<commit_message>
Add header and section borders spanning columns A-C.
Draw top/bottom borders on A1:C1 and on each display-key group
boundary so merged key blocks read as full-width sections.

Co-authored-by: EsaLongs <EsaLongs@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/preview/NP1PP_vs_C1Y_preview.xlsx
+++ b/preview/NP1PP_vs_C1Y_preview.xlsx
@@ -46,7 +46,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -54,18 +54,48 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+    </border>
+    <border>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+    </border>
+    <border>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -784,22 +814,22 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="inlineStr">
+      <c r="A25" s="5" t="inlineStr">
         <is>
           <t>AN2X8</t>
         </is>
       </c>
-      <c r="B25" s="3" t="n"/>
-      <c r="C25" s="3" t="inlineStr">
+      <c r="B25" s="6" t="n"/>
+      <c r="C25" s="6" t="inlineStr">
         <is>
           <t>AN2EEQMBDX8AR2COTC</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="n"/>
-      <c r="B26" s="3" t="n"/>
-      <c r="C26" s="3" t="inlineStr">
+      <c r="A26" s="7" t="n"/>
+      <c r="B26" s="8" t="n"/>
+      <c r="C26" s="8" t="inlineStr">
         <is>
           <t>AN2X8AR2COTC</t>
         </is>
@@ -1072,26 +1102,26 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="inlineStr">
+      <c r="A45" s="5" t="inlineStr">
         <is>
           <t>AO211D1</t>
         </is>
       </c>
-      <c r="B45" s="3" t="inlineStr">
+      <c r="B45" s="6" t="inlineStr">
         <is>
           <t>AO211D1COTMDB</t>
         </is>
       </c>
-      <c r="C45" s="3" t="inlineStr">
+      <c r="C45" s="6" t="inlineStr">
         <is>
           <t>AO211D1COT</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="n"/>
-      <c r="B46" s="3" t="n"/>
-      <c r="C46" s="3" t="inlineStr">
+      <c r="A46" s="7" t="n"/>
+      <c r="B46" s="8" t="n"/>
+      <c r="C46" s="8" t="inlineStr">
         <is>
           <t>AO211EEQMBDD1COT</t>
         </is>
@@ -1274,26 +1304,26 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="2" t="inlineStr">
+      <c r="A59" s="5" t="inlineStr">
         <is>
           <t>AO22D1</t>
         </is>
       </c>
-      <c r="B59" s="3" t="inlineStr">
+      <c r="B59" s="6" t="inlineStr">
         <is>
           <t>AO22D1COTMDB</t>
         </is>
       </c>
-      <c r="C59" s="3" t="inlineStr">
+      <c r="C59" s="6" t="inlineStr">
         <is>
           <t>AO22D1COT</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="2" t="n"/>
-      <c r="B60" s="3" t="n"/>
-      <c r="C60" s="3" t="inlineStr">
+      <c r="A60" s="7" t="n"/>
+      <c r="B60" s="8" t="n"/>
+      <c r="C60" s="8" t="inlineStr">
         <is>
           <t>AO22EEQMBDD1COT</t>
         </is>
@@ -1939,22 +1969,22 @@
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="2" t="inlineStr">
+      <c r="A104" s="5" t="inlineStr">
         <is>
           <t>AOI21X2</t>
         </is>
       </c>
-      <c r="B104" s="3" t="n"/>
-      <c r="C104" s="3" t="inlineStr">
+      <c r="B104" s="6" t="n"/>
+      <c r="C104" s="6" t="inlineStr">
         <is>
           <t>AOI21EEQMBDX2APBCOTC</t>
         </is>
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="2" t="n"/>
-      <c r="B105" s="3" t="n"/>
-      <c r="C105" s="3" t="inlineStr">
+      <c r="A105" s="7" t="n"/>
+      <c r="B105" s="8" t="n"/>
+      <c r="C105" s="8" t="inlineStr">
         <is>
           <t>AOI21X2APACOTC</t>
         </is>
@@ -1987,22 +2017,22 @@
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="2" t="inlineStr">
+      <c r="A108" s="5" t="inlineStr">
         <is>
           <t>AOI21X8</t>
         </is>
       </c>
-      <c r="B108" s="3" t="n"/>
-      <c r="C108" s="3" t="inlineStr">
+      <c r="B108" s="6" t="n"/>
+      <c r="C108" s="6" t="inlineStr">
         <is>
           <t>AOI21X8APACOTC</t>
         </is>
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="2" t="n"/>
-      <c r="B109" s="3" t="n"/>
-      <c r="C109" s="3" t="inlineStr">
+      <c r="A109" s="7" t="n"/>
+      <c r="B109" s="8" t="n"/>
+      <c r="C109" s="8" t="inlineStr">
         <is>
           <t>AOI21X8APBCOTC</t>
         </is>
@@ -2564,93 +2594,93 @@
       <c r="C148" s="3" t="n"/>
     </row>
     <row r="149">
-      <c r="A149" s="2" t="inlineStr">
+      <c r="A149" s="5" t="inlineStr">
         <is>
           <t>AOI22X1</t>
         </is>
       </c>
-      <c r="B149" s="3" t="n"/>
-      <c r="C149" s="3" t="inlineStr">
+      <c r="B149" s="6" t="n"/>
+      <c r="C149" s="6" t="inlineStr">
         <is>
           <t>AOI22X1APBCOTC</t>
         </is>
       </c>
     </row>
     <row r="150">
-      <c r="A150" s="2" t="n"/>
-      <c r="B150" s="3" t="n"/>
-      <c r="C150" s="3" t="inlineStr">
+      <c r="A150" s="9" t="n"/>
+      <c r="B150" s="10" t="n"/>
+      <c r="C150" s="10" t="inlineStr">
         <is>
           <t>AOI22X1APCCOTC</t>
         </is>
       </c>
     </row>
     <row r="151">
-      <c r="A151" s="2" t="n"/>
-      <c r="B151" s="3" t="n"/>
-      <c r="C151" s="3" t="inlineStr">
+      <c r="A151" s="9" t="n"/>
+      <c r="B151" s="10" t="n"/>
+      <c r="C151" s="10" t="inlineStr">
         <is>
           <t>AOI22X1APDCOTC</t>
         </is>
       </c>
     </row>
     <row r="152">
-      <c r="A152" s="2" t="n"/>
-      <c r="B152" s="3" t="n"/>
-      <c r="C152" s="3" t="inlineStr">
+      <c r="A152" s="9" t="n"/>
+      <c r="B152" s="10" t="n"/>
+      <c r="C152" s="10" t="inlineStr">
         <is>
           <t>AOI22X1APMCOTC</t>
         </is>
       </c>
     </row>
     <row r="153">
-      <c r="A153" s="2" t="n"/>
-      <c r="B153" s="3" t="n"/>
-      <c r="C153" s="3" t="inlineStr">
+      <c r="A153" s="7" t="n"/>
+      <c r="B153" s="8" t="n"/>
+      <c r="C153" s="8" t="inlineStr">
         <is>
           <t>AOI22X1APPCOTC</t>
         </is>
       </c>
     </row>
     <row r="154">
-      <c r="A154" s="2" t="inlineStr">
+      <c r="A154" s="5" t="inlineStr">
         <is>
           <t>AOI22X2</t>
         </is>
       </c>
-      <c r="B154" s="3" t="n"/>
-      <c r="C154" s="3" t="inlineStr">
+      <c r="B154" s="6" t="n"/>
+      <c r="C154" s="6" t="inlineStr">
         <is>
           <t>AOI22X2ANSCOTC</t>
         </is>
       </c>
     </row>
     <row r="155">
-      <c r="A155" s="2" t="n"/>
-      <c r="B155" s="3" t="n"/>
-      <c r="C155" s="3" t="inlineStr">
+      <c r="A155" s="7" t="n"/>
+      <c r="B155" s="8" t="n"/>
+      <c r="C155" s="8" t="inlineStr">
         <is>
           <t>AOI22X2APQCOTC</t>
         </is>
       </c>
     </row>
     <row r="156">
-      <c r="A156" s="2" t="inlineStr">
+      <c r="A156" s="5" t="inlineStr">
         <is>
           <t>AOI22X3</t>
         </is>
       </c>
-      <c r="B156" s="3" t="n"/>
-      <c r="C156" s="3" t="inlineStr">
+      <c r="B156" s="6" t="n"/>
+      <c r="C156" s="6" t="inlineStr">
         <is>
           <t>AOI22X3ANSCOTC</t>
         </is>
       </c>
     </row>
     <row r="157">
-      <c r="A157" s="2" t="n"/>
-      <c r="B157" s="3" t="n"/>
-      <c r="C157" s="3" t="inlineStr">
+      <c r="A157" s="7" t="n"/>
+      <c r="B157" s="8" t="n"/>
+      <c r="C157" s="8" t="inlineStr">
         <is>
           <t>AOI22X3APQCOT</t>
         </is>
@@ -3392,22 +3422,22 @@
       </c>
     </row>
     <row r="209">
-      <c r="A209" s="2" t="inlineStr">
+      <c r="A209" s="5" t="inlineStr">
         <is>
           <t>BUFX8</t>
         </is>
       </c>
-      <c r="B209" s="3" t="n"/>
-      <c r="C209" s="3" t="inlineStr">
+      <c r="B209" s="6" t="n"/>
+      <c r="C209" s="6" t="inlineStr">
         <is>
           <t>BUFX8AHACOT</t>
         </is>
       </c>
     </row>
     <row r="210">
-      <c r="A210" s="2" t="n"/>
-      <c r="B210" s="3" t="n"/>
-      <c r="C210" s="3" t="inlineStr">
+      <c r="A210" s="7" t="n"/>
+      <c r="B210" s="8" t="n"/>
+      <c r="C210" s="8" t="inlineStr">
         <is>
           <t>BUFX8AROCOT</t>
         </is>
@@ -3733,26 +3763,26 @@
       </c>
     </row>
     <row r="234">
-      <c r="A234" s="2" t="inlineStr">
+      <c r="A234" s="5" t="inlineStr">
         <is>
           <t>CKMUX2D8</t>
         </is>
       </c>
-      <c r="B234" s="3" t="inlineStr">
+      <c r="B234" s="6" t="inlineStr">
         <is>
           <t>CKMUX2D8COTM3CEQ</t>
         </is>
       </c>
-      <c r="C234" s="3" t="inlineStr">
+      <c r="C234" s="6" t="inlineStr">
         <is>
           <t>CKMUX2D8COT</t>
         </is>
       </c>
     </row>
     <row r="235">
-      <c r="A235" s="2" t="n"/>
-      <c r="B235" s="3" t="n"/>
-      <c r="C235" s="3" t="inlineStr">
+      <c r="A235" s="7" t="n"/>
+      <c r="B235" s="8" t="n"/>
+      <c r="C235" s="8" t="inlineStr">
         <is>
           <t>CKMUX2EEQMBDD8COT</t>
         </is>
@@ -4211,26 +4241,26 @@
       </c>
     </row>
     <row r="268">
-      <c r="A268" s="2" t="inlineStr">
+      <c r="A268" s="5" t="inlineStr">
         <is>
           <t>CMPE42D4</t>
         </is>
       </c>
-      <c r="B268" s="3" t="inlineStr">
+      <c r="B268" s="6" t="inlineStr">
         <is>
           <t>CMPE42D4COT</t>
         </is>
       </c>
-      <c r="C268" s="3" t="inlineStr">
+      <c r="C268" s="6" t="inlineStr">
         <is>
           <t>CMPE42D4OPTCOT</t>
         </is>
       </c>
     </row>
     <row r="269">
-      <c r="A269" s="2" t="n"/>
-      <c r="B269" s="3" t="n"/>
-      <c r="C269" s="3" t="inlineStr">
+      <c r="A269" s="7" t="n"/>
+      <c r="B269" s="8" t="n"/>
+      <c r="C269" s="8" t="inlineStr">
         <is>
           <t>CMPE42EEQMBDD4COT</t>
         </is>
@@ -4250,26 +4280,26 @@
       </c>
     </row>
     <row r="271">
-      <c r="A271" s="2" t="inlineStr">
+      <c r="A271" s="5" t="inlineStr">
         <is>
           <t>DC</t>
         </is>
       </c>
-      <c r="B271" s="3" t="inlineStr">
+      <c r="B271" s="6" t="inlineStr">
         <is>
           <t>DCAP4COT</t>
         </is>
       </c>
-      <c r="C271" s="3" t="n"/>
+      <c r="C271" s="6" t="n"/>
     </row>
     <row r="272">
-      <c r="A272" s="2" t="n"/>
-      <c r="B272" s="3" t="inlineStr">
+      <c r="A272" s="7" t="n"/>
+      <c r="B272" s="8" t="inlineStr">
         <is>
           <t>DCAP5COT</t>
         </is>
       </c>
-      <c r="C272" s="3" t="n"/>
+      <c r="C272" s="8" t="n"/>
     </row>
     <row r="273">
       <c r="A273" s="2" t="inlineStr">
@@ -6741,26 +6771,26 @@
       </c>
     </row>
     <row r="454">
-      <c r="A454" s="2" t="inlineStr">
+      <c r="A454" s="5" t="inlineStr">
         <is>
           <t>HDDID2</t>
         </is>
       </c>
-      <c r="B454" s="3" t="inlineStr">
+      <c r="B454" s="6" t="inlineStr">
         <is>
           <t>HDDID2A30COTARC</t>
         </is>
       </c>
-      <c r="C454" s="3" t="n"/>
+      <c r="C454" s="6" t="n"/>
     </row>
     <row r="455">
-      <c r="A455" s="2" t="n"/>
-      <c r="B455" s="3" t="inlineStr">
+      <c r="A455" s="7" t="n"/>
+      <c r="B455" s="8" t="inlineStr">
         <is>
           <t>HDDID2A40COTARC</t>
         </is>
       </c>
-      <c r="C455" s="3" t="n"/>
+      <c r="C455" s="8" t="n"/>
     </row>
     <row r="456">
       <c r="A456" s="2" t="inlineStr">
@@ -6776,26 +6806,26 @@
       <c r="C456" s="3" t="n"/>
     </row>
     <row r="457">
-      <c r="A457" s="2" t="inlineStr">
+      <c r="A457" s="5" t="inlineStr">
         <is>
           <t>IAO21D2</t>
         </is>
       </c>
-      <c r="B457" s="3" t="inlineStr">
+      <c r="B457" s="6" t="inlineStr">
         <is>
           <t>IAO21D2COT</t>
         </is>
       </c>
-      <c r="C457" s="3" t="inlineStr">
+      <c r="C457" s="6" t="inlineStr">
         <is>
           <t>IAO21D2COT3FIN</t>
         </is>
       </c>
     </row>
     <row r="458">
-      <c r="A458" s="2" t="n"/>
-      <c r="B458" s="3" t="n"/>
-      <c r="C458" s="3" t="inlineStr">
+      <c r="A458" s="7" t="n"/>
+      <c r="B458" s="8" t="n"/>
+      <c r="C458" s="8" t="inlineStr">
         <is>
           <t>IAO21EEQMBDD2COT</t>
         </is>
@@ -6879,26 +6909,26 @@
       </c>
     </row>
     <row r="464">
-      <c r="A464" s="2" t="inlineStr">
+      <c r="A464" s="5" t="inlineStr">
         <is>
           <t>IAOI21D1</t>
         </is>
       </c>
-      <c r="B464" s="3" t="inlineStr">
+      <c r="B464" s="6" t="inlineStr">
         <is>
           <t>IAOI21D1COTOPU</t>
         </is>
       </c>
-      <c r="C464" s="3" t="inlineStr">
+      <c r="C464" s="6" t="inlineStr">
         <is>
           <t>IAOI21D1COT</t>
         </is>
       </c>
     </row>
     <row r="465">
-      <c r="A465" s="2" t="n"/>
-      <c r="B465" s="3" t="n"/>
-      <c r="C465" s="3" t="inlineStr">
+      <c r="A465" s="7" t="n"/>
+      <c r="B465" s="8" t="n"/>
+      <c r="C465" s="8" t="inlineStr">
         <is>
           <t>IAOI21EEQMBDD1COT</t>
         </is>
@@ -9396,22 +9426,22 @@
       </c>
     </row>
     <row r="645">
-      <c r="A645" s="2" t="inlineStr">
+      <c r="A645" s="5" t="inlineStr">
         <is>
           <t>MX2X2</t>
         </is>
       </c>
-      <c r="B645" s="3" t="n"/>
-      <c r="C645" s="3" t="inlineStr">
+      <c r="B645" s="6" t="n"/>
+      <c r="C645" s="6" t="inlineStr">
         <is>
           <t>MX2X2ATACOTC</t>
         </is>
       </c>
     </row>
     <row r="646">
-      <c r="A646" s="2" t="n"/>
-      <c r="B646" s="3" t="n"/>
-      <c r="C646" s="3" t="inlineStr">
+      <c r="A646" s="7" t="n"/>
+      <c r="B646" s="8" t="n"/>
+      <c r="C646" s="8" t="inlineStr">
         <is>
           <t>MX2X2ATFCOTC</t>
         </is>
@@ -9431,53 +9461,53 @@
       </c>
     </row>
     <row r="648">
-      <c r="A648" s="2" t="inlineStr">
+      <c r="A648" s="5" t="inlineStr">
         <is>
           <t>MXI2X1</t>
         </is>
       </c>
-      <c r="B648" s="3" t="n"/>
-      <c r="C648" s="3" t="inlineStr">
+      <c r="B648" s="6" t="n"/>
+      <c r="C648" s="6" t="inlineStr">
         <is>
           <t>MXI2X1ATACOTC</t>
         </is>
       </c>
     </row>
     <row r="649">
-      <c r="A649" s="2" t="n"/>
-      <c r="B649" s="3" t="n"/>
-      <c r="C649" s="3" t="inlineStr">
+      <c r="A649" s="7" t="n"/>
+      <c r="B649" s="8" t="n"/>
+      <c r="C649" s="8" t="inlineStr">
         <is>
           <t>MXI2X1ATBCOTC</t>
         </is>
       </c>
     </row>
     <row r="650">
-      <c r="A650" s="2" t="inlineStr">
+      <c r="A650" s="5" t="inlineStr">
         <is>
           <t>MXI2X2</t>
         </is>
       </c>
-      <c r="B650" s="3" t="n"/>
-      <c r="C650" s="3" t="inlineStr">
+      <c r="B650" s="6" t="n"/>
+      <c r="C650" s="6" t="inlineStr">
         <is>
           <t>MXI2X2ATACOTC</t>
         </is>
       </c>
     </row>
     <row r="651">
-      <c r="A651" s="2" t="n"/>
-      <c r="B651" s="3" t="n"/>
-      <c r="C651" s="3" t="inlineStr">
+      <c r="A651" s="9" t="n"/>
+      <c r="B651" s="10" t="n"/>
+      <c r="C651" s="10" t="inlineStr">
         <is>
           <t>MXI2X2ATBCOTC</t>
         </is>
       </c>
     </row>
     <row r="652">
-      <c r="A652" s="2" t="n"/>
-      <c r="B652" s="3" t="n"/>
-      <c r="C652" s="3" t="inlineStr">
+      <c r="A652" s="7" t="n"/>
+      <c r="B652" s="8" t="n"/>
+      <c r="C652" s="8" t="inlineStr">
         <is>
           <t>MXI2X2ATSCOTC</t>
         </is>
@@ -9497,31 +9527,31 @@
       </c>
     </row>
     <row r="654">
-      <c r="A654" s="2" t="inlineStr">
+      <c r="A654" s="5" t="inlineStr">
         <is>
           <t>MXI2X4</t>
         </is>
       </c>
-      <c r="B654" s="3" t="n"/>
-      <c r="C654" s="3" t="inlineStr">
+      <c r="B654" s="6" t="n"/>
+      <c r="C654" s="6" t="inlineStr">
         <is>
           <t>MXI2X4ATACOTC</t>
         </is>
       </c>
     </row>
     <row r="655">
-      <c r="A655" s="2" t="n"/>
-      <c r="B655" s="3" t="n"/>
-      <c r="C655" s="3" t="inlineStr">
+      <c r="A655" s="9" t="n"/>
+      <c r="B655" s="10" t="n"/>
+      <c r="C655" s="10" t="inlineStr">
         <is>
           <t>MXI2X4ATBCOTC</t>
         </is>
       </c>
     </row>
     <row r="656">
-      <c r="A656" s="2" t="n"/>
-      <c r="B656" s="3" t="n"/>
-      <c r="C656" s="3" t="inlineStr">
+      <c r="A656" s="7" t="n"/>
+      <c r="B656" s="8" t="n"/>
+      <c r="C656" s="8" t="inlineStr">
         <is>
           <t>MXI2X4ATSCOTC</t>
         </is>
@@ -9541,22 +9571,22 @@
       </c>
     </row>
     <row r="658">
-      <c r="A658" s="2" t="inlineStr">
+      <c r="A658" s="5" t="inlineStr">
         <is>
           <t>MXI2X8</t>
         </is>
       </c>
-      <c r="B658" s="3" t="n"/>
-      <c r="C658" s="3" t="inlineStr">
+      <c r="B658" s="6" t="n"/>
+      <c r="C658" s="6" t="inlineStr">
         <is>
           <t>MXI2X8ATACOTC</t>
         </is>
       </c>
     </row>
     <row r="659">
-      <c r="A659" s="2" t="n"/>
-      <c r="B659" s="3" t="n"/>
-      <c r="C659" s="3" t="inlineStr">
+      <c r="A659" s="7" t="n"/>
+      <c r="B659" s="8" t="n"/>
+      <c r="C659" s="8" t="inlineStr">
         <is>
           <t>MXI2X8ATSCOTC</t>
         </is>
@@ -9843,53 +9873,53 @@
       <c r="C679" s="3" t="n"/>
     </row>
     <row r="680">
-      <c r="A680" s="2" t="inlineStr">
+      <c r="A680" s="5" t="inlineStr">
         <is>
           <t>ND2X1</t>
         </is>
       </c>
-      <c r="B680" s="3" t="n"/>
-      <c r="C680" s="3" t="inlineStr">
+      <c r="B680" s="6" t="n"/>
+      <c r="C680" s="6" t="inlineStr">
         <is>
           <t>ND2X1AKPCOTC</t>
         </is>
       </c>
     </row>
     <row r="681">
-      <c r="A681" s="2" t="n"/>
-      <c r="B681" s="3" t="n"/>
-      <c r="C681" s="3" t="inlineStr">
+      <c r="A681" s="7" t="n"/>
+      <c r="B681" s="8" t="n"/>
+      <c r="C681" s="8" t="inlineStr">
         <is>
           <t>ND2X1APNCOTC</t>
         </is>
       </c>
     </row>
     <row r="682">
-      <c r="A682" s="2" t="inlineStr">
+      <c r="A682" s="5" t="inlineStr">
         <is>
           <t>ND2X10</t>
         </is>
       </c>
-      <c r="B682" s="3" t="n"/>
-      <c r="C682" s="3" t="inlineStr">
+      <c r="B682" s="6" t="n"/>
+      <c r="C682" s="6" t="inlineStr">
         <is>
           <t>ND2X10AKPCOTC</t>
         </is>
       </c>
     </row>
     <row r="683">
-      <c r="A683" s="2" t="n"/>
-      <c r="B683" s="3" t="n"/>
-      <c r="C683" s="3" t="inlineStr">
+      <c r="A683" s="9" t="n"/>
+      <c r="B683" s="10" t="n"/>
+      <c r="C683" s="10" t="inlineStr">
         <is>
           <t>ND2X10APBCOTC</t>
         </is>
       </c>
     </row>
     <row r="684">
-      <c r="A684" s="2" t="n"/>
-      <c r="B684" s="3" t="n"/>
-      <c r="C684" s="3" t="inlineStr">
+      <c r="A684" s="7" t="n"/>
+      <c r="B684" s="8" t="n"/>
+      <c r="C684" s="8" t="inlineStr">
         <is>
           <t>ND2X10APNCOTC</t>
         </is>
@@ -9935,31 +9965,31 @@
       </c>
     </row>
     <row r="688">
-      <c r="A688" s="2" t="inlineStr">
+      <c r="A688" s="5" t="inlineStr">
         <is>
           <t>ND2X2</t>
         </is>
       </c>
-      <c r="B688" s="3" t="n"/>
-      <c r="C688" s="3" t="inlineStr">
+      <c r="B688" s="6" t="n"/>
+      <c r="C688" s="6" t="inlineStr">
         <is>
           <t>ND2X2AKPCOTC</t>
         </is>
       </c>
     </row>
     <row r="689">
-      <c r="A689" s="2" t="n"/>
-      <c r="B689" s="3" t="n"/>
-      <c r="C689" s="3" t="inlineStr">
+      <c r="A689" s="9" t="n"/>
+      <c r="B689" s="10" t="n"/>
+      <c r="C689" s="10" t="inlineStr">
         <is>
           <t>ND2X2APBCOTC</t>
         </is>
       </c>
     </row>
     <row r="690">
-      <c r="A690" s="2" t="n"/>
-      <c r="B690" s="3" t="n"/>
-      <c r="C690" s="3" t="inlineStr">
+      <c r="A690" s="7" t="n"/>
+      <c r="B690" s="8" t="n"/>
+      <c r="C690" s="8" t="inlineStr">
         <is>
           <t>ND2X2APNCOTC</t>
         </is>
@@ -9979,71 +10009,71 @@
       </c>
     </row>
     <row r="692">
-      <c r="A692" s="2" t="inlineStr">
+      <c r="A692" s="5" t="inlineStr">
         <is>
           <t>ND2X4</t>
         </is>
       </c>
-      <c r="B692" s="3" t="n"/>
-      <c r="C692" s="3" t="inlineStr">
+      <c r="B692" s="6" t="n"/>
+      <c r="C692" s="6" t="inlineStr">
         <is>
           <t>ND2X4APACOT3FINC</t>
         </is>
       </c>
     </row>
     <row r="693">
-      <c r="A693" s="2" t="n"/>
-      <c r="B693" s="3" t="n"/>
-      <c r="C693" s="3" t="inlineStr">
+      <c r="A693" s="9" t="n"/>
+      <c r="B693" s="10" t="n"/>
+      <c r="C693" s="10" t="inlineStr">
         <is>
           <t>ND2X4APBCOTC</t>
         </is>
       </c>
     </row>
     <row r="694">
-      <c r="A694" s="2" t="n"/>
-      <c r="B694" s="3" t="n"/>
-      <c r="C694" s="3" t="inlineStr">
+      <c r="A694" s="9" t="n"/>
+      <c r="B694" s="10" t="n"/>
+      <c r="C694" s="10" t="inlineStr">
         <is>
           <t>ND2X4APNCOTC</t>
         </is>
       </c>
     </row>
     <row r="695">
-      <c r="A695" s="2" t="n"/>
-      <c r="B695" s="3" t="n"/>
-      <c r="C695" s="3" t="inlineStr">
+      <c r="A695" s="7" t="n"/>
+      <c r="B695" s="8" t="n"/>
+      <c r="C695" s="8" t="inlineStr">
         <is>
           <t>ND2X4ARQCOT</t>
         </is>
       </c>
     </row>
     <row r="696">
-      <c r="A696" s="2" t="inlineStr">
+      <c r="A696" s="5" t="inlineStr">
         <is>
           <t>ND2X6</t>
         </is>
       </c>
-      <c r="B696" s="3" t="n"/>
-      <c r="C696" s="3" t="inlineStr">
+      <c r="B696" s="6" t="n"/>
+      <c r="C696" s="6" t="inlineStr">
         <is>
           <t>ND2X6AKPCOTC</t>
         </is>
       </c>
     </row>
     <row r="697">
-      <c r="A697" s="2" t="n"/>
-      <c r="B697" s="3" t="n"/>
-      <c r="C697" s="3" t="inlineStr">
+      <c r="A697" s="9" t="n"/>
+      <c r="B697" s="10" t="n"/>
+      <c r="C697" s="10" t="inlineStr">
         <is>
           <t>ND2X6APNCOTC</t>
         </is>
       </c>
     </row>
     <row r="698">
-      <c r="A698" s="2" t="n"/>
-      <c r="B698" s="3" t="n"/>
-      <c r="C698" s="3" t="inlineStr">
+      <c r="A698" s="7" t="n"/>
+      <c r="B698" s="8" t="n"/>
+      <c r="C698" s="8" t="inlineStr">
         <is>
           <t>ND2X6AROCOT</t>
         </is>
@@ -10063,31 +10093,31 @@
       </c>
     </row>
     <row r="700">
-      <c r="A700" s="2" t="inlineStr">
+      <c r="A700" s="5" t="inlineStr">
         <is>
           <t>ND2X8</t>
         </is>
       </c>
-      <c r="B700" s="3" t="n"/>
-      <c r="C700" s="3" t="inlineStr">
+      <c r="B700" s="6" t="n"/>
+      <c r="C700" s="6" t="inlineStr">
         <is>
           <t>ND2X8APACOT3FINC</t>
         </is>
       </c>
     </row>
     <row r="701">
-      <c r="A701" s="2" t="n"/>
-      <c r="B701" s="3" t="n"/>
-      <c r="C701" s="3" t="inlineStr">
+      <c r="A701" s="9" t="n"/>
+      <c r="B701" s="10" t="n"/>
+      <c r="C701" s="10" t="inlineStr">
         <is>
           <t>ND2X8APBCOTC</t>
         </is>
       </c>
     </row>
     <row r="702">
-      <c r="A702" s="2" t="n"/>
-      <c r="B702" s="3" t="n"/>
-      <c r="C702" s="3" t="inlineStr">
+      <c r="A702" s="7" t="n"/>
+      <c r="B702" s="8" t="n"/>
+      <c r="C702" s="8" t="inlineStr">
         <is>
           <t>ND2X8APNCOTC</t>
         </is>
@@ -10456,22 +10486,22 @@
       </c>
     </row>
     <row r="729">
-      <c r="A729" s="2" t="inlineStr">
+      <c r="A729" s="5" t="inlineStr">
         <is>
           <t>NR2N1X12</t>
         </is>
       </c>
-      <c r="B729" s="3" t="n"/>
-      <c r="C729" s="3" t="inlineStr">
+      <c r="B729" s="6" t="n"/>
+      <c r="C729" s="6" t="inlineStr">
         <is>
           <t>NR2N1X12APPCOTC</t>
         </is>
       </c>
     </row>
     <row r="730">
-      <c r="A730" s="2" t="n"/>
-      <c r="B730" s="3" t="n"/>
-      <c r="C730" s="3" t="inlineStr">
+      <c r="A730" s="7" t="n"/>
+      <c r="B730" s="8" t="n"/>
+      <c r="C730" s="8" t="inlineStr">
         <is>
           <t>NR2N1X12AROCOT</t>
         </is>
@@ -10621,159 +10651,159 @@
       </c>
     </row>
     <row r="742">
-      <c r="A742" s="2" t="inlineStr">
+      <c r="A742" s="5" t="inlineStr">
         <is>
           <t>NR2X1</t>
         </is>
       </c>
-      <c r="B742" s="3" t="n"/>
-      <c r="C742" s="3" t="inlineStr">
+      <c r="B742" s="6" t="n"/>
+      <c r="C742" s="6" t="inlineStr">
         <is>
           <t>NR2X1AKNCOTC</t>
         </is>
       </c>
     </row>
     <row r="743">
-      <c r="A743" s="2" t="n"/>
-      <c r="B743" s="3" t="n"/>
-      <c r="C743" s="3" t="inlineStr">
+      <c r="A743" s="9" t="n"/>
+      <c r="B743" s="10" t="n"/>
+      <c r="C743" s="10" t="inlineStr">
         <is>
           <t>NR2X1APACOTC</t>
         </is>
       </c>
     </row>
     <row r="744">
-      <c r="A744" s="2" t="n"/>
-      <c r="B744" s="3" t="n"/>
-      <c r="C744" s="3" t="inlineStr">
+      <c r="A744" s="7" t="n"/>
+      <c r="B744" s="8" t="n"/>
+      <c r="C744" s="8" t="inlineStr">
         <is>
           <t>NR2X1APPCOTC</t>
         </is>
       </c>
     </row>
     <row r="745">
-      <c r="A745" s="2" t="inlineStr">
+      <c r="A745" s="5" t="inlineStr">
         <is>
           <t>NR2X10</t>
         </is>
       </c>
-      <c r="B745" s="3" t="n"/>
-      <c r="C745" s="3" t="inlineStr">
+      <c r="B745" s="6" t="n"/>
+      <c r="C745" s="6" t="inlineStr">
         <is>
           <t>NR2X10APBCOTC</t>
         </is>
       </c>
     </row>
     <row r="746">
-      <c r="A746" s="2" t="n"/>
-      <c r="B746" s="3" t="n"/>
-      <c r="C746" s="3" t="inlineStr">
+      <c r="A746" s="7" t="n"/>
+      <c r="B746" s="8" t="n"/>
+      <c r="C746" s="8" t="inlineStr">
         <is>
           <t>NR2X10APPCOTC</t>
         </is>
       </c>
     </row>
     <row r="747">
-      <c r="A747" s="2" t="inlineStr">
+      <c r="A747" s="5" t="inlineStr">
         <is>
           <t>NR2X12</t>
         </is>
       </c>
-      <c r="B747" s="3" t="n"/>
-      <c r="C747" s="3" t="inlineStr">
+      <c r="B747" s="6" t="n"/>
+      <c r="C747" s="6" t="inlineStr">
         <is>
           <t>NR2X12AKNCOTC</t>
         </is>
       </c>
     </row>
     <row r="748">
-      <c r="A748" s="2" t="n"/>
-      <c r="B748" s="3" t="n"/>
-      <c r="C748" s="3" t="inlineStr">
+      <c r="A748" s="9" t="n"/>
+      <c r="B748" s="10" t="n"/>
+      <c r="C748" s="10" t="inlineStr">
         <is>
           <t>NR2X12APACOTC</t>
         </is>
       </c>
     </row>
     <row r="749">
-      <c r="A749" s="2" t="n"/>
-      <c r="B749" s="3" t="n"/>
-      <c r="C749" s="3" t="inlineStr">
+      <c r="A749" s="7" t="n"/>
+      <c r="B749" s="8" t="n"/>
+      <c r="C749" s="8" t="inlineStr">
         <is>
           <t>NR2X12APPCOTC</t>
         </is>
       </c>
     </row>
     <row r="750">
-      <c r="A750" s="2" t="inlineStr">
+      <c r="A750" s="5" t="inlineStr">
         <is>
           <t>NR2X14</t>
         </is>
       </c>
-      <c r="B750" s="3" t="n"/>
-      <c r="C750" s="3" t="inlineStr">
+      <c r="B750" s="6" t="n"/>
+      <c r="C750" s="6" t="inlineStr">
         <is>
           <t>NR2X14APBCOTC</t>
         </is>
       </c>
     </row>
     <row r="751">
-      <c r="A751" s="2" t="n"/>
-      <c r="B751" s="3" t="n"/>
-      <c r="C751" s="3" t="inlineStr">
+      <c r="A751" s="7" t="n"/>
+      <c r="B751" s="8" t="n"/>
+      <c r="C751" s="8" t="inlineStr">
         <is>
           <t>NR2X14APPCOTC</t>
         </is>
       </c>
     </row>
     <row r="752">
-      <c r="A752" s="2" t="inlineStr">
+      <c r="A752" s="5" t="inlineStr">
         <is>
           <t>NR2X16</t>
         </is>
       </c>
-      <c r="B752" s="3" t="n"/>
-      <c r="C752" s="3" t="inlineStr">
+      <c r="B752" s="6" t="n"/>
+      <c r="C752" s="6" t="inlineStr">
         <is>
           <t>NR2X16APACOTC</t>
         </is>
       </c>
     </row>
     <row r="753">
-      <c r="A753" s="2" t="n"/>
-      <c r="B753" s="3" t="n"/>
-      <c r="C753" s="3" t="inlineStr">
+      <c r="A753" s="9" t="n"/>
+      <c r="B753" s="10" t="n"/>
+      <c r="C753" s="10" t="inlineStr">
         <is>
           <t>NR2X16APBCOTC</t>
         </is>
       </c>
     </row>
     <row r="754">
-      <c r="A754" s="2" t="n"/>
-      <c r="B754" s="3" t="n"/>
-      <c r="C754" s="3" t="inlineStr">
+      <c r="A754" s="7" t="n"/>
+      <c r="B754" s="8" t="n"/>
+      <c r="C754" s="8" t="inlineStr">
         <is>
           <t>NR2X16APPCOTC</t>
         </is>
       </c>
     </row>
     <row r="755">
-      <c r="A755" s="2" t="inlineStr">
+      <c r="A755" s="5" t="inlineStr">
         <is>
           <t>NR2X2</t>
         </is>
       </c>
-      <c r="B755" s="3" t="n"/>
-      <c r="C755" s="3" t="inlineStr">
+      <c r="B755" s="6" t="n"/>
+      <c r="C755" s="6" t="inlineStr">
         <is>
           <t>NR2X2AKNCOT3FINC</t>
         </is>
       </c>
     </row>
     <row r="756">
-      <c r="A756" s="2" t="n"/>
-      <c r="B756" s="3" t="n"/>
-      <c r="C756" s="3" t="inlineStr">
+      <c r="A756" s="7" t="n"/>
+      <c r="B756" s="8" t="n"/>
+      <c r="C756" s="8" t="inlineStr">
         <is>
           <t>NR2X2APPCOT3FINC</t>
         </is>
@@ -10793,111 +10823,111 @@
       </c>
     </row>
     <row r="758">
-      <c r="A758" s="2" t="inlineStr">
+      <c r="A758" s="5" t="inlineStr">
         <is>
           <t>NR2X4</t>
         </is>
       </c>
-      <c r="B758" s="3" t="n"/>
-      <c r="C758" s="3" t="inlineStr">
+      <c r="B758" s="6" t="n"/>
+      <c r="C758" s="6" t="inlineStr">
         <is>
           <t>NR2X4AKNCOTC</t>
         </is>
       </c>
     </row>
     <row r="759">
-      <c r="A759" s="2" t="n"/>
-      <c r="B759" s="3" t="n"/>
-      <c r="C759" s="3" t="inlineStr">
+      <c r="A759" s="9" t="n"/>
+      <c r="B759" s="10" t="n"/>
+      <c r="C759" s="10" t="inlineStr">
         <is>
           <t>NR2X4APACOTC</t>
         </is>
       </c>
     </row>
     <row r="760">
-      <c r="A760" s="2" t="n"/>
-      <c r="B760" s="3" t="n"/>
-      <c r="C760" s="3" t="inlineStr">
+      <c r="A760" s="9" t="n"/>
+      <c r="B760" s="10" t="n"/>
+      <c r="C760" s="10" t="inlineStr">
         <is>
           <t>NR2X4APBCOTC</t>
         </is>
       </c>
     </row>
     <row r="761">
-      <c r="A761" s="2" t="n"/>
-      <c r="B761" s="3" t="n"/>
-      <c r="C761" s="3" t="inlineStr">
+      <c r="A761" s="7" t="n"/>
+      <c r="B761" s="8" t="n"/>
+      <c r="C761" s="8" t="inlineStr">
         <is>
           <t>NR2X4ARQCOT</t>
         </is>
       </c>
     </row>
     <row r="762">
-      <c r="A762" s="2" t="inlineStr">
+      <c r="A762" s="5" t="inlineStr">
         <is>
           <t>NR2X6</t>
         </is>
       </c>
-      <c r="B762" s="3" t="n"/>
-      <c r="C762" s="3" t="inlineStr">
+      <c r="B762" s="6" t="n"/>
+      <c r="C762" s="6" t="inlineStr">
         <is>
           <t>NR2X6APACOTC</t>
         </is>
       </c>
     </row>
     <row r="763">
-      <c r="A763" s="2" t="n"/>
-      <c r="B763" s="3" t="n"/>
-      <c r="C763" s="3" t="inlineStr">
+      <c r="A763" s="9" t="n"/>
+      <c r="B763" s="10" t="n"/>
+      <c r="C763" s="10" t="inlineStr">
         <is>
           <t>NR2X6APBCOTC</t>
         </is>
       </c>
     </row>
     <row r="764">
-      <c r="A764" s="2" t="n"/>
-      <c r="B764" s="3" t="n"/>
-      <c r="C764" s="3" t="inlineStr">
+      <c r="A764" s="7" t="n"/>
+      <c r="B764" s="8" t="n"/>
+      <c r="C764" s="8" t="inlineStr">
         <is>
           <t>NR2X6ARQCOT</t>
         </is>
       </c>
     </row>
     <row r="765">
-      <c r="A765" s="2" t="inlineStr">
+      <c r="A765" s="5" t="inlineStr">
         <is>
           <t>NR2X8</t>
         </is>
       </c>
-      <c r="B765" s="3" t="n"/>
-      <c r="C765" s="3" t="inlineStr">
+      <c r="B765" s="6" t="n"/>
+      <c r="C765" s="6" t="inlineStr">
         <is>
           <t>NR2X8APACOTC</t>
         </is>
       </c>
     </row>
     <row r="766">
-      <c r="A766" s="2" t="n"/>
-      <c r="B766" s="3" t="n"/>
-      <c r="C766" s="3" t="inlineStr">
+      <c r="A766" s="9" t="n"/>
+      <c r="B766" s="10" t="n"/>
+      <c r="C766" s="10" t="inlineStr">
         <is>
           <t>NR2X8APBCOTC</t>
         </is>
       </c>
     </row>
     <row r="767">
-      <c r="A767" s="2" t="n"/>
-      <c r="B767" s="3" t="n"/>
-      <c r="C767" s="3" t="inlineStr">
+      <c r="A767" s="9" t="n"/>
+      <c r="B767" s="10" t="n"/>
+      <c r="C767" s="10" t="inlineStr">
         <is>
           <t>NR2X8APPCOTC</t>
         </is>
       </c>
     </row>
     <row r="768">
-      <c r="A768" s="2" t="n"/>
-      <c r="B768" s="3" t="n"/>
-      <c r="C768" s="3" t="inlineStr">
+      <c r="A768" s="7" t="n"/>
+      <c r="B768" s="8" t="n"/>
+      <c r="C768" s="8" t="inlineStr">
         <is>
           <t>NR2X8AROCOT</t>
         </is>
@@ -11157,26 +11187,26 @@
       </c>
     </row>
     <row r="786">
-      <c r="A786" s="2" t="inlineStr">
+      <c r="A786" s="5" t="inlineStr">
         <is>
           <t>OA211D1</t>
         </is>
       </c>
-      <c r="B786" s="3" t="inlineStr">
+      <c r="B786" s="6" t="inlineStr">
         <is>
           <t>OA211D1COTMVM2OPU</t>
         </is>
       </c>
-      <c r="C786" s="3" t="inlineStr">
+      <c r="C786" s="6" t="inlineStr">
         <is>
           <t>OA211D1COT</t>
         </is>
       </c>
     </row>
     <row r="787">
-      <c r="A787" s="2" t="n"/>
-      <c r="B787" s="3" t="n"/>
-      <c r="C787" s="3" t="inlineStr">
+      <c r="A787" s="7" t="n"/>
+      <c r="B787" s="8" t="n"/>
+      <c r="C787" s="8" t="inlineStr">
         <is>
           <t>OA211EEQMBDD1COT</t>
         </is>
@@ -11304,26 +11334,26 @@
       <c r="C796" s="3" t="n"/>
     </row>
     <row r="797">
-      <c r="A797" s="2" t="inlineStr">
+      <c r="A797" s="5" t="inlineStr">
         <is>
           <t>OA222D1</t>
         </is>
       </c>
-      <c r="B797" s="3" t="inlineStr">
+      <c r="B797" s="6" t="inlineStr">
         <is>
           <t>OA222D1COTVIA</t>
         </is>
       </c>
-      <c r="C797" s="3" t="inlineStr">
+      <c r="C797" s="6" t="inlineStr">
         <is>
           <t>OA222D1COTA</t>
         </is>
       </c>
     </row>
     <row r="798">
-      <c r="A798" s="2" t="n"/>
-      <c r="B798" s="3" t="n"/>
-      <c r="C798" s="3" t="inlineStr">
+      <c r="A798" s="7" t="n"/>
+      <c r="B798" s="8" t="n"/>
+      <c r="C798" s="8" t="inlineStr">
         <is>
           <t>OA222EEQMBDD1COTA</t>
         </is>
@@ -11661,26 +11691,26 @@
       </c>
     </row>
     <row r="822">
-      <c r="A822" s="2" t="inlineStr">
+      <c r="A822" s="5" t="inlineStr">
         <is>
           <t>OAI21D1</t>
         </is>
       </c>
-      <c r="B822" s="3" t="inlineStr">
+      <c r="B822" s="6" t="inlineStr">
         <is>
           <t>OAI21D1COTOPTPA</t>
         </is>
       </c>
-      <c r="C822" s="3" t="inlineStr">
+      <c r="C822" s="6" t="inlineStr">
         <is>
           <t>OAI21D1COT</t>
         </is>
       </c>
     </row>
     <row r="823">
-      <c r="A823" s="2" t="n"/>
-      <c r="B823" s="3" t="n"/>
-      <c r="C823" s="3" t="inlineStr">
+      <c r="A823" s="7" t="n"/>
+      <c r="B823" s="8" t="n"/>
+      <c r="C823" s="8" t="inlineStr">
         <is>
           <t>OAI21EEQMBCD1COT</t>
         </is>
@@ -11799,22 +11829,22 @@
       </c>
     </row>
     <row r="832">
-      <c r="A832" s="2" t="inlineStr">
+      <c r="A832" s="5" t="inlineStr">
         <is>
           <t>OAI21N2X8</t>
         </is>
       </c>
-      <c r="B832" s="3" t="n"/>
-      <c r="C832" s="3" t="inlineStr">
+      <c r="B832" s="6" t="n"/>
+      <c r="C832" s="6" t="inlineStr">
         <is>
           <t>OAI21N2X8APACOTC</t>
         </is>
       </c>
     </row>
     <row r="833">
-      <c r="A833" s="2" t="n"/>
-      <c r="B833" s="3" t="n"/>
-      <c r="C833" s="3" t="inlineStr">
+      <c r="A833" s="7" t="n"/>
+      <c r="B833" s="8" t="n"/>
+      <c r="C833" s="8" t="inlineStr">
         <is>
           <t>OAI21N2X8COTC</t>
         </is>
@@ -12170,26 +12200,26 @@
       </c>
     </row>
     <row r="859">
-      <c r="A859" s="2" t="inlineStr">
+      <c r="A859" s="5" t="inlineStr">
         <is>
           <t>OAI2222D1</t>
         </is>
       </c>
-      <c r="B859" s="3" t="inlineStr">
+      <c r="B859" s="6" t="inlineStr">
         <is>
           <t>OAI2222D1COTOPTPA</t>
         </is>
       </c>
-      <c r="C859" s="3" t="inlineStr">
+      <c r="C859" s="6" t="inlineStr">
         <is>
           <t>OAI2222D1COTA</t>
         </is>
       </c>
     </row>
     <row r="860">
-      <c r="A860" s="2" t="n"/>
-      <c r="B860" s="3" t="n"/>
-      <c r="C860" s="3" t="inlineStr">
+      <c r="A860" s="7" t="n"/>
+      <c r="B860" s="8" t="n"/>
+      <c r="C860" s="8" t="inlineStr">
         <is>
           <t>OAI2222EEQMBDD1COTA</t>
         </is>
@@ -13145,22 +13175,22 @@
       </c>
     </row>
     <row r="926">
-      <c r="A926" s="2" t="inlineStr">
+      <c r="A926" s="5" t="inlineStr">
         <is>
           <t>OR2X4</t>
         </is>
       </c>
-      <c r="B926" s="3" t="n"/>
-      <c r="C926" s="3" t="inlineStr">
+      <c r="B926" s="6" t="n"/>
+      <c r="C926" s="6" t="inlineStr">
         <is>
           <t>OR2EEQMBDX4ARNCOTC</t>
         </is>
       </c>
     </row>
     <row r="927">
-      <c r="A927" s="2" t="n"/>
-      <c r="B927" s="3" t="n"/>
-      <c r="C927" s="3" t="inlineStr">
+      <c r="A927" s="7" t="n"/>
+      <c r="B927" s="8" t="n"/>
+      <c r="C927" s="8" t="inlineStr">
         <is>
           <t>OR2X4ARNCOTC</t>
         </is>
@@ -13193,31 +13223,31 @@
       </c>
     </row>
     <row r="930">
-      <c r="A930" s="2" t="inlineStr">
+      <c r="A930" s="5" t="inlineStr">
         <is>
           <t>OR2X8</t>
         </is>
       </c>
-      <c r="B930" s="3" t="n"/>
-      <c r="C930" s="3" t="inlineStr">
+      <c r="B930" s="6" t="n"/>
+      <c r="C930" s="6" t="inlineStr">
         <is>
           <t>OR2EEQMBDX8AR2COTC</t>
         </is>
       </c>
     </row>
     <row r="931">
-      <c r="A931" s="2" t="n"/>
-      <c r="B931" s="3" t="n"/>
-      <c r="C931" s="3" t="inlineStr">
+      <c r="A931" s="9" t="n"/>
+      <c r="B931" s="10" t="n"/>
+      <c r="C931" s="10" t="inlineStr">
         <is>
           <t>OR2X8AR2COT3FINC</t>
         </is>
       </c>
     </row>
     <row r="932">
-      <c r="A932" s="2" t="n"/>
-      <c r="B932" s="3" t="n"/>
-      <c r="C932" s="3" t="inlineStr">
+      <c r="A932" s="7" t="n"/>
+      <c r="B932" s="8" t="n"/>
+      <c r="C932" s="8" t="inlineStr">
         <is>
           <t>OR2X8ARNCOTC</t>
         </is>
@@ -13555,44 +13585,44 @@
       </c>
     </row>
     <row r="956">
-      <c r="A956" s="2" t="inlineStr">
+      <c r="A956" s="5" t="inlineStr">
         <is>
           <t>SDFFQNX0P5</t>
         </is>
       </c>
-      <c r="B956" s="3" t="n"/>
-      <c r="C956" s="3" t="inlineStr">
+      <c r="B956" s="6" t="n"/>
+      <c r="C956" s="6" t="inlineStr">
         <is>
           <t>SDFFQNX0P5AHCCOTC</t>
         </is>
       </c>
     </row>
     <row r="957">
-      <c r="A957" s="2" t="n"/>
-      <c r="B957" s="3" t="n"/>
-      <c r="C957" s="3" t="inlineStr">
+      <c r="A957" s="7" t="n"/>
+      <c r="B957" s="8" t="n"/>
+      <c r="C957" s="8" t="inlineStr">
         <is>
           <t>SDFFQNX0P5AHQCOTC</t>
         </is>
       </c>
     </row>
     <row r="958">
-      <c r="A958" s="2" t="inlineStr">
+      <c r="A958" s="5" t="inlineStr">
         <is>
           <t>SDFFQNX4</t>
         </is>
       </c>
-      <c r="B958" s="3" t="n"/>
-      <c r="C958" s="3" t="inlineStr">
+      <c r="B958" s="6" t="n"/>
+      <c r="C958" s="6" t="inlineStr">
         <is>
           <t>SDFFQNX4AHBCOTC</t>
         </is>
       </c>
     </row>
     <row r="959">
-      <c r="A959" s="2" t="n"/>
-      <c r="B959" s="3" t="n"/>
-      <c r="C959" s="3" t="inlineStr">
+      <c r="A959" s="7" t="n"/>
+      <c r="B959" s="8" t="n"/>
+      <c r="C959" s="8" t="inlineStr">
         <is>
           <t>SDFFQNX4AHQCOTC</t>
         </is>
@@ -14519,26 +14549,26 @@
       </c>
     </row>
     <row r="1028">
-      <c r="A1028" s="2" t="inlineStr">
+      <c r="A1028" s="5" t="inlineStr">
         <is>
           <t>XNR2D8</t>
         </is>
       </c>
-      <c r="B1028" s="3" t="inlineStr">
+      <c r="B1028" s="6" t="inlineStr">
         <is>
           <t>XNR2D8COTMDB</t>
         </is>
       </c>
-      <c r="C1028" s="3" t="inlineStr">
+      <c r="C1028" s="6" t="inlineStr">
         <is>
           <t>XNR2D8COT3FIN</t>
         </is>
       </c>
     </row>
     <row r="1029">
-      <c r="A1029" s="2" t="n"/>
-      <c r="B1029" s="3" t="n"/>
-      <c r="C1029" s="3" t="inlineStr">
+      <c r="A1029" s="7" t="n"/>
+      <c r="B1029" s="8" t="n"/>
+      <c r="C1029" s="8" t="inlineStr">
         <is>
           <t>XNR2EEQMBDD8COT</t>
         </is>
@@ -14696,22 +14726,22 @@
       </c>
     </row>
     <row r="1041">
-      <c r="A1041" s="2" t="inlineStr">
+      <c r="A1041" s="5" t="inlineStr">
         <is>
           <t>XNR2X2</t>
         </is>
       </c>
-      <c r="B1041" s="3" t="n"/>
-      <c r="C1041" s="3" t="inlineStr">
+      <c r="B1041" s="6" t="n"/>
+      <c r="C1041" s="6" t="inlineStr">
         <is>
           <t>XNR2X2ATACOTC</t>
         </is>
       </c>
     </row>
     <row r="1042">
-      <c r="A1042" s="2" t="n"/>
-      <c r="B1042" s="3" t="n"/>
-      <c r="C1042" s="3" t="inlineStr">
+      <c r="A1042" s="7" t="n"/>
+      <c r="B1042" s="8" t="n"/>
+      <c r="C1042" s="8" t="inlineStr">
         <is>
           <t>XNR2X2ATBCOTC</t>
         </is>
@@ -15200,22 +15230,22 @@
       </c>
     </row>
     <row r="1077">
-      <c r="A1077" s="2" t="inlineStr">
+      <c r="A1077" s="5" t="inlineStr">
         <is>
           <t>XOR2X1</t>
         </is>
       </c>
-      <c r="B1077" s="3" t="n"/>
-      <c r="C1077" s="3" t="inlineStr">
+      <c r="B1077" s="6" t="n"/>
+      <c r="C1077" s="6" t="inlineStr">
         <is>
           <t>XOR2X1ATACOTC</t>
         </is>
       </c>
     </row>
     <row r="1078">
-      <c r="A1078" s="2" t="n"/>
-      <c r="B1078" s="3" t="n"/>
-      <c r="C1078" s="3" t="inlineStr">
+      <c r="A1078" s="7" t="n"/>
+      <c r="B1078" s="8" t="n"/>
+      <c r="C1078" s="8" t="inlineStr">
         <is>
           <t>XOR2X1ATCCOTC</t>
         </is>

</xml_diff>

<commit_message>
Excel 排版增强 + --format-replace 正则替换 (#5)
* Freeze the Excel header row while scrolling.

Set worksheet.freeze_panes to A2 so row 1 stays visible.

Co-authored-by: EsaLongs <EsaLongs@users.noreply.github.com>

* Add header and section borders spanning columns A-C.

Draw top/bottom borders on A1:C1 and on each display-key group
boundary so merged key blocks read as full-width sections.

Co-authored-by: EsaLongs <EsaLongs@users.noreply.github.com>

* Add --format-replace for post-delete regex substitutions.

Parse quote-delimited "pattern ：replacement" mappings (half-width :
also supported) and apply them after --format-filter deletes.

Co-authored-by: EsaLongs <EsaLongs@users.noreply.github.com>

---------

Co-authored-by: Cursor Agent <cursoragent@cursor.com>
Co-authored-by: EsaLongs <EsaLongs@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/preview/NP1PP_vs_C1Y_preview.xlsx
+++ b/preview/NP1PP_vs_C1Y_preview.xlsx
@@ -46,7 +46,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -54,18 +54,48 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+    </border>
+    <border>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+    </border>
+    <border>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -784,22 +814,22 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="inlineStr">
+      <c r="A25" s="5" t="inlineStr">
         <is>
           <t>AN2X8</t>
         </is>
       </c>
-      <c r="B25" s="3" t="n"/>
-      <c r="C25" s="3" t="inlineStr">
+      <c r="B25" s="6" t="n"/>
+      <c r="C25" s="6" t="inlineStr">
         <is>
           <t>AN2EEQMBDX8AR2COTC</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="n"/>
-      <c r="B26" s="3" t="n"/>
-      <c r="C26" s="3" t="inlineStr">
+      <c r="A26" s="7" t="n"/>
+      <c r="B26" s="8" t="n"/>
+      <c r="C26" s="8" t="inlineStr">
         <is>
           <t>AN2X8AR2COTC</t>
         </is>
@@ -1072,26 +1102,26 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="inlineStr">
+      <c r="A45" s="5" t="inlineStr">
         <is>
           <t>AO211D1</t>
         </is>
       </c>
-      <c r="B45" s="3" t="inlineStr">
+      <c r="B45" s="6" t="inlineStr">
         <is>
           <t>AO211D1COTMDB</t>
         </is>
       </c>
-      <c r="C45" s="3" t="inlineStr">
+      <c r="C45" s="6" t="inlineStr">
         <is>
           <t>AO211D1COT</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="n"/>
-      <c r="B46" s="3" t="n"/>
-      <c r="C46" s="3" t="inlineStr">
+      <c r="A46" s="7" t="n"/>
+      <c r="B46" s="8" t="n"/>
+      <c r="C46" s="8" t="inlineStr">
         <is>
           <t>AO211EEQMBDD1COT</t>
         </is>
@@ -1274,26 +1304,26 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="2" t="inlineStr">
+      <c r="A59" s="5" t="inlineStr">
         <is>
           <t>AO22D1</t>
         </is>
       </c>
-      <c r="B59" s="3" t="inlineStr">
+      <c r="B59" s="6" t="inlineStr">
         <is>
           <t>AO22D1COTMDB</t>
         </is>
       </c>
-      <c r="C59" s="3" t="inlineStr">
+      <c r="C59" s="6" t="inlineStr">
         <is>
           <t>AO22D1COT</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="2" t="n"/>
-      <c r="B60" s="3" t="n"/>
-      <c r="C60" s="3" t="inlineStr">
+      <c r="A60" s="7" t="n"/>
+      <c r="B60" s="8" t="n"/>
+      <c r="C60" s="8" t="inlineStr">
         <is>
           <t>AO22EEQMBDD1COT</t>
         </is>
@@ -1939,22 +1969,22 @@
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="2" t="inlineStr">
+      <c r="A104" s="5" t="inlineStr">
         <is>
           <t>AOI21X2</t>
         </is>
       </c>
-      <c r="B104" s="3" t="n"/>
-      <c r="C104" s="3" t="inlineStr">
+      <c r="B104" s="6" t="n"/>
+      <c r="C104" s="6" t="inlineStr">
         <is>
           <t>AOI21EEQMBDX2APBCOTC</t>
         </is>
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="2" t="n"/>
-      <c r="B105" s="3" t="n"/>
-      <c r="C105" s="3" t="inlineStr">
+      <c r="A105" s="7" t="n"/>
+      <c r="B105" s="8" t="n"/>
+      <c r="C105" s="8" t="inlineStr">
         <is>
           <t>AOI21X2APACOTC</t>
         </is>
@@ -1987,22 +2017,22 @@
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="2" t="inlineStr">
+      <c r="A108" s="5" t="inlineStr">
         <is>
           <t>AOI21X8</t>
         </is>
       </c>
-      <c r="B108" s="3" t="n"/>
-      <c r="C108" s="3" t="inlineStr">
+      <c r="B108" s="6" t="n"/>
+      <c r="C108" s="6" t="inlineStr">
         <is>
           <t>AOI21X8APACOTC</t>
         </is>
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="2" t="n"/>
-      <c r="B109" s="3" t="n"/>
-      <c r="C109" s="3" t="inlineStr">
+      <c r="A109" s="7" t="n"/>
+      <c r="B109" s="8" t="n"/>
+      <c r="C109" s="8" t="inlineStr">
         <is>
           <t>AOI21X8APBCOTC</t>
         </is>
@@ -2564,93 +2594,93 @@
       <c r="C148" s="3" t="n"/>
     </row>
     <row r="149">
-      <c r="A149" s="2" t="inlineStr">
+      <c r="A149" s="5" t="inlineStr">
         <is>
           <t>AOI22X1</t>
         </is>
       </c>
-      <c r="B149" s="3" t="n"/>
-      <c r="C149" s="3" t="inlineStr">
+      <c r="B149" s="6" t="n"/>
+      <c r="C149" s="6" t="inlineStr">
         <is>
           <t>AOI22X1APBCOTC</t>
         </is>
       </c>
     </row>
     <row r="150">
-      <c r="A150" s="2" t="n"/>
-      <c r="B150" s="3" t="n"/>
-      <c r="C150" s="3" t="inlineStr">
+      <c r="A150" s="9" t="n"/>
+      <c r="B150" s="10" t="n"/>
+      <c r="C150" s="10" t="inlineStr">
         <is>
           <t>AOI22X1APCCOTC</t>
         </is>
       </c>
     </row>
     <row r="151">
-      <c r="A151" s="2" t="n"/>
-      <c r="B151" s="3" t="n"/>
-      <c r="C151" s="3" t="inlineStr">
+      <c r="A151" s="9" t="n"/>
+      <c r="B151" s="10" t="n"/>
+      <c r="C151" s="10" t="inlineStr">
         <is>
           <t>AOI22X1APDCOTC</t>
         </is>
       </c>
     </row>
     <row r="152">
-      <c r="A152" s="2" t="n"/>
-      <c r="B152" s="3" t="n"/>
-      <c r="C152" s="3" t="inlineStr">
+      <c r="A152" s="9" t="n"/>
+      <c r="B152" s="10" t="n"/>
+      <c r="C152" s="10" t="inlineStr">
         <is>
           <t>AOI22X1APMCOTC</t>
         </is>
       </c>
     </row>
     <row r="153">
-      <c r="A153" s="2" t="n"/>
-      <c r="B153" s="3" t="n"/>
-      <c r="C153" s="3" t="inlineStr">
+      <c r="A153" s="7" t="n"/>
+      <c r="B153" s="8" t="n"/>
+      <c r="C153" s="8" t="inlineStr">
         <is>
           <t>AOI22X1APPCOTC</t>
         </is>
       </c>
     </row>
     <row r="154">
-      <c r="A154" s="2" t="inlineStr">
+      <c r="A154" s="5" t="inlineStr">
         <is>
           <t>AOI22X2</t>
         </is>
       </c>
-      <c r="B154" s="3" t="n"/>
-      <c r="C154" s="3" t="inlineStr">
+      <c r="B154" s="6" t="n"/>
+      <c r="C154" s="6" t="inlineStr">
         <is>
           <t>AOI22X2ANSCOTC</t>
         </is>
       </c>
     </row>
     <row r="155">
-      <c r="A155" s="2" t="n"/>
-      <c r="B155" s="3" t="n"/>
-      <c r="C155" s="3" t="inlineStr">
+      <c r="A155" s="7" t="n"/>
+      <c r="B155" s="8" t="n"/>
+      <c r="C155" s="8" t="inlineStr">
         <is>
           <t>AOI22X2APQCOTC</t>
         </is>
       </c>
     </row>
     <row r="156">
-      <c r="A156" s="2" t="inlineStr">
+      <c r="A156" s="5" t="inlineStr">
         <is>
           <t>AOI22X3</t>
         </is>
       </c>
-      <c r="B156" s="3" t="n"/>
-      <c r="C156" s="3" t="inlineStr">
+      <c r="B156" s="6" t="n"/>
+      <c r="C156" s="6" t="inlineStr">
         <is>
           <t>AOI22X3ANSCOTC</t>
         </is>
       </c>
     </row>
     <row r="157">
-      <c r="A157" s="2" t="n"/>
-      <c r="B157" s="3" t="n"/>
-      <c r="C157" s="3" t="inlineStr">
+      <c r="A157" s="7" t="n"/>
+      <c r="B157" s="8" t="n"/>
+      <c r="C157" s="8" t="inlineStr">
         <is>
           <t>AOI22X3APQCOT</t>
         </is>
@@ -3392,22 +3422,22 @@
       </c>
     </row>
     <row r="209">
-      <c r="A209" s="2" t="inlineStr">
+      <c r="A209" s="5" t="inlineStr">
         <is>
           <t>BUFX8</t>
         </is>
       </c>
-      <c r="B209" s="3" t="n"/>
-      <c r="C209" s="3" t="inlineStr">
+      <c r="B209" s="6" t="n"/>
+      <c r="C209" s="6" t="inlineStr">
         <is>
           <t>BUFX8AHACOT</t>
         </is>
       </c>
     </row>
     <row r="210">
-      <c r="A210" s="2" t="n"/>
-      <c r="B210" s="3" t="n"/>
-      <c r="C210" s="3" t="inlineStr">
+      <c r="A210" s="7" t="n"/>
+      <c r="B210" s="8" t="n"/>
+      <c r="C210" s="8" t="inlineStr">
         <is>
           <t>BUFX8AROCOT</t>
         </is>
@@ -3733,26 +3763,26 @@
       </c>
     </row>
     <row r="234">
-      <c r="A234" s="2" t="inlineStr">
+      <c r="A234" s="5" t="inlineStr">
         <is>
           <t>CKMUX2D8</t>
         </is>
       </c>
-      <c r="B234" s="3" t="inlineStr">
+      <c r="B234" s="6" t="inlineStr">
         <is>
           <t>CKMUX2D8COTM3CEQ</t>
         </is>
       </c>
-      <c r="C234" s="3" t="inlineStr">
+      <c r="C234" s="6" t="inlineStr">
         <is>
           <t>CKMUX2D8COT</t>
         </is>
       </c>
     </row>
     <row r="235">
-      <c r="A235" s="2" t="n"/>
-      <c r="B235" s="3" t="n"/>
-      <c r="C235" s="3" t="inlineStr">
+      <c r="A235" s="7" t="n"/>
+      <c r="B235" s="8" t="n"/>
+      <c r="C235" s="8" t="inlineStr">
         <is>
           <t>CKMUX2EEQMBDD8COT</t>
         </is>
@@ -4211,26 +4241,26 @@
       </c>
     </row>
     <row r="268">
-      <c r="A268" s="2" t="inlineStr">
+      <c r="A268" s="5" t="inlineStr">
         <is>
           <t>CMPE42D4</t>
         </is>
       </c>
-      <c r="B268" s="3" t="inlineStr">
+      <c r="B268" s="6" t="inlineStr">
         <is>
           <t>CMPE42D4COT</t>
         </is>
       </c>
-      <c r="C268" s="3" t="inlineStr">
+      <c r="C268" s="6" t="inlineStr">
         <is>
           <t>CMPE42D4OPTCOT</t>
         </is>
       </c>
     </row>
     <row r="269">
-      <c r="A269" s="2" t="n"/>
-      <c r="B269" s="3" t="n"/>
-      <c r="C269" s="3" t="inlineStr">
+      <c r="A269" s="7" t="n"/>
+      <c r="B269" s="8" t="n"/>
+      <c r="C269" s="8" t="inlineStr">
         <is>
           <t>CMPE42EEQMBDD4COT</t>
         </is>
@@ -4250,26 +4280,26 @@
       </c>
     </row>
     <row r="271">
-      <c r="A271" s="2" t="inlineStr">
+      <c r="A271" s="5" t="inlineStr">
         <is>
           <t>DC</t>
         </is>
       </c>
-      <c r="B271" s="3" t="inlineStr">
+      <c r="B271" s="6" t="inlineStr">
         <is>
           <t>DCAP4COT</t>
         </is>
       </c>
-      <c r="C271" s="3" t="n"/>
+      <c r="C271" s="6" t="n"/>
     </row>
     <row r="272">
-      <c r="A272" s="2" t="n"/>
-      <c r="B272" s="3" t="inlineStr">
+      <c r="A272" s="7" t="n"/>
+      <c r="B272" s="8" t="inlineStr">
         <is>
           <t>DCAP5COT</t>
         </is>
       </c>
-      <c r="C272" s="3" t="n"/>
+      <c r="C272" s="8" t="n"/>
     </row>
     <row r="273">
       <c r="A273" s="2" t="inlineStr">
@@ -6741,26 +6771,26 @@
       </c>
     </row>
     <row r="454">
-      <c r="A454" s="2" t="inlineStr">
+      <c r="A454" s="5" t="inlineStr">
         <is>
           <t>HDDID2</t>
         </is>
       </c>
-      <c r="B454" s="3" t="inlineStr">
+      <c r="B454" s="6" t="inlineStr">
         <is>
           <t>HDDID2A30COTARC</t>
         </is>
       </c>
-      <c r="C454" s="3" t="n"/>
+      <c r="C454" s="6" t="n"/>
     </row>
     <row r="455">
-      <c r="A455" s="2" t="n"/>
-      <c r="B455" s="3" t="inlineStr">
+      <c r="A455" s="7" t="n"/>
+      <c r="B455" s="8" t="inlineStr">
         <is>
           <t>HDDID2A40COTARC</t>
         </is>
       </c>
-      <c r="C455" s="3" t="n"/>
+      <c r="C455" s="8" t="n"/>
     </row>
     <row r="456">
       <c r="A456" s="2" t="inlineStr">
@@ -6776,26 +6806,26 @@
       <c r="C456" s="3" t="n"/>
     </row>
     <row r="457">
-      <c r="A457" s="2" t="inlineStr">
+      <c r="A457" s="5" t="inlineStr">
         <is>
           <t>IAO21D2</t>
         </is>
       </c>
-      <c r="B457" s="3" t="inlineStr">
+      <c r="B457" s="6" t="inlineStr">
         <is>
           <t>IAO21D2COT</t>
         </is>
       </c>
-      <c r="C457" s="3" t="inlineStr">
+      <c r="C457" s="6" t="inlineStr">
         <is>
           <t>IAO21D2COT3FIN</t>
         </is>
       </c>
     </row>
     <row r="458">
-      <c r="A458" s="2" t="n"/>
-      <c r="B458" s="3" t="n"/>
-      <c r="C458" s="3" t="inlineStr">
+      <c r="A458" s="7" t="n"/>
+      <c r="B458" s="8" t="n"/>
+      <c r="C458" s="8" t="inlineStr">
         <is>
           <t>IAO21EEQMBDD2COT</t>
         </is>
@@ -6879,26 +6909,26 @@
       </c>
     </row>
     <row r="464">
-      <c r="A464" s="2" t="inlineStr">
+      <c r="A464" s="5" t="inlineStr">
         <is>
           <t>IAOI21D1</t>
         </is>
       </c>
-      <c r="B464" s="3" t="inlineStr">
+      <c r="B464" s="6" t="inlineStr">
         <is>
           <t>IAOI21D1COTOPU</t>
         </is>
       </c>
-      <c r="C464" s="3" t="inlineStr">
+      <c r="C464" s="6" t="inlineStr">
         <is>
           <t>IAOI21D1COT</t>
         </is>
       </c>
     </row>
     <row r="465">
-      <c r="A465" s="2" t="n"/>
-      <c r="B465" s="3" t="n"/>
-      <c r="C465" s="3" t="inlineStr">
+      <c r="A465" s="7" t="n"/>
+      <c r="B465" s="8" t="n"/>
+      <c r="C465" s="8" t="inlineStr">
         <is>
           <t>IAOI21EEQMBDD1COT</t>
         </is>
@@ -9396,22 +9426,22 @@
       </c>
     </row>
     <row r="645">
-      <c r="A645" s="2" t="inlineStr">
+      <c r="A645" s="5" t="inlineStr">
         <is>
           <t>MX2X2</t>
         </is>
       </c>
-      <c r="B645" s="3" t="n"/>
-      <c r="C645" s="3" t="inlineStr">
+      <c r="B645" s="6" t="n"/>
+      <c r="C645" s="6" t="inlineStr">
         <is>
           <t>MX2X2ATACOTC</t>
         </is>
       </c>
     </row>
     <row r="646">
-      <c r="A646" s="2" t="n"/>
-      <c r="B646" s="3" t="n"/>
-      <c r="C646" s="3" t="inlineStr">
+      <c r="A646" s="7" t="n"/>
+      <c r="B646" s="8" t="n"/>
+      <c r="C646" s="8" t="inlineStr">
         <is>
           <t>MX2X2ATFCOTC</t>
         </is>
@@ -9431,53 +9461,53 @@
       </c>
     </row>
     <row r="648">
-      <c r="A648" s="2" t="inlineStr">
+      <c r="A648" s="5" t="inlineStr">
         <is>
           <t>MXI2X1</t>
         </is>
       </c>
-      <c r="B648" s="3" t="n"/>
-      <c r="C648" s="3" t="inlineStr">
+      <c r="B648" s="6" t="n"/>
+      <c r="C648" s="6" t="inlineStr">
         <is>
           <t>MXI2X1ATACOTC</t>
         </is>
       </c>
     </row>
     <row r="649">
-      <c r="A649" s="2" t="n"/>
-      <c r="B649" s="3" t="n"/>
-      <c r="C649" s="3" t="inlineStr">
+      <c r="A649" s="7" t="n"/>
+      <c r="B649" s="8" t="n"/>
+      <c r="C649" s="8" t="inlineStr">
         <is>
           <t>MXI2X1ATBCOTC</t>
         </is>
       </c>
     </row>
     <row r="650">
-      <c r="A650" s="2" t="inlineStr">
+      <c r="A650" s="5" t="inlineStr">
         <is>
           <t>MXI2X2</t>
         </is>
       </c>
-      <c r="B650" s="3" t="n"/>
-      <c r="C650" s="3" t="inlineStr">
+      <c r="B650" s="6" t="n"/>
+      <c r="C650" s="6" t="inlineStr">
         <is>
           <t>MXI2X2ATACOTC</t>
         </is>
       </c>
     </row>
     <row r="651">
-      <c r="A651" s="2" t="n"/>
-      <c r="B651" s="3" t="n"/>
-      <c r="C651" s="3" t="inlineStr">
+      <c r="A651" s="9" t="n"/>
+      <c r="B651" s="10" t="n"/>
+      <c r="C651" s="10" t="inlineStr">
         <is>
           <t>MXI2X2ATBCOTC</t>
         </is>
       </c>
     </row>
     <row r="652">
-      <c r="A652" s="2" t="n"/>
-      <c r="B652" s="3" t="n"/>
-      <c r="C652" s="3" t="inlineStr">
+      <c r="A652" s="7" t="n"/>
+      <c r="B652" s="8" t="n"/>
+      <c r="C652" s="8" t="inlineStr">
         <is>
           <t>MXI2X2ATSCOTC</t>
         </is>
@@ -9497,31 +9527,31 @@
       </c>
     </row>
     <row r="654">
-      <c r="A654" s="2" t="inlineStr">
+      <c r="A654" s="5" t="inlineStr">
         <is>
           <t>MXI2X4</t>
         </is>
       </c>
-      <c r="B654" s="3" t="n"/>
-      <c r="C654" s="3" t="inlineStr">
+      <c r="B654" s="6" t="n"/>
+      <c r="C654" s="6" t="inlineStr">
         <is>
           <t>MXI2X4ATACOTC</t>
         </is>
       </c>
     </row>
     <row r="655">
-      <c r="A655" s="2" t="n"/>
-      <c r="B655" s="3" t="n"/>
-      <c r="C655" s="3" t="inlineStr">
+      <c r="A655" s="9" t="n"/>
+      <c r="B655" s="10" t="n"/>
+      <c r="C655" s="10" t="inlineStr">
         <is>
           <t>MXI2X4ATBCOTC</t>
         </is>
       </c>
     </row>
     <row r="656">
-      <c r="A656" s="2" t="n"/>
-      <c r="B656" s="3" t="n"/>
-      <c r="C656" s="3" t="inlineStr">
+      <c r="A656" s="7" t="n"/>
+      <c r="B656" s="8" t="n"/>
+      <c r="C656" s="8" t="inlineStr">
         <is>
           <t>MXI2X4ATSCOTC</t>
         </is>
@@ -9541,22 +9571,22 @@
       </c>
     </row>
     <row r="658">
-      <c r="A658" s="2" t="inlineStr">
+      <c r="A658" s="5" t="inlineStr">
         <is>
           <t>MXI2X8</t>
         </is>
       </c>
-      <c r="B658" s="3" t="n"/>
-      <c r="C658" s="3" t="inlineStr">
+      <c r="B658" s="6" t="n"/>
+      <c r="C658" s="6" t="inlineStr">
         <is>
           <t>MXI2X8ATACOTC</t>
         </is>
       </c>
     </row>
     <row r="659">
-      <c r="A659" s="2" t="n"/>
-      <c r="B659" s="3" t="n"/>
-      <c r="C659" s="3" t="inlineStr">
+      <c r="A659" s="7" t="n"/>
+      <c r="B659" s="8" t="n"/>
+      <c r="C659" s="8" t="inlineStr">
         <is>
           <t>MXI2X8ATSCOTC</t>
         </is>
@@ -9843,53 +9873,53 @@
       <c r="C679" s="3" t="n"/>
     </row>
     <row r="680">
-      <c r="A680" s="2" t="inlineStr">
+      <c r="A680" s="5" t="inlineStr">
         <is>
           <t>ND2X1</t>
         </is>
       </c>
-      <c r="B680" s="3" t="n"/>
-      <c r="C680" s="3" t="inlineStr">
+      <c r="B680" s="6" t="n"/>
+      <c r="C680" s="6" t="inlineStr">
         <is>
           <t>ND2X1AKPCOTC</t>
         </is>
       </c>
     </row>
     <row r="681">
-      <c r="A681" s="2" t="n"/>
-      <c r="B681" s="3" t="n"/>
-      <c r="C681" s="3" t="inlineStr">
+      <c r="A681" s="7" t="n"/>
+      <c r="B681" s="8" t="n"/>
+      <c r="C681" s="8" t="inlineStr">
         <is>
           <t>ND2X1APNCOTC</t>
         </is>
       </c>
     </row>
     <row r="682">
-      <c r="A682" s="2" t="inlineStr">
+      <c r="A682" s="5" t="inlineStr">
         <is>
           <t>ND2X10</t>
         </is>
       </c>
-      <c r="B682" s="3" t="n"/>
-      <c r="C682" s="3" t="inlineStr">
+      <c r="B682" s="6" t="n"/>
+      <c r="C682" s="6" t="inlineStr">
         <is>
           <t>ND2X10AKPCOTC</t>
         </is>
       </c>
     </row>
     <row r="683">
-      <c r="A683" s="2" t="n"/>
-      <c r="B683" s="3" t="n"/>
-      <c r="C683" s="3" t="inlineStr">
+      <c r="A683" s="9" t="n"/>
+      <c r="B683" s="10" t="n"/>
+      <c r="C683" s="10" t="inlineStr">
         <is>
           <t>ND2X10APBCOTC</t>
         </is>
       </c>
     </row>
     <row r="684">
-      <c r="A684" s="2" t="n"/>
-      <c r="B684" s="3" t="n"/>
-      <c r="C684" s="3" t="inlineStr">
+      <c r="A684" s="7" t="n"/>
+      <c r="B684" s="8" t="n"/>
+      <c r="C684" s="8" t="inlineStr">
         <is>
           <t>ND2X10APNCOTC</t>
         </is>
@@ -9935,31 +9965,31 @@
       </c>
     </row>
     <row r="688">
-      <c r="A688" s="2" t="inlineStr">
+      <c r="A688" s="5" t="inlineStr">
         <is>
           <t>ND2X2</t>
         </is>
       </c>
-      <c r="B688" s="3" t="n"/>
-      <c r="C688" s="3" t="inlineStr">
+      <c r="B688" s="6" t="n"/>
+      <c r="C688" s="6" t="inlineStr">
         <is>
           <t>ND2X2AKPCOTC</t>
         </is>
       </c>
     </row>
     <row r="689">
-      <c r="A689" s="2" t="n"/>
-      <c r="B689" s="3" t="n"/>
-      <c r="C689" s="3" t="inlineStr">
+      <c r="A689" s="9" t="n"/>
+      <c r="B689" s="10" t="n"/>
+      <c r="C689" s="10" t="inlineStr">
         <is>
           <t>ND2X2APBCOTC</t>
         </is>
       </c>
     </row>
     <row r="690">
-      <c r="A690" s="2" t="n"/>
-      <c r="B690" s="3" t="n"/>
-      <c r="C690" s="3" t="inlineStr">
+      <c r="A690" s="7" t="n"/>
+      <c r="B690" s="8" t="n"/>
+      <c r="C690" s="8" t="inlineStr">
         <is>
           <t>ND2X2APNCOTC</t>
         </is>
@@ -9979,71 +10009,71 @@
       </c>
     </row>
     <row r="692">
-      <c r="A692" s="2" t="inlineStr">
+      <c r="A692" s="5" t="inlineStr">
         <is>
           <t>ND2X4</t>
         </is>
       </c>
-      <c r="B692" s="3" t="n"/>
-      <c r="C692" s="3" t="inlineStr">
+      <c r="B692" s="6" t="n"/>
+      <c r="C692" s="6" t="inlineStr">
         <is>
           <t>ND2X4APACOT3FINC</t>
         </is>
       </c>
     </row>
     <row r="693">
-      <c r="A693" s="2" t="n"/>
-      <c r="B693" s="3" t="n"/>
-      <c r="C693" s="3" t="inlineStr">
+      <c r="A693" s="9" t="n"/>
+      <c r="B693" s="10" t="n"/>
+      <c r="C693" s="10" t="inlineStr">
         <is>
           <t>ND2X4APBCOTC</t>
         </is>
       </c>
     </row>
     <row r="694">
-      <c r="A694" s="2" t="n"/>
-      <c r="B694" s="3" t="n"/>
-      <c r="C694" s="3" t="inlineStr">
+      <c r="A694" s="9" t="n"/>
+      <c r="B694" s="10" t="n"/>
+      <c r="C694" s="10" t="inlineStr">
         <is>
           <t>ND2X4APNCOTC</t>
         </is>
       </c>
     </row>
     <row r="695">
-      <c r="A695" s="2" t="n"/>
-      <c r="B695" s="3" t="n"/>
-      <c r="C695" s="3" t="inlineStr">
+      <c r="A695" s="7" t="n"/>
+      <c r="B695" s="8" t="n"/>
+      <c r="C695" s="8" t="inlineStr">
         <is>
           <t>ND2X4ARQCOT</t>
         </is>
       </c>
     </row>
     <row r="696">
-      <c r="A696" s="2" t="inlineStr">
+      <c r="A696" s="5" t="inlineStr">
         <is>
           <t>ND2X6</t>
         </is>
       </c>
-      <c r="B696" s="3" t="n"/>
-      <c r="C696" s="3" t="inlineStr">
+      <c r="B696" s="6" t="n"/>
+      <c r="C696" s="6" t="inlineStr">
         <is>
           <t>ND2X6AKPCOTC</t>
         </is>
       </c>
     </row>
     <row r="697">
-      <c r="A697" s="2" t="n"/>
-      <c r="B697" s="3" t="n"/>
-      <c r="C697" s="3" t="inlineStr">
+      <c r="A697" s="9" t="n"/>
+      <c r="B697" s="10" t="n"/>
+      <c r="C697" s="10" t="inlineStr">
         <is>
           <t>ND2X6APNCOTC</t>
         </is>
       </c>
     </row>
     <row r="698">
-      <c r="A698" s="2" t="n"/>
-      <c r="B698" s="3" t="n"/>
-      <c r="C698" s="3" t="inlineStr">
+      <c r="A698" s="7" t="n"/>
+      <c r="B698" s="8" t="n"/>
+      <c r="C698" s="8" t="inlineStr">
         <is>
           <t>ND2X6AROCOT</t>
         </is>
@@ -10063,31 +10093,31 @@
       </c>
     </row>
     <row r="700">
-      <c r="A700" s="2" t="inlineStr">
+      <c r="A700" s="5" t="inlineStr">
         <is>
           <t>ND2X8</t>
         </is>
       </c>
-      <c r="B700" s="3" t="n"/>
-      <c r="C700" s="3" t="inlineStr">
+      <c r="B700" s="6" t="n"/>
+      <c r="C700" s="6" t="inlineStr">
         <is>
           <t>ND2X8APACOT3FINC</t>
         </is>
       </c>
     </row>
     <row r="701">
-      <c r="A701" s="2" t="n"/>
-      <c r="B701" s="3" t="n"/>
-      <c r="C701" s="3" t="inlineStr">
+      <c r="A701" s="9" t="n"/>
+      <c r="B701" s="10" t="n"/>
+      <c r="C701" s="10" t="inlineStr">
         <is>
           <t>ND2X8APBCOTC</t>
         </is>
       </c>
     </row>
     <row r="702">
-      <c r="A702" s="2" t="n"/>
-      <c r="B702" s="3" t="n"/>
-      <c r="C702" s="3" t="inlineStr">
+      <c r="A702" s="7" t="n"/>
+      <c r="B702" s="8" t="n"/>
+      <c r="C702" s="8" t="inlineStr">
         <is>
           <t>ND2X8APNCOTC</t>
         </is>
@@ -10456,22 +10486,22 @@
       </c>
     </row>
     <row r="729">
-      <c r="A729" s="2" t="inlineStr">
+      <c r="A729" s="5" t="inlineStr">
         <is>
           <t>NR2N1X12</t>
         </is>
       </c>
-      <c r="B729" s="3" t="n"/>
-      <c r="C729" s="3" t="inlineStr">
+      <c r="B729" s="6" t="n"/>
+      <c r="C729" s="6" t="inlineStr">
         <is>
           <t>NR2N1X12APPCOTC</t>
         </is>
       </c>
     </row>
     <row r="730">
-      <c r="A730" s="2" t="n"/>
-      <c r="B730" s="3" t="n"/>
-      <c r="C730" s="3" t="inlineStr">
+      <c r="A730" s="7" t="n"/>
+      <c r="B730" s="8" t="n"/>
+      <c r="C730" s="8" t="inlineStr">
         <is>
           <t>NR2N1X12AROCOT</t>
         </is>
@@ -10621,159 +10651,159 @@
       </c>
     </row>
     <row r="742">
-      <c r="A742" s="2" t="inlineStr">
+      <c r="A742" s="5" t="inlineStr">
         <is>
           <t>NR2X1</t>
         </is>
       </c>
-      <c r="B742" s="3" t="n"/>
-      <c r="C742" s="3" t="inlineStr">
+      <c r="B742" s="6" t="n"/>
+      <c r="C742" s="6" t="inlineStr">
         <is>
           <t>NR2X1AKNCOTC</t>
         </is>
       </c>
     </row>
     <row r="743">
-      <c r="A743" s="2" t="n"/>
-      <c r="B743" s="3" t="n"/>
-      <c r="C743" s="3" t="inlineStr">
+      <c r="A743" s="9" t="n"/>
+      <c r="B743" s="10" t="n"/>
+      <c r="C743" s="10" t="inlineStr">
         <is>
           <t>NR2X1APACOTC</t>
         </is>
       </c>
     </row>
     <row r="744">
-      <c r="A744" s="2" t="n"/>
-      <c r="B744" s="3" t="n"/>
-      <c r="C744" s="3" t="inlineStr">
+      <c r="A744" s="7" t="n"/>
+      <c r="B744" s="8" t="n"/>
+      <c r="C744" s="8" t="inlineStr">
         <is>
           <t>NR2X1APPCOTC</t>
         </is>
       </c>
     </row>
     <row r="745">
-      <c r="A745" s="2" t="inlineStr">
+      <c r="A745" s="5" t="inlineStr">
         <is>
           <t>NR2X10</t>
         </is>
       </c>
-      <c r="B745" s="3" t="n"/>
-      <c r="C745" s="3" t="inlineStr">
+      <c r="B745" s="6" t="n"/>
+      <c r="C745" s="6" t="inlineStr">
         <is>
           <t>NR2X10APBCOTC</t>
         </is>
       </c>
     </row>
     <row r="746">
-      <c r="A746" s="2" t="n"/>
-      <c r="B746" s="3" t="n"/>
-      <c r="C746" s="3" t="inlineStr">
+      <c r="A746" s="7" t="n"/>
+      <c r="B746" s="8" t="n"/>
+      <c r="C746" s="8" t="inlineStr">
         <is>
           <t>NR2X10APPCOTC</t>
         </is>
       </c>
     </row>
     <row r="747">
-      <c r="A747" s="2" t="inlineStr">
+      <c r="A747" s="5" t="inlineStr">
         <is>
           <t>NR2X12</t>
         </is>
       </c>
-      <c r="B747" s="3" t="n"/>
-      <c r="C747" s="3" t="inlineStr">
+      <c r="B747" s="6" t="n"/>
+      <c r="C747" s="6" t="inlineStr">
         <is>
           <t>NR2X12AKNCOTC</t>
         </is>
       </c>
     </row>
     <row r="748">
-      <c r="A748" s="2" t="n"/>
-      <c r="B748" s="3" t="n"/>
-      <c r="C748" s="3" t="inlineStr">
+      <c r="A748" s="9" t="n"/>
+      <c r="B748" s="10" t="n"/>
+      <c r="C748" s="10" t="inlineStr">
         <is>
           <t>NR2X12APACOTC</t>
         </is>
       </c>
     </row>
     <row r="749">
-      <c r="A749" s="2" t="n"/>
-      <c r="B749" s="3" t="n"/>
-      <c r="C749" s="3" t="inlineStr">
+      <c r="A749" s="7" t="n"/>
+      <c r="B749" s="8" t="n"/>
+      <c r="C749" s="8" t="inlineStr">
         <is>
           <t>NR2X12APPCOTC</t>
         </is>
       </c>
     </row>
     <row r="750">
-      <c r="A750" s="2" t="inlineStr">
+      <c r="A750" s="5" t="inlineStr">
         <is>
           <t>NR2X14</t>
         </is>
       </c>
-      <c r="B750" s="3" t="n"/>
-      <c r="C750" s="3" t="inlineStr">
+      <c r="B750" s="6" t="n"/>
+      <c r="C750" s="6" t="inlineStr">
         <is>
           <t>NR2X14APBCOTC</t>
         </is>
       </c>
     </row>
     <row r="751">
-      <c r="A751" s="2" t="n"/>
-      <c r="B751" s="3" t="n"/>
-      <c r="C751" s="3" t="inlineStr">
+      <c r="A751" s="7" t="n"/>
+      <c r="B751" s="8" t="n"/>
+      <c r="C751" s="8" t="inlineStr">
         <is>
           <t>NR2X14APPCOTC</t>
         </is>
       </c>
     </row>
     <row r="752">
-      <c r="A752" s="2" t="inlineStr">
+      <c r="A752" s="5" t="inlineStr">
         <is>
           <t>NR2X16</t>
         </is>
       </c>
-      <c r="B752" s="3" t="n"/>
-      <c r="C752" s="3" t="inlineStr">
+      <c r="B752" s="6" t="n"/>
+      <c r="C752" s="6" t="inlineStr">
         <is>
           <t>NR2X16APACOTC</t>
         </is>
       </c>
     </row>
     <row r="753">
-      <c r="A753" s="2" t="n"/>
-      <c r="B753" s="3" t="n"/>
-      <c r="C753" s="3" t="inlineStr">
+      <c r="A753" s="9" t="n"/>
+      <c r="B753" s="10" t="n"/>
+      <c r="C753" s="10" t="inlineStr">
         <is>
           <t>NR2X16APBCOTC</t>
         </is>
       </c>
     </row>
     <row r="754">
-      <c r="A754" s="2" t="n"/>
-      <c r="B754" s="3" t="n"/>
-      <c r="C754" s="3" t="inlineStr">
+      <c r="A754" s="7" t="n"/>
+      <c r="B754" s="8" t="n"/>
+      <c r="C754" s="8" t="inlineStr">
         <is>
           <t>NR2X16APPCOTC</t>
         </is>
       </c>
     </row>
     <row r="755">
-      <c r="A755" s="2" t="inlineStr">
+      <c r="A755" s="5" t="inlineStr">
         <is>
           <t>NR2X2</t>
         </is>
       </c>
-      <c r="B755" s="3" t="n"/>
-      <c r="C755" s="3" t="inlineStr">
+      <c r="B755" s="6" t="n"/>
+      <c r="C755" s="6" t="inlineStr">
         <is>
           <t>NR2X2AKNCOT3FINC</t>
         </is>
       </c>
     </row>
     <row r="756">
-      <c r="A756" s="2" t="n"/>
-      <c r="B756" s="3" t="n"/>
-      <c r="C756" s="3" t="inlineStr">
+      <c r="A756" s="7" t="n"/>
+      <c r="B756" s="8" t="n"/>
+      <c r="C756" s="8" t="inlineStr">
         <is>
           <t>NR2X2APPCOT3FINC</t>
         </is>
@@ -10793,111 +10823,111 @@
       </c>
     </row>
     <row r="758">
-      <c r="A758" s="2" t="inlineStr">
+      <c r="A758" s="5" t="inlineStr">
         <is>
           <t>NR2X4</t>
         </is>
       </c>
-      <c r="B758" s="3" t="n"/>
-      <c r="C758" s="3" t="inlineStr">
+      <c r="B758" s="6" t="n"/>
+      <c r="C758" s="6" t="inlineStr">
         <is>
           <t>NR2X4AKNCOTC</t>
         </is>
       </c>
     </row>
     <row r="759">
-      <c r="A759" s="2" t="n"/>
-      <c r="B759" s="3" t="n"/>
-      <c r="C759" s="3" t="inlineStr">
+      <c r="A759" s="9" t="n"/>
+      <c r="B759" s="10" t="n"/>
+      <c r="C759" s="10" t="inlineStr">
         <is>
           <t>NR2X4APACOTC</t>
         </is>
       </c>
     </row>
     <row r="760">
-      <c r="A760" s="2" t="n"/>
-      <c r="B760" s="3" t="n"/>
-      <c r="C760" s="3" t="inlineStr">
+      <c r="A760" s="9" t="n"/>
+      <c r="B760" s="10" t="n"/>
+      <c r="C760" s="10" t="inlineStr">
         <is>
           <t>NR2X4APBCOTC</t>
         </is>
       </c>
     </row>
     <row r="761">
-      <c r="A761" s="2" t="n"/>
-      <c r="B761" s="3" t="n"/>
-      <c r="C761" s="3" t="inlineStr">
+      <c r="A761" s="7" t="n"/>
+      <c r="B761" s="8" t="n"/>
+      <c r="C761" s="8" t="inlineStr">
         <is>
           <t>NR2X4ARQCOT</t>
         </is>
       </c>
     </row>
     <row r="762">
-      <c r="A762" s="2" t="inlineStr">
+      <c r="A762" s="5" t="inlineStr">
         <is>
           <t>NR2X6</t>
         </is>
       </c>
-      <c r="B762" s="3" t="n"/>
-      <c r="C762" s="3" t="inlineStr">
+      <c r="B762" s="6" t="n"/>
+      <c r="C762" s="6" t="inlineStr">
         <is>
           <t>NR2X6APACOTC</t>
         </is>
       </c>
     </row>
     <row r="763">
-      <c r="A763" s="2" t="n"/>
-      <c r="B763" s="3" t="n"/>
-      <c r="C763" s="3" t="inlineStr">
+      <c r="A763" s="9" t="n"/>
+      <c r="B763" s="10" t="n"/>
+      <c r="C763" s="10" t="inlineStr">
         <is>
           <t>NR2X6APBCOTC</t>
         </is>
       </c>
     </row>
     <row r="764">
-      <c r="A764" s="2" t="n"/>
-      <c r="B764" s="3" t="n"/>
-      <c r="C764" s="3" t="inlineStr">
+      <c r="A764" s="7" t="n"/>
+      <c r="B764" s="8" t="n"/>
+      <c r="C764" s="8" t="inlineStr">
         <is>
           <t>NR2X6ARQCOT</t>
         </is>
       </c>
     </row>
     <row r="765">
-      <c r="A765" s="2" t="inlineStr">
+      <c r="A765" s="5" t="inlineStr">
         <is>
           <t>NR2X8</t>
         </is>
       </c>
-      <c r="B765" s="3" t="n"/>
-      <c r="C765" s="3" t="inlineStr">
+      <c r="B765" s="6" t="n"/>
+      <c r="C765" s="6" t="inlineStr">
         <is>
           <t>NR2X8APACOTC</t>
         </is>
       </c>
     </row>
     <row r="766">
-      <c r="A766" s="2" t="n"/>
-      <c r="B766" s="3" t="n"/>
-      <c r="C766" s="3" t="inlineStr">
+      <c r="A766" s="9" t="n"/>
+      <c r="B766" s="10" t="n"/>
+      <c r="C766" s="10" t="inlineStr">
         <is>
           <t>NR2X8APBCOTC</t>
         </is>
       </c>
     </row>
     <row r="767">
-      <c r="A767" s="2" t="n"/>
-      <c r="B767" s="3" t="n"/>
-      <c r="C767" s="3" t="inlineStr">
+      <c r="A767" s="9" t="n"/>
+      <c r="B767" s="10" t="n"/>
+      <c r="C767" s="10" t="inlineStr">
         <is>
           <t>NR2X8APPCOTC</t>
         </is>
       </c>
     </row>
     <row r="768">
-      <c r="A768" s="2" t="n"/>
-      <c r="B768" s="3" t="n"/>
-      <c r="C768" s="3" t="inlineStr">
+      <c r="A768" s="7" t="n"/>
+      <c r="B768" s="8" t="n"/>
+      <c r="C768" s="8" t="inlineStr">
         <is>
           <t>NR2X8AROCOT</t>
         </is>
@@ -11157,26 +11187,26 @@
       </c>
     </row>
     <row r="786">
-      <c r="A786" s="2" t="inlineStr">
+      <c r="A786" s="5" t="inlineStr">
         <is>
           <t>OA211D1</t>
         </is>
       </c>
-      <c r="B786" s="3" t="inlineStr">
+      <c r="B786" s="6" t="inlineStr">
         <is>
           <t>OA211D1COTMVM2OPU</t>
         </is>
       </c>
-      <c r="C786" s="3" t="inlineStr">
+      <c r="C786" s="6" t="inlineStr">
         <is>
           <t>OA211D1COT</t>
         </is>
       </c>
     </row>
     <row r="787">
-      <c r="A787" s="2" t="n"/>
-      <c r="B787" s="3" t="n"/>
-      <c r="C787" s="3" t="inlineStr">
+      <c r="A787" s="7" t="n"/>
+      <c r="B787" s="8" t="n"/>
+      <c r="C787" s="8" t="inlineStr">
         <is>
           <t>OA211EEQMBDD1COT</t>
         </is>
@@ -11304,26 +11334,26 @@
       <c r="C796" s="3" t="n"/>
     </row>
     <row r="797">
-      <c r="A797" s="2" t="inlineStr">
+      <c r="A797" s="5" t="inlineStr">
         <is>
           <t>OA222D1</t>
         </is>
       </c>
-      <c r="B797" s="3" t="inlineStr">
+      <c r="B797" s="6" t="inlineStr">
         <is>
           <t>OA222D1COTVIA</t>
         </is>
       </c>
-      <c r="C797" s="3" t="inlineStr">
+      <c r="C797" s="6" t="inlineStr">
         <is>
           <t>OA222D1COTA</t>
         </is>
       </c>
     </row>
     <row r="798">
-      <c r="A798" s="2" t="n"/>
-      <c r="B798" s="3" t="n"/>
-      <c r="C798" s="3" t="inlineStr">
+      <c r="A798" s="7" t="n"/>
+      <c r="B798" s="8" t="n"/>
+      <c r="C798" s="8" t="inlineStr">
         <is>
           <t>OA222EEQMBDD1COTA</t>
         </is>
@@ -11661,26 +11691,26 @@
       </c>
     </row>
     <row r="822">
-      <c r="A822" s="2" t="inlineStr">
+      <c r="A822" s="5" t="inlineStr">
         <is>
           <t>OAI21D1</t>
         </is>
       </c>
-      <c r="B822" s="3" t="inlineStr">
+      <c r="B822" s="6" t="inlineStr">
         <is>
           <t>OAI21D1COTOPTPA</t>
         </is>
       </c>
-      <c r="C822" s="3" t="inlineStr">
+      <c r="C822" s="6" t="inlineStr">
         <is>
           <t>OAI21D1COT</t>
         </is>
       </c>
     </row>
     <row r="823">
-      <c r="A823" s="2" t="n"/>
-      <c r="B823" s="3" t="n"/>
-      <c r="C823" s="3" t="inlineStr">
+      <c r="A823" s="7" t="n"/>
+      <c r="B823" s="8" t="n"/>
+      <c r="C823" s="8" t="inlineStr">
         <is>
           <t>OAI21EEQMBCD1COT</t>
         </is>
@@ -11799,22 +11829,22 @@
       </c>
     </row>
     <row r="832">
-      <c r="A832" s="2" t="inlineStr">
+      <c r="A832" s="5" t="inlineStr">
         <is>
           <t>OAI21N2X8</t>
         </is>
       </c>
-      <c r="B832" s="3" t="n"/>
-      <c r="C832" s="3" t="inlineStr">
+      <c r="B832" s="6" t="n"/>
+      <c r="C832" s="6" t="inlineStr">
         <is>
           <t>OAI21N2X8APACOTC</t>
         </is>
       </c>
     </row>
     <row r="833">
-      <c r="A833" s="2" t="n"/>
-      <c r="B833" s="3" t="n"/>
-      <c r="C833" s="3" t="inlineStr">
+      <c r="A833" s="7" t="n"/>
+      <c r="B833" s="8" t="n"/>
+      <c r="C833" s="8" t="inlineStr">
         <is>
           <t>OAI21N2X8COTC</t>
         </is>
@@ -12170,26 +12200,26 @@
       </c>
     </row>
     <row r="859">
-      <c r="A859" s="2" t="inlineStr">
+      <c r="A859" s="5" t="inlineStr">
         <is>
           <t>OAI2222D1</t>
         </is>
       </c>
-      <c r="B859" s="3" t="inlineStr">
+      <c r="B859" s="6" t="inlineStr">
         <is>
           <t>OAI2222D1COTOPTPA</t>
         </is>
       </c>
-      <c r="C859" s="3" t="inlineStr">
+      <c r="C859" s="6" t="inlineStr">
         <is>
           <t>OAI2222D1COTA</t>
         </is>
       </c>
     </row>
     <row r="860">
-      <c r="A860" s="2" t="n"/>
-      <c r="B860" s="3" t="n"/>
-      <c r="C860" s="3" t="inlineStr">
+      <c r="A860" s="7" t="n"/>
+      <c r="B860" s="8" t="n"/>
+      <c r="C860" s="8" t="inlineStr">
         <is>
           <t>OAI2222EEQMBDD1COTA</t>
         </is>
@@ -13145,22 +13175,22 @@
       </c>
     </row>
     <row r="926">
-      <c r="A926" s="2" t="inlineStr">
+      <c r="A926" s="5" t="inlineStr">
         <is>
           <t>OR2X4</t>
         </is>
       </c>
-      <c r="B926" s="3" t="n"/>
-      <c r="C926" s="3" t="inlineStr">
+      <c r="B926" s="6" t="n"/>
+      <c r="C926" s="6" t="inlineStr">
         <is>
           <t>OR2EEQMBDX4ARNCOTC</t>
         </is>
       </c>
     </row>
     <row r="927">
-      <c r="A927" s="2" t="n"/>
-      <c r="B927" s="3" t="n"/>
-      <c r="C927" s="3" t="inlineStr">
+      <c r="A927" s="7" t="n"/>
+      <c r="B927" s="8" t="n"/>
+      <c r="C927" s="8" t="inlineStr">
         <is>
           <t>OR2X4ARNCOTC</t>
         </is>
@@ -13193,31 +13223,31 @@
       </c>
     </row>
     <row r="930">
-      <c r="A930" s="2" t="inlineStr">
+      <c r="A930" s="5" t="inlineStr">
         <is>
           <t>OR2X8</t>
         </is>
       </c>
-      <c r="B930" s="3" t="n"/>
-      <c r="C930" s="3" t="inlineStr">
+      <c r="B930" s="6" t="n"/>
+      <c r="C930" s="6" t="inlineStr">
         <is>
           <t>OR2EEQMBDX8AR2COTC</t>
         </is>
       </c>
     </row>
     <row r="931">
-      <c r="A931" s="2" t="n"/>
-      <c r="B931" s="3" t="n"/>
-      <c r="C931" s="3" t="inlineStr">
+      <c r="A931" s="9" t="n"/>
+      <c r="B931" s="10" t="n"/>
+      <c r="C931" s="10" t="inlineStr">
         <is>
           <t>OR2X8AR2COT3FINC</t>
         </is>
       </c>
     </row>
     <row r="932">
-      <c r="A932" s="2" t="n"/>
-      <c r="B932" s="3" t="n"/>
-      <c r="C932" s="3" t="inlineStr">
+      <c r="A932" s="7" t="n"/>
+      <c r="B932" s="8" t="n"/>
+      <c r="C932" s="8" t="inlineStr">
         <is>
           <t>OR2X8ARNCOTC</t>
         </is>
@@ -13555,44 +13585,44 @@
       </c>
     </row>
     <row r="956">
-      <c r="A956" s="2" t="inlineStr">
+      <c r="A956" s="5" t="inlineStr">
         <is>
           <t>SDFFQNX0P5</t>
         </is>
       </c>
-      <c r="B956" s="3" t="n"/>
-      <c r="C956" s="3" t="inlineStr">
+      <c r="B956" s="6" t="n"/>
+      <c r="C956" s="6" t="inlineStr">
         <is>
           <t>SDFFQNX0P5AHCCOTC</t>
         </is>
       </c>
     </row>
     <row r="957">
-      <c r="A957" s="2" t="n"/>
-      <c r="B957" s="3" t="n"/>
-      <c r="C957" s="3" t="inlineStr">
+      <c r="A957" s="7" t="n"/>
+      <c r="B957" s="8" t="n"/>
+      <c r="C957" s="8" t="inlineStr">
         <is>
           <t>SDFFQNX0P5AHQCOTC</t>
         </is>
       </c>
     </row>
     <row r="958">
-      <c r="A958" s="2" t="inlineStr">
+      <c r="A958" s="5" t="inlineStr">
         <is>
           <t>SDFFQNX4</t>
         </is>
       </c>
-      <c r="B958" s="3" t="n"/>
-      <c r="C958" s="3" t="inlineStr">
+      <c r="B958" s="6" t="n"/>
+      <c r="C958" s="6" t="inlineStr">
         <is>
           <t>SDFFQNX4AHBCOTC</t>
         </is>
       </c>
     </row>
     <row r="959">
-      <c r="A959" s="2" t="n"/>
-      <c r="B959" s="3" t="n"/>
-      <c r="C959" s="3" t="inlineStr">
+      <c r="A959" s="7" t="n"/>
+      <c r="B959" s="8" t="n"/>
+      <c r="C959" s="8" t="inlineStr">
         <is>
           <t>SDFFQNX4AHQCOTC</t>
         </is>
@@ -14519,26 +14549,26 @@
       </c>
     </row>
     <row r="1028">
-      <c r="A1028" s="2" t="inlineStr">
+      <c r="A1028" s="5" t="inlineStr">
         <is>
           <t>XNR2D8</t>
         </is>
       </c>
-      <c r="B1028" s="3" t="inlineStr">
+      <c r="B1028" s="6" t="inlineStr">
         <is>
           <t>XNR2D8COTMDB</t>
         </is>
       </c>
-      <c r="C1028" s="3" t="inlineStr">
+      <c r="C1028" s="6" t="inlineStr">
         <is>
           <t>XNR2D8COT3FIN</t>
         </is>
       </c>
     </row>
     <row r="1029">
-      <c r="A1029" s="2" t="n"/>
-      <c r="B1029" s="3" t="n"/>
-      <c r="C1029" s="3" t="inlineStr">
+      <c r="A1029" s="7" t="n"/>
+      <c r="B1029" s="8" t="n"/>
+      <c r="C1029" s="8" t="inlineStr">
         <is>
           <t>XNR2EEQMBDD8COT</t>
         </is>
@@ -14696,22 +14726,22 @@
       </c>
     </row>
     <row r="1041">
-      <c r="A1041" s="2" t="inlineStr">
+      <c r="A1041" s="5" t="inlineStr">
         <is>
           <t>XNR2X2</t>
         </is>
       </c>
-      <c r="B1041" s="3" t="n"/>
-      <c r="C1041" s="3" t="inlineStr">
+      <c r="B1041" s="6" t="n"/>
+      <c r="C1041" s="6" t="inlineStr">
         <is>
           <t>XNR2X2ATACOTC</t>
         </is>
       </c>
     </row>
     <row r="1042">
-      <c r="A1042" s="2" t="n"/>
-      <c r="B1042" s="3" t="n"/>
-      <c r="C1042" s="3" t="inlineStr">
+      <c r="A1042" s="7" t="n"/>
+      <c r="B1042" s="8" t="n"/>
+      <c r="C1042" s="8" t="inlineStr">
         <is>
           <t>XNR2X2ATBCOTC</t>
         </is>
@@ -15200,22 +15230,22 @@
       </c>
     </row>
     <row r="1077">
-      <c r="A1077" s="2" t="inlineStr">
+      <c r="A1077" s="5" t="inlineStr">
         <is>
           <t>XOR2X1</t>
         </is>
       </c>
-      <c r="B1077" s="3" t="n"/>
-      <c r="C1077" s="3" t="inlineStr">
+      <c r="B1077" s="6" t="n"/>
+      <c r="C1077" s="6" t="inlineStr">
         <is>
           <t>XOR2X1ATACOTC</t>
         </is>
       </c>
     </row>
     <row r="1078">
-      <c r="A1078" s="2" t="n"/>
-      <c r="B1078" s="3" t="n"/>
-      <c r="C1078" s="3" t="inlineStr">
+      <c r="A1078" s="7" t="n"/>
+      <c r="B1078" s="8" t="n"/>
+      <c r="C1078" s="8" t="inlineStr">
         <is>
           <t>XOR2X1ATCCOTC</t>
         </is>

</xml_diff>

<commit_message>
Remove header bottom border; keep freeze panes only.
Leave A1:C1 without a bottom edge so the frozen header separates
from data without an extra line.

Co-authored-by: EsaLongs <EsaLongs@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/preview/NP1PP_vs_C1Y_preview.xlsx
+++ b/preview/NP1PP_vs_C1Y_preview.xlsx
@@ -58,14 +58,14 @@
       <top style="thin">
         <color rgb="00000000"/>
       </top>
-      <bottom style="thin">
-        <color rgb="00000000"/>
-      </bottom>
     </border>
     <border>
       <top style="thin">
         <color rgb="00000000"/>
       </top>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
     </border>
     <border>
       <bottom style="thin">
@@ -79,15 +79,15 @@
   <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>

</xml_diff>

<commit_message>
Add ordered --function-keys prefix matching for column A.
Grouping is controlled by an explicit key list (CLI and/or file): first
valid prefix wins and is not overridden later. Digit-after-key blocking
keeps OAI22 from stealing OAI2211/FILL12; letter-tailed compounds still
need longer-first order. Refresh suggested keys (435) and docs.

Co-authored-by: EsaLongs <EsaLongs@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/preview/NP1PP_vs_C1Y_preview.xlsx
+++ b/preview/NP1PP_vs_C1Y_preview.xlsx
@@ -1811,30 +1811,26 @@
       </c>
     </row>
     <row r="132">
-      <c r="A132" s="9" t="inlineStr">
+      <c r="A132" s="2" t="inlineStr">
         <is>
           <t>AOI21OAI21</t>
         </is>
       </c>
-      <c r="B132" s="10" t="inlineStr">
+      <c r="B132" s="11" t="inlineStr">
+        <is>
+          <t>AOI21OAI21CCAD2COT</t>
+        </is>
+      </c>
+      <c r="C132" s="11" t="n"/>
+    </row>
+    <row r="133">
+      <c r="A133" s="4" t="n"/>
+      <c r="B133" s="6" t="inlineStr">
         <is>
           <t>AOI21OAI21CCMD2COT</t>
         </is>
       </c>
-      <c r="C132" s="10" t="n"/>
-    </row>
-    <row r="133">
-      <c r="A133" s="2" t="inlineStr">
-        <is>
-          <t>AOI21OAI21CCA</t>
-        </is>
-      </c>
-      <c r="B133" s="11" t="inlineStr">
-        <is>
-          <t>AOI21OAI21CCAD2COT</t>
-        </is>
-      </c>
-      <c r="C133" s="11" t="n"/>
+      <c r="C133" s="6" t="n"/>
     </row>
     <row r="134">
       <c r="A134" s="7" t="n"/>
@@ -2395,39 +2391,35 @@
       </c>
       <c r="B189" s="11" t="inlineStr">
         <is>
+          <t>AOI22OAI21CCAD1COT</t>
+        </is>
+      </c>
+      <c r="C189" s="11" t="n"/>
+    </row>
+    <row r="190">
+      <c r="A190" s="4" t="n"/>
+      <c r="B190" s="6" t="inlineStr">
+        <is>
           <t>AOI22OAI21CCMD1COT</t>
         </is>
       </c>
-      <c r="C189" s="11" t="n"/>
-    </row>
-    <row r="190">
-      <c r="A190" s="7" t="n"/>
-      <c r="B190" s="8" t="n"/>
-      <c r="C190" s="8" t="inlineStr">
-        <is>
-          <t>AOI22OAI21CCBD1COTA</t>
-        </is>
-      </c>
+      <c r="C190" s="6" t="n"/>
     </row>
     <row r="191">
-      <c r="A191" s="2" t="inlineStr">
-        <is>
-          <t>AOI22OAI21CCA</t>
-        </is>
-      </c>
-      <c r="B191" s="11" t="inlineStr">
-        <is>
-          <t>AOI22OAI21CCAD1COT</t>
-        </is>
-      </c>
-      <c r="C191" s="11" t="n"/>
+      <c r="A191" s="4" t="n"/>
+      <c r="B191" s="6" t="n"/>
+      <c r="C191" s="6" t="inlineStr">
+        <is>
+          <t>AOI22OAI21CCAD1COTA</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" s="7" t="n"/>
       <c r="B192" s="8" t="n"/>
       <c r="C192" s="8" t="inlineStr">
         <is>
-          <t>AOI22OAI21CCAD1COTA</t>
+          <t>AOI22OAI21CCBD1COTA</t>
         </is>
       </c>
     </row>
@@ -3748,35 +3740,27 @@
       </c>
     </row>
     <row r="305">
-      <c r="A305" s="7" t="n"/>
-      <c r="B305" s="8" t="n"/>
-      <c r="C305" s="8" t="inlineStr">
+      <c r="A305" s="4" t="n"/>
+      <c r="B305" s="6" t="n"/>
+      <c r="C305" s="6" t="inlineStr">
         <is>
           <t>CMPE32D4SFCOT</t>
         </is>
       </c>
     </row>
     <row r="306">
-      <c r="A306" s="9" t="inlineStr">
-        <is>
-          <t>CMPE32D4TGAR</t>
-        </is>
-      </c>
-      <c r="B306" s="10" t="n"/>
-      <c r="C306" s="10" t="inlineStr">
+      <c r="A306" s="4" t="n"/>
+      <c r="B306" s="6" t="n"/>
+      <c r="C306" s="6" t="inlineStr">
         <is>
           <t>CMPE32D4TGARCOT</t>
         </is>
       </c>
     </row>
     <row r="307">
-      <c r="A307" s="9" t="inlineStr">
-        <is>
-          <t>CMPE32D4XNRAR</t>
-        </is>
-      </c>
-      <c r="B307" s="10" t="n"/>
-      <c r="C307" s="10" t="inlineStr">
+      <c r="A307" s="7" t="n"/>
+      <c r="B307" s="8" t="n"/>
+      <c r="C307" s="8" t="inlineStr">
         <is>
           <t>CMPE32D4XNRARCOT</t>
         </is>
@@ -4838,78 +4822,74 @@
       <c r="C398" s="10" t="n"/>
     </row>
     <row r="399">
-      <c r="A399" s="9" t="inlineStr">
+      <c r="A399" s="2" t="inlineStr">
         <is>
           <t>FILL1</t>
         </is>
       </c>
-      <c r="B399" s="10" t="n"/>
-      <c r="C399" s="10" t="inlineStr">
+      <c r="B399" s="11" t="n"/>
+      <c r="C399" s="11" t="inlineStr">
         <is>
           <t>FILL1COT</t>
         </is>
       </c>
     </row>
     <row r="400">
-      <c r="A400" s="2" t="inlineStr">
+      <c r="A400" s="7" t="n"/>
+      <c r="B400" s="8" t="n"/>
+      <c r="C400" s="8" t="inlineStr">
+        <is>
+          <t>FILL1NOBCMCOT</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" s="2" t="inlineStr">
         <is>
           <t>FILL12</t>
         </is>
       </c>
-      <c r="B400" s="11" t="inlineStr">
+      <c r="B401" s="11" t="inlineStr">
         <is>
           <t>FILL12COT</t>
         </is>
       </c>
-      <c r="C400" s="11" t="n"/>
-    </row>
-    <row r="401">
-      <c r="A401" s="7" t="n"/>
-      <c r="B401" s="8" t="inlineStr">
+      <c r="C401" s="11" t="n"/>
+    </row>
+    <row r="402">
+      <c r="A402" s="7" t="n"/>
+      <c r="B402" s="8" t="inlineStr">
         <is>
           <t>FILL12VGCOT</t>
         </is>
       </c>
-      <c r="C401" s="8" t="n"/>
-    </row>
-    <row r="402">
-      <c r="A402" s="2" t="inlineStr">
+      <c r="C402" s="8" t="n"/>
+    </row>
+    <row r="403">
+      <c r="A403" s="2" t="inlineStr">
         <is>
           <t>FILL16</t>
         </is>
       </c>
-      <c r="B402" s="3" t="inlineStr">
+      <c r="B403" s="3" t="inlineStr">
         <is>
           <t>FILL16COT</t>
         </is>
       </c>
-      <c r="C402" s="3" t="inlineStr">
+      <c r="C403" s="3" t="inlineStr">
         <is>
           <t>FILL16COT</t>
         </is>
       </c>
     </row>
-    <row r="403">
-      <c r="A403" s="7" t="n"/>
-      <c r="B403" s="8" t="inlineStr">
+    <row r="404">
+      <c r="A404" s="7" t="n"/>
+      <c r="B404" s="8" t="inlineStr">
         <is>
           <t>FILL16VGCOT</t>
         </is>
       </c>
-      <c r="C403" s="8" t="n"/>
-    </row>
-    <row r="404">
-      <c r="A404" s="9" t="inlineStr">
-        <is>
-          <t>FILL1NOBCM</t>
-        </is>
-      </c>
-      <c r="B404" s="10" t="n"/>
-      <c r="C404" s="10" t="inlineStr">
-        <is>
-          <t>FILL1NOBCMCOT</t>
-        </is>
-      </c>
+      <c r="C404" s="8" t="n"/>
     </row>
     <row r="405">
       <c r="A405" s="2" t="inlineStr">
@@ -6618,22 +6598,18 @@
       <c r="C546" s="6" t="n"/>
     </row>
     <row r="547">
-      <c r="A547" s="7" t="n"/>
-      <c r="B547" s="8" t="inlineStr">
+      <c r="A547" s="4" t="n"/>
+      <c r="B547" s="6" t="inlineStr">
         <is>
           <t>IND2OPTPAD1COTOPU</t>
         </is>
       </c>
-      <c r="C547" s="8" t="n"/>
+      <c r="C547" s="6" t="n"/>
     </row>
     <row r="548">
-      <c r="A548" s="2" t="inlineStr">
-        <is>
-          <t>IND2DBA4</t>
-        </is>
-      </c>
-      <c r="B548" s="11" t="n"/>
-      <c r="C548" s="11" t="inlineStr">
+      <c r="A548" s="4" t="n"/>
+      <c r="B548" s="6" t="n"/>
+      <c r="C548" s="6" t="inlineStr">
         <is>
           <t>IND2DBA4AFOPTPAD8COT</t>
         </is>
@@ -6809,22 +6785,18 @@
       </c>
     </row>
     <row r="566">
-      <c r="A566" s="7" t="n"/>
-      <c r="B566" s="8" t="n"/>
-      <c r="C566" s="8" t="inlineStr">
+      <c r="A566" s="4" t="n"/>
+      <c r="B566" s="6" t="n"/>
+      <c r="C566" s="6" t="inlineStr">
         <is>
           <t>INR2D8COT3FIN</t>
         </is>
       </c>
     </row>
     <row r="567">
-      <c r="A567" s="2" t="inlineStr">
-        <is>
-          <t>INR2DBA4</t>
-        </is>
-      </c>
-      <c r="B567" s="11" t="n"/>
-      <c r="C567" s="11" t="inlineStr">
+      <c r="A567" s="4" t="n"/>
+      <c r="B567" s="6" t="n"/>
+      <c r="C567" s="6" t="inlineStr">
         <is>
           <t>INR2DBA4AFD8COT</t>
         </is>
@@ -7572,42 +7544,34 @@
       <c r="B633" s="6" t="n"/>
       <c r="C633" s="6" t="inlineStr">
         <is>
+          <t>LVLLHBUFFSNKCWBALD4COT</t>
+        </is>
+      </c>
+    </row>
+    <row r="634">
+      <c r="A634" s="4" t="n"/>
+      <c r="B634" s="6" t="n"/>
+      <c r="C634" s="6" t="inlineStr">
+        <is>
           <t>LVLLHBUFFSNKCWD4CNWBALCOT</t>
         </is>
       </c>
     </row>
-    <row r="634">
-      <c r="A634" s="7" t="n"/>
-      <c r="B634" s="8" t="n"/>
-      <c r="C634" s="8" t="inlineStr">
+    <row r="635">
+      <c r="A635" s="4" t="n"/>
+      <c r="B635" s="6" t="n"/>
+      <c r="C635" s="6" t="inlineStr">
+        <is>
+          <t>LVLLHBUFFSRCCWBALD1COT</t>
+        </is>
+      </c>
+    </row>
+    <row r="636">
+      <c r="A636" s="7" t="n"/>
+      <c r="B636" s="8" t="n"/>
+      <c r="C636" s="8" t="inlineStr">
         <is>
           <t>LVLLHBUFFSRCCWD8CNWCOTLN</t>
-        </is>
-      </c>
-    </row>
-    <row r="635">
-      <c r="A635" s="9" t="inlineStr">
-        <is>
-          <t>LVLLHBUFFSNKCWBAL</t>
-        </is>
-      </c>
-      <c r="B635" s="10" t="n"/>
-      <c r="C635" s="10" t="inlineStr">
-        <is>
-          <t>LVLLHBUFFSNKCWBALD4COT</t>
-        </is>
-      </c>
-    </row>
-    <row r="636">
-      <c r="A636" s="9" t="inlineStr">
-        <is>
-          <t>LVLLHBUFFSRCCWBAL</t>
-        </is>
-      </c>
-      <c r="B636" s="10" t="n"/>
-      <c r="C636" s="10" t="inlineStr">
-        <is>
-          <t>LVLLHBUFFSRCCWBALD1COT</t>
         </is>
       </c>
     </row>
@@ -7625,48 +7589,36 @@
       <c r="C637" s="11" t="n"/>
     </row>
     <row r="638">
-      <c r="A638" s="7" t="n"/>
-      <c r="B638" s="8" t="inlineStr">
+      <c r="A638" s="4" t="n"/>
+      <c r="B638" s="6" t="inlineStr">
         <is>
           <t>LVLLHCHSRCD4COTVIA</t>
         </is>
       </c>
-      <c r="C638" s="8" t="n"/>
+      <c r="C638" s="6" t="n"/>
     </row>
     <row r="639">
-      <c r="A639" s="9" t="inlineStr">
-        <is>
-          <t>LVLLHCHSNKCWBALRB</t>
-        </is>
-      </c>
-      <c r="B639" s="10" t="n"/>
-      <c r="C639" s="10" t="inlineStr">
+      <c r="A639" s="4" t="n"/>
+      <c r="B639" s="6" t="n"/>
+      <c r="C639" s="6" t="inlineStr">
         <is>
           <t>LVLLHCHSNKCWBALRBD2COT</t>
         </is>
       </c>
     </row>
     <row r="640">
-      <c r="A640" s="9" t="inlineStr">
-        <is>
-          <t>LVLLHCHSRCCWBALRB</t>
-        </is>
-      </c>
-      <c r="B640" s="10" t="n"/>
-      <c r="C640" s="10" t="inlineStr">
+      <c r="A640" s="4" t="n"/>
+      <c r="B640" s="6" t="n"/>
+      <c r="C640" s="6" t="inlineStr">
         <is>
           <t>LVLLHCHSRCCWBALRBD4COT</t>
         </is>
       </c>
     </row>
     <row r="641">
-      <c r="A641" s="2" t="inlineStr">
-        <is>
-          <t>LVLLHCHSRCCWRB</t>
-        </is>
-      </c>
-      <c r="B641" s="11" t="n"/>
-      <c r="C641" s="11" t="inlineStr">
+      <c r="A641" s="4" t="n"/>
+      <c r="B641" s="6" t="n"/>
+      <c r="C641" s="6" t="inlineStr">
         <is>
           <t>LVLLHCHSRCCWRBD4CNWCOT</t>
         </is>
@@ -7695,57 +7647,45 @@
       <c r="C643" s="11" t="n"/>
     </row>
     <row r="644">
-      <c r="A644" s="7" t="n"/>
-      <c r="B644" s="8" t="inlineStr">
+      <c r="A644" s="4" t="n"/>
+      <c r="B644" s="6" t="inlineStr">
         <is>
           <t>LVLLHCLSRCD4COT</t>
         </is>
       </c>
-      <c r="C644" s="8" t="n"/>
+      <c r="C644" s="6" t="n"/>
     </row>
     <row r="645">
-      <c r="A645" s="9" t="inlineStr">
-        <is>
-          <t>LVLLHCLSNKCWBALRB</t>
-        </is>
-      </c>
-      <c r="B645" s="10" t="n"/>
-      <c r="C645" s="10" t="inlineStr">
+      <c r="A645" s="4" t="n"/>
+      <c r="B645" s="6" t="n"/>
+      <c r="C645" s="6" t="inlineStr">
         <is>
           <t>LVLLHCLSNKCWBALRBD4COT</t>
         </is>
       </c>
     </row>
     <row r="646">
-      <c r="A646" s="2" t="inlineStr">
-        <is>
-          <t>LVLLHCLSNKCWRB</t>
-        </is>
-      </c>
-      <c r="B646" s="11" t="n"/>
-      <c r="C646" s="11" t="inlineStr">
+      <c r="A646" s="4" t="n"/>
+      <c r="B646" s="6" t="n"/>
+      <c r="C646" s="6" t="inlineStr">
         <is>
           <t>LVLLHCLSNKCWRBD2CNWCOT</t>
         </is>
       </c>
     </row>
     <row r="647">
-      <c r="A647" s="7" t="n"/>
-      <c r="B647" s="8" t="n"/>
-      <c r="C647" s="8" t="inlineStr">
+      <c r="A647" s="4" t="n"/>
+      <c r="B647" s="6" t="n"/>
+      <c r="C647" s="6" t="inlineStr">
         <is>
           <t>LVLLHCLSNKCWRBD2COT</t>
         </is>
       </c>
     </row>
     <row r="648">
-      <c r="A648" s="9" t="inlineStr">
-        <is>
-          <t>LVLLHCLSRCCWRB</t>
-        </is>
-      </c>
-      <c r="B648" s="10" t="n"/>
-      <c r="C648" s="10" t="inlineStr">
+      <c r="A648" s="7" t="n"/>
+      <c r="B648" s="8" t="n"/>
+      <c r="C648" s="8" t="inlineStr">
         <is>
           <t>LVLLHCLSRCCWRBD4CNWCOT</t>
         </is>
@@ -7851,111 +7791,111 @@
     <row r="658">
       <c r="A658" s="2" t="inlineStr">
         <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="B658" s="11" t="n"/>
-      <c r="C658" s="11" t="inlineStr">
-        <is>
-          <t>MX2X2ATACOTC</t>
-        </is>
-      </c>
+          <t>MAOI22</t>
+        </is>
+      </c>
+      <c r="B658" s="11" t="inlineStr">
+        <is>
+          <t>MAOI22D1COT</t>
+        </is>
+      </c>
+      <c r="C658" s="11" t="n"/>
     </row>
     <row r="659">
       <c r="A659" s="4" t="n"/>
-      <c r="B659" s="6" t="n"/>
-      <c r="C659" s="6" t="inlineStr">
-        <is>
-          <t>MX2X2ATFCOTC</t>
-        </is>
-      </c>
+      <c r="B659" s="6" t="inlineStr">
+        <is>
+          <t>MAOI22D2COTVIA</t>
+        </is>
+      </c>
+      <c r="C659" s="6" t="n"/>
     </row>
     <row r="660">
-      <c r="A660" s="7" t="n"/>
-      <c r="B660" s="8" t="n"/>
-      <c r="C660" s="8" t="inlineStr">
-        <is>
-          <t>MX2X8ATACOTC</t>
-        </is>
-      </c>
+      <c r="A660" s="4" t="n"/>
+      <c r="B660" s="6" t="inlineStr">
+        <is>
+          <t>MAOI22D4COTVIA</t>
+        </is>
+      </c>
+      <c r="C660" s="6" t="n"/>
     </row>
     <row r="661">
-      <c r="A661" s="2" t="inlineStr">
-        <is>
-          <t>MAOI22</t>
-        </is>
-      </c>
-      <c r="B661" s="11" t="inlineStr">
-        <is>
-          <t>MAOI22D1COT</t>
-        </is>
-      </c>
-      <c r="C661" s="11" t="n"/>
+      <c r="A661" s="7" t="n"/>
+      <c r="B661" s="8" t="n"/>
+      <c r="C661" s="8" t="inlineStr">
+        <is>
+          <t>MAOI22D4COT</t>
+        </is>
+      </c>
     </row>
     <row r="662">
-      <c r="A662" s="4" t="n"/>
-      <c r="B662" s="6" t="inlineStr">
-        <is>
-          <t>MAOI22D2COTVIA</t>
-        </is>
-      </c>
-      <c r="C662" s="6" t="n"/>
+      <c r="A662" s="2" t="inlineStr">
+        <is>
+          <t>MAOI222</t>
+        </is>
+      </c>
+      <c r="B662" s="11" t="inlineStr">
+        <is>
+          <t>MAOI222D1COT</t>
+        </is>
+      </c>
+      <c r="C662" s="11" t="n"/>
     </row>
     <row r="663">
       <c r="A663" s="4" t="n"/>
       <c r="B663" s="6" t="inlineStr">
         <is>
-          <t>MAOI22D4COTVIA</t>
+          <t>MAOI222D2COTVIA</t>
         </is>
       </c>
       <c r="C663" s="6" t="n"/>
     </row>
     <row r="664">
-      <c r="A664" s="7" t="n"/>
-      <c r="B664" s="8" t="n"/>
-      <c r="C664" s="8" t="inlineStr">
-        <is>
-          <t>MAOI22D4COT</t>
-        </is>
-      </c>
+      <c r="A664" s="4" t="n"/>
+      <c r="B664" s="6" t="inlineStr">
+        <is>
+          <t>MAOI222D4COTMDB</t>
+        </is>
+      </c>
+      <c r="C664" s="6" t="n"/>
     </row>
     <row r="665">
-      <c r="A665" s="2" t="inlineStr">
-        <is>
-          <t>MAOI222</t>
-        </is>
-      </c>
-      <c r="B665" s="11" t="inlineStr">
-        <is>
-          <t>MAOI222D1COT</t>
-        </is>
-      </c>
-      <c r="C665" s="11" t="n"/>
+      <c r="A665" s="4" t="n"/>
+      <c r="B665" s="6" t="n"/>
+      <c r="C665" s="6" t="inlineStr">
+        <is>
+          <t>MAOI222D2COT</t>
+        </is>
+      </c>
     </row>
     <row r="666">
-      <c r="A666" s="4" t="n"/>
-      <c r="B666" s="6" t="inlineStr">
-        <is>
-          <t>MAOI222D2COTVIA</t>
-        </is>
-      </c>
-      <c r="C666" s="6" t="n"/>
+      <c r="A666" s="7" t="n"/>
+      <c r="B666" s="8" t="n"/>
+      <c r="C666" s="8" t="inlineStr">
+        <is>
+          <t>MAOI222D4COT</t>
+        </is>
+      </c>
     </row>
     <row r="667">
-      <c r="A667" s="4" t="n"/>
-      <c r="B667" s="6" t="inlineStr">
-        <is>
-          <t>MAOI222D4COTMDB</t>
-        </is>
-      </c>
-      <c r="C667" s="6" t="n"/>
+      <c r="A667" s="2" t="inlineStr">
+        <is>
+          <t>MB2LHCNQ</t>
+        </is>
+      </c>
+      <c r="B667" s="11" t="inlineStr">
+        <is>
+          <t>MB2LHCNQD4COTVIAOPP</t>
+        </is>
+      </c>
+      <c r="C667" s="11" t="n"/>
     </row>
     <row r="668">
       <c r="A668" s="4" t="n"/>
       <c r="B668" s="6" t="n"/>
       <c r="C668" s="6" t="inlineStr">
         <is>
-          <t>MAOI222D2COT</t>
+          <t>MB2LHCNQD1ARCOT</t>
         </is>
       </c>
     </row>
@@ -7964,160 +7904,160 @@
       <c r="B669" s="8" t="n"/>
       <c r="C669" s="8" t="inlineStr">
         <is>
-          <t>MAOI222D4COT</t>
+          <t>MB2LHCNQD2ARSPCOT</t>
         </is>
       </c>
     </row>
     <row r="670">
       <c r="A670" s="2" t="inlineStr">
         <is>
-          <t>MB2LHCNQ</t>
+          <t>MB2LHQ</t>
         </is>
       </c>
       <c r="B670" s="11" t="inlineStr">
         <is>
-          <t>MB2LHCNQD4COTVIAOPP</t>
+          <t>MB2LHQD1COT</t>
         </is>
       </c>
       <c r="C670" s="11" t="n"/>
     </row>
     <row r="671">
-      <c r="A671" s="7" t="n"/>
-      <c r="B671" s="8" t="n"/>
-      <c r="C671" s="8" t="inlineStr">
-        <is>
-          <t>MB2LHCNQD1ARCOT</t>
+      <c r="A671" s="4" t="n"/>
+      <c r="B671" s="6" t="n"/>
+      <c r="C671" s="6" t="inlineStr">
+        <is>
+          <t>MB2LHQD2BFCOT</t>
         </is>
       </c>
     </row>
     <row r="672">
-      <c r="A672" s="9" t="inlineStr">
-        <is>
-          <t>MB2LHCNQD2ARSP</t>
-        </is>
-      </c>
-      <c r="B672" s="10" t="n"/>
-      <c r="C672" s="10" t="inlineStr">
-        <is>
-          <t>MB2LHCNQD2ARSPCOT</t>
+      <c r="A672" s="4" t="n"/>
+      <c r="B672" s="6" t="n"/>
+      <c r="C672" s="6" t="inlineStr">
+        <is>
+          <t>MB2LHQD2COT</t>
         </is>
       </c>
     </row>
     <row r="673">
-      <c r="A673" s="2" t="inlineStr">
-        <is>
-          <t>MB2LHQ</t>
-        </is>
-      </c>
-      <c r="B673" s="11" t="inlineStr">
-        <is>
-          <t>MB2LHQD1COT</t>
-        </is>
-      </c>
-      <c r="C673" s="11" t="n"/>
+      <c r="A673" s="7" t="n"/>
+      <c r="B673" s="8" t="n"/>
+      <c r="C673" s="8" t="inlineStr">
+        <is>
+          <t>MB2LHQD2FFCOT</t>
+        </is>
+      </c>
     </row>
     <row r="674">
-      <c r="A674" s="4" t="n"/>
-      <c r="B674" s="6" t="n"/>
-      <c r="C674" s="6" t="inlineStr">
-        <is>
-          <t>MB2LHQD2BFCOT</t>
-        </is>
-      </c>
+      <c r="A674" s="9" t="inlineStr">
+        <is>
+          <t>MB2LHSPCNQ</t>
+        </is>
+      </c>
+      <c r="B674" s="10" t="inlineStr">
+        <is>
+          <t>MB2LHSPCNQD2COTVIA</t>
+        </is>
+      </c>
+      <c r="C674" s="10" t="n"/>
     </row>
     <row r="675">
-      <c r="A675" s="4" t="n"/>
-      <c r="B675" s="6" t="n"/>
-      <c r="C675" s="6" t="inlineStr">
-        <is>
-          <t>MB2LHQD2COT</t>
-        </is>
-      </c>
+      <c r="A675" s="2" t="inlineStr">
+        <is>
+          <t>MB2LNCNQ</t>
+        </is>
+      </c>
+      <c r="B675" s="11" t="inlineStr">
+        <is>
+          <t>MB2LNCNQD4COTVIAOPP</t>
+        </is>
+      </c>
+      <c r="C675" s="11" t="n"/>
     </row>
     <row r="676">
       <c r="A676" s="7" t="n"/>
       <c r="B676" s="8" t="n"/>
       <c r="C676" s="8" t="inlineStr">
         <is>
-          <t>MB2LHQD2FFCOT</t>
+          <t>MB2LNCNQD4ARCOT</t>
         </is>
       </c>
     </row>
     <row r="677">
-      <c r="A677" s="9" t="inlineStr">
-        <is>
-          <t>MB2LHSPCNQ</t>
-        </is>
-      </c>
-      <c r="B677" s="10" t="inlineStr">
-        <is>
-          <t>MB2LHSPCNQD2COTVIA</t>
-        </is>
-      </c>
-      <c r="C677" s="10" t="n"/>
+      <c r="A677" s="2" t="inlineStr">
+        <is>
+          <t>MB2LNQ</t>
+        </is>
+      </c>
+      <c r="B677" s="11" t="inlineStr">
+        <is>
+          <t>MB2LNQD2COT</t>
+        </is>
+      </c>
+      <c r="C677" s="11" t="n"/>
     </row>
     <row r="678">
-      <c r="A678" s="2" t="inlineStr">
-        <is>
-          <t>MB2LNCNQ</t>
-        </is>
-      </c>
-      <c r="B678" s="11" t="inlineStr">
-        <is>
-          <t>MB2LNCNQD4COTVIAOPP</t>
-        </is>
-      </c>
-      <c r="C678" s="11" t="n"/>
+      <c r="A678" s="4" t="n"/>
+      <c r="B678" s="6" t="n"/>
+      <c r="C678" s="6" t="inlineStr">
+        <is>
+          <t>MB2LNQD1BFCOT</t>
+        </is>
+      </c>
     </row>
     <row r="679">
       <c r="A679" s="7" t="n"/>
       <c r="B679" s="8" t="n"/>
       <c r="C679" s="8" t="inlineStr">
         <is>
-          <t>MB2LNCNQD4ARCOT</t>
+          <t>MB2LNQD2FFCOT</t>
         </is>
       </c>
     </row>
     <row r="680">
-      <c r="A680" s="2" t="inlineStr">
-        <is>
-          <t>MB2LNQ</t>
-        </is>
-      </c>
-      <c r="B680" s="11" t="inlineStr">
-        <is>
-          <t>MB2LNQD2COT</t>
-        </is>
-      </c>
-      <c r="C680" s="11" t="n"/>
+      <c r="A680" s="9" t="inlineStr">
+        <is>
+          <t>MB2LNSPCNQ</t>
+        </is>
+      </c>
+      <c r="B680" s="10" t="inlineStr">
+        <is>
+          <t>MB2LNSPCNQD4COTM3CEQ</t>
+        </is>
+      </c>
+      <c r="C680" s="10" t="n"/>
     </row>
     <row r="681">
-      <c r="A681" s="4" t="n"/>
-      <c r="B681" s="6" t="n"/>
-      <c r="C681" s="6" t="inlineStr">
-        <is>
-          <t>MB2LNQD1BFCOT</t>
-        </is>
-      </c>
+      <c r="A681" s="2" t="inlineStr">
+        <is>
+          <t>MB2SRLSDFKRPQ</t>
+        </is>
+      </c>
+      <c r="B681" s="11" t="inlineStr">
+        <is>
+          <t>MB2SRLSDFKRPQD2COTONEOPU</t>
+        </is>
+      </c>
+      <c r="C681" s="11" t="n"/>
     </row>
     <row r="682">
       <c r="A682" s="7" t="n"/>
       <c r="B682" s="8" t="n"/>
       <c r="C682" s="8" t="inlineStr">
         <is>
-          <t>MB2LNQD2FFCOT</t>
+          <t>MB2SRLSDFKRPQD2COTSC4LP</t>
         </is>
       </c>
     </row>
     <row r="683">
       <c r="A683" s="9" t="inlineStr">
         <is>
-          <t>MB2LNSPCNQ</t>
+          <t>MB2SRLSDFQ</t>
         </is>
       </c>
       <c r="B683" s="10" t="inlineStr">
         <is>
-          <t>MB2LNSPCNQD4COTM3CEQ</t>
+          <t>MB2SRLSDFQD2COTONEOPU</t>
         </is>
       </c>
       <c r="C683" s="10" t="n"/>
@@ -8125,12 +8065,12 @@
     <row r="684">
       <c r="A684" s="2" t="inlineStr">
         <is>
-          <t>MB2SRLSDFKRPQ</t>
+          <t>MB2SRLSDFRPQ</t>
         </is>
       </c>
       <c r="B684" s="11" t="inlineStr">
         <is>
-          <t>MB2SRLSDFKRPQD2COTONEOPU</t>
+          <t>MB2SRLSDFRPQD2COTONEOPU</t>
         </is>
       </c>
       <c r="C684" s="11" t="n"/>
@@ -8140,344 +8080,340 @@
       <c r="B685" s="8" t="n"/>
       <c r="C685" s="8" t="inlineStr">
         <is>
-          <t>MB2SRLSDFKRPQD2COTSC4LP</t>
+          <t>MB2SRLSDFRPQD1COTSC5LP</t>
         </is>
       </c>
     </row>
     <row r="686">
       <c r="A686" s="9" t="inlineStr">
         <is>
-          <t>MB2SRLSDFQ</t>
+          <t>MB2SRLSDFSNQ</t>
         </is>
       </c>
       <c r="B686" s="10" t="inlineStr">
         <is>
-          <t>MB2SRLSDFQD2COTONEOPU</t>
+          <t>MB2SRLSDFSNQD2COTONEOPU</t>
         </is>
       </c>
       <c r="C686" s="10" t="n"/>
     </row>
     <row r="687">
-      <c r="A687" s="2" t="inlineStr">
-        <is>
-          <t>MB2SRLSDFRPQ</t>
-        </is>
-      </c>
-      <c r="B687" s="11" t="inlineStr">
-        <is>
-          <t>MB2SRLSDFRPQD2COTONEOPU</t>
-        </is>
-      </c>
-      <c r="C687" s="11" t="n"/>
+      <c r="A687" s="9" t="inlineStr">
+        <is>
+          <t>MB4LHQ</t>
+        </is>
+      </c>
+      <c r="B687" s="10" t="inlineStr">
+        <is>
+          <t>MB4LHQD4COT</t>
+        </is>
+      </c>
+      <c r="C687" s="10" t="n"/>
     </row>
     <row r="688">
-      <c r="A688" s="7" t="n"/>
-      <c r="B688" s="8" t="n"/>
-      <c r="C688" s="8" t="inlineStr">
-        <is>
-          <t>MB2SRLSDFRPQD1COTSC5LP</t>
-        </is>
-      </c>
+      <c r="A688" s="9" t="inlineStr">
+        <is>
+          <t>MB4LNQ</t>
+        </is>
+      </c>
+      <c r="B688" s="10" t="inlineStr">
+        <is>
+          <t>MB4LNQD1COTVIA</t>
+        </is>
+      </c>
+      <c r="C688" s="10" t="n"/>
     </row>
     <row r="689">
       <c r="A689" s="9" t="inlineStr">
         <is>
-          <t>MB2SRLSDFSNQ</t>
+          <t>MB4SRLSDFKRPQ</t>
         </is>
       </c>
       <c r="B689" s="10" t="inlineStr">
         <is>
-          <t>MB2SRLSDFSNQD2COTONEOPU</t>
+          <t>MB4SRLSDFKRPQD1COTVIA</t>
         </is>
       </c>
       <c r="C689" s="10" t="n"/>
     </row>
     <row r="690">
-      <c r="A690" s="9" t="inlineStr">
-        <is>
-          <t>MB4LHQ</t>
-        </is>
-      </c>
-      <c r="B690" s="10" t="inlineStr">
-        <is>
-          <t>MB4LHQD4COT</t>
-        </is>
-      </c>
-      <c r="C690" s="10" t="n"/>
+      <c r="A690" s="2" t="inlineStr">
+        <is>
+          <t>MB4SRLSDFQ</t>
+        </is>
+      </c>
+      <c r="B690" s="11" t="inlineStr">
+        <is>
+          <t>MB4SRLSDFQD1COTVIA</t>
+        </is>
+      </c>
+      <c r="C690" s="11" t="n"/>
     </row>
     <row r="691">
-      <c r="A691" s="9" t="inlineStr">
-        <is>
-          <t>MB4LNQ</t>
-        </is>
-      </c>
-      <c r="B691" s="10" t="inlineStr">
-        <is>
-          <t>MB4LNQD1COTVIA</t>
-        </is>
-      </c>
-      <c r="C691" s="10" t="n"/>
+      <c r="A691" s="7" t="n"/>
+      <c r="B691" s="8" t="n"/>
+      <c r="C691" s="8" t="inlineStr">
+        <is>
+          <t>MB4SRLSDFQD1COT</t>
+        </is>
+      </c>
     </row>
     <row r="692">
-      <c r="A692" s="9" t="inlineStr">
-        <is>
-          <t>MB4SRLSDFKRPQ</t>
-        </is>
-      </c>
-      <c r="B692" s="10" t="inlineStr">
-        <is>
-          <t>MB4SRLSDFKRPQD1COTVIA</t>
-        </is>
-      </c>
-      <c r="C692" s="10" t="n"/>
+      <c r="A692" s="2" t="inlineStr">
+        <is>
+          <t>MB4SRLSDFRPQ</t>
+        </is>
+      </c>
+      <c r="B692" s="11" t="inlineStr">
+        <is>
+          <t>MB4SRLSDFRPQD2COTOPUEEQ</t>
+        </is>
+      </c>
+      <c r="C692" s="11" t="n"/>
     </row>
     <row r="693">
-      <c r="A693" s="2" t="inlineStr">
-        <is>
-          <t>MB4SRLSDFQ</t>
-        </is>
-      </c>
-      <c r="B693" s="11" t="inlineStr">
-        <is>
-          <t>MB4SRLSDFQD1COTVIA</t>
-        </is>
-      </c>
-      <c r="C693" s="11" t="n"/>
+      <c r="A693" s="7" t="n"/>
+      <c r="B693" s="8" t="n"/>
+      <c r="C693" s="8" t="inlineStr">
+        <is>
+          <t>MB4SRLSDFRPQD1ONECOT</t>
+        </is>
+      </c>
     </row>
     <row r="694">
-      <c r="A694" s="7" t="n"/>
-      <c r="B694" s="8" t="n"/>
-      <c r="C694" s="8" t="inlineStr">
-        <is>
-          <t>MB4SRLSDFQD1COT</t>
-        </is>
-      </c>
+      <c r="A694" s="9" t="inlineStr">
+        <is>
+          <t>MB4SRLSDFSNQ</t>
+        </is>
+      </c>
+      <c r="B694" s="10" t="inlineStr">
+        <is>
+          <t>MB4SRLSDFSNQD1COTM3CEQ</t>
+        </is>
+      </c>
+      <c r="C694" s="10" t="n"/>
     </row>
     <row r="695">
-      <c r="A695" s="2" t="inlineStr">
-        <is>
-          <t>MB4SRLSDFRPQ</t>
-        </is>
-      </c>
-      <c r="B695" s="11" t="inlineStr">
-        <is>
-          <t>MB4SRLSDFRPQD2COTOPUEEQ</t>
-        </is>
-      </c>
-      <c r="C695" s="11" t="n"/>
+      <c r="A695" s="9" t="inlineStr">
+        <is>
+          <t>MCECNQ</t>
+        </is>
+      </c>
+      <c r="B695" s="10" t="n"/>
+      <c r="C695" s="10" t="inlineStr">
+        <is>
+          <t>MCECNQD1COT</t>
+        </is>
+      </c>
     </row>
     <row r="696">
-      <c r="A696" s="7" t="n"/>
-      <c r="B696" s="8" t="n"/>
-      <c r="C696" s="8" t="inlineStr">
-        <is>
-          <t>MB4SRLSDFRPQD1ONECOT</t>
+      <c r="A696" s="2" t="inlineStr">
+        <is>
+          <t>MOAI22</t>
+        </is>
+      </c>
+      <c r="B696" s="3" t="inlineStr">
+        <is>
+          <t>MOAI22D4COT</t>
+        </is>
+      </c>
+      <c r="C696" s="3" t="inlineStr">
+        <is>
+          <t>MOAI22D4COT</t>
         </is>
       </c>
     </row>
     <row r="697">
-      <c r="A697" s="9" t="inlineStr">
-        <is>
-          <t>MB4SRLSDFSNQ</t>
-        </is>
-      </c>
-      <c r="B697" s="10" t="inlineStr">
-        <is>
-          <t>MB4SRLSDFSNQD1COTM3CEQ</t>
-        </is>
-      </c>
-      <c r="C697" s="10" t="n"/>
+      <c r="A697" s="4" t="n"/>
+      <c r="B697" s="6" t="inlineStr">
+        <is>
+          <t>MOAI22D1COTVIAMVM2OPU</t>
+        </is>
+      </c>
+      <c r="C697" s="6" t="n"/>
     </row>
     <row r="698">
-      <c r="A698" s="9" t="inlineStr">
-        <is>
-          <t>MCECNQ</t>
-        </is>
-      </c>
-      <c r="B698" s="10" t="n"/>
-      <c r="C698" s="10" t="inlineStr">
-        <is>
-          <t>MCECNQD1COT</t>
-        </is>
-      </c>
+      <c r="A698" s="4" t="n"/>
+      <c r="B698" s="6" t="inlineStr">
+        <is>
+          <t>MOAI22D2COT</t>
+        </is>
+      </c>
+      <c r="C698" s="6" t="n"/>
     </row>
     <row r="699">
-      <c r="A699" s="2" t="inlineStr">
-        <is>
-          <t>MOAI22</t>
-        </is>
-      </c>
-      <c r="B699" s="3" t="inlineStr">
-        <is>
-          <t>MOAI22D4COT</t>
-        </is>
-      </c>
-      <c r="C699" s="3" t="inlineStr">
-        <is>
-          <t>MOAI22D4COT</t>
+      <c r="A699" s="4" t="n"/>
+      <c r="B699" s="6" t="n"/>
+      <c r="C699" s="6" t="inlineStr">
+        <is>
+          <t>MOAI22D0COT</t>
         </is>
       </c>
     </row>
     <row r="700">
-      <c r="A700" s="4" t="n"/>
-      <c r="B700" s="6" t="inlineStr">
-        <is>
-          <t>MOAI22D1COTVIAMVM2OPU</t>
-        </is>
-      </c>
-      <c r="C700" s="6" t="n"/>
+      <c r="A700" s="7" t="n"/>
+      <c r="B700" s="8" t="n"/>
+      <c r="C700" s="8" t="inlineStr">
+        <is>
+          <t>MOAI22D1COT</t>
+        </is>
+      </c>
     </row>
     <row r="701">
-      <c r="A701" s="4" t="n"/>
-      <c r="B701" s="6" t="inlineStr">
-        <is>
-          <t>MOAI22D2COT</t>
-        </is>
-      </c>
-      <c r="C701" s="6" t="n"/>
+      <c r="A701" s="2" t="inlineStr">
+        <is>
+          <t>MUX2</t>
+        </is>
+      </c>
+      <c r="B701" s="3" t="inlineStr">
+        <is>
+          <t>MUX2D6COT</t>
+        </is>
+      </c>
+      <c r="C701" s="3" t="inlineStr">
+        <is>
+          <t>MUX2D6COT</t>
+        </is>
+      </c>
     </row>
     <row r="702">
       <c r="A702" s="4" t="n"/>
-      <c r="B702" s="6" t="n"/>
-      <c r="C702" s="6" t="inlineStr">
-        <is>
-          <t>MOAI22D0COT</t>
-        </is>
-      </c>
+      <c r="B702" s="6" t="inlineStr">
+        <is>
+          <t>MUX2D2COT</t>
+        </is>
+      </c>
+      <c r="C702" s="6" t="n"/>
     </row>
     <row r="703">
-      <c r="A703" s="7" t="n"/>
-      <c r="B703" s="8" t="n"/>
-      <c r="C703" s="8" t="inlineStr">
-        <is>
-          <t>MOAI22D1COT</t>
-        </is>
-      </c>
+      <c r="A703" s="4" t="n"/>
+      <c r="B703" s="6" t="inlineStr">
+        <is>
+          <t>MUX2D8COTM3CEQ</t>
+        </is>
+      </c>
+      <c r="C703" s="6" t="n"/>
     </row>
     <row r="704">
-      <c r="A704" s="2" t="inlineStr">
-        <is>
-          <t>MUX2</t>
-        </is>
-      </c>
-      <c r="B704" s="3" t="inlineStr">
-        <is>
-          <t>MUX2D6COT</t>
-        </is>
-      </c>
-      <c r="C704" s="3" t="inlineStr">
-        <is>
-          <t>MUX2D6COT</t>
+      <c r="A704" s="4" t="n"/>
+      <c r="B704" s="6" t="n"/>
+      <c r="C704" s="6" t="inlineStr">
+        <is>
+          <t>MUX2D1COT</t>
         </is>
       </c>
     </row>
     <row r="705">
       <c r="A705" s="4" t="n"/>
-      <c r="B705" s="6" t="inlineStr">
-        <is>
-          <t>MUX2D2COT</t>
-        </is>
-      </c>
-      <c r="C705" s="6" t="n"/>
+      <c r="B705" s="6" t="n"/>
+      <c r="C705" s="6" t="inlineStr">
+        <is>
+          <t>MUX2D2COT3FIN</t>
+        </is>
+      </c>
     </row>
     <row r="706">
-      <c r="A706" s="4" t="n"/>
-      <c r="B706" s="6" t="inlineStr">
-        <is>
-          <t>MUX2D8COTM3CEQ</t>
-        </is>
-      </c>
-      <c r="C706" s="6" t="n"/>
+      <c r="A706" s="7" t="n"/>
+      <c r="B706" s="8" t="n"/>
+      <c r="C706" s="8" t="inlineStr">
+        <is>
+          <t>MUX2D8COT</t>
+        </is>
+      </c>
     </row>
     <row r="707">
-      <c r="A707" s="4" t="n"/>
-      <c r="B707" s="6" t="n"/>
-      <c r="C707" s="6" t="inlineStr">
-        <is>
-          <t>MUX2D1COT</t>
-        </is>
-      </c>
+      <c r="A707" s="2" t="inlineStr">
+        <is>
+          <t>MUX2AOI</t>
+        </is>
+      </c>
+      <c r="B707" s="11" t="inlineStr">
+        <is>
+          <t>MUX2AOID2COTVIA</t>
+        </is>
+      </c>
+      <c r="C707" s="11" t="n"/>
     </row>
     <row r="708">
-      <c r="A708" s="4" t="n"/>
-      <c r="B708" s="6" t="n"/>
-      <c r="C708" s="6" t="inlineStr">
-        <is>
-          <t>MUX2D2COT3FIN</t>
+      <c r="A708" s="7" t="n"/>
+      <c r="B708" s="8" t="n"/>
+      <c r="C708" s="8" t="inlineStr">
+        <is>
+          <t>MUX2AOID1COTA</t>
         </is>
       </c>
     </row>
     <row r="709">
-      <c r="A709" s="7" t="n"/>
-      <c r="B709" s="8" t="n"/>
-      <c r="C709" s="8" t="inlineStr">
-        <is>
-          <t>MUX2D8COT</t>
-        </is>
-      </c>
+      <c r="A709" s="9" t="inlineStr">
+        <is>
+          <t>MUX2I</t>
+        </is>
+      </c>
+      <c r="B709" s="10" t="inlineStr">
+        <is>
+          <t>MUX2ID2COTVIAMDB</t>
+        </is>
+      </c>
+      <c r="C709" s="10" t="n"/>
     </row>
     <row r="710">
       <c r="A710" s="2" t="inlineStr">
         <is>
-          <t>MUX2AOI</t>
+          <t>MUX2ND2</t>
         </is>
       </c>
       <c r="B710" s="11" t="inlineStr">
         <is>
-          <t>MUX2AOID2COTVIA</t>
+          <t>MUX2ND2CCBD2COT</t>
         </is>
       </c>
       <c r="C710" s="11" t="n"/>
     </row>
     <row r="711">
-      <c r="A711" s="7" t="n"/>
-      <c r="B711" s="8" t="n"/>
-      <c r="C711" s="8" t="inlineStr">
-        <is>
-          <t>MUX2AOID1COTA</t>
-        </is>
-      </c>
+      <c r="A711" s="4" t="n"/>
+      <c r="B711" s="6" t="inlineStr">
+        <is>
+          <t>MUX2ND2D1COT</t>
+        </is>
+      </c>
+      <c r="C711" s="6" t="n"/>
     </row>
     <row r="712">
-      <c r="A712" s="9" t="inlineStr">
-        <is>
-          <t>MUX2I</t>
-        </is>
-      </c>
-      <c r="B712" s="10" t="inlineStr">
-        <is>
-          <t>MUX2ID2COTVIAMDB</t>
-        </is>
-      </c>
-      <c r="C712" s="10" t="n"/>
+      <c r="A712" s="4" t="n"/>
+      <c r="B712" s="6" t="inlineStr">
+        <is>
+          <t>MUX2ND2D2COT</t>
+        </is>
+      </c>
+      <c r="C712" s="6" t="n"/>
     </row>
     <row r="713">
-      <c r="A713" s="2" t="inlineStr">
-        <is>
-          <t>MUX2ND2</t>
-        </is>
-      </c>
-      <c r="B713" s="11" t="inlineStr">
-        <is>
-          <t>MUX2ND2CCBD2COT</t>
-        </is>
-      </c>
-      <c r="C713" s="11" t="n"/>
+      <c r="A713" s="7" t="n"/>
+      <c r="B713" s="8" t="n"/>
+      <c r="C713" s="8" t="inlineStr">
+        <is>
+          <t>MUX2ND2CCBD2COTA</t>
+        </is>
+      </c>
     </row>
     <row r="714">
-      <c r="A714" s="4" t="n"/>
-      <c r="B714" s="6" t="inlineStr">
-        <is>
-          <t>MUX2ND2D1COT</t>
-        </is>
-      </c>
-      <c r="C714" s="6" t="n"/>
+      <c r="A714" s="2" t="inlineStr">
+        <is>
+          <t>MUX2NND2</t>
+        </is>
+      </c>
+      <c r="B714" s="11" t="inlineStr">
+        <is>
+          <t>MUX2NND2D1COTMDB</t>
+        </is>
+      </c>
+      <c r="C714" s="11" t="n"/>
     </row>
     <row r="715">
       <c r="A715" s="4" t="n"/>
       <c r="B715" s="6" t="inlineStr">
         <is>
-          <t>MUX2ND2D2COT</t>
+          <t>MUX2NND2D2COTMDB</t>
         </is>
       </c>
       <c r="C715" s="6" t="n"/>
@@ -8487,59 +8423,59 @@
       <c r="B716" s="8" t="n"/>
       <c r="C716" s="8" t="inlineStr">
         <is>
-          <t>MUX2ND2CCBD2COTA</t>
+          <t>MUX2NND2D2COTA</t>
         </is>
       </c>
     </row>
     <row r="717">
       <c r="A717" s="2" t="inlineStr">
         <is>
-          <t>MUX2NND2</t>
+          <t>MUX2NNR2</t>
         </is>
       </c>
       <c r="B717" s="11" t="inlineStr">
         <is>
-          <t>MUX2NND2D1COTMDB</t>
+          <t>MUX2NNR2D1COTMDB</t>
         </is>
       </c>
       <c r="C717" s="11" t="n"/>
     </row>
     <row r="718">
-      <c r="A718" s="4" t="n"/>
-      <c r="B718" s="6" t="inlineStr">
-        <is>
-          <t>MUX2NND2D2COTMDB</t>
-        </is>
-      </c>
-      <c r="C718" s="6" t="n"/>
+      <c r="A718" s="7" t="n"/>
+      <c r="B718" s="8" t="inlineStr">
+        <is>
+          <t>MUX2NNR2D2COTM3CEQ</t>
+        </is>
+      </c>
+      <c r="C718" s="8" t="n"/>
     </row>
     <row r="719">
-      <c r="A719" s="7" t="n"/>
-      <c r="B719" s="8" t="n"/>
-      <c r="C719" s="8" t="inlineStr">
-        <is>
-          <t>MUX2NND2D2COTA</t>
-        </is>
-      </c>
+      <c r="A719" s="2" t="inlineStr">
+        <is>
+          <t>MUX2NR2</t>
+        </is>
+      </c>
+      <c r="B719" s="11" t="inlineStr">
+        <is>
+          <t>MUX2NR2CCBD2COTEEQ</t>
+        </is>
+      </c>
+      <c r="C719" s="11" t="n"/>
     </row>
     <row r="720">
-      <c r="A720" s="2" t="inlineStr">
-        <is>
-          <t>MUX2NNR2</t>
-        </is>
-      </c>
-      <c r="B720" s="11" t="inlineStr">
-        <is>
-          <t>MUX2NNR2D1COTMDB</t>
-        </is>
-      </c>
-      <c r="C720" s="11" t="n"/>
+      <c r="A720" s="4" t="n"/>
+      <c r="B720" s="6" t="inlineStr">
+        <is>
+          <t>MUX2NR2D1COT</t>
+        </is>
+      </c>
+      <c r="C720" s="6" t="n"/>
     </row>
     <row r="721">
       <c r="A721" s="7" t="n"/>
       <c r="B721" s="8" t="inlineStr">
         <is>
-          <t>MUX2NNR2D2COTM3CEQ</t>
+          <t>MUX2NR2D2COT</t>
         </is>
       </c>
       <c r="C721" s="8" t="n"/>
@@ -8547,145 +8483,145 @@
     <row r="722">
       <c r="A722" s="2" t="inlineStr">
         <is>
-          <t>MUX2NR2</t>
-        </is>
-      </c>
-      <c r="B722" s="11" t="inlineStr">
-        <is>
-          <t>MUX2NR2CCBD2COTEEQ</t>
-        </is>
-      </c>
-      <c r="C722" s="11" t="n"/>
+          <t>MUX3</t>
+        </is>
+      </c>
+      <c r="B722" s="3" t="inlineStr">
+        <is>
+          <t>MUX3D4COT</t>
+        </is>
+      </c>
+      <c r="C722" s="3" t="inlineStr">
+        <is>
+          <t>MUX3D4COT</t>
+        </is>
+      </c>
     </row>
     <row r="723">
       <c r="A723" s="4" t="n"/>
-      <c r="B723" s="6" t="inlineStr">
-        <is>
-          <t>MUX2NR2D1COT</t>
-        </is>
-      </c>
-      <c r="C723" s="6" t="n"/>
+      <c r="B723" s="6" t="n"/>
+      <c r="C723" s="6" t="inlineStr">
+        <is>
+          <t>MUX3D0COT</t>
+        </is>
+      </c>
     </row>
     <row r="724">
       <c r="A724" s="7" t="n"/>
-      <c r="B724" s="8" t="inlineStr">
-        <is>
-          <t>MUX2NR2D2COT</t>
-        </is>
-      </c>
-      <c r="C724" s="8" t="n"/>
+      <c r="B724" s="8" t="n"/>
+      <c r="C724" s="8" t="inlineStr">
+        <is>
+          <t>MUX3OPTLD2COT</t>
+        </is>
+      </c>
     </row>
     <row r="725">
-      <c r="A725" s="2" t="inlineStr">
-        <is>
-          <t>MUX3</t>
-        </is>
-      </c>
-      <c r="B725" s="3" t="inlineStr">
-        <is>
-          <t>MUX3D4COT</t>
-        </is>
-      </c>
-      <c r="C725" s="3" t="inlineStr">
-        <is>
-          <t>MUX3D4COT</t>
-        </is>
-      </c>
+      <c r="A725" s="9" t="inlineStr">
+        <is>
+          <t>MUX3ND1</t>
+        </is>
+      </c>
+      <c r="B725" s="10" t="inlineStr">
+        <is>
+          <t>MUX3ND1COTOPU</t>
+        </is>
+      </c>
+      <c r="C725" s="10" t="n"/>
     </row>
     <row r="726">
-      <c r="A726" s="4" t="n"/>
-      <c r="B726" s="6" t="n"/>
-      <c r="C726" s="6" t="inlineStr">
-        <is>
-          <t>MUX3D0COT</t>
-        </is>
-      </c>
+      <c r="A726" s="2" t="inlineStr">
+        <is>
+          <t>MUX4</t>
+        </is>
+      </c>
+      <c r="B726" s="11" t="inlineStr">
+        <is>
+          <t>MUX4D1COTOPUEEQ</t>
+        </is>
+      </c>
+      <c r="C726" s="11" t="n"/>
     </row>
     <row r="727">
-      <c r="A727" s="7" t="n"/>
-      <c r="B727" s="8" t="n"/>
-      <c r="C727" s="8" t="inlineStr">
-        <is>
-          <t>MUX3OPTLD2COT</t>
-        </is>
-      </c>
+      <c r="A727" s="4" t="n"/>
+      <c r="B727" s="6" t="inlineStr">
+        <is>
+          <t>MUX4OPTDD1COTOPU</t>
+        </is>
+      </c>
+      <c r="C727" s="6" t="n"/>
     </row>
     <row r="728">
-      <c r="A728" s="9" t="inlineStr">
-        <is>
-          <t>MUX3ND1</t>
-        </is>
-      </c>
-      <c r="B728" s="10" t="inlineStr">
-        <is>
-          <t>MUX3ND1COTOPU</t>
-        </is>
-      </c>
-      <c r="C728" s="10" t="n"/>
+      <c r="A728" s="7" t="n"/>
+      <c r="B728" s="8" t="n"/>
+      <c r="C728" s="8" t="inlineStr">
+        <is>
+          <t>MUX4EEQMBDD1COT</t>
+        </is>
+      </c>
     </row>
     <row r="729">
-      <c r="A729" s="2" t="inlineStr">
-        <is>
-          <t>MUX4</t>
-        </is>
-      </c>
-      <c r="B729" s="11" t="inlineStr">
-        <is>
-          <t>MUX4D1COTOPUEEQ</t>
-        </is>
-      </c>
-      <c r="C729" s="11" t="n"/>
+      <c r="A729" s="9" t="inlineStr">
+        <is>
+          <t>MUX4N</t>
+        </is>
+      </c>
+      <c r="B729" s="10" t="n"/>
+      <c r="C729" s="10" t="inlineStr">
+        <is>
+          <t>MUX4NOPTLD2COT</t>
+        </is>
+      </c>
     </row>
     <row r="730">
-      <c r="A730" s="4" t="n"/>
-      <c r="B730" s="6" t="inlineStr">
-        <is>
-          <t>MUX4OPTDD1COTOPU</t>
-        </is>
-      </c>
-      <c r="C730" s="6" t="n"/>
+      <c r="A730" s="2" t="inlineStr">
+        <is>
+          <t>MUX8</t>
+        </is>
+      </c>
+      <c r="B730" s="11" t="inlineStr">
+        <is>
+          <t>MUX8D3COT</t>
+        </is>
+      </c>
+      <c r="C730" s="11" t="n"/>
     </row>
     <row r="731">
       <c r="A731" s="7" t="n"/>
       <c r="B731" s="8" t="n"/>
       <c r="C731" s="8" t="inlineStr">
         <is>
-          <t>MUX4EEQMBDD1COT</t>
+          <t>MUX8D3COTA</t>
         </is>
       </c>
     </row>
     <row r="732">
-      <c r="A732" s="9" t="inlineStr">
-        <is>
-          <t>MUX4N</t>
-        </is>
-      </c>
-      <c r="B732" s="10" t="n"/>
-      <c r="C732" s="10" t="inlineStr">
-        <is>
-          <t>MUX4NOPTLD2COT</t>
+      <c r="A732" s="2" t="inlineStr">
+        <is>
+          <t>MX2</t>
+        </is>
+      </c>
+      <c r="B732" s="11" t="n"/>
+      <c r="C732" s="11" t="inlineStr">
+        <is>
+          <t>MX2X2ATACOTC</t>
         </is>
       </c>
     </row>
     <row r="733">
-      <c r="A733" s="2" t="inlineStr">
-        <is>
-          <t>MUX8</t>
-        </is>
-      </c>
-      <c r="B733" s="11" t="inlineStr">
-        <is>
-          <t>MUX8D3COT</t>
-        </is>
-      </c>
-      <c r="C733" s="11" t="n"/>
+      <c r="A733" s="4" t="n"/>
+      <c r="B733" s="6" t="n"/>
+      <c r="C733" s="6" t="inlineStr">
+        <is>
+          <t>MX2X2ATFCOTC</t>
+        </is>
+      </c>
     </row>
     <row r="734">
       <c r="A734" s="7" t="n"/>
       <c r="B734" s="8" t="n"/>
       <c r="C734" s="8" t="inlineStr">
         <is>
-          <t>MUX8D3COTA</t>
+          <t>MX2X8ATACOTC</t>
         </is>
       </c>
     </row>
@@ -10710,7 +10646,7 @@
     <row r="945">
       <c r="A945" s="9" t="inlineStr">
         <is>
-          <t>OAI211INVCCA</t>
+          <t>OAI211INV</t>
         </is>
       </c>
       <c r="B945" s="10" t="inlineStr">
@@ -10812,7 +10748,7 @@
       </c>
       <c r="B954" s="11" t="inlineStr">
         <is>
-          <t>OAI21ND2CCBD4COTVIA</t>
+          <t>OAI21ND2CCAD1COTVIAG</t>
         </is>
       </c>
       <c r="C954" s="11" t="n"/>
@@ -10821,7 +10757,7 @@
       <c r="A955" s="4" t="n"/>
       <c r="B955" s="6" t="inlineStr">
         <is>
-          <t>OAI21ND2D1COT</t>
+          <t>OAI21ND2CCBD4COTVIA</t>
         </is>
       </c>
       <c r="C955" s="6" t="n"/>
@@ -10830,7 +10766,7 @@
       <c r="A956" s="4" t="n"/>
       <c r="B956" s="6" t="inlineStr">
         <is>
-          <t>OAI21ND2D2COT</t>
+          <t>OAI21ND2D1COT</t>
         </is>
       </c>
       <c r="C956" s="6" t="n"/>
@@ -10839,39 +10775,35 @@
       <c r="A957" s="4" t="n"/>
       <c r="B957" s="6" t="inlineStr">
         <is>
+          <t>OAI21ND2D2COT</t>
+        </is>
+      </c>
+      <c r="C957" s="6" t="n"/>
+    </row>
+    <row r="958">
+      <c r="A958" s="4" t="n"/>
+      <c r="B958" s="6" t="inlineStr">
+        <is>
           <t>OAI21ND2D4COT</t>
         </is>
       </c>
-      <c r="C957" s="6" t="n"/>
-    </row>
-    <row r="958">
-      <c r="A958" s="7" t="n"/>
-      <c r="B958" s="8" t="n"/>
-      <c r="C958" s="8" t="inlineStr">
-        <is>
-          <t>OAI21ND2CCBD4COTA</t>
-        </is>
-      </c>
+      <c r="C958" s="6" t="n"/>
     </row>
     <row r="959">
-      <c r="A959" s="2" t="inlineStr">
-        <is>
-          <t>OAI21ND2CCA</t>
-        </is>
-      </c>
-      <c r="B959" s="11" t="inlineStr">
-        <is>
-          <t>OAI21ND2CCAD1COTVIAG</t>
-        </is>
-      </c>
-      <c r="C959" s="11" t="n"/>
+      <c r="A959" s="4" t="n"/>
+      <c r="B959" s="6" t="n"/>
+      <c r="C959" s="6" t="inlineStr">
+        <is>
+          <t>OAI21ND2CCAD1COTA</t>
+        </is>
+      </c>
     </row>
     <row r="960">
       <c r="A960" s="7" t="n"/>
       <c r="B960" s="8" t="n"/>
       <c r="C960" s="8" t="inlineStr">
         <is>
-          <t>OAI21ND2CCAD1COTA</t>
+          <t>OAI21ND2CCBD4COTA</t>
         </is>
       </c>
     </row>
@@ -10883,39 +10815,35 @@
       </c>
       <c r="B961" s="11" t="inlineStr">
         <is>
+          <t>OAI21NR2CCAD1COT</t>
+        </is>
+      </c>
+      <c r="C961" s="11" t="n"/>
+    </row>
+    <row r="962">
+      <c r="A962" s="4" t="n"/>
+      <c r="B962" s="6" t="inlineStr">
+        <is>
           <t>OAI21NR2CCBD2COT</t>
         </is>
       </c>
-      <c r="C961" s="11" t="n"/>
-    </row>
-    <row r="962">
-      <c r="A962" s="7" t="n"/>
-      <c r="B962" s="8" t="n"/>
-      <c r="C962" s="8" t="inlineStr">
-        <is>
-          <t>OAI21NR2CCBD1COTA</t>
-        </is>
-      </c>
+      <c r="C962" s="6" t="n"/>
     </row>
     <row r="963">
-      <c r="A963" s="2" t="inlineStr">
-        <is>
-          <t>OAI21NR2CCA</t>
-        </is>
-      </c>
-      <c r="B963" s="11" t="inlineStr">
-        <is>
-          <t>OAI21NR2CCAD1COT</t>
-        </is>
-      </c>
-      <c r="C963" s="11" t="n"/>
+      <c r="A963" s="4" t="n"/>
+      <c r="B963" s="6" t="n"/>
+      <c r="C963" s="6" t="inlineStr">
+        <is>
+          <t>OAI21NR2CCAD2COTA</t>
+        </is>
+      </c>
     </row>
     <row r="964">
       <c r="A964" s="7" t="n"/>
       <c r="B964" s="8" t="n"/>
       <c r="C964" s="8" t="inlineStr">
         <is>
-          <t>OAI21NR2CCAD2COTA</t>
+          <t>OAI21NR2CCBD1COTA</t>
         </is>
       </c>
     </row>
@@ -11294,46 +11222,42 @@
       </c>
       <c r="B1000" s="11" t="inlineStr">
         <is>
-          <t>OAI22AOI21CCMD1COT</t>
+          <t>OAI22AOI21CCAD2COT</t>
         </is>
       </c>
       <c r="C1000" s="11" t="n"/>
     </row>
     <row r="1001">
       <c r="A1001" s="4" t="n"/>
-      <c r="B1001" s="6" t="n"/>
-      <c r="C1001" s="6" t="inlineStr">
+      <c r="B1001" s="6" t="inlineStr">
+        <is>
+          <t>OAI22AOI21CCMD1COT</t>
+        </is>
+      </c>
+      <c r="C1001" s="6" t="n"/>
+    </row>
+    <row r="1002">
+      <c r="A1002" s="4" t="n"/>
+      <c r="B1002" s="6" t="n"/>
+      <c r="C1002" s="6" t="inlineStr">
         <is>
           <t>OAI22AOI21CCBD4COTA</t>
         </is>
       </c>
     </row>
-    <row r="1002">
-      <c r="A1002" s="7" t="n"/>
-      <c r="B1002" s="8" t="n"/>
-      <c r="C1002" s="8" t="inlineStr">
+    <row r="1003">
+      <c r="A1003" s="7" t="n"/>
+      <c r="B1003" s="8" t="n"/>
+      <c r="C1003" s="8" t="inlineStr">
         <is>
           <t>OAI22AOI21CCMD2COTA</t>
         </is>
       </c>
-    </row>
-    <row r="1003">
-      <c r="A1003" s="9" t="inlineStr">
-        <is>
-          <t>OAI22AOI21CCA</t>
-        </is>
-      </c>
-      <c r="B1003" s="10" t="inlineStr">
-        <is>
-          <t>OAI22AOI21CCAD2COT</t>
-        </is>
-      </c>
-      <c r="C1003" s="10" t="n"/>
     </row>
     <row r="1004">
       <c r="A1004" s="2" t="inlineStr">
         <is>
-          <t>OAI22INVCCA</t>
+          <t>OAI22INV</t>
         </is>
       </c>
       <c r="B1004" s="11" t="inlineStr">
@@ -14101,88 +14025,85 @@
       <c r="C1261" s="10" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="229">
+  <mergeCells count="223">
     <mergeCell ref="A540:A543"/>
     <mergeCell ref="A378:A384"/>
-    <mergeCell ref="A729:A731"/>
     <mergeCell ref="A605:A606"/>
-    <mergeCell ref="A710:A711"/>
+    <mergeCell ref="A399:A400"/>
     <mergeCell ref="A268:A269"/>
+    <mergeCell ref="A701:A706"/>
     <mergeCell ref="A1139:A1140"/>
     <mergeCell ref="A649:A650"/>
-    <mergeCell ref="A673:A676"/>
     <mergeCell ref="A335:A336"/>
+    <mergeCell ref="A690:A691"/>
     <mergeCell ref="A966:A977"/>
     <mergeCell ref="A346:A347"/>
     <mergeCell ref="A30:A37"/>
     <mergeCell ref="A586:A587"/>
-    <mergeCell ref="A1141:A1142"/>
+    <mergeCell ref="A696:A700"/>
     <mergeCell ref="A413:A414"/>
     <mergeCell ref="A582:A583"/>
+    <mergeCell ref="A1141:A1142"/>
     <mergeCell ref="A236:A237"/>
     <mergeCell ref="A792:A795"/>
-    <mergeCell ref="A713:A716"/>
     <mergeCell ref="A71:A74"/>
+    <mergeCell ref="A189:A192"/>
     <mergeCell ref="A989:A990"/>
     <mergeCell ref="A1075:A1083"/>
     <mergeCell ref="A164:A167"/>
     <mergeCell ref="A785:A789"/>
+    <mergeCell ref="A675:A676"/>
     <mergeCell ref="A1175:A1178"/>
     <mergeCell ref="A244:A247"/>
     <mergeCell ref="A103:A114"/>
     <mergeCell ref="A1021:A1025"/>
     <mergeCell ref="A1232:A1236"/>
-    <mergeCell ref="A1036:A1040"/>
+    <mergeCell ref="A730:A731"/>
     <mergeCell ref="A1011:A1015"/>
     <mergeCell ref="A790:A791"/>
     <mergeCell ref="A905:A909"/>
     <mergeCell ref="A115:A118"/>
+    <mergeCell ref="A1036:A1040"/>
     <mergeCell ref="A501:A507"/>
-    <mergeCell ref="A544:A547"/>
+    <mergeCell ref="A961:A964"/>
     <mergeCell ref="A780:A781"/>
     <mergeCell ref="A320:A321"/>
+    <mergeCell ref="A403:A404"/>
+    <mergeCell ref="A714:A716"/>
     <mergeCell ref="A1143:A1144"/>
     <mergeCell ref="A577:A579"/>
-    <mergeCell ref="A400:A401"/>
     <mergeCell ref="A584:A585"/>
     <mergeCell ref="A286:A290"/>
     <mergeCell ref="A528:A532"/>
     <mergeCell ref="A480:A481"/>
-    <mergeCell ref="A191:A192"/>
     <mergeCell ref="A256:A257"/>
     <mergeCell ref="A427:A428"/>
-    <mergeCell ref="A699:A703"/>
     <mergeCell ref="A747:A779"/>
     <mergeCell ref="A1033:A1035"/>
     <mergeCell ref="A1105:A1106"/>
-    <mergeCell ref="A661:A664"/>
     <mergeCell ref="A119:A120"/>
-    <mergeCell ref="A725:A727"/>
-    <mergeCell ref="A402:A403"/>
+    <mergeCell ref="A569:A576"/>
     <mergeCell ref="A359:A360"/>
-    <mergeCell ref="A569:A576"/>
+    <mergeCell ref="A719:A721"/>
     <mergeCell ref="A653:A654"/>
     <mergeCell ref="A2:A6"/>
-    <mergeCell ref="A687:A688"/>
     <mergeCell ref="A1026:A1029"/>
-    <mergeCell ref="A556:A566"/>
     <mergeCell ref="A339:A340"/>
-    <mergeCell ref="A300:A305"/>
     <mergeCell ref="A177:A178"/>
     <mergeCell ref="A330:A331"/>
     <mergeCell ref="A388:A389"/>
     <mergeCell ref="A351:A352"/>
-    <mergeCell ref="A680:A682"/>
     <mergeCell ref="A513:A517"/>
     <mergeCell ref="A1246:A1250"/>
     <mergeCell ref="A135:A154"/>
     <mergeCell ref="A202:A206"/>
     <mergeCell ref="A168:A171"/>
+    <mergeCell ref="A556:A568"/>
+    <mergeCell ref="A300:A307"/>
+    <mergeCell ref="A662:A666"/>
     <mergeCell ref="A1196:A1200"/>
-    <mergeCell ref="A720:A721"/>
     <mergeCell ref="A374:A375"/>
     <mergeCell ref="A405:A406"/>
-    <mergeCell ref="A641:A642"/>
     <mergeCell ref="A454:A455"/>
     <mergeCell ref="A172:A174"/>
     <mergeCell ref="A596:A599"/>
@@ -14192,19 +14113,20 @@
     <mergeCell ref="A160:A163"/>
     <mergeCell ref="A64:A70"/>
     <mergeCell ref="A622:A623"/>
-    <mergeCell ref="A704:A709"/>
     <mergeCell ref="A121:A122"/>
     <mergeCell ref="A357:A358"/>
+    <mergeCell ref="A681:A682"/>
     <mergeCell ref="A1092:A1095"/>
     <mergeCell ref="A848:A849"/>
     <mergeCell ref="A344:A345"/>
     <mergeCell ref="A615:A616"/>
-    <mergeCell ref="A961:A962"/>
     <mergeCell ref="A947:A949"/>
-    <mergeCell ref="A658:A660"/>
     <mergeCell ref="A407:A408"/>
+    <mergeCell ref="A667:A669"/>
+    <mergeCell ref="A631:A636"/>
     <mergeCell ref="A337:A338"/>
     <mergeCell ref="A608:A609"/>
+    <mergeCell ref="A692:A693"/>
     <mergeCell ref="A126:A128"/>
     <mergeCell ref="A534:A539"/>
     <mergeCell ref="A1125:A1130"/>
@@ -14216,7 +14138,6 @@
     <mergeCell ref="A1201:A1217"/>
     <mergeCell ref="A473:A474"/>
     <mergeCell ref="A796:A797"/>
-    <mergeCell ref="A678:A679"/>
     <mergeCell ref="A1151:A1152"/>
     <mergeCell ref="A85:A102"/>
     <mergeCell ref="A551:A554"/>
@@ -14224,7 +14145,6 @@
     <mergeCell ref="A799:A801"/>
     <mergeCell ref="A264:A265"/>
     <mergeCell ref="A326:A327"/>
-    <mergeCell ref="A733:A734"/>
     <mergeCell ref="A1154:A1171"/>
     <mergeCell ref="A425:A426"/>
     <mergeCell ref="A860:A862"/>
@@ -14232,12 +14152,12 @@
     <mergeCell ref="A850:A859"/>
     <mergeCell ref="A376:A377"/>
     <mergeCell ref="A735:A746"/>
-    <mergeCell ref="A1000:A1002"/>
+    <mergeCell ref="A717:A718"/>
     <mergeCell ref="A368:A370"/>
-    <mergeCell ref="A670:A671"/>
-    <mergeCell ref="A695:A696"/>
+    <mergeCell ref="A643:A648"/>
     <mergeCell ref="A38:A48"/>
     <mergeCell ref="A497:A500"/>
+    <mergeCell ref="A726:A728"/>
     <mergeCell ref="A1016:A1020"/>
     <mergeCell ref="A409:A410"/>
     <mergeCell ref="A207:A209"/>
@@ -14246,10 +14166,10 @@
     <mergeCell ref="A1118:A1122"/>
     <mergeCell ref="A1224:A1227"/>
     <mergeCell ref="A898:A904"/>
-    <mergeCell ref="A646:A647"/>
     <mergeCell ref="A991:A999"/>
     <mergeCell ref="A179:A184"/>
     <mergeCell ref="A411:A412"/>
+    <mergeCell ref="A670:A673"/>
     <mergeCell ref="A651:A652"/>
     <mergeCell ref="A1004:A1005"/>
     <mergeCell ref="A1228:A1230"/>
@@ -14260,56 +14180,52 @@
     <mergeCell ref="A523:A527"/>
     <mergeCell ref="A391:A392"/>
     <mergeCell ref="A1100:A1101"/>
-    <mergeCell ref="A631:A634"/>
+    <mergeCell ref="A637:A642"/>
+    <mergeCell ref="A954:A960"/>
     <mergeCell ref="A978:A982"/>
+    <mergeCell ref="A707:A708"/>
     <mergeCell ref="A1219:A1223"/>
     <mergeCell ref="A985:A988"/>
     <mergeCell ref="A446:A447"/>
     <mergeCell ref="A617:A618"/>
-    <mergeCell ref="A954:A958"/>
     <mergeCell ref="A271:A277"/>
     <mergeCell ref="A1191:A1195"/>
-    <mergeCell ref="A567:A568"/>
     <mergeCell ref="A448:A449"/>
     <mergeCell ref="A210:A214"/>
     <mergeCell ref="A1135:A1136"/>
     <mergeCell ref="A876:A886"/>
     <mergeCell ref="A291:A294"/>
-    <mergeCell ref="A643:A644"/>
-    <mergeCell ref="A963:A964"/>
-    <mergeCell ref="A665:A669"/>
     <mergeCell ref="A432:A434"/>
     <mergeCell ref="A124:A125"/>
     <mergeCell ref="A1172:A1174"/>
     <mergeCell ref="A1006:A1007"/>
-    <mergeCell ref="A133:A134"/>
-    <mergeCell ref="A189:A190"/>
+    <mergeCell ref="A250:A255"/>
     <mergeCell ref="A57:A63"/>
-    <mergeCell ref="A250:A255"/>
-    <mergeCell ref="A959:A960"/>
     <mergeCell ref="A1041:A1067"/>
     <mergeCell ref="A943:A944"/>
     <mergeCell ref="A911:A928"/>
+    <mergeCell ref="A732:A734"/>
     <mergeCell ref="A261:A263"/>
     <mergeCell ref="A1030:A1032"/>
     <mergeCell ref="A950:A953"/>
     <mergeCell ref="A155:A159"/>
     <mergeCell ref="A308:A314"/>
-    <mergeCell ref="A1111:A1112"/>
+    <mergeCell ref="A658:A661"/>
     <mergeCell ref="A198:A201"/>
     <mergeCell ref="A722:A724"/>
-    <mergeCell ref="A1182:A1183"/>
+    <mergeCell ref="A544:A550"/>
     <mergeCell ref="A782:A784"/>
     <mergeCell ref="A518:A522"/>
-    <mergeCell ref="A1096:A1099"/>
+    <mergeCell ref="A132:A134"/>
+    <mergeCell ref="A1111:A1112"/>
+    <mergeCell ref="A1182:A1183"/>
+    <mergeCell ref="A401:A402"/>
     <mergeCell ref="A863:A875"/>
     <mergeCell ref="A684:A685"/>
+    <mergeCell ref="A1096:A1099"/>
+    <mergeCell ref="A1008:A1009"/>
     <mergeCell ref="A1185:A1188"/>
-    <mergeCell ref="A1008:A1009"/>
-    <mergeCell ref="A637:A638"/>
-    <mergeCell ref="A693:A694"/>
     <mergeCell ref="A7:A29"/>
-    <mergeCell ref="A548:A550"/>
     <mergeCell ref="A1113:A1114"/>
     <mergeCell ref="A929:A942"/>
     <mergeCell ref="A450:A451"/>
@@ -14317,17 +14233,19 @@
     <mergeCell ref="A589:A595"/>
     <mergeCell ref="A1103:A1104"/>
     <mergeCell ref="A215:A216"/>
+    <mergeCell ref="A677:A679"/>
     <mergeCell ref="A624:A626"/>
     <mergeCell ref="A75:A77"/>
     <mergeCell ref="A193:A197"/>
-    <mergeCell ref="A717:A719"/>
     <mergeCell ref="A892:A897"/>
+    <mergeCell ref="A1000:A1003"/>
     <mergeCell ref="A627:A628"/>
     <mergeCell ref="A78:A84"/>
     <mergeCell ref="A452:A453"/>
     <mergeCell ref="A50:A56"/>
     <mergeCell ref="A266:A267"/>
     <mergeCell ref="A129:A131"/>
+    <mergeCell ref="A710:A713"/>
     <mergeCell ref="A655:A657"/>
     <mergeCell ref="A279:A284"/>
     <mergeCell ref="A629:A630"/>

</xml_diff>

<commit_message>
Peel leftover layout suffixes from suggested function keys.
Strip HD/V2/IW/AAR/VPPVBB tails so CMPE42X1AAR, ISOCHSRCIW, HAC1V2,
TAPCELLVPPVBB, *HD and AP*HD collapse to clean roots (keep BHD).
Regenerate keys: 435 -> 431 with full coverage.

Co-authored-by: EsaLongs <EsaLongs@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/preview/NP1PP_vs_C1Y_preview.xlsx
+++ b/preview/NP1PP_vs_C1Y_preview.xlsx
@@ -2660,7 +2660,7 @@
     <row r="215">
       <c r="A215" s="2" t="inlineStr">
         <is>
-          <t>APBUFHD</t>
+          <t>APBUF</t>
         </is>
       </c>
       <c r="B215" s="11" t="inlineStr">
@@ -2682,7 +2682,7 @@
     <row r="217">
       <c r="A217" s="9" t="inlineStr">
         <is>
-          <t>APINVHD</t>
+          <t>APINV</t>
         </is>
       </c>
       <c r="B217" s="10" t="inlineStr">
@@ -3825,22 +3825,18 @@
       </c>
     </row>
     <row r="314">
-      <c r="A314" s="7" t="n"/>
-      <c r="B314" s="8" t="n"/>
-      <c r="C314" s="8" t="inlineStr">
+      <c r="A314" s="4" t="n"/>
+      <c r="B314" s="6" t="n"/>
+      <c r="C314" s="6" t="inlineStr">
         <is>
           <t>CMPE42EEQMBDD4COT</t>
         </is>
       </c>
     </row>
     <row r="315">
-      <c r="A315" s="9" t="inlineStr">
-        <is>
-          <t>CMPE42X1AAR</t>
-        </is>
-      </c>
-      <c r="B315" s="10" t="n"/>
-      <c r="C315" s="10" t="inlineStr">
+      <c r="A315" s="7" t="n"/>
+      <c r="B315" s="8" t="n"/>
+      <c r="C315" s="8" t="inlineStr">
         <is>
           <t>CMPE42X1AARCOTC</t>
         </is>
@@ -6170,22 +6166,18 @@
       </c>
     </row>
     <row r="507">
-      <c r="A507" s="7" t="n"/>
-      <c r="B507" s="8" t="n"/>
-      <c r="C507" s="8" t="inlineStr">
+      <c r="A507" s="4" t="n"/>
+      <c r="B507" s="6" t="n"/>
+      <c r="C507" s="6" t="inlineStr">
         <is>
           <t>HAC1D4ALPCOT</t>
         </is>
       </c>
     </row>
     <row r="508">
-      <c r="A508" s="9" t="inlineStr">
-        <is>
-          <t>HAC1V2</t>
-        </is>
-      </c>
-      <c r="B508" s="10" t="n"/>
-      <c r="C508" s="10" t="inlineStr">
+      <c r="A508" s="7" t="n"/>
+      <c r="B508" s="8" t="n"/>
+      <c r="C508" s="8" t="inlineStr">
         <is>
           <t>HAC1V2D4ALPCOT</t>
         </is>
@@ -7225,22 +7217,18 @@
       <c r="C605" s="11" t="n"/>
     </row>
     <row r="606">
-      <c r="A606" s="7" t="n"/>
-      <c r="B606" s="8" t="inlineStr">
+      <c r="A606" s="4" t="n"/>
+      <c r="B606" s="6" t="inlineStr">
         <is>
           <t>ISOCHSRCD4COT</t>
         </is>
       </c>
-      <c r="C606" s="8" t="n"/>
+      <c r="C606" s="6" t="n"/>
     </row>
     <row r="607">
-      <c r="A607" s="9" t="inlineStr">
-        <is>
-          <t>ISOCHSRCIW</t>
-        </is>
-      </c>
-      <c r="B607" s="10" t="n"/>
-      <c r="C607" s="10" t="inlineStr">
+      <c r="A607" s="7" t="n"/>
+      <c r="B607" s="8" t="n"/>
+      <c r="C607" s="8" t="inlineStr">
         <is>
           <t>ISOCHSRCIWD2COT</t>
         </is>
@@ -12085,7 +12073,7 @@
     <row r="1084">
       <c r="A1084" s="9" t="inlineStr">
         <is>
-          <t>RSDFQHD</t>
+          <t>RSDFQ</t>
         </is>
       </c>
       <c r="B1084" s="10" t="n"/>
@@ -12098,7 +12086,7 @@
     <row r="1085">
       <c r="A1085" s="9" t="inlineStr">
         <is>
-          <t>RSDFRPQHD</t>
+          <t>RSDFRPQ</t>
         </is>
       </c>
       <c r="B1085" s="10" t="n"/>
@@ -12111,7 +12099,7 @@
     <row r="1086">
       <c r="A1086" s="9" t="inlineStr">
         <is>
-          <t>RSDFSNQHD</t>
+          <t>RSDFSNQ</t>
         </is>
       </c>
       <c r="B1086" s="10" t="n"/>
@@ -12124,7 +12112,7 @@
     <row r="1087">
       <c r="A1087" s="9" t="inlineStr">
         <is>
-          <t>RSDFSRPQHD</t>
+          <t>RSDFSRPQ</t>
         </is>
       </c>
       <c r="B1087" s="10" t="n"/>
@@ -12806,30 +12794,26 @@
       <c r="C1146" s="10" t="n"/>
     </row>
     <row r="1147">
-      <c r="A1147" s="9" t="inlineStr">
+      <c r="A1147" s="2" t="inlineStr">
         <is>
           <t>TAPCELL</t>
         </is>
       </c>
-      <c r="B1147" s="12" t="inlineStr">
+      <c r="B1147" s="3" t="inlineStr">
         <is>
           <t>TAPCELLCOT</t>
         </is>
       </c>
-      <c r="C1147" s="12" t="inlineStr">
+      <c r="C1147" s="3" t="inlineStr">
         <is>
           <t>TAPCELLCOT</t>
         </is>
       </c>
     </row>
     <row r="1148">
-      <c r="A1148" s="9" t="inlineStr">
-        <is>
-          <t>TAPCELLVPPVBB</t>
-        </is>
-      </c>
-      <c r="B1148" s="10" t="n"/>
-      <c r="C1148" s="10" t="inlineStr">
+      <c r="A1148" s="7" t="n"/>
+      <c r="B1148" s="8" t="n"/>
+      <c r="C1148" s="8" t="inlineStr">
         <is>
           <t>TAPCELLVPPVBBCOT</t>
         </is>
@@ -14025,10 +14009,9 @@
       <c r="C1261" s="10" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="223">
+  <mergeCells count="224">
     <mergeCell ref="A540:A543"/>
     <mergeCell ref="A378:A384"/>
-    <mergeCell ref="A605:A606"/>
     <mergeCell ref="A399:A400"/>
     <mergeCell ref="A268:A269"/>
     <mergeCell ref="A701:A706"/>
@@ -14064,7 +14047,6 @@
     <mergeCell ref="A905:A909"/>
     <mergeCell ref="A115:A118"/>
     <mergeCell ref="A1036:A1040"/>
-    <mergeCell ref="A501:A507"/>
     <mergeCell ref="A961:A964"/>
     <mergeCell ref="A780:A781"/>
     <mergeCell ref="A320:A321"/>
@@ -14144,6 +14126,7 @@
     <mergeCell ref="A457:A458"/>
     <mergeCell ref="A799:A801"/>
     <mergeCell ref="A264:A265"/>
+    <mergeCell ref="A1147:A1148"/>
     <mergeCell ref="A326:A327"/>
     <mergeCell ref="A1154:A1171"/>
     <mergeCell ref="A425:A426"/>
@@ -14165,6 +14148,7 @@
     <mergeCell ref="A483:A484"/>
     <mergeCell ref="A1118:A1122"/>
     <mergeCell ref="A1224:A1227"/>
+    <mergeCell ref="A605:A607"/>
     <mergeCell ref="A898:A904"/>
     <mergeCell ref="A991:A999"/>
     <mergeCell ref="A179:A184"/>
@@ -14209,7 +14193,7 @@
     <mergeCell ref="A1030:A1032"/>
     <mergeCell ref="A950:A953"/>
     <mergeCell ref="A155:A159"/>
-    <mergeCell ref="A308:A314"/>
+    <mergeCell ref="A501:A508"/>
     <mergeCell ref="A658:A661"/>
     <mergeCell ref="A198:A201"/>
     <mergeCell ref="A722:A724"/>
@@ -14248,6 +14232,7 @@
     <mergeCell ref="A710:A713"/>
     <mergeCell ref="A655:A657"/>
     <mergeCell ref="A279:A284"/>
+    <mergeCell ref="A308:A315"/>
     <mergeCell ref="A629:A630"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add Chinese function briefs to merged column-A cells.
Each grouped key now displays as KEY plus a short Chinese label
(e.g. AN2/与门, ND2/与非门, SDFQ/扫描触发器) with wrap-enabled merges.

Co-authored-by: EsaLongs <EsaLongs@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/preview/NP1PP_vs_C1Y_preview.xlsx
+++ b/preview/NP1PP_vs_C1Y_preview.xlsx
@@ -466,7 +466,7 @@
   <dimension ref="A1:C1261"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
     <col width="55" customWidth="1" min="2" max="2"/>
     <col width="55" customWidth="1" min="3" max="3"/>
   </cols>
@@ -487,7 +487,8 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>AIOI21</t>
+          <t>AIOI21
+复合逻辑门</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -544,7 +545,8 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>AN2</t>
+          <t>AN2
+与门</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -767,7 +769,8 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>AN3</t>
+          <t>AN3
+与门</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
@@ -859,7 +862,8 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>AN4</t>
+          <t>AN4
+与门</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
@@ -970,7 +974,8 @@
     <row r="49">
       <c r="A49" s="9" t="inlineStr">
         <is>
-          <t>ANTENNA</t>
+          <t>ANTENNA
+天线二极管</t>
         </is>
       </c>
       <c r="B49" s="10" t="inlineStr">
@@ -983,7 +988,8 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>AO21</t>
+          <t>AO21
+与或门</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
@@ -1058,7 +1064,8 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>AO211</t>
+          <t>AO211
+与或门</t>
         </is>
       </c>
       <c r="B57" s="11" t="inlineStr">
@@ -1125,7 +1132,8 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>AO22</t>
+          <t>AO22
+与或门</t>
         </is>
       </c>
       <c r="B64" s="3" t="inlineStr">
@@ -1196,7 +1204,8 @@
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>AO222</t>
+          <t>AO222
+与或门</t>
         </is>
       </c>
       <c r="B71" s="11" t="inlineStr">
@@ -1236,7 +1245,8 @@
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>AO33</t>
+          <t>AO33
+与或门</t>
         </is>
       </c>
       <c r="B75" s="11" t="inlineStr">
@@ -1267,7 +1277,8 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>AOAI211</t>
+          <t>AOAI211
+复合逻辑门</t>
         </is>
       </c>
       <c r="B78" s="3" t="inlineStr">
@@ -1346,7 +1357,8 @@
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>AOI21</t>
+          <t>AOI21
+与或非门</t>
         </is>
       </c>
       <c r="B85" s="11" t="inlineStr">
@@ -1512,7 +1524,8 @@
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>AOI211</t>
+          <t>AOI211
+与或非门</t>
         </is>
       </c>
       <c r="B103" s="3" t="inlineStr">
@@ -1632,7 +1645,8 @@
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
         <is>
-          <t>AOI2111</t>
+          <t>AOI2111
+与或非门</t>
         </is>
       </c>
       <c r="B115" s="11" t="inlineStr">
@@ -1672,7 +1686,8 @@
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
         <is>
-          <t>AOI211INV</t>
+          <t>AOI211INV
+复合逻辑门</t>
         </is>
       </c>
       <c r="B119" s="11" t="inlineStr">
@@ -1694,7 +1709,8 @@
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
         <is>
-          <t>AOI21AOI21</t>
+          <t>AOI21AOI21
+复合逻辑门</t>
         </is>
       </c>
       <c r="B121" s="11" t="inlineStr">
@@ -1716,7 +1732,8 @@
     <row r="123">
       <c r="A123" s="9" t="inlineStr">
         <is>
-          <t>AOI21B1</t>
+          <t>AOI21B1
+与或非门</t>
         </is>
       </c>
       <c r="B123" s="10" t="n"/>
@@ -1729,7 +1746,8 @@
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>AOI21N2</t>
+          <t>AOI21N2
+与或非门</t>
         </is>
       </c>
       <c r="B124" s="11" t="n"/>
@@ -1751,7 +1769,8 @@
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>AOI21ND2</t>
+          <t>AOI21ND2
+与或非门</t>
         </is>
       </c>
       <c r="B126" s="11" t="inlineStr">
@@ -1782,7 +1801,8 @@
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
         <is>
-          <t>AOI21NR2</t>
+          <t>AOI21NR2
+与或非门</t>
         </is>
       </c>
       <c r="B129" s="11" t="inlineStr">
@@ -1813,7 +1833,8 @@
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
         <is>
-          <t>AOI21OAI21</t>
+          <t>AOI21OAI21
+复合逻辑门</t>
         </is>
       </c>
       <c r="B132" s="11" t="inlineStr">
@@ -1844,7 +1865,8 @@
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
         <is>
-          <t>AOI22</t>
+          <t>AOI22
+与或非门</t>
         </is>
       </c>
       <c r="B135" s="11" t="inlineStr">
@@ -2028,7 +2050,8 @@
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
         <is>
-          <t>AOI221</t>
+          <t>AOI221
+与或非门</t>
         </is>
       </c>
       <c r="B155" s="3" t="inlineStr">
@@ -2081,7 +2104,8 @@
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
         <is>
-          <t>AOI2211</t>
+          <t>AOI2211
+与或非门</t>
         </is>
       </c>
       <c r="B160" s="11" t="inlineStr">
@@ -2121,7 +2145,8 @@
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
         <is>
-          <t>AOI222</t>
+          <t>AOI222
+与或非门</t>
         </is>
       </c>
       <c r="B164" s="3" t="inlineStr">
@@ -2169,7 +2194,8 @@
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
         <is>
-          <t>AOI2221</t>
+          <t>AOI2221
+与或非门</t>
         </is>
       </c>
       <c r="B168" s="11" t="inlineStr">
@@ -2209,7 +2235,8 @@
     <row r="172">
       <c r="A172" s="2" t="inlineStr">
         <is>
-          <t>AOI2222</t>
+          <t>AOI2222
+与或非门</t>
         </is>
       </c>
       <c r="B172" s="11" t="inlineStr">
@@ -2240,7 +2267,8 @@
     <row r="175">
       <c r="A175" s="9" t="inlineStr">
         <is>
-          <t>AOI22AOI21</t>
+          <t>AOI22AOI21
+复合逻辑门</t>
         </is>
       </c>
       <c r="B175" s="10" t="inlineStr">
@@ -2253,7 +2281,8 @@
     <row r="176">
       <c r="A176" s="9" t="inlineStr">
         <is>
-          <t>AOI22AOI22</t>
+          <t>AOI22AOI22
+复合逻辑门</t>
         </is>
       </c>
       <c r="B176" s="10" t="inlineStr">
@@ -2266,7 +2295,8 @@
     <row r="177">
       <c r="A177" s="2" t="inlineStr">
         <is>
-          <t>AOI22INV</t>
+          <t>AOI22INV
+复合逻辑门</t>
         </is>
       </c>
       <c r="B177" s="11" t="inlineStr">
@@ -2288,7 +2318,8 @@
     <row r="179">
       <c r="A179" s="2" t="inlineStr">
         <is>
-          <t>AOI22ND2</t>
+          <t>AOI22ND2
+与或非门</t>
         </is>
       </c>
       <c r="B179" s="11" t="inlineStr">
@@ -2346,7 +2377,8 @@
     <row r="185">
       <c r="A185" s="2" t="inlineStr">
         <is>
-          <t>AOI22NR2</t>
+          <t>AOI22NR2
+与或非门</t>
         </is>
       </c>
       <c r="B185" s="11" t="inlineStr">
@@ -2386,7 +2418,8 @@
     <row r="189">
       <c r="A189" s="2" t="inlineStr">
         <is>
-          <t>AOI22OAI21</t>
+          <t>AOI22OAI21
+复合逻辑门</t>
         </is>
       </c>
       <c r="B189" s="11" t="inlineStr">
@@ -2426,7 +2459,8 @@
     <row r="193">
       <c r="A193" s="2" t="inlineStr">
         <is>
-          <t>AOI31</t>
+          <t>AOI31
+与或非门</t>
         </is>
       </c>
       <c r="B193" s="11" t="inlineStr">
@@ -2475,7 +2509,8 @@
     <row r="198">
       <c r="A198" s="2" t="inlineStr">
         <is>
-          <t>AOI311</t>
+          <t>AOI311
+与或非门</t>
         </is>
       </c>
       <c r="B198" s="3" t="inlineStr">
@@ -2519,7 +2554,8 @@
     <row r="202">
       <c r="A202" s="2" t="inlineStr">
         <is>
-          <t>AOI32</t>
+          <t>AOI32
+与或非门</t>
         </is>
       </c>
       <c r="B202" s="3" t="inlineStr">
@@ -2572,7 +2608,8 @@
     <row r="207">
       <c r="A207" s="2" t="inlineStr">
         <is>
-          <t>AOI321</t>
+          <t>AOI321
+与或非门</t>
         </is>
       </c>
       <c r="B207" s="11" t="inlineStr">
@@ -2603,7 +2640,8 @@
     <row r="210">
       <c r="A210" s="2" t="inlineStr">
         <is>
-          <t>AOI33</t>
+          <t>AOI33
+与或非门</t>
         </is>
       </c>
       <c r="B210" s="3" t="inlineStr">
@@ -2660,7 +2698,8 @@
     <row r="215">
       <c r="A215" s="2" t="inlineStr">
         <is>
-          <t>APBUF</t>
+          <t>APBUF
+缓冲器</t>
         </is>
       </c>
       <c r="B215" s="11" t="inlineStr">
@@ -2682,7 +2721,8 @@
     <row r="217">
       <c r="A217" s="9" t="inlineStr">
         <is>
-          <t>APINV</t>
+          <t>APINV
+反相器</t>
         </is>
       </c>
       <c r="B217" s="10" t="inlineStr">
@@ -2695,7 +2735,8 @@
     <row r="218">
       <c r="A218" s="9" t="inlineStr">
         <is>
-          <t>APTIEH</t>
+          <t>APTIEH
+电平钳位</t>
         </is>
       </c>
       <c r="B218" s="12" t="inlineStr">
@@ -2712,7 +2753,8 @@
     <row r="219">
       <c r="A219" s="9" t="inlineStr">
         <is>
-          <t>APTIEL</t>
+          <t>APTIEL
+电平钳位</t>
         </is>
       </c>
       <c r="B219" s="10" t="inlineStr">
@@ -2725,7 +2767,8 @@
     <row r="220">
       <c r="A220" s="9" t="inlineStr">
         <is>
-          <t>BENCGRF</t>
+          <t>BENCGRF
+编码器</t>
         </is>
       </c>
       <c r="B220" s="10" t="n"/>
@@ -2738,7 +2781,8 @@
     <row r="221">
       <c r="A221" s="9" t="inlineStr">
         <is>
-          <t>BHD</t>
+          <t>BHD
+总线保持器</t>
         </is>
       </c>
       <c r="B221" s="12" t="inlineStr">
@@ -2755,7 +2799,8 @@
     <row r="222">
       <c r="A222" s="9" t="inlineStr">
         <is>
-          <t>BOUNDARYCNREXRN</t>
+          <t>BOUNDARYCNREXRN
+边界/版图单元</t>
         </is>
       </c>
       <c r="B222" s="12" t="inlineStr">
@@ -2772,7 +2817,8 @@
     <row r="223">
       <c r="A223" s="9" t="inlineStr">
         <is>
-          <t>BOUNDARYCNREXRN6</t>
+          <t>BOUNDARYCNREXRN6
+边界/版图单元</t>
         </is>
       </c>
       <c r="B223" s="10" t="n"/>
@@ -2785,7 +2831,8 @@
     <row r="224">
       <c r="A224" s="9" t="inlineStr">
         <is>
-          <t>BOUNDARYCNREXRP</t>
+          <t>BOUNDARYCNREXRP
+边界/版图单元</t>
         </is>
       </c>
       <c r="B224" s="12" t="inlineStr">
@@ -2802,7 +2849,8 @@
     <row r="225">
       <c r="A225" s="9" t="inlineStr">
         <is>
-          <t>BOUNDARYCNRINRN6</t>
+          <t>BOUNDARYCNRINRN6
+边界/版图单元</t>
         </is>
       </c>
       <c r="B225" s="10" t="n"/>
@@ -2815,7 +2863,8 @@
     <row r="226">
       <c r="A226" s="9" t="inlineStr">
         <is>
-          <t>BOUNDARYCNRINRP6</t>
+          <t>BOUNDARYCNRINRP6
+边界/版图单元</t>
         </is>
       </c>
       <c r="B226" s="10" t="n"/>
@@ -2828,7 +2877,8 @@
     <row r="227">
       <c r="A227" s="9" t="inlineStr">
         <is>
-          <t>BOUNDARYCOLN1</t>
+          <t>BOUNDARYCOLN1
+边界/版图单元</t>
         </is>
       </c>
       <c r="B227" s="12" t="inlineStr">
@@ -2845,7 +2895,8 @@
     <row r="228">
       <c r="A228" s="9" t="inlineStr">
         <is>
-          <t>BOUNDARYCOLN2</t>
+          <t>BOUNDARYCOLN2
+边界/版图单元</t>
         </is>
       </c>
       <c r="B228" s="12" t="inlineStr">
@@ -2862,7 +2913,8 @@
     <row r="229">
       <c r="A229" s="9" t="inlineStr">
         <is>
-          <t>BOUNDARYCOLN3</t>
+          <t>BOUNDARYCOLN3
+边界/版图单元</t>
         </is>
       </c>
       <c r="B229" s="10" t="n"/>
@@ -2875,7 +2927,8 @@
     <row r="230">
       <c r="A230" s="9" t="inlineStr">
         <is>
-          <t>BOUNDARYCOLNGAP</t>
+          <t>BOUNDARYCOLNGAP
+边界/版图单元</t>
         </is>
       </c>
       <c r="B230" s="10" t="inlineStr">
@@ -2888,7 +2941,8 @@
     <row r="231">
       <c r="A231" s="9" t="inlineStr">
         <is>
-          <t>BOUNDARYCOLP1</t>
+          <t>BOUNDARYCOLP1
+边界/版图单元</t>
         </is>
       </c>
       <c r="B231" s="12" t="inlineStr">
@@ -2905,7 +2959,8 @@
     <row r="232">
       <c r="A232" s="9" t="inlineStr">
         <is>
-          <t>BOUNDARYCOLP2</t>
+          <t>BOUNDARYCOLP2
+边界/版图单元</t>
         </is>
       </c>
       <c r="B232" s="10" t="inlineStr">
@@ -2918,7 +2973,8 @@
     <row r="233">
       <c r="A233" s="9" t="inlineStr">
         <is>
-          <t>BOUNDARYCOLP3</t>
+          <t>BOUNDARYCOLP3
+边界/版图单元</t>
         </is>
       </c>
       <c r="B233" s="10" t="n"/>
@@ -2931,7 +2987,8 @@
     <row r="234">
       <c r="A234" s="9" t="inlineStr">
         <is>
-          <t>BOUNDARYCOLPGAP</t>
+          <t>BOUNDARYCOLPGAP
+边界/版图单元</t>
         </is>
       </c>
       <c r="B234" s="12" t="inlineStr">
@@ -2948,7 +3005,8 @@
     <row r="235">
       <c r="A235" s="9" t="inlineStr">
         <is>
-          <t>BOUNDARYICNREXRN6</t>
+          <t>BOUNDARYICNREXRN6
+边界/版图单元</t>
         </is>
       </c>
       <c r="B235" s="12" t="inlineStr">
@@ -2965,7 +3023,8 @@
     <row r="236">
       <c r="A236" s="2" t="inlineStr">
         <is>
-          <t>BOUNDARYICNREXRP6</t>
+          <t>BOUNDARYICNREXRP6
+边界/版图单元</t>
         </is>
       </c>
       <c r="B236" s="3" t="inlineStr">
@@ -2991,7 +3050,8 @@
     <row r="238">
       <c r="A238" s="9" t="inlineStr">
         <is>
-          <t>BOUNDARYROW6</t>
+          <t>BOUNDARYROW6
+边界/版图单元</t>
         </is>
       </c>
       <c r="B238" s="10" t="inlineStr">
@@ -3004,7 +3064,8 @@
     <row r="239">
       <c r="A239" s="9" t="inlineStr">
         <is>
-          <t>BOUNDARYROW7</t>
+          <t>BOUNDARYROW7
+边界/版图单元</t>
         </is>
       </c>
       <c r="B239" s="10" t="inlineStr">
@@ -3017,7 +3078,8 @@
     <row r="240">
       <c r="A240" s="9" t="inlineStr">
         <is>
-          <t>BOUNDARY_HD1A20</t>
+          <t>BOUNDARY_HD1A20
+边界/版图单元</t>
         </is>
       </c>
       <c r="B240" s="10" t="n"/>
@@ -3030,7 +3092,8 @@
     <row r="241">
       <c r="A241" s="9" t="inlineStr">
         <is>
-          <t>BOUNDARY_HD2A30F</t>
+          <t>BOUNDARY_HD2A30F
+边界/版图单元</t>
         </is>
       </c>
       <c r="B241" s="10" t="n"/>
@@ -3043,7 +3106,8 @@
     <row r="242">
       <c r="A242" s="9" t="inlineStr">
         <is>
-          <t>BOUNDARY_HDDID1A40</t>
+          <t>BOUNDARY_HDDID1A40
+边界/版图单元</t>
         </is>
       </c>
       <c r="B242" s="10" t="inlineStr">
@@ -3056,7 +3120,8 @@
     <row r="243">
       <c r="A243" s="9" t="inlineStr">
         <is>
-          <t>BOUNDARY_HDDID2A30</t>
+          <t>BOUNDARY_HDDID2A30
+边界/版图单元</t>
         </is>
       </c>
       <c r="B243" s="10" t="inlineStr">
@@ -3069,7 +3134,8 @@
     <row r="244">
       <c r="A244" s="2" t="inlineStr">
         <is>
-          <t>BUF</t>
+          <t>BUF
+缓冲器</t>
         </is>
       </c>
       <c r="B244" s="11" t="n"/>
@@ -3109,7 +3175,8 @@
     <row r="248">
       <c r="A248" s="9" t="inlineStr">
         <is>
-          <t>BUFF</t>
+          <t>BUFF
+缓冲器</t>
         </is>
       </c>
       <c r="B248" s="10" t="inlineStr">
@@ -3122,7 +3189,8 @@
     <row r="249">
       <c r="A249" s="9" t="inlineStr">
         <is>
-          <t>BUFT</t>
+          <t>BUFT
+三态缓冲器</t>
         </is>
       </c>
       <c r="B249" s="10" t="inlineStr">
@@ -3135,7 +3203,8 @@
     <row r="250">
       <c r="A250" s="2" t="inlineStr">
         <is>
-          <t>CKAN2</t>
+          <t>CKAN2
+时钟与门</t>
         </is>
       </c>
       <c r="B250" s="3" t="inlineStr">
@@ -3201,7 +3270,8 @@
     <row r="256">
       <c r="A256" s="2" t="inlineStr">
         <is>
-          <t>CKB</t>
+          <t>CKB
+时钟缓冲/反相</t>
         </is>
       </c>
       <c r="B256" s="11" t="inlineStr">
@@ -3223,7 +3293,8 @@
     <row r="258">
       <c r="A258" s="2" t="inlineStr">
         <is>
-          <t>CKLHQ</t>
+          <t>CKLHQ
+时钟锁存器</t>
         </is>
       </c>
       <c r="B258" s="11" t="inlineStr">
@@ -3245,7 +3316,8 @@
     <row r="260">
       <c r="A260" s="9" t="inlineStr">
         <is>
-          <t>CKLNCNQ</t>
+          <t>CKLNCNQ
+时钟锁存器</t>
         </is>
       </c>
       <c r="B260" s="10" t="inlineStr">
@@ -3258,7 +3330,8 @@
     <row r="261">
       <c r="A261" s="2" t="inlineStr">
         <is>
-          <t>CKLNQ</t>
+          <t>CKLNQ
+时钟锁存器</t>
         </is>
       </c>
       <c r="B261" s="11" t="inlineStr">
@@ -3289,7 +3362,8 @@
     <row r="264">
       <c r="A264" s="2" t="inlineStr">
         <is>
-          <t>CKLVLLHBUFF</t>
+          <t>CKLVLLHBUFF
+电平转换器</t>
         </is>
       </c>
       <c r="B264" s="11" t="inlineStr">
@@ -3311,7 +3385,8 @@
     <row r="266">
       <c r="A266" s="2" t="inlineStr">
         <is>
-          <t>CKLVLLHCH</t>
+          <t>CKLVLLHCH
+电平转换器</t>
         </is>
       </c>
       <c r="B266" s="11" t="inlineStr">
@@ -3333,7 +3408,8 @@
     <row r="268">
       <c r="A268" s="2" t="inlineStr">
         <is>
-          <t>CKLVLLHCL</t>
+          <t>CKLVLLHCL
+电平转换器</t>
         </is>
       </c>
       <c r="B268" s="11" t="inlineStr">
@@ -3355,7 +3431,8 @@
     <row r="270">
       <c r="A270" s="9" t="inlineStr">
         <is>
-          <t>CKLVU</t>
+          <t>CKLVU
+电平转换器</t>
         </is>
       </c>
       <c r="B270" s="10" t="n"/>
@@ -3368,7 +3445,8 @@
     <row r="271">
       <c r="A271" s="2" t="inlineStr">
         <is>
-          <t>CKMUX2</t>
+          <t>CKMUX2
+时钟多路选择器</t>
         </is>
       </c>
       <c r="B271" s="3" t="inlineStr">
@@ -3443,7 +3521,8 @@
     <row r="278">
       <c r="A278" s="9" t="inlineStr">
         <is>
-          <t>CKN</t>
+          <t>CKN
+时钟单元</t>
         </is>
       </c>
       <c r="B278" s="10" t="n"/>
@@ -3456,7 +3535,8 @@
     <row r="279">
       <c r="A279" s="2" t="inlineStr">
         <is>
-          <t>CKND2</t>
+          <t>CKND2
+时钟与非门</t>
         </is>
       </c>
       <c r="B279" s="11" t="inlineStr">
@@ -3514,7 +3594,8 @@
     <row r="285">
       <c r="A285" s="9" t="inlineStr">
         <is>
-          <t>CKND24</t>
+          <t>CKND24
+时钟与非门</t>
         </is>
       </c>
       <c r="B285" s="10" t="inlineStr">
@@ -3527,7 +3608,8 @@
     <row r="286">
       <c r="A286" s="2" t="inlineStr">
         <is>
-          <t>CKNR2</t>
+          <t>CKNR2
+时钟或非门</t>
         </is>
       </c>
       <c r="B286" s="3" t="inlineStr">
@@ -3588,7 +3670,8 @@
     <row r="291">
       <c r="A291" s="2" t="inlineStr">
         <is>
-          <t>CKOR2</t>
+          <t>CKOR2
+时钟或门</t>
         </is>
       </c>
       <c r="B291" s="3" t="inlineStr">
@@ -3640,7 +3723,8 @@
     <row r="295">
       <c r="A295" s="2" t="inlineStr">
         <is>
-          <t>CKXOR2</t>
+          <t>CKXOR2
+时钟或门</t>
         </is>
       </c>
       <c r="B295" s="3" t="inlineStr">
@@ -3693,7 +3777,8 @@
     <row r="300">
       <c r="A300" s="2" t="inlineStr">
         <is>
-          <t>CMPE32</t>
+          <t>CMPE32
+比较器</t>
         </is>
       </c>
       <c r="B300" s="11" t="inlineStr">
@@ -3769,7 +3854,8 @@
     <row r="308">
       <c r="A308" s="2" t="inlineStr">
         <is>
-          <t>CMPE42</t>
+          <t>CMPE42
+比较器</t>
         </is>
       </c>
       <c r="B308" s="11" t="inlineStr">
@@ -3845,7 +3931,8 @@
     <row r="316">
       <c r="A316" s="9" t="inlineStr">
         <is>
-          <t>DCAP10</t>
+          <t>DCAP10
+去耦电容</t>
         </is>
       </c>
       <c r="B316" s="10" t="inlineStr">
@@ -3858,7 +3945,8 @@
     <row r="317">
       <c r="A317" s="9" t="inlineStr">
         <is>
-          <t>DCAP16</t>
+          <t>DCAP16
+去耦电容</t>
         </is>
       </c>
       <c r="B317" s="10" t="n"/>
@@ -3871,7 +3959,8 @@
     <row r="318">
       <c r="A318" s="9" t="inlineStr">
         <is>
-          <t>DCAP20</t>
+          <t>DCAP20
+去耦电容</t>
         </is>
       </c>
       <c r="B318" s="10" t="inlineStr">
@@ -3884,7 +3973,8 @@
     <row r="319">
       <c r="A319" s="9" t="inlineStr">
         <is>
-          <t>DCAP32</t>
+          <t>DCAP32
+去耦电容</t>
         </is>
       </c>
       <c r="B319" s="10" t="n"/>
@@ -3897,7 +3987,8 @@
     <row r="320">
       <c r="A320" s="2" t="inlineStr">
         <is>
-          <t>DCAP4</t>
+          <t>DCAP4
+去耦电容</t>
         </is>
       </c>
       <c r="B320" s="11" t="inlineStr">
@@ -3919,7 +4010,8 @@
     <row r="322">
       <c r="A322" s="9" t="inlineStr">
         <is>
-          <t>DCAP40</t>
+          <t>DCAP40
+去耦电容</t>
         </is>
       </c>
       <c r="B322" s="10" t="inlineStr">
@@ -3932,7 +4024,8 @@
     <row r="323">
       <c r="A323" s="9" t="inlineStr">
         <is>
-          <t>DCAP5</t>
+          <t>DCAP5
+去耦电容</t>
         </is>
       </c>
       <c r="B323" s="10" t="inlineStr">
@@ -3945,7 +4038,8 @@
     <row r="324">
       <c r="A324" s="9" t="inlineStr">
         <is>
-          <t>DCAP64</t>
+          <t>DCAP64
+去耦电容</t>
         </is>
       </c>
       <c r="B324" s="10" t="n"/>
@@ -3958,7 +4052,8 @@
     <row r="325">
       <c r="A325" s="9" t="inlineStr">
         <is>
-          <t>DCAP8</t>
+          <t>DCAP8
+去耦电容</t>
         </is>
       </c>
       <c r="B325" s="10" t="n"/>
@@ -3971,7 +4066,8 @@
     <row r="326">
       <c r="A326" s="2" t="inlineStr">
         <is>
-          <t>DCCKB</t>
+          <t>DCCKB
+时钟缓冲/反相</t>
         </is>
       </c>
       <c r="B326" s="11" t="inlineStr">
@@ -3993,7 +4089,8 @@
     <row r="328">
       <c r="A328" s="9" t="inlineStr">
         <is>
-          <t>DCCKND12</t>
+          <t>DCCKND12
+时钟与非门</t>
         </is>
       </c>
       <c r="B328" s="10" t="inlineStr">
@@ -4006,7 +4103,8 @@
     <row r="329">
       <c r="A329" s="9" t="inlineStr">
         <is>
-          <t>DCCKND20</t>
+          <t>DCCKND20
+时钟与非门</t>
         </is>
       </c>
       <c r="B329" s="10" t="n"/>
@@ -4019,7 +4117,8 @@
     <row r="330">
       <c r="A330" s="2" t="inlineStr">
         <is>
-          <t>DELA</t>
+          <t>DELA
+延时单元</t>
         </is>
       </c>
       <c r="B330" s="11" t="inlineStr">
@@ -4041,7 +4140,8 @@
     <row r="332">
       <c r="A332" s="2" t="inlineStr">
         <is>
-          <t>DELB</t>
+          <t>DELB
+延时单元</t>
         </is>
       </c>
       <c r="B332" s="11" t="inlineStr">
@@ -4063,7 +4163,8 @@
     <row r="334">
       <c r="A334" s="9" t="inlineStr">
         <is>
-          <t>DELC</t>
+          <t>DELC
+延时单元</t>
         </is>
       </c>
       <c r="B334" s="10" t="inlineStr">
@@ -4076,7 +4177,8 @@
     <row r="335">
       <c r="A335" s="2" t="inlineStr">
         <is>
-          <t>DELD</t>
+          <t>DELD
+延时单元</t>
         </is>
       </c>
       <c r="B335" s="11" t="inlineStr">
@@ -4098,7 +4200,8 @@
     <row r="337">
       <c r="A337" s="2" t="inlineStr">
         <is>
-          <t>DELE</t>
+          <t>DELE
+延时单元</t>
         </is>
       </c>
       <c r="B337" s="11" t="inlineStr">
@@ -4120,7 +4223,8 @@
     <row r="339">
       <c r="A339" s="2" t="inlineStr">
         <is>
-          <t>DELF</t>
+          <t>DELF
+延时单元</t>
         </is>
       </c>
       <c r="B339" s="11" t="inlineStr">
@@ -4142,7 +4246,8 @@
     <row r="341">
       <c r="A341" s="9" t="inlineStr">
         <is>
-          <t>DELG</t>
+          <t>DELG
+延时单元</t>
         </is>
       </c>
       <c r="B341" s="10" t="inlineStr">
@@ -4155,7 +4260,8 @@
     <row r="342">
       <c r="A342" s="2" t="inlineStr">
         <is>
-          <t>DFKRPQ</t>
+          <t>DFKRPQ
+D触发器</t>
         </is>
       </c>
       <c r="B342" s="11" t="inlineStr">
@@ -4177,7 +4283,8 @@
     <row r="344">
       <c r="A344" s="2" t="inlineStr">
         <is>
-          <t>DFKSNQ</t>
+          <t>DFKSNQ
+D触发器</t>
         </is>
       </c>
       <c r="B344" s="11" t="inlineStr">
@@ -4199,7 +4306,8 @@
     <row r="346">
       <c r="A346" s="2" t="inlineStr">
         <is>
-          <t>DFKSRPQ</t>
+          <t>DFKSRPQ
+D触发器</t>
         </is>
       </c>
       <c r="B346" s="11" t="inlineStr">
@@ -4221,7 +4329,8 @@
     <row r="348">
       <c r="A348" s="9" t="inlineStr">
         <is>
-          <t>DFMQ</t>
+          <t>DFMQ
+D触发器</t>
         </is>
       </c>
       <c r="B348" s="10" t="inlineStr">
@@ -4234,7 +4343,8 @@
     <row r="349">
       <c r="A349" s="9" t="inlineStr">
         <is>
-          <t>DFNQ</t>
+          <t>DFNQ
+D触发器</t>
         </is>
       </c>
       <c r="B349" s="10" t="inlineStr">
@@ -4247,7 +4357,8 @@
     <row r="350">
       <c r="A350" s="9" t="inlineStr">
         <is>
-          <t>DFNQND2</t>
+          <t>DFNQND2
+D触发器</t>
         </is>
       </c>
       <c r="B350" s="10" t="inlineStr">
@@ -4260,7 +4371,8 @@
     <row r="351">
       <c r="A351" s="2" t="inlineStr">
         <is>
-          <t>DFNRPQ</t>
+          <t>DFNRPQ
+D触发器</t>
         </is>
       </c>
       <c r="B351" s="11" t="inlineStr">
@@ -4282,7 +4394,8 @@
     <row r="353">
       <c r="A353" s="9" t="inlineStr">
         <is>
-          <t>DFNRPQND1</t>
+          <t>DFNRPQND1
+D触发器</t>
         </is>
       </c>
       <c r="B353" s="10" t="n"/>
@@ -4295,7 +4408,8 @@
     <row r="354">
       <c r="A354" s="9" t="inlineStr">
         <is>
-          <t>DFNRPQND2</t>
+          <t>DFNRPQND2
+D触发器</t>
         </is>
       </c>
       <c r="B354" s="10" t="inlineStr">
@@ -4308,7 +4422,8 @@
     <row r="355">
       <c r="A355" s="9" t="inlineStr">
         <is>
-          <t>DFNSNQ</t>
+          <t>DFNSNQ
+D触发器</t>
         </is>
       </c>
       <c r="B355" s="10" t="inlineStr">
@@ -4321,7 +4436,8 @@
     <row r="356">
       <c r="A356" s="9" t="inlineStr">
         <is>
-          <t>DFNSNQND1</t>
+          <t>DFNSNQND1
+D触发器</t>
         </is>
       </c>
       <c r="B356" s="10" t="inlineStr">
@@ -4334,7 +4450,8 @@
     <row r="357">
       <c r="A357" s="2" t="inlineStr">
         <is>
-          <t>DFNSRPQ</t>
+          <t>DFNSRPQ
+D触发器</t>
         </is>
       </c>
       <c r="B357" s="11" t="inlineStr">
@@ -4356,7 +4473,8 @@
     <row r="359">
       <c r="A359" s="2" t="inlineStr">
         <is>
-          <t>DFQ</t>
+          <t>DFQ
+D触发器</t>
         </is>
       </c>
       <c r="B359" s="11" t="inlineStr">
@@ -4378,7 +4496,8 @@
     <row r="361">
       <c r="A361" s="9" t="inlineStr">
         <is>
-          <t>DFQN</t>
+          <t>DFQN
+D触发器</t>
         </is>
       </c>
       <c r="B361" s="10" t="n"/>
@@ -4391,7 +4510,8 @@
     <row r="362">
       <c r="A362" s="9" t="inlineStr">
         <is>
-          <t>DFQND1</t>
+          <t>DFQND1
+D触发器</t>
         </is>
       </c>
       <c r="B362" s="10" t="inlineStr">
@@ -4404,7 +4524,8 @@
     <row r="363">
       <c r="A363" s="2" t="inlineStr">
         <is>
-          <t>DFRPQ</t>
+          <t>DFRPQ
+D触发器</t>
         </is>
       </c>
       <c r="B363" s="11" t="inlineStr">
@@ -4435,7 +4556,8 @@
     <row r="366">
       <c r="A366" s="9" t="inlineStr">
         <is>
-          <t>DFRPQND1</t>
+          <t>DFRPQND1
+D触发器</t>
         </is>
       </c>
       <c r="B366" s="10" t="inlineStr">
@@ -4448,7 +4570,8 @@
     <row r="367">
       <c r="A367" s="9" t="inlineStr">
         <is>
-          <t>DFRPQND2</t>
+          <t>DFRPQND2
+D触发器</t>
         </is>
       </c>
       <c r="B367" s="10" t="n"/>
@@ -4461,7 +4584,8 @@
     <row r="368">
       <c r="A368" s="2" t="inlineStr">
         <is>
-          <t>DFSNQ</t>
+          <t>DFSNQ
+D触发器</t>
         </is>
       </c>
       <c r="B368" s="11" t="inlineStr">
@@ -4492,7 +4616,8 @@
     <row r="371">
       <c r="A371" s="9" t="inlineStr">
         <is>
-          <t>DFSNQND2</t>
+          <t>DFSNQND2
+D触发器</t>
         </is>
       </c>
       <c r="B371" s="10" t="n"/>
@@ -4505,7 +4630,8 @@
     <row r="372">
       <c r="A372" s="9" t="inlineStr">
         <is>
-          <t>DFSNQND4</t>
+          <t>DFSNQND4
+D触发器</t>
         </is>
       </c>
       <c r="B372" s="10" t="inlineStr">
@@ -4518,7 +4644,8 @@
     <row r="373">
       <c r="A373" s="9" t="inlineStr">
         <is>
-          <t>DFSRPQ</t>
+          <t>DFSRPQ
+D触发器</t>
         </is>
       </c>
       <c r="B373" s="10" t="inlineStr">
@@ -4531,7 +4658,8 @@
     <row r="374">
       <c r="A374" s="2" t="inlineStr">
         <is>
-          <t>EDFQ</t>
+          <t>EDFQ
+扫描触发器</t>
         </is>
       </c>
       <c r="B374" s="11" t="inlineStr">
@@ -4553,7 +4681,8 @@
     <row r="376">
       <c r="A376" s="2" t="inlineStr">
         <is>
-          <t>EDFRPQ</t>
+          <t>EDFRPQ
+扫描触发器</t>
         </is>
       </c>
       <c r="B376" s="11" t="inlineStr">
@@ -4575,7 +4704,8 @@
     <row r="378">
       <c r="A378" s="2" t="inlineStr">
         <is>
-          <t>FA1</t>
+          <t>FA1
+全加器</t>
         </is>
       </c>
       <c r="B378" s="3" t="inlineStr">
@@ -4646,7 +4776,8 @@
     <row r="385">
       <c r="A385" s="9" t="inlineStr">
         <is>
-          <t>FA1ND1</t>
+          <t>FA1ND1
+全加器</t>
         </is>
       </c>
       <c r="B385" s="10" t="n"/>
@@ -4659,7 +4790,8 @@
     <row r="386">
       <c r="A386" s="9" t="inlineStr">
         <is>
-          <t>FA1SND1</t>
+          <t>FA1SND1
+全加器</t>
         </is>
       </c>
       <c r="B386" s="10" t="inlineStr">
@@ -4672,7 +4804,8 @@
     <row r="387">
       <c r="A387" s="9" t="inlineStr">
         <is>
-          <t>FA1SND4</t>
+          <t>FA1SND4
+全加器</t>
         </is>
       </c>
       <c r="B387" s="10" t="n"/>
@@ -4685,7 +4818,8 @@
     <row r="388">
       <c r="A388" s="2" t="inlineStr">
         <is>
-          <t>FCICO</t>
+          <t>FCICO
+进位逻辑</t>
         </is>
       </c>
       <c r="B388" s="11" t="inlineStr">
@@ -4707,7 +4841,8 @@
     <row r="390">
       <c r="A390" s="9" t="inlineStr">
         <is>
-          <t>FCICOND1</t>
+          <t>FCICOND1
+进位逻辑</t>
         </is>
       </c>
       <c r="B390" s="10" t="inlineStr">
@@ -4720,7 +4855,8 @@
     <row r="391">
       <c r="A391" s="2" t="inlineStr">
         <is>
-          <t>FCIS</t>
+          <t>FCIS
+进位逻辑</t>
         </is>
       </c>
       <c r="B391" s="11" t="inlineStr">
@@ -4742,7 +4878,8 @@
     <row r="393">
       <c r="A393" s="9" t="inlineStr">
         <is>
-          <t>FCISND2</t>
+          <t>FCISND2
+进位逻辑</t>
         </is>
       </c>
       <c r="B393" s="10" t="inlineStr">
@@ -4755,7 +4892,8 @@
     <row r="394">
       <c r="A394" s="9" t="inlineStr">
         <is>
-          <t>FCISND4</t>
+          <t>FCISND4
+进位逻辑</t>
         </is>
       </c>
       <c r="B394" s="10" t="n"/>
@@ -4768,7 +4906,8 @@
     <row r="395">
       <c r="A395" s="9" t="inlineStr">
         <is>
-          <t>FCONSND1</t>
+          <t>FCONSND1
+进位逻辑</t>
         </is>
       </c>
       <c r="B395" s="10" t="inlineStr">
@@ -4781,7 +4920,8 @@
     <row r="396">
       <c r="A396" s="9" t="inlineStr">
         <is>
-          <t>FCSICOND1</t>
+          <t>FCSICOND1
+进位逻辑</t>
         </is>
       </c>
       <c r="B396" s="10" t="inlineStr">
@@ -4794,7 +4934,8 @@
     <row r="397">
       <c r="A397" s="9" t="inlineStr">
         <is>
-          <t>FIICOND1</t>
+          <t>FIICOND1
+进位逻辑</t>
         </is>
       </c>
       <c r="B397" s="10" t="n"/>
@@ -4807,7 +4948,8 @@
     <row r="398">
       <c r="A398" s="9" t="inlineStr">
         <is>
-          <t>FIICOND4</t>
+          <t>FIICOND4
+进位逻辑</t>
         </is>
       </c>
       <c r="B398" s="10" t="inlineStr">
@@ -4820,7 +4962,8 @@
     <row r="399">
       <c r="A399" s="2" t="inlineStr">
         <is>
-          <t>FILL1</t>
+          <t>FILL1
+填充单元</t>
         </is>
       </c>
       <c r="B399" s="11" t="n"/>
@@ -4842,7 +4985,8 @@
     <row r="401">
       <c r="A401" s="2" t="inlineStr">
         <is>
-          <t>FILL12</t>
+          <t>FILL12
+填充单元</t>
         </is>
       </c>
       <c r="B401" s="11" t="inlineStr">
@@ -4864,7 +5008,8 @@
     <row r="403">
       <c r="A403" s="2" t="inlineStr">
         <is>
-          <t>FILL16</t>
+          <t>FILL16
+填充单元</t>
         </is>
       </c>
       <c r="B403" s="3" t="inlineStr">
@@ -4890,7 +5035,8 @@
     <row r="405">
       <c r="A405" s="2" t="inlineStr">
         <is>
-          <t>FILL2</t>
+          <t>FILL2
+填充单元</t>
         </is>
       </c>
       <c r="B405" s="11" t="inlineStr">
@@ -4912,7 +5058,8 @@
     <row r="407">
       <c r="A407" s="2" t="inlineStr">
         <is>
-          <t>FILL3</t>
+          <t>FILL3
+填充单元</t>
         </is>
       </c>
       <c r="B407" s="3" t="inlineStr">
@@ -4938,7 +5085,8 @@
     <row r="409">
       <c r="A409" s="2" t="inlineStr">
         <is>
-          <t>FILL32</t>
+          <t>FILL32
+填充单元</t>
         </is>
       </c>
       <c r="B409" s="11" t="inlineStr">
@@ -4960,7 +5108,8 @@
     <row r="411">
       <c r="A411" s="2" t="inlineStr">
         <is>
-          <t>FILL4</t>
+          <t>FILL4
+填充单元</t>
         </is>
       </c>
       <c r="B411" s="3" t="inlineStr">
@@ -4986,7 +5135,8 @@
     <row r="413">
       <c r="A413" s="2" t="inlineStr">
         <is>
-          <t>FILL64</t>
+          <t>FILL64
+填充单元</t>
         </is>
       </c>
       <c r="B413" s="3" t="inlineStr">
@@ -5012,7 +5162,8 @@
     <row r="415">
       <c r="A415" s="2" t="inlineStr">
         <is>
-          <t>FILL8</t>
+          <t>FILL8
+填充单元</t>
         </is>
       </c>
       <c r="B415" s="11" t="inlineStr">
@@ -5034,7 +5185,8 @@
     <row r="417">
       <c r="A417" s="9" t="inlineStr">
         <is>
-          <t>GAN2</t>
+          <t>GAN2
+与门</t>
         </is>
       </c>
       <c r="B417" s="10" t="inlineStr">
@@ -5047,7 +5199,8 @@
     <row r="418">
       <c r="A418" s="9" t="inlineStr">
         <is>
-          <t>GAN3</t>
+          <t>GAN3
+与门</t>
         </is>
       </c>
       <c r="B418" s="10" t="inlineStr">
@@ -5060,7 +5213,8 @@
     <row r="419">
       <c r="A419" s="9" t="inlineStr">
         <is>
-          <t>GAN4</t>
+          <t>GAN4
+与门</t>
         </is>
       </c>
       <c r="B419" s="10" t="inlineStr">
@@ -5073,7 +5227,8 @@
     <row r="420">
       <c r="A420" s="9" t="inlineStr">
         <is>
-          <t>GAND3</t>
+          <t>GAND3
+与门</t>
         </is>
       </c>
       <c r="B420" s="10" t="n"/>
@@ -5086,7 +5241,8 @@
     <row r="421">
       <c r="A421" s="9" t="inlineStr">
         <is>
-          <t>GAO21</t>
+          <t>GAO21
+与或门</t>
         </is>
       </c>
       <c r="B421" s="12" t="inlineStr">
@@ -5103,7 +5259,8 @@
     <row r="422">
       <c r="A422" s="9" t="inlineStr">
         <is>
-          <t>GAO22</t>
+          <t>GAO22
+与或门</t>
         </is>
       </c>
       <c r="B422" s="12" t="inlineStr">
@@ -5120,7 +5277,8 @@
     <row r="423">
       <c r="A423" s="9" t="inlineStr">
         <is>
-          <t>GAO31</t>
+          <t>GAO31
+与或门</t>
         </is>
       </c>
       <c r="B423" s="10" t="n"/>
@@ -5133,7 +5291,8 @@
     <row r="424">
       <c r="A424" s="9" t="inlineStr">
         <is>
-          <t>GAO32</t>
+          <t>GAO32
+与或门</t>
         </is>
       </c>
       <c r="B424" s="10" t="n"/>
@@ -5146,7 +5305,8 @@
     <row r="425">
       <c r="A425" s="2" t="inlineStr">
         <is>
-          <t>GAOI21</t>
+          <t>GAOI21
+与或非门</t>
         </is>
       </c>
       <c r="B425" s="11" t="inlineStr">
@@ -5168,7 +5328,8 @@
     <row r="427">
       <c r="A427" s="2" t="inlineStr">
         <is>
-          <t>GAOI22</t>
+          <t>GAOI22
+与或非门</t>
         </is>
       </c>
       <c r="B427" s="11" t="inlineStr">
@@ -5190,7 +5351,8 @@
     <row r="429">
       <c r="A429" s="9" t="inlineStr">
         <is>
-          <t>GAOI33</t>
+          <t>GAOI33
+与或非门</t>
         </is>
       </c>
       <c r="B429" s="10" t="n"/>
@@ -5203,7 +5365,8 @@
     <row r="430">
       <c r="A430" s="9" t="inlineStr">
         <is>
-          <t>GBUFF</t>
+          <t>GBUFF
+缓冲器</t>
         </is>
       </c>
       <c r="B430" s="10" t="inlineStr">
@@ -5216,7 +5379,8 @@
     <row r="431">
       <c r="A431" s="9" t="inlineStr">
         <is>
-          <t>GCKLNQ</t>
+          <t>GCKLNQ
+时钟锁存器</t>
         </is>
       </c>
       <c r="B431" s="10" t="inlineStr">
@@ -5229,7 +5393,8 @@
     <row r="432">
       <c r="A432" s="2" t="inlineStr">
         <is>
-          <t>GCKNQ</t>
+          <t>GCKNQ
+时钟单元</t>
         </is>
       </c>
       <c r="B432" s="11" t="n"/>
@@ -5260,7 +5425,8 @@
     <row r="435">
       <c r="A435" s="9" t="inlineStr">
         <is>
-          <t>GDCAP12</t>
+          <t>GDCAP12
+去耦电容</t>
         </is>
       </c>
       <c r="B435" s="10" t="inlineStr">
@@ -5273,7 +5439,8 @@
     <row r="436">
       <c r="A436" s="9" t="inlineStr">
         <is>
-          <t>GDCAP2</t>
+          <t>GDCAP2
+去耦电容</t>
         </is>
       </c>
       <c r="B436" s="10" t="inlineStr">
@@ -5286,7 +5453,8 @@
     <row r="437">
       <c r="A437" s="9" t="inlineStr">
         <is>
-          <t>GDCAP4</t>
+          <t>GDCAP4
+去耦电容</t>
         </is>
       </c>
       <c r="B437" s="10" t="inlineStr">
@@ -5299,7 +5467,8 @@
     <row r="438">
       <c r="A438" s="9" t="inlineStr">
         <is>
-          <t>GDCAP6</t>
+          <t>GDCAP6
+去耦电容</t>
         </is>
       </c>
       <c r="B438" s="10" t="inlineStr">
@@ -5312,7 +5481,8 @@
     <row r="439">
       <c r="A439" s="9" t="inlineStr">
         <is>
-          <t>GDCAP8</t>
+          <t>GDCAP8
+去耦电容</t>
         </is>
       </c>
       <c r="B439" s="10" t="inlineStr">
@@ -5325,7 +5495,8 @@
     <row r="440">
       <c r="A440" s="9" t="inlineStr">
         <is>
-          <t>GDFQ</t>
+          <t>GDFQ
+D触发器</t>
         </is>
       </c>
       <c r="B440" s="12" t="inlineStr">
@@ -5342,7 +5513,8 @@
     <row r="441">
       <c r="A441" s="9" t="inlineStr">
         <is>
-          <t>GDFRPQ</t>
+          <t>GDFRPQ
+D触发器</t>
         </is>
       </c>
       <c r="B441" s="10" t="inlineStr">
@@ -5355,7 +5527,8 @@
     <row r="442">
       <c r="A442" s="9" t="inlineStr">
         <is>
-          <t>GDFSNQ</t>
+          <t>GDFSNQ
+D触发器</t>
         </is>
       </c>
       <c r="B442" s="12" t="inlineStr">
@@ -5372,7 +5545,8 @@
     <row r="443">
       <c r="A443" s="9" t="inlineStr">
         <is>
-          <t>GFILL1</t>
+          <t>GFILL1
+填充单元</t>
         </is>
       </c>
       <c r="B443" s="10" t="inlineStr">
@@ -5385,7 +5559,8 @@
     <row r="444">
       <c r="A444" s="9" t="inlineStr">
         <is>
-          <t>GFILL11</t>
+          <t>GFILL11
+填充单元</t>
         </is>
       </c>
       <c r="B444" s="10" t="inlineStr">
@@ -5398,7 +5573,8 @@
     <row r="445">
       <c r="A445" s="9" t="inlineStr">
         <is>
-          <t>GFILL12</t>
+          <t>GFILL12
+填充单元</t>
         </is>
       </c>
       <c r="B445" s="10" t="inlineStr">
@@ -5411,7 +5587,8 @@
     <row r="446">
       <c r="A446" s="2" t="inlineStr">
         <is>
-          <t>GFILL2</t>
+          <t>GFILL2
+填充单元</t>
         </is>
       </c>
       <c r="B446" s="11" t="inlineStr">
@@ -5433,7 +5610,8 @@
     <row r="448">
       <c r="A448" s="2" t="inlineStr">
         <is>
-          <t>GFILL3</t>
+          <t>GFILL3
+填充单元</t>
         </is>
       </c>
       <c r="B448" s="11" t="inlineStr">
@@ -5455,7 +5633,8 @@
     <row r="450">
       <c r="A450" s="2" t="inlineStr">
         <is>
-          <t>GFILL4</t>
+          <t>GFILL4
+填充单元</t>
         </is>
       </c>
       <c r="B450" s="11" t="inlineStr">
@@ -5477,7 +5656,8 @@
     <row r="452">
       <c r="A452" s="2" t="inlineStr">
         <is>
-          <t>GFILL5</t>
+          <t>GFILL5
+填充单元</t>
         </is>
       </c>
       <c r="B452" s="11" t="inlineStr">
@@ -5499,7 +5679,8 @@
     <row r="454">
       <c r="A454" s="2" t="inlineStr">
         <is>
-          <t>GFILL6</t>
+          <t>GFILL6
+填充单元</t>
         </is>
       </c>
       <c r="B454" s="11" t="inlineStr">
@@ -5521,7 +5702,8 @@
     <row r="456">
       <c r="A456" s="9" t="inlineStr">
         <is>
-          <t>GFILL7</t>
+          <t>GFILL7
+填充单元</t>
         </is>
       </c>
       <c r="B456" s="10" t="inlineStr">
@@ -5534,7 +5716,8 @@
     <row r="457">
       <c r="A457" s="2" t="inlineStr">
         <is>
-          <t>GFILL8</t>
+          <t>GFILL8
+填充单元</t>
         </is>
       </c>
       <c r="B457" s="11" t="inlineStr">
@@ -5556,7 +5739,8 @@
     <row r="459">
       <c r="A459" s="9" t="inlineStr">
         <is>
-          <t>GFILL9</t>
+          <t>GFILL9
+填充单元</t>
         </is>
       </c>
       <c r="B459" s="10" t="inlineStr">
@@ -5569,7 +5753,8 @@
     <row r="460">
       <c r="A460" s="9" t="inlineStr">
         <is>
-          <t>GIND4</t>
+          <t>GIND4
+与非门</t>
         </is>
       </c>
       <c r="B460" s="10" t="n"/>
@@ -5582,7 +5767,8 @@
     <row r="461">
       <c r="A461" s="9" t="inlineStr">
         <is>
-          <t>GINV</t>
+          <t>GINV
+反相器</t>
         </is>
       </c>
       <c r="B461" s="10" t="inlineStr">
@@ -5595,7 +5781,8 @@
     <row r="462">
       <c r="A462" s="9" t="inlineStr">
         <is>
-          <t>GLAHQ</t>
+          <t>GLAHQ
+锁存器</t>
         </is>
       </c>
       <c r="B462" s="10" t="n"/>
@@ -5608,7 +5795,8 @@
     <row r="463">
       <c r="A463" s="9" t="inlineStr">
         <is>
-          <t>GLHCNQ</t>
+          <t>GLHCNQ
+锁存器</t>
         </is>
       </c>
       <c r="B463" s="10" t="inlineStr">
@@ -5621,7 +5809,8 @@
     <row r="464">
       <c r="A464" s="9" t="inlineStr">
         <is>
-          <t>GLHQ</t>
+          <t>GLHQ
+锁存器</t>
         </is>
       </c>
       <c r="B464" s="10" t="inlineStr">
@@ -5634,7 +5823,8 @@
     <row r="465">
       <c r="A465" s="9" t="inlineStr">
         <is>
-          <t>GLNCNQ</t>
+          <t>GLNCNQ
+锁存器</t>
         </is>
       </c>
       <c r="B465" s="10" t="inlineStr">
@@ -5647,7 +5837,8 @@
     <row r="466">
       <c r="A466" s="9" t="inlineStr">
         <is>
-          <t>GLNQ</t>
+          <t>GLNQ
+锁存器</t>
         </is>
       </c>
       <c r="B466" s="10" t="inlineStr">
@@ -5660,7 +5851,8 @@
     <row r="467">
       <c r="A467" s="9" t="inlineStr">
         <is>
-          <t>GMUX2</t>
+          <t>GMUX2
+多路选择器</t>
         </is>
       </c>
       <c r="B467" s="12" t="inlineStr">
@@ -5677,7 +5869,8 @@
     <row r="468">
       <c r="A468" s="9" t="inlineStr">
         <is>
-          <t>GMUX2ND1</t>
+          <t>GMUX2ND1
+复合多路选择器</t>
         </is>
       </c>
       <c r="B468" s="10" t="inlineStr">
@@ -5690,7 +5883,8 @@
     <row r="469">
       <c r="A469" s="9" t="inlineStr">
         <is>
-          <t>GNAND2</t>
+          <t>GNAND2
+与非门</t>
         </is>
       </c>
       <c r="B469" s="10" t="n"/>
@@ -5703,7 +5897,8 @@
     <row r="470">
       <c r="A470" s="9" t="inlineStr">
         <is>
-          <t>GND2</t>
+          <t>GND2
+与非门</t>
         </is>
       </c>
       <c r="B470" s="10" t="inlineStr">
@@ -5716,7 +5911,8 @@
     <row r="471">
       <c r="A471" s="9" t="inlineStr">
         <is>
-          <t>GND3</t>
+          <t>GND3
+与非门</t>
         </is>
       </c>
       <c r="B471" s="10" t="inlineStr">
@@ -5729,7 +5925,8 @@
     <row r="472">
       <c r="A472" s="9" t="inlineStr">
         <is>
-          <t>GNOR4</t>
+          <t>GNOR4
+或非门</t>
         </is>
       </c>
       <c r="B472" s="10" t="n"/>
@@ -5742,7 +5939,8 @@
     <row r="473">
       <c r="A473" s="2" t="inlineStr">
         <is>
-          <t>GNR2</t>
+          <t>GNR2
+或非门</t>
         </is>
       </c>
       <c r="B473" s="11" t="inlineStr">
@@ -5764,7 +5962,8 @@
     <row r="475">
       <c r="A475" s="9" t="inlineStr">
         <is>
-          <t>GNR3</t>
+          <t>GNR3
+或非门</t>
         </is>
       </c>
       <c r="B475" s="10" t="inlineStr">
@@ -5777,7 +5976,8 @@
     <row r="476">
       <c r="A476" s="9" t="inlineStr">
         <is>
-          <t>GNR4</t>
+          <t>GNR4
+或非门</t>
         </is>
       </c>
       <c r="B476" s="10" t="inlineStr">
@@ -5790,7 +5990,8 @@
     <row r="477">
       <c r="A477" s="9" t="inlineStr">
         <is>
-          <t>GOA21</t>
+          <t>GOA21
+或与门</t>
         </is>
       </c>
       <c r="B477" s="12" t="inlineStr">
@@ -5807,7 +6008,8 @@
     <row r="478">
       <c r="A478" s="9" t="inlineStr">
         <is>
-          <t>GOA22</t>
+          <t>GOA22
+或与门</t>
         </is>
       </c>
       <c r="B478" s="12" t="inlineStr">
@@ -5824,7 +6026,8 @@
     <row r="479">
       <c r="A479" s="9" t="inlineStr">
         <is>
-          <t>GOA32</t>
+          <t>GOA32
+或与门</t>
         </is>
       </c>
       <c r="B479" s="10" t="n"/>
@@ -5837,7 +6040,8 @@
     <row r="480">
       <c r="A480" s="2" t="inlineStr">
         <is>
-          <t>GOAI21</t>
+          <t>GOAI21
+或与非门</t>
         </is>
       </c>
       <c r="B480" s="11" t="inlineStr">
@@ -5859,7 +6063,8 @@
     <row r="482">
       <c r="A482" s="9" t="inlineStr">
         <is>
-          <t>GOAI211</t>
+          <t>GOAI211
+或与非门</t>
         </is>
       </c>
       <c r="B482" s="10" t="n"/>
@@ -5872,7 +6077,8 @@
     <row r="483">
       <c r="A483" s="2" t="inlineStr">
         <is>
-          <t>GOAI22</t>
+          <t>GOAI22
+或与非门</t>
         </is>
       </c>
       <c r="B483" s="3" t="inlineStr">
@@ -5898,7 +6104,8 @@
     <row r="485">
       <c r="A485" s="9" t="inlineStr">
         <is>
-          <t>GOAI33</t>
+          <t>GOAI33
+或与非门</t>
         </is>
       </c>
       <c r="B485" s="10" t="n"/>
@@ -5911,7 +6118,8 @@
     <row r="486">
       <c r="A486" s="9" t="inlineStr">
         <is>
-          <t>GOR2</t>
+          <t>GOR2
+或门</t>
         </is>
       </c>
       <c r="B486" s="12" t="inlineStr">
@@ -5928,7 +6136,8 @@
     <row r="487">
       <c r="A487" s="9" t="inlineStr">
         <is>
-          <t>GOR3</t>
+          <t>GOR3
+或门</t>
         </is>
       </c>
       <c r="B487" s="10" t="inlineStr">
@@ -5941,7 +6150,8 @@
     <row r="488">
       <c r="A488" s="9" t="inlineStr">
         <is>
-          <t>GOR4</t>
+          <t>GOR4
+或门</t>
         </is>
       </c>
       <c r="B488" s="12" t="inlineStr">
@@ -5958,7 +6168,8 @@
     <row r="489">
       <c r="A489" s="9" t="inlineStr">
         <is>
-          <t>GPULL0</t>
+          <t>GPULL0
+上拉/下拉</t>
         </is>
       </c>
       <c r="B489" s="10" t="n"/>
@@ -5971,7 +6182,8 @@
     <row r="490">
       <c r="A490" s="9" t="inlineStr">
         <is>
-          <t>GSDFQ</t>
+          <t>GSDFQ
+扫描触发器</t>
         </is>
       </c>
       <c r="B490" s="10" t="inlineStr">
@@ -5984,7 +6196,8 @@
     <row r="491">
       <c r="A491" s="9" t="inlineStr">
         <is>
-          <t>GSDFRPQ</t>
+          <t>GSDFRPQ
+扫描触发器</t>
         </is>
       </c>
       <c r="B491" s="10" t="inlineStr">
@@ -5997,7 +6210,8 @@
     <row r="492">
       <c r="A492" s="9" t="inlineStr">
         <is>
-          <t>GSDFSNQ</t>
+          <t>GSDFSNQ
+扫描触发器</t>
         </is>
       </c>
       <c r="B492" s="12" t="inlineStr">
@@ -6014,7 +6228,8 @@
     <row r="493">
       <c r="A493" s="9" t="inlineStr">
         <is>
-          <t>GTIEHXP</t>
+          <t>GTIEHXP
+电平钳位</t>
         </is>
       </c>
       <c r="B493" s="10" t="inlineStr">
@@ -6027,7 +6242,8 @@
     <row r="494">
       <c r="A494" s="9" t="inlineStr">
         <is>
-          <t>GTIELXN</t>
+          <t>GTIELXN
+电平钳位</t>
         </is>
       </c>
       <c r="B494" s="10" t="inlineStr">
@@ -6040,7 +6256,8 @@
     <row r="495">
       <c r="A495" s="9" t="inlineStr">
         <is>
-          <t>GXNR2</t>
+          <t>GXNR2
+同或门</t>
         </is>
       </c>
       <c r="B495" s="10" t="inlineStr">
@@ -6053,7 +6270,8 @@
     <row r="496">
       <c r="A496" s="9" t="inlineStr">
         <is>
-          <t>GXOR2</t>
+          <t>GXOR2
+异或门</t>
         </is>
       </c>
       <c r="B496" s="10" t="inlineStr">
@@ -6066,7 +6284,8 @@
     <row r="497">
       <c r="A497" s="2" t="inlineStr">
         <is>
-          <t>HA1</t>
+          <t>HA1
+半加器</t>
         </is>
       </c>
       <c r="B497" s="3" t="inlineStr">
@@ -6110,7 +6329,8 @@
     <row r="501">
       <c r="A501" s="2" t="inlineStr">
         <is>
-          <t>HAC1</t>
+          <t>HAC1
+半加器</t>
         </is>
       </c>
       <c r="B501" s="11" t="inlineStr">
@@ -6186,7 +6406,8 @@
     <row r="509">
       <c r="A509" s="9" t="inlineStr">
         <is>
-          <t>HDDICWYX2A20</t>
+          <t>HDDICWYX2A20
+边界/版图单元</t>
         </is>
       </c>
       <c r="B509" s="10" t="n"/>
@@ -6199,7 +6420,8 @@
     <row r="510">
       <c r="A510" s="9" t="inlineStr">
         <is>
-          <t>HDDICWYX2B30</t>
+          <t>HDDICWYX2B30
+边界/版图单元</t>
         </is>
       </c>
       <c r="B510" s="10" t="n"/>
@@ -6212,7 +6434,8 @@
     <row r="511">
       <c r="A511" s="9" t="inlineStr">
         <is>
-          <t>HDDID2A30</t>
+          <t>HDDID2A30
+边界/版图单元</t>
         </is>
       </c>
       <c r="B511" s="10" t="inlineStr">
@@ -6225,7 +6448,8 @@
     <row r="512">
       <c r="A512" s="9" t="inlineStr">
         <is>
-          <t>HDDID2A40</t>
+          <t>HDDID2A40
+边界/版图单元</t>
         </is>
       </c>
       <c r="B512" s="10" t="inlineStr">
@@ -6238,7 +6462,8 @@
     <row r="513">
       <c r="A513" s="2" t="inlineStr">
         <is>
-          <t>IAO21</t>
+          <t>IAO21
+复合逻辑门</t>
         </is>
       </c>
       <c r="B513" s="11" t="inlineStr">
@@ -6287,7 +6512,8 @@
     <row r="518">
       <c r="A518" s="2" t="inlineStr">
         <is>
-          <t>IAO22</t>
+          <t>IAO22
+复合逻辑门</t>
         </is>
       </c>
       <c r="B518" s="3" t="inlineStr">
@@ -6344,7 +6570,8 @@
     <row r="523">
       <c r="A523" s="2" t="inlineStr">
         <is>
-          <t>IAOI21</t>
+          <t>IAOI21
+复合逻辑门</t>
         </is>
       </c>
       <c r="B523" s="3" t="inlineStr">
@@ -6397,7 +6624,8 @@
     <row r="528">
       <c r="A528" s="2" t="inlineStr">
         <is>
-          <t>IIND3</t>
+          <t>IIND3
+与非门</t>
         </is>
       </c>
       <c r="B528" s="11" t="inlineStr">
@@ -6446,7 +6674,8 @@
     <row r="533">
       <c r="A533" s="9" t="inlineStr">
         <is>
-          <t>IIND4</t>
+          <t>IIND4
+与非门</t>
         </is>
       </c>
       <c r="B533" s="10" t="inlineStr">
@@ -6459,7 +6688,8 @@
     <row r="534">
       <c r="A534" s="2" t="inlineStr">
         <is>
-          <t>IINR3</t>
+          <t>IINR3
+或非门</t>
         </is>
       </c>
       <c r="B534" s="3" t="inlineStr">
@@ -6521,7 +6751,8 @@
     <row r="540">
       <c r="A540" s="2" t="inlineStr">
         <is>
-          <t>IINR4</t>
+          <t>IINR4
+或非门</t>
         </is>
       </c>
       <c r="B540" s="11" t="inlineStr">
@@ -6561,7 +6792,8 @@
     <row r="544">
       <c r="A544" s="2" t="inlineStr">
         <is>
-          <t>IND2</t>
+          <t>IND2
+与非门</t>
         </is>
       </c>
       <c r="B544" s="11" t="inlineStr">
@@ -6628,7 +6860,8 @@
     <row r="551">
       <c r="A551" s="2" t="inlineStr">
         <is>
-          <t>IND3</t>
+          <t>IND3
+与非门</t>
         </is>
       </c>
       <c r="B551" s="11" t="inlineStr">
@@ -6668,7 +6901,8 @@
     <row r="555">
       <c r="A555" s="9" t="inlineStr">
         <is>
-          <t>IND4</t>
+          <t>IND4
+与非门</t>
         </is>
       </c>
       <c r="B555" s="10" t="inlineStr">
@@ -6681,7 +6915,8 @@
     <row r="556">
       <c r="A556" s="2" t="inlineStr">
         <is>
-          <t>INR2</t>
+          <t>INR2
+或非门</t>
         </is>
       </c>
       <c r="B556" s="3" t="inlineStr">
@@ -6806,7 +7041,8 @@
     <row r="569">
       <c r="A569" s="2" t="inlineStr">
         <is>
-          <t>INR3</t>
+          <t>INR3
+或非门</t>
         </is>
       </c>
       <c r="B569" s="3" t="inlineStr">
@@ -6890,7 +7126,8 @@
     <row r="577">
       <c r="A577" s="2" t="inlineStr">
         <is>
-          <t>INR4</t>
+          <t>INR4
+或非门</t>
         </is>
       </c>
       <c r="B577" s="3" t="inlineStr">
@@ -6929,7 +7166,8 @@
     <row r="580">
       <c r="A580" s="9" t="inlineStr">
         <is>
-          <t>INV</t>
+          <t>INV
+反相器</t>
         </is>
       </c>
       <c r="B580" s="10" t="inlineStr">
@@ -6942,7 +7180,8 @@
     <row r="581">
       <c r="A581" s="9" t="inlineStr">
         <is>
-          <t>INVAAOI21</t>
+          <t>INVAAOI21
+复合逻辑门</t>
         </is>
       </c>
       <c r="B581" s="10" t="inlineStr">
@@ -6955,7 +7194,8 @@
     <row r="582">
       <c r="A582" s="2" t="inlineStr">
         <is>
-          <t>INVAOAI21</t>
+          <t>INVAOAI21
+复合逻辑门</t>
         </is>
       </c>
       <c r="B582" s="11" t="inlineStr">
@@ -6977,7 +7217,8 @@
     <row r="584">
       <c r="A584" s="2" t="inlineStr">
         <is>
-          <t>INVBAOI21</t>
+          <t>INVBAOI21
+复合逻辑门</t>
         </is>
       </c>
       <c r="B584" s="11" t="inlineStr">
@@ -6999,7 +7240,8 @@
     <row r="586">
       <c r="A586" s="2" t="inlineStr">
         <is>
-          <t>INVBOAI21</t>
+          <t>INVBOAI21
+复合逻辑门</t>
         </is>
       </c>
       <c r="B586" s="11" t="inlineStr">
@@ -7021,7 +7263,8 @@
     <row r="588">
       <c r="A588" s="9" t="inlineStr">
         <is>
-          <t>INVPAD</t>
+          <t>INVPAD
+焊盘反相器</t>
         </is>
       </c>
       <c r="B588" s="10" t="inlineStr">
@@ -7034,7 +7277,8 @@
     <row r="589">
       <c r="A589" s="2" t="inlineStr">
         <is>
-          <t>IOA21</t>
+          <t>IOA21
+复合逻辑门</t>
         </is>
       </c>
       <c r="B589" s="3" t="inlineStr">
@@ -7105,7 +7349,8 @@
     <row r="596">
       <c r="A596" s="2" t="inlineStr">
         <is>
-          <t>IOA22</t>
+          <t>IOA22
+复合逻辑门</t>
         </is>
       </c>
       <c r="B596" s="3" t="inlineStr">
@@ -7149,7 +7394,8 @@
     <row r="600">
       <c r="A600" s="2" t="inlineStr">
         <is>
-          <t>IOAI21</t>
+          <t>IOAI21
+复合逻辑门</t>
         </is>
       </c>
       <c r="B600" s="3" t="inlineStr">
@@ -7206,7 +7452,8 @@
     <row r="605">
       <c r="A605" s="2" t="inlineStr">
         <is>
-          <t>ISOCH</t>
+          <t>ISOCH
+电平转换器</t>
         </is>
       </c>
       <c r="B605" s="11" t="inlineStr">
@@ -7237,7 +7484,8 @@
     <row r="608">
       <c r="A608" s="2" t="inlineStr">
         <is>
-          <t>ISOCL</t>
+          <t>ISOCL
+电平转换器</t>
         </is>
       </c>
       <c r="B608" s="11" t="inlineStr">
@@ -7259,7 +7507,8 @@
     <row r="610">
       <c r="A610" s="9" t="inlineStr">
         <is>
-          <t>ISOH</t>
+          <t>ISOH
+电平转换器</t>
         </is>
       </c>
       <c r="B610" s="10" t="n"/>
@@ -7272,7 +7521,8 @@
     <row r="611">
       <c r="A611" s="9" t="inlineStr">
         <is>
-          <t>ISOHFR</t>
+          <t>ISOHFR
+电平转换器</t>
         </is>
       </c>
       <c r="B611" s="10" t="n"/>
@@ -7285,7 +7535,8 @@
     <row r="612">
       <c r="A612" s="9" t="inlineStr">
         <is>
-          <t>ISOL</t>
+          <t>ISOL
+电平转换器</t>
         </is>
       </c>
       <c r="B612" s="10" t="n"/>
@@ -7298,7 +7549,8 @@
     <row r="613">
       <c r="A613" s="9" t="inlineStr">
         <is>
-          <t>LHCNQ</t>
+          <t>LHCNQ
+锁存器</t>
         </is>
       </c>
       <c r="B613" s="10" t="inlineStr">
@@ -7311,7 +7563,8 @@
     <row r="614">
       <c r="A614" s="9" t="inlineStr">
         <is>
-          <t>LHCSNQ</t>
+          <t>LHCSNQ
+锁存器</t>
         </is>
       </c>
       <c r="B614" s="10" t="inlineStr">
@@ -7324,7 +7577,8 @@
     <row r="615">
       <c r="A615" s="2" t="inlineStr">
         <is>
-          <t>LHQ</t>
+          <t>LHQ
+锁存器</t>
         </is>
       </c>
       <c r="B615" s="11" t="inlineStr">
@@ -7346,7 +7600,8 @@
     <row r="617">
       <c r="A617" s="2" t="inlineStr">
         <is>
-          <t>LHSNQ</t>
+          <t>LHSNQ
+锁存器</t>
         </is>
       </c>
       <c r="B617" s="11" t="inlineStr">
@@ -7368,7 +7623,8 @@
     <row r="619">
       <c r="A619" s="9" t="inlineStr">
         <is>
-          <t>LNCNQ</t>
+          <t>LNCNQ
+锁存器</t>
         </is>
       </c>
       <c r="B619" s="10" t="inlineStr">
@@ -7381,7 +7637,8 @@
     <row r="620">
       <c r="A620" s="9" t="inlineStr">
         <is>
-          <t>LNCSNQ</t>
+          <t>LNCSNQ
+锁存器</t>
         </is>
       </c>
       <c r="B620" s="12" t="inlineStr">
@@ -7398,7 +7655,8 @@
     <row r="621">
       <c r="A621" s="9" t="inlineStr">
         <is>
-          <t>LNQ</t>
+          <t>LNQ
+锁存器</t>
         </is>
       </c>
       <c r="B621" s="10" t="inlineStr">
@@ -7411,7 +7669,8 @@
     <row r="622">
       <c r="A622" s="2" t="inlineStr">
         <is>
-          <t>LNSNQ</t>
+          <t>LNSNQ
+锁存器</t>
         </is>
       </c>
       <c r="B622" s="11" t="inlineStr">
@@ -7433,7 +7692,8 @@
     <row r="624">
       <c r="A624" s="2" t="inlineStr">
         <is>
-          <t>LVLHLBUFF</t>
+          <t>LVLHLBUFF
+电平转换器</t>
         </is>
       </c>
       <c r="B624" s="11" t="inlineStr">
@@ -7464,7 +7724,8 @@
     <row r="627">
       <c r="A627" s="2" t="inlineStr">
         <is>
-          <t>LVLHLCH</t>
+          <t>LVLHLCH
+电平转换器</t>
         </is>
       </c>
       <c r="B627" s="11" t="inlineStr">
@@ -7486,7 +7747,8 @@
     <row r="629">
       <c r="A629" s="2" t="inlineStr">
         <is>
-          <t>LVLHLCL</t>
+          <t>LVLHLCL
+电平转换器</t>
         </is>
       </c>
       <c r="B629" s="11" t="inlineStr">
@@ -7508,7 +7770,8 @@
     <row r="631">
       <c r="A631" s="2" t="inlineStr">
         <is>
-          <t>LVLLHBUFF</t>
+          <t>LVLLHBUFF
+电平转换器</t>
         </is>
       </c>
       <c r="B631" s="11" t="inlineStr">
@@ -7566,7 +7829,8 @@
     <row r="637">
       <c r="A637" s="2" t="inlineStr">
         <is>
-          <t>LVLLHCH</t>
+          <t>LVLLHCH
+电平转换器</t>
         </is>
       </c>
       <c r="B637" s="11" t="inlineStr">
@@ -7624,7 +7888,8 @@
     <row r="643">
       <c r="A643" s="2" t="inlineStr">
         <is>
-          <t>LVLLHCL</t>
+          <t>LVLLHCL
+电平转换器</t>
         </is>
       </c>
       <c r="B643" s="11" t="inlineStr">
@@ -7682,7 +7947,8 @@
     <row r="649">
       <c r="A649" s="2" t="inlineStr">
         <is>
-          <t>LVUAN2</t>
+          <t>LVUAN2
+电平转换器</t>
         </is>
       </c>
       <c r="B649" s="11" t="n"/>
@@ -7704,7 +7970,8 @@
     <row r="651">
       <c r="A651" s="2" t="inlineStr">
         <is>
-          <t>LVUFRAN2</t>
+          <t>LVUFRAN2
+电平转换器</t>
         </is>
       </c>
       <c r="B651" s="11" t="n"/>
@@ -7726,7 +7993,8 @@
     <row r="653">
       <c r="A653" s="2" t="inlineStr">
         <is>
-          <t>LVUFROR2N1</t>
+          <t>LVUFROR2N1
+电平转换器</t>
         </is>
       </c>
       <c r="B653" s="11" t="n"/>
@@ -7748,7 +8016,8 @@
     <row r="655">
       <c r="A655" s="2" t="inlineStr">
         <is>
-          <t>LVUOR2N1</t>
+          <t>LVUOR2N1
+电平转换器</t>
         </is>
       </c>
       <c r="B655" s="11" t="n"/>
@@ -7779,7 +8048,8 @@
     <row r="658">
       <c r="A658" s="2" t="inlineStr">
         <is>
-          <t>MAOI22</t>
+          <t>MAOI22
+复合逻辑门</t>
         </is>
       </c>
       <c r="B658" s="11" t="inlineStr">
@@ -7819,7 +8089,8 @@
     <row r="662">
       <c r="A662" s="2" t="inlineStr">
         <is>
-          <t>MAOI222</t>
+          <t>MAOI222
+复合逻辑门</t>
         </is>
       </c>
       <c r="B662" s="11" t="inlineStr">
@@ -7868,7 +8139,8 @@
     <row r="667">
       <c r="A667" s="2" t="inlineStr">
         <is>
-          <t>MB2LHCNQ</t>
+          <t>MB2LHCNQ
+多比特锁存器</t>
         </is>
       </c>
       <c r="B667" s="11" t="inlineStr">
@@ -7899,7 +8171,8 @@
     <row r="670">
       <c r="A670" s="2" t="inlineStr">
         <is>
-          <t>MB2LHQ</t>
+          <t>MB2LHQ
+多比特锁存器</t>
         </is>
       </c>
       <c r="B670" s="11" t="inlineStr">
@@ -7939,7 +8212,8 @@
     <row r="674">
       <c r="A674" s="9" t="inlineStr">
         <is>
-          <t>MB2LHSPCNQ</t>
+          <t>MB2LHSPCNQ
+多比特锁存器</t>
         </is>
       </c>
       <c r="B674" s="10" t="inlineStr">
@@ -7952,7 +8226,8 @@
     <row r="675">
       <c r="A675" s="2" t="inlineStr">
         <is>
-          <t>MB2LNCNQ</t>
+          <t>MB2LNCNQ
+多比特锁存器</t>
         </is>
       </c>
       <c r="B675" s="11" t="inlineStr">
@@ -7974,7 +8249,8 @@
     <row r="677">
       <c r="A677" s="2" t="inlineStr">
         <is>
-          <t>MB2LNQ</t>
+          <t>MB2LNQ
+多比特锁存器</t>
         </is>
       </c>
       <c r="B677" s="11" t="inlineStr">
@@ -8005,7 +8281,8 @@
     <row r="680">
       <c r="A680" s="9" t="inlineStr">
         <is>
-          <t>MB2LNSPCNQ</t>
+          <t>MB2LNSPCNQ
+多比特锁存器</t>
         </is>
       </c>
       <c r="B680" s="10" t="inlineStr">
@@ -8018,7 +8295,8 @@
     <row r="681">
       <c r="A681" s="2" t="inlineStr">
         <is>
-          <t>MB2SRLSDFKRPQ</t>
+          <t>MB2SRLSDFKRPQ
+多比特触发器</t>
         </is>
       </c>
       <c r="B681" s="11" t="inlineStr">
@@ -8040,7 +8318,8 @@
     <row r="683">
       <c r="A683" s="9" t="inlineStr">
         <is>
-          <t>MB2SRLSDFQ</t>
+          <t>MB2SRLSDFQ
+多比特触发器</t>
         </is>
       </c>
       <c r="B683" s="10" t="inlineStr">
@@ -8053,7 +8332,8 @@
     <row r="684">
       <c r="A684" s="2" t="inlineStr">
         <is>
-          <t>MB2SRLSDFRPQ</t>
+          <t>MB2SRLSDFRPQ
+多比特触发器</t>
         </is>
       </c>
       <c r="B684" s="11" t="inlineStr">
@@ -8075,7 +8355,8 @@
     <row r="686">
       <c r="A686" s="9" t="inlineStr">
         <is>
-          <t>MB2SRLSDFSNQ</t>
+          <t>MB2SRLSDFSNQ
+多比特触发器</t>
         </is>
       </c>
       <c r="B686" s="10" t="inlineStr">
@@ -8088,7 +8369,8 @@
     <row r="687">
       <c r="A687" s="9" t="inlineStr">
         <is>
-          <t>MB4LHQ</t>
+          <t>MB4LHQ
+多比特锁存器</t>
         </is>
       </c>
       <c r="B687" s="10" t="inlineStr">
@@ -8101,7 +8383,8 @@
     <row r="688">
       <c r="A688" s="9" t="inlineStr">
         <is>
-          <t>MB4LNQ</t>
+          <t>MB4LNQ
+多比特锁存器</t>
         </is>
       </c>
       <c r="B688" s="10" t="inlineStr">
@@ -8114,7 +8397,8 @@
     <row r="689">
       <c r="A689" s="9" t="inlineStr">
         <is>
-          <t>MB4SRLSDFKRPQ</t>
+          <t>MB4SRLSDFKRPQ
+多比特触发器</t>
         </is>
       </c>
       <c r="B689" s="10" t="inlineStr">
@@ -8127,7 +8411,8 @@
     <row r="690">
       <c r="A690" s="2" t="inlineStr">
         <is>
-          <t>MB4SRLSDFQ</t>
+          <t>MB4SRLSDFQ
+多比特触发器</t>
         </is>
       </c>
       <c r="B690" s="11" t="inlineStr">
@@ -8149,7 +8434,8 @@
     <row r="692">
       <c r="A692" s="2" t="inlineStr">
         <is>
-          <t>MB4SRLSDFRPQ</t>
+          <t>MB4SRLSDFRPQ
+多比特触发器</t>
         </is>
       </c>
       <c r="B692" s="11" t="inlineStr">
@@ -8171,7 +8457,8 @@
     <row r="694">
       <c r="A694" s="9" t="inlineStr">
         <is>
-          <t>MB4SRLSDFSNQ</t>
+          <t>MB4SRLSDFSNQ
+多比特触发器</t>
         </is>
       </c>
       <c r="B694" s="10" t="inlineStr">
@@ -8184,7 +8471,8 @@
     <row r="695">
       <c r="A695" s="9" t="inlineStr">
         <is>
-          <t>MCECNQ</t>
+          <t>MCECNQ
+多比特锁存器</t>
         </is>
       </c>
       <c r="B695" s="10" t="n"/>
@@ -8197,7 +8485,8 @@
     <row r="696">
       <c r="A696" s="2" t="inlineStr">
         <is>
-          <t>MOAI22</t>
+          <t>MOAI22
+复合逻辑门</t>
         </is>
       </c>
       <c r="B696" s="3" t="inlineStr">
@@ -8250,7 +8539,8 @@
     <row r="701">
       <c r="A701" s="2" t="inlineStr">
         <is>
-          <t>MUX2</t>
+          <t>MUX2
+多路选择器</t>
         </is>
       </c>
       <c r="B701" s="3" t="inlineStr">
@@ -8312,7 +8602,8 @@
     <row r="707">
       <c r="A707" s="2" t="inlineStr">
         <is>
-          <t>MUX2AOI</t>
+          <t>MUX2AOI
+复合多路选择器</t>
         </is>
       </c>
       <c r="B707" s="11" t="inlineStr">
@@ -8334,7 +8625,8 @@
     <row r="709">
       <c r="A709" s="9" t="inlineStr">
         <is>
-          <t>MUX2I</t>
+          <t>MUX2I
+反相多路选择器</t>
         </is>
       </c>
       <c r="B709" s="10" t="inlineStr">
@@ -8347,7 +8639,8 @@
     <row r="710">
       <c r="A710" s="2" t="inlineStr">
         <is>
-          <t>MUX2ND2</t>
+          <t>MUX2ND2
+复合多路选择器</t>
         </is>
       </c>
       <c r="B710" s="11" t="inlineStr">
@@ -8387,7 +8680,8 @@
     <row r="714">
       <c r="A714" s="2" t="inlineStr">
         <is>
-          <t>MUX2NND2</t>
+          <t>MUX2NND2
+复合多路选择器</t>
         </is>
       </c>
       <c r="B714" s="11" t="inlineStr">
@@ -8418,7 +8712,8 @@
     <row r="717">
       <c r="A717" s="2" t="inlineStr">
         <is>
-          <t>MUX2NNR2</t>
+          <t>MUX2NNR2
+复合多路选择器</t>
         </is>
       </c>
       <c r="B717" s="11" t="inlineStr">
@@ -8440,7 +8735,8 @@
     <row r="719">
       <c r="A719" s="2" t="inlineStr">
         <is>
-          <t>MUX2NR2</t>
+          <t>MUX2NR2
+复合多路选择器</t>
         </is>
       </c>
       <c r="B719" s="11" t="inlineStr">
@@ -8471,7 +8767,8 @@
     <row r="722">
       <c r="A722" s="2" t="inlineStr">
         <is>
-          <t>MUX3</t>
+          <t>MUX3
+多路选择器</t>
         </is>
       </c>
       <c r="B722" s="3" t="inlineStr">
@@ -8506,7 +8803,8 @@
     <row r="725">
       <c r="A725" s="9" t="inlineStr">
         <is>
-          <t>MUX3ND1</t>
+          <t>MUX3ND1
+复合多路选择器</t>
         </is>
       </c>
       <c r="B725" s="10" t="inlineStr">
@@ -8519,7 +8817,8 @@
     <row r="726">
       <c r="A726" s="2" t="inlineStr">
         <is>
-          <t>MUX4</t>
+          <t>MUX4
+多路选择器</t>
         </is>
       </c>
       <c r="B726" s="11" t="inlineStr">
@@ -8550,7 +8849,8 @@
     <row r="729">
       <c r="A729" s="9" t="inlineStr">
         <is>
-          <t>MUX4N</t>
+          <t>MUX4N
+多路选择器</t>
         </is>
       </c>
       <c r="B729" s="10" t="n"/>
@@ -8563,7 +8863,8 @@
     <row r="730">
       <c r="A730" s="2" t="inlineStr">
         <is>
-          <t>MUX8</t>
+          <t>MUX8
+多路选择器</t>
         </is>
       </c>
       <c r="B730" s="11" t="inlineStr">
@@ -8585,7 +8886,8 @@
     <row r="732">
       <c r="A732" s="2" t="inlineStr">
         <is>
-          <t>MX2</t>
+          <t>MX2
+多路选择器</t>
         </is>
       </c>
       <c r="B732" s="11" t="n"/>
@@ -8616,7 +8918,8 @@
     <row r="735">
       <c r="A735" s="2" t="inlineStr">
         <is>
-          <t>MXI2</t>
+          <t>MXI2
+反相多路选择器</t>
         </is>
       </c>
       <c r="B735" s="11" t="n"/>
@@ -8728,7 +9031,8 @@
     <row r="747">
       <c r="A747" s="2" t="inlineStr">
         <is>
-          <t>ND2</t>
+          <t>ND2
+与非门</t>
         </is>
       </c>
       <c r="B747" s="3" t="inlineStr">
@@ -9041,7 +9345,8 @@
     <row r="780">
       <c r="A780" s="2" t="inlineStr">
         <is>
-          <t>ND2AOI21</t>
+          <t>ND2AOI21
+复合逻辑门</t>
         </is>
       </c>
       <c r="B780" s="11" t="inlineStr">
@@ -9063,7 +9368,8 @@
     <row r="782">
       <c r="A782" s="2" t="inlineStr">
         <is>
-          <t>ND2IOA21</t>
+          <t>ND2IOA21
+与非门</t>
         </is>
       </c>
       <c r="B782" s="11" t="inlineStr">
@@ -9094,7 +9400,8 @@
     <row r="785">
       <c r="A785" s="2" t="inlineStr">
         <is>
-          <t>ND2N1</t>
+          <t>ND2N1
+与非门</t>
         </is>
       </c>
       <c r="B785" s="11" t="n"/>
@@ -9143,7 +9450,8 @@
     <row r="790">
       <c r="A790" s="2" t="inlineStr">
         <is>
-          <t>ND2OAI21</t>
+          <t>ND2OAI21
+复合逻辑门</t>
         </is>
       </c>
       <c r="B790" s="11" t="inlineStr">
@@ -9165,7 +9473,8 @@
     <row r="792">
       <c r="A792" s="2" t="inlineStr">
         <is>
-          <t>ND3</t>
+          <t>ND3
+与非门</t>
         </is>
       </c>
       <c r="B792" s="11" t="inlineStr">
@@ -9205,7 +9514,8 @@
     <row r="796">
       <c r="A796" s="2" t="inlineStr">
         <is>
-          <t>ND3N1</t>
+          <t>ND3N1
+与非门</t>
         </is>
       </c>
       <c r="B796" s="11" t="n"/>
@@ -9227,7 +9537,8 @@
     <row r="798">
       <c r="A798" s="9" t="inlineStr">
         <is>
-          <t>ND3N2</t>
+          <t>ND3N2
+与非门</t>
         </is>
       </c>
       <c r="B798" s="10" t="n"/>
@@ -9240,7 +9551,8 @@
     <row r="799">
       <c r="A799" s="2" t="inlineStr">
         <is>
-          <t>ND4</t>
+          <t>ND4
+与非门</t>
         </is>
       </c>
       <c r="B799" s="11" t="inlineStr">
@@ -9271,7 +9583,8 @@
     <row r="802">
       <c r="A802" s="9" t="inlineStr">
         <is>
-          <t>ND4N1</t>
+          <t>ND4N1
+与非门</t>
         </is>
       </c>
       <c r="B802" s="10" t="n"/>
@@ -9284,7 +9597,8 @@
     <row r="803">
       <c r="A803" s="2" t="inlineStr">
         <is>
-          <t>NR2</t>
+          <t>NR2
+或非门</t>
         </is>
       </c>
       <c r="B803" s="3" t="inlineStr">
@@ -9697,7 +10011,8 @@
     <row r="848">
       <c r="A848" s="2" t="inlineStr">
         <is>
-          <t>NR2AOI21</t>
+          <t>NR2AOI21
+复合逻辑门</t>
         </is>
       </c>
       <c r="B848" s="11" t="inlineStr">
@@ -9719,7 +10034,8 @@
     <row r="850">
       <c r="A850" s="2" t="inlineStr">
         <is>
-          <t>NR2N1</t>
+          <t>NR2N1
+或非门</t>
         </is>
       </c>
       <c r="B850" s="11" t="n"/>
@@ -9813,7 +10129,8 @@
     <row r="860">
       <c r="A860" s="2" t="inlineStr">
         <is>
-          <t>NR2ND2</t>
+          <t>NR2ND2
+或非门</t>
         </is>
       </c>
       <c r="B860" s="11" t="inlineStr">
@@ -9844,7 +10161,8 @@
     <row r="863">
       <c r="A863" s="2" t="inlineStr">
         <is>
-          <t>NR3</t>
+          <t>NR3
+或非门</t>
         </is>
       </c>
       <c r="B863" s="3" t="inlineStr">
@@ -9969,7 +10287,8 @@
     <row r="876">
       <c r="A876" s="2" t="inlineStr">
         <is>
-          <t>NR4</t>
+          <t>NR4
+或非门</t>
         </is>
       </c>
       <c r="B876" s="11" t="inlineStr">
@@ -10072,7 +10391,8 @@
     <row r="887">
       <c r="A887" s="2" t="inlineStr">
         <is>
-          <t>OA21</t>
+          <t>OA21
+或与门</t>
         </is>
       </c>
       <c r="B887" s="3" t="inlineStr">
@@ -10125,7 +10445,8 @@
     <row r="892">
       <c r="A892" s="2" t="inlineStr">
         <is>
-          <t>OA211</t>
+          <t>OA211
+或与门</t>
         </is>
       </c>
       <c r="B892" s="11" t="inlineStr">
@@ -10183,7 +10504,8 @@
     <row r="898">
       <c r="A898" s="2" t="inlineStr">
         <is>
-          <t>OA22</t>
+          <t>OA22
+或与门</t>
         </is>
       </c>
       <c r="B898" s="3" t="inlineStr">
@@ -10254,7 +10576,8 @@
     <row r="905">
       <c r="A905" s="2" t="inlineStr">
         <is>
-          <t>OA222</t>
+          <t>OA222
+或与门</t>
         </is>
       </c>
       <c r="B905" s="11" t="inlineStr">
@@ -10303,7 +10626,8 @@
     <row r="910">
       <c r="A910" s="9" t="inlineStr">
         <is>
-          <t>OA2222</t>
+          <t>OA2222
+或与门</t>
         </is>
       </c>
       <c r="B910" s="10" t="inlineStr">
@@ -10316,7 +10640,8 @@
     <row r="911">
       <c r="A911" s="2" t="inlineStr">
         <is>
-          <t>OAI21</t>
+          <t>OAI21
+或与非门</t>
         </is>
       </c>
       <c r="B911" s="11" t="inlineStr">
@@ -10482,7 +10807,8 @@
     <row r="929">
       <c r="A929" s="2" t="inlineStr">
         <is>
-          <t>OAI211</t>
+          <t>OAI211
+或与非门</t>
         </is>
       </c>
       <c r="B929" s="11" t="inlineStr">
@@ -10612,7 +10938,8 @@
     <row r="943">
       <c r="A943" s="2" t="inlineStr">
         <is>
-          <t>OAI2111</t>
+          <t>OAI2111
+或与非门</t>
         </is>
       </c>
       <c r="B943" s="11" t="inlineStr">
@@ -10634,7 +10961,8 @@
     <row r="945">
       <c r="A945" s="9" t="inlineStr">
         <is>
-          <t>OAI211INV</t>
+          <t>OAI211INV
+复合逻辑门</t>
         </is>
       </c>
       <c r="B945" s="10" t="inlineStr">
@@ -10647,7 +10975,8 @@
     <row r="946">
       <c r="A946" s="9" t="inlineStr">
         <is>
-          <t>OAI21AOI21</t>
+          <t>OAI21AOI21
+复合逻辑门</t>
         </is>
       </c>
       <c r="B946" s="10" t="n"/>
@@ -10660,7 +10989,8 @@
     <row r="947">
       <c r="A947" s="2" t="inlineStr">
         <is>
-          <t>OAI21AOI22</t>
+          <t>OAI21AOI22
+复合逻辑门</t>
         </is>
       </c>
       <c r="B947" s="11" t="inlineStr">
@@ -10691,7 +11021,8 @@
     <row r="950">
       <c r="A950" s="2" t="inlineStr">
         <is>
-          <t>OAI21N2</t>
+          <t>OAI21N2
+或与非门</t>
         </is>
       </c>
       <c r="B950" s="11" t="n"/>
@@ -10731,7 +11062,8 @@
     <row r="954">
       <c r="A954" s="2" t="inlineStr">
         <is>
-          <t>OAI21ND2</t>
+          <t>OAI21ND2
+或与非门</t>
         </is>
       </c>
       <c r="B954" s="11" t="inlineStr">
@@ -10798,7 +11130,8 @@
     <row r="961">
       <c r="A961" s="2" t="inlineStr">
         <is>
-          <t>OAI21NR2</t>
+          <t>OAI21NR2
+或与非门</t>
         </is>
       </c>
       <c r="B961" s="11" t="inlineStr">
@@ -10838,7 +11171,8 @@
     <row r="965">
       <c r="A965" s="9" t="inlineStr">
         <is>
-          <t>OAI21OAI21</t>
+          <t>OAI21OAI21
+复合逻辑门</t>
         </is>
       </c>
       <c r="B965" s="10" t="n"/>
@@ -10851,7 +11185,8 @@
     <row r="966">
       <c r="A966" s="2" t="inlineStr">
         <is>
-          <t>OAI22</t>
+          <t>OAI22
+或与非门</t>
         </is>
       </c>
       <c r="B966" s="3" t="inlineStr">
@@ -10971,7 +11306,8 @@
     <row r="978">
       <c r="A978" s="2" t="inlineStr">
         <is>
-          <t>OAI221</t>
+          <t>OAI221
+或与非门</t>
         </is>
       </c>
       <c r="B978" s="3" t="inlineStr">
@@ -11028,7 +11364,8 @@
     <row r="983">
       <c r="A983" s="2" t="inlineStr">
         <is>
-          <t>OAI2211</t>
+          <t>OAI2211
+或与非门</t>
         </is>
       </c>
       <c r="B983" s="11" t="inlineStr">
@@ -11050,7 +11387,8 @@
     <row r="985">
       <c r="A985" s="2" t="inlineStr">
         <is>
-          <t>OAI222</t>
+          <t>OAI222
+或与非门</t>
         </is>
       </c>
       <c r="B985" s="3" t="inlineStr">
@@ -11098,7 +11436,8 @@
     <row r="989">
       <c r="A989" s="2" t="inlineStr">
         <is>
-          <t>OAI2221</t>
+          <t>OAI2221
+或与非门</t>
         </is>
       </c>
       <c r="B989" s="11" t="inlineStr">
@@ -11120,7 +11459,8 @@
     <row r="991">
       <c r="A991" s="2" t="inlineStr">
         <is>
-          <t>OAI2222</t>
+          <t>OAI2222
+或与非门</t>
         </is>
       </c>
       <c r="B991" s="11" t="inlineStr">
@@ -11205,7 +11545,8 @@
     <row r="1000">
       <c r="A1000" s="2" t="inlineStr">
         <is>
-          <t>OAI22AOI21</t>
+          <t>OAI22AOI21
+复合逻辑门</t>
         </is>
       </c>
       <c r="B1000" s="11" t="inlineStr">
@@ -11245,7 +11586,8 @@
     <row r="1004">
       <c r="A1004" s="2" t="inlineStr">
         <is>
-          <t>OAI22INV</t>
+          <t>OAI22INV
+复合逻辑门</t>
         </is>
       </c>
       <c r="B1004" s="11" t="inlineStr">
@@ -11267,7 +11609,8 @@
     <row r="1006">
       <c r="A1006" s="2" t="inlineStr">
         <is>
-          <t>OAI22ND2</t>
+          <t>OAI22ND2
+或与非门</t>
         </is>
       </c>
       <c r="B1006" s="11" t="inlineStr">
@@ -11289,7 +11632,8 @@
     <row r="1008">
       <c r="A1008" s="2" t="inlineStr">
         <is>
-          <t>OAI22NR2</t>
+          <t>OAI22NR2
+或与非门</t>
         </is>
       </c>
       <c r="B1008" s="11" t="inlineStr">
@@ -11311,7 +11655,8 @@
     <row r="1010">
       <c r="A1010" s="9" t="inlineStr">
         <is>
-          <t>OAI22OAI21</t>
+          <t>OAI22OAI21
+复合逻辑门</t>
         </is>
       </c>
       <c r="B1010" s="10" t="n"/>
@@ -11324,7 +11669,8 @@
     <row r="1011">
       <c r="A1011" s="2" t="inlineStr">
         <is>
-          <t>OAI31</t>
+          <t>OAI31
+或与非门</t>
         </is>
       </c>
       <c r="B1011" s="11" t="inlineStr">
@@ -11373,7 +11719,8 @@
     <row r="1016">
       <c r="A1016" s="2" t="inlineStr">
         <is>
-          <t>OAI311</t>
+          <t>OAI311
+或与非门</t>
         </is>
       </c>
       <c r="B1016" s="3" t="inlineStr">
@@ -11426,7 +11773,8 @@
     <row r="1021">
       <c r="A1021" s="2" t="inlineStr">
         <is>
-          <t>OAI32</t>
+          <t>OAI32
+或与非门</t>
         </is>
       </c>
       <c r="B1021" s="3" t="inlineStr">
@@ -11479,7 +11827,8 @@
     <row r="1026">
       <c r="A1026" s="2" t="inlineStr">
         <is>
-          <t>OAI321</t>
+          <t>OAI321
+或与非门</t>
         </is>
       </c>
       <c r="B1026" s="11" t="inlineStr">
@@ -11519,7 +11868,8 @@
     <row r="1030">
       <c r="A1030" s="2" t="inlineStr">
         <is>
-          <t>OAI33</t>
+          <t>OAI33
+或与非门</t>
         </is>
       </c>
       <c r="B1030" s="11" t="inlineStr">
@@ -11550,7 +11900,8 @@
     <row r="1033">
       <c r="A1033" s="2" t="inlineStr">
         <is>
-          <t>OAOI211</t>
+          <t>OAOI211
+复合逻辑门</t>
         </is>
       </c>
       <c r="B1033" s="3" t="inlineStr">
@@ -11585,7 +11936,8 @@
     <row r="1036">
       <c r="A1036" s="2" t="inlineStr">
         <is>
-          <t>OIAI21</t>
+          <t>OIAI21
+复合逻辑门</t>
         </is>
       </c>
       <c r="B1036" s="3" t="inlineStr">
@@ -11638,7 +11990,8 @@
     <row r="1041">
       <c r="A1041" s="2" t="inlineStr">
         <is>
-          <t>OR2</t>
+          <t>OR2
+或门</t>
         </is>
       </c>
       <c r="B1041" s="3" t="inlineStr">
@@ -11897,7 +12250,8 @@
     <row r="1068">
       <c r="A1068" s="2" t="inlineStr">
         <is>
-          <t>OR3</t>
+          <t>OR3
+或门</t>
         </is>
       </c>
       <c r="B1068" s="3" t="inlineStr">
@@ -11984,7 +12338,8 @@
     <row r="1075">
       <c r="A1075" s="2" t="inlineStr">
         <is>
-          <t>OR4</t>
+          <t>OR4
+或门</t>
         </is>
       </c>
       <c r="B1075" s="3" t="inlineStr">
@@ -12073,7 +12428,8 @@
     <row r="1084">
       <c r="A1084" s="9" t="inlineStr">
         <is>
-          <t>RSDFQ</t>
+          <t>RSDFQ
+扫描触发器</t>
         </is>
       </c>
       <c r="B1084" s="10" t="n"/>
@@ -12086,7 +12442,8 @@
     <row r="1085">
       <c r="A1085" s="9" t="inlineStr">
         <is>
-          <t>RSDFRPQ</t>
+          <t>RSDFRPQ
+扫描触发器</t>
         </is>
       </c>
       <c r="B1085" s="10" t="n"/>
@@ -12099,7 +12456,8 @@
     <row r="1086">
       <c r="A1086" s="9" t="inlineStr">
         <is>
-          <t>RSDFSNQ</t>
+          <t>RSDFSNQ
+扫描触发器</t>
         </is>
       </c>
       <c r="B1086" s="10" t="n"/>
@@ -12112,7 +12470,8 @@
     <row r="1087">
       <c r="A1087" s="9" t="inlineStr">
         <is>
-          <t>RSDFSRPQ</t>
+          <t>RSDFSRPQ
+扫描触发器</t>
         </is>
       </c>
       <c r="B1087" s="10" t="n"/>
@@ -12125,7 +12484,8 @@
     <row r="1088">
       <c r="A1088" s="9" t="inlineStr">
         <is>
-          <t>SD2FFQN</t>
+          <t>SD2FFQN
+扫描触发器</t>
         </is>
       </c>
       <c r="B1088" s="10" t="n"/>
@@ -12138,7 +12498,8 @@
     <row r="1089">
       <c r="A1089" s="9" t="inlineStr">
         <is>
-          <t>SDFFACPQ</t>
+          <t>SDFFACPQ
+扫描触发器</t>
         </is>
       </c>
       <c r="B1089" s="10" t="n"/>
@@ -12151,7 +12512,8 @@
     <row r="1090">
       <c r="A1090" s="9" t="inlineStr">
         <is>
-          <t>SDFFASNQ</t>
+          <t>SDFFASNQ
+扫描触发器</t>
         </is>
       </c>
       <c r="B1090" s="10" t="n"/>
@@ -12164,7 +12526,8 @@
     <row r="1091">
       <c r="A1091" s="9" t="inlineStr">
         <is>
-          <t>SDFFEACPQ</t>
+          <t>SDFFEACPQ
+扫描触发器</t>
         </is>
       </c>
       <c r="B1091" s="10" t="n"/>
@@ -12177,7 +12540,8 @@
     <row r="1092">
       <c r="A1092" s="2" t="inlineStr">
         <is>
-          <t>SDFFQ</t>
+          <t>SDFFQ
+扫描触发器</t>
         </is>
       </c>
       <c r="B1092" s="11" t="n"/>
@@ -12217,7 +12581,8 @@
     <row r="1096">
       <c r="A1096" s="2" t="inlineStr">
         <is>
-          <t>SDFFQN</t>
+          <t>SDFFQN
+扫描触发器</t>
         </is>
       </c>
       <c r="B1096" s="11" t="n"/>
@@ -12257,7 +12622,8 @@
     <row r="1100">
       <c r="A1100" s="2" t="inlineStr">
         <is>
-          <t>SDFKRPQ</t>
+          <t>SDFKRPQ
+扫描触发器</t>
         </is>
       </c>
       <c r="B1100" s="11" t="inlineStr">
@@ -12279,7 +12645,8 @@
     <row r="1102">
       <c r="A1102" s="9" t="inlineStr">
         <is>
-          <t>SDFKSNQ</t>
+          <t>SDFKSNQ
+扫描触发器</t>
         </is>
       </c>
       <c r="B1102" s="10" t="inlineStr">
@@ -12292,7 +12659,8 @@
     <row r="1103">
       <c r="A1103" s="2" t="inlineStr">
         <is>
-          <t>SDFKSRPQ</t>
+          <t>SDFKSRPQ
+扫描触发器</t>
         </is>
       </c>
       <c r="B1103" s="11" t="inlineStr">
@@ -12314,7 +12682,8 @@
     <row r="1105">
       <c r="A1105" s="2" t="inlineStr">
         <is>
-          <t>SDFMQ</t>
+          <t>SDFMQ
+扫描触发器</t>
         </is>
       </c>
       <c r="B1105" s="11" t="inlineStr">
@@ -12336,7 +12705,8 @@
     <row r="1107">
       <c r="A1107" s="2" t="inlineStr">
         <is>
-          <t>SDFNQ</t>
+          <t>SDFNQ
+扫描触发器</t>
         </is>
       </c>
       <c r="B1107" s="11" t="inlineStr">
@@ -12358,7 +12728,8 @@
     <row r="1109">
       <c r="A1109" s="9" t="inlineStr">
         <is>
-          <t>SDFNQND2</t>
+          <t>SDFNQND2
+扫描触发器</t>
         </is>
       </c>
       <c r="B1109" s="10" t="inlineStr">
@@ -12371,7 +12742,8 @@
     <row r="1110">
       <c r="A1110" s="9" t="inlineStr">
         <is>
-          <t>SDFNRPQ</t>
+          <t>SDFNRPQ
+扫描触发器</t>
         </is>
       </c>
       <c r="B1110" s="10" t="inlineStr">
@@ -12384,7 +12756,8 @@
     <row r="1111">
       <c r="A1111" s="2" t="inlineStr">
         <is>
-          <t>SDFNRPQND2</t>
+          <t>SDFNRPQND2
+扫描触发器</t>
         </is>
       </c>
       <c r="B1111" s="11" t="inlineStr">
@@ -12406,7 +12779,8 @@
     <row r="1113">
       <c r="A1113" s="2" t="inlineStr">
         <is>
-          <t>SDFNSNQ</t>
+          <t>SDFNSNQ
+扫描触发器</t>
         </is>
       </c>
       <c r="B1113" s="11" t="inlineStr">
@@ -12428,7 +12802,8 @@
     <row r="1115">
       <c r="A1115" s="9" t="inlineStr">
         <is>
-          <t>SDFNSNQND0</t>
+          <t>SDFNSNQND0
+扫描触发器</t>
         </is>
       </c>
       <c r="B1115" s="10" t="n"/>
@@ -12441,7 +12816,8 @@
     <row r="1116">
       <c r="A1116" s="9" t="inlineStr">
         <is>
-          <t>SDFNSNQND1</t>
+          <t>SDFNSNQND1
+扫描触发器</t>
         </is>
       </c>
       <c r="B1116" s="10" t="inlineStr">
@@ -12454,7 +12830,8 @@
     <row r="1117">
       <c r="A1117" s="9" t="inlineStr">
         <is>
-          <t>SDFNSRPQ</t>
+          <t>SDFNSRPQ
+扫描触发器</t>
         </is>
       </c>
       <c r="B1117" s="10" t="inlineStr">
@@ -12467,7 +12844,8 @@
     <row r="1118">
       <c r="A1118" s="2" t="inlineStr">
         <is>
-          <t>SDFQ</t>
+          <t>SDFQ
+扫描触发器</t>
         </is>
       </c>
       <c r="B1118" s="11" t="inlineStr">
@@ -12516,7 +12894,8 @@
     <row r="1123">
       <c r="A1123" s="9" t="inlineStr">
         <is>
-          <t>SDFQND1</t>
+          <t>SDFQND1
+扫描触发器</t>
         </is>
       </c>
       <c r="B1123" s="10" t="inlineStr">
@@ -12529,7 +12908,8 @@
     <row r="1124">
       <c r="A1124" s="9" t="inlineStr">
         <is>
-          <t>SDFQND2</t>
+          <t>SDFQND2
+扫描触发器</t>
         </is>
       </c>
       <c r="B1124" s="10" t="n"/>
@@ -12542,7 +12922,8 @@
     <row r="1125">
       <c r="A1125" s="2" t="inlineStr">
         <is>
-          <t>SDFRPQ</t>
+          <t>SDFRPQ
+扫描触发器</t>
         </is>
       </c>
       <c r="B1125" s="11" t="inlineStr">
@@ -12600,7 +12981,8 @@
     <row r="1131">
       <c r="A1131" s="9" t="inlineStr">
         <is>
-          <t>SDFRPQND4</t>
+          <t>SDFRPQND4
+扫描触发器</t>
         </is>
       </c>
       <c r="B1131" s="10" t="inlineStr">
@@ -12613,7 +12995,8 @@
     <row r="1132">
       <c r="A1132" s="9" t="inlineStr">
         <is>
-          <t>SDFSNQ</t>
+          <t>SDFSNQ
+扫描触发器</t>
         </is>
       </c>
       <c r="B1132" s="10" t="inlineStr">
@@ -12626,7 +13009,8 @@
     <row r="1133">
       <c r="A1133" s="9" t="inlineStr">
         <is>
-          <t>SDFSNQND2</t>
+          <t>SDFSNQND2
+扫描触发器</t>
         </is>
       </c>
       <c r="B1133" s="10" t="n"/>
@@ -12639,7 +13023,8 @@
     <row r="1134">
       <c r="A1134" s="9" t="inlineStr">
         <is>
-          <t>SDFSNQND4</t>
+          <t>SDFSNQND4
+扫描触发器</t>
         </is>
       </c>
       <c r="B1134" s="10" t="inlineStr">
@@ -12652,7 +13037,8 @@
     <row r="1135">
       <c r="A1135" s="2" t="inlineStr">
         <is>
-          <t>SDFSRPQ</t>
+          <t>SDFSRPQ
+扫描触发器</t>
         </is>
       </c>
       <c r="B1135" s="11" t="inlineStr">
@@ -12674,7 +13060,8 @@
     <row r="1137">
       <c r="A1137" s="9" t="inlineStr">
         <is>
-          <t>SDFSYNC1Q</t>
+          <t>SDFSYNC1Q
+同步触发器</t>
         </is>
       </c>
       <c r="B1137" s="10" t="n"/>
@@ -12687,7 +13074,8 @@
     <row r="1138">
       <c r="A1138" s="9" t="inlineStr">
         <is>
-          <t>SDFSYNC1RPQ</t>
+          <t>SDFSYNC1RPQ
+同步触发器</t>
         </is>
       </c>
       <c r="B1138" s="10" t="n"/>
@@ -12700,7 +13088,8 @@
     <row r="1139">
       <c r="A1139" s="2" t="inlineStr">
         <is>
-          <t>SEDFQ</t>
+          <t>SEDFQ
+扫描触发器</t>
         </is>
       </c>
       <c r="B1139" s="11" t="inlineStr">
@@ -12722,7 +13111,8 @@
     <row r="1141">
       <c r="A1141" s="2" t="inlineStr">
         <is>
-          <t>SEDFRPQ</t>
+          <t>SEDFRPQ
+扫描触发器</t>
         </is>
       </c>
       <c r="B1141" s="11" t="inlineStr">
@@ -12744,7 +13134,8 @@
     <row r="1143">
       <c r="A1143" s="2" t="inlineStr">
         <is>
-          <t>SYNLHCNQ</t>
+          <t>SYNLHCNQ
+同步器</t>
         </is>
       </c>
       <c r="B1143" s="11" t="inlineStr">
@@ -12766,7 +13157,8 @@
     <row r="1145">
       <c r="A1145" s="9" t="inlineStr">
         <is>
-          <t>SYNLHQ</t>
+          <t>SYNLHQ
+同步器</t>
         </is>
       </c>
       <c r="B1145" s="12" t="inlineStr">
@@ -12783,7 +13175,8 @@
     <row r="1146">
       <c r="A1146" s="9" t="inlineStr">
         <is>
-          <t>SYNLHSNQ</t>
+          <t>SYNLHSNQ
+同步器</t>
         </is>
       </c>
       <c r="B1146" s="10" t="inlineStr">
@@ -12796,7 +13189,8 @@
     <row r="1147">
       <c r="A1147" s="2" t="inlineStr">
         <is>
-          <t>TAPCELL</t>
+          <t>TAPCELL
+阱敲击单元</t>
         </is>
       </c>
       <c r="B1147" s="3" t="inlineStr">
@@ -12822,7 +13216,8 @@
     <row r="1149">
       <c r="A1149" s="9" t="inlineStr">
         <is>
-          <t>TIEHXP</t>
+          <t>TIEHXP
+电平钳位</t>
         </is>
       </c>
       <c r="B1149" s="10" t="inlineStr">
@@ -12835,7 +13230,8 @@
     <row r="1150">
       <c r="A1150" s="9" t="inlineStr">
         <is>
-          <t>TIELXN</t>
+          <t>TIELXN
+电平钳位</t>
         </is>
       </c>
       <c r="B1150" s="12" t="inlineStr">
@@ -12852,7 +13248,8 @@
     <row r="1151">
       <c r="A1151" s="2" t="inlineStr">
         <is>
-          <t>W2AO22</t>
+          <t>W2AO22
+复合逻辑门</t>
         </is>
       </c>
       <c r="B1151" s="11" t="n"/>
@@ -12874,7 +13271,8 @@
     <row r="1153">
       <c r="A1153" s="9" t="inlineStr">
         <is>
-          <t>WAO22OA22</t>
+          <t>WAO22OA22
+复合逻辑门</t>
         </is>
       </c>
       <c r="B1153" s="10" t="n"/>
@@ -12887,7 +13285,8 @@
     <row r="1154">
       <c r="A1154" s="2" t="inlineStr">
         <is>
-          <t>XNR2</t>
+          <t>XNR2
+同或门</t>
         </is>
       </c>
       <c r="B1154" s="3" t="inlineStr">
@@ -13057,7 +13456,8 @@
     <row r="1172">
       <c r="A1172" s="2" t="inlineStr">
         <is>
-          <t>XNR2AOI21</t>
+          <t>XNR2AOI21
+复合逻辑门</t>
         </is>
       </c>
       <c r="B1172" s="11" t="inlineStr">
@@ -13088,7 +13488,8 @@
     <row r="1175">
       <c r="A1175" s="2" t="inlineStr">
         <is>
-          <t>XNR2AOI22</t>
+          <t>XNR2AOI22
+复合逻辑门</t>
         </is>
       </c>
       <c r="B1175" s="11" t="inlineStr">
@@ -13128,7 +13529,8 @@
     <row r="1179">
       <c r="A1179" s="2" t="inlineStr">
         <is>
-          <t>XNR2ND2</t>
+          <t>XNR2ND2
+同或门</t>
         </is>
       </c>
       <c r="B1179" s="11" t="inlineStr">
@@ -13159,7 +13561,8 @@
     <row r="1182">
       <c r="A1182" s="2" t="inlineStr">
         <is>
-          <t>XNR2NR2</t>
+          <t>XNR2NR2
+同或门</t>
         </is>
       </c>
       <c r="B1182" s="11" t="inlineStr">
@@ -13181,7 +13584,8 @@
     <row r="1184">
       <c r="A1184" s="9" t="inlineStr">
         <is>
-          <t>XNR2OAI21</t>
+          <t>XNR2OAI21
+复合逻辑门</t>
         </is>
       </c>
       <c r="B1184" s="10" t="inlineStr">
@@ -13194,7 +13598,8 @@
     <row r="1185">
       <c r="A1185" s="2" t="inlineStr">
         <is>
-          <t>XNR2OAI22</t>
+          <t>XNR2OAI22
+复合逻辑门</t>
         </is>
       </c>
       <c r="B1185" s="11" t="inlineStr">
@@ -13234,7 +13639,8 @@
     <row r="1189">
       <c r="A1189" s="9" t="inlineStr">
         <is>
-          <t>XNR2XNR2</t>
+          <t>XNR2XNR2
+复合逻辑门</t>
         </is>
       </c>
       <c r="B1189" s="10" t="inlineStr">
@@ -13247,7 +13653,8 @@
     <row r="1190">
       <c r="A1190" s="9" t="inlineStr">
         <is>
-          <t>XNR2XOR2</t>
+          <t>XNR2XOR2
+复合逻辑门</t>
         </is>
       </c>
       <c r="B1190" s="10" t="inlineStr">
@@ -13260,7 +13667,8 @@
     <row r="1191">
       <c r="A1191" s="2" t="inlineStr">
         <is>
-          <t>XNR3</t>
+          <t>XNR3
+同或门</t>
         </is>
       </c>
       <c r="B1191" s="11" t="inlineStr">
@@ -13309,7 +13717,8 @@
     <row r="1196">
       <c r="A1196" s="2" t="inlineStr">
         <is>
-          <t>XNR4</t>
+          <t>XNR4
+同或门</t>
         </is>
       </c>
       <c r="B1196" s="11" t="inlineStr">
@@ -13358,7 +13767,8 @@
     <row r="1201">
       <c r="A1201" s="2" t="inlineStr">
         <is>
-          <t>XOR2</t>
+          <t>XOR2
+异或门</t>
         </is>
       </c>
       <c r="B1201" s="3" t="inlineStr">
@@ -13523,7 +13933,8 @@
     <row r="1218">
       <c r="A1218" s="9" t="inlineStr">
         <is>
-          <t>XOR2AOI21</t>
+          <t>XOR2AOI21
+复合逻辑门</t>
         </is>
       </c>
       <c r="B1218" s="10" t="inlineStr">
@@ -13536,7 +13947,8 @@
     <row r="1219">
       <c r="A1219" s="2" t="inlineStr">
         <is>
-          <t>XOR2AOI22</t>
+          <t>XOR2AOI22
+复合逻辑门</t>
         </is>
       </c>
       <c r="B1219" s="11" t="inlineStr">
@@ -13585,7 +13997,8 @@
     <row r="1224">
       <c r="A1224" s="2" t="inlineStr">
         <is>
-          <t>XOR2ND2</t>
+          <t>XOR2ND2
+异或门</t>
         </is>
       </c>
       <c r="B1224" s="11" t="inlineStr">
@@ -13625,7 +14038,8 @@
     <row r="1228">
       <c r="A1228" s="2" t="inlineStr">
         <is>
-          <t>XOR2NR2</t>
+          <t>XOR2NR2
+异或门</t>
         </is>
       </c>
       <c r="B1228" s="11" t="inlineStr">
@@ -13656,7 +14070,8 @@
     <row r="1231">
       <c r="A1231" s="9" t="inlineStr">
         <is>
-          <t>XOR2OAI21</t>
+          <t>XOR2OAI21
+复合逻辑门</t>
         </is>
       </c>
       <c r="B1231" s="10" t="inlineStr">
@@ -13669,7 +14084,8 @@
     <row r="1232">
       <c r="A1232" s="2" t="inlineStr">
         <is>
-          <t>XOR2OAI22</t>
+          <t>XOR2OAI22
+复合逻辑门</t>
         </is>
       </c>
       <c r="B1232" s="11" t="inlineStr">
@@ -13718,7 +14134,8 @@
     <row r="1237">
       <c r="A1237" s="9" t="inlineStr">
         <is>
-          <t>XOR2XNR2</t>
+          <t>XOR2XNR2
+复合逻辑门</t>
         </is>
       </c>
       <c r="B1237" s="10" t="inlineStr">
@@ -13731,7 +14148,8 @@
     <row r="1238">
       <c r="A1238" s="9" t="inlineStr">
         <is>
-          <t>XOR2XOR2</t>
+          <t>XOR2XOR2
+复合逻辑门</t>
         </is>
       </c>
       <c r="B1238" s="10" t="inlineStr">
@@ -13744,7 +14162,8 @@
     <row r="1239">
       <c r="A1239" s="2" t="inlineStr">
         <is>
-          <t>XOR3</t>
+          <t>XOR3
+异或门</t>
         </is>
       </c>
       <c r="B1239" s="3" t="inlineStr">
@@ -13815,7 +14234,8 @@
     <row r="1246">
       <c r="A1246" s="2" t="inlineStr">
         <is>
-          <t>XOR4</t>
+          <t>XOR4
+异或门</t>
         </is>
       </c>
       <c r="B1246" s="3" t="inlineStr">
@@ -13868,7 +14288,8 @@
     <row r="1251">
       <c r="A1251" s="9" t="inlineStr">
         <is>
-          <t>Y2SDFFQ</t>
+          <t>Y2SDFFQ
+扫描触发器</t>
         </is>
       </c>
       <c r="B1251" s="10" t="n"/>
@@ -13881,7 +14302,8 @@
     <row r="1252">
       <c r="A1252" s="9" t="inlineStr">
         <is>
-          <t>Y2SDFQ</t>
+          <t>Y2SDFQ
+扫描触发器</t>
         </is>
       </c>
       <c r="B1252" s="10" t="inlineStr">
@@ -13894,7 +14316,8 @@
     <row r="1253">
       <c r="A1253" s="9" t="inlineStr">
         <is>
-          <t>Y2SDFRPQ</t>
+          <t>Y2SDFRPQ
+扫描触发器</t>
         </is>
       </c>
       <c r="B1253" s="10" t="inlineStr">
@@ -13907,7 +14330,8 @@
     <row r="1254">
       <c r="A1254" s="9" t="inlineStr">
         <is>
-          <t>Y2SDFSNQ</t>
+          <t>Y2SDFSNQ
+扫描触发器</t>
         </is>
       </c>
       <c r="B1254" s="10" t="inlineStr">
@@ -13920,7 +14344,8 @@
     <row r="1255">
       <c r="A1255" s="9" t="inlineStr">
         <is>
-          <t>Y3SDFFACPQ</t>
+          <t>Y3SDFFACPQ
+扫描触发器</t>
         </is>
       </c>
       <c r="B1255" s="10" t="n"/>
@@ -13933,7 +14358,8 @@
     <row r="1256">
       <c r="A1256" s="9" t="inlineStr">
         <is>
-          <t>Y3SDFQ</t>
+          <t>Y3SDFQ
+扫描触发器</t>
         </is>
       </c>
       <c r="B1256" s="10" t="inlineStr">
@@ -13946,7 +14372,8 @@
     <row r="1257">
       <c r="A1257" s="9" t="inlineStr">
         <is>
-          <t>Y3SDFRPQ</t>
+          <t>Y3SDFRPQ
+扫描触发器</t>
         </is>
       </c>
       <c r="B1257" s="10" t="inlineStr">
@@ -13959,7 +14386,8 @@
     <row r="1258">
       <c r="A1258" s="9" t="inlineStr">
         <is>
-          <t>Y3SDFSNQ</t>
+          <t>Y3SDFSNQ
+扫描触发器</t>
         </is>
       </c>
       <c r="B1258" s="10" t="inlineStr">
@@ -13972,7 +14400,8 @@
     <row r="1259">
       <c r="A1259" s="9" t="inlineStr">
         <is>
-          <t>YSDFQ</t>
+          <t>YSDFQ
+扫描触发器</t>
         </is>
       </c>
       <c r="B1259" s="10" t="inlineStr">
@@ -13985,7 +14414,8 @@
     <row r="1260">
       <c r="A1260" s="9" t="inlineStr">
         <is>
-          <t>YSDFRPQ</t>
+          <t>YSDFRPQ
+扫描触发器</t>
         </is>
       </c>
       <c r="B1260" s="10" t="inlineStr">
@@ -13998,7 +14428,8 @@
     <row r="1261">
       <c r="A1261" s="9" t="inlineStr">
         <is>
-          <t>YSDFSNQ</t>
+          <t>YSDFSNQ
+扫描触发器</t>
         </is>
       </c>
       <c r="B1261" s="10" t="inlineStr">

</xml_diff>

<commit_message>
Fix Chinese labels for CKXOR, compounds, and EDF cells.
XOR is checked before OR in clock keys; compound detection no longer
swallows ND/NR; EDF* maps to enable flip-flops, SEDF* stays scan.

Co-authored-by: EsaLongs <EsaLongs@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/preview/NP1PP_vs_C1Y_preview.xlsx
+++ b/preview/NP1PP_vs_C1Y_preview.xlsx
@@ -1770,7 +1770,7 @@
       <c r="A126" s="2" t="inlineStr">
         <is>
           <t>AOI21ND2
-与或非门</t>
+复合逻辑门</t>
         </is>
       </c>
       <c r="B126" s="11" t="inlineStr">
@@ -1802,7 +1802,7 @@
       <c r="A129" s="2" t="inlineStr">
         <is>
           <t>AOI21NR2
-与或非门</t>
+复合逻辑门</t>
         </is>
       </c>
       <c r="B129" s="11" t="inlineStr">
@@ -2319,7 +2319,7 @@
       <c r="A179" s="2" t="inlineStr">
         <is>
           <t>AOI22ND2
-与或非门</t>
+复合逻辑门</t>
         </is>
       </c>
       <c r="B179" s="11" t="inlineStr">
@@ -2378,7 +2378,7 @@
       <c r="A185" s="2" t="inlineStr">
         <is>
           <t>AOI22NR2
-与或非门</t>
+复合逻辑门</t>
         </is>
       </c>
       <c r="B185" s="11" t="inlineStr">
@@ -3724,7 +3724,7 @@
       <c r="A295" s="2" t="inlineStr">
         <is>
           <t>CKXOR2
-时钟或门</t>
+时钟异或门</t>
         </is>
       </c>
       <c r="B295" s="3" t="inlineStr">
@@ -4659,7 +4659,7 @@
       <c r="A374" s="2" t="inlineStr">
         <is>
           <t>EDFQ
-扫描触发器</t>
+使能触发器</t>
         </is>
       </c>
       <c r="B374" s="11" t="inlineStr">
@@ -4682,7 +4682,7 @@
       <c r="A376" s="2" t="inlineStr">
         <is>
           <t>EDFRPQ
-扫描触发器</t>
+使能触发器</t>
         </is>
       </c>
       <c r="B376" s="11" t="inlineStr">
@@ -9369,7 +9369,7 @@
       <c r="A782" s="2" t="inlineStr">
         <is>
           <t>ND2IOA21
-与非门</t>
+复合逻辑门</t>
         </is>
       </c>
       <c r="B782" s="11" t="inlineStr">
@@ -10130,7 +10130,7 @@
       <c r="A860" s="2" t="inlineStr">
         <is>
           <t>NR2ND2
-或非门</t>
+复合逻辑门</t>
         </is>
       </c>
       <c r="B860" s="11" t="inlineStr">
@@ -11063,7 +11063,7 @@
       <c r="A954" s="2" t="inlineStr">
         <is>
           <t>OAI21ND2
-或与非门</t>
+复合逻辑门</t>
         </is>
       </c>
       <c r="B954" s="11" t="inlineStr">
@@ -11131,7 +11131,7 @@
       <c r="A961" s="2" t="inlineStr">
         <is>
           <t>OAI21NR2
-或与非门</t>
+复合逻辑门</t>
         </is>
       </c>
       <c r="B961" s="11" t="inlineStr">
@@ -11610,7 +11610,7 @@
       <c r="A1006" s="2" t="inlineStr">
         <is>
           <t>OAI22ND2
-或与非门</t>
+复合逻辑门</t>
         </is>
       </c>
       <c r="B1006" s="11" t="inlineStr">
@@ -11633,7 +11633,7 @@
       <c r="A1008" s="2" t="inlineStr">
         <is>
           <t>OAI22NR2
-或与非门</t>
+复合逻辑门</t>
         </is>
       </c>
       <c r="B1008" s="11" t="inlineStr">
@@ -13530,7 +13530,7 @@
       <c r="A1179" s="2" t="inlineStr">
         <is>
           <t>XNR2ND2
-同或门</t>
+复合逻辑门</t>
         </is>
       </c>
       <c r="B1179" s="11" t="inlineStr">
@@ -13562,7 +13562,7 @@
       <c r="A1182" s="2" t="inlineStr">
         <is>
           <t>XNR2NR2
-同或门</t>
+复合逻辑门</t>
         </is>
       </c>
       <c r="B1182" s="11" t="inlineStr">
@@ -13998,7 +13998,7 @@
       <c r="A1224" s="2" t="inlineStr">
         <is>
           <t>XOR2ND2
-异或门</t>
+复合逻辑门</t>
         </is>
       </c>
       <c r="B1224" s="11" t="inlineStr">
@@ -14039,7 +14039,7 @@
       <c r="A1228" s="2" t="inlineStr">
         <is>
           <t>XOR2NR2
-异或门</t>
+复合逻辑门</t>
         </is>
       </c>
       <c r="B1228" s="11" t="inlineStr">

</xml_diff>

<commit_message>
Label ISO* cells as isolation units, not level shifters.
Keep LVL/LVU/CKLV* as level shifters; refresh zh catalog and preview.

Co-authored-by: EsaLongs <EsaLongs@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/preview/NP1PP_vs_C1Y_preview.xlsx
+++ b/preview/NP1PP_vs_C1Y_preview.xlsx
@@ -7453,7 +7453,7 @@
       <c r="A605" s="2" t="inlineStr">
         <is>
           <t>ISOCH
-电平转换器</t>
+隔离单元</t>
         </is>
       </c>
       <c r="B605" s="11" t="inlineStr">
@@ -7485,7 +7485,7 @@
       <c r="A608" s="2" t="inlineStr">
         <is>
           <t>ISOCL
-电平转换器</t>
+隔离单元</t>
         </is>
       </c>
       <c r="B608" s="11" t="inlineStr">
@@ -7508,7 +7508,7 @@
       <c r="A610" s="9" t="inlineStr">
         <is>
           <t>ISOH
-电平转换器</t>
+隔离单元</t>
         </is>
       </c>
       <c r="B610" s="10" t="n"/>
@@ -7522,7 +7522,7 @@
       <c r="A611" s="9" t="inlineStr">
         <is>
           <t>ISOHFR
-电平转换器</t>
+隔离单元</t>
         </is>
       </c>
       <c r="B611" s="10" t="n"/>
@@ -7536,7 +7536,7 @@
       <c r="A612" s="9" t="inlineStr">
         <is>
           <t>ISOL
-电平转换器</t>
+隔离单元</t>
         </is>
       </c>
       <c r="B612" s="10" t="n"/>

</xml_diff>

<commit_message>
Refine Chinese labels for CMPE, CKN/GCKNQ, and MUX4N.
Map compressors, clock inverter/gated-clock, and inverted mux more precisely.

Co-authored-by: EsaLongs <EsaLongs@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/preview/NP1PP_vs_C1Y_preview.xlsx
+++ b/preview/NP1PP_vs_C1Y_preview.xlsx
@@ -3522,7 +3522,7 @@
       <c r="A278" s="9" t="inlineStr">
         <is>
           <t>CKN
-时钟单元</t>
+时钟缓冲/反相</t>
         </is>
       </c>
       <c r="B278" s="10" t="n"/>
@@ -3778,7 +3778,7 @@
       <c r="A300" s="2" t="inlineStr">
         <is>
           <t>CMPE32
-比较器</t>
+压缩器</t>
         </is>
       </c>
       <c r="B300" s="11" t="inlineStr">
@@ -3855,7 +3855,7 @@
       <c r="A308" s="2" t="inlineStr">
         <is>
           <t>CMPE42
-比较器</t>
+压缩器</t>
         </is>
       </c>
       <c r="B308" s="11" t="inlineStr">
@@ -5394,7 +5394,7 @@
       <c r="A432" s="2" t="inlineStr">
         <is>
           <t>GCKNQ
-时钟单元</t>
+门控时钟</t>
         </is>
       </c>
       <c r="B432" s="11" t="n"/>
@@ -8850,7 +8850,7 @@
       <c r="A729" s="9" t="inlineStr">
         <is>
           <t>MUX4N
-多路选择器</t>
+反相多路选择器</t>
         </is>
       </c>
       <c r="B729" s="10" t="n"/>

</xml_diff>

<commit_message>
Peel B1/N2 device variants from function roots.
Collapse AOI21B1/AOI21N2/OAI21N2 and *N1 device tails into base
gates (keep AN2 and real compounds like AOI21ND2). Keys 431->423.

Co-authored-by: EsaLongs <EsaLongs@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/preview/NP1PP_vs_C1Y_preview.xlsx
+++ b/preview/NP1PP_vs_C1Y_preview.xlsx
@@ -1427,7 +1427,7 @@
       <c r="B92" s="6" t="n"/>
       <c r="C92" s="6" t="inlineStr">
         <is>
-          <t>AOI21D1COT</t>
+          <t>AOI21B1X6COTC</t>
         </is>
       </c>
     </row>
@@ -1436,7 +1436,7 @@
       <c r="B93" s="6" t="n"/>
       <c r="C93" s="6" t="inlineStr">
         <is>
-          <t>AOI21D3COT</t>
+          <t>AOI21D1COT</t>
         </is>
       </c>
     </row>
@@ -1445,7 +1445,7 @@
       <c r="B94" s="6" t="n"/>
       <c r="C94" s="6" t="inlineStr">
         <is>
-          <t>AOI21D4COT</t>
+          <t>AOI21D3COT</t>
         </is>
       </c>
     </row>
@@ -1454,7 +1454,7 @@
       <c r="B95" s="6" t="n"/>
       <c r="C95" s="6" t="inlineStr">
         <is>
-          <t>AOI21D8COT</t>
+          <t>AOI21D4COT</t>
         </is>
       </c>
     </row>
@@ -1463,7 +1463,7 @@
       <c r="B96" s="6" t="n"/>
       <c r="C96" s="6" t="inlineStr">
         <is>
-          <t>AOI21EEQMBDX2APBCOTC</t>
+          <t>AOI21D8COT</t>
         </is>
       </c>
     </row>
@@ -1472,7 +1472,7 @@
       <c r="B97" s="6" t="n"/>
       <c r="C97" s="6" t="inlineStr">
         <is>
-          <t>AOI21SKND3COT</t>
+          <t>AOI21EEQMBDX2APBCOTC</t>
         </is>
       </c>
     </row>
@@ -1481,7 +1481,7 @@
       <c r="B98" s="6" t="n"/>
       <c r="C98" s="6" t="inlineStr">
         <is>
-          <t>AOI21X2APACOTC</t>
+          <t>AOI21N2X2APACOTC</t>
         </is>
       </c>
     </row>
@@ -1490,7 +1490,7 @@
       <c r="B99" s="6" t="n"/>
       <c r="C99" s="6" t="inlineStr">
         <is>
-          <t>AOI21X4APBCOTC</t>
+          <t>AOI21N2X4APACOTC</t>
         </is>
       </c>
     </row>
@@ -1499,7 +1499,7 @@
       <c r="B100" s="6" t="n"/>
       <c r="C100" s="6" t="inlineStr">
         <is>
-          <t>AOI21X6APACOTC</t>
+          <t>AOI21SKND3COT</t>
         </is>
       </c>
     </row>
@@ -1508,82 +1508,82 @@
       <c r="B101" s="6" t="n"/>
       <c r="C101" s="6" t="inlineStr">
         <is>
+          <t>AOI21X2APACOTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="4" t="n"/>
+      <c r="B102" s="6" t="n"/>
+      <c r="C102" s="6" t="inlineStr">
+        <is>
+          <t>AOI21X4APBCOTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="4" t="n"/>
+      <c r="B103" s="6" t="n"/>
+      <c r="C103" s="6" t="inlineStr">
+        <is>
+          <t>AOI21X6APACOTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="4" t="n"/>
+      <c r="B104" s="6" t="n"/>
+      <c r="C104" s="6" t="inlineStr">
+        <is>
           <t>AOI21X8APACOTC</t>
         </is>
       </c>
     </row>
-    <row r="102">
-      <c r="A102" s="7" t="n"/>
-      <c r="B102" s="8" t="n"/>
-      <c r="C102" s="8" t="inlineStr">
+    <row r="105">
+      <c r="A105" s="7" t="n"/>
+      <c r="B105" s="8" t="n"/>
+      <c r="C105" s="8" t="inlineStr">
         <is>
           <t>AOI21X8APBCOTC</t>
         </is>
       </c>
     </row>
-    <row r="103">
-      <c r="A103" s="2" t="inlineStr">
+    <row r="106">
+      <c r="A106" s="2" t="inlineStr">
         <is>
           <t>AOI211
 与或非门</t>
         </is>
       </c>
-      <c r="B103" s="3" t="inlineStr">
+      <c r="B106" s="3" t="inlineStr">
         <is>
           <t>AOI211D2COT</t>
         </is>
       </c>
-      <c r="C103" s="3" t="inlineStr">
+      <c r="C106" s="3" t="inlineStr">
         <is>
           <t>AOI211D2COT</t>
         </is>
       </c>
-    </row>
-    <row r="104">
-      <c r="A104" s="4" t="n"/>
-      <c r="B104" s="5" t="inlineStr">
-        <is>
-          <t>AOI211D3COT</t>
-        </is>
-      </c>
-      <c r="C104" s="5" t="inlineStr">
-        <is>
-          <t>AOI211D3COT</t>
-        </is>
-      </c>
-    </row>
-    <row r="105">
-      <c r="A105" s="4" t="n"/>
-      <c r="B105" s="6" t="inlineStr">
-        <is>
-          <t>AOI211D1COTOPTPA</t>
-        </is>
-      </c>
-      <c r="C105" s="6" t="n"/>
-    </row>
-    <row r="106">
-      <c r="A106" s="4" t="n"/>
-      <c r="B106" s="6" t="inlineStr">
-        <is>
-          <t>AOI211D4COT</t>
-        </is>
-      </c>
-      <c r="C106" s="6" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="4" t="n"/>
-      <c r="B107" s="6" t="inlineStr">
-        <is>
-          <t>AOI211D6COTSKR</t>
-        </is>
-      </c>
-      <c r="C107" s="6" t="n"/>
+      <c r="B107" s="5" t="inlineStr">
+        <is>
+          <t>AOI211D3COT</t>
+        </is>
+      </c>
+      <c r="C107" s="5" t="inlineStr">
+        <is>
+          <t>AOI211D3COT</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="4" t="n"/>
       <c r="B108" s="6" t="inlineStr">
         <is>
-          <t>AOI211D8COTSKF</t>
+          <t>AOI211D1COTOPTPA</t>
         </is>
       </c>
       <c r="C108" s="6" t="n"/>
@@ -1592,177 +1592,167 @@
       <c r="A109" s="4" t="n"/>
       <c r="B109" s="6" t="inlineStr">
         <is>
-          <t>AOI211OPTPAD1COTOPU</t>
+          <t>AOI211D4COT</t>
         </is>
       </c>
       <c r="C109" s="6" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="4" t="n"/>
-      <c r="B110" s="6" t="n"/>
-      <c r="C110" s="6" t="inlineStr">
-        <is>
-          <t>AOI211D0COT</t>
-        </is>
-      </c>
+      <c r="B110" s="6" t="inlineStr">
+        <is>
+          <t>AOI211D6COTSKR</t>
+        </is>
+      </c>
+      <c r="C110" s="6" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="4" t="n"/>
-      <c r="B111" s="6" t="n"/>
-      <c r="C111" s="6" t="inlineStr">
-        <is>
-          <t>AOI211D1COT</t>
-        </is>
-      </c>
+      <c r="B111" s="6" t="inlineStr">
+        <is>
+          <t>AOI211D8COTSKF</t>
+        </is>
+      </c>
+      <c r="C111" s="6" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="4" t="n"/>
-      <c r="B112" s="6" t="n"/>
-      <c r="C112" s="6" t="inlineStr">
-        <is>
-          <t>AOI211D8COT</t>
-        </is>
-      </c>
+      <c r="B112" s="6" t="inlineStr">
+        <is>
+          <t>AOI211OPTPAD1COTOPU</t>
+        </is>
+      </c>
+      <c r="C112" s="6" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="4" t="n"/>
       <c r="B113" s="6" t="n"/>
       <c r="C113" s="6" t="inlineStr">
         <is>
+          <t>AOI211D0COT</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="4" t="n"/>
+      <c r="B114" s="6" t="n"/>
+      <c r="C114" s="6" t="inlineStr">
+        <is>
+          <t>AOI211D1COT</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="4" t="n"/>
+      <c r="B115" s="6" t="n"/>
+      <c r="C115" s="6" t="inlineStr">
+        <is>
+          <t>AOI211D8COT</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="4" t="n"/>
+      <c r="B116" s="6" t="n"/>
+      <c r="C116" s="6" t="inlineStr">
+        <is>
           <t>AOI211X1APBCOTC</t>
         </is>
       </c>
     </row>
-    <row r="114">
-      <c r="A114" s="7" t="n"/>
-      <c r="B114" s="8" t="n"/>
-      <c r="C114" s="8" t="inlineStr">
+    <row r="117">
+      <c r="A117" s="7" t="n"/>
+      <c r="B117" s="8" t="n"/>
+      <c r="C117" s="8" t="inlineStr">
         <is>
           <t>AOI211X4APBCOTC</t>
         </is>
       </c>
     </row>
-    <row r="115">
-      <c r="A115" s="2" t="inlineStr">
+    <row r="118">
+      <c r="A118" s="2" t="inlineStr">
         <is>
           <t>AOI2111
 与或非门</t>
         </is>
       </c>
-      <c r="B115" s="11" t="inlineStr">
+      <c r="B118" s="11" t="inlineStr">
         <is>
           <t>AOI2111D1COT</t>
         </is>
       </c>
-      <c r="C115" s="11" t="n"/>
-    </row>
-    <row r="116">
-      <c r="A116" s="4" t="n"/>
-      <c r="B116" s="6" t="inlineStr">
+      <c r="C118" s="11" t="n"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="4" t="n"/>
+      <c r="B119" s="6" t="inlineStr">
         <is>
           <t>AOI2111D2COT</t>
         </is>
       </c>
-      <c r="C116" s="6" t="n"/>
-    </row>
-    <row r="117">
-      <c r="A117" s="4" t="n"/>
-      <c r="B117" s="6" t="n"/>
-      <c r="C117" s="6" t="inlineStr">
+      <c r="C119" s="6" t="n"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="4" t="n"/>
+      <c r="B120" s="6" t="n"/>
+      <c r="C120" s="6" t="inlineStr">
         <is>
           <t>AOI2111D1COTA</t>
         </is>
       </c>
     </row>
-    <row r="118">
-      <c r="A118" s="7" t="n"/>
-      <c r="B118" s="8" t="n"/>
-      <c r="C118" s="8" t="inlineStr">
+    <row r="121">
+      <c r="A121" s="7" t="n"/>
+      <c r="B121" s="8" t="n"/>
+      <c r="C121" s="8" t="inlineStr">
         <is>
           <t>AOI2111D2COTA</t>
         </is>
       </c>
     </row>
-    <row r="119">
-      <c r="A119" s="2" t="inlineStr">
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
         <is>
           <t>AOI211INV
 复合逻辑门</t>
         </is>
       </c>
-      <c r="B119" s="11" t="inlineStr">
+      <c r="B122" s="11" t="inlineStr">
         <is>
           <t>AOI211INVCCMD1COTVIAG</t>
         </is>
       </c>
-      <c r="C119" s="11" t="n"/>
-    </row>
-    <row r="120">
-      <c r="A120" s="7" t="n"/>
-      <c r="B120" s="8" t="n"/>
-      <c r="C120" s="8" t="inlineStr">
+      <c r="C122" s="11" t="n"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="7" t="n"/>
+      <c r="B123" s="8" t="n"/>
+      <c r="C123" s="8" t="inlineStr">
         <is>
           <t>AOI211INVCCMD2COTA</t>
         </is>
       </c>
     </row>
-    <row r="121">
-      <c r="A121" s="2" t="inlineStr">
+    <row r="124">
+      <c r="A124" s="2" t="inlineStr">
         <is>
           <t>AOI21AOI21
 复合逻辑门</t>
         </is>
       </c>
-      <c r="B121" s="11" t="inlineStr">
+      <c r="B124" s="11" t="inlineStr">
         <is>
           <t>AOI21AOI21CCMD1COT</t>
         </is>
       </c>
-      <c r="C121" s="11" t="n"/>
-    </row>
-    <row r="122">
-      <c r="A122" s="7" t="n"/>
-      <c r="B122" s="8" t="n"/>
-      <c r="C122" s="8" t="inlineStr">
-        <is>
-          <t>AOI21AOI21CCMD1COTA</t>
-        </is>
-      </c>
-    </row>
-    <row r="123">
-      <c r="A123" s="9" t="inlineStr">
-        <is>
-          <t>AOI21B1
-与或非门</t>
-        </is>
-      </c>
-      <c r="B123" s="10" t="n"/>
-      <c r="C123" s="10" t="inlineStr">
-        <is>
-          <t>AOI21B1X6COTC</t>
-        </is>
-      </c>
-    </row>
-    <row r="124">
-      <c r="A124" s="2" t="inlineStr">
-        <is>
-          <t>AOI21N2
-与或非门</t>
-        </is>
-      </c>
-      <c r="B124" s="11" t="n"/>
-      <c r="C124" s="11" t="inlineStr">
-        <is>
-          <t>AOI21N2X2APACOTC</t>
-        </is>
-      </c>
+      <c r="C124" s="11" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="7" t="n"/>
       <c r="B125" s="8" t="n"/>
       <c r="C125" s="8" t="inlineStr">
         <is>
-          <t>AOI21N2X4APACOTC</t>
+          <t>AOI21AOI21CCMD1COTA</t>
         </is>
       </c>
     </row>
@@ -7993,7 +7983,7 @@
     <row r="653">
       <c r="A653" s="2" t="inlineStr">
         <is>
-          <t>LVUFROR2N1
+          <t>LVUFROR2
 电平转换器</t>
         </is>
       </c>
@@ -8016,7 +8006,7 @@
     <row r="655">
       <c r="A655" s="2" t="inlineStr">
         <is>
-          <t>LVUOR2N1
+          <t>LVUOR2
 电平转换器</t>
         </is>
       </c>
@@ -9140,7 +9130,7 @@
       <c r="B757" s="6" t="n"/>
       <c r="C757" s="6" t="inlineStr">
         <is>
-          <t>ND2X10AKPCOTC</t>
+          <t>ND2N1X10APNCOTC</t>
         </is>
       </c>
     </row>
@@ -9149,7 +9139,7 @@
       <c r="B758" s="6" t="n"/>
       <c r="C758" s="6" t="inlineStr">
         <is>
-          <t>ND2X10APBCOTC</t>
+          <t>ND2N1X12APNCOTC</t>
         </is>
       </c>
     </row>
@@ -9158,7 +9148,7 @@
       <c r="B759" s="6" t="n"/>
       <c r="C759" s="6" t="inlineStr">
         <is>
-          <t>ND2X10APNCOTC</t>
+          <t>ND2N1X2AFCOTC</t>
         </is>
       </c>
     </row>
@@ -9167,7 +9157,7 @@
       <c r="B760" s="6" t="n"/>
       <c r="C760" s="6" t="inlineStr">
         <is>
-          <t>ND2X12AKPCOTC</t>
+          <t>ND2N1X4APNCOTC</t>
         </is>
       </c>
     </row>
@@ -9176,7 +9166,7 @@
       <c r="B761" s="6" t="n"/>
       <c r="C761" s="6" t="inlineStr">
         <is>
-          <t>ND2X14APBCOTC</t>
+          <t>ND2N1X6APNCOTC</t>
         </is>
       </c>
     </row>
@@ -9185,7 +9175,7 @@
       <c r="B762" s="6" t="n"/>
       <c r="C762" s="6" t="inlineStr">
         <is>
-          <t>ND2X16APNCOTC</t>
+          <t>ND2X10AKPCOTC</t>
         </is>
       </c>
     </row>
@@ -9194,7 +9184,7 @@
       <c r="B763" s="6" t="n"/>
       <c r="C763" s="6" t="inlineStr">
         <is>
-          <t>ND2X1AKPCOTC</t>
+          <t>ND2X10APBCOTC</t>
         </is>
       </c>
     </row>
@@ -9203,7 +9193,7 @@
       <c r="B764" s="6" t="n"/>
       <c r="C764" s="6" t="inlineStr">
         <is>
-          <t>ND2X1APNCOTC</t>
+          <t>ND2X10APNCOTC</t>
         </is>
       </c>
     </row>
@@ -9212,7 +9202,7 @@
       <c r="B765" s="6" t="n"/>
       <c r="C765" s="6" t="inlineStr">
         <is>
-          <t>ND2X2AKPCOTC</t>
+          <t>ND2X12AKPCOTC</t>
         </is>
       </c>
     </row>
@@ -9221,7 +9211,7 @@
       <c r="B766" s="6" t="n"/>
       <c r="C766" s="6" t="inlineStr">
         <is>
-          <t>ND2X2APBCOTC</t>
+          <t>ND2X14APBCOTC</t>
         </is>
       </c>
     </row>
@@ -9230,7 +9220,7 @@
       <c r="B767" s="6" t="n"/>
       <c r="C767" s="6" t="inlineStr">
         <is>
-          <t>ND2X2APNCOTC</t>
+          <t>ND2X16APNCOTC</t>
         </is>
       </c>
     </row>
@@ -9239,7 +9229,7 @@
       <c r="B768" s="6" t="n"/>
       <c r="C768" s="6" t="inlineStr">
         <is>
-          <t>ND2X3AKPCOT3FINC</t>
+          <t>ND2X1AKPCOTC</t>
         </is>
       </c>
     </row>
@@ -9248,7 +9238,7 @@
       <c r="B769" s="6" t="n"/>
       <c r="C769" s="6" t="inlineStr">
         <is>
-          <t>ND2X4APACOT3FINC</t>
+          <t>ND2X1APNCOTC</t>
         </is>
       </c>
     </row>
@@ -9257,7 +9247,7 @@
       <c r="B770" s="6" t="n"/>
       <c r="C770" s="6" t="inlineStr">
         <is>
-          <t>ND2X4APBCOTC</t>
+          <t>ND2X2AKPCOTC</t>
         </is>
       </c>
     </row>
@@ -9266,7 +9256,7 @@
       <c r="B771" s="6" t="n"/>
       <c r="C771" s="6" t="inlineStr">
         <is>
-          <t>ND2X4APNCOTC</t>
+          <t>ND2X2APBCOTC</t>
         </is>
       </c>
     </row>
@@ -9275,7 +9265,7 @@
       <c r="B772" s="6" t="n"/>
       <c r="C772" s="6" t="inlineStr">
         <is>
-          <t>ND2X4ARQCOT</t>
+          <t>ND2X2APNCOTC</t>
         </is>
       </c>
     </row>
@@ -9284,7 +9274,7 @@
       <c r="B773" s="6" t="n"/>
       <c r="C773" s="6" t="inlineStr">
         <is>
-          <t>ND2X6AKPCOTC</t>
+          <t>ND2X3AKPCOT3FINC</t>
         </is>
       </c>
     </row>
@@ -9293,7 +9283,7 @@
       <c r="B774" s="6" t="n"/>
       <c r="C774" s="6" t="inlineStr">
         <is>
-          <t>ND2X6APNCOTC</t>
+          <t>ND2X4APACOT3FINC</t>
         </is>
       </c>
     </row>
@@ -9302,7 +9292,7 @@
       <c r="B775" s="6" t="n"/>
       <c r="C775" s="6" t="inlineStr">
         <is>
-          <t>ND2X6AROAFCOT</t>
+          <t>ND2X4APBCOTC</t>
         </is>
       </c>
     </row>
@@ -9311,7 +9301,7 @@
       <c r="B776" s="6" t="n"/>
       <c r="C776" s="6" t="inlineStr">
         <is>
-          <t>ND2X6AROCOT</t>
+          <t>ND2X4APNCOTC</t>
         </is>
       </c>
     </row>
@@ -9320,7 +9310,7 @@
       <c r="B777" s="6" t="n"/>
       <c r="C777" s="6" t="inlineStr">
         <is>
-          <t>ND2X8APACOT3FINC</t>
+          <t>ND2X4ARQCOT</t>
         </is>
       </c>
     </row>
@@ -9329,123 +9319,118 @@
       <c r="B778" s="6" t="n"/>
       <c r="C778" s="6" t="inlineStr">
         <is>
+          <t>ND2X6AKPCOTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="779">
+      <c r="A779" s="4" t="n"/>
+      <c r="B779" s="6" t="n"/>
+      <c r="C779" s="6" t="inlineStr">
+        <is>
+          <t>ND2X6APNCOTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="780">
+      <c r="A780" s="4" t="n"/>
+      <c r="B780" s="6" t="n"/>
+      <c r="C780" s="6" t="inlineStr">
+        <is>
+          <t>ND2X6AROAFCOT</t>
+        </is>
+      </c>
+    </row>
+    <row r="781">
+      <c r="A781" s="4" t="n"/>
+      <c r="B781" s="6" t="n"/>
+      <c r="C781" s="6" t="inlineStr">
+        <is>
+          <t>ND2X6AROCOT</t>
+        </is>
+      </c>
+    </row>
+    <row r="782">
+      <c r="A782" s="4" t="n"/>
+      <c r="B782" s="6" t="n"/>
+      <c r="C782" s="6" t="inlineStr">
+        <is>
+          <t>ND2X8APACOT3FINC</t>
+        </is>
+      </c>
+    </row>
+    <row r="783">
+      <c r="A783" s="4" t="n"/>
+      <c r="B783" s="6" t="n"/>
+      <c r="C783" s="6" t="inlineStr">
+        <is>
           <t>ND2X8APBCOTC</t>
         </is>
       </c>
     </row>
-    <row r="779">
-      <c r="A779" s="7" t="n"/>
-      <c r="B779" s="8" t="n"/>
-      <c r="C779" s="8" t="inlineStr">
+    <row r="784">
+      <c r="A784" s="7" t="n"/>
+      <c r="B784" s="8" t="n"/>
+      <c r="C784" s="8" t="inlineStr">
         <is>
           <t>ND2X8APNCOTC</t>
         </is>
       </c>
     </row>
-    <row r="780">
-      <c r="A780" s="2" t="inlineStr">
+    <row r="785">
+      <c r="A785" s="2" t="inlineStr">
         <is>
           <t>ND2AOI21
 复合逻辑门</t>
         </is>
       </c>
-      <c r="B780" s="11" t="inlineStr">
+      <c r="B785" s="11" t="inlineStr">
         <is>
           <t>ND2AOI21CCBD1COT</t>
         </is>
       </c>
-      <c r="C780" s="11" t="n"/>
-    </row>
-    <row r="781">
-      <c r="A781" s="7" t="n"/>
-      <c r="B781" s="8" t="n"/>
-      <c r="C781" s="8" t="inlineStr">
+      <c r="C785" s="11" t="n"/>
+    </row>
+    <row r="786">
+      <c r="A786" s="7" t="n"/>
+      <c r="B786" s="8" t="n"/>
+      <c r="C786" s="8" t="inlineStr">
         <is>
           <t>ND2AOI21CCBD4COTA</t>
         </is>
       </c>
     </row>
-    <row r="782">
-      <c r="A782" s="2" t="inlineStr">
+    <row r="787">
+      <c r="A787" s="2" t="inlineStr">
         <is>
           <t>ND2IOA21
 复合逻辑门</t>
         </is>
       </c>
-      <c r="B782" s="11" t="inlineStr">
+      <c r="B787" s="11" t="inlineStr">
         <is>
           <t>ND2IOA21D1COT</t>
         </is>
       </c>
-      <c r="C782" s="11" t="n"/>
-    </row>
-    <row r="783">
-      <c r="A783" s="4" t="n"/>
-      <c r="B783" s="6" t="inlineStr">
-        <is>
-          <t>ND2IOA21D2COTVIA</t>
-        </is>
-      </c>
-      <c r="C783" s="6" t="n"/>
-    </row>
-    <row r="784">
-      <c r="A784" s="7" t="n"/>
-      <c r="B784" s="8" t="inlineStr">
-        <is>
-          <t>ND2IOA21D4COT</t>
-        </is>
-      </c>
-      <c r="C784" s="8" t="n"/>
-    </row>
-    <row r="785">
-      <c r="A785" s="2" t="inlineStr">
-        <is>
-          <t>ND2N1
-与非门</t>
-        </is>
-      </c>
-      <c r="B785" s="11" t="n"/>
-      <c r="C785" s="11" t="inlineStr">
-        <is>
-          <t>ND2N1X10APNCOTC</t>
-        </is>
-      </c>
-    </row>
-    <row r="786">
-      <c r="A786" s="4" t="n"/>
-      <c r="B786" s="6" t="n"/>
-      <c r="C786" s="6" t="inlineStr">
-        <is>
-          <t>ND2N1X12APNCOTC</t>
-        </is>
-      </c>
-    </row>
-    <row r="787">
-      <c r="A787" s="4" t="n"/>
-      <c r="B787" s="6" t="n"/>
-      <c r="C787" s="6" t="inlineStr">
-        <is>
-          <t>ND2N1X2AFCOTC</t>
-        </is>
-      </c>
+      <c r="C787" s="11" t="n"/>
     </row>
     <row r="788">
       <c r="A788" s="4" t="n"/>
-      <c r="B788" s="6" t="n"/>
-      <c r="C788" s="6" t="inlineStr">
-        <is>
-          <t>ND2N1X4APNCOTC</t>
-        </is>
-      </c>
+      <c r="B788" s="6" t="inlineStr">
+        <is>
+          <t>ND2IOA21D2COTVIA</t>
+        </is>
+      </c>
+      <c r="C788" s="6" t="n"/>
     </row>
     <row r="789">
       <c r="A789" s="7" t="n"/>
-      <c r="B789" s="8" t="n"/>
-      <c r="C789" s="8" t="inlineStr">
-        <is>
-          <t>ND2N1X6APNCOTC</t>
-        </is>
-      </c>
+      <c r="B789" s="8" t="inlineStr">
+        <is>
+          <t>ND2IOA21D4COT</t>
+        </is>
+      </c>
+      <c r="C789" s="8" t="n"/>
     </row>
     <row r="790">
       <c r="A790" s="2" t="inlineStr">
@@ -9498,53 +9483,43 @@
       <c r="B794" s="6" t="n"/>
       <c r="C794" s="6" t="inlineStr">
         <is>
+          <t>ND3N1X4AFCOTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="795">
+      <c r="A795" s="4" t="n"/>
+      <c r="B795" s="6" t="n"/>
+      <c r="C795" s="6" t="inlineStr">
+        <is>
+          <t>ND3N1X8AFCOTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="796">
+      <c r="A796" s="4" t="n"/>
+      <c r="B796" s="6" t="n"/>
+      <c r="C796" s="6" t="inlineStr">
+        <is>
+          <t>ND3N2X6COTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="797">
+      <c r="A797" s="4" t="n"/>
+      <c r="B797" s="6" t="n"/>
+      <c r="C797" s="6" t="inlineStr">
+        <is>
           <t>ND3X3APACOTC</t>
         </is>
       </c>
     </row>
-    <row r="795">
-      <c r="A795" s="7" t="n"/>
-      <c r="B795" s="8" t="n"/>
-      <c r="C795" s="8" t="inlineStr">
+    <row r="798">
+      <c r="A798" s="7" t="n"/>
+      <c r="B798" s="8" t="n"/>
+      <c r="C798" s="8" t="inlineStr">
         <is>
           <t>ND3X6APACOTC</t>
-        </is>
-      </c>
-    </row>
-    <row r="796">
-      <c r="A796" s="2" t="inlineStr">
-        <is>
-          <t>ND3N1
-与非门</t>
-        </is>
-      </c>
-      <c r="B796" s="11" t="n"/>
-      <c r="C796" s="11" t="inlineStr">
-        <is>
-          <t>ND3N1X4AFCOTC</t>
-        </is>
-      </c>
-    </row>
-    <row r="797">
-      <c r="A797" s="7" t="n"/>
-      <c r="B797" s="8" t="n"/>
-      <c r="C797" s="8" t="inlineStr">
-        <is>
-          <t>ND3N1X8AFCOTC</t>
-        </is>
-      </c>
-    </row>
-    <row r="798">
-      <c r="A798" s="9" t="inlineStr">
-        <is>
-          <t>ND3N2
-与非门</t>
-        </is>
-      </c>
-      <c r="B798" s="10" t="n"/>
-      <c r="C798" s="10" t="inlineStr">
-        <is>
-          <t>ND3N2X6COTC</t>
         </is>
       </c>
     </row>
@@ -9572,23 +9547,18 @@
       <c r="C800" s="6" t="n"/>
     </row>
     <row r="801">
-      <c r="A801" s="7" t="n"/>
-      <c r="B801" s="8" t="n"/>
-      <c r="C801" s="8" t="inlineStr">
+      <c r="A801" s="4" t="n"/>
+      <c r="B801" s="6" t="n"/>
+      <c r="C801" s="6" t="inlineStr">
         <is>
           <t>ND4D0COT</t>
         </is>
       </c>
     </row>
     <row r="802">
-      <c r="A802" s="9" t="inlineStr">
-        <is>
-          <t>ND4N1
-与非门</t>
-        </is>
-      </c>
-      <c r="B802" s="10" t="n"/>
-      <c r="C802" s="10" t="inlineStr">
+      <c r="A802" s="7" t="n"/>
+      <c r="B802" s="8" t="n"/>
+      <c r="C802" s="8" t="inlineStr">
         <is>
           <t>ND4N1X6COTC</t>
         </is>
@@ -9761,7 +9731,7 @@
       <c r="B820" s="6" t="n"/>
       <c r="C820" s="6" t="inlineStr">
         <is>
-          <t>NR2SKPD12COT3FIN</t>
+          <t>NR2N1X10APPCOTC</t>
         </is>
       </c>
     </row>
@@ -9770,7 +9740,7 @@
       <c r="B821" s="6" t="n"/>
       <c r="C821" s="6" t="inlineStr">
         <is>
-          <t>NR2X10APBCOTC</t>
+          <t>NR2N1X12APPCOTC</t>
         </is>
       </c>
     </row>
@@ -9779,7 +9749,7 @@
       <c r="B822" s="6" t="n"/>
       <c r="C822" s="6" t="inlineStr">
         <is>
-          <t>NR2X10APPCOTC</t>
+          <t>NR2N1X12AROAFCOT</t>
         </is>
       </c>
     </row>
@@ -9788,7 +9758,7 @@
       <c r="B823" s="6" t="n"/>
       <c r="C823" s="6" t="inlineStr">
         <is>
-          <t>NR2X12AKNCOTC</t>
+          <t>NR2N1X12AROCOT</t>
         </is>
       </c>
     </row>
@@ -9797,7 +9767,7 @@
       <c r="B824" s="6" t="n"/>
       <c r="C824" s="6" t="inlineStr">
         <is>
-          <t>NR2X12APACOTC</t>
+          <t>NR2N1X14APPCOTC</t>
         </is>
       </c>
     </row>
@@ -9806,7 +9776,7 @@
       <c r="B825" s="6" t="n"/>
       <c r="C825" s="6" t="inlineStr">
         <is>
-          <t>NR2X12APPCOTC</t>
+          <t>NR2N1X16APPCOTC</t>
         </is>
       </c>
     </row>
@@ -9815,7 +9785,7 @@
       <c r="B826" s="6" t="n"/>
       <c r="C826" s="6" t="inlineStr">
         <is>
-          <t>NR2X14APBCOTC</t>
+          <t>NR2N1X1APPCOTC</t>
         </is>
       </c>
     </row>
@@ -9824,7 +9794,7 @@
       <c r="B827" s="6" t="n"/>
       <c r="C827" s="6" t="inlineStr">
         <is>
-          <t>NR2X14APPCOTC</t>
+          <t>NR2N1X4APPCOTC</t>
         </is>
       </c>
     </row>
@@ -9833,7 +9803,7 @@
       <c r="B828" s="6" t="n"/>
       <c r="C828" s="6" t="inlineStr">
         <is>
-          <t>NR2X16APACOTC</t>
+          <t>NR2N1X6APPCOTC</t>
         </is>
       </c>
     </row>
@@ -9842,7 +9812,7 @@
       <c r="B829" s="6" t="n"/>
       <c r="C829" s="6" t="inlineStr">
         <is>
-          <t>NR2X16APBCOTC</t>
+          <t>NR2N1X8APPCOTC</t>
         </is>
       </c>
     </row>
@@ -9851,7 +9821,7 @@
       <c r="B830" s="6" t="n"/>
       <c r="C830" s="6" t="inlineStr">
         <is>
-          <t>NR2X16APPCOTC</t>
+          <t>NR2SKPD12COT3FIN</t>
         </is>
       </c>
     </row>
@@ -9860,7 +9830,7 @@
       <c r="B831" s="6" t="n"/>
       <c r="C831" s="6" t="inlineStr">
         <is>
-          <t>NR2X1AKNCOTC</t>
+          <t>NR2X10APBCOTC</t>
         </is>
       </c>
     </row>
@@ -9869,7 +9839,7 @@
       <c r="B832" s="6" t="n"/>
       <c r="C832" s="6" t="inlineStr">
         <is>
-          <t>NR2X1APACOTC</t>
+          <t>NR2X10APPCOTC</t>
         </is>
       </c>
     </row>
@@ -9878,7 +9848,7 @@
       <c r="B833" s="6" t="n"/>
       <c r="C833" s="6" t="inlineStr">
         <is>
-          <t>NR2X1APPCOTC</t>
+          <t>NR2X12AKNCOTC</t>
         </is>
       </c>
     </row>
@@ -9887,7 +9857,7 @@
       <c r="B834" s="6" t="n"/>
       <c r="C834" s="6" t="inlineStr">
         <is>
-          <t>NR2X2AKNCOT3FINC</t>
+          <t>NR2X12APACOTC</t>
         </is>
       </c>
     </row>
@@ -9896,7 +9866,7 @@
       <c r="B835" s="6" t="n"/>
       <c r="C835" s="6" t="inlineStr">
         <is>
-          <t>NR2X2APPCOT3FINC</t>
+          <t>NR2X12APPCOTC</t>
         </is>
       </c>
     </row>
@@ -9905,7 +9875,7 @@
       <c r="B836" s="6" t="n"/>
       <c r="C836" s="6" t="inlineStr">
         <is>
-          <t>NR2X3AKNCOT3FINC</t>
+          <t>NR2X14APBCOTC</t>
         </is>
       </c>
     </row>
@@ -9914,7 +9884,7 @@
       <c r="B837" s="6" t="n"/>
       <c r="C837" s="6" t="inlineStr">
         <is>
-          <t>NR2X4AKNCOTC</t>
+          <t>NR2X14APPCOTC</t>
         </is>
       </c>
     </row>
@@ -9923,7 +9893,7 @@
       <c r="B838" s="6" t="n"/>
       <c r="C838" s="6" t="inlineStr">
         <is>
-          <t>NR2X4APACOTC</t>
+          <t>NR2X16APACOTC</t>
         </is>
       </c>
     </row>
@@ -9932,7 +9902,7 @@
       <c r="B839" s="6" t="n"/>
       <c r="C839" s="6" t="inlineStr">
         <is>
-          <t>NR2X4APBCOTC</t>
+          <t>NR2X16APBCOTC</t>
         </is>
       </c>
     </row>
@@ -9941,7 +9911,7 @@
       <c r="B840" s="6" t="n"/>
       <c r="C840" s="6" t="inlineStr">
         <is>
-          <t>NR2X4ARQCOT</t>
+          <t>NR2X16APPCOTC</t>
         </is>
       </c>
     </row>
@@ -9950,7 +9920,7 @@
       <c r="B841" s="6" t="n"/>
       <c r="C841" s="6" t="inlineStr">
         <is>
-          <t>NR2X6APACOTC</t>
+          <t>NR2X1AKNCOTC</t>
         </is>
       </c>
     </row>
@@ -9959,7 +9929,7 @@
       <c r="B842" s="6" t="n"/>
       <c r="C842" s="6" t="inlineStr">
         <is>
-          <t>NR2X6APBCOTC</t>
+          <t>NR2X1APACOTC</t>
         </is>
       </c>
     </row>
@@ -9968,7 +9938,7 @@
       <c r="B843" s="6" t="n"/>
       <c r="C843" s="6" t="inlineStr">
         <is>
-          <t>NR2X6ARQCOT</t>
+          <t>NR2X1APPCOTC</t>
         </is>
       </c>
     </row>
@@ -9977,7 +9947,7 @@
       <c r="B844" s="6" t="n"/>
       <c r="C844" s="6" t="inlineStr">
         <is>
-          <t>NR2X8APACOTC</t>
+          <t>NR2X2AKNCOT3FINC</t>
         </is>
       </c>
     </row>
@@ -9986,7 +9956,7 @@
       <c r="B845" s="6" t="n"/>
       <c r="C845" s="6" t="inlineStr">
         <is>
-          <t>NR2X8APBCOTC</t>
+          <t>NR2X2APPCOT3FINC</t>
         </is>
       </c>
     </row>
@@ -9995,53 +9965,43 @@
       <c r="B846" s="6" t="n"/>
       <c r="C846" s="6" t="inlineStr">
         <is>
-          <t>NR2X8APPCOTC</t>
+          <t>NR2X3AKNCOT3FINC</t>
         </is>
       </c>
     </row>
     <row r="847">
-      <c r="A847" s="7" t="n"/>
-      <c r="B847" s="8" t="n"/>
-      <c r="C847" s="8" t="inlineStr">
-        <is>
-          <t>NR2X8AROCOT</t>
+      <c r="A847" s="4" t="n"/>
+      <c r="B847" s="6" t="n"/>
+      <c r="C847" s="6" t="inlineStr">
+        <is>
+          <t>NR2X4AKNCOTC</t>
         </is>
       </c>
     </row>
     <row r="848">
-      <c r="A848" s="2" t="inlineStr">
-        <is>
-          <t>NR2AOI21
-复合逻辑门</t>
-        </is>
-      </c>
-      <c r="B848" s="11" t="inlineStr">
-        <is>
-          <t>NR2AOI21CCBD4COT</t>
-        </is>
-      </c>
-      <c r="C848" s="11" t="n"/>
+      <c r="A848" s="4" t="n"/>
+      <c r="B848" s="6" t="n"/>
+      <c r="C848" s="6" t="inlineStr">
+        <is>
+          <t>NR2X4APACOTC</t>
+        </is>
+      </c>
     </row>
     <row r="849">
-      <c r="A849" s="7" t="n"/>
-      <c r="B849" s="8" t="n"/>
-      <c r="C849" s="8" t="inlineStr">
-        <is>
-          <t>NR2AOI21CCBD2COT</t>
+      <c r="A849" s="4" t="n"/>
+      <c r="B849" s="6" t="n"/>
+      <c r="C849" s="6" t="inlineStr">
+        <is>
+          <t>NR2X4APBCOTC</t>
         </is>
       </c>
     </row>
     <row r="850">
-      <c r="A850" s="2" t="inlineStr">
-        <is>
-          <t>NR2N1
-或非门</t>
-        </is>
-      </c>
-      <c r="B850" s="11" t="n"/>
-      <c r="C850" s="11" t="inlineStr">
-        <is>
-          <t>NR2N1X10APPCOTC</t>
+      <c r="A850" s="4" t="n"/>
+      <c r="B850" s="6" t="n"/>
+      <c r="C850" s="6" t="inlineStr">
+        <is>
+          <t>NR2X4ARQCOT</t>
         </is>
       </c>
     </row>
@@ -10050,7 +10010,7 @@
       <c r="B851" s="6" t="n"/>
       <c r="C851" s="6" t="inlineStr">
         <is>
-          <t>NR2N1X12APPCOTC</t>
+          <t>NR2X6APACOTC</t>
         </is>
       </c>
     </row>
@@ -10059,7 +10019,7 @@
       <c r="B852" s="6" t="n"/>
       <c r="C852" s="6" t="inlineStr">
         <is>
-          <t>NR2N1X12AROAFCOT</t>
+          <t>NR2X6APBCOTC</t>
         </is>
       </c>
     </row>
@@ -10068,7 +10028,7 @@
       <c r="B853" s="6" t="n"/>
       <c r="C853" s="6" t="inlineStr">
         <is>
-          <t>NR2N1X12AROCOT</t>
+          <t>NR2X6ARQCOT</t>
         </is>
       </c>
     </row>
@@ -10077,7 +10037,7 @@
       <c r="B854" s="6" t="n"/>
       <c r="C854" s="6" t="inlineStr">
         <is>
-          <t>NR2N1X14APPCOTC</t>
+          <t>NR2X8APACOTC</t>
         </is>
       </c>
     </row>
@@ -10086,7 +10046,7 @@
       <c r="B855" s="6" t="n"/>
       <c r="C855" s="6" t="inlineStr">
         <is>
-          <t>NR2N1X16APPCOTC</t>
+          <t>NR2X8APBCOTC</t>
         </is>
       </c>
     </row>
@@ -10095,34 +10055,39 @@
       <c r="B856" s="6" t="n"/>
       <c r="C856" s="6" t="inlineStr">
         <is>
-          <t>NR2N1X1APPCOTC</t>
+          <t>NR2X8APPCOTC</t>
         </is>
       </c>
     </row>
     <row r="857">
-      <c r="A857" s="4" t="n"/>
-      <c r="B857" s="6" t="n"/>
-      <c r="C857" s="6" t="inlineStr">
-        <is>
-          <t>NR2N1X4APPCOTC</t>
+      <c r="A857" s="7" t="n"/>
+      <c r="B857" s="8" t="n"/>
+      <c r="C857" s="8" t="inlineStr">
+        <is>
+          <t>NR2X8AROCOT</t>
         </is>
       </c>
     </row>
     <row r="858">
-      <c r="A858" s="4" t="n"/>
-      <c r="B858" s="6" t="n"/>
-      <c r="C858" s="6" t="inlineStr">
-        <is>
-          <t>NR2N1X6APPCOTC</t>
-        </is>
-      </c>
+      <c r="A858" s="2" t="inlineStr">
+        <is>
+          <t>NR2AOI21
+复合逻辑门</t>
+        </is>
+      </c>
+      <c r="B858" s="11" t="inlineStr">
+        <is>
+          <t>NR2AOI21CCBD4COT</t>
+        </is>
+      </c>
+      <c r="C858" s="11" t="n"/>
     </row>
     <row r="859">
       <c r="A859" s="7" t="n"/>
       <c r="B859" s="8" t="n"/>
       <c r="C859" s="8" t="inlineStr">
         <is>
-          <t>NR2N1X8APPCOTC</t>
+          <t>NR2AOI21CCBD2COT</t>
         </is>
       </c>
     </row>
@@ -10755,7 +10720,7 @@
       <c r="B923" s="6" t="n"/>
       <c r="C923" s="6" t="inlineStr">
         <is>
-          <t>OAI21OPTLD4COT</t>
+          <t>OAI21N2X2APACOTC</t>
         </is>
       </c>
     </row>
@@ -10764,7 +10729,7 @@
       <c r="B924" s="6" t="n"/>
       <c r="C924" s="6" t="inlineStr">
         <is>
-          <t>OAI21X1APACOTC</t>
+          <t>OAI21N2X6APACOTC</t>
         </is>
       </c>
     </row>
@@ -10773,7 +10738,7 @@
       <c r="B925" s="6" t="n"/>
       <c r="C925" s="6" t="inlineStr">
         <is>
-          <t>OAI21X3APACOTC</t>
+          <t>OAI21N2X8APACOTC</t>
         </is>
       </c>
     </row>
@@ -10782,7 +10747,7 @@
       <c r="B926" s="6" t="n"/>
       <c r="C926" s="6" t="inlineStr">
         <is>
-          <t>OAI21X4APACOTC</t>
+          <t>OAI21N2X8COTC</t>
         </is>
       </c>
     </row>
@@ -10791,74 +10756,74 @@
       <c r="B927" s="6" t="n"/>
       <c r="C927" s="6" t="inlineStr">
         <is>
+          <t>OAI21OPTLD4COT</t>
+        </is>
+      </c>
+    </row>
+    <row r="928">
+      <c r="A928" s="4" t="n"/>
+      <c r="B928" s="6" t="n"/>
+      <c r="C928" s="6" t="inlineStr">
+        <is>
+          <t>OAI21X1APACOTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="929">
+      <c r="A929" s="4" t="n"/>
+      <c r="B929" s="6" t="n"/>
+      <c r="C929" s="6" t="inlineStr">
+        <is>
+          <t>OAI21X3APACOTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="930">
+      <c r="A930" s="4" t="n"/>
+      <c r="B930" s="6" t="n"/>
+      <c r="C930" s="6" t="inlineStr">
+        <is>
+          <t>OAI21X4APACOTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="931">
+      <c r="A931" s="4" t="n"/>
+      <c r="B931" s="6" t="n"/>
+      <c r="C931" s="6" t="inlineStr">
+        <is>
           <t>OAI21X6APACOTC</t>
         </is>
       </c>
     </row>
-    <row r="928">
-      <c r="A928" s="7" t="n"/>
-      <c r="B928" s="8" t="n"/>
-      <c r="C928" s="8" t="inlineStr">
+    <row r="932">
+      <c r="A932" s="7" t="n"/>
+      <c r="B932" s="8" t="n"/>
+      <c r="C932" s="8" t="inlineStr">
         <is>
           <t>OAI21X8APACOTC</t>
         </is>
       </c>
     </row>
-    <row r="929">
-      <c r="A929" s="2" t="inlineStr">
+    <row r="933">
+      <c r="A933" s="2" t="inlineStr">
         <is>
           <t>OAI211
 或与非门</t>
         </is>
       </c>
-      <c r="B929" s="11" t="inlineStr">
+      <c r="B933" s="11" t="inlineStr">
         <is>
           <t>OAI211D1COTOPU</t>
         </is>
       </c>
-      <c r="C929" s="11" t="n"/>
-    </row>
-    <row r="930">
-      <c r="A930" s="4" t="n"/>
-      <c r="B930" s="6" t="inlineStr">
-        <is>
-          <t>OAI211D2COT</t>
-        </is>
-      </c>
-      <c r="C930" s="6" t="n"/>
-    </row>
-    <row r="931">
-      <c r="A931" s="4" t="n"/>
-      <c r="B931" s="6" t="inlineStr">
-        <is>
-          <t>OAI211D3COTSKF</t>
-        </is>
-      </c>
-      <c r="C931" s="6" t="n"/>
-    </row>
-    <row r="932">
-      <c r="A932" s="4" t="n"/>
-      <c r="B932" s="6" t="inlineStr">
-        <is>
-          <t>OAI211D4COTOPTPA</t>
-        </is>
-      </c>
-      <c r="C932" s="6" t="n"/>
-    </row>
-    <row r="933">
-      <c r="A933" s="4" t="n"/>
-      <c r="B933" s="6" t="inlineStr">
-        <is>
-          <t>OAI211D6COTOPTPA</t>
-        </is>
-      </c>
-      <c r="C933" s="6" t="n"/>
+      <c r="C933" s="11" t="n"/>
     </row>
     <row r="934">
       <c r="A934" s="4" t="n"/>
       <c r="B934" s="6" t="inlineStr">
         <is>
-          <t>OAI211D8COTSKR</t>
+          <t>OAI211D2COT</t>
         </is>
       </c>
       <c r="C934" s="6" t="n"/>
@@ -10867,53 +10832,53 @@
       <c r="A935" s="4" t="n"/>
       <c r="B935" s="6" t="inlineStr">
         <is>
-          <t>OAI211OPTPAD1COTOPU</t>
+          <t>OAI211D3COTSKF</t>
         </is>
       </c>
       <c r="C935" s="6" t="n"/>
     </row>
     <row r="936">
       <c r="A936" s="4" t="n"/>
-      <c r="B936" s="6" t="n"/>
-      <c r="C936" s="6" t="inlineStr">
-        <is>
-          <t>OAI211D1COT</t>
-        </is>
-      </c>
+      <c r="B936" s="6" t="inlineStr">
+        <is>
+          <t>OAI211D4COTOPTPA</t>
+        </is>
+      </c>
+      <c r="C936" s="6" t="n"/>
     </row>
     <row r="937">
       <c r="A937" s="4" t="n"/>
-      <c r="B937" s="6" t="n"/>
-      <c r="C937" s="6" t="inlineStr">
-        <is>
-          <t>OAI211D3COT</t>
-        </is>
-      </c>
+      <c r="B937" s="6" t="inlineStr">
+        <is>
+          <t>OAI211D6COTOPTPA</t>
+        </is>
+      </c>
+      <c r="C937" s="6" t="n"/>
     </row>
     <row r="938">
       <c r="A938" s="4" t="n"/>
-      <c r="B938" s="6" t="n"/>
-      <c r="C938" s="6" t="inlineStr">
-        <is>
-          <t>OAI211D4COT</t>
-        </is>
-      </c>
+      <c r="B938" s="6" t="inlineStr">
+        <is>
+          <t>OAI211D8COTSKR</t>
+        </is>
+      </c>
+      <c r="C938" s="6" t="n"/>
     </row>
     <row r="939">
       <c r="A939" s="4" t="n"/>
-      <c r="B939" s="6" t="n"/>
-      <c r="C939" s="6" t="inlineStr">
-        <is>
-          <t>OAI211D6COT</t>
-        </is>
-      </c>
+      <c r="B939" s="6" t="inlineStr">
+        <is>
+          <t>OAI211OPTPAD1COTOPU</t>
+        </is>
+      </c>
+      <c r="C939" s="6" t="n"/>
     </row>
     <row r="940">
       <c r="A940" s="4" t="n"/>
       <c r="B940" s="6" t="n"/>
       <c r="C940" s="6" t="inlineStr">
         <is>
-          <t>OAI211D8COT</t>
+          <t>OAI211D1COT</t>
         </is>
       </c>
     </row>
@@ -10922,142 +10887,137 @@
       <c r="B941" s="6" t="n"/>
       <c r="C941" s="6" t="inlineStr">
         <is>
+          <t>OAI211D3COT</t>
+        </is>
+      </c>
+    </row>
+    <row r="942">
+      <c r="A942" s="4" t="n"/>
+      <c r="B942" s="6" t="n"/>
+      <c r="C942" s="6" t="inlineStr">
+        <is>
+          <t>OAI211D4COT</t>
+        </is>
+      </c>
+    </row>
+    <row r="943">
+      <c r="A943" s="4" t="n"/>
+      <c r="B943" s="6" t="n"/>
+      <c r="C943" s="6" t="inlineStr">
+        <is>
+          <t>OAI211D6COT</t>
+        </is>
+      </c>
+    </row>
+    <row r="944">
+      <c r="A944" s="4" t="n"/>
+      <c r="B944" s="6" t="n"/>
+      <c r="C944" s="6" t="inlineStr">
+        <is>
+          <t>OAI211D8COT</t>
+        </is>
+      </c>
+    </row>
+    <row r="945">
+      <c r="A945" s="4" t="n"/>
+      <c r="B945" s="6" t="n"/>
+      <c r="C945" s="6" t="inlineStr">
+        <is>
           <t>OAI211OPTPAD6COT</t>
         </is>
       </c>
     </row>
-    <row r="942">
-      <c r="A942" s="7" t="n"/>
-      <c r="B942" s="8" t="n"/>
-      <c r="C942" s="8" t="inlineStr">
+    <row r="946">
+      <c r="A946" s="7" t="n"/>
+      <c r="B946" s="8" t="n"/>
+      <c r="C946" s="8" t="inlineStr">
         <is>
           <t>OAI211X2APBCOTC</t>
         </is>
       </c>
     </row>
-    <row r="943">
-      <c r="A943" s="2" t="inlineStr">
+    <row r="947">
+      <c r="A947" s="2" t="inlineStr">
         <is>
           <t>OAI2111
 或与非门</t>
         </is>
       </c>
-      <c r="B943" s="11" t="inlineStr">
+      <c r="B947" s="11" t="inlineStr">
         <is>
           <t>OAI2111D1COT</t>
         </is>
       </c>
-      <c r="C943" s="11" t="n"/>
-    </row>
-    <row r="944">
-      <c r="A944" s="7" t="n"/>
-      <c r="B944" s="8" t="inlineStr">
+      <c r="C947" s="11" t="n"/>
+    </row>
+    <row r="948">
+      <c r="A948" s="7" t="n"/>
+      <c r="B948" s="8" t="inlineStr">
         <is>
           <t>OAI2111D2COT</t>
         </is>
       </c>
-      <c r="C944" s="8" t="n"/>
-    </row>
-    <row r="945">
-      <c r="A945" s="9" t="inlineStr">
+      <c r="C948" s="8" t="n"/>
+    </row>
+    <row r="949">
+      <c r="A949" s="9" t="inlineStr">
         <is>
           <t>OAI211INV
 复合逻辑门</t>
         </is>
       </c>
-      <c r="B945" s="10" t="inlineStr">
+      <c r="B949" s="10" t="inlineStr">
         <is>
           <t>OAI211INVCCAD1COTVIAG</t>
         </is>
       </c>
-      <c r="C945" s="10" t="n"/>
-    </row>
-    <row r="946">
-      <c r="A946" s="9" t="inlineStr">
+      <c r="C949" s="10" t="n"/>
+    </row>
+    <row r="950">
+      <c r="A950" s="9" t="inlineStr">
         <is>
           <t>OAI21AOI21
 复合逻辑门</t>
         </is>
       </c>
-      <c r="B946" s="10" t="n"/>
-      <c r="C946" s="10" t="inlineStr">
+      <c r="B950" s="10" t="n"/>
+      <c r="C950" s="10" t="inlineStr">
         <is>
           <t>OAI21AOI21CCBD4COTA</t>
         </is>
       </c>
     </row>
-    <row r="947">
-      <c r="A947" s="2" t="inlineStr">
+    <row r="951">
+      <c r="A951" s="2" t="inlineStr">
         <is>
           <t>OAI21AOI22
 复合逻辑门</t>
         </is>
       </c>
-      <c r="B947" s="11" t="inlineStr">
+      <c r="B951" s="11" t="inlineStr">
         <is>
           <t>OAI21AOI22D1COT</t>
         </is>
       </c>
-      <c r="C947" s="11" t="n"/>
-    </row>
-    <row r="948">
-      <c r="A948" s="4" t="n"/>
-      <c r="B948" s="6" t="inlineStr">
-        <is>
-          <t>OAI21AOI22D2COT</t>
-        </is>
-      </c>
-      <c r="C948" s="6" t="n"/>
-    </row>
-    <row r="949">
-      <c r="A949" s="7" t="n"/>
-      <c r="B949" s="8" t="inlineStr">
-        <is>
-          <t>OAI21AOI22D4COT</t>
-        </is>
-      </c>
-      <c r="C949" s="8" t="n"/>
-    </row>
-    <row r="950">
-      <c r="A950" s="2" t="inlineStr">
-        <is>
-          <t>OAI21N2
-或与非门</t>
-        </is>
-      </c>
-      <c r="B950" s="11" t="n"/>
-      <c r="C950" s="11" t="inlineStr">
-        <is>
-          <t>OAI21N2X2APACOTC</t>
-        </is>
-      </c>
-    </row>
-    <row r="951">
-      <c r="A951" s="4" t="n"/>
-      <c r="B951" s="6" t="n"/>
-      <c r="C951" s="6" t="inlineStr">
-        <is>
-          <t>OAI21N2X6APACOTC</t>
-        </is>
-      </c>
+      <c r="C951" s="11" t="n"/>
     </row>
     <row r="952">
       <c r="A952" s="4" t="n"/>
-      <c r="B952" s="6" t="n"/>
-      <c r="C952" s="6" t="inlineStr">
-        <is>
-          <t>OAI21N2X8APACOTC</t>
-        </is>
-      </c>
+      <c r="B952" s="6" t="inlineStr">
+        <is>
+          <t>OAI21AOI22D2COT</t>
+        </is>
+      </c>
+      <c r="C952" s="6" t="n"/>
     </row>
     <row r="953">
       <c r="A953" s="7" t="n"/>
-      <c r="B953" s="8" t="n"/>
-      <c r="C953" s="8" t="inlineStr">
-        <is>
-          <t>OAI21N2X8COTC</t>
-        </is>
-      </c>
+      <c r="B953" s="8" t="inlineStr">
+        <is>
+          <t>OAI21AOI22D4COT</t>
+        </is>
+      </c>
+      <c r="C953" s="8" t="n"/>
     </row>
     <row r="954">
       <c r="A954" s="2" t="inlineStr">
@@ -14440,14 +14400,16 @@
       <c r="C1261" s="10" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="224">
+  <mergeCells count="219">
     <mergeCell ref="A540:A543"/>
+    <mergeCell ref="A106:A117"/>
     <mergeCell ref="A378:A384"/>
     <mergeCell ref="A399:A400"/>
     <mergeCell ref="A268:A269"/>
     <mergeCell ref="A701:A706"/>
     <mergeCell ref="A1139:A1140"/>
     <mergeCell ref="A649:A650"/>
+    <mergeCell ref="A947:A948"/>
     <mergeCell ref="A335:A336"/>
     <mergeCell ref="A690:A691"/>
     <mergeCell ref="A966:A977"/>
@@ -14459,27 +14421,22 @@
     <mergeCell ref="A582:A583"/>
     <mergeCell ref="A1141:A1142"/>
     <mergeCell ref="A236:A237"/>
-    <mergeCell ref="A792:A795"/>
     <mergeCell ref="A71:A74"/>
     <mergeCell ref="A189:A192"/>
     <mergeCell ref="A989:A990"/>
     <mergeCell ref="A1075:A1083"/>
     <mergeCell ref="A164:A167"/>
-    <mergeCell ref="A785:A789"/>
     <mergeCell ref="A675:A676"/>
     <mergeCell ref="A1175:A1178"/>
     <mergeCell ref="A244:A247"/>
-    <mergeCell ref="A103:A114"/>
     <mergeCell ref="A1021:A1025"/>
     <mergeCell ref="A1232:A1236"/>
     <mergeCell ref="A730:A731"/>
     <mergeCell ref="A1011:A1015"/>
     <mergeCell ref="A790:A791"/>
     <mergeCell ref="A905:A909"/>
-    <mergeCell ref="A115:A118"/>
     <mergeCell ref="A1036:A1040"/>
     <mergeCell ref="A961:A964"/>
-    <mergeCell ref="A780:A781"/>
     <mergeCell ref="A320:A321"/>
     <mergeCell ref="A403:A404"/>
     <mergeCell ref="A714:A716"/>
@@ -14491,10 +14448,8 @@
     <mergeCell ref="A480:A481"/>
     <mergeCell ref="A256:A257"/>
     <mergeCell ref="A427:A428"/>
-    <mergeCell ref="A747:A779"/>
     <mergeCell ref="A1033:A1035"/>
     <mergeCell ref="A1105:A1106"/>
-    <mergeCell ref="A119:A120"/>
     <mergeCell ref="A569:A576"/>
     <mergeCell ref="A359:A360"/>
     <mergeCell ref="A719:A721"/>
@@ -14526,14 +14481,13 @@
     <mergeCell ref="A160:A163"/>
     <mergeCell ref="A64:A70"/>
     <mergeCell ref="A622:A623"/>
-    <mergeCell ref="A121:A122"/>
+    <mergeCell ref="A858:A859"/>
+    <mergeCell ref="A787:A789"/>
     <mergeCell ref="A357:A358"/>
     <mergeCell ref="A681:A682"/>
     <mergeCell ref="A1092:A1095"/>
-    <mergeCell ref="A848:A849"/>
     <mergeCell ref="A344:A345"/>
     <mergeCell ref="A615:A616"/>
-    <mergeCell ref="A947:A949"/>
     <mergeCell ref="A407:A408"/>
     <mergeCell ref="A667:A669"/>
     <mergeCell ref="A631:A636"/>
@@ -14543,27 +14497,24 @@
     <mergeCell ref="A126:A128"/>
     <mergeCell ref="A534:A539"/>
     <mergeCell ref="A1125:A1130"/>
-    <mergeCell ref="A803:A847"/>
     <mergeCell ref="A1068:A1074"/>
     <mergeCell ref="A1239:A1245"/>
     <mergeCell ref="A983:A984"/>
     <mergeCell ref="A887:A891"/>
     <mergeCell ref="A1201:A1217"/>
     <mergeCell ref="A473:A474"/>
-    <mergeCell ref="A796:A797"/>
     <mergeCell ref="A1151:A1152"/>
-    <mergeCell ref="A85:A102"/>
     <mergeCell ref="A551:A554"/>
     <mergeCell ref="A457:A458"/>
-    <mergeCell ref="A799:A801"/>
     <mergeCell ref="A264:A265"/>
     <mergeCell ref="A1147:A1148"/>
     <mergeCell ref="A326:A327"/>
+    <mergeCell ref="A118:A121"/>
+    <mergeCell ref="A951:A953"/>
     <mergeCell ref="A1154:A1171"/>
     <mergeCell ref="A425:A426"/>
     <mergeCell ref="A860:A862"/>
     <mergeCell ref="A600:A604"/>
-    <mergeCell ref="A850:A859"/>
     <mergeCell ref="A376:A377"/>
     <mergeCell ref="A735:A746"/>
     <mergeCell ref="A717:A718"/>
@@ -14583,15 +14534,19 @@
     <mergeCell ref="A898:A904"/>
     <mergeCell ref="A991:A999"/>
     <mergeCell ref="A179:A184"/>
+    <mergeCell ref="A122:A123"/>
     <mergeCell ref="A411:A412"/>
+    <mergeCell ref="A651:A652"/>
     <mergeCell ref="A670:A673"/>
-    <mergeCell ref="A651:A652"/>
     <mergeCell ref="A1004:A1005"/>
     <mergeCell ref="A1228:A1230"/>
     <mergeCell ref="A258:A259"/>
     <mergeCell ref="A185:A188"/>
+    <mergeCell ref="A933:A946"/>
     <mergeCell ref="A363:A365"/>
     <mergeCell ref="A1107:A1108"/>
+    <mergeCell ref="A747:A784"/>
+    <mergeCell ref="A799:A802"/>
     <mergeCell ref="A523:A527"/>
     <mergeCell ref="A391:A392"/>
     <mergeCell ref="A1100:A1101"/>
@@ -14601,11 +14556,14 @@
     <mergeCell ref="A707:A708"/>
     <mergeCell ref="A1219:A1223"/>
     <mergeCell ref="A985:A988"/>
+    <mergeCell ref="A85:A105"/>
     <mergeCell ref="A446:A447"/>
     <mergeCell ref="A617:A618"/>
     <mergeCell ref="A271:A277"/>
+    <mergeCell ref="A785:A786"/>
     <mergeCell ref="A1191:A1195"/>
     <mergeCell ref="A448:A449"/>
+    <mergeCell ref="A792:A798"/>
     <mergeCell ref="A210:A214"/>
     <mergeCell ref="A1135:A1136"/>
     <mergeCell ref="A876:A886"/>
@@ -14617,19 +14575,17 @@
     <mergeCell ref="A250:A255"/>
     <mergeCell ref="A57:A63"/>
     <mergeCell ref="A1041:A1067"/>
-    <mergeCell ref="A943:A944"/>
-    <mergeCell ref="A911:A928"/>
     <mergeCell ref="A732:A734"/>
     <mergeCell ref="A261:A263"/>
     <mergeCell ref="A1030:A1032"/>
-    <mergeCell ref="A950:A953"/>
     <mergeCell ref="A155:A159"/>
+    <mergeCell ref="A803:A857"/>
     <mergeCell ref="A501:A508"/>
     <mergeCell ref="A658:A661"/>
     <mergeCell ref="A198:A201"/>
     <mergeCell ref="A722:A724"/>
     <mergeCell ref="A544:A550"/>
-    <mergeCell ref="A782:A784"/>
+    <mergeCell ref="A911:A932"/>
     <mergeCell ref="A518:A522"/>
     <mergeCell ref="A132:A134"/>
     <mergeCell ref="A1111:A1112"/>
@@ -14642,7 +14598,6 @@
     <mergeCell ref="A1185:A1188"/>
     <mergeCell ref="A7:A29"/>
     <mergeCell ref="A1113:A1114"/>
-    <mergeCell ref="A929:A942"/>
     <mergeCell ref="A450:A451"/>
     <mergeCell ref="A332:A333"/>
     <mergeCell ref="A589:A595"/>

</xml_diff>

<commit_message>
Peel B1/N2 device variants from function roots. (#11)
Collapse AOI21B1/AOI21N2/OAI21N2 and *N1 device tails into base
gates (keep AN2 and real compounds like AOI21ND2). Keys 431->423.

Co-authored-by: Cursor Agent <cursoragent@cursor.com>
Co-authored-by: EsaLongs <EsaLongs@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/preview/NP1PP_vs_C1Y_preview.xlsx
+++ b/preview/NP1PP_vs_C1Y_preview.xlsx
@@ -1427,7 +1427,7 @@
       <c r="B92" s="6" t="n"/>
       <c r="C92" s="6" t="inlineStr">
         <is>
-          <t>AOI21D1COT</t>
+          <t>AOI21B1X6COTC</t>
         </is>
       </c>
     </row>
@@ -1436,7 +1436,7 @@
       <c r="B93" s="6" t="n"/>
       <c r="C93" s="6" t="inlineStr">
         <is>
-          <t>AOI21D3COT</t>
+          <t>AOI21D1COT</t>
         </is>
       </c>
     </row>
@@ -1445,7 +1445,7 @@
       <c r="B94" s="6" t="n"/>
       <c r="C94" s="6" t="inlineStr">
         <is>
-          <t>AOI21D4COT</t>
+          <t>AOI21D3COT</t>
         </is>
       </c>
     </row>
@@ -1454,7 +1454,7 @@
       <c r="B95" s="6" t="n"/>
       <c r="C95" s="6" t="inlineStr">
         <is>
-          <t>AOI21D8COT</t>
+          <t>AOI21D4COT</t>
         </is>
       </c>
     </row>
@@ -1463,7 +1463,7 @@
       <c r="B96" s="6" t="n"/>
       <c r="C96" s="6" t="inlineStr">
         <is>
-          <t>AOI21EEQMBDX2APBCOTC</t>
+          <t>AOI21D8COT</t>
         </is>
       </c>
     </row>
@@ -1472,7 +1472,7 @@
       <c r="B97" s="6" t="n"/>
       <c r="C97" s="6" t="inlineStr">
         <is>
-          <t>AOI21SKND3COT</t>
+          <t>AOI21EEQMBDX2APBCOTC</t>
         </is>
       </c>
     </row>
@@ -1481,7 +1481,7 @@
       <c r="B98" s="6" t="n"/>
       <c r="C98" s="6" t="inlineStr">
         <is>
-          <t>AOI21X2APACOTC</t>
+          <t>AOI21N2X2APACOTC</t>
         </is>
       </c>
     </row>
@@ -1490,7 +1490,7 @@
       <c r="B99" s="6" t="n"/>
       <c r="C99" s="6" t="inlineStr">
         <is>
-          <t>AOI21X4APBCOTC</t>
+          <t>AOI21N2X4APACOTC</t>
         </is>
       </c>
     </row>
@@ -1499,7 +1499,7 @@
       <c r="B100" s="6" t="n"/>
       <c r="C100" s="6" t="inlineStr">
         <is>
-          <t>AOI21X6APACOTC</t>
+          <t>AOI21SKND3COT</t>
         </is>
       </c>
     </row>
@@ -1508,82 +1508,82 @@
       <c r="B101" s="6" t="n"/>
       <c r="C101" s="6" t="inlineStr">
         <is>
+          <t>AOI21X2APACOTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="4" t="n"/>
+      <c r="B102" s="6" t="n"/>
+      <c r="C102" s="6" t="inlineStr">
+        <is>
+          <t>AOI21X4APBCOTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="4" t="n"/>
+      <c r="B103" s="6" t="n"/>
+      <c r="C103" s="6" t="inlineStr">
+        <is>
+          <t>AOI21X6APACOTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="4" t="n"/>
+      <c r="B104" s="6" t="n"/>
+      <c r="C104" s="6" t="inlineStr">
+        <is>
           <t>AOI21X8APACOTC</t>
         </is>
       </c>
     </row>
-    <row r="102">
-      <c r="A102" s="7" t="n"/>
-      <c r="B102" s="8" t="n"/>
-      <c r="C102" s="8" t="inlineStr">
+    <row r="105">
+      <c r="A105" s="7" t="n"/>
+      <c r="B105" s="8" t="n"/>
+      <c r="C105" s="8" t="inlineStr">
         <is>
           <t>AOI21X8APBCOTC</t>
         </is>
       </c>
     </row>
-    <row r="103">
-      <c r="A103" s="2" t="inlineStr">
+    <row r="106">
+      <c r="A106" s="2" t="inlineStr">
         <is>
           <t>AOI211
 与或非门</t>
         </is>
       </c>
-      <c r="B103" s="3" t="inlineStr">
+      <c r="B106" s="3" t="inlineStr">
         <is>
           <t>AOI211D2COT</t>
         </is>
       </c>
-      <c r="C103" s="3" t="inlineStr">
+      <c r="C106" s="3" t="inlineStr">
         <is>
           <t>AOI211D2COT</t>
         </is>
       </c>
-    </row>
-    <row r="104">
-      <c r="A104" s="4" t="n"/>
-      <c r="B104" s="5" t="inlineStr">
-        <is>
-          <t>AOI211D3COT</t>
-        </is>
-      </c>
-      <c r="C104" s="5" t="inlineStr">
-        <is>
-          <t>AOI211D3COT</t>
-        </is>
-      </c>
-    </row>
-    <row r="105">
-      <c r="A105" s="4" t="n"/>
-      <c r="B105" s="6" t="inlineStr">
-        <is>
-          <t>AOI211D1COTOPTPA</t>
-        </is>
-      </c>
-      <c r="C105" s="6" t="n"/>
-    </row>
-    <row r="106">
-      <c r="A106" s="4" t="n"/>
-      <c r="B106" s="6" t="inlineStr">
-        <is>
-          <t>AOI211D4COT</t>
-        </is>
-      </c>
-      <c r="C106" s="6" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="4" t="n"/>
-      <c r="B107" s="6" t="inlineStr">
-        <is>
-          <t>AOI211D6COTSKR</t>
-        </is>
-      </c>
-      <c r="C107" s="6" t="n"/>
+      <c r="B107" s="5" t="inlineStr">
+        <is>
+          <t>AOI211D3COT</t>
+        </is>
+      </c>
+      <c r="C107" s="5" t="inlineStr">
+        <is>
+          <t>AOI211D3COT</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="4" t="n"/>
       <c r="B108" s="6" t="inlineStr">
         <is>
-          <t>AOI211D8COTSKF</t>
+          <t>AOI211D1COTOPTPA</t>
         </is>
       </c>
       <c r="C108" s="6" t="n"/>
@@ -1592,177 +1592,167 @@
       <c r="A109" s="4" t="n"/>
       <c r="B109" s="6" t="inlineStr">
         <is>
-          <t>AOI211OPTPAD1COTOPU</t>
+          <t>AOI211D4COT</t>
         </is>
       </c>
       <c r="C109" s="6" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="4" t="n"/>
-      <c r="B110" s="6" t="n"/>
-      <c r="C110" s="6" t="inlineStr">
-        <is>
-          <t>AOI211D0COT</t>
-        </is>
-      </c>
+      <c r="B110" s="6" t="inlineStr">
+        <is>
+          <t>AOI211D6COTSKR</t>
+        </is>
+      </c>
+      <c r="C110" s="6" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="4" t="n"/>
-      <c r="B111" s="6" t="n"/>
-      <c r="C111" s="6" t="inlineStr">
-        <is>
-          <t>AOI211D1COT</t>
-        </is>
-      </c>
+      <c r="B111" s="6" t="inlineStr">
+        <is>
+          <t>AOI211D8COTSKF</t>
+        </is>
+      </c>
+      <c r="C111" s="6" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="4" t="n"/>
-      <c r="B112" s="6" t="n"/>
-      <c r="C112" s="6" t="inlineStr">
-        <is>
-          <t>AOI211D8COT</t>
-        </is>
-      </c>
+      <c r="B112" s="6" t="inlineStr">
+        <is>
+          <t>AOI211OPTPAD1COTOPU</t>
+        </is>
+      </c>
+      <c r="C112" s="6" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="4" t="n"/>
       <c r="B113" s="6" t="n"/>
       <c r="C113" s="6" t="inlineStr">
         <is>
+          <t>AOI211D0COT</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="4" t="n"/>
+      <c r="B114" s="6" t="n"/>
+      <c r="C114" s="6" t="inlineStr">
+        <is>
+          <t>AOI211D1COT</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="4" t="n"/>
+      <c r="B115" s="6" t="n"/>
+      <c r="C115" s="6" t="inlineStr">
+        <is>
+          <t>AOI211D8COT</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="4" t="n"/>
+      <c r="B116" s="6" t="n"/>
+      <c r="C116" s="6" t="inlineStr">
+        <is>
           <t>AOI211X1APBCOTC</t>
         </is>
       </c>
     </row>
-    <row r="114">
-      <c r="A114" s="7" t="n"/>
-      <c r="B114" s="8" t="n"/>
-      <c r="C114" s="8" t="inlineStr">
+    <row r="117">
+      <c r="A117" s="7" t="n"/>
+      <c r="B117" s="8" t="n"/>
+      <c r="C117" s="8" t="inlineStr">
         <is>
           <t>AOI211X4APBCOTC</t>
         </is>
       </c>
     </row>
-    <row r="115">
-      <c r="A115" s="2" t="inlineStr">
+    <row r="118">
+      <c r="A118" s="2" t="inlineStr">
         <is>
           <t>AOI2111
 与或非门</t>
         </is>
       </c>
-      <c r="B115" s="11" t="inlineStr">
+      <c r="B118" s="11" t="inlineStr">
         <is>
           <t>AOI2111D1COT</t>
         </is>
       </c>
-      <c r="C115" s="11" t="n"/>
-    </row>
-    <row r="116">
-      <c r="A116" s="4" t="n"/>
-      <c r="B116" s="6" t="inlineStr">
+      <c r="C118" s="11" t="n"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="4" t="n"/>
+      <c r="B119" s="6" t="inlineStr">
         <is>
           <t>AOI2111D2COT</t>
         </is>
       </c>
-      <c r="C116" s="6" t="n"/>
-    </row>
-    <row r="117">
-      <c r="A117" s="4" t="n"/>
-      <c r="B117" s="6" t="n"/>
-      <c r="C117" s="6" t="inlineStr">
+      <c r="C119" s="6" t="n"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="4" t="n"/>
+      <c r="B120" s="6" t="n"/>
+      <c r="C120" s="6" t="inlineStr">
         <is>
           <t>AOI2111D1COTA</t>
         </is>
       </c>
     </row>
-    <row r="118">
-      <c r="A118" s="7" t="n"/>
-      <c r="B118" s="8" t="n"/>
-      <c r="C118" s="8" t="inlineStr">
+    <row r="121">
+      <c r="A121" s="7" t="n"/>
+      <c r="B121" s="8" t="n"/>
+      <c r="C121" s="8" t="inlineStr">
         <is>
           <t>AOI2111D2COTA</t>
         </is>
       </c>
     </row>
-    <row r="119">
-      <c r="A119" s="2" t="inlineStr">
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
         <is>
           <t>AOI211INV
 复合逻辑门</t>
         </is>
       </c>
-      <c r="B119" s="11" t="inlineStr">
+      <c r="B122" s="11" t="inlineStr">
         <is>
           <t>AOI211INVCCMD1COTVIAG</t>
         </is>
       </c>
-      <c r="C119" s="11" t="n"/>
-    </row>
-    <row r="120">
-      <c r="A120" s="7" t="n"/>
-      <c r="B120" s="8" t="n"/>
-      <c r="C120" s="8" t="inlineStr">
+      <c r="C122" s="11" t="n"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="7" t="n"/>
+      <c r="B123" s="8" t="n"/>
+      <c r="C123" s="8" t="inlineStr">
         <is>
           <t>AOI211INVCCMD2COTA</t>
         </is>
       </c>
     </row>
-    <row r="121">
-      <c r="A121" s="2" t="inlineStr">
+    <row r="124">
+      <c r="A124" s="2" t="inlineStr">
         <is>
           <t>AOI21AOI21
 复合逻辑门</t>
         </is>
       </c>
-      <c r="B121" s="11" t="inlineStr">
+      <c r="B124" s="11" t="inlineStr">
         <is>
           <t>AOI21AOI21CCMD1COT</t>
         </is>
       </c>
-      <c r="C121" s="11" t="n"/>
-    </row>
-    <row r="122">
-      <c r="A122" s="7" t="n"/>
-      <c r="B122" s="8" t="n"/>
-      <c r="C122" s="8" t="inlineStr">
-        <is>
-          <t>AOI21AOI21CCMD1COTA</t>
-        </is>
-      </c>
-    </row>
-    <row r="123">
-      <c r="A123" s="9" t="inlineStr">
-        <is>
-          <t>AOI21B1
-与或非门</t>
-        </is>
-      </c>
-      <c r="B123" s="10" t="n"/>
-      <c r="C123" s="10" t="inlineStr">
-        <is>
-          <t>AOI21B1X6COTC</t>
-        </is>
-      </c>
-    </row>
-    <row r="124">
-      <c r="A124" s="2" t="inlineStr">
-        <is>
-          <t>AOI21N2
-与或非门</t>
-        </is>
-      </c>
-      <c r="B124" s="11" t="n"/>
-      <c r="C124" s="11" t="inlineStr">
-        <is>
-          <t>AOI21N2X2APACOTC</t>
-        </is>
-      </c>
+      <c r="C124" s="11" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="7" t="n"/>
       <c r="B125" s="8" t="n"/>
       <c r="C125" s="8" t="inlineStr">
         <is>
-          <t>AOI21N2X4APACOTC</t>
+          <t>AOI21AOI21CCMD1COTA</t>
         </is>
       </c>
     </row>
@@ -7993,7 +7983,7 @@
     <row r="653">
       <c r="A653" s="2" t="inlineStr">
         <is>
-          <t>LVUFROR2N1
+          <t>LVUFROR2
 电平转换器</t>
         </is>
       </c>
@@ -8016,7 +8006,7 @@
     <row r="655">
       <c r="A655" s="2" t="inlineStr">
         <is>
-          <t>LVUOR2N1
+          <t>LVUOR2
 电平转换器</t>
         </is>
       </c>
@@ -9140,7 +9130,7 @@
       <c r="B757" s="6" t="n"/>
       <c r="C757" s="6" t="inlineStr">
         <is>
-          <t>ND2X10AKPCOTC</t>
+          <t>ND2N1X10APNCOTC</t>
         </is>
       </c>
     </row>
@@ -9149,7 +9139,7 @@
       <c r="B758" s="6" t="n"/>
       <c r="C758" s="6" t="inlineStr">
         <is>
-          <t>ND2X10APBCOTC</t>
+          <t>ND2N1X12APNCOTC</t>
         </is>
       </c>
     </row>
@@ -9158,7 +9148,7 @@
       <c r="B759" s="6" t="n"/>
       <c r="C759" s="6" t="inlineStr">
         <is>
-          <t>ND2X10APNCOTC</t>
+          <t>ND2N1X2AFCOTC</t>
         </is>
       </c>
     </row>
@@ -9167,7 +9157,7 @@
       <c r="B760" s="6" t="n"/>
       <c r="C760" s="6" t="inlineStr">
         <is>
-          <t>ND2X12AKPCOTC</t>
+          <t>ND2N1X4APNCOTC</t>
         </is>
       </c>
     </row>
@@ -9176,7 +9166,7 @@
       <c r="B761" s="6" t="n"/>
       <c r="C761" s="6" t="inlineStr">
         <is>
-          <t>ND2X14APBCOTC</t>
+          <t>ND2N1X6APNCOTC</t>
         </is>
       </c>
     </row>
@@ -9185,7 +9175,7 @@
       <c r="B762" s="6" t="n"/>
       <c r="C762" s="6" t="inlineStr">
         <is>
-          <t>ND2X16APNCOTC</t>
+          <t>ND2X10AKPCOTC</t>
         </is>
       </c>
     </row>
@@ -9194,7 +9184,7 @@
       <c r="B763" s="6" t="n"/>
       <c r="C763" s="6" t="inlineStr">
         <is>
-          <t>ND2X1AKPCOTC</t>
+          <t>ND2X10APBCOTC</t>
         </is>
       </c>
     </row>
@@ -9203,7 +9193,7 @@
       <c r="B764" s="6" t="n"/>
       <c r="C764" s="6" t="inlineStr">
         <is>
-          <t>ND2X1APNCOTC</t>
+          <t>ND2X10APNCOTC</t>
         </is>
       </c>
     </row>
@@ -9212,7 +9202,7 @@
       <c r="B765" s="6" t="n"/>
       <c r="C765" s="6" t="inlineStr">
         <is>
-          <t>ND2X2AKPCOTC</t>
+          <t>ND2X12AKPCOTC</t>
         </is>
       </c>
     </row>
@@ -9221,7 +9211,7 @@
       <c r="B766" s="6" t="n"/>
       <c r="C766" s="6" t="inlineStr">
         <is>
-          <t>ND2X2APBCOTC</t>
+          <t>ND2X14APBCOTC</t>
         </is>
       </c>
     </row>
@@ -9230,7 +9220,7 @@
       <c r="B767" s="6" t="n"/>
       <c r="C767" s="6" t="inlineStr">
         <is>
-          <t>ND2X2APNCOTC</t>
+          <t>ND2X16APNCOTC</t>
         </is>
       </c>
     </row>
@@ -9239,7 +9229,7 @@
       <c r="B768" s="6" t="n"/>
       <c r="C768" s="6" t="inlineStr">
         <is>
-          <t>ND2X3AKPCOT3FINC</t>
+          <t>ND2X1AKPCOTC</t>
         </is>
       </c>
     </row>
@@ -9248,7 +9238,7 @@
       <c r="B769" s="6" t="n"/>
       <c r="C769" s="6" t="inlineStr">
         <is>
-          <t>ND2X4APACOT3FINC</t>
+          <t>ND2X1APNCOTC</t>
         </is>
       </c>
     </row>
@@ -9257,7 +9247,7 @@
       <c r="B770" s="6" t="n"/>
       <c r="C770" s="6" t="inlineStr">
         <is>
-          <t>ND2X4APBCOTC</t>
+          <t>ND2X2AKPCOTC</t>
         </is>
       </c>
     </row>
@@ -9266,7 +9256,7 @@
       <c r="B771" s="6" t="n"/>
       <c r="C771" s="6" t="inlineStr">
         <is>
-          <t>ND2X4APNCOTC</t>
+          <t>ND2X2APBCOTC</t>
         </is>
       </c>
     </row>
@@ -9275,7 +9265,7 @@
       <c r="B772" s="6" t="n"/>
       <c r="C772" s="6" t="inlineStr">
         <is>
-          <t>ND2X4ARQCOT</t>
+          <t>ND2X2APNCOTC</t>
         </is>
       </c>
     </row>
@@ -9284,7 +9274,7 @@
       <c r="B773" s="6" t="n"/>
       <c r="C773" s="6" t="inlineStr">
         <is>
-          <t>ND2X6AKPCOTC</t>
+          <t>ND2X3AKPCOT3FINC</t>
         </is>
       </c>
     </row>
@@ -9293,7 +9283,7 @@
       <c r="B774" s="6" t="n"/>
       <c r="C774" s="6" t="inlineStr">
         <is>
-          <t>ND2X6APNCOTC</t>
+          <t>ND2X4APACOT3FINC</t>
         </is>
       </c>
     </row>
@@ -9302,7 +9292,7 @@
       <c r="B775" s="6" t="n"/>
       <c r="C775" s="6" t="inlineStr">
         <is>
-          <t>ND2X6AROAFCOT</t>
+          <t>ND2X4APBCOTC</t>
         </is>
       </c>
     </row>
@@ -9311,7 +9301,7 @@
       <c r="B776" s="6" t="n"/>
       <c r="C776" s="6" t="inlineStr">
         <is>
-          <t>ND2X6AROCOT</t>
+          <t>ND2X4APNCOTC</t>
         </is>
       </c>
     </row>
@@ -9320,7 +9310,7 @@
       <c r="B777" s="6" t="n"/>
       <c r="C777" s="6" t="inlineStr">
         <is>
-          <t>ND2X8APACOT3FINC</t>
+          <t>ND2X4ARQCOT</t>
         </is>
       </c>
     </row>
@@ -9329,123 +9319,118 @@
       <c r="B778" s="6" t="n"/>
       <c r="C778" s="6" t="inlineStr">
         <is>
+          <t>ND2X6AKPCOTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="779">
+      <c r="A779" s="4" t="n"/>
+      <c r="B779" s="6" t="n"/>
+      <c r="C779" s="6" t="inlineStr">
+        <is>
+          <t>ND2X6APNCOTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="780">
+      <c r="A780" s="4" t="n"/>
+      <c r="B780" s="6" t="n"/>
+      <c r="C780" s="6" t="inlineStr">
+        <is>
+          <t>ND2X6AROAFCOT</t>
+        </is>
+      </c>
+    </row>
+    <row r="781">
+      <c r="A781" s="4" t="n"/>
+      <c r="B781" s="6" t="n"/>
+      <c r="C781" s="6" t="inlineStr">
+        <is>
+          <t>ND2X6AROCOT</t>
+        </is>
+      </c>
+    </row>
+    <row r="782">
+      <c r="A782" s="4" t="n"/>
+      <c r="B782" s="6" t="n"/>
+      <c r="C782" s="6" t="inlineStr">
+        <is>
+          <t>ND2X8APACOT3FINC</t>
+        </is>
+      </c>
+    </row>
+    <row r="783">
+      <c r="A783" s="4" t="n"/>
+      <c r="B783" s="6" t="n"/>
+      <c r="C783" s="6" t="inlineStr">
+        <is>
           <t>ND2X8APBCOTC</t>
         </is>
       </c>
     </row>
-    <row r="779">
-      <c r="A779" s="7" t="n"/>
-      <c r="B779" s="8" t="n"/>
-      <c r="C779" s="8" t="inlineStr">
+    <row r="784">
+      <c r="A784" s="7" t="n"/>
+      <c r="B784" s="8" t="n"/>
+      <c r="C784" s="8" t="inlineStr">
         <is>
           <t>ND2X8APNCOTC</t>
         </is>
       </c>
     </row>
-    <row r="780">
-      <c r="A780" s="2" t="inlineStr">
+    <row r="785">
+      <c r="A785" s="2" t="inlineStr">
         <is>
           <t>ND2AOI21
 复合逻辑门</t>
         </is>
       </c>
-      <c r="B780" s="11" t="inlineStr">
+      <c r="B785" s="11" t="inlineStr">
         <is>
           <t>ND2AOI21CCBD1COT</t>
         </is>
       </c>
-      <c r="C780" s="11" t="n"/>
-    </row>
-    <row r="781">
-      <c r="A781" s="7" t="n"/>
-      <c r="B781" s="8" t="n"/>
-      <c r="C781" s="8" t="inlineStr">
+      <c r="C785" s="11" t="n"/>
+    </row>
+    <row r="786">
+      <c r="A786" s="7" t="n"/>
+      <c r="B786" s="8" t="n"/>
+      <c r="C786" s="8" t="inlineStr">
         <is>
           <t>ND2AOI21CCBD4COTA</t>
         </is>
       </c>
     </row>
-    <row r="782">
-      <c r="A782" s="2" t="inlineStr">
+    <row r="787">
+      <c r="A787" s="2" t="inlineStr">
         <is>
           <t>ND2IOA21
 复合逻辑门</t>
         </is>
       </c>
-      <c r="B782" s="11" t="inlineStr">
+      <c r="B787" s="11" t="inlineStr">
         <is>
           <t>ND2IOA21D1COT</t>
         </is>
       </c>
-      <c r="C782" s="11" t="n"/>
-    </row>
-    <row r="783">
-      <c r="A783" s="4" t="n"/>
-      <c r="B783" s="6" t="inlineStr">
-        <is>
-          <t>ND2IOA21D2COTVIA</t>
-        </is>
-      </c>
-      <c r="C783" s="6" t="n"/>
-    </row>
-    <row r="784">
-      <c r="A784" s="7" t="n"/>
-      <c r="B784" s="8" t="inlineStr">
-        <is>
-          <t>ND2IOA21D4COT</t>
-        </is>
-      </c>
-      <c r="C784" s="8" t="n"/>
-    </row>
-    <row r="785">
-      <c r="A785" s="2" t="inlineStr">
-        <is>
-          <t>ND2N1
-与非门</t>
-        </is>
-      </c>
-      <c r="B785" s="11" t="n"/>
-      <c r="C785" s="11" t="inlineStr">
-        <is>
-          <t>ND2N1X10APNCOTC</t>
-        </is>
-      </c>
-    </row>
-    <row r="786">
-      <c r="A786" s="4" t="n"/>
-      <c r="B786" s="6" t="n"/>
-      <c r="C786" s="6" t="inlineStr">
-        <is>
-          <t>ND2N1X12APNCOTC</t>
-        </is>
-      </c>
-    </row>
-    <row r="787">
-      <c r="A787" s="4" t="n"/>
-      <c r="B787" s="6" t="n"/>
-      <c r="C787" s="6" t="inlineStr">
-        <is>
-          <t>ND2N1X2AFCOTC</t>
-        </is>
-      </c>
+      <c r="C787" s="11" t="n"/>
     </row>
     <row r="788">
       <c r="A788" s="4" t="n"/>
-      <c r="B788" s="6" t="n"/>
-      <c r="C788" s="6" t="inlineStr">
-        <is>
-          <t>ND2N1X4APNCOTC</t>
-        </is>
-      </c>
+      <c r="B788" s="6" t="inlineStr">
+        <is>
+          <t>ND2IOA21D2COTVIA</t>
+        </is>
+      </c>
+      <c r="C788" s="6" t="n"/>
     </row>
     <row r="789">
       <c r="A789" s="7" t="n"/>
-      <c r="B789" s="8" t="n"/>
-      <c r="C789" s="8" t="inlineStr">
-        <is>
-          <t>ND2N1X6APNCOTC</t>
-        </is>
-      </c>
+      <c r="B789" s="8" t="inlineStr">
+        <is>
+          <t>ND2IOA21D4COT</t>
+        </is>
+      </c>
+      <c r="C789" s="8" t="n"/>
     </row>
     <row r="790">
       <c r="A790" s="2" t="inlineStr">
@@ -9498,53 +9483,43 @@
       <c r="B794" s="6" t="n"/>
       <c r="C794" s="6" t="inlineStr">
         <is>
+          <t>ND3N1X4AFCOTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="795">
+      <c r="A795" s="4" t="n"/>
+      <c r="B795" s="6" t="n"/>
+      <c r="C795" s="6" t="inlineStr">
+        <is>
+          <t>ND3N1X8AFCOTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="796">
+      <c r="A796" s="4" t="n"/>
+      <c r="B796" s="6" t="n"/>
+      <c r="C796" s="6" t="inlineStr">
+        <is>
+          <t>ND3N2X6COTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="797">
+      <c r="A797" s="4" t="n"/>
+      <c r="B797" s="6" t="n"/>
+      <c r="C797" s="6" t="inlineStr">
+        <is>
           <t>ND3X3APACOTC</t>
         </is>
       </c>
     </row>
-    <row r="795">
-      <c r="A795" s="7" t="n"/>
-      <c r="B795" s="8" t="n"/>
-      <c r="C795" s="8" t="inlineStr">
+    <row r="798">
+      <c r="A798" s="7" t="n"/>
+      <c r="B798" s="8" t="n"/>
+      <c r="C798" s="8" t="inlineStr">
         <is>
           <t>ND3X6APACOTC</t>
-        </is>
-      </c>
-    </row>
-    <row r="796">
-      <c r="A796" s="2" t="inlineStr">
-        <is>
-          <t>ND3N1
-与非门</t>
-        </is>
-      </c>
-      <c r="B796" s="11" t="n"/>
-      <c r="C796" s="11" t="inlineStr">
-        <is>
-          <t>ND3N1X4AFCOTC</t>
-        </is>
-      </c>
-    </row>
-    <row r="797">
-      <c r="A797" s="7" t="n"/>
-      <c r="B797" s="8" t="n"/>
-      <c r="C797" s="8" t="inlineStr">
-        <is>
-          <t>ND3N1X8AFCOTC</t>
-        </is>
-      </c>
-    </row>
-    <row r="798">
-      <c r="A798" s="9" t="inlineStr">
-        <is>
-          <t>ND3N2
-与非门</t>
-        </is>
-      </c>
-      <c r="B798" s="10" t="n"/>
-      <c r="C798" s="10" t="inlineStr">
-        <is>
-          <t>ND3N2X6COTC</t>
         </is>
       </c>
     </row>
@@ -9572,23 +9547,18 @@
       <c r="C800" s="6" t="n"/>
     </row>
     <row r="801">
-      <c r="A801" s="7" t="n"/>
-      <c r="B801" s="8" t="n"/>
-      <c r="C801" s="8" t="inlineStr">
+      <c r="A801" s="4" t="n"/>
+      <c r="B801" s="6" t="n"/>
+      <c r="C801" s="6" t="inlineStr">
         <is>
           <t>ND4D0COT</t>
         </is>
       </c>
     </row>
     <row r="802">
-      <c r="A802" s="9" t="inlineStr">
-        <is>
-          <t>ND4N1
-与非门</t>
-        </is>
-      </c>
-      <c r="B802" s="10" t="n"/>
-      <c r="C802" s="10" t="inlineStr">
+      <c r="A802" s="7" t="n"/>
+      <c r="B802" s="8" t="n"/>
+      <c r="C802" s="8" t="inlineStr">
         <is>
           <t>ND4N1X6COTC</t>
         </is>
@@ -9761,7 +9731,7 @@
       <c r="B820" s="6" t="n"/>
       <c r="C820" s="6" t="inlineStr">
         <is>
-          <t>NR2SKPD12COT3FIN</t>
+          <t>NR2N1X10APPCOTC</t>
         </is>
       </c>
     </row>
@@ -9770,7 +9740,7 @@
       <c r="B821" s="6" t="n"/>
       <c r="C821" s="6" t="inlineStr">
         <is>
-          <t>NR2X10APBCOTC</t>
+          <t>NR2N1X12APPCOTC</t>
         </is>
       </c>
     </row>
@@ -9779,7 +9749,7 @@
       <c r="B822" s="6" t="n"/>
       <c r="C822" s="6" t="inlineStr">
         <is>
-          <t>NR2X10APPCOTC</t>
+          <t>NR2N1X12AROAFCOT</t>
         </is>
       </c>
     </row>
@@ -9788,7 +9758,7 @@
       <c r="B823" s="6" t="n"/>
       <c r="C823" s="6" t="inlineStr">
         <is>
-          <t>NR2X12AKNCOTC</t>
+          <t>NR2N1X12AROCOT</t>
         </is>
       </c>
     </row>
@@ -9797,7 +9767,7 @@
       <c r="B824" s="6" t="n"/>
       <c r="C824" s="6" t="inlineStr">
         <is>
-          <t>NR2X12APACOTC</t>
+          <t>NR2N1X14APPCOTC</t>
         </is>
       </c>
     </row>
@@ -9806,7 +9776,7 @@
       <c r="B825" s="6" t="n"/>
       <c r="C825" s="6" t="inlineStr">
         <is>
-          <t>NR2X12APPCOTC</t>
+          <t>NR2N1X16APPCOTC</t>
         </is>
       </c>
     </row>
@@ -9815,7 +9785,7 @@
       <c r="B826" s="6" t="n"/>
       <c r="C826" s="6" t="inlineStr">
         <is>
-          <t>NR2X14APBCOTC</t>
+          <t>NR2N1X1APPCOTC</t>
         </is>
       </c>
     </row>
@@ -9824,7 +9794,7 @@
       <c r="B827" s="6" t="n"/>
       <c r="C827" s="6" t="inlineStr">
         <is>
-          <t>NR2X14APPCOTC</t>
+          <t>NR2N1X4APPCOTC</t>
         </is>
       </c>
     </row>
@@ -9833,7 +9803,7 @@
       <c r="B828" s="6" t="n"/>
       <c r="C828" s="6" t="inlineStr">
         <is>
-          <t>NR2X16APACOTC</t>
+          <t>NR2N1X6APPCOTC</t>
         </is>
       </c>
     </row>
@@ -9842,7 +9812,7 @@
       <c r="B829" s="6" t="n"/>
       <c r="C829" s="6" t="inlineStr">
         <is>
-          <t>NR2X16APBCOTC</t>
+          <t>NR2N1X8APPCOTC</t>
         </is>
       </c>
     </row>
@@ -9851,7 +9821,7 @@
       <c r="B830" s="6" t="n"/>
       <c r="C830" s="6" t="inlineStr">
         <is>
-          <t>NR2X16APPCOTC</t>
+          <t>NR2SKPD12COT3FIN</t>
         </is>
       </c>
     </row>
@@ -9860,7 +9830,7 @@
       <c r="B831" s="6" t="n"/>
       <c r="C831" s="6" t="inlineStr">
         <is>
-          <t>NR2X1AKNCOTC</t>
+          <t>NR2X10APBCOTC</t>
         </is>
       </c>
     </row>
@@ -9869,7 +9839,7 @@
       <c r="B832" s="6" t="n"/>
       <c r="C832" s="6" t="inlineStr">
         <is>
-          <t>NR2X1APACOTC</t>
+          <t>NR2X10APPCOTC</t>
         </is>
       </c>
     </row>
@@ -9878,7 +9848,7 @@
       <c r="B833" s="6" t="n"/>
       <c r="C833" s="6" t="inlineStr">
         <is>
-          <t>NR2X1APPCOTC</t>
+          <t>NR2X12AKNCOTC</t>
         </is>
       </c>
     </row>
@@ -9887,7 +9857,7 @@
       <c r="B834" s="6" t="n"/>
       <c r="C834" s="6" t="inlineStr">
         <is>
-          <t>NR2X2AKNCOT3FINC</t>
+          <t>NR2X12APACOTC</t>
         </is>
       </c>
     </row>
@@ -9896,7 +9866,7 @@
       <c r="B835" s="6" t="n"/>
       <c r="C835" s="6" t="inlineStr">
         <is>
-          <t>NR2X2APPCOT3FINC</t>
+          <t>NR2X12APPCOTC</t>
         </is>
       </c>
     </row>
@@ -9905,7 +9875,7 @@
       <c r="B836" s="6" t="n"/>
       <c r="C836" s="6" t="inlineStr">
         <is>
-          <t>NR2X3AKNCOT3FINC</t>
+          <t>NR2X14APBCOTC</t>
         </is>
       </c>
     </row>
@@ -9914,7 +9884,7 @@
       <c r="B837" s="6" t="n"/>
       <c r="C837" s="6" t="inlineStr">
         <is>
-          <t>NR2X4AKNCOTC</t>
+          <t>NR2X14APPCOTC</t>
         </is>
       </c>
     </row>
@@ -9923,7 +9893,7 @@
       <c r="B838" s="6" t="n"/>
       <c r="C838" s="6" t="inlineStr">
         <is>
-          <t>NR2X4APACOTC</t>
+          <t>NR2X16APACOTC</t>
         </is>
       </c>
     </row>
@@ -9932,7 +9902,7 @@
       <c r="B839" s="6" t="n"/>
       <c r="C839" s="6" t="inlineStr">
         <is>
-          <t>NR2X4APBCOTC</t>
+          <t>NR2X16APBCOTC</t>
         </is>
       </c>
     </row>
@@ -9941,7 +9911,7 @@
       <c r="B840" s="6" t="n"/>
       <c r="C840" s="6" t="inlineStr">
         <is>
-          <t>NR2X4ARQCOT</t>
+          <t>NR2X16APPCOTC</t>
         </is>
       </c>
     </row>
@@ -9950,7 +9920,7 @@
       <c r="B841" s="6" t="n"/>
       <c r="C841" s="6" t="inlineStr">
         <is>
-          <t>NR2X6APACOTC</t>
+          <t>NR2X1AKNCOTC</t>
         </is>
       </c>
     </row>
@@ -9959,7 +9929,7 @@
       <c r="B842" s="6" t="n"/>
       <c r="C842" s="6" t="inlineStr">
         <is>
-          <t>NR2X6APBCOTC</t>
+          <t>NR2X1APACOTC</t>
         </is>
       </c>
     </row>
@@ -9968,7 +9938,7 @@
       <c r="B843" s="6" t="n"/>
       <c r="C843" s="6" t="inlineStr">
         <is>
-          <t>NR2X6ARQCOT</t>
+          <t>NR2X1APPCOTC</t>
         </is>
       </c>
     </row>
@@ -9977,7 +9947,7 @@
       <c r="B844" s="6" t="n"/>
       <c r="C844" s="6" t="inlineStr">
         <is>
-          <t>NR2X8APACOTC</t>
+          <t>NR2X2AKNCOT3FINC</t>
         </is>
       </c>
     </row>
@@ -9986,7 +9956,7 @@
       <c r="B845" s="6" t="n"/>
       <c r="C845" s="6" t="inlineStr">
         <is>
-          <t>NR2X8APBCOTC</t>
+          <t>NR2X2APPCOT3FINC</t>
         </is>
       </c>
     </row>
@@ -9995,53 +9965,43 @@
       <c r="B846" s="6" t="n"/>
       <c r="C846" s="6" t="inlineStr">
         <is>
-          <t>NR2X8APPCOTC</t>
+          <t>NR2X3AKNCOT3FINC</t>
         </is>
       </c>
     </row>
     <row r="847">
-      <c r="A847" s="7" t="n"/>
-      <c r="B847" s="8" t="n"/>
-      <c r="C847" s="8" t="inlineStr">
-        <is>
-          <t>NR2X8AROCOT</t>
+      <c r="A847" s="4" t="n"/>
+      <c r="B847" s="6" t="n"/>
+      <c r="C847" s="6" t="inlineStr">
+        <is>
+          <t>NR2X4AKNCOTC</t>
         </is>
       </c>
     </row>
     <row r="848">
-      <c r="A848" s="2" t="inlineStr">
-        <is>
-          <t>NR2AOI21
-复合逻辑门</t>
-        </is>
-      </c>
-      <c r="B848" s="11" t="inlineStr">
-        <is>
-          <t>NR2AOI21CCBD4COT</t>
-        </is>
-      </c>
-      <c r="C848" s="11" t="n"/>
+      <c r="A848" s="4" t="n"/>
+      <c r="B848" s="6" t="n"/>
+      <c r="C848" s="6" t="inlineStr">
+        <is>
+          <t>NR2X4APACOTC</t>
+        </is>
+      </c>
     </row>
     <row r="849">
-      <c r="A849" s="7" t="n"/>
-      <c r="B849" s="8" t="n"/>
-      <c r="C849" s="8" t="inlineStr">
-        <is>
-          <t>NR2AOI21CCBD2COT</t>
+      <c r="A849" s="4" t="n"/>
+      <c r="B849" s="6" t="n"/>
+      <c r="C849" s="6" t="inlineStr">
+        <is>
+          <t>NR2X4APBCOTC</t>
         </is>
       </c>
     </row>
     <row r="850">
-      <c r="A850" s="2" t="inlineStr">
-        <is>
-          <t>NR2N1
-或非门</t>
-        </is>
-      </c>
-      <c r="B850" s="11" t="n"/>
-      <c r="C850" s="11" t="inlineStr">
-        <is>
-          <t>NR2N1X10APPCOTC</t>
+      <c r="A850" s="4" t="n"/>
+      <c r="B850" s="6" t="n"/>
+      <c r="C850" s="6" t="inlineStr">
+        <is>
+          <t>NR2X4ARQCOT</t>
         </is>
       </c>
     </row>
@@ -10050,7 +10010,7 @@
       <c r="B851" s="6" t="n"/>
       <c r="C851" s="6" t="inlineStr">
         <is>
-          <t>NR2N1X12APPCOTC</t>
+          <t>NR2X6APACOTC</t>
         </is>
       </c>
     </row>
@@ -10059,7 +10019,7 @@
       <c r="B852" s="6" t="n"/>
       <c r="C852" s="6" t="inlineStr">
         <is>
-          <t>NR2N1X12AROAFCOT</t>
+          <t>NR2X6APBCOTC</t>
         </is>
       </c>
     </row>
@@ -10068,7 +10028,7 @@
       <c r="B853" s="6" t="n"/>
       <c r="C853" s="6" t="inlineStr">
         <is>
-          <t>NR2N1X12AROCOT</t>
+          <t>NR2X6ARQCOT</t>
         </is>
       </c>
     </row>
@@ -10077,7 +10037,7 @@
       <c r="B854" s="6" t="n"/>
       <c r="C854" s="6" t="inlineStr">
         <is>
-          <t>NR2N1X14APPCOTC</t>
+          <t>NR2X8APACOTC</t>
         </is>
       </c>
     </row>
@@ -10086,7 +10046,7 @@
       <c r="B855" s="6" t="n"/>
       <c r="C855" s="6" t="inlineStr">
         <is>
-          <t>NR2N1X16APPCOTC</t>
+          <t>NR2X8APBCOTC</t>
         </is>
       </c>
     </row>
@@ -10095,34 +10055,39 @@
       <c r="B856" s="6" t="n"/>
       <c r="C856" s="6" t="inlineStr">
         <is>
-          <t>NR2N1X1APPCOTC</t>
+          <t>NR2X8APPCOTC</t>
         </is>
       </c>
     </row>
     <row r="857">
-      <c r="A857" s="4" t="n"/>
-      <c r="B857" s="6" t="n"/>
-      <c r="C857" s="6" t="inlineStr">
-        <is>
-          <t>NR2N1X4APPCOTC</t>
+      <c r="A857" s="7" t="n"/>
+      <c r="B857" s="8" t="n"/>
+      <c r="C857" s="8" t="inlineStr">
+        <is>
+          <t>NR2X8AROCOT</t>
         </is>
       </c>
     </row>
     <row r="858">
-      <c r="A858" s="4" t="n"/>
-      <c r="B858" s="6" t="n"/>
-      <c r="C858" s="6" t="inlineStr">
-        <is>
-          <t>NR2N1X6APPCOTC</t>
-        </is>
-      </c>
+      <c r="A858" s="2" t="inlineStr">
+        <is>
+          <t>NR2AOI21
+复合逻辑门</t>
+        </is>
+      </c>
+      <c r="B858" s="11" t="inlineStr">
+        <is>
+          <t>NR2AOI21CCBD4COT</t>
+        </is>
+      </c>
+      <c r="C858" s="11" t="n"/>
     </row>
     <row r="859">
       <c r="A859" s="7" t="n"/>
       <c r="B859" s="8" t="n"/>
       <c r="C859" s="8" t="inlineStr">
         <is>
-          <t>NR2N1X8APPCOTC</t>
+          <t>NR2AOI21CCBD2COT</t>
         </is>
       </c>
     </row>
@@ -10755,7 +10720,7 @@
       <c r="B923" s="6" t="n"/>
       <c r="C923" s="6" t="inlineStr">
         <is>
-          <t>OAI21OPTLD4COT</t>
+          <t>OAI21N2X2APACOTC</t>
         </is>
       </c>
     </row>
@@ -10764,7 +10729,7 @@
       <c r="B924" s="6" t="n"/>
       <c r="C924" s="6" t="inlineStr">
         <is>
-          <t>OAI21X1APACOTC</t>
+          <t>OAI21N2X6APACOTC</t>
         </is>
       </c>
     </row>
@@ -10773,7 +10738,7 @@
       <c r="B925" s="6" t="n"/>
       <c r="C925" s="6" t="inlineStr">
         <is>
-          <t>OAI21X3APACOTC</t>
+          <t>OAI21N2X8APACOTC</t>
         </is>
       </c>
     </row>
@@ -10782,7 +10747,7 @@
       <c r="B926" s="6" t="n"/>
       <c r="C926" s="6" t="inlineStr">
         <is>
-          <t>OAI21X4APACOTC</t>
+          <t>OAI21N2X8COTC</t>
         </is>
       </c>
     </row>
@@ -10791,74 +10756,74 @@
       <c r="B927" s="6" t="n"/>
       <c r="C927" s="6" t="inlineStr">
         <is>
+          <t>OAI21OPTLD4COT</t>
+        </is>
+      </c>
+    </row>
+    <row r="928">
+      <c r="A928" s="4" t="n"/>
+      <c r="B928" s="6" t="n"/>
+      <c r="C928" s="6" t="inlineStr">
+        <is>
+          <t>OAI21X1APACOTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="929">
+      <c r="A929" s="4" t="n"/>
+      <c r="B929" s="6" t="n"/>
+      <c r="C929" s="6" t="inlineStr">
+        <is>
+          <t>OAI21X3APACOTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="930">
+      <c r="A930" s="4" t="n"/>
+      <c r="B930" s="6" t="n"/>
+      <c r="C930" s="6" t="inlineStr">
+        <is>
+          <t>OAI21X4APACOTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="931">
+      <c r="A931" s="4" t="n"/>
+      <c r="B931" s="6" t="n"/>
+      <c r="C931" s="6" t="inlineStr">
+        <is>
           <t>OAI21X6APACOTC</t>
         </is>
       </c>
     </row>
-    <row r="928">
-      <c r="A928" s="7" t="n"/>
-      <c r="B928" s="8" t="n"/>
-      <c r="C928" s="8" t="inlineStr">
+    <row r="932">
+      <c r="A932" s="7" t="n"/>
+      <c r="B932" s="8" t="n"/>
+      <c r="C932" s="8" t="inlineStr">
         <is>
           <t>OAI21X8APACOTC</t>
         </is>
       </c>
     </row>
-    <row r="929">
-      <c r="A929" s="2" t="inlineStr">
+    <row r="933">
+      <c r="A933" s="2" t="inlineStr">
         <is>
           <t>OAI211
 或与非门</t>
         </is>
       </c>
-      <c r="B929" s="11" t="inlineStr">
+      <c r="B933" s="11" t="inlineStr">
         <is>
           <t>OAI211D1COTOPU</t>
         </is>
       </c>
-      <c r="C929" s="11" t="n"/>
-    </row>
-    <row r="930">
-      <c r="A930" s="4" t="n"/>
-      <c r="B930" s="6" t="inlineStr">
-        <is>
-          <t>OAI211D2COT</t>
-        </is>
-      </c>
-      <c r="C930" s="6" t="n"/>
-    </row>
-    <row r="931">
-      <c r="A931" s="4" t="n"/>
-      <c r="B931" s="6" t="inlineStr">
-        <is>
-          <t>OAI211D3COTSKF</t>
-        </is>
-      </c>
-      <c r="C931" s="6" t="n"/>
-    </row>
-    <row r="932">
-      <c r="A932" s="4" t="n"/>
-      <c r="B932" s="6" t="inlineStr">
-        <is>
-          <t>OAI211D4COTOPTPA</t>
-        </is>
-      </c>
-      <c r="C932" s="6" t="n"/>
-    </row>
-    <row r="933">
-      <c r="A933" s="4" t="n"/>
-      <c r="B933" s="6" t="inlineStr">
-        <is>
-          <t>OAI211D6COTOPTPA</t>
-        </is>
-      </c>
-      <c r="C933" s="6" t="n"/>
+      <c r="C933" s="11" t="n"/>
     </row>
     <row r="934">
       <c r="A934" s="4" t="n"/>
       <c r="B934" s="6" t="inlineStr">
         <is>
-          <t>OAI211D8COTSKR</t>
+          <t>OAI211D2COT</t>
         </is>
       </c>
       <c r="C934" s="6" t="n"/>
@@ -10867,53 +10832,53 @@
       <c r="A935" s="4" t="n"/>
       <c r="B935" s="6" t="inlineStr">
         <is>
-          <t>OAI211OPTPAD1COTOPU</t>
+          <t>OAI211D3COTSKF</t>
         </is>
       </c>
       <c r="C935" s="6" t="n"/>
     </row>
     <row r="936">
       <c r="A936" s="4" t="n"/>
-      <c r="B936" s="6" t="n"/>
-      <c r="C936" s="6" t="inlineStr">
-        <is>
-          <t>OAI211D1COT</t>
-        </is>
-      </c>
+      <c r="B936" s="6" t="inlineStr">
+        <is>
+          <t>OAI211D4COTOPTPA</t>
+        </is>
+      </c>
+      <c r="C936" s="6" t="n"/>
     </row>
     <row r="937">
       <c r="A937" s="4" t="n"/>
-      <c r="B937" s="6" t="n"/>
-      <c r="C937" s="6" t="inlineStr">
-        <is>
-          <t>OAI211D3COT</t>
-        </is>
-      </c>
+      <c r="B937" s="6" t="inlineStr">
+        <is>
+          <t>OAI211D6COTOPTPA</t>
+        </is>
+      </c>
+      <c r="C937" s="6" t="n"/>
     </row>
     <row r="938">
       <c r="A938" s="4" t="n"/>
-      <c r="B938" s="6" t="n"/>
-      <c r="C938" s="6" t="inlineStr">
-        <is>
-          <t>OAI211D4COT</t>
-        </is>
-      </c>
+      <c r="B938" s="6" t="inlineStr">
+        <is>
+          <t>OAI211D8COTSKR</t>
+        </is>
+      </c>
+      <c r="C938" s="6" t="n"/>
     </row>
     <row r="939">
       <c r="A939" s="4" t="n"/>
-      <c r="B939" s="6" t="n"/>
-      <c r="C939" s="6" t="inlineStr">
-        <is>
-          <t>OAI211D6COT</t>
-        </is>
-      </c>
+      <c r="B939" s="6" t="inlineStr">
+        <is>
+          <t>OAI211OPTPAD1COTOPU</t>
+        </is>
+      </c>
+      <c r="C939" s="6" t="n"/>
     </row>
     <row r="940">
       <c r="A940" s="4" t="n"/>
       <c r="B940" s="6" t="n"/>
       <c r="C940" s="6" t="inlineStr">
         <is>
-          <t>OAI211D8COT</t>
+          <t>OAI211D1COT</t>
         </is>
       </c>
     </row>
@@ -10922,142 +10887,137 @@
       <c r="B941" s="6" t="n"/>
       <c r="C941" s="6" t="inlineStr">
         <is>
+          <t>OAI211D3COT</t>
+        </is>
+      </c>
+    </row>
+    <row r="942">
+      <c r="A942" s="4" t="n"/>
+      <c r="B942" s="6" t="n"/>
+      <c r="C942" s="6" t="inlineStr">
+        <is>
+          <t>OAI211D4COT</t>
+        </is>
+      </c>
+    </row>
+    <row r="943">
+      <c r="A943" s="4" t="n"/>
+      <c r="B943" s="6" t="n"/>
+      <c r="C943" s="6" t="inlineStr">
+        <is>
+          <t>OAI211D6COT</t>
+        </is>
+      </c>
+    </row>
+    <row r="944">
+      <c r="A944" s="4" t="n"/>
+      <c r="B944" s="6" t="n"/>
+      <c r="C944" s="6" t="inlineStr">
+        <is>
+          <t>OAI211D8COT</t>
+        </is>
+      </c>
+    </row>
+    <row r="945">
+      <c r="A945" s="4" t="n"/>
+      <c r="B945" s="6" t="n"/>
+      <c r="C945" s="6" t="inlineStr">
+        <is>
           <t>OAI211OPTPAD6COT</t>
         </is>
       </c>
     </row>
-    <row r="942">
-      <c r="A942" s="7" t="n"/>
-      <c r="B942" s="8" t="n"/>
-      <c r="C942" s="8" t="inlineStr">
+    <row r="946">
+      <c r="A946" s="7" t="n"/>
+      <c r="B946" s="8" t="n"/>
+      <c r="C946" s="8" t="inlineStr">
         <is>
           <t>OAI211X2APBCOTC</t>
         </is>
       </c>
     </row>
-    <row r="943">
-      <c r="A943" s="2" t="inlineStr">
+    <row r="947">
+      <c r="A947" s="2" t="inlineStr">
         <is>
           <t>OAI2111
 或与非门</t>
         </is>
       </c>
-      <c r="B943" s="11" t="inlineStr">
+      <c r="B947" s="11" t="inlineStr">
         <is>
           <t>OAI2111D1COT</t>
         </is>
       </c>
-      <c r="C943" s="11" t="n"/>
-    </row>
-    <row r="944">
-      <c r="A944" s="7" t="n"/>
-      <c r="B944" s="8" t="inlineStr">
+      <c r="C947" s="11" t="n"/>
+    </row>
+    <row r="948">
+      <c r="A948" s="7" t="n"/>
+      <c r="B948" s="8" t="inlineStr">
         <is>
           <t>OAI2111D2COT</t>
         </is>
       </c>
-      <c r="C944" s="8" t="n"/>
-    </row>
-    <row r="945">
-      <c r="A945" s="9" t="inlineStr">
+      <c r="C948" s="8" t="n"/>
+    </row>
+    <row r="949">
+      <c r="A949" s="9" t="inlineStr">
         <is>
           <t>OAI211INV
 复合逻辑门</t>
         </is>
       </c>
-      <c r="B945" s="10" t="inlineStr">
+      <c r="B949" s="10" t="inlineStr">
         <is>
           <t>OAI211INVCCAD1COTVIAG</t>
         </is>
       </c>
-      <c r="C945" s="10" t="n"/>
-    </row>
-    <row r="946">
-      <c r="A946" s="9" t="inlineStr">
+      <c r="C949" s="10" t="n"/>
+    </row>
+    <row r="950">
+      <c r="A950" s="9" t="inlineStr">
         <is>
           <t>OAI21AOI21
 复合逻辑门</t>
         </is>
       </c>
-      <c r="B946" s="10" t="n"/>
-      <c r="C946" s="10" t="inlineStr">
+      <c r="B950" s="10" t="n"/>
+      <c r="C950" s="10" t="inlineStr">
         <is>
           <t>OAI21AOI21CCBD4COTA</t>
         </is>
       </c>
     </row>
-    <row r="947">
-      <c r="A947" s="2" t="inlineStr">
+    <row r="951">
+      <c r="A951" s="2" t="inlineStr">
         <is>
           <t>OAI21AOI22
 复合逻辑门</t>
         </is>
       </c>
-      <c r="B947" s="11" t="inlineStr">
+      <c r="B951" s="11" t="inlineStr">
         <is>
           <t>OAI21AOI22D1COT</t>
         </is>
       </c>
-      <c r="C947" s="11" t="n"/>
-    </row>
-    <row r="948">
-      <c r="A948" s="4" t="n"/>
-      <c r="B948" s="6" t="inlineStr">
-        <is>
-          <t>OAI21AOI22D2COT</t>
-        </is>
-      </c>
-      <c r="C948" s="6" t="n"/>
-    </row>
-    <row r="949">
-      <c r="A949" s="7" t="n"/>
-      <c r="B949" s="8" t="inlineStr">
-        <is>
-          <t>OAI21AOI22D4COT</t>
-        </is>
-      </c>
-      <c r="C949" s="8" t="n"/>
-    </row>
-    <row r="950">
-      <c r="A950" s="2" t="inlineStr">
-        <is>
-          <t>OAI21N2
-或与非门</t>
-        </is>
-      </c>
-      <c r="B950" s="11" t="n"/>
-      <c r="C950" s="11" t="inlineStr">
-        <is>
-          <t>OAI21N2X2APACOTC</t>
-        </is>
-      </c>
-    </row>
-    <row r="951">
-      <c r="A951" s="4" t="n"/>
-      <c r="B951" s="6" t="n"/>
-      <c r="C951" s="6" t="inlineStr">
-        <is>
-          <t>OAI21N2X6APACOTC</t>
-        </is>
-      </c>
+      <c r="C951" s="11" t="n"/>
     </row>
     <row r="952">
       <c r="A952" s="4" t="n"/>
-      <c r="B952" s="6" t="n"/>
-      <c r="C952" s="6" t="inlineStr">
-        <is>
-          <t>OAI21N2X8APACOTC</t>
-        </is>
-      </c>
+      <c r="B952" s="6" t="inlineStr">
+        <is>
+          <t>OAI21AOI22D2COT</t>
+        </is>
+      </c>
+      <c r="C952" s="6" t="n"/>
     </row>
     <row r="953">
       <c r="A953" s="7" t="n"/>
-      <c r="B953" s="8" t="n"/>
-      <c r="C953" s="8" t="inlineStr">
-        <is>
-          <t>OAI21N2X8COTC</t>
-        </is>
-      </c>
+      <c r="B953" s="8" t="inlineStr">
+        <is>
+          <t>OAI21AOI22D4COT</t>
+        </is>
+      </c>
+      <c r="C953" s="8" t="n"/>
     </row>
     <row r="954">
       <c r="A954" s="2" t="inlineStr">
@@ -14440,14 +14400,16 @@
       <c r="C1261" s="10" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="224">
+  <mergeCells count="219">
     <mergeCell ref="A540:A543"/>
+    <mergeCell ref="A106:A117"/>
     <mergeCell ref="A378:A384"/>
     <mergeCell ref="A399:A400"/>
     <mergeCell ref="A268:A269"/>
     <mergeCell ref="A701:A706"/>
     <mergeCell ref="A1139:A1140"/>
     <mergeCell ref="A649:A650"/>
+    <mergeCell ref="A947:A948"/>
     <mergeCell ref="A335:A336"/>
     <mergeCell ref="A690:A691"/>
     <mergeCell ref="A966:A977"/>
@@ -14459,27 +14421,22 @@
     <mergeCell ref="A582:A583"/>
     <mergeCell ref="A1141:A1142"/>
     <mergeCell ref="A236:A237"/>
-    <mergeCell ref="A792:A795"/>
     <mergeCell ref="A71:A74"/>
     <mergeCell ref="A189:A192"/>
     <mergeCell ref="A989:A990"/>
     <mergeCell ref="A1075:A1083"/>
     <mergeCell ref="A164:A167"/>
-    <mergeCell ref="A785:A789"/>
     <mergeCell ref="A675:A676"/>
     <mergeCell ref="A1175:A1178"/>
     <mergeCell ref="A244:A247"/>
-    <mergeCell ref="A103:A114"/>
     <mergeCell ref="A1021:A1025"/>
     <mergeCell ref="A1232:A1236"/>
     <mergeCell ref="A730:A731"/>
     <mergeCell ref="A1011:A1015"/>
     <mergeCell ref="A790:A791"/>
     <mergeCell ref="A905:A909"/>
-    <mergeCell ref="A115:A118"/>
     <mergeCell ref="A1036:A1040"/>
     <mergeCell ref="A961:A964"/>
-    <mergeCell ref="A780:A781"/>
     <mergeCell ref="A320:A321"/>
     <mergeCell ref="A403:A404"/>
     <mergeCell ref="A714:A716"/>
@@ -14491,10 +14448,8 @@
     <mergeCell ref="A480:A481"/>
     <mergeCell ref="A256:A257"/>
     <mergeCell ref="A427:A428"/>
-    <mergeCell ref="A747:A779"/>
     <mergeCell ref="A1033:A1035"/>
     <mergeCell ref="A1105:A1106"/>
-    <mergeCell ref="A119:A120"/>
     <mergeCell ref="A569:A576"/>
     <mergeCell ref="A359:A360"/>
     <mergeCell ref="A719:A721"/>
@@ -14526,14 +14481,13 @@
     <mergeCell ref="A160:A163"/>
     <mergeCell ref="A64:A70"/>
     <mergeCell ref="A622:A623"/>
-    <mergeCell ref="A121:A122"/>
+    <mergeCell ref="A858:A859"/>
+    <mergeCell ref="A787:A789"/>
     <mergeCell ref="A357:A358"/>
     <mergeCell ref="A681:A682"/>
     <mergeCell ref="A1092:A1095"/>
-    <mergeCell ref="A848:A849"/>
     <mergeCell ref="A344:A345"/>
     <mergeCell ref="A615:A616"/>
-    <mergeCell ref="A947:A949"/>
     <mergeCell ref="A407:A408"/>
     <mergeCell ref="A667:A669"/>
     <mergeCell ref="A631:A636"/>
@@ -14543,27 +14497,24 @@
     <mergeCell ref="A126:A128"/>
     <mergeCell ref="A534:A539"/>
     <mergeCell ref="A1125:A1130"/>
-    <mergeCell ref="A803:A847"/>
     <mergeCell ref="A1068:A1074"/>
     <mergeCell ref="A1239:A1245"/>
     <mergeCell ref="A983:A984"/>
     <mergeCell ref="A887:A891"/>
     <mergeCell ref="A1201:A1217"/>
     <mergeCell ref="A473:A474"/>
-    <mergeCell ref="A796:A797"/>
     <mergeCell ref="A1151:A1152"/>
-    <mergeCell ref="A85:A102"/>
     <mergeCell ref="A551:A554"/>
     <mergeCell ref="A457:A458"/>
-    <mergeCell ref="A799:A801"/>
     <mergeCell ref="A264:A265"/>
     <mergeCell ref="A1147:A1148"/>
     <mergeCell ref="A326:A327"/>
+    <mergeCell ref="A118:A121"/>
+    <mergeCell ref="A951:A953"/>
     <mergeCell ref="A1154:A1171"/>
     <mergeCell ref="A425:A426"/>
     <mergeCell ref="A860:A862"/>
     <mergeCell ref="A600:A604"/>
-    <mergeCell ref="A850:A859"/>
     <mergeCell ref="A376:A377"/>
     <mergeCell ref="A735:A746"/>
     <mergeCell ref="A717:A718"/>
@@ -14583,15 +14534,19 @@
     <mergeCell ref="A898:A904"/>
     <mergeCell ref="A991:A999"/>
     <mergeCell ref="A179:A184"/>
+    <mergeCell ref="A122:A123"/>
     <mergeCell ref="A411:A412"/>
+    <mergeCell ref="A651:A652"/>
     <mergeCell ref="A670:A673"/>
-    <mergeCell ref="A651:A652"/>
     <mergeCell ref="A1004:A1005"/>
     <mergeCell ref="A1228:A1230"/>
     <mergeCell ref="A258:A259"/>
     <mergeCell ref="A185:A188"/>
+    <mergeCell ref="A933:A946"/>
     <mergeCell ref="A363:A365"/>
     <mergeCell ref="A1107:A1108"/>
+    <mergeCell ref="A747:A784"/>
+    <mergeCell ref="A799:A802"/>
     <mergeCell ref="A523:A527"/>
     <mergeCell ref="A391:A392"/>
     <mergeCell ref="A1100:A1101"/>
@@ -14601,11 +14556,14 @@
     <mergeCell ref="A707:A708"/>
     <mergeCell ref="A1219:A1223"/>
     <mergeCell ref="A985:A988"/>
+    <mergeCell ref="A85:A105"/>
     <mergeCell ref="A446:A447"/>
     <mergeCell ref="A617:A618"/>
     <mergeCell ref="A271:A277"/>
+    <mergeCell ref="A785:A786"/>
     <mergeCell ref="A1191:A1195"/>
     <mergeCell ref="A448:A449"/>
+    <mergeCell ref="A792:A798"/>
     <mergeCell ref="A210:A214"/>
     <mergeCell ref="A1135:A1136"/>
     <mergeCell ref="A876:A886"/>
@@ -14617,19 +14575,17 @@
     <mergeCell ref="A250:A255"/>
     <mergeCell ref="A57:A63"/>
     <mergeCell ref="A1041:A1067"/>
-    <mergeCell ref="A943:A944"/>
-    <mergeCell ref="A911:A928"/>
     <mergeCell ref="A732:A734"/>
     <mergeCell ref="A261:A263"/>
     <mergeCell ref="A1030:A1032"/>
-    <mergeCell ref="A950:A953"/>
     <mergeCell ref="A155:A159"/>
+    <mergeCell ref="A803:A857"/>
     <mergeCell ref="A501:A508"/>
     <mergeCell ref="A658:A661"/>
     <mergeCell ref="A198:A201"/>
     <mergeCell ref="A722:A724"/>
     <mergeCell ref="A544:A550"/>
-    <mergeCell ref="A782:A784"/>
+    <mergeCell ref="A911:A932"/>
     <mergeCell ref="A518:A522"/>
     <mergeCell ref="A132:A134"/>
     <mergeCell ref="A1111:A1112"/>
@@ -14642,7 +14598,6 @@
     <mergeCell ref="A1185:A1188"/>
     <mergeCell ref="A7:A29"/>
     <mergeCell ref="A1113:A1114"/>
-    <mergeCell ref="A929:A942"/>
     <mergeCell ref="A450:A451"/>
     <mergeCell ref="A332:A333"/>
     <mergeCell ref="A589:A595"/>

</xml_diff>

<commit_message>
Collapse layout cell families into BOUNDARY/HDDICWY/HDDID.
All BOUNDARY* variants share one key; HDDICWY* and HDDID* sized
layout cells likewise. Keys 423->401 with full coverage.

Co-authored-by: EsaLongs <EsaLongs@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/preview/NP1PP_vs_C1Y_preview.xlsx
+++ b/preview/NP1PP_vs_C1Y_preview.xlsx
@@ -2787,339 +2787,239 @@
       </c>
     </row>
     <row r="222">
-      <c r="A222" s="9" t="inlineStr">
-        <is>
-          <t>BOUNDARYCNREXRN
+      <c r="A222" s="2" t="inlineStr">
+        <is>
+          <t>BOUNDARY
 边界/版图单元</t>
         </is>
       </c>
-      <c r="B222" s="12" t="inlineStr">
+      <c r="B222" s="3" t="inlineStr">
         <is>
           <t>BOUNDARYCNREXRNCOT</t>
         </is>
       </c>
-      <c r="C222" s="12" t="inlineStr">
+      <c r="C222" s="3" t="inlineStr">
         <is>
           <t>BOUNDARYCNREXRNCOT</t>
         </is>
       </c>
     </row>
     <row r="223">
-      <c r="A223" s="9" t="inlineStr">
-        <is>
-          <t>BOUNDARYCNREXRN6
-边界/版图单元</t>
-        </is>
-      </c>
-      <c r="B223" s="10" t="n"/>
-      <c r="C223" s="10" t="inlineStr">
+      <c r="A223" s="4" t="n"/>
+      <c r="B223" s="5" t="inlineStr">
+        <is>
+          <t>BOUNDARYCNREXRPCOT</t>
+        </is>
+      </c>
+      <c r="C223" s="5" t="inlineStr">
+        <is>
+          <t>BOUNDARYCNREXRPCOT</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" s="4" t="n"/>
+      <c r="B224" s="5" t="inlineStr">
+        <is>
+          <t>BOUNDARYCOLN1COT</t>
+        </is>
+      </c>
+      <c r="C224" s="5" t="inlineStr">
+        <is>
+          <t>BOUNDARYCOLN1COT</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="4" t="n"/>
+      <c r="B225" s="5" t="inlineStr">
+        <is>
+          <t>BOUNDARYCOLN2COT</t>
+        </is>
+      </c>
+      <c r="C225" s="5" t="inlineStr">
+        <is>
+          <t>BOUNDARYCOLN2COT</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="4" t="n"/>
+      <c r="B226" s="5" t="inlineStr">
+        <is>
+          <t>BOUNDARYCOLP1COT</t>
+        </is>
+      </c>
+      <c r="C226" s="5" t="inlineStr">
+        <is>
+          <t>BOUNDARYCOLP1COT</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="4" t="n"/>
+      <c r="B227" s="5" t="inlineStr">
+        <is>
+          <t>BOUNDARYCOLPGAPCOT</t>
+        </is>
+      </c>
+      <c r="C227" s="5" t="inlineStr">
+        <is>
+          <t>BOUNDARYCOLPGAPCOT</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="4" t="n"/>
+      <c r="B228" s="5" t="inlineStr">
+        <is>
+          <t>BOUNDARYICNREXRN6COT</t>
+        </is>
+      </c>
+      <c r="C228" s="5" t="inlineStr">
+        <is>
+          <t>BOUNDARYICNREXRN6COT</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="4" t="n"/>
+      <c r="B229" s="5" t="inlineStr">
+        <is>
+          <t>BOUNDARYICNREXRP6COT</t>
+        </is>
+      </c>
+      <c r="C229" s="5" t="inlineStr">
+        <is>
+          <t>BOUNDARYICNREXRP6COT</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" s="4" t="n"/>
+      <c r="B230" s="6" t="inlineStr">
+        <is>
+          <t>BOUNDARYCOLNGAPCOT</t>
+        </is>
+      </c>
+      <c r="C230" s="6" t="n"/>
+    </row>
+    <row r="231">
+      <c r="A231" s="4" t="n"/>
+      <c r="B231" s="6" t="inlineStr">
+        <is>
+          <t>BOUNDARYCOLP2COT</t>
+        </is>
+      </c>
+      <c r="C231" s="6" t="n"/>
+    </row>
+    <row r="232">
+      <c r="A232" s="4" t="n"/>
+      <c r="B232" s="6" t="inlineStr">
+        <is>
+          <t>BOUNDARYROW6COT</t>
+        </is>
+      </c>
+      <c r="C232" s="6" t="n"/>
+    </row>
+    <row r="233">
+      <c r="A233" s="4" t="n"/>
+      <c r="B233" s="6" t="inlineStr">
+        <is>
+          <t>BOUNDARYROW7COT</t>
+        </is>
+      </c>
+      <c r="C233" s="6" t="n"/>
+    </row>
+    <row r="234">
+      <c r="A234" s="4" t="n"/>
+      <c r="B234" s="6" t="inlineStr">
+        <is>
+          <t>BOUNDARY_HDDID1A40COTARC</t>
+        </is>
+      </c>
+      <c r="C234" s="6" t="n"/>
+    </row>
+    <row r="235">
+      <c r="A235" s="4" t="n"/>
+      <c r="B235" s="6" t="inlineStr">
+        <is>
+          <t>BOUNDARY_HDDID2A30COT</t>
+        </is>
+      </c>
+      <c r="C235" s="6" t="n"/>
+    </row>
+    <row r="236">
+      <c r="A236" s="4" t="n"/>
+      <c r="B236" s="6" t="n"/>
+      <c r="C236" s="6" t="inlineStr">
         <is>
           <t>BOUNDARYCNREXRN6COT</t>
         </is>
       </c>
     </row>
-    <row r="224">
-      <c r="A224" s="9" t="inlineStr">
-        <is>
-          <t>BOUNDARYCNREXRP
-边界/版图单元</t>
-        </is>
-      </c>
-      <c r="B224" s="12" t="inlineStr">
-        <is>
-          <t>BOUNDARYCNREXRPCOT</t>
-        </is>
-      </c>
-      <c r="C224" s="12" t="inlineStr">
-        <is>
-          <t>BOUNDARYCNREXRPCOT</t>
-        </is>
-      </c>
-    </row>
-    <row r="225">
-      <c r="A225" s="9" t="inlineStr">
-        <is>
-          <t>BOUNDARYCNRINRN6
-边界/版图单元</t>
-        </is>
-      </c>
-      <c r="B225" s="10" t="n"/>
-      <c r="C225" s="10" t="inlineStr">
+    <row r="237">
+      <c r="A237" s="4" t="n"/>
+      <c r="B237" s="6" t="n"/>
+      <c r="C237" s="6" t="inlineStr">
         <is>
           <t>BOUNDARYCNRINRN6COT</t>
         </is>
       </c>
     </row>
-    <row r="226">
-      <c r="A226" s="9" t="inlineStr">
-        <is>
-          <t>BOUNDARYCNRINRP6
-边界/版图单元</t>
-        </is>
-      </c>
-      <c r="B226" s="10" t="n"/>
-      <c r="C226" s="10" t="inlineStr">
+    <row r="238">
+      <c r="A238" s="4" t="n"/>
+      <c r="B238" s="6" t="n"/>
+      <c r="C238" s="6" t="inlineStr">
         <is>
           <t>BOUNDARYCNRINRP6COT</t>
         </is>
       </c>
     </row>
-    <row r="227">
-      <c r="A227" s="9" t="inlineStr">
-        <is>
-          <t>BOUNDARYCOLN1
-边界/版图单元</t>
-        </is>
-      </c>
-      <c r="B227" s="12" t="inlineStr">
-        <is>
-          <t>BOUNDARYCOLN1COT</t>
-        </is>
-      </c>
-      <c r="C227" s="12" t="inlineStr">
-        <is>
-          <t>BOUNDARYCOLN1COT</t>
-        </is>
-      </c>
-    </row>
-    <row r="228">
-      <c r="A228" s="9" t="inlineStr">
-        <is>
-          <t>BOUNDARYCOLN2
-边界/版图单元</t>
-        </is>
-      </c>
-      <c r="B228" s="12" t="inlineStr">
-        <is>
-          <t>BOUNDARYCOLN2COT</t>
-        </is>
-      </c>
-      <c r="C228" s="12" t="inlineStr">
-        <is>
-          <t>BOUNDARYCOLN2COT</t>
-        </is>
-      </c>
-    </row>
-    <row r="229">
-      <c r="A229" s="9" t="inlineStr">
-        <is>
-          <t>BOUNDARYCOLN3
-边界/版图单元</t>
-        </is>
-      </c>
-      <c r="B229" s="10" t="n"/>
-      <c r="C229" s="10" t="inlineStr">
+    <row r="239">
+      <c r="A239" s="4" t="n"/>
+      <c r="B239" s="6" t="n"/>
+      <c r="C239" s="6" t="inlineStr">
         <is>
           <t>BOUNDARYCOLN3COT</t>
         </is>
       </c>
     </row>
-    <row r="230">
-      <c r="A230" s="9" t="inlineStr">
-        <is>
-          <t>BOUNDARYCOLNGAP
-边界/版图单元</t>
-        </is>
-      </c>
-      <c r="B230" s="10" t="inlineStr">
-        <is>
-          <t>BOUNDARYCOLNGAPCOT</t>
-        </is>
-      </c>
-      <c r="C230" s="10" t="n"/>
-    </row>
-    <row r="231">
-      <c r="A231" s="9" t="inlineStr">
-        <is>
-          <t>BOUNDARYCOLP1
-边界/版图单元</t>
-        </is>
-      </c>
-      <c r="B231" s="12" t="inlineStr">
-        <is>
-          <t>BOUNDARYCOLP1COT</t>
-        </is>
-      </c>
-      <c r="C231" s="12" t="inlineStr">
-        <is>
-          <t>BOUNDARYCOLP1COT</t>
-        </is>
-      </c>
-    </row>
-    <row r="232">
-      <c r="A232" s="9" t="inlineStr">
-        <is>
-          <t>BOUNDARYCOLP2
-边界/版图单元</t>
-        </is>
-      </c>
-      <c r="B232" s="10" t="inlineStr">
-        <is>
-          <t>BOUNDARYCOLP2COT</t>
-        </is>
-      </c>
-      <c r="C232" s="10" t="n"/>
-    </row>
-    <row r="233">
-      <c r="A233" s="9" t="inlineStr">
-        <is>
-          <t>BOUNDARYCOLP3
-边界/版图单元</t>
-        </is>
-      </c>
-      <c r="B233" s="10" t="n"/>
-      <c r="C233" s="10" t="inlineStr">
+    <row r="240">
+      <c r="A240" s="4" t="n"/>
+      <c r="B240" s="6" t="n"/>
+      <c r="C240" s="6" t="inlineStr">
         <is>
           <t>BOUNDARYCOLP3COT</t>
         </is>
       </c>
     </row>
-    <row r="234">
-      <c r="A234" s="9" t="inlineStr">
-        <is>
-          <t>BOUNDARYCOLPGAP
-边界/版图单元</t>
-        </is>
-      </c>
-      <c r="B234" s="12" t="inlineStr">
-        <is>
-          <t>BOUNDARYCOLPGAPCOT</t>
-        </is>
-      </c>
-      <c r="C234" s="12" t="inlineStr">
-        <is>
-          <t>BOUNDARYCOLPGAPCOT</t>
-        </is>
-      </c>
-    </row>
-    <row r="235">
-      <c r="A235" s="9" t="inlineStr">
-        <is>
-          <t>BOUNDARYICNREXRN6
-边界/版图单元</t>
-        </is>
-      </c>
-      <c r="B235" s="12" t="inlineStr">
-        <is>
-          <t>BOUNDARYICNREXRN6COT</t>
-        </is>
-      </c>
-      <c r="C235" s="12" t="inlineStr">
-        <is>
-          <t>BOUNDARYICNREXRN6COT</t>
-        </is>
-      </c>
-    </row>
-    <row r="236">
-      <c r="A236" s="2" t="inlineStr">
-        <is>
-          <t>BOUNDARYICNREXRP6
-边界/版图单元</t>
-        </is>
-      </c>
-      <c r="B236" s="3" t="inlineStr">
-        <is>
-          <t>BOUNDARYICNREXRP6COT</t>
-        </is>
-      </c>
-      <c r="C236" s="3" t="inlineStr">
-        <is>
-          <t>BOUNDARYICNREXRP6COT</t>
-        </is>
-      </c>
-    </row>
-    <row r="237">
-      <c r="A237" s="7" t="n"/>
-      <c r="B237" s="8" t="n"/>
-      <c r="C237" s="8" t="inlineStr">
+    <row r="241">
+      <c r="A241" s="4" t="n"/>
+      <c r="B241" s="6" t="n"/>
+      <c r="C241" s="6" t="inlineStr">
         <is>
           <t>BOUNDARYICNREXRP6ICCCOT</t>
         </is>
       </c>
     </row>
-    <row r="238">
-      <c r="A238" s="9" t="inlineStr">
-        <is>
-          <t>BOUNDARYROW6
-边界/版图单元</t>
-        </is>
-      </c>
-      <c r="B238" s="10" t="inlineStr">
-        <is>
-          <t>BOUNDARYROW6COT</t>
-        </is>
-      </c>
-      <c r="C238" s="10" t="n"/>
-    </row>
-    <row r="239">
-      <c r="A239" s="9" t="inlineStr">
-        <is>
-          <t>BOUNDARYROW7
-边界/版图单元</t>
-        </is>
-      </c>
-      <c r="B239" s="10" t="inlineStr">
-        <is>
-          <t>BOUNDARYROW7COT</t>
-        </is>
-      </c>
-      <c r="C239" s="10" t="n"/>
-    </row>
-    <row r="240">
-      <c r="A240" s="9" t="inlineStr">
-        <is>
-          <t>BOUNDARY_HD1A20
-边界/版图单元</t>
-        </is>
-      </c>
-      <c r="B240" s="10" t="n"/>
-      <c r="C240" s="10" t="inlineStr">
+    <row r="242">
+      <c r="A242" s="4" t="n"/>
+      <c r="B242" s="6" t="n"/>
+      <c r="C242" s="6" t="inlineStr">
         <is>
           <t>BOUNDARY_HD1A20COTC</t>
         </is>
       </c>
     </row>
-    <row r="241">
-      <c r="A241" s="9" t="inlineStr">
-        <is>
-          <t>BOUNDARY_HD2A30F
-边界/版图单元</t>
-        </is>
-      </c>
-      <c r="B241" s="10" t="n"/>
-      <c r="C241" s="10" t="inlineStr">
+    <row r="243">
+      <c r="A243" s="7" t="n"/>
+      <c r="B243" s="8" t="n"/>
+      <c r="C243" s="8" t="inlineStr">
         <is>
           <t>BOUNDARY_HD2A30FCOTC</t>
         </is>
       </c>
-    </row>
-    <row r="242">
-      <c r="A242" s="9" t="inlineStr">
-        <is>
-          <t>BOUNDARY_HDDID1A40
-边界/版图单元</t>
-        </is>
-      </c>
-      <c r="B242" s="10" t="inlineStr">
-        <is>
-          <t>BOUNDARY_HDDID1A40COTARC</t>
-        </is>
-      </c>
-      <c r="C242" s="10" t="n"/>
-    </row>
-    <row r="243">
-      <c r="A243" s="9" t="inlineStr">
-        <is>
-          <t>BOUNDARY_HDDID2A30
-边界/版图单元</t>
-        </is>
-      </c>
-      <c r="B243" s="10" t="inlineStr">
-        <is>
-          <t>BOUNDARY_HDDID2A30COT</t>
-        </is>
-      </c>
-      <c r="C243" s="10" t="n"/>
     </row>
     <row r="244">
       <c r="A244" s="2" t="inlineStr">
@@ -6394,60 +6294,50 @@
       </c>
     </row>
     <row r="509">
-      <c r="A509" s="9" t="inlineStr">
-        <is>
-          <t>HDDICWYX2A20
+      <c r="A509" s="2" t="inlineStr">
+        <is>
+          <t>HDDICWY
 边界/版图单元</t>
         </is>
       </c>
-      <c r="B509" s="10" t="n"/>
-      <c r="C509" s="10" t="inlineStr">
+      <c r="B509" s="11" t="n"/>
+      <c r="C509" s="11" t="inlineStr">
         <is>
           <t>HDDICWYX2A20COT</t>
         </is>
       </c>
     </row>
     <row r="510">
-      <c r="A510" s="9" t="inlineStr">
-        <is>
-          <t>HDDICWYX2B30
+      <c r="A510" s="7" t="n"/>
+      <c r="B510" s="8" t="n"/>
+      <c r="C510" s="8" t="inlineStr">
+        <is>
+          <t>HDDICWYX2B30COT</t>
+        </is>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" s="2" t="inlineStr">
+        <is>
+          <t>HDDID
 边界/版图单元</t>
         </is>
       </c>
-      <c r="B510" s="10" t="n"/>
-      <c r="C510" s="10" t="inlineStr">
-        <is>
-          <t>HDDICWYX2B30COT</t>
-        </is>
-      </c>
-    </row>
-    <row r="511">
-      <c r="A511" s="9" t="inlineStr">
-        <is>
-          <t>HDDID2A30
-边界/版图单元</t>
-        </is>
-      </c>
-      <c r="B511" s="10" t="inlineStr">
+      <c r="B511" s="11" t="inlineStr">
         <is>
           <t>HDDID2A30COTARC</t>
         </is>
       </c>
-      <c r="C511" s="10" t="n"/>
+      <c r="C511" s="11" t="n"/>
     </row>
     <row r="512">
-      <c r="A512" s="9" t="inlineStr">
-        <is>
-          <t>HDDID2A40
-边界/版图单元</t>
-        </is>
-      </c>
-      <c r="B512" s="10" t="inlineStr">
+      <c r="A512" s="7" t="n"/>
+      <c r="B512" s="8" t="inlineStr">
         <is>
           <t>HDDID2A40COTARC</t>
         </is>
       </c>
-      <c r="C512" s="10" t="n"/>
+      <c r="C512" s="8" t="n"/>
     </row>
     <row r="513">
       <c r="A513" s="2" t="inlineStr">
@@ -14400,7 +14290,7 @@
       <c r="C1261" s="10" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="219">
+  <mergeCells count="221">
     <mergeCell ref="A540:A543"/>
     <mergeCell ref="A106:A117"/>
     <mergeCell ref="A378:A384"/>
@@ -14420,7 +14310,6 @@
     <mergeCell ref="A413:A414"/>
     <mergeCell ref="A582:A583"/>
     <mergeCell ref="A1141:A1142"/>
-    <mergeCell ref="A236:A237"/>
     <mergeCell ref="A71:A74"/>
     <mergeCell ref="A189:A192"/>
     <mergeCell ref="A989:A990"/>
@@ -14548,6 +14437,7 @@
     <mergeCell ref="A747:A784"/>
     <mergeCell ref="A799:A802"/>
     <mergeCell ref="A523:A527"/>
+    <mergeCell ref="A509:A510"/>
     <mergeCell ref="A391:A392"/>
     <mergeCell ref="A1100:A1101"/>
     <mergeCell ref="A637:A642"/>
@@ -14559,6 +14449,7 @@
     <mergeCell ref="A85:A105"/>
     <mergeCell ref="A446:A447"/>
     <mergeCell ref="A617:A618"/>
+    <mergeCell ref="A511:A512"/>
     <mergeCell ref="A271:A277"/>
     <mergeCell ref="A785:A786"/>
     <mergeCell ref="A1191:A1195"/>
@@ -14612,6 +14503,7 @@
     <mergeCell ref="A627:A628"/>
     <mergeCell ref="A78:A84"/>
     <mergeCell ref="A452:A453"/>
+    <mergeCell ref="A222:A243"/>
     <mergeCell ref="A50:A56"/>
     <mergeCell ref="A266:A267"/>
     <mergeCell ref="A129:A131"/>

</xml_diff>

<commit_message>
Collapse scan/multibit FF keys by truncating after SDF.
SDFQ/SDFRPQ/SDFSNQ/SDFF* share SDF; RSDF/GSDF/Y*SDF and MB*SRLSDF
likewise drop Q/RPQ/SNQ tails. Keys 401->355.

Co-authored-by: EsaLongs <EsaLongs@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/preview/NP1PP_vs_C1Y_preview.xlsx
+++ b/preview/NP1PP_vs_C1Y_preview.xlsx
@@ -6070,50 +6070,40 @@
       </c>
     </row>
     <row r="490">
-      <c r="A490" s="9" t="inlineStr">
-        <is>
-          <t>GSDFQ
+      <c r="A490" s="2" t="inlineStr">
+        <is>
+          <t>GSDF
 扫描触发器</t>
         </is>
       </c>
-      <c r="B490" s="10" t="inlineStr">
+      <c r="B490" s="3" t="inlineStr">
+        <is>
+          <t>GSDFSNQD1COT</t>
+        </is>
+      </c>
+      <c r="C490" s="3" t="inlineStr">
+        <is>
+          <t>GSDFSNQD1COT</t>
+        </is>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" s="4" t="n"/>
+      <c r="B491" s="6" t="inlineStr">
         <is>
           <t>GSDFQD1COTVIA</t>
         </is>
       </c>
-      <c r="C490" s="10" t="n"/>
-    </row>
-    <row r="491">
-      <c r="A491" s="9" t="inlineStr">
-        <is>
-          <t>GSDFRPQ
-扫描触发器</t>
-        </is>
-      </c>
-      <c r="B491" s="10" t="inlineStr">
+      <c r="C491" s="6" t="n"/>
+    </row>
+    <row r="492">
+      <c r="A492" s="7" t="n"/>
+      <c r="B492" s="8" t="inlineStr">
         <is>
           <t>GSDFRPQD1COT</t>
         </is>
       </c>
-      <c r="C491" s="10" t="n"/>
-    </row>
-    <row r="492">
-      <c r="A492" s="9" t="inlineStr">
-        <is>
-          <t>GSDFSNQ
-扫描触发器</t>
-        </is>
-      </c>
-      <c r="B492" s="12" t="inlineStr">
-        <is>
-          <t>GSDFSNQD1COT</t>
-        </is>
-      </c>
-      <c r="C492" s="12" t="inlineStr">
-        <is>
-          <t>GSDFSNQD1COT</t>
-        </is>
-      </c>
+      <c r="C492" s="8" t="n"/>
     </row>
     <row r="493">
       <c r="A493" s="9" t="inlineStr">
@@ -8175,7 +8165,7 @@
     <row r="681">
       <c r="A681" s="2" t="inlineStr">
         <is>
-          <t>MB2SRLSDFKRPQ
+          <t>MB2SRLSDF
 多比特触发器</t>
         </is>
       </c>
@@ -8187,64 +8177,49 @@
       <c r="C681" s="11" t="n"/>
     </row>
     <row r="682">
-      <c r="A682" s="7" t="n"/>
-      <c r="B682" s="8" t="n"/>
-      <c r="C682" s="8" t="inlineStr">
+      <c r="A682" s="4" t="n"/>
+      <c r="B682" s="6" t="inlineStr">
+        <is>
+          <t>MB2SRLSDFQD2COTONEOPU</t>
+        </is>
+      </c>
+      <c r="C682" s="6" t="n"/>
+    </row>
+    <row r="683">
+      <c r="A683" s="4" t="n"/>
+      <c r="B683" s="6" t="inlineStr">
+        <is>
+          <t>MB2SRLSDFRPQD2COTONEOPU</t>
+        </is>
+      </c>
+      <c r="C683" s="6" t="n"/>
+    </row>
+    <row r="684">
+      <c r="A684" s="4" t="n"/>
+      <c r="B684" s="6" t="inlineStr">
+        <is>
+          <t>MB2SRLSDFSNQD2COTONEOPU</t>
+        </is>
+      </c>
+      <c r="C684" s="6" t="n"/>
+    </row>
+    <row r="685">
+      <c r="A685" s="4" t="n"/>
+      <c r="B685" s="6" t="n"/>
+      <c r="C685" s="6" t="inlineStr">
         <is>
           <t>MB2SRLSDFKRPQD2COTSC4LP</t>
         </is>
       </c>
     </row>
-    <row r="683">
-      <c r="A683" s="9" t="inlineStr">
-        <is>
-          <t>MB2SRLSDFQ
-多比特触发器</t>
-        </is>
-      </c>
-      <c r="B683" s="10" t="inlineStr">
-        <is>
-          <t>MB2SRLSDFQD2COTONEOPU</t>
-        </is>
-      </c>
-      <c r="C683" s="10" t="n"/>
-    </row>
-    <row r="684">
-      <c r="A684" s="2" t="inlineStr">
-        <is>
-          <t>MB2SRLSDFRPQ
-多比特触发器</t>
-        </is>
-      </c>
-      <c r="B684" s="11" t="inlineStr">
-        <is>
-          <t>MB2SRLSDFRPQD2COTONEOPU</t>
-        </is>
-      </c>
-      <c r="C684" s="11" t="n"/>
-    </row>
-    <row r="685">
-      <c r="A685" s="7" t="n"/>
-      <c r="B685" s="8" t="n"/>
-      <c r="C685" s="8" t="inlineStr">
+    <row r="686">
+      <c r="A686" s="7" t="n"/>
+      <c r="B686" s="8" t="n"/>
+      <c r="C686" s="8" t="inlineStr">
         <is>
           <t>MB2SRLSDFRPQD1COTSC5LP</t>
         </is>
       </c>
-    </row>
-    <row r="686">
-      <c r="A686" s="9" t="inlineStr">
-        <is>
-          <t>MB2SRLSDFSNQ
-多比特触发器</t>
-        </is>
-      </c>
-      <c r="B686" s="10" t="inlineStr">
-        <is>
-          <t>MB2SRLSDFSNQD2COTONEOPU</t>
-        </is>
-      </c>
-      <c r="C686" s="10" t="n"/>
     </row>
     <row r="687">
       <c r="A687" s="9" t="inlineStr">
@@ -8275,78 +8250,63 @@
       <c r="C688" s="10" t="n"/>
     </row>
     <row r="689">
-      <c r="A689" s="9" t="inlineStr">
-        <is>
-          <t>MB4SRLSDFKRPQ
+      <c r="A689" s="2" t="inlineStr">
+        <is>
+          <t>MB4SRLSDF
 多比特触发器</t>
         </is>
       </c>
-      <c r="B689" s="10" t="inlineStr">
+      <c r="B689" s="11" t="inlineStr">
         <is>
           <t>MB4SRLSDFKRPQD1COTVIA</t>
         </is>
       </c>
-      <c r="C689" s="10" t="n"/>
+      <c r="C689" s="11" t="n"/>
     </row>
     <row r="690">
-      <c r="A690" s="2" t="inlineStr">
-        <is>
-          <t>MB4SRLSDFQ
-多比特触发器</t>
-        </is>
-      </c>
-      <c r="B690" s="11" t="inlineStr">
+      <c r="A690" s="4" t="n"/>
+      <c r="B690" s="6" t="inlineStr">
         <is>
           <t>MB4SRLSDFQD1COTVIA</t>
         </is>
       </c>
-      <c r="C690" s="11" t="n"/>
+      <c r="C690" s="6" t="n"/>
     </row>
     <row r="691">
-      <c r="A691" s="7" t="n"/>
-      <c r="B691" s="8" t="n"/>
-      <c r="C691" s="8" t="inlineStr">
+      <c r="A691" s="4" t="n"/>
+      <c r="B691" s="6" t="inlineStr">
+        <is>
+          <t>MB4SRLSDFRPQD2COTOPUEEQ</t>
+        </is>
+      </c>
+      <c r="C691" s="6" t="n"/>
+    </row>
+    <row r="692">
+      <c r="A692" s="4" t="n"/>
+      <c r="B692" s="6" t="inlineStr">
+        <is>
+          <t>MB4SRLSDFSNQD1COTM3CEQ</t>
+        </is>
+      </c>
+      <c r="C692" s="6" t="n"/>
+    </row>
+    <row r="693">
+      <c r="A693" s="4" t="n"/>
+      <c r="B693" s="6" t="n"/>
+      <c r="C693" s="6" t="inlineStr">
         <is>
           <t>MB4SRLSDFQD1COT</t>
         </is>
       </c>
     </row>
-    <row r="692">
-      <c r="A692" s="2" t="inlineStr">
-        <is>
-          <t>MB4SRLSDFRPQ
-多比特触发器</t>
-        </is>
-      </c>
-      <c r="B692" s="11" t="inlineStr">
-        <is>
-          <t>MB4SRLSDFRPQD2COTOPUEEQ</t>
-        </is>
-      </c>
-      <c r="C692" s="11" t="n"/>
-    </row>
-    <row r="693">
-      <c r="A693" s="7" t="n"/>
-      <c r="B693" s="8" t="n"/>
-      <c r="C693" s="8" t="inlineStr">
+    <row r="694">
+      <c r="A694" s="7" t="n"/>
+      <c r="B694" s="8" t="n"/>
+      <c r="C694" s="8" t="inlineStr">
         <is>
           <t>MB4SRLSDFRPQD1ONECOT</t>
         </is>
       </c>
-    </row>
-    <row r="694">
-      <c r="A694" s="9" t="inlineStr">
-        <is>
-          <t>MB4SRLSDFSNQ
-多比特触发器</t>
-        </is>
-      </c>
-      <c r="B694" s="10" t="inlineStr">
-        <is>
-          <t>MB4SRLSDFSNQD1COTM3CEQ</t>
-        </is>
-      </c>
-      <c r="C694" s="10" t="n"/>
     </row>
     <row r="695">
       <c r="A695" s="9" t="inlineStr">
@@ -12276,56 +12236,41 @@
       </c>
     </row>
     <row r="1084">
-      <c r="A1084" s="9" t="inlineStr">
-        <is>
-          <t>RSDFQ
+      <c r="A1084" s="2" t="inlineStr">
+        <is>
+          <t>RSDF
 扫描触发器</t>
         </is>
       </c>
-      <c r="B1084" s="10" t="n"/>
-      <c r="C1084" s="10" t="inlineStr">
+      <c r="B1084" s="11" t="n"/>
+      <c r="C1084" s="11" t="inlineStr">
         <is>
           <t>RSDFQHDCWD1COT</t>
         </is>
       </c>
     </row>
     <row r="1085">
-      <c r="A1085" s="9" t="inlineStr">
-        <is>
-          <t>RSDFRPQ
-扫描触发器</t>
-        </is>
-      </c>
-      <c r="B1085" s="10" t="n"/>
-      <c r="C1085" s="10" t="inlineStr">
+      <c r="A1085" s="4" t="n"/>
+      <c r="B1085" s="6" t="n"/>
+      <c r="C1085" s="6" t="inlineStr">
         <is>
           <t>RSDFRPQHDCWD1COT</t>
         </is>
       </c>
     </row>
     <row r="1086">
-      <c r="A1086" s="9" t="inlineStr">
-        <is>
-          <t>RSDFSNQ
-扫描触发器</t>
-        </is>
-      </c>
-      <c r="B1086" s="10" t="n"/>
-      <c r="C1086" s="10" t="inlineStr">
+      <c r="A1086" s="4" t="n"/>
+      <c r="B1086" s="6" t="n"/>
+      <c r="C1086" s="6" t="inlineStr">
         <is>
           <t>RSDFSNQHDCWD1COT</t>
         </is>
       </c>
     </row>
     <row r="1087">
-      <c r="A1087" s="9" t="inlineStr">
-        <is>
-          <t>RSDFSRPQ
-扫描触发器</t>
-        </is>
-      </c>
-      <c r="B1087" s="10" t="n"/>
-      <c r="C1087" s="10" t="inlineStr">
+      <c r="A1087" s="7" t="n"/>
+      <c r="B1087" s="8" t="n"/>
+      <c r="C1087" s="8" t="inlineStr">
         <is>
           <t>RSDFSRPQHDCWD1COT</t>
         </is>
@@ -12346,371 +12291,286 @@
       </c>
     </row>
     <row r="1089">
-      <c r="A1089" s="9" t="inlineStr">
-        <is>
-          <t>SDFFACPQ
+      <c r="A1089" s="2" t="inlineStr">
+        <is>
+          <t>SDF
 扫描触发器</t>
         </is>
       </c>
-      <c r="B1089" s="10" t="n"/>
-      <c r="C1089" s="10" t="inlineStr">
-        <is>
-          <t>SDFFACPQX4ASBCOTC</t>
-        </is>
-      </c>
+      <c r="B1089" s="11" t="inlineStr">
+        <is>
+          <t>SDFKRPQD1COTVIASC4LPM3CEQ</t>
+        </is>
+      </c>
+      <c r="C1089" s="11" t="n"/>
     </row>
     <row r="1090">
-      <c r="A1090" s="9" t="inlineStr">
-        <is>
-          <t>SDFFASNQ
-扫描触发器</t>
-        </is>
-      </c>
-      <c r="B1090" s="10" t="n"/>
-      <c r="C1090" s="10" t="inlineStr">
-        <is>
-          <t>SDFFASNQX2ATBCOTC</t>
-        </is>
-      </c>
+      <c r="A1090" s="4" t="n"/>
+      <c r="B1090" s="6" t="inlineStr">
+        <is>
+          <t>SDFKSNQD1COT</t>
+        </is>
+      </c>
+      <c r="C1090" s="6" t="n"/>
     </row>
     <row r="1091">
-      <c r="A1091" s="9" t="inlineStr">
-        <is>
-          <t>SDFFEACPQ
-扫描触发器</t>
-        </is>
-      </c>
-      <c r="B1091" s="10" t="n"/>
-      <c r="C1091" s="10" t="inlineStr">
-        <is>
-          <t>SDFFEACPQX4ASBCOTC</t>
-        </is>
-      </c>
+      <c r="A1091" s="4" t="n"/>
+      <c r="B1091" s="6" t="inlineStr">
+        <is>
+          <t>SDFKSRPQD4COTOPU</t>
+        </is>
+      </c>
+      <c r="C1091" s="6" t="n"/>
     </row>
     <row r="1092">
-      <c r="A1092" s="2" t="inlineStr">
-        <is>
-          <t>SDFFQ
-扫描触发器</t>
-        </is>
-      </c>
-      <c r="B1092" s="11" t="n"/>
-      <c r="C1092" s="11" t="inlineStr">
-        <is>
-          <t>SDFFQX1ASBCOTC</t>
-        </is>
-      </c>
+      <c r="A1092" s="4" t="n"/>
+      <c r="B1092" s="6" t="inlineStr">
+        <is>
+          <t>SDFMQD1COT</t>
+        </is>
+      </c>
+      <c r="C1092" s="6" t="n"/>
     </row>
     <row r="1093">
       <c r="A1093" s="4" t="n"/>
-      <c r="B1093" s="6" t="n"/>
-      <c r="C1093" s="6" t="inlineStr">
-        <is>
-          <t>SDFFQX4ATBCOTC</t>
-        </is>
-      </c>
+      <c r="B1093" s="6" t="inlineStr">
+        <is>
+          <t>SDFNQD2COTOPU</t>
+        </is>
+      </c>
+      <c r="C1093" s="6" t="n"/>
     </row>
     <row r="1094">
       <c r="A1094" s="4" t="n"/>
-      <c r="B1094" s="6" t="n"/>
-      <c r="C1094" s="6" t="inlineStr">
-        <is>
-          <t>SDFFQX6AHCCOTC</t>
-        </is>
-      </c>
+      <c r="B1094" s="6" t="inlineStr">
+        <is>
+          <t>SDFNQND2COTOPU</t>
+        </is>
+      </c>
+      <c r="C1094" s="6" t="n"/>
     </row>
     <row r="1095">
-      <c r="A1095" s="7" t="n"/>
-      <c r="B1095" s="8" t="n"/>
-      <c r="C1095" s="8" t="inlineStr">
-        <is>
-          <t>SDFFQX8COTC</t>
-        </is>
-      </c>
+      <c r="A1095" s="4" t="n"/>
+      <c r="B1095" s="6" t="inlineStr">
+        <is>
+          <t>SDFNRPQD4COT</t>
+        </is>
+      </c>
+      <c r="C1095" s="6" t="n"/>
     </row>
     <row r="1096">
-      <c r="A1096" s="2" t="inlineStr">
-        <is>
-          <t>SDFFQN
-扫描触发器</t>
-        </is>
-      </c>
-      <c r="B1096" s="11" t="n"/>
-      <c r="C1096" s="11" t="inlineStr">
-        <is>
-          <t>SDFFQNX0P5AHCCOTC</t>
-        </is>
-      </c>
+      <c r="A1096" s="4" t="n"/>
+      <c r="B1096" s="6" t="inlineStr">
+        <is>
+          <t>SDFNRPQND2COTMVM3OPU</t>
+        </is>
+      </c>
+      <c r="C1096" s="6" t="n"/>
     </row>
     <row r="1097">
       <c r="A1097" s="4" t="n"/>
-      <c r="B1097" s="6" t="n"/>
-      <c r="C1097" s="6" t="inlineStr">
-        <is>
-          <t>SDFFQNX0P5AHQCOTC</t>
-        </is>
-      </c>
+      <c r="B1097" s="6" t="inlineStr">
+        <is>
+          <t>SDFNSNQD2COT</t>
+        </is>
+      </c>
+      <c r="C1097" s="6" t="n"/>
     </row>
     <row r="1098">
       <c r="A1098" s="4" t="n"/>
-      <c r="B1098" s="6" t="n"/>
-      <c r="C1098" s="6" t="inlineStr">
+      <c r="B1098" s="6" t="inlineStr">
+        <is>
+          <t>SDFNSNQND1COTM3CEQ</t>
+        </is>
+      </c>
+      <c r="C1098" s="6" t="n"/>
+    </row>
+    <row r="1099">
+      <c r="A1099" s="4" t="n"/>
+      <c r="B1099" s="6" t="inlineStr">
+        <is>
+          <t>SDFNSRPQD4COT</t>
+        </is>
+      </c>
+      <c r="C1099" s="6" t="n"/>
+    </row>
+    <row r="1100">
+      <c r="A1100" s="4" t="n"/>
+      <c r="B1100" s="6" t="inlineStr">
+        <is>
+          <t>SDFQD2COTOPTTMIM3CEQ</t>
+        </is>
+      </c>
+      <c r="C1100" s="6" t="n"/>
+    </row>
+    <row r="1101">
+      <c r="A1101" s="4" t="n"/>
+      <c r="B1101" s="6" t="inlineStr">
+        <is>
+          <t>SDFQND1COT</t>
+        </is>
+      </c>
+      <c r="C1101" s="6" t="n"/>
+    </row>
+    <row r="1102">
+      <c r="A1102" s="4" t="n"/>
+      <c r="B1102" s="6" t="inlineStr">
+        <is>
+          <t>SDFRPQD4COTOPTBB</t>
+        </is>
+      </c>
+      <c r="C1102" s="6" t="n"/>
+    </row>
+    <row r="1103">
+      <c r="A1103" s="4" t="n"/>
+      <c r="B1103" s="6" t="inlineStr">
+        <is>
+          <t>SDFRPQND4COTOPU</t>
+        </is>
+      </c>
+      <c r="C1103" s="6" t="n"/>
+    </row>
+    <row r="1104">
+      <c r="A1104" s="4" t="n"/>
+      <c r="B1104" s="6" t="inlineStr">
+        <is>
+          <t>SDFSNQD8COTOPTBBM3CEQ</t>
+        </is>
+      </c>
+      <c r="C1104" s="6" t="n"/>
+    </row>
+    <row r="1105">
+      <c r="A1105" s="4" t="n"/>
+      <c r="B1105" s="6" t="inlineStr">
+        <is>
+          <t>SDFSNQND4COTOPU</t>
+        </is>
+      </c>
+      <c r="C1105" s="6" t="n"/>
+    </row>
+    <row r="1106">
+      <c r="A1106" s="4" t="n"/>
+      <c r="B1106" s="6" t="inlineStr">
+        <is>
+          <t>SDFSRPQD2COT</t>
+        </is>
+      </c>
+      <c r="C1106" s="6" t="n"/>
+    </row>
+    <row r="1107">
+      <c r="A1107" s="4" t="n"/>
+      <c r="B1107" s="6" t="n"/>
+      <c r="C1107" s="6" t="inlineStr">
+        <is>
+          <t>SDFFACPQX4ASBCOTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1108">
+      <c r="A1108" s="4" t="n"/>
+      <c r="B1108" s="6" t="n"/>
+      <c r="C1108" s="6" t="inlineStr">
+        <is>
+          <t>SDFFASNQX2ATBCOTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1109">
+      <c r="A1109" s="4" t="n"/>
+      <c r="B1109" s="6" t="n"/>
+      <c r="C1109" s="6" t="inlineStr">
+        <is>
+          <t>SDFFEACPQX4ASBCOTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1110">
+      <c r="A1110" s="4" t="n"/>
+      <c r="B1110" s="6" t="n"/>
+      <c r="C1110" s="6" t="inlineStr">
+        <is>
+          <t>SDFFQNX0P5AHCCOTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1111">
+      <c r="A1111" s="4" t="n"/>
+      <c r="B1111" s="6" t="n"/>
+      <c r="C1111" s="6" t="inlineStr">
+        <is>
+          <t>SDFFQNX0P5AHQCOTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1112">
+      <c r="A1112" s="4" t="n"/>
+      <c r="B1112" s="6" t="n"/>
+      <c r="C1112" s="6" t="inlineStr">
         <is>
           <t>SDFFQNX4AHBCOTC</t>
         </is>
       </c>
     </row>
-    <row r="1099">
-      <c r="A1099" s="7" t="n"/>
-      <c r="B1099" s="8" t="n"/>
-      <c r="C1099" s="8" t="inlineStr">
+    <row r="1113">
+      <c r="A1113" s="4" t="n"/>
+      <c r="B1113" s="6" t="n"/>
+      <c r="C1113" s="6" t="inlineStr">
         <is>
           <t>SDFFQNX4AHQCOTC</t>
         </is>
       </c>
     </row>
-    <row r="1100">
-      <c r="A1100" s="2" t="inlineStr">
-        <is>
-          <t>SDFKRPQ
-扫描触发器</t>
-        </is>
-      </c>
-      <c r="B1100" s="11" t="inlineStr">
-        <is>
-          <t>SDFKRPQD1COTVIASC4LPM3CEQ</t>
-        </is>
-      </c>
-      <c r="C1100" s="11" t="n"/>
-    </row>
-    <row r="1101">
-      <c r="A1101" s="7" t="n"/>
-      <c r="B1101" s="8" t="n"/>
-      <c r="C1101" s="8" t="inlineStr">
+    <row r="1114">
+      <c r="A1114" s="4" t="n"/>
+      <c r="B1114" s="6" t="n"/>
+      <c r="C1114" s="6" t="inlineStr">
+        <is>
+          <t>SDFFQX1ASBCOTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1115">
+      <c r="A1115" s="4" t="n"/>
+      <c r="B1115" s="6" t="n"/>
+      <c r="C1115" s="6" t="inlineStr">
+        <is>
+          <t>SDFFQX4ATBCOTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1116">
+      <c r="A1116" s="4" t="n"/>
+      <c r="B1116" s="6" t="n"/>
+      <c r="C1116" s="6" t="inlineStr">
+        <is>
+          <t>SDFFQX6AHCCOTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1117">
+      <c r="A1117" s="4" t="n"/>
+      <c r="B1117" s="6" t="n"/>
+      <c r="C1117" s="6" t="inlineStr">
+        <is>
+          <t>SDFFQX8COTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1118">
+      <c r="A1118" s="4" t="n"/>
+      <c r="B1118" s="6" t="n"/>
+      <c r="C1118" s="6" t="inlineStr">
         <is>
           <t>SDFKRPQD2ONECOT</t>
         </is>
       </c>
-    </row>
-    <row r="1102">
-      <c r="A1102" s="9" t="inlineStr">
-        <is>
-          <t>SDFKSNQ
-扫描触发器</t>
-        </is>
-      </c>
-      <c r="B1102" s="10" t="inlineStr">
-        <is>
-          <t>SDFKSNQD1COT</t>
-        </is>
-      </c>
-      <c r="C1102" s="10" t="n"/>
-    </row>
-    <row r="1103">
-      <c r="A1103" s="2" t="inlineStr">
-        <is>
-          <t>SDFKSRPQ
-扫描触发器</t>
-        </is>
-      </c>
-      <c r="B1103" s="11" t="inlineStr">
-        <is>
-          <t>SDFKSRPQD4COTOPU</t>
-        </is>
-      </c>
-      <c r="C1103" s="11" t="n"/>
-    </row>
-    <row r="1104">
-      <c r="A1104" s="7" t="n"/>
-      <c r="B1104" s="8" t="n"/>
-      <c r="C1104" s="8" t="inlineStr">
-        <is>
-          <t>SDFKSRPQEEQMBDD2COT</t>
-        </is>
-      </c>
-    </row>
-    <row r="1105">
-      <c r="A1105" s="2" t="inlineStr">
-        <is>
-          <t>SDFMQ
-扫描触发器</t>
-        </is>
-      </c>
-      <c r="B1105" s="11" t="inlineStr">
-        <is>
-          <t>SDFMQD1COT</t>
-        </is>
-      </c>
-      <c r="C1105" s="11" t="n"/>
-    </row>
-    <row r="1106">
-      <c r="A1106" s="7" t="n"/>
-      <c r="B1106" s="8" t="n"/>
-      <c r="C1106" s="8" t="inlineStr">
-        <is>
-          <t>SDFMQD6COT</t>
-        </is>
-      </c>
-    </row>
-    <row r="1107">
-      <c r="A1107" s="2" t="inlineStr">
-        <is>
-          <t>SDFNQ
-扫描触发器</t>
-        </is>
-      </c>
-      <c r="B1107" s="11" t="inlineStr">
-        <is>
-          <t>SDFNQD2COTOPU</t>
-        </is>
-      </c>
-      <c r="C1107" s="11" t="n"/>
-    </row>
-    <row r="1108">
-      <c r="A1108" s="7" t="n"/>
-      <c r="B1108" s="8" t="n"/>
-      <c r="C1108" s="8" t="inlineStr">
-        <is>
-          <t>SDFNQD0COT</t>
-        </is>
-      </c>
-    </row>
-    <row r="1109">
-      <c r="A1109" s="9" t="inlineStr">
-        <is>
-          <t>SDFNQND2
-扫描触发器</t>
-        </is>
-      </c>
-      <c r="B1109" s="10" t="inlineStr">
-        <is>
-          <t>SDFNQND2COTOPU</t>
-        </is>
-      </c>
-      <c r="C1109" s="10" t="n"/>
-    </row>
-    <row r="1110">
-      <c r="A1110" s="9" t="inlineStr">
-        <is>
-          <t>SDFNRPQ
-扫描触发器</t>
-        </is>
-      </c>
-      <c r="B1110" s="10" t="inlineStr">
-        <is>
-          <t>SDFNRPQD4COT</t>
-        </is>
-      </c>
-      <c r="C1110" s="10" t="n"/>
-    </row>
-    <row r="1111">
-      <c r="A1111" s="2" t="inlineStr">
-        <is>
-          <t>SDFNRPQND2
-扫描触发器</t>
-        </is>
-      </c>
-      <c r="B1111" s="11" t="inlineStr">
-        <is>
-          <t>SDFNRPQND2COTMVM3OPU</t>
-        </is>
-      </c>
-      <c r="C1111" s="11" t="n"/>
-    </row>
-    <row r="1112">
-      <c r="A1112" s="7" t="n"/>
-      <c r="B1112" s="8" t="n"/>
-      <c r="C1112" s="8" t="inlineStr">
-        <is>
-          <t>SDFNRPQND2COT</t>
-        </is>
-      </c>
-    </row>
-    <row r="1113">
-      <c r="A1113" s="2" t="inlineStr">
-        <is>
-          <t>SDFNSNQ
-扫描触发器</t>
-        </is>
-      </c>
-      <c r="B1113" s="11" t="inlineStr">
-        <is>
-          <t>SDFNSNQD2COT</t>
-        </is>
-      </c>
-      <c r="C1113" s="11" t="n"/>
-    </row>
-    <row r="1114">
-      <c r="A1114" s="7" t="n"/>
-      <c r="B1114" s="8" t="n"/>
-      <c r="C1114" s="8" t="inlineStr">
-        <is>
-          <t>SDFNSNQD1COT</t>
-        </is>
-      </c>
-    </row>
-    <row r="1115">
-      <c r="A1115" s="9" t="inlineStr">
-        <is>
-          <t>SDFNSNQND0
-扫描触发器</t>
-        </is>
-      </c>
-      <c r="B1115" s="10" t="n"/>
-      <c r="C1115" s="10" t="inlineStr">
-        <is>
-          <t>SDFNSNQND0COT</t>
-        </is>
-      </c>
-    </row>
-    <row r="1116">
-      <c r="A1116" s="9" t="inlineStr">
-        <is>
-          <t>SDFNSNQND1
-扫描触发器</t>
-        </is>
-      </c>
-      <c r="B1116" s="10" t="inlineStr">
-        <is>
-          <t>SDFNSNQND1COTM3CEQ</t>
-        </is>
-      </c>
-      <c r="C1116" s="10" t="n"/>
-    </row>
-    <row r="1117">
-      <c r="A1117" s="9" t="inlineStr">
-        <is>
-          <t>SDFNSRPQ
-扫描触发器</t>
-        </is>
-      </c>
-      <c r="B1117" s="10" t="inlineStr">
-        <is>
-          <t>SDFNSRPQD4COT</t>
-        </is>
-      </c>
-      <c r="C1117" s="10" t="n"/>
-    </row>
-    <row r="1118">
-      <c r="A1118" s="2" t="inlineStr">
-        <is>
-          <t>SDFQ
-扫描触发器</t>
-        </is>
-      </c>
-      <c r="B1118" s="11" t="inlineStr">
-        <is>
-          <t>SDFQD2COTOPTTMIM3CEQ</t>
-        </is>
-      </c>
-      <c r="C1118" s="11" t="n"/>
     </row>
     <row r="1119">
       <c r="A1119" s="4" t="n"/>
       <c r="B1119" s="6" t="n"/>
       <c r="C1119" s="6" t="inlineStr">
         <is>
-          <t>SDFQOPTBBOPTLD4COT</t>
+          <t>SDFKSRPQEEQMBDD2COT</t>
         </is>
       </c>
     </row>
@@ -12719,7 +12579,7 @@
       <c r="B1120" s="6" t="n"/>
       <c r="C1120" s="6" t="inlineStr">
         <is>
-          <t>SDFQOPTBCUSS1D2COT</t>
+          <t>SDFMQD6COT</t>
         </is>
       </c>
     </row>
@@ -12728,67 +12588,52 @@
       <c r="B1121" s="6" t="n"/>
       <c r="C1121" s="6" t="inlineStr">
         <is>
-          <t>SDFQOPTQD6COT</t>
+          <t>SDFNQD0COT</t>
         </is>
       </c>
     </row>
     <row r="1122">
-      <c r="A1122" s="7" t="n"/>
-      <c r="B1122" s="8" t="n"/>
-      <c r="C1122" s="8" t="inlineStr">
-        <is>
-          <t>SDFQOPTSV1D1COT</t>
+      <c r="A1122" s="4" t="n"/>
+      <c r="B1122" s="6" t="n"/>
+      <c r="C1122" s="6" t="inlineStr">
+        <is>
+          <t>SDFNRPQND2COT</t>
         </is>
       </c>
     </row>
     <row r="1123">
-      <c r="A1123" s="9" t="inlineStr">
-        <is>
-          <t>SDFQND1
-扫描触发器</t>
-        </is>
-      </c>
-      <c r="B1123" s="10" t="inlineStr">
-        <is>
-          <t>SDFQND1COT</t>
-        </is>
-      </c>
-      <c r="C1123" s="10" t="n"/>
+      <c r="A1123" s="4" t="n"/>
+      <c r="B1123" s="6" t="n"/>
+      <c r="C1123" s="6" t="inlineStr">
+        <is>
+          <t>SDFNSNQD1COT</t>
+        </is>
+      </c>
     </row>
     <row r="1124">
-      <c r="A1124" s="9" t="inlineStr">
-        <is>
-          <t>SDFQND2
-扫描触发器</t>
-        </is>
-      </c>
-      <c r="B1124" s="10" t="n"/>
-      <c r="C1124" s="10" t="inlineStr">
+      <c r="A1124" s="4" t="n"/>
+      <c r="B1124" s="6" t="n"/>
+      <c r="C1124" s="6" t="inlineStr">
+        <is>
+          <t>SDFNSNQND0COT</t>
+        </is>
+      </c>
+    </row>
+    <row r="1125">
+      <c r="A1125" s="4" t="n"/>
+      <c r="B1125" s="6" t="n"/>
+      <c r="C1125" s="6" t="inlineStr">
         <is>
           <t>SDFQND2COT</t>
         </is>
       </c>
-    </row>
-    <row r="1125">
-      <c r="A1125" s="2" t="inlineStr">
-        <is>
-          <t>SDFRPQ
-扫描触发器</t>
-        </is>
-      </c>
-      <c r="B1125" s="11" t="inlineStr">
-        <is>
-          <t>SDFRPQD4COTOPTBB</t>
-        </is>
-      </c>
-      <c r="C1125" s="11" t="n"/>
     </row>
     <row r="1126">
       <c r="A1126" s="4" t="n"/>
       <c r="B1126" s="6" t="n"/>
       <c r="C1126" s="6" t="inlineStr">
         <is>
-          <t>SDFRPQD1COT</t>
+          <t>SDFQOPTBBOPTLD4COT</t>
         </is>
       </c>
     </row>
@@ -12797,7 +12642,7 @@
       <c r="B1127" s="6" t="n"/>
       <c r="C1127" s="6" t="inlineStr">
         <is>
-          <t>SDFRPQOPTQD8COT</t>
+          <t>SDFQOPTBCUSS1D2COT</t>
         </is>
       </c>
     </row>
@@ -12806,7 +12651,7 @@
       <c r="B1128" s="6" t="n"/>
       <c r="C1128" s="6" t="inlineStr">
         <is>
-          <t>SDFRPQOPTQV3D8COT</t>
+          <t>SDFQOPTQD6COT</t>
         </is>
       </c>
     </row>
@@ -12815,121 +12660,86 @@
       <c r="B1129" s="6" t="n"/>
       <c r="C1129" s="6" t="inlineStr">
         <is>
+          <t>SDFQOPTSV1D1COT</t>
+        </is>
+      </c>
+    </row>
+    <row r="1130">
+      <c r="A1130" s="4" t="n"/>
+      <c r="B1130" s="6" t="n"/>
+      <c r="C1130" s="6" t="inlineStr">
+        <is>
+          <t>SDFRPQD1COT</t>
+        </is>
+      </c>
+    </row>
+    <row r="1131">
+      <c r="A1131" s="4" t="n"/>
+      <c r="B1131" s="6" t="n"/>
+      <c r="C1131" s="6" t="inlineStr">
+        <is>
+          <t>SDFRPQOPTQD8COT</t>
+        </is>
+      </c>
+    </row>
+    <row r="1132">
+      <c r="A1132" s="4" t="n"/>
+      <c r="B1132" s="6" t="n"/>
+      <c r="C1132" s="6" t="inlineStr">
+        <is>
+          <t>SDFRPQOPTQV3D8COT</t>
+        </is>
+      </c>
+    </row>
+    <row r="1133">
+      <c r="A1133" s="4" t="n"/>
+      <c r="B1133" s="6" t="n"/>
+      <c r="C1133" s="6" t="inlineStr">
+        <is>
           <t>SDFRPQOPTQV4D8COT</t>
         </is>
       </c>
     </row>
-    <row r="1130">
-      <c r="A1130" s="7" t="n"/>
-      <c r="B1130" s="8" t="n"/>
-      <c r="C1130" s="8" t="inlineStr">
+    <row r="1134">
+      <c r="A1134" s="4" t="n"/>
+      <c r="B1134" s="6" t="n"/>
+      <c r="C1134" s="6" t="inlineStr">
         <is>
           <t>SDFRPQOPTSV1D2COT</t>
         </is>
       </c>
     </row>
-    <row r="1131">
-      <c r="A1131" s="9" t="inlineStr">
-        <is>
-          <t>SDFRPQND4
-扫描触发器</t>
-        </is>
-      </c>
-      <c r="B1131" s="10" t="inlineStr">
-        <is>
-          <t>SDFRPQND4COTOPU</t>
-        </is>
-      </c>
-      <c r="C1131" s="10" t="n"/>
-    </row>
-    <row r="1132">
-      <c r="A1132" s="9" t="inlineStr">
-        <is>
-          <t>SDFSNQ
-扫描触发器</t>
-        </is>
-      </c>
-      <c r="B1132" s="10" t="inlineStr">
-        <is>
-          <t>SDFSNQD8COTOPTBBM3CEQ</t>
-        </is>
-      </c>
-      <c r="C1132" s="10" t="n"/>
-    </row>
-    <row r="1133">
-      <c r="A1133" s="9" t="inlineStr">
-        <is>
-          <t>SDFSNQND2
-扫描触发器</t>
-        </is>
-      </c>
-      <c r="B1133" s="10" t="n"/>
-      <c r="C1133" s="10" t="inlineStr">
+    <row r="1135">
+      <c r="A1135" s="4" t="n"/>
+      <c r="B1135" s="6" t="n"/>
+      <c r="C1135" s="6" t="inlineStr">
         <is>
           <t>SDFSNQND2COT</t>
         </is>
       </c>
     </row>
-    <row r="1134">
-      <c r="A1134" s="9" t="inlineStr">
-        <is>
-          <t>SDFSNQND4
-扫描触发器</t>
-        </is>
-      </c>
-      <c r="B1134" s="10" t="inlineStr">
-        <is>
-          <t>SDFSNQND4COTOPU</t>
-        </is>
-      </c>
-      <c r="C1134" s="10" t="n"/>
-    </row>
-    <row r="1135">
-      <c r="A1135" s="2" t="inlineStr">
-        <is>
-          <t>SDFSRPQ
-扫描触发器</t>
-        </is>
-      </c>
-      <c r="B1135" s="11" t="inlineStr">
-        <is>
-          <t>SDFSRPQD2COT</t>
-        </is>
-      </c>
-      <c r="C1135" s="11" t="n"/>
-    </row>
     <row r="1136">
-      <c r="A1136" s="7" t="n"/>
-      <c r="B1136" s="8" t="n"/>
-      <c r="C1136" s="8" t="inlineStr">
+      <c r="A1136" s="4" t="n"/>
+      <c r="B1136" s="6" t="n"/>
+      <c r="C1136" s="6" t="inlineStr">
         <is>
           <t>SDFSRPQEEQMBDD1COT</t>
         </is>
       </c>
     </row>
     <row r="1137">
-      <c r="A1137" s="9" t="inlineStr">
-        <is>
-          <t>SDFSYNC1Q
-同步触发器</t>
-        </is>
-      </c>
-      <c r="B1137" s="10" t="n"/>
-      <c r="C1137" s="10" t="inlineStr">
+      <c r="A1137" s="4" t="n"/>
+      <c r="B1137" s="6" t="n"/>
+      <c r="C1137" s="6" t="inlineStr">
         <is>
           <t>SDFSYNC1QD1COT</t>
         </is>
       </c>
     </row>
     <row r="1138">
-      <c r="A1138" s="9" t="inlineStr">
-        <is>
-          <t>SDFSYNC1RPQ
-同步触发器</t>
-        </is>
-      </c>
-      <c r="B1138" s="10" t="n"/>
-      <c r="C1138" s="10" t="inlineStr">
+      <c r="A1138" s="7" t="n"/>
+      <c r="B1138" s="8" t="n"/>
+      <c r="C1138" s="8" t="inlineStr">
         <is>
           <t>SDFSYNC1RPQD1COT</t>
         </is>
@@ -14136,161 +13946,121 @@
       </c>
     </row>
     <row r="1251">
-      <c r="A1251" s="9" t="inlineStr">
-        <is>
-          <t>Y2SDFFQ
+      <c r="A1251" s="2" t="inlineStr">
+        <is>
+          <t>Y2SDF
 扫描触发器</t>
         </is>
       </c>
-      <c r="B1251" s="10" t="n"/>
-      <c r="C1251" s="10" t="inlineStr">
+      <c r="B1251" s="11" t="inlineStr">
+        <is>
+          <t>Y2SDFQD1COTM3CEQ</t>
+        </is>
+      </c>
+      <c r="C1251" s="11" t="n"/>
+    </row>
+    <row r="1252">
+      <c r="A1252" s="4" t="n"/>
+      <c r="B1252" s="6" t="inlineStr">
+        <is>
+          <t>Y2SDFRPQD1COTM3CEQ</t>
+        </is>
+      </c>
+      <c r="C1252" s="6" t="n"/>
+    </row>
+    <row r="1253">
+      <c r="A1253" s="4" t="n"/>
+      <c r="B1253" s="6" t="inlineStr">
+        <is>
+          <t>Y2SDFSNQD1COTVIA</t>
+        </is>
+      </c>
+      <c r="C1253" s="6" t="n"/>
+    </row>
+    <row r="1254">
+      <c r="A1254" s="7" t="n"/>
+      <c r="B1254" s="8" t="n"/>
+      <c r="C1254" s="8" t="inlineStr">
         <is>
           <t>Y2SDFFQX1COTC</t>
         </is>
       </c>
     </row>
-    <row r="1252">
-      <c r="A1252" s="9" t="inlineStr">
-        <is>
-          <t>Y2SDFQ
+    <row r="1255">
+      <c r="A1255" s="2" t="inlineStr">
+        <is>
+          <t>Y3SDF
 扫描触发器</t>
         </is>
       </c>
-      <c r="B1252" s="10" t="inlineStr">
-        <is>
-          <t>Y2SDFQD1COTM3CEQ</t>
-        </is>
-      </c>
-      <c r="C1252" s="10" t="n"/>
-    </row>
-    <row r="1253">
-      <c r="A1253" s="9" t="inlineStr">
-        <is>
-          <t>Y2SDFRPQ
+      <c r="B1255" s="11" t="inlineStr">
+        <is>
+          <t>Y3SDFQD1COTVIAM3CEQ</t>
+        </is>
+      </c>
+      <c r="C1255" s="11" t="n"/>
+    </row>
+    <row r="1256">
+      <c r="A1256" s="4" t="n"/>
+      <c r="B1256" s="6" t="inlineStr">
+        <is>
+          <t>Y3SDFRPQD1COTVIA</t>
+        </is>
+      </c>
+      <c r="C1256" s="6" t="n"/>
+    </row>
+    <row r="1257">
+      <c r="A1257" s="4" t="n"/>
+      <c r="B1257" s="6" t="inlineStr">
+        <is>
+          <t>Y3SDFSNQD1COTM3CEQ</t>
+        </is>
+      </c>
+      <c r="C1257" s="6" t="n"/>
+    </row>
+    <row r="1258">
+      <c r="A1258" s="7" t="n"/>
+      <c r="B1258" s="8" t="n"/>
+      <c r="C1258" s="8" t="inlineStr">
+        <is>
+          <t>Y3SDFFACPQX1COTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1259">
+      <c r="A1259" s="2" t="inlineStr">
+        <is>
+          <t>YSDF
 扫描触发器</t>
         </is>
       </c>
-      <c r="B1253" s="10" t="inlineStr">
-        <is>
-          <t>Y2SDFRPQD1COTM3CEQ</t>
-        </is>
-      </c>
-      <c r="C1253" s="10" t="n"/>
-    </row>
-    <row r="1254">
-      <c r="A1254" s="9" t="inlineStr">
-        <is>
-          <t>Y2SDFSNQ
-扫描触发器</t>
-        </is>
-      </c>
-      <c r="B1254" s="10" t="inlineStr">
-        <is>
-          <t>Y2SDFSNQD1COTVIA</t>
-        </is>
-      </c>
-      <c r="C1254" s="10" t="n"/>
-    </row>
-    <row r="1255">
-      <c r="A1255" s="9" t="inlineStr">
-        <is>
-          <t>Y3SDFFACPQ
-扫描触发器</t>
-        </is>
-      </c>
-      <c r="B1255" s="10" t="n"/>
-      <c r="C1255" s="10" t="inlineStr">
-        <is>
-          <t>Y3SDFFACPQX1COTC</t>
-        </is>
-      </c>
-    </row>
-    <row r="1256">
-      <c r="A1256" s="9" t="inlineStr">
-        <is>
-          <t>Y3SDFQ
-扫描触发器</t>
-        </is>
-      </c>
-      <c r="B1256" s="10" t="inlineStr">
-        <is>
-          <t>Y3SDFQD1COTVIAM3CEQ</t>
-        </is>
-      </c>
-      <c r="C1256" s="10" t="n"/>
-    </row>
-    <row r="1257">
-      <c r="A1257" s="9" t="inlineStr">
-        <is>
-          <t>Y3SDFRPQ
-扫描触发器</t>
-        </is>
-      </c>
-      <c r="B1257" s="10" t="inlineStr">
-        <is>
-          <t>Y3SDFRPQD1COTVIA</t>
-        </is>
-      </c>
-      <c r="C1257" s="10" t="n"/>
-    </row>
-    <row r="1258">
-      <c r="A1258" s="9" t="inlineStr">
-        <is>
-          <t>Y3SDFSNQ
-扫描触发器</t>
-        </is>
-      </c>
-      <c r="B1258" s="10" t="inlineStr">
-        <is>
-          <t>Y3SDFSNQD1COTM3CEQ</t>
-        </is>
-      </c>
-      <c r="C1258" s="10" t="n"/>
-    </row>
-    <row r="1259">
-      <c r="A1259" s="9" t="inlineStr">
-        <is>
-          <t>YSDFQ
-扫描触发器</t>
-        </is>
-      </c>
-      <c r="B1259" s="10" t="inlineStr">
+      <c r="B1259" s="11" t="inlineStr">
         <is>
           <t>YSDFQD1COT</t>
         </is>
       </c>
-      <c r="C1259" s="10" t="n"/>
+      <c r="C1259" s="11" t="n"/>
     </row>
     <row r="1260">
-      <c r="A1260" s="9" t="inlineStr">
-        <is>
-          <t>YSDFRPQ
-扫描触发器</t>
-        </is>
-      </c>
-      <c r="B1260" s="10" t="inlineStr">
+      <c r="A1260" s="4" t="n"/>
+      <c r="B1260" s="6" t="inlineStr">
         <is>
           <t>YSDFRPQD1COT</t>
         </is>
       </c>
-      <c r="C1260" s="10" t="n"/>
+      <c r="C1260" s="6" t="n"/>
     </row>
     <row r="1261">
-      <c r="A1261" s="9" t="inlineStr">
-        <is>
-          <t>YSDFSNQ
-扫描触发器</t>
-        </is>
-      </c>
-      <c r="B1261" s="10" t="inlineStr">
+      <c r="A1261" s="7" t="n"/>
+      <c r="B1261" s="8" t="inlineStr">
         <is>
           <t>YSDFSNQD1COT</t>
         </is>
       </c>
-      <c r="C1261" s="10" t="n"/>
+      <c r="C1261" s="8" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="221">
+  <mergeCells count="214">
     <mergeCell ref="A540:A543"/>
     <mergeCell ref="A106:A117"/>
     <mergeCell ref="A378:A384"/>
@@ -14301,7 +14071,6 @@
     <mergeCell ref="A649:A650"/>
     <mergeCell ref="A947:A948"/>
     <mergeCell ref="A335:A336"/>
-    <mergeCell ref="A690:A691"/>
     <mergeCell ref="A966:A977"/>
     <mergeCell ref="A346:A347"/>
     <mergeCell ref="A30:A37"/>
@@ -14338,12 +14107,13 @@
     <mergeCell ref="A256:A257"/>
     <mergeCell ref="A427:A428"/>
     <mergeCell ref="A1033:A1035"/>
-    <mergeCell ref="A1105:A1106"/>
+    <mergeCell ref="A1251:A1254"/>
     <mergeCell ref="A569:A576"/>
     <mergeCell ref="A359:A360"/>
     <mergeCell ref="A719:A721"/>
     <mergeCell ref="A653:A654"/>
     <mergeCell ref="A2:A6"/>
+    <mergeCell ref="A1259:A1261"/>
     <mergeCell ref="A1026:A1029"/>
     <mergeCell ref="A339:A340"/>
     <mergeCell ref="A177:A178"/>
@@ -14373,19 +14143,17 @@
     <mergeCell ref="A858:A859"/>
     <mergeCell ref="A787:A789"/>
     <mergeCell ref="A357:A358"/>
-    <mergeCell ref="A681:A682"/>
-    <mergeCell ref="A1092:A1095"/>
     <mergeCell ref="A344:A345"/>
     <mergeCell ref="A615:A616"/>
+    <mergeCell ref="A681:A686"/>
     <mergeCell ref="A407:A408"/>
     <mergeCell ref="A667:A669"/>
     <mergeCell ref="A631:A636"/>
     <mergeCell ref="A337:A338"/>
     <mergeCell ref="A608:A609"/>
-    <mergeCell ref="A692:A693"/>
     <mergeCell ref="A126:A128"/>
     <mergeCell ref="A534:A539"/>
-    <mergeCell ref="A1125:A1130"/>
+    <mergeCell ref="A1084:A1087"/>
     <mergeCell ref="A1068:A1074"/>
     <mergeCell ref="A1239:A1245"/>
     <mergeCell ref="A983:A984"/>
@@ -14417,7 +14185,7 @@
     <mergeCell ref="A207:A209"/>
     <mergeCell ref="A295:A299"/>
     <mergeCell ref="A483:A484"/>
-    <mergeCell ref="A1118:A1122"/>
+    <mergeCell ref="A490:A492"/>
     <mergeCell ref="A1224:A1227"/>
     <mergeCell ref="A605:A607"/>
     <mergeCell ref="A898:A904"/>
@@ -14433,19 +14201,18 @@
     <mergeCell ref="A185:A188"/>
     <mergeCell ref="A933:A946"/>
     <mergeCell ref="A363:A365"/>
-    <mergeCell ref="A1107:A1108"/>
     <mergeCell ref="A747:A784"/>
     <mergeCell ref="A799:A802"/>
     <mergeCell ref="A523:A527"/>
     <mergeCell ref="A509:A510"/>
     <mergeCell ref="A391:A392"/>
-    <mergeCell ref="A1100:A1101"/>
     <mergeCell ref="A637:A642"/>
     <mergeCell ref="A954:A960"/>
     <mergeCell ref="A978:A982"/>
     <mergeCell ref="A707:A708"/>
     <mergeCell ref="A1219:A1223"/>
     <mergeCell ref="A985:A988"/>
+    <mergeCell ref="A1255:A1258"/>
     <mergeCell ref="A85:A105"/>
     <mergeCell ref="A446:A447"/>
     <mergeCell ref="A617:A618"/>
@@ -14456,10 +14223,10 @@
     <mergeCell ref="A448:A449"/>
     <mergeCell ref="A792:A798"/>
     <mergeCell ref="A210:A214"/>
-    <mergeCell ref="A1135:A1136"/>
     <mergeCell ref="A876:A886"/>
     <mergeCell ref="A291:A294"/>
     <mergeCell ref="A432:A434"/>
+    <mergeCell ref="A1089:A1138"/>
     <mergeCell ref="A124:A125"/>
     <mergeCell ref="A1172:A1174"/>
     <mergeCell ref="A1006:A1007"/>
@@ -14479,20 +14246,16 @@
     <mergeCell ref="A911:A932"/>
     <mergeCell ref="A518:A522"/>
     <mergeCell ref="A132:A134"/>
-    <mergeCell ref="A1111:A1112"/>
     <mergeCell ref="A1182:A1183"/>
     <mergeCell ref="A401:A402"/>
+    <mergeCell ref="A689:A694"/>
     <mergeCell ref="A863:A875"/>
-    <mergeCell ref="A684:A685"/>
-    <mergeCell ref="A1096:A1099"/>
+    <mergeCell ref="A1185:A1188"/>
     <mergeCell ref="A1008:A1009"/>
-    <mergeCell ref="A1185:A1188"/>
     <mergeCell ref="A7:A29"/>
-    <mergeCell ref="A1113:A1114"/>
     <mergeCell ref="A450:A451"/>
     <mergeCell ref="A332:A333"/>
     <mergeCell ref="A589:A595"/>
-    <mergeCell ref="A1103:A1104"/>
     <mergeCell ref="A215:A216"/>
     <mergeCell ref="A677:A679"/>
     <mergeCell ref="A624:A626"/>

</xml_diff>

<commit_message>
Collapse all flip-flop families by truncating after DF/SDF stems.
DF/GDF/EDF/SEDF/SDFF/SD2FF and SDF* share one key per stem; Q/RPQ/SNQ
tails are dropped. Keys 355->333 with full coverage.

Co-authored-by: EsaLongs <EsaLongs@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/preview/NP1PP_vs_C1Y_preview.xlsx
+++ b/preview/NP1PP_vs_C1Y_preview.xlsx
@@ -4150,7 +4150,7 @@
     <row r="342">
       <c r="A342" s="2" t="inlineStr">
         <is>
-          <t>DFKRPQ
+          <t>DF
 D触发器</t>
         </is>
       </c>
@@ -4162,393 +4162,288 @@
       <c r="C342" s="11" t="n"/>
     </row>
     <row r="343">
-      <c r="A343" s="7" t="n"/>
-      <c r="B343" s="8" t="n"/>
-      <c r="C343" s="8" t="inlineStr">
+      <c r="A343" s="4" t="n"/>
+      <c r="B343" s="6" t="inlineStr">
+        <is>
+          <t>DFKSNQD4COT</t>
+        </is>
+      </c>
+      <c r="C343" s="6" t="n"/>
+    </row>
+    <row r="344">
+      <c r="A344" s="4" t="n"/>
+      <c r="B344" s="6" t="inlineStr">
+        <is>
+          <t>DFKSRPQD1COTOPU</t>
+        </is>
+      </c>
+      <c r="C344" s="6" t="n"/>
+    </row>
+    <row r="345">
+      <c r="A345" s="4" t="n"/>
+      <c r="B345" s="6" t="inlineStr">
+        <is>
+          <t>DFMQD1COT</t>
+        </is>
+      </c>
+      <c r="C345" s="6" t="n"/>
+    </row>
+    <row r="346">
+      <c r="A346" s="4" t="n"/>
+      <c r="B346" s="6" t="inlineStr">
+        <is>
+          <t>DFNQD2COTOPU</t>
+        </is>
+      </c>
+      <c r="C346" s="6" t="n"/>
+    </row>
+    <row r="347">
+      <c r="A347" s="4" t="n"/>
+      <c r="B347" s="6" t="inlineStr">
+        <is>
+          <t>DFNQND2COT</t>
+        </is>
+      </c>
+      <c r="C347" s="6" t="n"/>
+    </row>
+    <row r="348">
+      <c r="A348" s="4" t="n"/>
+      <c r="B348" s="6" t="inlineStr">
+        <is>
+          <t>DFNRPQD1COTMVM3OPU</t>
+        </is>
+      </c>
+      <c r="C348" s="6" t="n"/>
+    </row>
+    <row r="349">
+      <c r="A349" s="4" t="n"/>
+      <c r="B349" s="6" t="inlineStr">
+        <is>
+          <t>DFNRPQND2COT</t>
+        </is>
+      </c>
+      <c r="C349" s="6" t="n"/>
+    </row>
+    <row r="350">
+      <c r="A350" s="4" t="n"/>
+      <c r="B350" s="6" t="inlineStr">
+        <is>
+          <t>DFNSNQD2COT</t>
+        </is>
+      </c>
+      <c r="C350" s="6" t="n"/>
+    </row>
+    <row r="351">
+      <c r="A351" s="4" t="n"/>
+      <c r="B351" s="6" t="inlineStr">
+        <is>
+          <t>DFNSNQND1COTMVM3OPU</t>
+        </is>
+      </c>
+      <c r="C351" s="6" t="n"/>
+    </row>
+    <row r="352">
+      <c r="A352" s="4" t="n"/>
+      <c r="B352" s="6" t="inlineStr">
+        <is>
+          <t>DFNSRPQD4COTVIAOPU</t>
+        </is>
+      </c>
+      <c r="C352" s="6" t="n"/>
+    </row>
+    <row r="353">
+      <c r="A353" s="4" t="n"/>
+      <c r="B353" s="6" t="inlineStr">
+        <is>
+          <t>DFQD2COTOPU</t>
+        </is>
+      </c>
+      <c r="C353" s="6" t="n"/>
+    </row>
+    <row r="354">
+      <c r="A354" s="4" t="n"/>
+      <c r="B354" s="6" t="inlineStr">
+        <is>
+          <t>DFQND1COTOPU</t>
+        </is>
+      </c>
+      <c r="C354" s="6" t="n"/>
+    </row>
+    <row r="355">
+      <c r="A355" s="4" t="n"/>
+      <c r="B355" s="6" t="inlineStr">
+        <is>
+          <t>DFRPQD2COTOPU</t>
+        </is>
+      </c>
+      <c r="C355" s="6" t="n"/>
+    </row>
+    <row r="356">
+      <c r="A356" s="4" t="n"/>
+      <c r="B356" s="6" t="inlineStr">
+        <is>
+          <t>DFRPQND1COTMVM3OPU</t>
+        </is>
+      </c>
+      <c r="C356" s="6" t="n"/>
+    </row>
+    <row r="357">
+      <c r="A357" s="4" t="n"/>
+      <c r="B357" s="6" t="inlineStr">
+        <is>
+          <t>DFSNQD2COTMVM3OPU</t>
+        </is>
+      </c>
+      <c r="C357" s="6" t="n"/>
+    </row>
+    <row r="358">
+      <c r="A358" s="4" t="n"/>
+      <c r="B358" s="6" t="inlineStr">
+        <is>
+          <t>DFSNQND4COTOPU</t>
+        </is>
+      </c>
+      <c r="C358" s="6" t="n"/>
+    </row>
+    <row r="359">
+      <c r="A359" s="4" t="n"/>
+      <c r="B359" s="6" t="inlineStr">
+        <is>
+          <t>DFSRPQD1COTOPU</t>
+        </is>
+      </c>
+      <c r="C359" s="6" t="n"/>
+    </row>
+    <row r="360">
+      <c r="A360" s="4" t="n"/>
+      <c r="B360" s="6" t="n"/>
+      <c r="C360" s="6" t="inlineStr">
         <is>
           <t>DFKRPQD1COT</t>
         </is>
       </c>
     </row>
-    <row r="344">
-      <c r="A344" s="2" t="inlineStr">
-        <is>
-          <t>DFKSNQ
-D触发器</t>
-        </is>
-      </c>
-      <c r="B344" s="11" t="inlineStr">
-        <is>
-          <t>DFKSNQD4COT</t>
-        </is>
-      </c>
-      <c r="C344" s="11" t="n"/>
-    </row>
-    <row r="345">
-      <c r="A345" s="7" t="n"/>
-      <c r="B345" s="8" t="n"/>
-      <c r="C345" s="8" t="inlineStr">
+    <row r="361">
+      <c r="A361" s="4" t="n"/>
+      <c r="B361" s="6" t="n"/>
+      <c r="C361" s="6" t="inlineStr">
         <is>
           <t>DFKSNQD0COT</t>
         </is>
       </c>
     </row>
-    <row r="346">
-      <c r="A346" s="2" t="inlineStr">
-        <is>
-          <t>DFKSRPQ
-D触发器</t>
-        </is>
-      </c>
-      <c r="B346" s="11" t="inlineStr">
-        <is>
-          <t>DFKSRPQD1COTOPU</t>
-        </is>
-      </c>
-      <c r="C346" s="11" t="n"/>
-    </row>
-    <row r="347">
-      <c r="A347" s="7" t="n"/>
-      <c r="B347" s="8" t="n"/>
-      <c r="C347" s="8" t="inlineStr">
+    <row r="362">
+      <c r="A362" s="4" t="n"/>
+      <c r="B362" s="6" t="n"/>
+      <c r="C362" s="6" t="inlineStr">
         <is>
           <t>DFKSRPQD0COT</t>
         </is>
       </c>
     </row>
-    <row r="348">
-      <c r="A348" s="9" t="inlineStr">
-        <is>
-          <t>DFMQ
-D触发器</t>
-        </is>
-      </c>
-      <c r="B348" s="10" t="inlineStr">
-        <is>
-          <t>DFMQD1COT</t>
-        </is>
-      </c>
-      <c r="C348" s="10" t="n"/>
-    </row>
-    <row r="349">
-      <c r="A349" s="9" t="inlineStr">
-        <is>
-          <t>DFNQ
-D触发器</t>
-        </is>
-      </c>
-      <c r="B349" s="10" t="inlineStr">
-        <is>
-          <t>DFNQD2COTOPU</t>
-        </is>
-      </c>
-      <c r="C349" s="10" t="n"/>
-    </row>
-    <row r="350">
-      <c r="A350" s="9" t="inlineStr">
-        <is>
-          <t>DFNQND2
-D触发器</t>
-        </is>
-      </c>
-      <c r="B350" s="10" t="inlineStr">
-        <is>
-          <t>DFNQND2COT</t>
-        </is>
-      </c>
-      <c r="C350" s="10" t="n"/>
-    </row>
-    <row r="351">
-      <c r="A351" s="2" t="inlineStr">
-        <is>
-          <t>DFNRPQ
-D触发器</t>
-        </is>
-      </c>
-      <c r="B351" s="11" t="inlineStr">
-        <is>
-          <t>DFNRPQD1COTMVM3OPU</t>
-        </is>
-      </c>
-      <c r="C351" s="11" t="n"/>
-    </row>
-    <row r="352">
-      <c r="A352" s="7" t="n"/>
-      <c r="B352" s="8" t="n"/>
-      <c r="C352" s="8" t="inlineStr">
+    <row r="363">
+      <c r="A363" s="4" t="n"/>
+      <c r="B363" s="6" t="n"/>
+      <c r="C363" s="6" t="inlineStr">
         <is>
           <t>DFNRPQD1COT</t>
         </is>
       </c>
-    </row>
-    <row r="353">
-      <c r="A353" s="9" t="inlineStr">
-        <is>
-          <t>DFNRPQND1
-D触发器</t>
-        </is>
-      </c>
-      <c r="B353" s="10" t="n"/>
-      <c r="C353" s="10" t="inlineStr">
-        <is>
-          <t>DFNRPQND1COT</t>
-        </is>
-      </c>
-    </row>
-    <row r="354">
-      <c r="A354" s="9" t="inlineStr">
-        <is>
-          <t>DFNRPQND2
-D触发器</t>
-        </is>
-      </c>
-      <c r="B354" s="10" t="inlineStr">
-        <is>
-          <t>DFNRPQND2COT</t>
-        </is>
-      </c>
-      <c r="C354" s="10" t="n"/>
-    </row>
-    <row r="355">
-      <c r="A355" s="9" t="inlineStr">
-        <is>
-          <t>DFNSNQ
-D触发器</t>
-        </is>
-      </c>
-      <c r="B355" s="10" t="inlineStr">
-        <is>
-          <t>DFNSNQD2COT</t>
-        </is>
-      </c>
-      <c r="C355" s="10" t="n"/>
-    </row>
-    <row r="356">
-      <c r="A356" s="9" t="inlineStr">
-        <is>
-          <t>DFNSNQND1
-D触发器</t>
-        </is>
-      </c>
-      <c r="B356" s="10" t="inlineStr">
-        <is>
-          <t>DFNSNQND1COTMVM3OPU</t>
-        </is>
-      </c>
-      <c r="C356" s="10" t="n"/>
-    </row>
-    <row r="357">
-      <c r="A357" s="2" t="inlineStr">
-        <is>
-          <t>DFNSRPQ
-D触发器</t>
-        </is>
-      </c>
-      <c r="B357" s="11" t="inlineStr">
-        <is>
-          <t>DFNSRPQD4COTVIAOPU</t>
-        </is>
-      </c>
-      <c r="C357" s="11" t="n"/>
-    </row>
-    <row r="358">
-      <c r="A358" s="7" t="n"/>
-      <c r="B358" s="8" t="n"/>
-      <c r="C358" s="8" t="inlineStr">
-        <is>
-          <t>DFNSRPQEEQMBDD4COT</t>
-        </is>
-      </c>
-    </row>
-    <row r="359">
-      <c r="A359" s="2" t="inlineStr">
-        <is>
-          <t>DFQ
-D触发器</t>
-        </is>
-      </c>
-      <c r="B359" s="11" t="inlineStr">
-        <is>
-          <t>DFQD2COTOPU</t>
-        </is>
-      </c>
-      <c r="C359" s="11" t="n"/>
-    </row>
-    <row r="360">
-      <c r="A360" s="7" t="n"/>
-      <c r="B360" s="8" t="n"/>
-      <c r="C360" s="8" t="inlineStr">
-        <is>
-          <t>DFQOPTLD2COT</t>
-        </is>
-      </c>
-    </row>
-    <row r="361">
-      <c r="A361" s="9" t="inlineStr">
-        <is>
-          <t>DFQN
-D触发器</t>
-        </is>
-      </c>
-      <c r="B361" s="10" t="n"/>
-      <c r="C361" s="10" t="inlineStr">
-        <is>
-          <t>DFQNOPTLD2COT</t>
-        </is>
-      </c>
-    </row>
-    <row r="362">
-      <c r="A362" s="9" t="inlineStr">
-        <is>
-          <t>DFQND1
-D触发器</t>
-        </is>
-      </c>
-      <c r="B362" s="10" t="inlineStr">
-        <is>
-          <t>DFQND1COTOPU</t>
-        </is>
-      </c>
-      <c r="C362" s="10" t="n"/>
-    </row>
-    <row r="363">
-      <c r="A363" s="2" t="inlineStr">
-        <is>
-          <t>DFRPQ
-D触发器</t>
-        </is>
-      </c>
-      <c r="B363" s="11" t="inlineStr">
-        <is>
-          <t>DFRPQD2COTOPU</t>
-        </is>
-      </c>
-      <c r="C363" s="11" t="n"/>
     </row>
     <row r="364">
       <c r="A364" s="4" t="n"/>
       <c r="B364" s="6" t="n"/>
       <c r="C364" s="6" t="inlineStr">
         <is>
+          <t>DFNRPQND1COT</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" s="4" t="n"/>
+      <c r="B365" s="6" t="n"/>
+      <c r="C365" s="6" t="inlineStr">
+        <is>
+          <t>DFNSRPQEEQMBDD4COT</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" s="4" t="n"/>
+      <c r="B366" s="6" t="n"/>
+      <c r="C366" s="6" t="inlineStr">
+        <is>
+          <t>DFQNOPTLD2COT</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" s="4" t="n"/>
+      <c r="B367" s="6" t="n"/>
+      <c r="C367" s="6" t="inlineStr">
+        <is>
+          <t>DFQOPTLD2COT</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" s="4" t="n"/>
+      <c r="B368" s="6" t="n"/>
+      <c r="C368" s="6" t="inlineStr">
+        <is>
           <t>DFRPQEEQMBDD4COT</t>
         </is>
       </c>
-    </row>
-    <row r="365">
-      <c r="A365" s="7" t="n"/>
-      <c r="B365" s="8" t="n"/>
-      <c r="C365" s="8" t="inlineStr">
-        <is>
-          <t>DFRPQOPTLD4COT</t>
-        </is>
-      </c>
-    </row>
-    <row r="366">
-      <c r="A366" s="9" t="inlineStr">
-        <is>
-          <t>DFRPQND1
-D触发器</t>
-        </is>
-      </c>
-      <c r="B366" s="10" t="inlineStr">
-        <is>
-          <t>DFRPQND1COTMVM3OPU</t>
-        </is>
-      </c>
-      <c r="C366" s="10" t="n"/>
-    </row>
-    <row r="367">
-      <c r="A367" s="9" t="inlineStr">
-        <is>
-          <t>DFRPQND2
-D触发器</t>
-        </is>
-      </c>
-      <c r="B367" s="10" t="n"/>
-      <c r="C367" s="10" t="inlineStr">
-        <is>
-          <t>DFRPQND2COT</t>
-        </is>
-      </c>
-    </row>
-    <row r="368">
-      <c r="A368" s="2" t="inlineStr">
-        <is>
-          <t>DFSNQ
-D触发器</t>
-        </is>
-      </c>
-      <c r="B368" s="11" t="inlineStr">
-        <is>
-          <t>DFSNQD2COTMVM3OPU</t>
-        </is>
-      </c>
-      <c r="C368" s="11" t="n"/>
     </row>
     <row r="369">
       <c r="A369" s="4" t="n"/>
       <c r="B369" s="6" t="n"/>
       <c r="C369" s="6" t="inlineStr">
         <is>
+          <t>DFRPQND2COT</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" s="4" t="n"/>
+      <c r="B370" s="6" t="n"/>
+      <c r="C370" s="6" t="inlineStr">
+        <is>
+          <t>DFRPQOPTLD4COT</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" s="4" t="n"/>
+      <c r="B371" s="6" t="n"/>
+      <c r="C371" s="6" t="inlineStr">
+        <is>
           <t>DFSNQD4COT</t>
         </is>
       </c>
     </row>
-    <row r="370">
-      <c r="A370" s="7" t="n"/>
-      <c r="B370" s="8" t="n"/>
-      <c r="C370" s="8" t="inlineStr">
+    <row r="372">
+      <c r="A372" s="4" t="n"/>
+      <c r="B372" s="6" t="n"/>
+      <c r="C372" s="6" t="inlineStr">
+        <is>
+          <t>DFSNQND2COT</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" s="7" t="n"/>
+      <c r="B373" s="8" t="n"/>
+      <c r="C373" s="8" t="inlineStr">
         <is>
           <t>DFSNQOPTLD4COT</t>
         </is>
       </c>
-    </row>
-    <row r="371">
-      <c r="A371" s="9" t="inlineStr">
-        <is>
-          <t>DFSNQND2
-D触发器</t>
-        </is>
-      </c>
-      <c r="B371" s="10" t="n"/>
-      <c r="C371" s="10" t="inlineStr">
-        <is>
-          <t>DFSNQND2COT</t>
-        </is>
-      </c>
-    </row>
-    <row r="372">
-      <c r="A372" s="9" t="inlineStr">
-        <is>
-          <t>DFSNQND4
-D触发器</t>
-        </is>
-      </c>
-      <c r="B372" s="10" t="inlineStr">
-        <is>
-          <t>DFSNQND4COTOPU</t>
-        </is>
-      </c>
-      <c r="C372" s="10" t="n"/>
-    </row>
-    <row r="373">
-      <c r="A373" s="9" t="inlineStr">
-        <is>
-          <t>DFSRPQ
-D触发器</t>
-        </is>
-      </c>
-      <c r="B373" s="10" t="inlineStr">
-        <is>
-          <t>DFSRPQD1COTOPU</t>
-        </is>
-      </c>
-      <c r="C373" s="10" t="n"/>
     </row>
     <row r="374">
       <c r="A374" s="2" t="inlineStr">
         <is>
-          <t>EDFQ
+          <t>EDF
 使能触发器</t>
         </is>
       </c>
@@ -4560,27 +4455,22 @@
       <c r="C374" s="11" t="n"/>
     </row>
     <row r="375">
-      <c r="A375" s="7" t="n"/>
-      <c r="B375" s="8" t="n"/>
-      <c r="C375" s="8" t="inlineStr">
+      <c r="A375" s="4" t="n"/>
+      <c r="B375" s="6" t="inlineStr">
+        <is>
+          <t>EDFRPQD2COTVIA</t>
+        </is>
+      </c>
+      <c r="C375" s="6" t="n"/>
+    </row>
+    <row r="376">
+      <c r="A376" s="4" t="n"/>
+      <c r="B376" s="6" t="n"/>
+      <c r="C376" s="6" t="inlineStr">
         <is>
           <t>EDFQD2COT</t>
         </is>
       </c>
-    </row>
-    <row r="376">
-      <c r="A376" s="2" t="inlineStr">
-        <is>
-          <t>EDFRPQ
-使能触发器</t>
-        </is>
-      </c>
-      <c r="B376" s="11" t="inlineStr">
-        <is>
-          <t>EDFRPQD2COTVIA</t>
-        </is>
-      </c>
-      <c r="C376" s="11" t="n"/>
     </row>
     <row r="377">
       <c r="A377" s="7" t="n"/>
@@ -5383,54 +5273,44 @@
       <c r="C439" s="10" t="n"/>
     </row>
     <row r="440">
-      <c r="A440" s="9" t="inlineStr">
-        <is>
-          <t>GDFQ
+      <c r="A440" s="2" t="inlineStr">
+        <is>
+          <t>GDF
 D触发器</t>
         </is>
       </c>
-      <c r="B440" s="12" t="inlineStr">
+      <c r="B440" s="3" t="inlineStr">
         <is>
           <t>GDFQD1COT</t>
         </is>
       </c>
-      <c r="C440" s="12" t="inlineStr">
+      <c r="C440" s="3" t="inlineStr">
         <is>
           <t>GDFQD1COT</t>
         </is>
       </c>
     </row>
     <row r="441">
-      <c r="A441" s="9" t="inlineStr">
-        <is>
-          <t>GDFRPQ
-D触发器</t>
-        </is>
-      </c>
-      <c r="B441" s="10" t="inlineStr">
+      <c r="A441" s="4" t="n"/>
+      <c r="B441" s="5" t="inlineStr">
+        <is>
+          <t>GDFSNQD1COT</t>
+        </is>
+      </c>
+      <c r="C441" s="5" t="inlineStr">
+        <is>
+          <t>GDFSNQD1COT</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" s="7" t="n"/>
+      <c r="B442" s="8" t="inlineStr">
         <is>
           <t>GDFRPQD1COT</t>
         </is>
       </c>
-      <c r="C441" s="10" t="n"/>
-    </row>
-    <row r="442">
-      <c r="A442" s="9" t="inlineStr">
-        <is>
-          <t>GDFSNQ
-D触发器</t>
-        </is>
-      </c>
-      <c r="B442" s="12" t="inlineStr">
-        <is>
-          <t>GDFSNQD1COT</t>
-        </is>
-      </c>
-      <c r="C442" s="12" t="inlineStr">
-        <is>
-          <t>GDFSNQD1COT</t>
-        </is>
-      </c>
+      <c r="C442" s="8" t="n"/>
     </row>
     <row r="443">
       <c r="A443" s="9" t="inlineStr">
@@ -12279,7 +12159,7 @@
     <row r="1088">
       <c r="A1088" s="9" t="inlineStr">
         <is>
-          <t>SD2FFQN
+          <t>SD2FF
 扫描触发器</t>
         </is>
       </c>
@@ -12462,7 +12342,7 @@
       <c r="B1107" s="6" t="n"/>
       <c r="C1107" s="6" t="inlineStr">
         <is>
-          <t>SDFFACPQX4ASBCOTC</t>
+          <t>SDFKRPQD2ONECOT</t>
         </is>
       </c>
     </row>
@@ -12471,7 +12351,7 @@
       <c r="B1108" s="6" t="n"/>
       <c r="C1108" s="6" t="inlineStr">
         <is>
-          <t>SDFFASNQX2ATBCOTC</t>
+          <t>SDFKSRPQEEQMBDD2COT</t>
         </is>
       </c>
     </row>
@@ -12480,7 +12360,7 @@
       <c r="B1109" s="6" t="n"/>
       <c r="C1109" s="6" t="inlineStr">
         <is>
-          <t>SDFFEACPQX4ASBCOTC</t>
+          <t>SDFMQD6COT</t>
         </is>
       </c>
     </row>
@@ -12489,7 +12369,7 @@
       <c r="B1110" s="6" t="n"/>
       <c r="C1110" s="6" t="inlineStr">
         <is>
-          <t>SDFFQNX0P5AHCCOTC</t>
+          <t>SDFNQD0COT</t>
         </is>
       </c>
     </row>
@@ -12498,7 +12378,7 @@
       <c r="B1111" s="6" t="n"/>
       <c r="C1111" s="6" t="inlineStr">
         <is>
-          <t>SDFFQNX0P5AHQCOTC</t>
+          <t>SDFNRPQND2COT</t>
         </is>
       </c>
     </row>
@@ -12507,7 +12387,7 @@
       <c r="B1112" s="6" t="n"/>
       <c r="C1112" s="6" t="inlineStr">
         <is>
-          <t>SDFFQNX4AHBCOTC</t>
+          <t>SDFNSNQD1COT</t>
         </is>
       </c>
     </row>
@@ -12516,7 +12396,7 @@
       <c r="B1113" s="6" t="n"/>
       <c r="C1113" s="6" t="inlineStr">
         <is>
-          <t>SDFFQNX4AHQCOTC</t>
+          <t>SDFNSNQND0COT</t>
         </is>
       </c>
     </row>
@@ -12525,7 +12405,7 @@
       <c r="B1114" s="6" t="n"/>
       <c r="C1114" s="6" t="inlineStr">
         <is>
-          <t>SDFFQX1ASBCOTC</t>
+          <t>SDFQND2COT</t>
         </is>
       </c>
     </row>
@@ -12534,7 +12414,7 @@
       <c r="B1115" s="6" t="n"/>
       <c r="C1115" s="6" t="inlineStr">
         <is>
-          <t>SDFFQX4ATBCOTC</t>
+          <t>SDFQOPTBBOPTLD4COT</t>
         </is>
       </c>
     </row>
@@ -12543,7 +12423,7 @@
       <c r="B1116" s="6" t="n"/>
       <c r="C1116" s="6" t="inlineStr">
         <is>
-          <t>SDFFQX6AHCCOTC</t>
+          <t>SDFQOPTBCUSS1D2COT</t>
         </is>
       </c>
     </row>
@@ -12552,7 +12432,7 @@
       <c r="B1117" s="6" t="n"/>
       <c r="C1117" s="6" t="inlineStr">
         <is>
-          <t>SDFFQX8COTC</t>
+          <t>SDFQOPTQD6COT</t>
         </is>
       </c>
     </row>
@@ -12561,7 +12441,7 @@
       <c r="B1118" s="6" t="n"/>
       <c r="C1118" s="6" t="inlineStr">
         <is>
-          <t>SDFKRPQD2ONECOT</t>
+          <t>SDFQOPTSV1D1COT</t>
         </is>
       </c>
     </row>
@@ -12570,7 +12450,7 @@
       <c r="B1119" s="6" t="n"/>
       <c r="C1119" s="6" t="inlineStr">
         <is>
-          <t>SDFKSRPQEEQMBDD2COT</t>
+          <t>SDFRPQD1COT</t>
         </is>
       </c>
     </row>
@@ -12579,7 +12459,7 @@
       <c r="B1120" s="6" t="n"/>
       <c r="C1120" s="6" t="inlineStr">
         <is>
-          <t>SDFMQD6COT</t>
+          <t>SDFRPQOPTQD8COT</t>
         </is>
       </c>
     </row>
@@ -12588,7 +12468,7 @@
       <c r="B1121" s="6" t="n"/>
       <c r="C1121" s="6" t="inlineStr">
         <is>
-          <t>SDFNQD0COT</t>
+          <t>SDFRPQOPTQV3D8COT</t>
         </is>
       </c>
     </row>
@@ -12597,7 +12477,7 @@
       <c r="B1122" s="6" t="n"/>
       <c r="C1122" s="6" t="inlineStr">
         <is>
-          <t>SDFNRPQND2COT</t>
+          <t>SDFRPQOPTQV4D8COT</t>
         </is>
       </c>
     </row>
@@ -12606,7 +12486,7 @@
       <c r="B1123" s="6" t="n"/>
       <c r="C1123" s="6" t="inlineStr">
         <is>
-          <t>SDFNSNQD1COT</t>
+          <t>SDFRPQOPTSV1D2COT</t>
         </is>
       </c>
     </row>
@@ -12615,7 +12495,7 @@
       <c r="B1124" s="6" t="n"/>
       <c r="C1124" s="6" t="inlineStr">
         <is>
-          <t>SDFNSNQND0COT</t>
+          <t>SDFSNQND2COT</t>
         </is>
       </c>
     </row>
@@ -12624,7 +12504,7 @@
       <c r="B1125" s="6" t="n"/>
       <c r="C1125" s="6" t="inlineStr">
         <is>
-          <t>SDFQND2COT</t>
+          <t>SDFSRPQEEQMBDD1COT</t>
         </is>
       </c>
     </row>
@@ -12633,25 +12513,30 @@
       <c r="B1126" s="6" t="n"/>
       <c r="C1126" s="6" t="inlineStr">
         <is>
-          <t>SDFQOPTBBOPTLD4COT</t>
+          <t>SDFSYNC1QD1COT</t>
         </is>
       </c>
     </row>
     <row r="1127">
-      <c r="A1127" s="4" t="n"/>
-      <c r="B1127" s="6" t="n"/>
-      <c r="C1127" s="6" t="inlineStr">
-        <is>
-          <t>SDFQOPTBCUSS1D2COT</t>
+      <c r="A1127" s="7" t="n"/>
+      <c r="B1127" s="8" t="n"/>
+      <c r="C1127" s="8" t="inlineStr">
+        <is>
+          <t>SDFSYNC1RPQD1COT</t>
         </is>
       </c>
     </row>
     <row r="1128">
-      <c r="A1128" s="4" t="n"/>
-      <c r="B1128" s="6" t="n"/>
-      <c r="C1128" s="6" t="inlineStr">
-        <is>
-          <t>SDFQOPTQD6COT</t>
+      <c r="A1128" s="2" t="inlineStr">
+        <is>
+          <t>SDFF
+扫描触发器</t>
+        </is>
+      </c>
+      <c r="B1128" s="11" t="n"/>
+      <c r="C1128" s="11" t="inlineStr">
+        <is>
+          <t>SDFFACPQX4ASBCOTC</t>
         </is>
       </c>
     </row>
@@ -12660,7 +12545,7 @@
       <c r="B1129" s="6" t="n"/>
       <c r="C1129" s="6" t="inlineStr">
         <is>
-          <t>SDFQOPTSV1D1COT</t>
+          <t>SDFFASNQX2ATBCOTC</t>
         </is>
       </c>
     </row>
@@ -12669,7 +12554,7 @@
       <c r="B1130" s="6" t="n"/>
       <c r="C1130" s="6" t="inlineStr">
         <is>
-          <t>SDFRPQD1COT</t>
+          <t>SDFFEACPQX4ASBCOTC</t>
         </is>
       </c>
     </row>
@@ -12678,7 +12563,7 @@
       <c r="B1131" s="6" t="n"/>
       <c r="C1131" s="6" t="inlineStr">
         <is>
-          <t>SDFRPQOPTQD8COT</t>
+          <t>SDFFQNX0P5AHCCOTC</t>
         </is>
       </c>
     </row>
@@ -12687,7 +12572,7 @@
       <c r="B1132" s="6" t="n"/>
       <c r="C1132" s="6" t="inlineStr">
         <is>
-          <t>SDFRPQOPTQV3D8COT</t>
+          <t>SDFFQNX0P5AHQCOTC</t>
         </is>
       </c>
     </row>
@@ -12696,7 +12581,7 @@
       <c r="B1133" s="6" t="n"/>
       <c r="C1133" s="6" t="inlineStr">
         <is>
-          <t>SDFRPQOPTQV4D8COT</t>
+          <t>SDFFQNX4AHBCOTC</t>
         </is>
       </c>
     </row>
@@ -12705,7 +12590,7 @@
       <c r="B1134" s="6" t="n"/>
       <c r="C1134" s="6" t="inlineStr">
         <is>
-          <t>SDFRPQOPTSV1D2COT</t>
+          <t>SDFFQNX4AHQCOTC</t>
         </is>
       </c>
     </row>
@@ -12714,7 +12599,7 @@
       <c r="B1135" s="6" t="n"/>
       <c r="C1135" s="6" t="inlineStr">
         <is>
-          <t>SDFSNQND2COT</t>
+          <t>SDFFQX1ASBCOTC</t>
         </is>
       </c>
     </row>
@@ -12723,7 +12608,7 @@
       <c r="B1136" s="6" t="n"/>
       <c r="C1136" s="6" t="inlineStr">
         <is>
-          <t>SDFSRPQEEQMBDD1COT</t>
+          <t>SDFFQX4ATBCOTC</t>
         </is>
       </c>
     </row>
@@ -12732,7 +12617,7 @@
       <c r="B1137" s="6" t="n"/>
       <c r="C1137" s="6" t="inlineStr">
         <is>
-          <t>SDFSYNC1QD1COT</t>
+          <t>SDFFQX6AHCCOTC</t>
         </is>
       </c>
     </row>
@@ -12741,14 +12626,14 @@
       <c r="B1138" s="8" t="n"/>
       <c r="C1138" s="8" t="inlineStr">
         <is>
-          <t>SDFSYNC1RPQD1COT</t>
+          <t>SDFFQX8COTC</t>
         </is>
       </c>
     </row>
     <row r="1139">
       <c r="A1139" s="2" t="inlineStr">
         <is>
-          <t>SEDFQ
+          <t>SEDF
 扫描触发器</t>
         </is>
       </c>
@@ -12760,27 +12645,22 @@
       <c r="C1139" s="11" t="n"/>
     </row>
     <row r="1140">
-      <c r="A1140" s="7" t="n"/>
-      <c r="B1140" s="8" t="n"/>
-      <c r="C1140" s="8" t="inlineStr">
+      <c r="A1140" s="4" t="n"/>
+      <c r="B1140" s="6" t="inlineStr">
+        <is>
+          <t>SEDFRPQD2COT</t>
+        </is>
+      </c>
+      <c r="C1140" s="6" t="n"/>
+    </row>
+    <row r="1141">
+      <c r="A1141" s="4" t="n"/>
+      <c r="B1141" s="6" t="n"/>
+      <c r="C1141" s="6" t="inlineStr">
         <is>
           <t>SEDFQD0COT</t>
         </is>
       </c>
-    </row>
-    <row r="1141">
-      <c r="A1141" s="2" t="inlineStr">
-        <is>
-          <t>SEDFRPQ
-扫描触发器</t>
-        </is>
-      </c>
-      <c r="B1141" s="11" t="inlineStr">
-        <is>
-          <t>SEDFRPQD2COT</t>
-        </is>
-      </c>
-      <c r="C1141" s="11" t="n"/>
     </row>
     <row r="1142">
       <c r="A1142" s="7" t="n"/>
@@ -13969,18 +13849,23 @@
       <c r="C1252" s="6" t="n"/>
     </row>
     <row r="1253">
-      <c r="A1253" s="4" t="n"/>
-      <c r="B1253" s="6" t="inlineStr">
+      <c r="A1253" s="7" t="n"/>
+      <c r="B1253" s="8" t="inlineStr">
         <is>
           <t>Y2SDFSNQD1COTVIA</t>
         </is>
       </c>
-      <c r="C1253" s="6" t="n"/>
+      <c r="C1253" s="8" t="n"/>
     </row>
     <row r="1254">
-      <c r="A1254" s="7" t="n"/>
-      <c r="B1254" s="8" t="n"/>
-      <c r="C1254" s="8" t="inlineStr">
+      <c r="A1254" s="9" t="inlineStr">
+        <is>
+          <t>Y2SDFF
+扫描触发器</t>
+        </is>
+      </c>
+      <c r="B1254" s="10" t="n"/>
+      <c r="C1254" s="10" t="inlineStr">
         <is>
           <t>Y2SDFFQX1COTC</t>
         </is>
@@ -14010,18 +13895,23 @@
       <c r="C1256" s="6" t="n"/>
     </row>
     <row r="1257">
-      <c r="A1257" s="4" t="n"/>
-      <c r="B1257" s="6" t="inlineStr">
+      <c r="A1257" s="7" t="n"/>
+      <c r="B1257" s="8" t="inlineStr">
         <is>
           <t>Y3SDFSNQD1COTM3CEQ</t>
         </is>
       </c>
-      <c r="C1257" s="6" t="n"/>
+      <c r="C1257" s="8" t="n"/>
     </row>
     <row r="1258">
-      <c r="A1258" s="7" t="n"/>
-      <c r="B1258" s="8" t="n"/>
-      <c r="C1258" s="8" t="inlineStr">
+      <c r="A1258" s="9" t="inlineStr">
+        <is>
+          <t>Y3SDFF
+扫描触发器</t>
+        </is>
+      </c>
+      <c r="B1258" s="10" t="n"/>
+      <c r="C1258" s="10" t="inlineStr">
         <is>
           <t>Y3SDFFACPQX1COTC</t>
         </is>
@@ -14060,34 +13950,34 @@
       <c r="C1261" s="8" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="214">
+  <mergeCells count="207">
     <mergeCell ref="A540:A543"/>
     <mergeCell ref="A106:A117"/>
     <mergeCell ref="A378:A384"/>
     <mergeCell ref="A399:A400"/>
     <mergeCell ref="A268:A269"/>
     <mergeCell ref="A701:A706"/>
-    <mergeCell ref="A1139:A1140"/>
     <mergeCell ref="A649:A650"/>
     <mergeCell ref="A947:A948"/>
     <mergeCell ref="A335:A336"/>
     <mergeCell ref="A966:A977"/>
-    <mergeCell ref="A346:A347"/>
+    <mergeCell ref="A586:A587"/>
     <mergeCell ref="A30:A37"/>
-    <mergeCell ref="A586:A587"/>
     <mergeCell ref="A696:A700"/>
     <mergeCell ref="A413:A414"/>
     <mergeCell ref="A582:A583"/>
-    <mergeCell ref="A1141:A1142"/>
+    <mergeCell ref="A1255:A1257"/>
     <mergeCell ref="A71:A74"/>
     <mergeCell ref="A189:A192"/>
+    <mergeCell ref="A374:A377"/>
     <mergeCell ref="A989:A990"/>
     <mergeCell ref="A1075:A1083"/>
     <mergeCell ref="A164:A167"/>
     <mergeCell ref="A675:A676"/>
-    <mergeCell ref="A1175:A1178"/>
+    <mergeCell ref="A1128:A1138"/>
     <mergeCell ref="A244:A247"/>
     <mergeCell ref="A1021:A1025"/>
+    <mergeCell ref="A1175:A1178"/>
     <mergeCell ref="A1232:A1236"/>
     <mergeCell ref="A730:A731"/>
     <mergeCell ref="A1011:A1015"/>
@@ -14104,12 +13994,11 @@
     <mergeCell ref="A286:A290"/>
     <mergeCell ref="A528:A532"/>
     <mergeCell ref="A480:A481"/>
+    <mergeCell ref="A427:A428"/>
+    <mergeCell ref="A440:A442"/>
     <mergeCell ref="A256:A257"/>
-    <mergeCell ref="A427:A428"/>
     <mergeCell ref="A1033:A1035"/>
-    <mergeCell ref="A1251:A1254"/>
     <mergeCell ref="A569:A576"/>
-    <mergeCell ref="A359:A360"/>
     <mergeCell ref="A719:A721"/>
     <mergeCell ref="A653:A654"/>
     <mergeCell ref="A2:A6"/>
@@ -14119,7 +14008,6 @@
     <mergeCell ref="A177:A178"/>
     <mergeCell ref="A330:A331"/>
     <mergeCell ref="A388:A389"/>
-    <mergeCell ref="A351:A352"/>
     <mergeCell ref="A513:A517"/>
     <mergeCell ref="A1246:A1250"/>
     <mergeCell ref="A135:A154"/>
@@ -14129,21 +14017,17 @@
     <mergeCell ref="A300:A307"/>
     <mergeCell ref="A662:A666"/>
     <mergeCell ref="A1196:A1200"/>
-    <mergeCell ref="A374:A375"/>
     <mergeCell ref="A405:A406"/>
     <mergeCell ref="A454:A455"/>
     <mergeCell ref="A172:A174"/>
     <mergeCell ref="A596:A599"/>
     <mergeCell ref="A415:A416"/>
     <mergeCell ref="A1179:A1181"/>
-    <mergeCell ref="A342:A343"/>
     <mergeCell ref="A160:A163"/>
     <mergeCell ref="A64:A70"/>
     <mergeCell ref="A622:A623"/>
     <mergeCell ref="A858:A859"/>
     <mergeCell ref="A787:A789"/>
-    <mergeCell ref="A357:A358"/>
-    <mergeCell ref="A344:A345"/>
     <mergeCell ref="A615:A616"/>
     <mergeCell ref="A681:A686"/>
     <mergeCell ref="A407:A408"/>
@@ -14156,8 +14040,10 @@
     <mergeCell ref="A1084:A1087"/>
     <mergeCell ref="A1068:A1074"/>
     <mergeCell ref="A1239:A1245"/>
+    <mergeCell ref="A342:A373"/>
+    <mergeCell ref="A887:A891"/>
     <mergeCell ref="A983:A984"/>
-    <mergeCell ref="A887:A891"/>
+    <mergeCell ref="A1089:A1127"/>
     <mergeCell ref="A1201:A1217"/>
     <mergeCell ref="A473:A474"/>
     <mergeCell ref="A1151:A1152"/>
@@ -14172,16 +14058,15 @@
     <mergeCell ref="A425:A426"/>
     <mergeCell ref="A860:A862"/>
     <mergeCell ref="A600:A604"/>
-    <mergeCell ref="A376:A377"/>
     <mergeCell ref="A735:A746"/>
     <mergeCell ref="A717:A718"/>
-    <mergeCell ref="A368:A370"/>
     <mergeCell ref="A643:A648"/>
     <mergeCell ref="A38:A48"/>
     <mergeCell ref="A497:A500"/>
     <mergeCell ref="A726:A728"/>
     <mergeCell ref="A1016:A1020"/>
     <mergeCell ref="A409:A410"/>
+    <mergeCell ref="A1251:A1253"/>
     <mergeCell ref="A207:A209"/>
     <mergeCell ref="A295:A299"/>
     <mergeCell ref="A483:A484"/>
@@ -14200,7 +14085,6 @@
     <mergeCell ref="A258:A259"/>
     <mergeCell ref="A185:A188"/>
     <mergeCell ref="A933:A946"/>
-    <mergeCell ref="A363:A365"/>
     <mergeCell ref="A747:A784"/>
     <mergeCell ref="A799:A802"/>
     <mergeCell ref="A523:A527"/>
@@ -14212,11 +14096,11 @@
     <mergeCell ref="A707:A708"/>
     <mergeCell ref="A1219:A1223"/>
     <mergeCell ref="A985:A988"/>
-    <mergeCell ref="A1255:A1258"/>
     <mergeCell ref="A85:A105"/>
     <mergeCell ref="A446:A447"/>
     <mergeCell ref="A617:A618"/>
     <mergeCell ref="A511:A512"/>
+    <mergeCell ref="A1139:A1142"/>
     <mergeCell ref="A271:A277"/>
     <mergeCell ref="A785:A786"/>
     <mergeCell ref="A1191:A1195"/>
@@ -14226,7 +14110,6 @@
     <mergeCell ref="A876:A886"/>
     <mergeCell ref="A291:A294"/>
     <mergeCell ref="A432:A434"/>
-    <mergeCell ref="A1089:A1138"/>
     <mergeCell ref="A124:A125"/>
     <mergeCell ref="A1172:A1174"/>
     <mergeCell ref="A1006:A1007"/>

</xml_diff>

<commit_message>
Drop level-shifter CH/CL domain sides from function keys.
LVLHLCH/CL and LVLLHCH/CL (and CKLVLLH*) collapse to LVLHL/LVLLH.
Keys 333->330; ISOCH/ISOCL unchanged.

Co-authored-by: EsaLongs <EsaLongs@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/preview/NP1PP_vs_C1Y_preview.xlsx
+++ b/preview/NP1PP_vs_C1Y_preview.xlsx
@@ -3252,45 +3252,40 @@
     <row r="264">
       <c r="A264" s="2" t="inlineStr">
         <is>
-          <t>CKLVLLHBUFF
+          <t>CKLVLLH
 电平转换器</t>
         </is>
       </c>
       <c r="B264" s="11" t="inlineStr">
         <is>
-          <t>CKLVLLHBUFFSNKD6COT</t>
+          <t>CKLVLLHCHSNKD2COT</t>
         </is>
       </c>
       <c r="C264" s="11" t="n"/>
     </row>
     <row r="265">
-      <c r="A265" s="7" t="n"/>
-      <c r="B265" s="8" t="inlineStr">
-        <is>
-          <t>CKLVLLHBUFFSRCD2COT</t>
-        </is>
-      </c>
-      <c r="C265" s="8" t="n"/>
+      <c r="A265" s="4" t="n"/>
+      <c r="B265" s="6" t="inlineStr">
+        <is>
+          <t>CKLVLLHCHSRCD4COT</t>
+        </is>
+      </c>
+      <c r="C265" s="6" t="n"/>
     </row>
     <row r="266">
-      <c r="A266" s="2" t="inlineStr">
-        <is>
-          <t>CKLVLLHCH
-电平转换器</t>
-        </is>
-      </c>
-      <c r="B266" s="11" t="inlineStr">
-        <is>
-          <t>CKLVLLHCHSNKD2COT</t>
-        </is>
-      </c>
-      <c r="C266" s="11" t="n"/>
+      <c r="A266" s="4" t="n"/>
+      <c r="B266" s="6" t="inlineStr">
+        <is>
+          <t>CKLVLLHCLSNKD4COT</t>
+        </is>
+      </c>
+      <c r="C266" s="6" t="n"/>
     </row>
     <row r="267">
       <c r="A267" s="7" t="n"/>
       <c r="B267" s="8" t="inlineStr">
         <is>
-          <t>CKLVLLHCHSRCD4COT</t>
+          <t>CKLVLLHCLSRCD2COT</t>
         </is>
       </c>
       <c r="C267" s="8" t="n"/>
@@ -3298,13 +3293,13 @@
     <row r="268">
       <c r="A268" s="2" t="inlineStr">
         <is>
-          <t>CKLVLLHCL
+          <t>CKLVLLHBUFF
 电平转换器</t>
         </is>
       </c>
       <c r="B268" s="11" t="inlineStr">
         <is>
-          <t>CKLVLLHCLSNKD4COT</t>
+          <t>CKLVLLHBUFFSNKD6COT</t>
         </is>
       </c>
       <c r="C268" s="11" t="n"/>
@@ -3313,7 +3308,7 @@
       <c r="A269" s="7" t="n"/>
       <c r="B269" s="8" t="inlineStr">
         <is>
-          <t>CKLVLLHCLSRCD2COT</t>
+          <t>CKLVLLHBUFFSRCD2COT</t>
         </is>
       </c>
       <c r="C269" s="8" t="n"/>
@@ -7442,91 +7437,86 @@
     <row r="624">
       <c r="A624" s="2" t="inlineStr">
         <is>
+          <t>LVLHL
+电平转换器</t>
+        </is>
+      </c>
+      <c r="B624" s="11" t="inlineStr">
+        <is>
+          <t>LVLHLCHSNKD1COT</t>
+        </is>
+      </c>
+      <c r="C624" s="11" t="n"/>
+    </row>
+    <row r="625">
+      <c r="A625" s="4" t="n"/>
+      <c r="B625" s="6" t="inlineStr">
+        <is>
+          <t>LVLHLCLSNKD4COT</t>
+        </is>
+      </c>
+      <c r="C625" s="6" t="n"/>
+    </row>
+    <row r="626">
+      <c r="A626" s="4" t="n"/>
+      <c r="B626" s="6" t="n"/>
+      <c r="C626" s="6" t="inlineStr">
+        <is>
+          <t>LVLHLCHSNKCWD2COT</t>
+        </is>
+      </c>
+    </row>
+    <row r="627">
+      <c r="A627" s="7" t="n"/>
+      <c r="B627" s="8" t="n"/>
+      <c r="C627" s="8" t="inlineStr">
+        <is>
+          <t>LVLHLCLSNKCWD1CNWCOT</t>
+        </is>
+      </c>
+    </row>
+    <row r="628">
+      <c r="A628" s="2" t="inlineStr">
+        <is>
           <t>LVLHLBUFF
 电平转换器</t>
         </is>
       </c>
-      <c r="B624" s="11" t="inlineStr">
+      <c r="B628" s="11" t="inlineStr">
         <is>
           <t>LVLHLBUFFSNKD2COT</t>
         </is>
       </c>
-      <c r="C624" s="11" t="n"/>
-    </row>
-    <row r="625">
-      <c r="A625" s="4" t="n"/>
-      <c r="B625" s="6" t="n"/>
-      <c r="C625" s="6" t="inlineStr">
+      <c r="C628" s="11" t="n"/>
+    </row>
+    <row r="629">
+      <c r="A629" s="4" t="n"/>
+      <c r="B629" s="6" t="n"/>
+      <c r="C629" s="6" t="inlineStr">
         <is>
           <t>LVLHLBUFFSNKCWD2CNWCOT</t>
         </is>
       </c>
-    </row>
-    <row r="626">
-      <c r="A626" s="7" t="n"/>
-      <c r="B626" s="8" t="n"/>
-      <c r="C626" s="8" t="inlineStr">
-        <is>
-          <t>LVLHLBUFFSNKCWD2COT</t>
-        </is>
-      </c>
-    </row>
-    <row r="627">
-      <c r="A627" s="2" t="inlineStr">
-        <is>
-          <t>LVLHLCH
-电平转换器</t>
-        </is>
-      </c>
-      <c r="B627" s="11" t="inlineStr">
-        <is>
-          <t>LVLHLCHSNKD1COT</t>
-        </is>
-      </c>
-      <c r="C627" s="11" t="n"/>
-    </row>
-    <row r="628">
-      <c r="A628" s="7" t="n"/>
-      <c r="B628" s="8" t="n"/>
-      <c r="C628" s="8" t="inlineStr">
-        <is>
-          <t>LVLHLCHSNKCWD2COT</t>
-        </is>
-      </c>
-    </row>
-    <row r="629">
-      <c r="A629" s="2" t="inlineStr">
-        <is>
-          <t>LVLHLCL
-电平转换器</t>
-        </is>
-      </c>
-      <c r="B629" s="11" t="inlineStr">
-        <is>
-          <t>LVLHLCLSNKD4COT</t>
-        </is>
-      </c>
-      <c r="C629" s="11" t="n"/>
     </row>
     <row r="630">
       <c r="A630" s="7" t="n"/>
       <c r="B630" s="8" t="n"/>
       <c r="C630" s="8" t="inlineStr">
         <is>
-          <t>LVLHLCLSNKCWD1CNWCOT</t>
+          <t>LVLHLBUFFSNKCWD2COT</t>
         </is>
       </c>
     </row>
     <row r="631">
       <c r="A631" s="2" t="inlineStr">
         <is>
-          <t>LVLLHBUFF
+          <t>LVLLH
 电平转换器</t>
         </is>
       </c>
       <c r="B631" s="11" t="inlineStr">
         <is>
-          <t>LVLLHBUFFSNKD8COTLN</t>
+          <t>LVLLHCHSNKD4COT</t>
         </is>
       </c>
       <c r="C631" s="11" t="n"/>
@@ -7535,76 +7525,71 @@
       <c r="A632" s="4" t="n"/>
       <c r="B632" s="6" t="inlineStr">
         <is>
-          <t>LVLLHBUFFSRCD1COT</t>
+          <t>LVLLHCHSRCD4COTVIA</t>
         </is>
       </c>
       <c r="C632" s="6" t="n"/>
     </row>
     <row r="633">
       <c r="A633" s="4" t="n"/>
-      <c r="B633" s="6" t="n"/>
-      <c r="C633" s="6" t="inlineStr">
-        <is>
-          <t>LVLLHBUFFSNKCWBALD4COT</t>
-        </is>
-      </c>
+      <c r="B633" s="6" t="inlineStr">
+        <is>
+          <t>LVLLHCLSNKD4COT</t>
+        </is>
+      </c>
+      <c r="C633" s="6" t="n"/>
     </row>
     <row r="634">
       <c r="A634" s="4" t="n"/>
-      <c r="B634" s="6" t="n"/>
-      <c r="C634" s="6" t="inlineStr">
-        <is>
-          <t>LVLLHBUFFSNKCWD4CNWBALCOT</t>
-        </is>
-      </c>
+      <c r="B634" s="6" t="inlineStr">
+        <is>
+          <t>LVLLHCLSRCD4COT</t>
+        </is>
+      </c>
+      <c r="C634" s="6" t="n"/>
     </row>
     <row r="635">
       <c r="A635" s="4" t="n"/>
       <c r="B635" s="6" t="n"/>
       <c r="C635" s="6" t="inlineStr">
         <is>
-          <t>LVLLHBUFFSRCCWBALD1COT</t>
+          <t>LVLLHCHSNKCWBALRBD2COT</t>
         </is>
       </c>
     </row>
     <row r="636">
-      <c r="A636" s="7" t="n"/>
-      <c r="B636" s="8" t="n"/>
-      <c r="C636" s="8" t="inlineStr">
-        <is>
-          <t>LVLLHBUFFSRCCWD8CNWCOTLN</t>
+      <c r="A636" s="4" t="n"/>
+      <c r="B636" s="6" t="n"/>
+      <c r="C636" s="6" t="inlineStr">
+        <is>
+          <t>LVLLHCHSRCCWBALRBD4COT</t>
         </is>
       </c>
     </row>
     <row r="637">
-      <c r="A637" s="2" t="inlineStr">
-        <is>
-          <t>LVLLHCH
-电平转换器</t>
-        </is>
-      </c>
-      <c r="B637" s="11" t="inlineStr">
-        <is>
-          <t>LVLLHCHSNKD4COT</t>
-        </is>
-      </c>
-      <c r="C637" s="11" t="n"/>
+      <c r="A637" s="4" t="n"/>
+      <c r="B637" s="6" t="n"/>
+      <c r="C637" s="6" t="inlineStr">
+        <is>
+          <t>LVLLHCHSRCCWRBD4CNWCOT</t>
+        </is>
+      </c>
     </row>
     <row r="638">
       <c r="A638" s="4" t="n"/>
-      <c r="B638" s="6" t="inlineStr">
-        <is>
-          <t>LVLLHCHSRCD4COTVIA</t>
-        </is>
-      </c>
-      <c r="C638" s="6" t="n"/>
+      <c r="B638" s="6" t="n"/>
+      <c r="C638" s="6" t="inlineStr">
+        <is>
+          <t>LVLLHCHSRCCWRBD4COT</t>
+        </is>
+      </c>
     </row>
     <row r="639">
       <c r="A639" s="4" t="n"/>
       <c r="B639" s="6" t="n"/>
       <c r="C639" s="6" t="inlineStr">
         <is>
-          <t>LVLLHCHSNKCWBALRBD2COT</t>
+          <t>LVLLHCLSNKCWBALRBD4COT</t>
         </is>
       </c>
     </row>
@@ -7613,7 +7598,7 @@
       <c r="B640" s="6" t="n"/>
       <c r="C640" s="6" t="inlineStr">
         <is>
-          <t>LVLLHCHSRCCWBALRBD4COT</t>
+          <t>LVLLHCLSNKCWRBD2CNWCOT</t>
         </is>
       </c>
     </row>
@@ -7622,7 +7607,7 @@
       <c r="B641" s="6" t="n"/>
       <c r="C641" s="6" t="inlineStr">
         <is>
-          <t>LVLLHCHSRCCWRBD4CNWCOT</t>
+          <t>LVLLHCLSNKCWRBD2COT</t>
         </is>
       </c>
     </row>
@@ -7631,20 +7616,20 @@
       <c r="B642" s="8" t="n"/>
       <c r="C642" s="8" t="inlineStr">
         <is>
-          <t>LVLLHCHSRCCWRBD4COT</t>
+          <t>LVLLHCLSRCCWRBD4CNWCOT</t>
         </is>
       </c>
     </row>
     <row r="643">
       <c r="A643" s="2" t="inlineStr">
         <is>
-          <t>LVLLHCL
+          <t>LVLLHBUFF
 电平转换器</t>
         </is>
       </c>
       <c r="B643" s="11" t="inlineStr">
         <is>
-          <t>LVLLHCLSNKD4COT</t>
+          <t>LVLLHBUFFSNKD8COTLN</t>
         </is>
       </c>
       <c r="C643" s="11" t="n"/>
@@ -7653,7 +7638,7 @@
       <c r="A644" s="4" t="n"/>
       <c r="B644" s="6" t="inlineStr">
         <is>
-          <t>LVLLHCLSRCD4COT</t>
+          <t>LVLLHBUFFSRCD1COT</t>
         </is>
       </c>
       <c r="C644" s="6" t="n"/>
@@ -7663,7 +7648,7 @@
       <c r="B645" s="6" t="n"/>
       <c r="C645" s="6" t="inlineStr">
         <is>
-          <t>LVLLHCLSNKCWBALRBD4COT</t>
+          <t>LVLLHBUFFSNKCWBALD4COT</t>
         </is>
       </c>
     </row>
@@ -7672,7 +7657,7 @@
       <c r="B646" s="6" t="n"/>
       <c r="C646" s="6" t="inlineStr">
         <is>
-          <t>LVLLHCLSNKCWRBD2CNWCOT</t>
+          <t>LVLLHBUFFSNKCWD4CNWBALCOT</t>
         </is>
       </c>
     </row>
@@ -7681,7 +7666,7 @@
       <c r="B647" s="6" t="n"/>
       <c r="C647" s="6" t="inlineStr">
         <is>
-          <t>LVLLHCLSNKCWRBD2COT</t>
+          <t>LVLLHBUFFSRCCWBALD1COT</t>
         </is>
       </c>
     </row>
@@ -7690,7 +7675,7 @@
       <c r="B648" s="8" t="n"/>
       <c r="C648" s="8" t="inlineStr">
         <is>
-          <t>LVLLHCLSRCCWRBD4CNWCOT</t>
+          <t>LVLLHBUFFSRCCWD8CNWCOTLN</t>
         </is>
       </c>
     </row>
@@ -13950,7 +13935,7 @@
       <c r="C1261" s="8" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="207">
+  <mergeCells count="204">
     <mergeCell ref="A540:A543"/>
     <mergeCell ref="A106:A117"/>
     <mergeCell ref="A378:A384"/>
@@ -14017,6 +14002,7 @@
     <mergeCell ref="A300:A307"/>
     <mergeCell ref="A662:A666"/>
     <mergeCell ref="A1196:A1200"/>
+    <mergeCell ref="A624:A627"/>
     <mergeCell ref="A405:A406"/>
     <mergeCell ref="A454:A455"/>
     <mergeCell ref="A172:A174"/>
@@ -14032,7 +14018,6 @@
     <mergeCell ref="A681:A686"/>
     <mergeCell ref="A407:A408"/>
     <mergeCell ref="A667:A669"/>
-    <mergeCell ref="A631:A636"/>
     <mergeCell ref="A337:A338"/>
     <mergeCell ref="A608:A609"/>
     <mergeCell ref="A126:A128"/>
@@ -14046,10 +14031,10 @@
     <mergeCell ref="A1089:A1127"/>
     <mergeCell ref="A1201:A1217"/>
     <mergeCell ref="A473:A474"/>
+    <mergeCell ref="A631:A642"/>
     <mergeCell ref="A1151:A1152"/>
     <mergeCell ref="A551:A554"/>
     <mergeCell ref="A457:A458"/>
-    <mergeCell ref="A264:A265"/>
     <mergeCell ref="A1147:A1148"/>
     <mergeCell ref="A326:A327"/>
     <mergeCell ref="A118:A121"/>
@@ -14061,6 +14046,7 @@
     <mergeCell ref="A735:A746"/>
     <mergeCell ref="A717:A718"/>
     <mergeCell ref="A643:A648"/>
+    <mergeCell ref="A264:A267"/>
     <mergeCell ref="A38:A48"/>
     <mergeCell ref="A497:A500"/>
     <mergeCell ref="A726:A728"/>
@@ -14090,7 +14076,6 @@
     <mergeCell ref="A523:A527"/>
     <mergeCell ref="A509:A510"/>
     <mergeCell ref="A391:A392"/>
-    <mergeCell ref="A637:A642"/>
     <mergeCell ref="A954:A960"/>
     <mergeCell ref="A978:A982"/>
     <mergeCell ref="A707:A708"/>
@@ -14139,25 +14124,22 @@
     <mergeCell ref="A450:A451"/>
     <mergeCell ref="A332:A333"/>
     <mergeCell ref="A589:A595"/>
+    <mergeCell ref="A628:A630"/>
     <mergeCell ref="A215:A216"/>
     <mergeCell ref="A677:A679"/>
-    <mergeCell ref="A624:A626"/>
     <mergeCell ref="A75:A77"/>
     <mergeCell ref="A193:A197"/>
     <mergeCell ref="A892:A897"/>
     <mergeCell ref="A1000:A1003"/>
-    <mergeCell ref="A627:A628"/>
     <mergeCell ref="A78:A84"/>
     <mergeCell ref="A452:A453"/>
     <mergeCell ref="A222:A243"/>
     <mergeCell ref="A50:A56"/>
-    <mergeCell ref="A266:A267"/>
     <mergeCell ref="A129:A131"/>
     <mergeCell ref="A710:A713"/>
     <mergeCell ref="A655:A657"/>
     <mergeCell ref="A279:A284"/>
     <mergeCell ref="A308:A315"/>
-    <mergeCell ref="A629:A630"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Strip remaining non-functional KEY tails from five audit findings.
Merge ISOCH/CL into ISOH/ISOL; peel TIE XP/XN; fix ND-drive false
protection; drop LVL*BUFF and BUFF→BUF; clear ISOHFR and LVUFR*.
Keys 330->317 with full coverage.

Co-authored-by: EsaLongs <EsaLongs@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/preview/NP1PP_vs_C1Y_preview.xlsx
+++ b/preview/NP1PP_vs_C1Y_preview.xlsx
@@ -3028,19 +3028,19 @@
 缓冲器</t>
         </is>
       </c>
-      <c r="B244" s="11" t="n"/>
-      <c r="C244" s="11" t="inlineStr">
-        <is>
-          <t>BUFX16AHBCOT</t>
-        </is>
-      </c>
+      <c r="B244" s="11" t="inlineStr">
+        <is>
+          <t>BUFFD10COTSKRMDB</t>
+        </is>
+      </c>
+      <c r="C244" s="11" t="n"/>
     </row>
     <row r="245">
       <c r="A245" s="4" t="n"/>
       <c r="B245" s="6" t="n"/>
       <c r="C245" s="6" t="inlineStr">
         <is>
-          <t>BUFX4ARQCOT</t>
+          <t>BUFX16AHBCOT</t>
         </is>
       </c>
     </row>
@@ -3049,32 +3049,27 @@
       <c r="B246" s="6" t="n"/>
       <c r="C246" s="6" t="inlineStr">
         <is>
+          <t>BUFX4ARQCOT</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" s="4" t="n"/>
+      <c r="B247" s="6" t="n"/>
+      <c r="C247" s="6" t="inlineStr">
+        <is>
           <t>BUFX8AHACOT</t>
         </is>
       </c>
     </row>
-    <row r="247">
-      <c r="A247" s="7" t="n"/>
-      <c r="B247" s="8" t="n"/>
-      <c r="C247" s="8" t="inlineStr">
+    <row r="248">
+      <c r="A248" s="7" t="n"/>
+      <c r="B248" s="8" t="n"/>
+      <c r="C248" s="8" t="inlineStr">
         <is>
           <t>BUFX8AROCOT</t>
         </is>
       </c>
-    </row>
-    <row r="248">
-      <c r="A248" s="9" t="inlineStr">
-        <is>
-          <t>BUFF
-缓冲器</t>
-        </is>
-      </c>
-      <c r="B248" s="10" t="inlineStr">
-        <is>
-          <t>BUFFD10COTSKRMDB</t>
-        </is>
-      </c>
-      <c r="C248" s="10" t="n"/>
     </row>
     <row r="249">
       <c r="A249" s="9" t="inlineStr">
@@ -3258,7 +3253,7 @@
       </c>
       <c r="B264" s="11" t="inlineStr">
         <is>
-          <t>CKLVLLHCHSNKD2COT</t>
+          <t>CKLVLLHBUFFSNKD6COT</t>
         </is>
       </c>
       <c r="C264" s="11" t="n"/>
@@ -3267,7 +3262,7 @@
       <c r="A265" s="4" t="n"/>
       <c r="B265" s="6" t="inlineStr">
         <is>
-          <t>CKLVLLHCHSRCD4COT</t>
+          <t>CKLVLLHBUFFSRCD2COT</t>
         </is>
       </c>
       <c r="C265" s="6" t="n"/>
@@ -3276,39 +3271,34 @@
       <c r="A266" s="4" t="n"/>
       <c r="B266" s="6" t="inlineStr">
         <is>
+          <t>CKLVLLHCHSNKD2COT</t>
+        </is>
+      </c>
+      <c r="C266" s="6" t="n"/>
+    </row>
+    <row r="267">
+      <c r="A267" s="4" t="n"/>
+      <c r="B267" s="6" t="inlineStr">
+        <is>
+          <t>CKLVLLHCHSRCD4COT</t>
+        </is>
+      </c>
+      <c r="C267" s="6" t="n"/>
+    </row>
+    <row r="268">
+      <c r="A268" s="4" t="n"/>
+      <c r="B268" s="6" t="inlineStr">
+        <is>
           <t>CKLVLLHCLSNKD4COT</t>
         </is>
       </c>
-      <c r="C266" s="6" t="n"/>
-    </row>
-    <row r="267">
-      <c r="A267" s="7" t="n"/>
-      <c r="B267" s="8" t="inlineStr">
-        <is>
-          <t>CKLVLLHCLSRCD2COT</t>
-        </is>
-      </c>
-      <c r="C267" s="8" t="n"/>
-    </row>
-    <row r="268">
-      <c r="A268" s="2" t="inlineStr">
-        <is>
-          <t>CKLVLLHBUFF
-电平转换器</t>
-        </is>
-      </c>
-      <c r="B268" s="11" t="inlineStr">
-        <is>
-          <t>CKLVLLHBUFFSNKD6COT</t>
-        </is>
-      </c>
-      <c r="C268" s="11" t="n"/>
+      <c r="C268" s="6" t="n"/>
     </row>
     <row r="269">
       <c r="A269" s="7" t="n"/>
       <c r="B269" s="8" t="inlineStr">
         <is>
-          <t>CKLVLLHBUFFSRCD2COT</t>
+          <t>CKLVLLHCLSRCD2COT</t>
         </is>
       </c>
       <c r="C269" s="8" t="n"/>
@@ -3972,28 +3962,23 @@
       </c>
     </row>
     <row r="328">
-      <c r="A328" s="9" t="inlineStr">
-        <is>
-          <t>DCCKND12
-时钟与非门</t>
-        </is>
-      </c>
-      <c r="B328" s="10" t="inlineStr">
+      <c r="A328" s="2" t="inlineStr">
+        <is>
+          <t>DCCKN
+时钟单元</t>
+        </is>
+      </c>
+      <c r="B328" s="11" t="inlineStr">
         <is>
           <t>DCCKND12COTDH</t>
         </is>
       </c>
-      <c r="C328" s="10" t="n"/>
+      <c r="C328" s="11" t="n"/>
     </row>
     <row r="329">
-      <c r="A329" s="9" t="inlineStr">
-        <is>
-          <t>DCCKND20
-时钟与非门</t>
-        </is>
-      </c>
-      <c r="B329" s="10" t="n"/>
-      <c r="C329" s="10" t="inlineStr">
+      <c r="A329" s="7" t="n"/>
+      <c r="B329" s="8" t="n"/>
+      <c r="C329" s="8" t="inlineStr">
         <is>
           <t>DCCKND20COT</t>
         </is>
@@ -4551,7 +4536,7 @@
     <row r="385">
       <c r="A385" s="9" t="inlineStr">
         <is>
-          <t>FA1ND1
+          <t>FA1N
 全加器</t>
         </is>
       </c>
@@ -4563,28 +4548,23 @@
       </c>
     </row>
     <row r="386">
-      <c r="A386" s="9" t="inlineStr">
-        <is>
-          <t>FA1SND1
+      <c r="A386" s="2" t="inlineStr">
+        <is>
+          <t>FA1SN
 全加器</t>
         </is>
       </c>
-      <c r="B386" s="10" t="inlineStr">
+      <c r="B386" s="11" t="inlineStr">
         <is>
           <t>FA1SND1COT</t>
         </is>
       </c>
-      <c r="C386" s="10" t="n"/>
+      <c r="C386" s="11" t="n"/>
     </row>
     <row r="387">
-      <c r="A387" s="9" t="inlineStr">
-        <is>
-          <t>FA1SND4
-全加器</t>
-        </is>
-      </c>
-      <c r="B387" s="10" t="n"/>
-      <c r="C387" s="10" t="inlineStr">
+      <c r="A387" s="7" t="n"/>
+      <c r="B387" s="8" t="n"/>
+      <c r="C387" s="8" t="inlineStr">
         <is>
           <t>FA1SND4COTCOT</t>
         </is>
@@ -4616,7 +4596,7 @@
     <row r="390">
       <c r="A390" s="9" t="inlineStr">
         <is>
-          <t>FCICOND1
+          <t>FCICON
 进位逻辑</t>
         </is>
       </c>
@@ -4651,28 +4631,23 @@
       </c>
     </row>
     <row r="393">
-      <c r="A393" s="9" t="inlineStr">
-        <is>
-          <t>FCISND2
+      <c r="A393" s="2" t="inlineStr">
+        <is>
+          <t>FCISN
 进位逻辑</t>
         </is>
       </c>
-      <c r="B393" s="10" t="inlineStr">
+      <c r="B393" s="11" t="inlineStr">
         <is>
           <t>FCISND2COT</t>
         </is>
       </c>
-      <c r="C393" s="10" t="n"/>
+      <c r="C393" s="11" t="n"/>
     </row>
     <row r="394">
-      <c r="A394" s="9" t="inlineStr">
-        <is>
-          <t>FCISND4
-进位逻辑</t>
-        </is>
-      </c>
-      <c r="B394" s="10" t="n"/>
-      <c r="C394" s="10" t="inlineStr">
+      <c r="A394" s="7" t="n"/>
+      <c r="B394" s="8" t="n"/>
+      <c r="C394" s="8" t="inlineStr">
         <is>
           <t>FCISND4COT</t>
         </is>
@@ -4681,7 +4656,7 @@
     <row r="395">
       <c r="A395" s="9" t="inlineStr">
         <is>
-          <t>FCONSND1
+          <t>FCONSN
 进位逻辑</t>
         </is>
       </c>
@@ -4695,7 +4670,7 @@
     <row r="396">
       <c r="A396" s="9" t="inlineStr">
         <is>
-          <t>FCSICOND1
+          <t>FCSICON
 进位逻辑</t>
         </is>
       </c>
@@ -4707,32 +4682,27 @@
       <c r="C396" s="10" t="n"/>
     </row>
     <row r="397">
-      <c r="A397" s="9" t="inlineStr">
-        <is>
-          <t>FIICOND1
+      <c r="A397" s="2" t="inlineStr">
+        <is>
+          <t>FIICON
 进位逻辑</t>
         </is>
       </c>
-      <c r="B397" s="10" t="n"/>
-      <c r="C397" s="10" t="inlineStr">
+      <c r="B397" s="11" t="inlineStr">
+        <is>
+          <t>FIICOND4COT</t>
+        </is>
+      </c>
+      <c r="C397" s="11" t="n"/>
+    </row>
+    <row r="398">
+      <c r="A398" s="7" t="n"/>
+      <c r="B398" s="8" t="n"/>
+      <c r="C398" s="8" t="inlineStr">
         <is>
           <t>FIICOND1COT</t>
         </is>
       </c>
-    </row>
-    <row r="398">
-      <c r="A398" s="9" t="inlineStr">
-        <is>
-          <t>FIICOND4
-进位逻辑</t>
-        </is>
-      </c>
-      <c r="B398" s="10" t="inlineStr">
-        <is>
-          <t>FIICOND4COT</t>
-        </is>
-      </c>
-      <c r="C398" s="10" t="n"/>
     </row>
     <row r="399">
       <c r="A399" s="2" t="inlineStr">
@@ -5634,8 +5604,8 @@
     <row r="468">
       <c r="A468" s="9" t="inlineStr">
         <is>
-          <t>GMUX2ND1
-复合多路选择器</t>
+          <t>GMUX2N
+反相多路选择器</t>
         </is>
       </c>
       <c r="B468" s="10" t="inlineStr">
@@ -5983,7 +5953,7 @@
     <row r="493">
       <c r="A493" s="9" t="inlineStr">
         <is>
-          <t>GTIEHXP
+          <t>GTIEH
 电平钳位</t>
         </is>
       </c>
@@ -5997,7 +5967,7 @@
     <row r="494">
       <c r="A494" s="9" t="inlineStr">
         <is>
-          <t>GTIELXN
+          <t>GTIEL
 电平钳位</t>
         </is>
       </c>
@@ -7197,7 +7167,7 @@
     <row r="605">
       <c r="A605" s="2" t="inlineStr">
         <is>
-          <t>ISOCH
+          <t>ISOH
 隔离单元</t>
         </is>
       </c>
@@ -7218,74 +7188,59 @@
       <c r="C606" s="6" t="n"/>
     </row>
     <row r="607">
-      <c r="A607" s="7" t="n"/>
-      <c r="B607" s="8" t="n"/>
-      <c r="C607" s="8" t="inlineStr">
+      <c r="A607" s="4" t="n"/>
+      <c r="B607" s="6" t="n"/>
+      <c r="C607" s="6" t="inlineStr">
         <is>
           <t>ISOCHSRCIWD2COT</t>
         </is>
       </c>
     </row>
     <row r="608">
-      <c r="A608" s="2" t="inlineStr">
-        <is>
-          <t>ISOCL
-隔离单元</t>
-        </is>
-      </c>
-      <c r="B608" s="11" t="inlineStr">
-        <is>
-          <t>ISOCLSNKD1COT</t>
-        </is>
-      </c>
-      <c r="C608" s="11" t="n"/>
+      <c r="A608" s="4" t="n"/>
+      <c r="B608" s="6" t="n"/>
+      <c r="C608" s="6" t="inlineStr">
+        <is>
+          <t>ISOHFRX4COTC</t>
+        </is>
+      </c>
     </row>
     <row r="609">
       <c r="A609" s="7" t="n"/>
-      <c r="B609" s="8" t="inlineStr">
-        <is>
-          <t>ISOCLSRCD1COT</t>
-        </is>
-      </c>
-      <c r="C609" s="8" t="n"/>
+      <c r="B609" s="8" t="n"/>
+      <c r="C609" s="8" t="inlineStr">
+        <is>
+          <t>ISOHX2COTC</t>
+        </is>
+      </c>
     </row>
     <row r="610">
-      <c r="A610" s="9" t="inlineStr">
-        <is>
-          <t>ISOH
-隔离单元</t>
-        </is>
-      </c>
-      <c r="B610" s="10" t="n"/>
-      <c r="C610" s="10" t="inlineStr">
-        <is>
-          <t>ISOHX2COTC</t>
-        </is>
-      </c>
-    </row>
-    <row r="611">
-      <c r="A611" s="9" t="inlineStr">
-        <is>
-          <t>ISOHFR
-隔离单元</t>
-        </is>
-      </c>
-      <c r="B611" s="10" t="n"/>
-      <c r="C611" s="10" t="inlineStr">
-        <is>
-          <t>ISOHFRX4COTC</t>
-        </is>
-      </c>
-    </row>
-    <row r="612">
-      <c r="A612" s="9" t="inlineStr">
+      <c r="A610" s="2" t="inlineStr">
         <is>
           <t>ISOL
 隔离单元</t>
         </is>
       </c>
-      <c r="B612" s="10" t="n"/>
-      <c r="C612" s="10" t="inlineStr">
+      <c r="B610" s="11" t="inlineStr">
+        <is>
+          <t>ISOCLSNKD1COT</t>
+        </is>
+      </c>
+      <c r="C610" s="11" t="n"/>
+    </row>
+    <row r="611">
+      <c r="A611" s="4" t="n"/>
+      <c r="B611" s="6" t="inlineStr">
+        <is>
+          <t>ISOCLSRCD1COT</t>
+        </is>
+      </c>
+      <c r="C611" s="6" t="n"/>
+    </row>
+    <row r="612">
+      <c r="A612" s="7" t="n"/>
+      <c r="B612" s="8" t="n"/>
+      <c r="C612" s="8" t="inlineStr">
         <is>
           <t>ISOLX2COTC</t>
         </is>
@@ -7443,7 +7398,7 @@
       </c>
       <c r="B624" s="11" t="inlineStr">
         <is>
-          <t>LVLHLCHSNKD1COT</t>
+          <t>LVLHLBUFFSNKD2COT</t>
         </is>
       </c>
       <c r="C624" s="11" t="n"/>
@@ -7452,49 +7407,44 @@
       <c r="A625" s="4" t="n"/>
       <c r="B625" s="6" t="inlineStr">
         <is>
-          <t>LVLHLCLSNKD4COT</t>
+          <t>LVLHLCHSNKD1COT</t>
         </is>
       </c>
       <c r="C625" s="6" t="n"/>
     </row>
     <row r="626">
       <c r="A626" s="4" t="n"/>
-      <c r="B626" s="6" t="n"/>
-      <c r="C626" s="6" t="inlineStr">
-        <is>
-          <t>LVLHLCHSNKCWD2COT</t>
-        </is>
-      </c>
+      <c r="B626" s="6" t="inlineStr">
+        <is>
+          <t>LVLHLCLSNKD4COT</t>
+        </is>
+      </c>
+      <c r="C626" s="6" t="n"/>
     </row>
     <row r="627">
-      <c r="A627" s="7" t="n"/>
-      <c r="B627" s="8" t="n"/>
-      <c r="C627" s="8" t="inlineStr">
-        <is>
-          <t>LVLHLCLSNKCWD1CNWCOT</t>
+      <c r="A627" s="4" t="n"/>
+      <c r="B627" s="6" t="n"/>
+      <c r="C627" s="6" t="inlineStr">
+        <is>
+          <t>LVLHLBUFFSNKCWD2CNWCOT</t>
         </is>
       </c>
     </row>
     <row r="628">
-      <c r="A628" s="2" t="inlineStr">
-        <is>
-          <t>LVLHLBUFF
-电平转换器</t>
-        </is>
-      </c>
-      <c r="B628" s="11" t="inlineStr">
-        <is>
-          <t>LVLHLBUFFSNKD2COT</t>
-        </is>
-      </c>
-      <c r="C628" s="11" t="n"/>
+      <c r="A628" s="4" t="n"/>
+      <c r="B628" s="6" t="n"/>
+      <c r="C628" s="6" t="inlineStr">
+        <is>
+          <t>LVLHLBUFFSNKCWD2COT</t>
+        </is>
+      </c>
     </row>
     <row r="629">
       <c r="A629" s="4" t="n"/>
       <c r="B629" s="6" t="n"/>
       <c r="C629" s="6" t="inlineStr">
         <is>
-          <t>LVLHLBUFFSNKCWD2CNWCOT</t>
+          <t>LVLHLCHSNKCWD2COT</t>
         </is>
       </c>
     </row>
@@ -7503,7 +7453,7 @@
       <c r="B630" s="8" t="n"/>
       <c r="C630" s="8" t="inlineStr">
         <is>
-          <t>LVLHLBUFFSNKCWD2COT</t>
+          <t>LVLHLCLSNKCWD1CNWCOT</t>
         </is>
       </c>
     </row>
@@ -7516,7 +7466,7 @@
       </c>
       <c r="B631" s="11" t="inlineStr">
         <is>
-          <t>LVLLHCHSNKD4COT</t>
+          <t>LVLLHBUFFSNKD8COTLN</t>
         </is>
       </c>
       <c r="C631" s="11" t="n"/>
@@ -7525,7 +7475,7 @@
       <c r="A632" s="4" t="n"/>
       <c r="B632" s="6" t="inlineStr">
         <is>
-          <t>LVLLHCHSRCD4COTVIA</t>
+          <t>LVLLHBUFFSRCD1COT</t>
         </is>
       </c>
       <c r="C632" s="6" t="n"/>
@@ -7534,7 +7484,7 @@
       <c r="A633" s="4" t="n"/>
       <c r="B633" s="6" t="inlineStr">
         <is>
-          <t>LVLLHCLSNKD4COT</t>
+          <t>LVLLHCHSNKD4COT</t>
         </is>
       </c>
       <c r="C633" s="6" t="n"/>
@@ -7543,35 +7493,35 @@
       <c r="A634" s="4" t="n"/>
       <c r="B634" s="6" t="inlineStr">
         <is>
-          <t>LVLLHCLSRCD4COT</t>
+          <t>LVLLHCHSRCD4COTVIA</t>
         </is>
       </c>
       <c r="C634" s="6" t="n"/>
     </row>
     <row r="635">
       <c r="A635" s="4" t="n"/>
-      <c r="B635" s="6" t="n"/>
-      <c r="C635" s="6" t="inlineStr">
-        <is>
-          <t>LVLLHCHSNKCWBALRBD2COT</t>
-        </is>
-      </c>
+      <c r="B635" s="6" t="inlineStr">
+        <is>
+          <t>LVLLHCLSNKD4COT</t>
+        </is>
+      </c>
+      <c r="C635" s="6" t="n"/>
     </row>
     <row r="636">
       <c r="A636" s="4" t="n"/>
-      <c r="B636" s="6" t="n"/>
-      <c r="C636" s="6" t="inlineStr">
-        <is>
-          <t>LVLLHCHSRCCWBALRBD4COT</t>
-        </is>
-      </c>
+      <c r="B636" s="6" t="inlineStr">
+        <is>
+          <t>LVLLHCLSRCD4COT</t>
+        </is>
+      </c>
+      <c r="C636" s="6" t="n"/>
     </row>
     <row r="637">
       <c r="A637" s="4" t="n"/>
       <c r="B637" s="6" t="n"/>
       <c r="C637" s="6" t="inlineStr">
         <is>
-          <t>LVLLHCHSRCCWRBD4CNWCOT</t>
+          <t>LVLLHBUFFSNKCWBALD4COT</t>
         </is>
       </c>
     </row>
@@ -7580,7 +7530,7 @@
       <c r="B638" s="6" t="n"/>
       <c r="C638" s="6" t="inlineStr">
         <is>
-          <t>LVLLHCHSRCCWRBD4COT</t>
+          <t>LVLLHBUFFSNKCWD4CNWBALCOT</t>
         </is>
       </c>
     </row>
@@ -7589,7 +7539,7 @@
       <c r="B639" s="6" t="n"/>
       <c r="C639" s="6" t="inlineStr">
         <is>
-          <t>LVLLHCLSNKCWBALRBD4COT</t>
+          <t>LVLLHBUFFSRCCWBALD1COT</t>
         </is>
       </c>
     </row>
@@ -7598,7 +7548,7 @@
       <c r="B640" s="6" t="n"/>
       <c r="C640" s="6" t="inlineStr">
         <is>
-          <t>LVLLHCLSNKCWRBD2CNWCOT</t>
+          <t>LVLLHBUFFSRCCWD8CNWCOTLN</t>
         </is>
       </c>
     </row>
@@ -7607,48 +7557,43 @@
       <c r="B641" s="6" t="n"/>
       <c r="C641" s="6" t="inlineStr">
         <is>
-          <t>LVLLHCLSNKCWRBD2COT</t>
+          <t>LVLLHCHSNKCWBALRBD2COT</t>
         </is>
       </c>
     </row>
     <row r="642">
-      <c r="A642" s="7" t="n"/>
-      <c r="B642" s="8" t="n"/>
-      <c r="C642" s="8" t="inlineStr">
-        <is>
-          <t>LVLLHCLSRCCWRBD4CNWCOT</t>
+      <c r="A642" s="4" t="n"/>
+      <c r="B642" s="6" t="n"/>
+      <c r="C642" s="6" t="inlineStr">
+        <is>
+          <t>LVLLHCHSRCCWBALRBD4COT</t>
         </is>
       </c>
     </row>
     <row r="643">
-      <c r="A643" s="2" t="inlineStr">
-        <is>
-          <t>LVLLHBUFF
-电平转换器</t>
-        </is>
-      </c>
-      <c r="B643" s="11" t="inlineStr">
-        <is>
-          <t>LVLLHBUFFSNKD8COTLN</t>
-        </is>
-      </c>
-      <c r="C643" s="11" t="n"/>
+      <c r="A643" s="4" t="n"/>
+      <c r="B643" s="6" t="n"/>
+      <c r="C643" s="6" t="inlineStr">
+        <is>
+          <t>LVLLHCHSRCCWRBD4CNWCOT</t>
+        </is>
+      </c>
     </row>
     <row r="644">
       <c r="A644" s="4" t="n"/>
-      <c r="B644" s="6" t="inlineStr">
-        <is>
-          <t>LVLLHBUFFSRCD1COT</t>
-        </is>
-      </c>
-      <c r="C644" s="6" t="n"/>
+      <c r="B644" s="6" t="n"/>
+      <c r="C644" s="6" t="inlineStr">
+        <is>
+          <t>LVLLHCHSRCCWRBD4COT</t>
+        </is>
+      </c>
     </row>
     <row r="645">
       <c r="A645" s="4" t="n"/>
       <c r="B645" s="6" t="n"/>
       <c r="C645" s="6" t="inlineStr">
         <is>
-          <t>LVLLHBUFFSNKCWBALD4COT</t>
+          <t>LVLLHCLSNKCWBALRBD4COT</t>
         </is>
       </c>
     </row>
@@ -7657,7 +7602,7 @@
       <c r="B646" s="6" t="n"/>
       <c r="C646" s="6" t="inlineStr">
         <is>
-          <t>LVLLHBUFFSNKCWD4CNWBALCOT</t>
+          <t>LVLLHCLSNKCWRBD2CNWCOT</t>
         </is>
       </c>
     </row>
@@ -7666,7 +7611,7 @@
       <c r="B647" s="6" t="n"/>
       <c r="C647" s="6" t="inlineStr">
         <is>
-          <t>LVLLHBUFFSRCCWBALD1COT</t>
+          <t>LVLLHCLSNKCWRBD2COT</t>
         </is>
       </c>
     </row>
@@ -7675,7 +7620,7 @@
       <c r="B648" s="8" t="n"/>
       <c r="C648" s="8" t="inlineStr">
         <is>
-          <t>LVLLHBUFFSRCCWD8CNWCOTLN</t>
+          <t>LVLLHCLSRCCWRBD4CNWCOT</t>
         </is>
       </c>
     </row>
@@ -7694,23 +7639,18 @@
       </c>
     </row>
     <row r="650">
-      <c r="A650" s="7" t="n"/>
-      <c r="B650" s="8" t="n"/>
-      <c r="C650" s="8" t="inlineStr">
+      <c r="A650" s="4" t="n"/>
+      <c r="B650" s="6" t="n"/>
+      <c r="C650" s="6" t="inlineStr">
         <is>
           <t>LVUAN2X4COTC</t>
         </is>
       </c>
     </row>
     <row r="651">
-      <c r="A651" s="2" t="inlineStr">
-        <is>
-          <t>LVUFRAN2
-电平转换器</t>
-        </is>
-      </c>
-      <c r="B651" s="11" t="n"/>
-      <c r="C651" s="11" t="inlineStr">
+      <c r="A651" s="4" t="n"/>
+      <c r="B651" s="6" t="n"/>
+      <c r="C651" s="6" t="inlineStr">
         <is>
           <t>LVUFRAN2X2COTC</t>
         </is>
@@ -7728,7 +7668,7 @@
     <row r="653">
       <c r="A653" s="2" t="inlineStr">
         <is>
-          <t>LVUFROR2
+          <t>LVUOR2
 电平转换器</t>
         </is>
       </c>
@@ -7740,23 +7680,18 @@
       </c>
     </row>
     <row r="654">
-      <c r="A654" s="7" t="n"/>
-      <c r="B654" s="8" t="n"/>
-      <c r="C654" s="8" t="inlineStr">
+      <c r="A654" s="4" t="n"/>
+      <c r="B654" s="6" t="n"/>
+      <c r="C654" s="6" t="inlineStr">
         <is>
           <t>LVUFROR2N1X4COTC</t>
         </is>
       </c>
     </row>
     <row r="655">
-      <c r="A655" s="2" t="inlineStr">
-        <is>
-          <t>LVUOR2
-电平转换器</t>
-        </is>
-      </c>
-      <c r="B655" s="11" t="n"/>
-      <c r="C655" s="11" t="inlineStr">
+      <c r="A655" s="4" t="n"/>
+      <c r="B655" s="6" t="n"/>
+      <c r="C655" s="6" t="inlineStr">
         <is>
           <t>LVUOR2N1X1COTC</t>
         </is>
@@ -8385,8 +8320,8 @@
     <row r="714">
       <c r="A714" s="2" t="inlineStr">
         <is>
-          <t>MUX2NND2
-复合多路选择器</t>
+          <t>MUX2NN
+多路选择器</t>
         </is>
       </c>
       <c r="B714" s="11" t="inlineStr">
@@ -8508,8 +8443,8 @@
     <row r="725">
       <c r="A725" s="9" t="inlineStr">
         <is>
-          <t>MUX3ND1
-复合多路选择器</t>
+          <t>MUX3N
+反相多路选择器</t>
         </is>
       </c>
       <c r="B725" s="10" t="inlineStr">
@@ -12741,7 +12676,7 @@
     <row r="1149">
       <c r="A1149" s="9" t="inlineStr">
         <is>
-          <t>TIEHXP
+          <t>TIEH
 电平钳位</t>
         </is>
       </c>
@@ -12755,7 +12690,7 @@
     <row r="1150">
       <c r="A1150" s="9" t="inlineStr">
         <is>
-          <t>TIELXN
+          <t>TIEL
 电平钳位</t>
         </is>
       </c>
@@ -13935,32 +13870,33 @@
       <c r="C1261" s="8" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="204">
+  <mergeCells count="203">
     <mergeCell ref="A540:A543"/>
     <mergeCell ref="A106:A117"/>
     <mergeCell ref="A378:A384"/>
     <mergeCell ref="A399:A400"/>
-    <mergeCell ref="A268:A269"/>
     <mergeCell ref="A701:A706"/>
-    <mergeCell ref="A649:A650"/>
     <mergeCell ref="A947:A948"/>
     <mergeCell ref="A335:A336"/>
+    <mergeCell ref="A397:A398"/>
     <mergeCell ref="A966:A977"/>
     <mergeCell ref="A586:A587"/>
     <mergeCell ref="A30:A37"/>
     <mergeCell ref="A696:A700"/>
     <mergeCell ref="A413:A414"/>
     <mergeCell ref="A582:A583"/>
+    <mergeCell ref="A649:A652"/>
     <mergeCell ref="A1255:A1257"/>
+    <mergeCell ref="A631:A648"/>
     <mergeCell ref="A71:A74"/>
     <mergeCell ref="A189:A192"/>
     <mergeCell ref="A374:A377"/>
     <mergeCell ref="A989:A990"/>
+    <mergeCell ref="A605:A609"/>
     <mergeCell ref="A1075:A1083"/>
     <mergeCell ref="A164:A167"/>
     <mergeCell ref="A675:A676"/>
     <mergeCell ref="A1128:A1138"/>
-    <mergeCell ref="A244:A247"/>
     <mergeCell ref="A1021:A1025"/>
     <mergeCell ref="A1175:A1178"/>
     <mergeCell ref="A1232:A1236"/>
@@ -13985,9 +13921,8 @@
     <mergeCell ref="A1033:A1035"/>
     <mergeCell ref="A569:A576"/>
     <mergeCell ref="A719:A721"/>
-    <mergeCell ref="A653:A654"/>
+    <mergeCell ref="A1259:A1261"/>
     <mergeCell ref="A2:A6"/>
-    <mergeCell ref="A1259:A1261"/>
     <mergeCell ref="A1026:A1029"/>
     <mergeCell ref="A339:A340"/>
     <mergeCell ref="A177:A178"/>
@@ -14002,7 +13937,7 @@
     <mergeCell ref="A300:A307"/>
     <mergeCell ref="A662:A666"/>
     <mergeCell ref="A1196:A1200"/>
-    <mergeCell ref="A624:A627"/>
+    <mergeCell ref="A264:A269"/>
     <mergeCell ref="A405:A406"/>
     <mergeCell ref="A454:A455"/>
     <mergeCell ref="A172:A174"/>
@@ -14018,8 +13953,8 @@
     <mergeCell ref="A681:A686"/>
     <mergeCell ref="A407:A408"/>
     <mergeCell ref="A667:A669"/>
+    <mergeCell ref="A328:A329"/>
     <mergeCell ref="A337:A338"/>
-    <mergeCell ref="A608:A609"/>
     <mergeCell ref="A126:A128"/>
     <mergeCell ref="A534:A539"/>
     <mergeCell ref="A1084:A1087"/>
@@ -14031,7 +13966,6 @@
     <mergeCell ref="A1089:A1127"/>
     <mergeCell ref="A1201:A1217"/>
     <mergeCell ref="A473:A474"/>
-    <mergeCell ref="A631:A642"/>
     <mergeCell ref="A1151:A1152"/>
     <mergeCell ref="A551:A554"/>
     <mergeCell ref="A457:A458"/>
@@ -14045,8 +13979,6 @@
     <mergeCell ref="A600:A604"/>
     <mergeCell ref="A735:A746"/>
     <mergeCell ref="A717:A718"/>
-    <mergeCell ref="A643:A648"/>
-    <mergeCell ref="A264:A267"/>
     <mergeCell ref="A38:A48"/>
     <mergeCell ref="A497:A500"/>
     <mergeCell ref="A726:A728"/>
@@ -14058,13 +13990,12 @@
     <mergeCell ref="A483:A484"/>
     <mergeCell ref="A490:A492"/>
     <mergeCell ref="A1224:A1227"/>
-    <mergeCell ref="A605:A607"/>
     <mergeCell ref="A898:A904"/>
     <mergeCell ref="A991:A999"/>
+    <mergeCell ref="A610:A612"/>
     <mergeCell ref="A179:A184"/>
     <mergeCell ref="A122:A123"/>
     <mergeCell ref="A411:A412"/>
-    <mergeCell ref="A651:A652"/>
     <mergeCell ref="A670:A673"/>
     <mergeCell ref="A1004:A1005"/>
     <mergeCell ref="A1228:A1230"/>
@@ -14087,11 +14018,13 @@
     <mergeCell ref="A511:A512"/>
     <mergeCell ref="A1139:A1142"/>
     <mergeCell ref="A271:A277"/>
+    <mergeCell ref="A624:A630"/>
     <mergeCell ref="A785:A786"/>
     <mergeCell ref="A1191:A1195"/>
     <mergeCell ref="A448:A449"/>
     <mergeCell ref="A792:A798"/>
     <mergeCell ref="A210:A214"/>
+    <mergeCell ref="A244:A248"/>
     <mergeCell ref="A876:A886"/>
     <mergeCell ref="A291:A294"/>
     <mergeCell ref="A432:A434"/>
@@ -14104,6 +14037,7 @@
     <mergeCell ref="A732:A734"/>
     <mergeCell ref="A261:A263"/>
     <mergeCell ref="A1030:A1032"/>
+    <mergeCell ref="A393:A394"/>
     <mergeCell ref="A155:A159"/>
     <mergeCell ref="A803:A857"/>
     <mergeCell ref="A501:A508"/>
@@ -14115,6 +14049,7 @@
     <mergeCell ref="A518:A522"/>
     <mergeCell ref="A132:A134"/>
     <mergeCell ref="A1182:A1183"/>
+    <mergeCell ref="A386:A387"/>
     <mergeCell ref="A401:A402"/>
     <mergeCell ref="A689:A694"/>
     <mergeCell ref="A863:A875"/>
@@ -14124,12 +14059,12 @@
     <mergeCell ref="A450:A451"/>
     <mergeCell ref="A332:A333"/>
     <mergeCell ref="A589:A595"/>
-    <mergeCell ref="A628:A630"/>
     <mergeCell ref="A215:A216"/>
     <mergeCell ref="A677:A679"/>
     <mergeCell ref="A75:A77"/>
     <mergeCell ref="A193:A197"/>
     <mergeCell ref="A892:A897"/>
+    <mergeCell ref="A653:A657"/>
     <mergeCell ref="A1000:A1003"/>
     <mergeCell ref="A78:A84"/>
     <mergeCell ref="A452:A453"/>
@@ -14137,7 +14072,6 @@
     <mergeCell ref="A50:A56"/>
     <mergeCell ref="A129:A131"/>
     <mergeCell ref="A710:A713"/>
-    <mergeCell ref="A655:A657"/>
     <mergeCell ref="A279:A284"/>
     <mergeCell ref="A308:A315"/>
   </mergeCells>

</xml_diff>

<commit_message>
Regenerate keys after MUX2NND2 compound fix.
Co-authored-by: EsaLongs <EsaLongs@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/preview/NP1PP_vs_C1Y_preview.xlsx
+++ b/preview/NP1PP_vs_C1Y_preview.xlsx
@@ -8320,8 +8320,8 @@
     <row r="714">
       <c r="A714" s="2" t="inlineStr">
         <is>
-          <t>MUX2NN
-多路选择器</t>
+          <t>MUX2NND2
+复合多路选择器</t>
         </is>
       </c>
       <c r="B714" s="11" t="inlineStr">

</xml_diff>

<commit_message>
Keep Excel column B as English KEY only.
Chinese remains only in column A; column B no longer repeats the label.

Co-authored-by: EsaLongs <EsaLongs@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/preview/NP1PP_vs_C1Y_preview.xlsx
+++ b/preview/NP1PP_vs_C1Y_preview.xlsx
@@ -498,8 +498,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>DF
-D触发器</t>
+          <t>DF</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
@@ -823,8 +822,7 @@
       <c r="A34" s="2" t="n"/>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>GDF
-D触发器</t>
+          <t>GDF</t>
         </is>
       </c>
       <c r="C34" s="8" t="inlineStr">
@@ -870,8 +868,7 @@
       </c>
       <c r="B37" s="10" t="inlineStr">
         <is>
-          <t>BUFT
-三态缓冲器</t>
+          <t>BUFT</t>
         </is>
       </c>
       <c r="C37" s="11" t="inlineStr">
@@ -889,8 +886,7 @@
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>GPULL0
-上拉/下拉</t>
+          <t>GPULL0</t>
         </is>
       </c>
       <c r="C38" s="11" t="n"/>
@@ -904,8 +900,7 @@
       <c r="A39" s="10" t="n"/>
       <c r="B39" s="10" t="inlineStr">
         <is>
-          <t>GPULL1
-上拉/下拉</t>
+          <t>GPULL1</t>
         </is>
       </c>
       <c r="C39" s="11" t="n"/>
@@ -923,8 +918,7 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>AO21
-与或门</t>
+          <t>AO21</t>
         </is>
       </c>
       <c r="C40" s="8" t="inlineStr">
@@ -1006,8 +1000,7 @@
       <c r="A47" s="2" t="n"/>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>AO211
-与或门</t>
+          <t>AO211</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
@@ -1081,8 +1074,7 @@
       <c r="A54" s="2" t="n"/>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>AO22
-与或门</t>
+          <t>AO22</t>
         </is>
       </c>
       <c r="C54" s="8" t="inlineStr">
@@ -1160,8 +1152,7 @@
       <c r="A61" s="2" t="n"/>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>AO222
-与或门</t>
+          <t>AO222</t>
         </is>
       </c>
       <c r="C61" s="3" t="inlineStr">
@@ -1205,8 +1196,7 @@
       <c r="A65" s="2" t="n"/>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>AO33
-与或门</t>
+          <t>AO33</t>
         </is>
       </c>
       <c r="C65" s="3" t="inlineStr">
@@ -1240,8 +1230,7 @@
       <c r="A68" s="10" t="n"/>
       <c r="B68" s="10" t="inlineStr">
         <is>
-          <t>GAO21
-与或门</t>
+          <t>GAO21</t>
         </is>
       </c>
       <c r="C68" s="12" t="inlineStr">
@@ -1259,8 +1248,7 @@
       <c r="A69" s="10" t="n"/>
       <c r="B69" s="10" t="inlineStr">
         <is>
-          <t>GAO22
-与或门</t>
+          <t>GAO22</t>
         </is>
       </c>
       <c r="C69" s="12" t="inlineStr">
@@ -1278,8 +1266,7 @@
       <c r="A70" s="10" t="n"/>
       <c r="B70" s="10" t="inlineStr">
         <is>
-          <t>GAO31
-与或门</t>
+          <t>GAO31</t>
         </is>
       </c>
       <c r="C70" s="11" t="n"/>
@@ -1293,8 +1280,7 @@
       <c r="A71" s="10" t="n"/>
       <c r="B71" s="10" t="inlineStr">
         <is>
-          <t>GAO32
-与或门</t>
+          <t>GAO32</t>
         </is>
       </c>
       <c r="C71" s="11" t="n"/>
@@ -1312,8 +1298,7 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>AOI21
-与或非门</t>
+          <t>AOI21</t>
         </is>
       </c>
       <c r="C72" s="3" t="inlineStr">
@@ -1527,8 +1512,7 @@
       <c r="A93" s="2" t="n"/>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>AOI211
-与或非门</t>
+          <t>AOI211</t>
         </is>
       </c>
       <c r="C93" s="8" t="inlineStr">
@@ -1660,8 +1644,7 @@
       <c r="A105" s="2" t="n"/>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>AOI2111
-与或非门</t>
+          <t>AOI2111</t>
         </is>
       </c>
       <c r="C105" s="3" t="inlineStr">
@@ -1705,8 +1688,7 @@
       <c r="A109" s="2" t="n"/>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>AOI22
-与或非门</t>
+          <t>AOI22</t>
         </is>
       </c>
       <c r="C109" s="3" t="inlineStr">
@@ -1910,8 +1892,7 @@
       <c r="A129" s="2" t="n"/>
       <c r="B129" s="2" t="inlineStr">
         <is>
-          <t>AOI221
-与或非门</t>
+          <t>AOI221</t>
         </is>
       </c>
       <c r="C129" s="8" t="inlineStr">
@@ -1969,8 +1950,7 @@
       <c r="A134" s="2" t="n"/>
       <c r="B134" s="2" t="inlineStr">
         <is>
-          <t>AOI2211
-与或非门</t>
+          <t>AOI2211</t>
         </is>
       </c>
       <c r="C134" s="3" t="inlineStr">
@@ -2014,8 +1994,7 @@
       <c r="A138" s="2" t="n"/>
       <c r="B138" s="2" t="inlineStr">
         <is>
-          <t>AOI222
-与或非门</t>
+          <t>AOI222</t>
         </is>
       </c>
       <c r="C138" s="8" t="inlineStr">
@@ -2067,8 +2046,7 @@
       <c r="A142" s="2" t="n"/>
       <c r="B142" s="2" t="inlineStr">
         <is>
-          <t>AOI2221
-与或非门</t>
+          <t>AOI2221</t>
         </is>
       </c>
       <c r="C142" s="3" t="inlineStr">
@@ -2112,8 +2090,7 @@
       <c r="A146" s="2" t="n"/>
       <c r="B146" s="2" t="inlineStr">
         <is>
-          <t>AOI2222
-与或非门</t>
+          <t>AOI2222</t>
         </is>
       </c>
       <c r="C146" s="3" t="inlineStr">
@@ -2147,8 +2124,7 @@
       <c r="A149" s="2" t="n"/>
       <c r="B149" s="2" t="inlineStr">
         <is>
-          <t>AOI31
-与或非门</t>
+          <t>AOI31</t>
         </is>
       </c>
       <c r="C149" s="3" t="inlineStr">
@@ -2202,8 +2178,7 @@
       <c r="A154" s="2" t="n"/>
       <c r="B154" s="2" t="inlineStr">
         <is>
-          <t>AOI311
-与或非门</t>
+          <t>AOI311</t>
         </is>
       </c>
       <c r="C154" s="8" t="inlineStr">
@@ -2251,8 +2226,7 @@
       <c r="A158" s="2" t="n"/>
       <c r="B158" s="2" t="inlineStr">
         <is>
-          <t>AOI32
-与或非门</t>
+          <t>AOI32</t>
         </is>
       </c>
       <c r="C158" s="8" t="inlineStr">
@@ -2310,8 +2284,7 @@
       <c r="A163" s="2" t="n"/>
       <c r="B163" s="2" t="inlineStr">
         <is>
-          <t>AOI321
-与或非门</t>
+          <t>AOI321</t>
         </is>
       </c>
       <c r="C163" s="3" t="inlineStr">
@@ -2345,8 +2318,7 @@
       <c r="A166" s="2" t="n"/>
       <c r="B166" s="2" t="inlineStr">
         <is>
-          <t>AOI33
-与或非门</t>
+          <t>AOI33</t>
         </is>
       </c>
       <c r="C166" s="8" t="inlineStr">
@@ -2408,8 +2380,7 @@
       <c r="A171" s="2" t="n"/>
       <c r="B171" s="2" t="inlineStr">
         <is>
-          <t>GAOI21
-与或非门</t>
+          <t>GAOI21</t>
         </is>
       </c>
       <c r="C171" s="3" t="inlineStr">
@@ -2433,8 +2404,7 @@
       <c r="A173" s="10" t="n"/>
       <c r="B173" s="10" t="inlineStr">
         <is>
-          <t>GAOI211
-与或非门</t>
+          <t>GAOI211</t>
         </is>
       </c>
       <c r="C173" s="11" t="n"/>
@@ -2448,8 +2418,7 @@
       <c r="A174" s="2" t="n"/>
       <c r="B174" s="2" t="inlineStr">
         <is>
-          <t>GAOI22
-与或非门</t>
+          <t>GAOI22</t>
         </is>
       </c>
       <c r="C174" s="3" t="inlineStr">
@@ -2473,8 +2442,7 @@
       <c r="A176" s="10" t="n"/>
       <c r="B176" s="10" t="inlineStr">
         <is>
-          <t>GAOI31
-与或非门</t>
+          <t>GAOI31</t>
         </is>
       </c>
       <c r="C176" s="11" t="n"/>
@@ -2488,8 +2456,7 @@
       <c r="A177" s="10" t="n"/>
       <c r="B177" s="10" t="inlineStr">
         <is>
-          <t>GAOI32
-与或非门</t>
+          <t>GAOI32</t>
         </is>
       </c>
       <c r="C177" s="11" t="n"/>
@@ -2503,8 +2470,7 @@
       <c r="A178" s="10" t="n"/>
       <c r="B178" s="10" t="inlineStr">
         <is>
-          <t>GAOI33
-与或非门</t>
+          <t>GAOI33</t>
         </is>
       </c>
       <c r="C178" s="11" t="n"/>
@@ -2522,8 +2488,7 @@
       </c>
       <c r="B179" s="2" t="inlineStr">
         <is>
-          <t>AN2
-与门</t>
+          <t>AN2</t>
         </is>
       </c>
       <c r="C179" s="8" t="inlineStr">
@@ -2769,8 +2734,7 @@
       <c r="A202" s="2" t="n"/>
       <c r="B202" s="2" t="inlineStr">
         <is>
-          <t>AN3
-与门</t>
+          <t>AN3</t>
         </is>
       </c>
       <c r="C202" s="8" t="inlineStr">
@@ -2870,8 +2834,7 @@
       <c r="A210" s="2" t="n"/>
       <c r="B210" s="2" t="inlineStr">
         <is>
-          <t>AN4
-与门</t>
+          <t>AN4</t>
         </is>
       </c>
       <c r="C210" s="8" t="inlineStr">
@@ -2993,8 +2956,7 @@
       <c r="A221" s="10" t="n"/>
       <c r="B221" s="10" t="inlineStr">
         <is>
-          <t>GAN2
-与门</t>
+          <t>GAN2</t>
         </is>
       </c>
       <c r="C221" s="11" t="inlineStr">
@@ -3008,8 +2970,7 @@
       <c r="A222" s="2" t="n"/>
       <c r="B222" s="2" t="inlineStr">
         <is>
-          <t>GAN3
-与门</t>
+          <t>GAN3</t>
         </is>
       </c>
       <c r="C222" s="3" t="inlineStr">
@@ -3033,8 +2994,7 @@
       <c r="A224" s="10" t="n"/>
       <c r="B224" s="10" t="inlineStr">
         <is>
-          <t>GAN4
-与门</t>
+          <t>GAN4</t>
         </is>
       </c>
       <c r="C224" s="11" t="inlineStr">
@@ -3052,8 +3012,7 @@
       </c>
       <c r="B225" s="2" t="inlineStr">
         <is>
-          <t>GND2
-与非门</t>
+          <t>GND2</t>
         </is>
       </c>
       <c r="C225" s="3" t="inlineStr">
@@ -3077,8 +3036,7 @@
       <c r="A227" s="10" t="n"/>
       <c r="B227" s="10" t="inlineStr">
         <is>
-          <t>GND3
-与非门</t>
+          <t>GND3</t>
         </is>
       </c>
       <c r="C227" s="11" t="inlineStr">
@@ -3092,8 +3050,7 @@
       <c r="A228" s="2" t="n"/>
       <c r="B228" s="2" t="inlineStr">
         <is>
-          <t>GND4
-与非门</t>
+          <t>GND4</t>
         </is>
       </c>
       <c r="C228" s="3" t="inlineStr">
@@ -3117,8 +3074,7 @@
       <c r="A230" s="2" t="n"/>
       <c r="B230" s="2" t="inlineStr">
         <is>
-          <t>IIND3
-与非门</t>
+          <t>IIND3</t>
         </is>
       </c>
       <c r="C230" s="3" t="inlineStr">
@@ -3172,8 +3128,7 @@
       <c r="A235" s="10" t="n"/>
       <c r="B235" s="10" t="inlineStr">
         <is>
-          <t>IIND4
-与非门</t>
+          <t>IIND4</t>
         </is>
       </c>
       <c r="C235" s="11" t="inlineStr">
@@ -3187,8 +3142,7 @@
       <c r="A236" s="2" t="n"/>
       <c r="B236" s="2" t="inlineStr">
         <is>
-          <t>IND2
-与非门</t>
+          <t>IND2</t>
         </is>
       </c>
       <c r="C236" s="3" t="inlineStr">
@@ -3262,8 +3216,7 @@
       <c r="A243" s="2" t="n"/>
       <c r="B243" s="2" t="inlineStr">
         <is>
-          <t>IND3
-与非门</t>
+          <t>IND3</t>
         </is>
       </c>
       <c r="C243" s="3" t="inlineStr">
@@ -3307,8 +3260,7 @@
       <c r="A247" s="10" t="n"/>
       <c r="B247" s="10" t="inlineStr">
         <is>
-          <t>IND4
-与非门</t>
+          <t>IND4</t>
         </is>
       </c>
       <c r="C247" s="11" t="inlineStr">
@@ -3322,8 +3274,7 @@
       <c r="A248" s="2" t="n"/>
       <c r="B248" s="2" t="inlineStr">
         <is>
-          <t>ND2
-与非门</t>
+          <t>ND2</t>
         </is>
       </c>
       <c r="C248" s="8" t="inlineStr">
@@ -3719,8 +3670,7 @@
       <c r="A286" s="2" t="n"/>
       <c r="B286" s="2" t="inlineStr">
         <is>
-          <t>ND3
-与非门</t>
+          <t>ND3</t>
         </is>
       </c>
       <c r="C286" s="3" t="inlineStr">
@@ -3794,8 +3744,7 @@
       <c r="A293" s="2" t="n"/>
       <c r="B293" s="2" t="inlineStr">
         <is>
-          <t>ND4
-与非门</t>
+          <t>ND4</t>
         </is>
       </c>
       <c r="C293" s="3" t="inlineStr">
@@ -3843,8 +3792,7 @@
       </c>
       <c r="B297" s="10" t="inlineStr">
         <is>
-          <t>SDFFE
-使能扫描触发器</t>
+          <t>SDFFE</t>
         </is>
       </c>
       <c r="C297" s="11" t="n"/>
@@ -3862,8 +3810,7 @@
       </c>
       <c r="B298" s="2" t="inlineStr">
         <is>
-          <t>EDF
-使能触发器</t>
+          <t>EDF</t>
         </is>
       </c>
       <c r="C298" s="3" t="inlineStr">
@@ -3911,8 +3858,7 @@
       </c>
       <c r="B302" s="2" t="inlineStr">
         <is>
-          <t>FA1
-全加器</t>
+          <t>FA1</t>
         </is>
       </c>
       <c r="C302" s="8" t="inlineStr">
@@ -4024,8 +3970,7 @@
       </c>
       <c r="B312" s="2" t="inlineStr">
         <is>
-          <t>HA1
-半加器</t>
+          <t>HA1</t>
         </is>
       </c>
       <c r="C312" s="8" t="inlineStr">
@@ -4073,8 +4018,7 @@
       <c r="A316" s="2" t="n"/>
       <c r="B316" s="2" t="inlineStr">
         <is>
-          <t>HAC1
-半加器</t>
+          <t>HAC1</t>
         </is>
       </c>
       <c r="C316" s="3" t="inlineStr">
@@ -4158,8 +4102,7 @@
       <c r="A324" s="10" t="n"/>
       <c r="B324" s="10" t="inlineStr">
         <is>
-          <t>HAN1
-半加器</t>
+          <t>HAN1</t>
         </is>
       </c>
       <c r="C324" s="11" t="n"/>
@@ -4177,8 +4120,7 @@
       </c>
       <c r="B325" s="2" t="inlineStr">
         <is>
-          <t>CMPE32
-压缩器</t>
+          <t>CMPE32</t>
         </is>
       </c>
       <c r="C325" s="3" t="inlineStr">
@@ -4262,8 +4204,7 @@
       <c r="A333" s="2" t="n"/>
       <c r="B333" s="2" t="inlineStr">
         <is>
-          <t>CMPE42
-压缩器</t>
+          <t>CMPE42</t>
         </is>
       </c>
       <c r="C333" s="3" t="inlineStr">
@@ -4351,8 +4292,7 @@
       </c>
       <c r="B341" s="10" t="inlineStr">
         <is>
-          <t>DCAP10
-去耦电容</t>
+          <t>DCAP10</t>
         </is>
       </c>
       <c r="C341" s="11" t="inlineStr">
@@ -4366,8 +4306,7 @@
       <c r="A342" s="10" t="n"/>
       <c r="B342" s="10" t="inlineStr">
         <is>
-          <t>DCAP16
-去耦电容</t>
+          <t>DCAP16</t>
         </is>
       </c>
       <c r="C342" s="11" t="n"/>
@@ -4381,8 +4320,7 @@
       <c r="A343" s="10" t="n"/>
       <c r="B343" s="10" t="inlineStr">
         <is>
-          <t>DCAP20
-去耦电容</t>
+          <t>DCAP20</t>
         </is>
       </c>
       <c r="C343" s="11" t="inlineStr">
@@ -4396,8 +4334,7 @@
       <c r="A344" s="10" t="n"/>
       <c r="B344" s="10" t="inlineStr">
         <is>
-          <t>DCAP32
-去耦电容</t>
+          <t>DCAP32</t>
         </is>
       </c>
       <c r="C344" s="11" t="n"/>
@@ -4411,8 +4348,7 @@
       <c r="A345" s="2" t="n"/>
       <c r="B345" s="2" t="inlineStr">
         <is>
-          <t>DCAP4
-去耦电容</t>
+          <t>DCAP4</t>
         </is>
       </c>
       <c r="C345" s="3" t="inlineStr">
@@ -4436,8 +4372,7 @@
       <c r="A347" s="10" t="n"/>
       <c r="B347" s="10" t="inlineStr">
         <is>
-          <t>DCAP40
-去耦电容</t>
+          <t>DCAP40</t>
         </is>
       </c>
       <c r="C347" s="11" t="inlineStr">
@@ -4451,8 +4386,7 @@
       <c r="A348" s="10" t="n"/>
       <c r="B348" s="10" t="inlineStr">
         <is>
-          <t>DCAP5
-去耦电容</t>
+          <t>DCAP5</t>
         </is>
       </c>
       <c r="C348" s="11" t="inlineStr">
@@ -4466,8 +4400,7 @@
       <c r="A349" s="10" t="n"/>
       <c r="B349" s="10" t="inlineStr">
         <is>
-          <t>DCAP64
-去耦电容</t>
+          <t>DCAP64</t>
         </is>
       </c>
       <c r="C349" s="11" t="n"/>
@@ -4481,8 +4414,7 @@
       <c r="A350" s="10" t="n"/>
       <c r="B350" s="10" t="inlineStr">
         <is>
-          <t>DCAP8
-去耦电容</t>
+          <t>DCAP8</t>
         </is>
       </c>
       <c r="C350" s="11" t="n"/>
@@ -4496,8 +4428,7 @@
       <c r="A351" s="10" t="n"/>
       <c r="B351" s="10" t="inlineStr">
         <is>
-          <t>GDCAP10
-去耦电容</t>
+          <t>GDCAP10</t>
         </is>
       </c>
       <c r="C351" s="11" t="n"/>
@@ -4511,8 +4442,7 @@
       <c r="A352" s="2" t="n"/>
       <c r="B352" s="2" t="inlineStr">
         <is>
-          <t>GDCAP12
-去耦电容</t>
+          <t>GDCAP12</t>
         </is>
       </c>
       <c r="C352" s="3" t="inlineStr">
@@ -4536,8 +4466,7 @@
       <c r="A354" s="2" t="n"/>
       <c r="B354" s="2" t="inlineStr">
         <is>
-          <t>GDCAP2
-去耦电容</t>
+          <t>GDCAP2</t>
         </is>
       </c>
       <c r="C354" s="3" t="inlineStr">
@@ -4561,8 +4490,7 @@
       <c r="A356" s="2" t="n"/>
       <c r="B356" s="2" t="inlineStr">
         <is>
-          <t>GDCAP4
-去耦电容</t>
+          <t>GDCAP4</t>
         </is>
       </c>
       <c r="C356" s="3" t="inlineStr">
@@ -4586,8 +4514,7 @@
       <c r="A358" s="2" t="n"/>
       <c r="B358" s="2" t="inlineStr">
         <is>
-          <t>GDCAP6
-去耦电容</t>
+          <t>GDCAP6</t>
         </is>
       </c>
       <c r="C358" s="3" t="inlineStr">
@@ -4611,8 +4538,7 @@
       <c r="A360" s="2" t="n"/>
       <c r="B360" s="2" t="inlineStr">
         <is>
-          <t>GDCAP8
-去耦电容</t>
+          <t>GDCAP8</t>
         </is>
       </c>
       <c r="C360" s="3" t="inlineStr">
@@ -4640,8 +4566,7 @@
       </c>
       <c r="B362" s="10" t="inlineStr">
         <is>
-          <t>APINV
-反相器</t>
+          <t>APINV</t>
         </is>
       </c>
       <c r="C362" s="11" t="inlineStr">
@@ -4655,8 +4580,7 @@
       <c r="A363" s="2" t="n"/>
       <c r="B363" s="2" t="inlineStr">
         <is>
-          <t>GINV
-反相器</t>
+          <t>GINV</t>
         </is>
       </c>
       <c r="C363" s="3" t="inlineStr">
@@ -4710,8 +4634,7 @@
       <c r="A368" s="10" t="n"/>
       <c r="B368" s="10" t="inlineStr">
         <is>
-          <t>INV
-反相器</t>
+          <t>INV</t>
         </is>
       </c>
       <c r="C368" s="11" t="inlineStr">
@@ -4729,8 +4652,7 @@
       </c>
       <c r="B369" s="10" t="inlineStr">
         <is>
-          <t>GMUX2N
-反相多路选择器</t>
+          <t>GMUX2N</t>
         </is>
       </c>
       <c r="C369" s="11" t="inlineStr">
@@ -4744,8 +4666,7 @@
       <c r="A370" s="10" t="n"/>
       <c r="B370" s="10" t="inlineStr">
         <is>
-          <t>MUX2I
-反相多路选择器</t>
+          <t>MUX2I</t>
         </is>
       </c>
       <c r="C370" s="11" t="inlineStr">
@@ -4759,8 +4680,7 @@
       <c r="A371" s="10" t="n"/>
       <c r="B371" s="10" t="inlineStr">
         <is>
-          <t>MUX3N
-反相多路选择器</t>
+          <t>MUX3N</t>
         </is>
       </c>
       <c r="C371" s="11" t="inlineStr">
@@ -4774,8 +4694,7 @@
       <c r="A372" s="10" t="n"/>
       <c r="B372" s="10" t="inlineStr">
         <is>
-          <t>MUX4N
-反相多路选择器</t>
+          <t>MUX4N</t>
         </is>
       </c>
       <c r="C372" s="11" t="n"/>
@@ -4789,8 +4708,7 @@
       <c r="A373" s="2" t="n"/>
       <c r="B373" s="2" t="inlineStr">
         <is>
-          <t>MXI2
-反相多路选择器</t>
+          <t>MXI2</t>
         </is>
       </c>
       <c r="C373" s="3" t="n"/>
@@ -4918,8 +4836,7 @@
       </c>
       <c r="B385" s="2" t="inlineStr">
         <is>
-          <t>GXNR2
-同或门</t>
+          <t>GXNR2</t>
         </is>
       </c>
       <c r="C385" s="3" t="inlineStr">
@@ -4943,8 +4860,7 @@
       <c r="A387" s="2" t="n"/>
       <c r="B387" s="2" t="inlineStr">
         <is>
-          <t>XNR2
-同或门</t>
+          <t>XNR2</t>
         </is>
       </c>
       <c r="C387" s="8" t="inlineStr">
@@ -5132,8 +5048,7 @@
       <c r="A405" s="2" t="n"/>
       <c r="B405" s="2" t="inlineStr">
         <is>
-          <t>XNR3
-同或门</t>
+          <t>XNR3</t>
         </is>
       </c>
       <c r="C405" s="3" t="inlineStr">
@@ -5187,8 +5102,7 @@
       <c r="A410" s="2" t="n"/>
       <c r="B410" s="2" t="inlineStr">
         <is>
-          <t>XNR4
-同或门</t>
+          <t>XNR4</t>
         </is>
       </c>
       <c r="C410" s="3" t="inlineStr">
@@ -5246,8 +5160,7 @@
       </c>
       <c r="B415" s="2" t="inlineStr">
         <is>
-          <t>SYNLHCNQ
-同步器</t>
+          <t>SYNLHCNQ</t>
         </is>
       </c>
       <c r="C415" s="3" t="inlineStr">
@@ -5271,8 +5184,7 @@
       <c r="A417" s="10" t="n"/>
       <c r="B417" s="10" t="inlineStr">
         <is>
-          <t>SYNLHQ
-同步器</t>
+          <t>SYNLHQ</t>
         </is>
       </c>
       <c r="C417" s="12" t="inlineStr">
@@ -5290,8 +5202,7 @@
       <c r="A418" s="10" t="n"/>
       <c r="B418" s="10" t="inlineStr">
         <is>
-          <t>SYNLHRPQ
-同步器</t>
+          <t>SYNLHRPQ</t>
         </is>
       </c>
       <c r="C418" s="11" t="n"/>
@@ -5305,8 +5216,7 @@
       <c r="A419" s="10" t="n"/>
       <c r="B419" s="10" t="inlineStr">
         <is>
-          <t>SYNLHSNQ
-同步器</t>
+          <t>SYNLHSNQ</t>
         </is>
       </c>
       <c r="C419" s="11" t="inlineStr">
@@ -5324,8 +5234,7 @@
       </c>
       <c r="B420" s="2" t="inlineStr">
         <is>
-          <t>SDFSYNC1
-同步触发器</t>
+          <t>SDFSYNC1</t>
         </is>
       </c>
       <c r="C420" s="3" t="n"/>
@@ -5353,8 +5262,7 @@
       </c>
       <c r="B422" s="2" t="inlineStr">
         <is>
-          <t>FILL1
-填充单元</t>
+          <t>FILL1</t>
         </is>
       </c>
       <c r="C422" s="3" t="n"/>
@@ -5378,8 +5286,7 @@
       <c r="A424" s="2" t="n"/>
       <c r="B424" s="2" t="inlineStr">
         <is>
-          <t>FILL12
-填充单元</t>
+          <t>FILL12</t>
         </is>
       </c>
       <c r="C424" s="3" t="inlineStr">
@@ -5403,8 +5310,7 @@
       <c r="A426" s="2" t="n"/>
       <c r="B426" s="2" t="inlineStr">
         <is>
-          <t>FILL16
-填充单元</t>
+          <t>FILL16</t>
         </is>
       </c>
       <c r="C426" s="8" t="inlineStr">
@@ -5432,8 +5338,7 @@
       <c r="A428" s="2" t="n"/>
       <c r="B428" s="2" t="inlineStr">
         <is>
-          <t>FILL2
-填充单元</t>
+          <t>FILL2</t>
         </is>
       </c>
       <c r="C428" s="3" t="inlineStr">
@@ -5457,8 +5362,7 @@
       <c r="A430" s="2" t="n"/>
       <c r="B430" s="2" t="inlineStr">
         <is>
-          <t>FILL3
-填充单元</t>
+          <t>FILL3</t>
         </is>
       </c>
       <c r="C430" s="8" t="inlineStr">
@@ -5486,8 +5390,7 @@
       <c r="A432" s="2" t="n"/>
       <c r="B432" s="2" t="inlineStr">
         <is>
-          <t>FILL32
-填充单元</t>
+          <t>FILL32</t>
         </is>
       </c>
       <c r="C432" s="3" t="inlineStr">
@@ -5511,8 +5414,7 @@
       <c r="A434" s="2" t="n"/>
       <c r="B434" s="2" t="inlineStr">
         <is>
-          <t>FILL4
-填充单元</t>
+          <t>FILL4</t>
         </is>
       </c>
       <c r="C434" s="8" t="inlineStr">
@@ -5540,8 +5442,7 @@
       <c r="A436" s="2" t="n"/>
       <c r="B436" s="2" t="inlineStr">
         <is>
-          <t>FILL64
-填充单元</t>
+          <t>FILL64</t>
         </is>
       </c>
       <c r="C436" s="8" t="inlineStr">
@@ -5569,8 +5470,7 @@
       <c r="A438" s="2" t="n"/>
       <c r="B438" s="2" t="inlineStr">
         <is>
-          <t>FILL8
-填充单元</t>
+          <t>FILL8</t>
         </is>
       </c>
       <c r="C438" s="3" t="inlineStr">
@@ -5594,8 +5494,7 @@
       <c r="A440" s="2" t="n"/>
       <c r="B440" s="2" t="inlineStr">
         <is>
-          <t>GFILL1
-填充单元</t>
+          <t>GFILL1</t>
         </is>
       </c>
       <c r="C440" s="3" t="inlineStr">
@@ -5619,8 +5518,7 @@
       <c r="A442" s="10" t="n"/>
       <c r="B442" s="10" t="inlineStr">
         <is>
-          <t>GFILL10
-填充单元</t>
+          <t>GFILL10</t>
         </is>
       </c>
       <c r="C442" s="11" t="n"/>
@@ -5634,8 +5532,7 @@
       <c r="A443" s="2" t="n"/>
       <c r="B443" s="2" t="inlineStr">
         <is>
-          <t>GFILL11
-填充单元</t>
+          <t>GFILL11</t>
         </is>
       </c>
       <c r="C443" s="3" t="inlineStr">
@@ -5669,8 +5566,7 @@
       <c r="A446" s="2" t="n"/>
       <c r="B446" s="2" t="inlineStr">
         <is>
-          <t>GFILL12
-填充单元</t>
+          <t>GFILL12</t>
         </is>
       </c>
       <c r="C446" s="3" t="inlineStr">
@@ -5694,8 +5590,7 @@
       <c r="A448" s="2" t="n"/>
       <c r="B448" s="2" t="inlineStr">
         <is>
-          <t>GFILL2
-填充单元</t>
+          <t>GFILL2</t>
         </is>
       </c>
       <c r="C448" s="3" t="inlineStr">
@@ -5739,8 +5634,7 @@
       <c r="A452" s="2" t="n"/>
       <c r="B452" s="2" t="inlineStr">
         <is>
-          <t>GFILL3
-填充单元</t>
+          <t>GFILL3</t>
         </is>
       </c>
       <c r="C452" s="3" t="inlineStr">
@@ -5784,8 +5678,7 @@
       <c r="A456" s="2" t="n"/>
       <c r="B456" s="2" t="inlineStr">
         <is>
-          <t>GFILL4
-填充单元</t>
+          <t>GFILL4</t>
         </is>
       </c>
       <c r="C456" s="3" t="inlineStr">
@@ -5829,8 +5722,7 @@
       <c r="A460" s="2" t="n"/>
       <c r="B460" s="2" t="inlineStr">
         <is>
-          <t>GFILL5
-填充单元</t>
+          <t>GFILL5</t>
         </is>
       </c>
       <c r="C460" s="3" t="inlineStr">
@@ -5874,8 +5766,7 @@
       <c r="A464" s="2" t="n"/>
       <c r="B464" s="2" t="inlineStr">
         <is>
-          <t>GFILL6
-填充单元</t>
+          <t>GFILL6</t>
         </is>
       </c>
       <c r="C464" s="3" t="inlineStr">
@@ -5919,8 +5810,7 @@
       <c r="A468" s="2" t="n"/>
       <c r="B468" s="2" t="inlineStr">
         <is>
-          <t>GFILL7
-填充单元</t>
+          <t>GFILL7</t>
         </is>
       </c>
       <c r="C468" s="3" t="inlineStr">
@@ -5954,8 +5844,7 @@
       <c r="A471" s="2" t="n"/>
       <c r="B471" s="2" t="inlineStr">
         <is>
-          <t>GFILL8
-填充单元</t>
+          <t>GFILL8</t>
         </is>
       </c>
       <c r="C471" s="3" t="inlineStr">
@@ -5999,8 +5888,7 @@
       <c r="A475" s="2" t="n"/>
       <c r="B475" s="2" t="inlineStr">
         <is>
-          <t>GFILL9
-填充单元</t>
+          <t>GFILL9</t>
         </is>
       </c>
       <c r="C475" s="3" t="inlineStr">
@@ -6038,8 +5926,7 @@
       </c>
       <c r="B478" s="2" t="inlineStr">
         <is>
-          <t>MUX2AOI
-复合多路选择器</t>
+          <t>MUX2AOI</t>
         </is>
       </c>
       <c r="C478" s="3" t="inlineStr">
@@ -6063,8 +5950,7 @@
       <c r="A480" s="2" t="n"/>
       <c r="B480" s="2" t="inlineStr">
         <is>
-          <t>MUX2ND2
-复合多路选择器</t>
+          <t>MUX2ND2</t>
         </is>
       </c>
       <c r="C480" s="3" t="inlineStr">
@@ -6108,8 +5994,7 @@
       <c r="A484" s="2" t="n"/>
       <c r="B484" s="2" t="inlineStr">
         <is>
-          <t>MUX2NND2
-复合多路选择器</t>
+          <t>MUX2NND2</t>
         </is>
       </c>
       <c r="C484" s="3" t="inlineStr">
@@ -6143,8 +6028,7 @@
       <c r="A487" s="2" t="n"/>
       <c r="B487" s="2" t="inlineStr">
         <is>
-          <t>MUX2NNR2
-复合多路选择器</t>
+          <t>MUX2NNR2</t>
         </is>
       </c>
       <c r="C487" s="3" t="inlineStr">
@@ -6168,8 +6052,7 @@
       <c r="A489" s="2" t="n"/>
       <c r="B489" s="2" t="inlineStr">
         <is>
-          <t>MUX2NR2
-复合多路选择器</t>
+          <t>MUX2NR2</t>
         </is>
       </c>
       <c r="C489" s="3" t="inlineStr">
@@ -6207,8 +6090,7 @@
       </c>
       <c r="B492" s="2" t="inlineStr">
         <is>
-          <t>AIOI21
-复合逻辑门</t>
+          <t>AIOI21</t>
         </is>
       </c>
       <c r="C492" s="8" t="inlineStr">
@@ -6270,8 +6152,7 @@
       <c r="A497" s="2" t="n"/>
       <c r="B497" s="2" t="inlineStr">
         <is>
-          <t>AOAI211
-复合逻辑门</t>
+          <t>AOAI211</t>
         </is>
       </c>
       <c r="C497" s="8" t="inlineStr">
@@ -6357,8 +6238,7 @@
       <c r="A504" s="2" t="n"/>
       <c r="B504" s="2" t="inlineStr">
         <is>
-          <t>AOI211INV
-复合逻辑门</t>
+          <t>AOI211INV</t>
         </is>
       </c>
       <c r="C504" s="3" t="inlineStr">
@@ -6382,8 +6262,7 @@
       <c r="A506" s="2" t="n"/>
       <c r="B506" s="2" t="inlineStr">
         <is>
-          <t>AOI21AOI21
-复合逻辑门</t>
+          <t>AOI21AOI21</t>
         </is>
       </c>
       <c r="C506" s="3" t="inlineStr">
@@ -6407,8 +6286,7 @@
       <c r="A508" s="2" t="n"/>
       <c r="B508" s="2" t="inlineStr">
         <is>
-          <t>AOI21ND2
-复合逻辑门</t>
+          <t>AOI21ND2</t>
         </is>
       </c>
       <c r="C508" s="3" t="inlineStr">
@@ -6442,8 +6320,7 @@
       <c r="A511" s="2" t="n"/>
       <c r="B511" s="2" t="inlineStr">
         <is>
-          <t>AOI21NR2
-复合逻辑门</t>
+          <t>AOI21NR2</t>
         </is>
       </c>
       <c r="C511" s="3" t="inlineStr">
@@ -6477,8 +6354,7 @@
       <c r="A514" s="2" t="n"/>
       <c r="B514" s="2" t="inlineStr">
         <is>
-          <t>AOI21OAI21
-复合逻辑门</t>
+          <t>AOI21OAI21</t>
         </is>
       </c>
       <c r="C514" s="3" t="inlineStr">
@@ -6512,8 +6388,7 @@
       <c r="A517" s="10" t="n"/>
       <c r="B517" s="10" t="inlineStr">
         <is>
-          <t>AOI22AOI21
-复合逻辑门</t>
+          <t>AOI22AOI21</t>
         </is>
       </c>
       <c r="C517" s="11" t="inlineStr">
@@ -6527,8 +6402,7 @@
       <c r="A518" s="10" t="n"/>
       <c r="B518" s="10" t="inlineStr">
         <is>
-          <t>AOI22AOI22
-复合逻辑门</t>
+          <t>AOI22AOI22</t>
         </is>
       </c>
       <c r="C518" s="11" t="inlineStr">
@@ -6542,8 +6416,7 @@
       <c r="A519" s="2" t="n"/>
       <c r="B519" s="2" t="inlineStr">
         <is>
-          <t>AOI22INV
-复合逻辑门</t>
+          <t>AOI22INV</t>
         </is>
       </c>
       <c r="C519" s="3" t="inlineStr">
@@ -6567,8 +6440,7 @@
       <c r="A521" s="2" t="n"/>
       <c r="B521" s="2" t="inlineStr">
         <is>
-          <t>AOI22ND2
-复合逻辑门</t>
+          <t>AOI22ND2</t>
         </is>
       </c>
       <c r="C521" s="3" t="inlineStr">
@@ -6632,8 +6504,7 @@
       <c r="A527" s="2" t="n"/>
       <c r="B527" s="2" t="inlineStr">
         <is>
-          <t>AOI22NR2
-复合逻辑门</t>
+          <t>AOI22NR2</t>
         </is>
       </c>
       <c r="C527" s="3" t="inlineStr">
@@ -6677,8 +6548,7 @@
       <c r="A531" s="2" t="n"/>
       <c r="B531" s="2" t="inlineStr">
         <is>
-          <t>AOI22OAI21
-复合逻辑门</t>
+          <t>AOI22OAI21</t>
         </is>
       </c>
       <c r="C531" s="3" t="inlineStr">
@@ -6722,8 +6592,7 @@
       <c r="A535" s="2" t="n"/>
       <c r="B535" s="2" t="inlineStr">
         <is>
-          <t>IAO21
-复合逻辑门</t>
+          <t>IAO21</t>
         </is>
       </c>
       <c r="C535" s="3" t="inlineStr">
@@ -6777,8 +6646,7 @@
       <c r="A540" s="2" t="n"/>
       <c r="B540" s="2" t="inlineStr">
         <is>
-          <t>IAO22
-复合逻辑门</t>
+          <t>IAO22</t>
         </is>
       </c>
       <c r="C540" s="8" t="inlineStr">
@@ -6840,8 +6708,7 @@
       <c r="A545" s="2" t="n"/>
       <c r="B545" s="2" t="inlineStr">
         <is>
-          <t>IAOI21
-复合逻辑门</t>
+          <t>IAOI21</t>
         </is>
       </c>
       <c r="C545" s="8" t="inlineStr">
@@ -6899,8 +6766,7 @@
       <c r="A550" s="10" t="n"/>
       <c r="B550" s="10" t="inlineStr">
         <is>
-          <t>INVAAOI21
-复合逻辑门</t>
+          <t>INVAAOI21</t>
         </is>
       </c>
       <c r="C550" s="11" t="inlineStr">
@@ -6914,8 +6780,7 @@
       <c r="A551" s="2" t="n"/>
       <c r="B551" s="2" t="inlineStr">
         <is>
-          <t>INVAOAI21
-复合逻辑门</t>
+          <t>INVAOAI21</t>
         </is>
       </c>
       <c r="C551" s="3" t="inlineStr">
@@ -6939,8 +6804,7 @@
       <c r="A553" s="2" t="n"/>
       <c r="B553" s="2" t="inlineStr">
         <is>
-          <t>INVBAOI21
-复合逻辑门</t>
+          <t>INVBAOI21</t>
         </is>
       </c>
       <c r="C553" s="3" t="inlineStr">
@@ -6964,8 +6828,7 @@
       <c r="A555" s="2" t="n"/>
       <c r="B555" s="2" t="inlineStr">
         <is>
-          <t>INVBOAI21
-复合逻辑门</t>
+          <t>INVBOAI21</t>
         </is>
       </c>
       <c r="C555" s="3" t="inlineStr">
@@ -6989,8 +6852,7 @@
       <c r="A557" s="2" t="n"/>
       <c r="B557" s="2" t="inlineStr">
         <is>
-          <t>IOA21
-复合逻辑门</t>
+          <t>IOA21</t>
         </is>
       </c>
       <c r="C557" s="8" t="inlineStr">
@@ -7068,8 +6930,7 @@
       <c r="A564" s="2" t="n"/>
       <c r="B564" s="2" t="inlineStr">
         <is>
-          <t>IOA22
-复合逻辑门</t>
+          <t>IOA22</t>
         </is>
       </c>
       <c r="C564" s="8" t="inlineStr">
@@ -7117,8 +6978,7 @@
       <c r="A568" s="2" t="n"/>
       <c r="B568" s="2" t="inlineStr">
         <is>
-          <t>IOAI21
-复合逻辑门</t>
+          <t>IOAI21</t>
         </is>
       </c>
       <c r="C568" s="8" t="inlineStr">
@@ -7180,8 +7040,7 @@
       <c r="A573" s="2" t="n"/>
       <c r="B573" s="2" t="inlineStr">
         <is>
-          <t>MAOI22
-复合逻辑门</t>
+          <t>MAOI22</t>
         </is>
       </c>
       <c r="C573" s="3" t="inlineStr">
@@ -7225,8 +7084,7 @@
       <c r="A577" s="2" t="n"/>
       <c r="B577" s="2" t="inlineStr">
         <is>
-          <t>MAOI222
-复合逻辑门</t>
+          <t>MAOI222</t>
         </is>
       </c>
       <c r="C577" s="3" t="inlineStr">
@@ -7280,8 +7138,7 @@
       <c r="A582" s="2" t="n"/>
       <c r="B582" s="2" t="inlineStr">
         <is>
-          <t>MOAI22
-复合逻辑门</t>
+          <t>MOAI22</t>
         </is>
       </c>
       <c r="C582" s="8" t="inlineStr">
@@ -7339,8 +7196,7 @@
       <c r="A587" s="2" t="n"/>
       <c r="B587" s="2" t="inlineStr">
         <is>
-          <t>ND2AOI21
-复合逻辑门</t>
+          <t>ND2AOI21</t>
         </is>
       </c>
       <c r="C587" s="3" t="inlineStr">
@@ -7364,8 +7220,7 @@
       <c r="A589" s="2" t="n"/>
       <c r="B589" s="2" t="inlineStr">
         <is>
-          <t>ND2IOA21
-复合逻辑门</t>
+          <t>ND2IOA21</t>
         </is>
       </c>
       <c r="C589" s="3" t="inlineStr">
@@ -7399,8 +7254,7 @@
       <c r="A592" s="2" t="n"/>
       <c r="B592" s="2" t="inlineStr">
         <is>
-          <t>ND2OAI21
-复合逻辑门</t>
+          <t>ND2OAI21</t>
         </is>
       </c>
       <c r="C592" s="3" t="inlineStr">
@@ -7424,8 +7278,7 @@
       <c r="A594" s="2" t="n"/>
       <c r="B594" s="2" t="inlineStr">
         <is>
-          <t>NR2AOI21
-复合逻辑门</t>
+          <t>NR2AOI21</t>
         </is>
       </c>
       <c r="C594" s="3" t="inlineStr">
@@ -7449,8 +7302,7 @@
       <c r="A596" s="2" t="n"/>
       <c r="B596" s="2" t="inlineStr">
         <is>
-          <t>NR2ND2
-复合逻辑门</t>
+          <t>NR2ND2</t>
         </is>
       </c>
       <c r="C596" s="3" t="inlineStr">
@@ -7484,8 +7336,7 @@
       <c r="A599" s="10" t="n"/>
       <c r="B599" s="10" t="inlineStr">
         <is>
-          <t>OAI211INV
-复合逻辑门</t>
+          <t>OAI211INV</t>
         </is>
       </c>
       <c r="C599" s="11" t="inlineStr">
@@ -7499,8 +7350,7 @@
       <c r="A600" s="10" t="n"/>
       <c r="B600" s="10" t="inlineStr">
         <is>
-          <t>OAI21AOI21
-复合逻辑门</t>
+          <t>OAI21AOI21</t>
         </is>
       </c>
       <c r="C600" s="11" t="n"/>
@@ -7514,8 +7364,7 @@
       <c r="A601" s="2" t="n"/>
       <c r="B601" s="2" t="inlineStr">
         <is>
-          <t>OAI21AOI22
-复合逻辑门</t>
+          <t>OAI21AOI22</t>
         </is>
       </c>
       <c r="C601" s="3" t="inlineStr">
@@ -7549,8 +7398,7 @@
       <c r="A604" s="2" t="n"/>
       <c r="B604" s="2" t="inlineStr">
         <is>
-          <t>OAI21ND2
-复合逻辑门</t>
+          <t>OAI21ND2</t>
         </is>
       </c>
       <c r="C604" s="3" t="inlineStr">
@@ -7624,8 +7472,7 @@
       <c r="A611" s="2" t="n"/>
       <c r="B611" s="2" t="inlineStr">
         <is>
-          <t>OAI21NR2
-复合逻辑门</t>
+          <t>OAI21NR2</t>
         </is>
       </c>
       <c r="C611" s="3" t="inlineStr">
@@ -7669,8 +7516,7 @@
       <c r="A615" s="10" t="n"/>
       <c r="B615" s="10" t="inlineStr">
         <is>
-          <t>OAI21OAI21
-复合逻辑门</t>
+          <t>OAI21OAI21</t>
         </is>
       </c>
       <c r="C615" s="11" t="n"/>
@@ -7684,8 +7530,7 @@
       <c r="A616" s="2" t="n"/>
       <c r="B616" s="2" t="inlineStr">
         <is>
-          <t>OAI22AOI21
-复合逻辑门</t>
+          <t>OAI22AOI21</t>
         </is>
       </c>
       <c r="C616" s="3" t="inlineStr">
@@ -7729,8 +7574,7 @@
       <c r="A620" s="2" t="n"/>
       <c r="B620" s="2" t="inlineStr">
         <is>
-          <t>OAI22INV
-复合逻辑门</t>
+          <t>OAI22INV</t>
         </is>
       </c>
       <c r="C620" s="3" t="inlineStr">
@@ -7754,8 +7598,7 @@
       <c r="A622" s="2" t="n"/>
       <c r="B622" s="2" t="inlineStr">
         <is>
-          <t>OAI22ND2
-复合逻辑门</t>
+          <t>OAI22ND2</t>
         </is>
       </c>
       <c r="C622" s="3" t="inlineStr">
@@ -7779,8 +7622,7 @@
       <c r="A624" s="2" t="n"/>
       <c r="B624" s="2" t="inlineStr">
         <is>
-          <t>OAI22NR2
-复合逻辑门</t>
+          <t>OAI22NR2</t>
         </is>
       </c>
       <c r="C624" s="3" t="inlineStr">
@@ -7804,8 +7646,7 @@
       <c r="A626" s="10" t="n"/>
       <c r="B626" s="10" t="inlineStr">
         <is>
-          <t>OAI22OAI21
-复合逻辑门</t>
+          <t>OAI22OAI21</t>
         </is>
       </c>
       <c r="C626" s="11" t="n"/>
@@ -7819,8 +7660,7 @@
       <c r="A627" s="2" t="n"/>
       <c r="B627" s="2" t="inlineStr">
         <is>
-          <t>OAOI211
-复合逻辑门</t>
+          <t>OAOI211</t>
         </is>
       </c>
       <c r="C627" s="8" t="inlineStr">
@@ -7858,8 +7698,7 @@
       <c r="A630" s="2" t="n"/>
       <c r="B630" s="2" t="inlineStr">
         <is>
-          <t>OIAI21
-复合逻辑门</t>
+          <t>OIAI21</t>
         </is>
       </c>
       <c r="C630" s="8" t="inlineStr">
@@ -7917,8 +7756,7 @@
       <c r="A635" s="2" t="n"/>
       <c r="B635" s="2" t="inlineStr">
         <is>
-          <t>W2AO22
-复合逻辑门</t>
+          <t>W2AO22</t>
         </is>
       </c>
       <c r="C635" s="3" t="n"/>
@@ -7942,8 +7780,7 @@
       <c r="A637" s="10" t="n"/>
       <c r="B637" s="10" t="inlineStr">
         <is>
-          <t>W2AOI22
-复合逻辑门</t>
+          <t>W2AOI22</t>
         </is>
       </c>
       <c r="C637" s="11" t="n"/>
@@ -7957,8 +7794,7 @@
       <c r="A638" s="10" t="n"/>
       <c r="B638" s="10" t="inlineStr">
         <is>
-          <t>WAN2OR2
-复合逻辑门</t>
+          <t>WAN2OR2</t>
         </is>
       </c>
       <c r="C638" s="11" t="n"/>
@@ -7972,8 +7808,7 @@
       <c r="A639" s="10" t="n"/>
       <c r="B639" s="10" t="inlineStr">
         <is>
-          <t>WAO21OA21
-复合逻辑门</t>
+          <t>WAO21OA21</t>
         </is>
       </c>
       <c r="C639" s="11" t="n"/>
@@ -7987,8 +7822,7 @@
       <c r="A640" s="10" t="n"/>
       <c r="B640" s="10" t="inlineStr">
         <is>
-          <t>WAO22OA22
-复合逻辑门</t>
+          <t>WAO22OA22</t>
         </is>
       </c>
       <c r="C640" s="11" t="n"/>
@@ -8002,8 +7836,7 @@
       <c r="A641" s="2" t="n"/>
       <c r="B641" s="2" t="inlineStr">
         <is>
-          <t>XNR2AOI21
-复合逻辑门</t>
+          <t>XNR2AOI21</t>
         </is>
       </c>
       <c r="C641" s="3" t="inlineStr">
@@ -8037,8 +7870,7 @@
       <c r="A644" s="2" t="n"/>
       <c r="B644" s="2" t="inlineStr">
         <is>
-          <t>XNR2AOI22
-复合逻辑门</t>
+          <t>XNR2AOI22</t>
         </is>
       </c>
       <c r="C644" s="3" t="inlineStr">
@@ -8082,8 +7914,7 @@
       <c r="A648" s="2" t="n"/>
       <c r="B648" s="2" t="inlineStr">
         <is>
-          <t>XNR2ND2
-复合逻辑门</t>
+          <t>XNR2ND2</t>
         </is>
       </c>
       <c r="C648" s="3" t="inlineStr">
@@ -8117,8 +7948,7 @@
       <c r="A651" s="2" t="n"/>
       <c r="B651" s="2" t="inlineStr">
         <is>
-          <t>XNR2NR2
-复合逻辑门</t>
+          <t>XNR2NR2</t>
         </is>
       </c>
       <c r="C651" s="3" t="inlineStr">
@@ -8142,8 +7972,7 @@
       <c r="A653" s="10" t="n"/>
       <c r="B653" s="10" t="inlineStr">
         <is>
-          <t>XNR2OAI21
-复合逻辑门</t>
+          <t>XNR2OAI21</t>
         </is>
       </c>
       <c r="C653" s="11" t="inlineStr">
@@ -8157,8 +7986,7 @@
       <c r="A654" s="2" t="n"/>
       <c r="B654" s="2" t="inlineStr">
         <is>
-          <t>XNR2OAI22
-复合逻辑门</t>
+          <t>XNR2OAI22</t>
         </is>
       </c>
       <c r="C654" s="3" t="inlineStr">
@@ -8202,8 +8030,7 @@
       <c r="A658" s="10" t="n"/>
       <c r="B658" s="10" t="inlineStr">
         <is>
-          <t>XNR2XNR2
-复合逻辑门</t>
+          <t>XNR2XNR2</t>
         </is>
       </c>
       <c r="C658" s="11" t="inlineStr">
@@ -8217,8 +8044,7 @@
       <c r="A659" s="10" t="n"/>
       <c r="B659" s="10" t="inlineStr">
         <is>
-          <t>XNR2XOR2
-复合逻辑门</t>
+          <t>XNR2XOR2</t>
         </is>
       </c>
       <c r="C659" s="11" t="inlineStr">
@@ -8232,8 +8058,7 @@
       <c r="A660" s="10" t="n"/>
       <c r="B660" s="10" t="inlineStr">
         <is>
-          <t>XOR2AOI21
-复合逻辑门</t>
+          <t>XOR2AOI21</t>
         </is>
       </c>
       <c r="C660" s="11" t="inlineStr">
@@ -8247,8 +8072,7 @@
       <c r="A661" s="2" t="n"/>
       <c r="B661" s="2" t="inlineStr">
         <is>
-          <t>XOR2AOI22
-复合逻辑门</t>
+          <t>XOR2AOI22</t>
         </is>
       </c>
       <c r="C661" s="3" t="inlineStr">
@@ -8302,8 +8126,7 @@
       <c r="A666" s="2" t="n"/>
       <c r="B666" s="2" t="inlineStr">
         <is>
-          <t>XOR2ND2
-复合逻辑门</t>
+          <t>XOR2ND2</t>
         </is>
       </c>
       <c r="C666" s="3" t="inlineStr">
@@ -8347,8 +8170,7 @@
       <c r="A670" s="2" t="n"/>
       <c r="B670" s="2" t="inlineStr">
         <is>
-          <t>XOR2NR2
-复合逻辑门</t>
+          <t>XOR2NR2</t>
         </is>
       </c>
       <c r="C670" s="3" t="inlineStr">
@@ -8382,8 +8204,7 @@
       <c r="A673" s="10" t="n"/>
       <c r="B673" s="10" t="inlineStr">
         <is>
-          <t>XOR2OAI21
-复合逻辑门</t>
+          <t>XOR2OAI21</t>
         </is>
       </c>
       <c r="C673" s="11" t="inlineStr">
@@ -8397,8 +8218,7 @@
       <c r="A674" s="2" t="n"/>
       <c r="B674" s="2" t="inlineStr">
         <is>
-          <t>XOR2OAI22
-复合逻辑门</t>
+          <t>XOR2OAI22</t>
         </is>
       </c>
       <c r="C674" s="3" t="inlineStr">
@@ -8452,8 +8272,7 @@
       <c r="A679" s="10" t="n"/>
       <c r="B679" s="10" t="inlineStr">
         <is>
-          <t>XOR2XNR2
-复合逻辑门</t>
+          <t>XOR2XNR2</t>
         </is>
       </c>
       <c r="C679" s="11" t="inlineStr">
@@ -8467,8 +8286,7 @@
       <c r="A680" s="10" t="n"/>
       <c r="B680" s="10" t="inlineStr">
         <is>
-          <t>XOR2XOR2
-复合逻辑门</t>
+          <t>XOR2XOR2</t>
         </is>
       </c>
       <c r="C680" s="11" t="inlineStr">
@@ -8486,8 +8304,7 @@
       </c>
       <c r="B681" s="2" t="inlineStr">
         <is>
-          <t>MCESNQSYN
-多比特同步器</t>
+          <t>MCESNQSYN</t>
         </is>
       </c>
       <c r="C681" s="3" t="n"/>
@@ -8525,8 +8342,7 @@
       </c>
       <c r="B684" s="2" t="inlineStr">
         <is>
-          <t>MB2SRLSDF
-多比特触发器</t>
+          <t>MB2SRLSDF</t>
         </is>
       </c>
       <c r="C684" s="3" t="inlineStr">
@@ -8590,8 +8406,7 @@
       <c r="A690" s="2" t="n"/>
       <c r="B690" s="2" t="inlineStr">
         <is>
-          <t>MB4SRLSDF
-多比特触发器</t>
+          <t>MB4SRLSDF</t>
         </is>
       </c>
       <c r="C690" s="3" t="inlineStr">
@@ -8659,8 +8474,7 @@
       </c>
       <c r="B696" s="2" t="inlineStr">
         <is>
-          <t>MB2LHCNQ
-多比特锁存器</t>
+          <t>MB2LHCNQ</t>
         </is>
       </c>
       <c r="C696" s="3" t="inlineStr">
@@ -8694,8 +8508,7 @@
       <c r="A699" s="2" t="n"/>
       <c r="B699" s="2" t="inlineStr">
         <is>
-          <t>MB2LHQ
-多比特锁存器</t>
+          <t>MB2LHQ</t>
         </is>
       </c>
       <c r="C699" s="3" t="inlineStr">
@@ -8739,8 +8552,7 @@
       <c r="A703" s="10" t="n"/>
       <c r="B703" s="10" t="inlineStr">
         <is>
-          <t>MB2LHSPCNQ
-多比特锁存器</t>
+          <t>MB2LHSPCNQ</t>
         </is>
       </c>
       <c r="C703" s="11" t="inlineStr">
@@ -8754,8 +8566,7 @@
       <c r="A704" s="2" t="n"/>
       <c r="B704" s="2" t="inlineStr">
         <is>
-          <t>MB2LNCNQ
-多比特锁存器</t>
+          <t>MB2LNCNQ</t>
         </is>
       </c>
       <c r="C704" s="3" t="inlineStr">
@@ -8779,8 +8590,7 @@
       <c r="A706" s="2" t="n"/>
       <c r="B706" s="2" t="inlineStr">
         <is>
-          <t>MB2LNQ
-多比特锁存器</t>
+          <t>MB2LNQ</t>
         </is>
       </c>
       <c r="C706" s="3" t="inlineStr">
@@ -8814,8 +8624,7 @@
       <c r="A709" s="10" t="n"/>
       <c r="B709" s="10" t="inlineStr">
         <is>
-          <t>MB2LNSPCNQ
-多比特锁存器</t>
+          <t>MB2LNSPCNQ</t>
         </is>
       </c>
       <c r="C709" s="11" t="inlineStr">
@@ -8829,8 +8638,7 @@
       <c r="A710" s="10" t="n"/>
       <c r="B710" s="10" t="inlineStr">
         <is>
-          <t>MB4LHQ
-多比特锁存器</t>
+          <t>MB4LHQ</t>
         </is>
       </c>
       <c r="C710" s="11" t="inlineStr">
@@ -8844,8 +8652,7 @@
       <c r="A711" s="10" t="n"/>
       <c r="B711" s="10" t="inlineStr">
         <is>
-          <t>MB4LNQ
-多比特锁存器</t>
+          <t>MB4LNQ</t>
         </is>
       </c>
       <c r="C711" s="11" t="inlineStr">
@@ -8859,8 +8666,7 @@
       <c r="A712" s="10" t="n"/>
       <c r="B712" s="10" t="inlineStr">
         <is>
-          <t>MCECNQ
-多比特锁存器</t>
+          <t>MCECNQ</t>
         </is>
       </c>
       <c r="C712" s="11" t="n"/>
@@ -8874,8 +8680,7 @@
       <c r="A713" s="2" t="n"/>
       <c r="B713" s="2" t="inlineStr">
         <is>
-          <t>MCESNQ
-多比特锁存器</t>
+          <t>MCESNQ</t>
         </is>
       </c>
       <c r="C713" s="3" t="n"/>
@@ -8913,8 +8718,7 @@
       </c>
       <c r="B716" s="10" t="inlineStr">
         <is>
-          <t>GMUX2
-多路选择器</t>
+          <t>GMUX2</t>
         </is>
       </c>
       <c r="C716" s="12" t="inlineStr">
@@ -8932,8 +8736,7 @@
       <c r="A717" s="2" t="n"/>
       <c r="B717" s="2" t="inlineStr">
         <is>
-          <t>MUX2
-多路选择器</t>
+          <t>MUX2</t>
         </is>
       </c>
       <c r="C717" s="8" t="inlineStr">
@@ -9001,8 +8804,7 @@
       <c r="A723" s="2" t="n"/>
       <c r="B723" s="2" t="inlineStr">
         <is>
-          <t>MUX3
-多路选择器</t>
+          <t>MUX3</t>
         </is>
       </c>
       <c r="C723" s="8" t="inlineStr">
@@ -9040,8 +8842,7 @@
       <c r="A726" s="2" t="n"/>
       <c r="B726" s="2" t="inlineStr">
         <is>
-          <t>MUX4
-多路选择器</t>
+          <t>MUX4</t>
         </is>
       </c>
       <c r="C726" s="3" t="inlineStr">
@@ -9075,8 +8876,7 @@
       <c r="A729" s="2" t="n"/>
       <c r="B729" s="2" t="inlineStr">
         <is>
-          <t>MUX8
-多路选择器</t>
+          <t>MUX8</t>
         </is>
       </c>
       <c r="C729" s="3" t="inlineStr">
@@ -9100,8 +8900,7 @@
       <c r="A731" s="2" t="n"/>
       <c r="B731" s="2" t="inlineStr">
         <is>
-          <t>MX2
-多路选择器</t>
+          <t>MX2</t>
         </is>
       </c>
       <c r="C731" s="3" t="n"/>
@@ -9139,8 +8938,7 @@
       </c>
       <c r="B734" s="10" t="inlineStr">
         <is>
-          <t>ANTENNA
-天线二极管</t>
+          <t>ANTENNA</t>
         </is>
       </c>
       <c r="C734" s="11" t="inlineStr">
@@ -9158,8 +8956,7 @@
       </c>
       <c r="B735" s="2" t="inlineStr">
         <is>
-          <t>DELA
-延时单元</t>
+          <t>DELA</t>
         </is>
       </c>
       <c r="C735" s="3" t="inlineStr">
@@ -9183,8 +8980,7 @@
       <c r="A737" s="2" t="n"/>
       <c r="B737" s="2" t="inlineStr">
         <is>
-          <t>DELB
-延时单元</t>
+          <t>DELB</t>
         </is>
       </c>
       <c r="C737" s="3" t="inlineStr">
@@ -9208,8 +9004,7 @@
       <c r="A739" s="10" t="n"/>
       <c r="B739" s="10" t="inlineStr">
         <is>
-          <t>DELC
-延时单元</t>
+          <t>DELC</t>
         </is>
       </c>
       <c r="C739" s="11" t="inlineStr">
@@ -9223,8 +9018,7 @@
       <c r="A740" s="2" t="n"/>
       <c r="B740" s="2" t="inlineStr">
         <is>
-          <t>DELD
-延时单元</t>
+          <t>DELD</t>
         </is>
       </c>
       <c r="C740" s="3" t="inlineStr">
@@ -9248,8 +9042,7 @@
       <c r="A742" s="2" t="n"/>
       <c r="B742" s="2" t="inlineStr">
         <is>
-          <t>DELE
-延时单元</t>
+          <t>DELE</t>
         </is>
       </c>
       <c r="C742" s="3" t="inlineStr">
@@ -9273,8 +9066,7 @@
       <c r="A744" s="2" t="n"/>
       <c r="B744" s="2" t="inlineStr">
         <is>
-          <t>DELF
-延时单元</t>
+          <t>DELF</t>
         </is>
       </c>
       <c r="C744" s="3" t="inlineStr">
@@ -9298,8 +9090,7 @@
       <c r="A746" s="10" t="n"/>
       <c r="B746" s="10" t="inlineStr">
         <is>
-          <t>DELG
-延时单元</t>
+          <t>DELG</t>
         </is>
       </c>
       <c r="C746" s="11" t="inlineStr">
@@ -9317,8 +9108,7 @@
       </c>
       <c r="B747" s="10" t="inlineStr">
         <is>
-          <t>GXOR2
-异或门</t>
+          <t>GXOR2</t>
         </is>
       </c>
       <c r="C747" s="11" t="inlineStr">
@@ -9332,8 +9122,7 @@
       <c r="A748" s="2" t="n"/>
       <c r="B748" s="2" t="inlineStr">
         <is>
-          <t>XOR2
-异或门</t>
+          <t>XOR2</t>
         </is>
       </c>
       <c r="C748" s="8" t="inlineStr">
@@ -9515,8 +9304,7 @@
       <c r="A765" s="2" t="n"/>
       <c r="B765" s="2" t="inlineStr">
         <is>
-          <t>XOR3
-异或门</t>
+          <t>XOR3</t>
         </is>
       </c>
       <c r="C765" s="8" t="inlineStr">
@@ -9594,8 +9382,7 @@
       <c r="A772" s="2" t="n"/>
       <c r="B772" s="2" t="inlineStr">
         <is>
-          <t>XOR4
-异或门</t>
+          <t>XOR4</t>
         </is>
       </c>
       <c r="C772" s="8" t="inlineStr">
@@ -9657,8 +9444,7 @@
       </c>
       <c r="B777" s="10" t="inlineStr">
         <is>
-          <t>BHD
-总线保持器</t>
+          <t>BHD</t>
         </is>
       </c>
       <c r="C777" s="12" t="inlineStr">
@@ -9680,8 +9466,7 @@
       </c>
       <c r="B778" s="10" t="inlineStr">
         <is>
-          <t>GOA21
-或与门</t>
+          <t>GOA21</t>
         </is>
       </c>
       <c r="C778" s="12" t="inlineStr">
@@ -9699,8 +9484,7 @@
       <c r="A779" s="10" t="n"/>
       <c r="B779" s="10" t="inlineStr">
         <is>
-          <t>GOA22
-或与门</t>
+          <t>GOA22</t>
         </is>
       </c>
       <c r="C779" s="12" t="inlineStr">
@@ -9718,8 +9502,7 @@
       <c r="A780" s="10" t="n"/>
       <c r="B780" s="10" t="inlineStr">
         <is>
-          <t>GOA31
-或与门</t>
+          <t>GOA31</t>
         </is>
       </c>
       <c r="C780" s="11" t="n"/>
@@ -9733,8 +9516,7 @@
       <c r="A781" s="10" t="n"/>
       <c r="B781" s="10" t="inlineStr">
         <is>
-          <t>GOA32
-或与门</t>
+          <t>GOA32</t>
         </is>
       </c>
       <c r="C781" s="11" t="n"/>
@@ -9748,8 +9530,7 @@
       <c r="A782" s="2" t="n"/>
       <c r="B782" s="2" t="inlineStr">
         <is>
-          <t>OA21
-或与门</t>
+          <t>OA21</t>
         </is>
       </c>
       <c r="C782" s="8" t="inlineStr">
@@ -9807,8 +9588,7 @@
       <c r="A787" s="2" t="n"/>
       <c r="B787" s="2" t="inlineStr">
         <is>
-          <t>OA211
-或与门</t>
+          <t>OA211</t>
         </is>
       </c>
       <c r="C787" s="3" t="inlineStr">
@@ -9872,8 +9652,7 @@
       <c r="A793" s="2" t="n"/>
       <c r="B793" s="2" t="inlineStr">
         <is>
-          <t>OA22
-或与门</t>
+          <t>OA22</t>
         </is>
       </c>
       <c r="C793" s="8" t="inlineStr">
@@ -9951,8 +9730,7 @@
       <c r="A800" s="2" t="n"/>
       <c r="B800" s="2" t="inlineStr">
         <is>
-          <t>OA222
-或与门</t>
+          <t>OA222</t>
         </is>
       </c>
       <c r="C800" s="3" t="inlineStr">
@@ -10006,8 +9784,7 @@
       <c r="A805" s="10" t="n"/>
       <c r="B805" s="10" t="inlineStr">
         <is>
-          <t>OA2222
-或与门</t>
+          <t>OA2222</t>
         </is>
       </c>
       <c r="C805" s="11" t="inlineStr">
@@ -10025,8 +9802,7 @@
       </c>
       <c r="B806" s="2" t="inlineStr">
         <is>
-          <t>GOAI21
-或与非门</t>
+          <t>GOAI21</t>
         </is>
       </c>
       <c r="C806" s="3" t="inlineStr">
@@ -10050,8 +9826,7 @@
       <c r="A808" s="10" t="n"/>
       <c r="B808" s="10" t="inlineStr">
         <is>
-          <t>GOAI211
-或与非门</t>
+          <t>GOAI211</t>
         </is>
       </c>
       <c r="C808" s="11" t="n"/>
@@ -10065,8 +9840,7 @@
       <c r="A809" s="2" t="n"/>
       <c r="B809" s="2" t="inlineStr">
         <is>
-          <t>GOAI22
-或与非门</t>
+          <t>GOAI22</t>
         </is>
       </c>
       <c r="C809" s="8" t="inlineStr">
@@ -10094,8 +9868,7 @@
       <c r="A811" s="10" t="n"/>
       <c r="B811" s="10" t="inlineStr">
         <is>
-          <t>GOAI31
-或与非门</t>
+          <t>GOAI31</t>
         </is>
       </c>
       <c r="C811" s="11" t="n"/>
@@ -10109,8 +9882,7 @@
       <c r="A812" s="10" t="n"/>
       <c r="B812" s="10" t="inlineStr">
         <is>
-          <t>GOAI32
-或与非门</t>
+          <t>GOAI32</t>
         </is>
       </c>
       <c r="C812" s="11" t="n"/>
@@ -10124,8 +9896,7 @@
       <c r="A813" s="10" t="n"/>
       <c r="B813" s="10" t="inlineStr">
         <is>
-          <t>GOAI33
-或与非门</t>
+          <t>GOAI33</t>
         </is>
       </c>
       <c r="C813" s="11" t="n"/>
@@ -10139,8 +9910,7 @@
       <c r="A814" s="2" t="n"/>
       <c r="B814" s="2" t="inlineStr">
         <is>
-          <t>OAI21
-或与非门</t>
+          <t>OAI21</t>
         </is>
       </c>
       <c r="C814" s="3" t="inlineStr">
@@ -10364,8 +10134,7 @@
       <c r="A836" s="2" t="n"/>
       <c r="B836" s="2" t="inlineStr">
         <is>
-          <t>OAI211
-或与非门</t>
+          <t>OAI211</t>
         </is>
       </c>
       <c r="C836" s="3" t="inlineStr">
@@ -10509,8 +10278,7 @@
       <c r="A850" s="2" t="n"/>
       <c r="B850" s="2" t="inlineStr">
         <is>
-          <t>OAI2111
-或与非门</t>
+          <t>OAI2111</t>
         </is>
       </c>
       <c r="C850" s="3" t="inlineStr">
@@ -10534,8 +10302,7 @@
       <c r="A852" s="2" t="n"/>
       <c r="B852" s="2" t="inlineStr">
         <is>
-          <t>OAI22
-或与非门</t>
+          <t>OAI22</t>
         </is>
       </c>
       <c r="C852" s="8" t="inlineStr">
@@ -10667,8 +10434,7 @@
       <c r="A864" s="2" t="n"/>
       <c r="B864" s="2" t="inlineStr">
         <is>
-          <t>OAI221
-或与非门</t>
+          <t>OAI221</t>
         </is>
       </c>
       <c r="C864" s="8" t="inlineStr">
@@ -10730,8 +10496,7 @@
       <c r="A869" s="2" t="n"/>
       <c r="B869" s="2" t="inlineStr">
         <is>
-          <t>OAI2211
-或与非门</t>
+          <t>OAI2211</t>
         </is>
       </c>
       <c r="C869" s="3" t="inlineStr">
@@ -10755,8 +10520,7 @@
       <c r="A871" s="2" t="n"/>
       <c r="B871" s="2" t="inlineStr">
         <is>
-          <t>OAI222
-或与非门</t>
+          <t>OAI222</t>
         </is>
       </c>
       <c r="C871" s="8" t="inlineStr">
@@ -10808,8 +10572,7 @@
       <c r="A875" s="2" t="n"/>
       <c r="B875" s="2" t="inlineStr">
         <is>
-          <t>OAI2221
-或与非门</t>
+          <t>OAI2221</t>
         </is>
       </c>
       <c r="C875" s="3" t="inlineStr">
@@ -10833,8 +10596,7 @@
       <c r="A877" s="2" t="n"/>
       <c r="B877" s="2" t="inlineStr">
         <is>
-          <t>OAI2222
-或与非门</t>
+          <t>OAI2222</t>
         </is>
       </c>
       <c r="C877" s="3" t="inlineStr">
@@ -10928,8 +10690,7 @@
       <c r="A886" s="2" t="n"/>
       <c r="B886" s="2" t="inlineStr">
         <is>
-          <t>OAI31
-或与非门</t>
+          <t>OAI31</t>
         </is>
       </c>
       <c r="C886" s="3" t="inlineStr">
@@ -10983,8 +10744,7 @@
       <c r="A891" s="2" t="n"/>
       <c r="B891" s="2" t="inlineStr">
         <is>
-          <t>OAI311
-或与非门</t>
+          <t>OAI311</t>
         </is>
       </c>
       <c r="C891" s="8" t="inlineStr">
@@ -11042,8 +10802,7 @@
       <c r="A896" s="2" t="n"/>
       <c r="B896" s="2" t="inlineStr">
         <is>
-          <t>OAI32
-或与非门</t>
+          <t>OAI32</t>
         </is>
       </c>
       <c r="C896" s="8" t="inlineStr">
@@ -11101,8 +10860,7 @@
       <c r="A901" s="2" t="n"/>
       <c r="B901" s="2" t="inlineStr">
         <is>
-          <t>OAI321
-或与非门</t>
+          <t>OAI321</t>
         </is>
       </c>
       <c r="C901" s="3" t="inlineStr">
@@ -11146,8 +10904,7 @@
       <c r="A905" s="2" t="n"/>
       <c r="B905" s="2" t="inlineStr">
         <is>
-          <t>OAI33
-或与非门</t>
+          <t>OAI33</t>
         </is>
       </c>
       <c r="C905" s="3" t="inlineStr">
@@ -11185,8 +10942,7 @@
       </c>
       <c r="B908" s="10" t="inlineStr">
         <is>
-          <t>GOR2
-或门</t>
+          <t>GOR2</t>
         </is>
       </c>
       <c r="C908" s="12" t="inlineStr">
@@ -11204,8 +10960,7 @@
       <c r="A909" s="10" t="n"/>
       <c r="B909" s="10" t="inlineStr">
         <is>
-          <t>GOR3
-或门</t>
+          <t>GOR3</t>
         </is>
       </c>
       <c r="C909" s="11" t="inlineStr">
@@ -11219,8 +10974,7 @@
       <c r="A910" s="10" t="n"/>
       <c r="B910" s="10" t="inlineStr">
         <is>
-          <t>GOR4
-或门</t>
+          <t>GOR4</t>
         </is>
       </c>
       <c r="C910" s="12" t="inlineStr">
@@ -11238,8 +10992,7 @@
       <c r="A911" s="2" t="n"/>
       <c r="B911" s="2" t="inlineStr">
         <is>
-          <t>OR2
-或门</t>
+          <t>OR2</t>
         </is>
       </c>
       <c r="C911" s="8" t="inlineStr">
@@ -11525,8 +11278,7 @@
       <c r="A938" s="2" t="n"/>
       <c r="B938" s="2" t="inlineStr">
         <is>
-          <t>OR3
-或门</t>
+          <t>OR3</t>
         </is>
       </c>
       <c r="C938" s="8" t="inlineStr">
@@ -11620,8 +11372,7 @@
       <c r="A945" s="2" t="n"/>
       <c r="B945" s="2" t="inlineStr">
         <is>
-          <t>OR4
-或门</t>
+          <t>OR4</t>
         </is>
       </c>
       <c r="C945" s="8" t="inlineStr">
@@ -11723,8 +11474,7 @@
       </c>
       <c r="B954" s="2" t="inlineStr">
         <is>
-          <t>GNR2
-或非门</t>
+          <t>GNR2</t>
         </is>
       </c>
       <c r="C954" s="3" t="inlineStr">
@@ -11748,8 +11498,7 @@
       <c r="A956" s="10" t="n"/>
       <c r="B956" s="10" t="inlineStr">
         <is>
-          <t>GNR3
-或非门</t>
+          <t>GNR3</t>
         </is>
       </c>
       <c r="C956" s="11" t="inlineStr">
@@ -11763,8 +11512,7 @@
       <c r="A957" s="2" t="n"/>
       <c r="B957" s="2" t="inlineStr">
         <is>
-          <t>GNR4
-或非门</t>
+          <t>GNR4</t>
         </is>
       </c>
       <c r="C957" s="3" t="inlineStr">
@@ -11788,8 +11536,7 @@
       <c r="A959" s="2" t="n"/>
       <c r="B959" s="2" t="inlineStr">
         <is>
-          <t>IINR3
-或非门</t>
+          <t>IINR3</t>
         </is>
       </c>
       <c r="C959" s="8" t="inlineStr">
@@ -11857,8 +11604,7 @@
       <c r="A965" s="2" t="n"/>
       <c r="B965" s="2" t="inlineStr">
         <is>
-          <t>IINR4
-或非门</t>
+          <t>IINR4</t>
         </is>
       </c>
       <c r="C965" s="3" t="inlineStr">
@@ -11902,8 +11648,7 @@
       <c r="A969" s="2" t="n"/>
       <c r="B969" s="2" t="inlineStr">
         <is>
-          <t>INR2
-或非门</t>
+          <t>INR2</t>
         </is>
       </c>
       <c r="C969" s="8" t="inlineStr">
@@ -12041,8 +11786,7 @@
       <c r="A982" s="2" t="n"/>
       <c r="B982" s="2" t="inlineStr">
         <is>
-          <t>INR3
-或非门</t>
+          <t>INR3</t>
         </is>
       </c>
       <c r="C982" s="8" t="inlineStr">
@@ -12134,8 +11878,7 @@
       <c r="A990" s="2" t="n"/>
       <c r="B990" s="2" t="inlineStr">
         <is>
-          <t>INR4
-或非门</t>
+          <t>INR4</t>
         </is>
       </c>
       <c r="C990" s="8" t="inlineStr">
@@ -12177,8 +11920,7 @@
       <c r="A993" s="2" t="n"/>
       <c r="B993" s="2" t="inlineStr">
         <is>
-          <t>NR2
-或非门</t>
+          <t>NR2</t>
         </is>
       </c>
       <c r="C993" s="8" t="inlineStr">
@@ -12736,8 +12478,7 @@
       <c r="A1048" s="2" t="n"/>
       <c r="B1048" s="2" t="inlineStr">
         <is>
-          <t>NR3
-或非门</t>
+          <t>NR3</t>
         </is>
       </c>
       <c r="C1048" s="8" t="inlineStr">
@@ -12875,8 +12616,7 @@
       <c r="A1061" s="2" t="n"/>
       <c r="B1061" s="2" t="inlineStr">
         <is>
-          <t>NR4
-或非门</t>
+          <t>NR4</t>
         </is>
       </c>
       <c r="C1061" s="3" t="inlineStr">
@@ -12994,8 +12734,7 @@
       </c>
       <c r="B1072" s="2" t="inlineStr">
         <is>
-          <t>GSDF
-扫描触发器</t>
+          <t>GSDF</t>
         </is>
       </c>
       <c r="C1072" s="8" t="inlineStr">
@@ -13033,8 +12772,7 @@
       <c r="A1075" s="2" t="n"/>
       <c r="B1075" s="2" t="inlineStr">
         <is>
-          <t>RSDF
-扫描触发器</t>
+          <t>RSDF</t>
         </is>
       </c>
       <c r="C1075" s="3" t="n"/>
@@ -13078,8 +12816,7 @@
       <c r="A1079" s="10" t="n"/>
       <c r="B1079" s="10" t="inlineStr">
         <is>
-          <t>SD2FF
-扫描触发器</t>
+          <t>SD2FF</t>
         </is>
       </c>
       <c r="C1079" s="11" t="n"/>
@@ -13093,8 +12830,7 @@
       <c r="A1080" s="2" t="n"/>
       <c r="B1080" s="2" t="inlineStr">
         <is>
-          <t>SDF
-扫描触发器</t>
+          <t>SDF</t>
         </is>
       </c>
       <c r="C1080" s="3" t="inlineStr">
@@ -13468,8 +13204,7 @@
       <c r="A1117" s="2" t="n"/>
       <c r="B1117" s="2" t="inlineStr">
         <is>
-          <t>SDFF
-扫描触发器</t>
+          <t>SDFF</t>
         </is>
       </c>
       <c r="C1117" s="3" t="n"/>
@@ -13573,8 +13308,7 @@
       <c r="A1127" s="2" t="n"/>
       <c r="B1127" s="2" t="inlineStr">
         <is>
-          <t>SEDF
-扫描触发器</t>
+          <t>SEDF</t>
         </is>
       </c>
       <c r="C1127" s="3" t="inlineStr">
@@ -13618,8 +13352,7 @@
       <c r="A1131" s="2" t="n"/>
       <c r="B1131" s="2" t="inlineStr">
         <is>
-          <t>Y2SDF
-扫描触发器</t>
+          <t>Y2SDF</t>
         </is>
       </c>
       <c r="C1131" s="3" t="inlineStr">
@@ -13653,8 +13386,7 @@
       <c r="A1134" s="10" t="n"/>
       <c r="B1134" s="10" t="inlineStr">
         <is>
-          <t>Y2SDFF
-扫描触发器</t>
+          <t>Y2SDFF</t>
         </is>
       </c>
       <c r="C1134" s="11" t="n"/>
@@ -13668,8 +13400,7 @@
       <c r="A1135" s="2" t="n"/>
       <c r="B1135" s="2" t="inlineStr">
         <is>
-          <t>Y3SDF
-扫描触发器</t>
+          <t>Y3SDF</t>
         </is>
       </c>
       <c r="C1135" s="3" t="inlineStr">
@@ -13703,8 +13434,7 @@
       <c r="A1138" s="10" t="n"/>
       <c r="B1138" s="10" t="inlineStr">
         <is>
-          <t>Y3SDFF
-扫描触发器</t>
+          <t>Y3SDFF</t>
         </is>
       </c>
       <c r="C1138" s="11" t="n"/>
@@ -13718,8 +13448,7 @@
       <c r="A1139" s="2" t="n"/>
       <c r="B1139" s="2" t="inlineStr">
         <is>
-          <t>YSDF
-扫描触发器</t>
+          <t>YSDF</t>
         </is>
       </c>
       <c r="C1139" s="3" t="inlineStr">
@@ -13757,8 +13486,7 @@
       </c>
       <c r="B1142" s="2" t="inlineStr">
         <is>
-          <t>CKAN2
-时钟与门</t>
+          <t>CKAN2</t>
         </is>
       </c>
       <c r="C1142" s="8" t="inlineStr">
@@ -13834,8 +13562,7 @@
       </c>
       <c r="B1148" s="2" t="inlineStr">
         <is>
-          <t>CKND2
-时钟与非门</t>
+          <t>CKND2</t>
         </is>
       </c>
       <c r="C1148" s="3" t="inlineStr">
@@ -13903,8 +13630,7 @@
       </c>
       <c r="B1154" s="2" t="inlineStr">
         <is>
-          <t>DCCKN
-时钟单元</t>
+          <t>DCCKN</t>
         </is>
       </c>
       <c r="C1154" s="3" t="inlineStr">
@@ -13932,8 +13658,7 @@
       </c>
       <c r="B1156" s="2" t="inlineStr">
         <is>
-          <t>CKMUX2
-时钟多路选择器</t>
+          <t>CKMUX2</t>
         </is>
       </c>
       <c r="C1156" s="8" t="inlineStr">
@@ -14019,8 +13744,7 @@
       </c>
       <c r="B1163" s="2" t="inlineStr">
         <is>
-          <t>CKXOR2
-时钟异或门</t>
+          <t>CKXOR2</t>
         </is>
       </c>
       <c r="C1163" s="8" t="inlineStr">
@@ -14082,8 +13806,7 @@
       </c>
       <c r="B1168" s="2" t="inlineStr">
         <is>
-          <t>CKOR2
-时钟或门</t>
+          <t>CKOR2</t>
         </is>
       </c>
       <c r="C1168" s="8" t="inlineStr">
@@ -14143,8 +13866,7 @@
       </c>
       <c r="B1172" s="2" t="inlineStr">
         <is>
-          <t>CKNR2
-时钟或非门</t>
+          <t>CKNR2</t>
         </is>
       </c>
       <c r="C1172" s="8" t="inlineStr">
@@ -14214,8 +13936,7 @@
       </c>
       <c r="B1177" s="2" t="inlineStr">
         <is>
-          <t>CKB
-时钟缓冲/反相</t>
+          <t>CKB</t>
         </is>
       </c>
       <c r="C1177" s="3" t="inlineStr">
@@ -14239,8 +13960,7 @@
       <c r="A1179" s="2" t="n"/>
       <c r="B1179" s="2" t="inlineStr">
         <is>
-          <t>CKN
-时钟缓冲/反相</t>
+          <t>CKN</t>
         </is>
       </c>
       <c r="C1179" s="3" t="inlineStr">
@@ -14264,8 +13984,7 @@
       <c r="A1181" s="2" t="n"/>
       <c r="B1181" s="2" t="inlineStr">
         <is>
-          <t>DCCKB
-时钟缓冲/反相</t>
+          <t>DCCKB</t>
         </is>
       </c>
       <c r="C1181" s="3" t="inlineStr">
@@ -14293,8 +14012,7 @@
       </c>
       <c r="B1183" s="2" t="inlineStr">
         <is>
-          <t>CKLHQ
-时钟锁存器</t>
+          <t>CKLHQ</t>
         </is>
       </c>
       <c r="C1183" s="3" t="inlineStr">
@@ -14318,8 +14036,7 @@
       <c r="A1185" s="10" t="n"/>
       <c r="B1185" s="10" t="inlineStr">
         <is>
-          <t>CKLNCNQ
-时钟锁存器</t>
+          <t>CKLNCNQ</t>
         </is>
       </c>
       <c r="C1185" s="11" t="inlineStr">
@@ -14333,8 +14050,7 @@
       <c r="A1186" s="2" t="n"/>
       <c r="B1186" s="2" t="inlineStr">
         <is>
-          <t>CKLNQ
-时钟锁存器</t>
+          <t>CKLNQ</t>
         </is>
       </c>
       <c r="C1186" s="3" t="inlineStr">
@@ -14368,8 +14084,7 @@
       <c r="A1189" s="10" t="n"/>
       <c r="B1189" s="10" t="inlineStr">
         <is>
-          <t>GCKLNQ
-时钟锁存器</t>
+          <t>GCKLNQ</t>
         </is>
       </c>
       <c r="C1189" s="11" t="inlineStr">
@@ -14387,8 +14102,7 @@
       </c>
       <c r="B1190" s="10" t="inlineStr">
         <is>
-          <t>INVPAD
-焊盘反相器</t>
+          <t>INVPAD</t>
         </is>
       </c>
       <c r="C1190" s="11" t="inlineStr">
@@ -14406,8 +14120,7 @@
       </c>
       <c r="B1191" s="2" t="inlineStr">
         <is>
-          <t>CKLVLLH
-电平转换器</t>
+          <t>CKLVLLH</t>
         </is>
       </c>
       <c r="C1191" s="3" t="inlineStr">
@@ -14471,8 +14184,7 @@
       <c r="A1197" s="10" t="n"/>
       <c r="B1197" s="10" t="inlineStr">
         <is>
-          <t>CKLVU
-电平转换器</t>
+          <t>CKLVU</t>
         </is>
       </c>
       <c r="C1197" s="11" t="n"/>
@@ -14486,8 +14198,7 @@
       <c r="A1198" s="2" t="n"/>
       <c r="B1198" s="2" t="inlineStr">
         <is>
-          <t>LVLHL
-电平转换器</t>
+          <t>LVLHL</t>
         </is>
       </c>
       <c r="C1198" s="3" t="inlineStr">
@@ -14561,8 +14272,7 @@
       <c r="A1205" s="2" t="n"/>
       <c r="B1205" s="2" t="inlineStr">
         <is>
-          <t>LVLLH
-电平转换器</t>
+          <t>LVLLH</t>
         </is>
       </c>
       <c r="C1205" s="3" t="inlineStr">
@@ -14746,8 +14456,7 @@
       <c r="A1223" s="2" t="n"/>
       <c r="B1223" s="2" t="inlineStr">
         <is>
-          <t>LVU
-电平转换器</t>
+          <t>LVU</t>
         </is>
       </c>
       <c r="C1223" s="3" t="n"/>
@@ -14831,8 +14540,7 @@
       <c r="A1231" s="2" t="n"/>
       <c r="B1231" s="2" t="inlineStr">
         <is>
-          <t>LVUAN2
-电平转换器</t>
+          <t>LVUAN2</t>
         </is>
       </c>
       <c r="C1231" s="3" t="n"/>
@@ -14876,8 +14584,7 @@
       <c r="A1235" s="2" t="n"/>
       <c r="B1235" s="2" t="inlineStr">
         <is>
-          <t>LVUOR2
-电平转换器</t>
+          <t>LVUOR2</t>
         </is>
       </c>
       <c r="C1235" s="3" t="n"/>
@@ -14935,8 +14642,7 @@
       </c>
       <c r="B1240" s="10" t="inlineStr">
         <is>
-          <t>APTIEH
-电平钳位</t>
+          <t>APTIEH</t>
         </is>
       </c>
       <c r="C1240" s="12" t="inlineStr">
@@ -14954,8 +14660,7 @@
       <c r="A1241" s="10" t="n"/>
       <c r="B1241" s="10" t="inlineStr">
         <is>
-          <t>APTIEL
-电平钳位</t>
+          <t>APTIEL</t>
         </is>
       </c>
       <c r="C1241" s="11" t="inlineStr">
@@ -14969,8 +14674,7 @@
       <c r="A1242" s="10" t="n"/>
       <c r="B1242" s="10" t="inlineStr">
         <is>
-          <t>GTIEH
-电平钳位</t>
+          <t>GTIEH</t>
         </is>
       </c>
       <c r="C1242" s="11" t="inlineStr">
@@ -14984,8 +14688,7 @@
       <c r="A1243" s="10" t="n"/>
       <c r="B1243" s="10" t="inlineStr">
         <is>
-          <t>GTIEL
-电平钳位</t>
+          <t>GTIEL</t>
         </is>
       </c>
       <c r="C1243" s="11" t="inlineStr">
@@ -14999,8 +14702,7 @@
       <c r="A1244" s="10" t="n"/>
       <c r="B1244" s="10" t="inlineStr">
         <is>
-          <t>TIEH
-电平钳位</t>
+          <t>TIEH</t>
         </is>
       </c>
       <c r="C1244" s="11" t="inlineStr">
@@ -15014,8 +14716,7 @@
       <c r="A1245" s="10" t="n"/>
       <c r="B1245" s="10" t="inlineStr">
         <is>
-          <t>TIEL
-电平钳位</t>
+          <t>TIEL</t>
         </is>
       </c>
       <c r="C1245" s="12" t="inlineStr">
@@ -15037,8 +14738,7 @@
       </c>
       <c r="B1246" s="2" t="inlineStr">
         <is>
-          <t>APBUF
-缓冲器</t>
+          <t>APBUF</t>
         </is>
       </c>
       <c r="C1246" s="3" t="inlineStr">
@@ -15062,8 +14762,7 @@
       <c r="A1248" s="2" t="n"/>
       <c r="B1248" s="2" t="inlineStr">
         <is>
-          <t>BUF
-缓冲器</t>
+          <t>BUF</t>
         </is>
       </c>
       <c r="C1248" s="3" t="inlineStr">
@@ -15117,8 +14816,7 @@
       <c r="A1253" s="2" t="n"/>
       <c r="B1253" s="2" t="inlineStr">
         <is>
-          <t>GBUFF
-缓冲器</t>
+          <t>GBUFF</t>
         </is>
       </c>
       <c r="C1253" s="3" t="inlineStr">
@@ -15176,8 +14874,7 @@
       </c>
       <c r="B1258" s="2" t="inlineStr">
         <is>
-          <t>BENC
-编码器</t>
+          <t>BENC</t>
         </is>
       </c>
       <c r="C1258" s="3" t="n"/>
@@ -15211,8 +14908,7 @@
       <c r="A1261" s="10" t="n"/>
       <c r="B1261" s="10" t="inlineStr">
         <is>
-          <t>BENCGRF
-编码器</t>
+          <t>BENCGRF</t>
         </is>
       </c>
       <c r="C1261" s="11" t="n"/>
@@ -15230,8 +14926,7 @@
       </c>
       <c r="B1262" s="2" t="inlineStr">
         <is>
-          <t>BML
-辅助单元</t>
+          <t>BML</t>
         </is>
       </c>
       <c r="C1262" s="3" t="n"/>
@@ -15269,8 +14964,7 @@
       </c>
       <c r="B1265" s="2" t="inlineStr">
         <is>
-          <t>BOUNDARY
-边界/版图单元</t>
+          <t>BOUNDARY</t>
         </is>
       </c>
       <c r="C1265" s="8" t="inlineStr">
@@ -15526,8 +15220,7 @@
       <c r="A1287" s="2" t="n"/>
       <c r="B1287" s="2" t="inlineStr">
         <is>
-          <t>HDDICWY
-边界/版图单元</t>
+          <t>HDDICWY</t>
         </is>
       </c>
       <c r="C1287" s="3" t="n"/>
@@ -15551,8 +15244,7 @@
       <c r="A1289" s="2" t="n"/>
       <c r="B1289" s="2" t="inlineStr">
         <is>
-          <t>HDDID
-边界/版图单元</t>
+          <t>HDDID</t>
         </is>
       </c>
       <c r="C1289" s="3" t="inlineStr">
@@ -15580,8 +15272,7 @@
       </c>
       <c r="B1291" s="2" t="inlineStr">
         <is>
-          <t>FCICO
-进位逻辑</t>
+          <t>FCICO</t>
         </is>
       </c>
       <c r="C1291" s="3" t="inlineStr">
@@ -15605,8 +15296,7 @@
       <c r="A1293" s="10" t="n"/>
       <c r="B1293" s="10" t="inlineStr">
         <is>
-          <t>FCICON
-进位逻辑</t>
+          <t>FCICON</t>
         </is>
       </c>
       <c r="C1293" s="11" t="inlineStr">
@@ -15620,8 +15310,7 @@
       <c r="A1294" s="2" t="n"/>
       <c r="B1294" s="2" t="inlineStr">
         <is>
-          <t>FCIS
-进位逻辑</t>
+          <t>FCIS</t>
         </is>
       </c>
       <c r="C1294" s="3" t="inlineStr">
@@ -15645,8 +15334,7 @@
       <c r="A1296" s="2" t="n"/>
       <c r="B1296" s="2" t="inlineStr">
         <is>
-          <t>FCISN
-进位逻辑</t>
+          <t>FCISN</t>
         </is>
       </c>
       <c r="C1296" s="3" t="inlineStr">
@@ -15670,8 +15358,7 @@
       <c r="A1298" s="10" t="n"/>
       <c r="B1298" s="10" t="inlineStr">
         <is>
-          <t>FCONSN
-进位逻辑</t>
+          <t>FCONSN</t>
         </is>
       </c>
       <c r="C1298" s="11" t="inlineStr">
@@ -15685,8 +15372,7 @@
       <c r="A1299" s="10" t="n"/>
       <c r="B1299" s="10" t="inlineStr">
         <is>
-          <t>FCSICON
-进位逻辑</t>
+          <t>FCSICON</t>
         </is>
       </c>
       <c r="C1299" s="11" t="inlineStr">
@@ -15700,8 +15386,7 @@
       <c r="A1300" s="2" t="n"/>
       <c r="B1300" s="2" t="inlineStr">
         <is>
-          <t>FIICON
-进位逻辑</t>
+          <t>FIICON</t>
         </is>
       </c>
       <c r="C1300" s="3" t="inlineStr">
@@ -15729,8 +15414,7 @@
       </c>
       <c r="B1302" s="10" t="inlineStr">
         <is>
-          <t>GLAHQ
-锁存器</t>
+          <t>GLAHQ</t>
         </is>
       </c>
       <c r="C1302" s="11" t="n"/>
@@ -15744,8 +15428,7 @@
       <c r="A1303" s="10" t="n"/>
       <c r="B1303" s="10" t="inlineStr">
         <is>
-          <t>GLAHRNQ
-锁存器</t>
+          <t>GLAHRNQ</t>
         </is>
       </c>
       <c r="C1303" s="11" t="n"/>
@@ -15759,8 +15442,7 @@
       <c r="A1304" s="10" t="n"/>
       <c r="B1304" s="10" t="inlineStr">
         <is>
-          <t>GLHCNQ
-锁存器</t>
+          <t>GLHCNQ</t>
         </is>
       </c>
       <c r="C1304" s="11" t="inlineStr">
@@ -15774,8 +15456,7 @@
       <c r="A1305" s="10" t="n"/>
       <c r="B1305" s="10" t="inlineStr">
         <is>
-          <t>GLHQ
-锁存器</t>
+          <t>GLHQ</t>
         </is>
       </c>
       <c r="C1305" s="11" t="inlineStr">
@@ -15789,8 +15470,7 @@
       <c r="A1306" s="10" t="n"/>
       <c r="B1306" s="10" t="inlineStr">
         <is>
-          <t>GLNCNQ
-锁存器</t>
+          <t>GLNCNQ</t>
         </is>
       </c>
       <c r="C1306" s="11" t="inlineStr">
@@ -15804,8 +15484,7 @@
       <c r="A1307" s="10" t="n"/>
       <c r="B1307" s="10" t="inlineStr">
         <is>
-          <t>GLNQ
-锁存器</t>
+          <t>GLNQ</t>
         </is>
       </c>
       <c r="C1307" s="11" t="inlineStr">
@@ -15819,8 +15498,7 @@
       <c r="A1308" s="10" t="n"/>
       <c r="B1308" s="10" t="inlineStr">
         <is>
-          <t>LHCNQ
-锁存器</t>
+          <t>LHCNQ</t>
         </is>
       </c>
       <c r="C1308" s="11" t="inlineStr">
@@ -15834,8 +15512,7 @@
       <c r="A1309" s="10" t="n"/>
       <c r="B1309" s="10" t="inlineStr">
         <is>
-          <t>LHCSNQ
-锁存器</t>
+          <t>LHCSNQ</t>
         </is>
       </c>
       <c r="C1309" s="11" t="inlineStr">
@@ -15849,8 +15526,7 @@
       <c r="A1310" s="2" t="n"/>
       <c r="B1310" s="2" t="inlineStr">
         <is>
-          <t>LHQ
-锁存器</t>
+          <t>LHQ</t>
         </is>
       </c>
       <c r="C1310" s="3" t="inlineStr">
@@ -15874,8 +15550,7 @@
       <c r="A1312" s="2" t="n"/>
       <c r="B1312" s="2" t="inlineStr">
         <is>
-          <t>LHSNQ
-锁存器</t>
+          <t>LHSNQ</t>
         </is>
       </c>
       <c r="C1312" s="3" t="inlineStr">
@@ -15899,8 +15574,7 @@
       <c r="A1314" s="10" t="n"/>
       <c r="B1314" s="10" t="inlineStr">
         <is>
-          <t>LNCNQ
-锁存器</t>
+          <t>LNCNQ</t>
         </is>
       </c>
       <c r="C1314" s="11" t="inlineStr">
@@ -15914,8 +15588,7 @@
       <c r="A1315" s="10" t="n"/>
       <c r="B1315" s="10" t="inlineStr">
         <is>
-          <t>LNCSNQ
-锁存器</t>
+          <t>LNCSNQ</t>
         </is>
       </c>
       <c r="C1315" s="12" t="inlineStr">
@@ -15933,8 +15606,7 @@
       <c r="A1316" s="10" t="n"/>
       <c r="B1316" s="10" t="inlineStr">
         <is>
-          <t>LNQ
-锁存器</t>
+          <t>LNQ</t>
         </is>
       </c>
       <c r="C1316" s="11" t="inlineStr">
@@ -15948,8 +15620,7 @@
       <c r="A1317" s="2" t="n"/>
       <c r="B1317" s="2" t="inlineStr">
         <is>
-          <t>LNSNQ
-锁存器</t>
+          <t>LNSNQ</t>
         </is>
       </c>
       <c r="C1317" s="3" t="inlineStr">
@@ -15977,8 +15648,7 @@
       </c>
       <c r="B1319" s="2" t="inlineStr">
         <is>
-          <t>GCKNQ
-门控时钟</t>
+          <t>GCKNQ</t>
         </is>
       </c>
       <c r="C1319" s="3" t="n"/>
@@ -16016,8 +15686,7 @@
       </c>
       <c r="B1322" s="2" t="inlineStr">
         <is>
-          <t>TAPCELL
-阱敲击单元</t>
+          <t>TAPCELL</t>
         </is>
       </c>
       <c r="C1322" s="8" t="inlineStr">
@@ -16049,8 +15718,7 @@
       </c>
       <c r="B1324" s="2" t="inlineStr">
         <is>
-          <t>ISOH
-隔离单元</t>
+          <t>ISOH</t>
         </is>
       </c>
       <c r="C1324" s="3" t="inlineStr">
@@ -16104,8 +15772,7 @@
       <c r="A1329" s="2" t="n"/>
       <c r="B1329" s="2" t="inlineStr">
         <is>
-          <t>ISOL
-隔离单元</t>
+          <t>ISOL</t>
         </is>
       </c>
       <c r="C1329" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Refine B-family merges per structure/LH-LN/Y-scan rules.
Compound keys ignore 21/22 digits and group by boolean skeleton;
latches only split LH vs LN; scan FFs only split Y vs non-Y.

Co-authored-by: EsaLongs <EsaLongs@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/preview/NP1PP_vs_C1Y_preview.xlsx
+++ b/preview/NP1PP_vs_C1Y_preview.xlsx
@@ -3722,7 +3722,7 @@
       </c>
       <c r="B302" s="2" t="inlineStr">
         <is>
-          <t>FA1</t>
+          <t>FA</t>
         </is>
       </c>
       <c r="C302" s="8" t="inlineStr">
@@ -5021,7 +5021,7 @@
       </c>
       <c r="B420" s="2" t="inlineStr">
         <is>
-          <t>SDFSYNC1</t>
+          <t>SDFSYNC</t>
         </is>
       </c>
       <c r="C420" s="3" t="n"/>
@@ -5787,7 +5787,8 @@
       </c>
       <c r="B492" s="2" t="inlineStr">
         <is>
-          <t>AIOI21</t>
+          <t>AIOI
+复合·AIOI</t>
         </is>
       </c>
       <c r="C492" s="8" t="inlineStr">
@@ -5849,7 +5850,8 @@
       <c r="A497" s="2" t="n"/>
       <c r="B497" s="2" t="inlineStr">
         <is>
-          <t>AOAI211</t>
+          <t>AOAI
+复合·AOAI</t>
         </is>
       </c>
       <c r="C497" s="8" t="inlineStr">
@@ -5935,39 +5937,36 @@
       <c r="A504" s="2" t="n"/>
       <c r="B504" s="2" t="inlineStr">
         <is>
-          <t>AOI211INV</t>
+          <t>AOIAOI
+复合·AOIAOI</t>
         </is>
       </c>
       <c r="C504" s="3" t="inlineStr">
         <is>
-          <t>AOI211INVCCMD1COTVIAG</t>
+          <t>AOI21AOI21CCMD1COT</t>
         </is>
       </c>
       <c r="D504" s="3" t="n"/>
     </row>
     <row r="505">
-      <c r="A505" s="6" t="n"/>
-      <c r="B505" s="6" t="n"/>
-      <c r="C505" s="7" t="n"/>
-      <c r="D505" s="7" t="inlineStr">
-        <is>
-          <t>AOI211INVCCMD2COTA</t>
-        </is>
-      </c>
+      <c r="A505" s="4" t="n"/>
+      <c r="B505" s="4" t="n"/>
+      <c r="C505" s="5" t="inlineStr">
+        <is>
+          <t>AOI22AOI21CCMD2COTVIA</t>
+        </is>
+      </c>
+      <c r="D505" s="5" t="n"/>
     </row>
     <row r="506">
-      <c r="A506" s="2" t="n"/>
-      <c r="B506" s="2" t="inlineStr">
-        <is>
-          <t>AOI21AOI21</t>
-        </is>
-      </c>
-      <c r="C506" s="3" t="inlineStr">
-        <is>
-          <t>AOI21AOI21CCMD1COT</t>
-        </is>
-      </c>
-      <c r="D506" s="3" t="n"/>
+      <c r="A506" s="4" t="n"/>
+      <c r="B506" s="4" t="n"/>
+      <c r="C506" s="5" t="inlineStr">
+        <is>
+          <t>AOI22AOI22CCMD2COTM3CEQ</t>
+        </is>
+      </c>
+      <c r="D506" s="5" t="n"/>
     </row>
     <row r="507">
       <c r="A507" s="6" t="n"/>
@@ -5983,12 +5982,13 @@
       <c r="A508" s="2" t="n"/>
       <c r="B508" s="2" t="inlineStr">
         <is>
-          <t>AOI21ND2</t>
+          <t>AOIINV
+复合·AOIINV</t>
         </is>
       </c>
       <c r="C508" s="3" t="inlineStr">
         <is>
-          <t>AOI21ND2CCBD1COT</t>
+          <t>AOI211INVCCMD1COTVIAG</t>
         </is>
       </c>
       <c r="D508" s="3" t="n"/>
@@ -5998,130 +5998,115 @@
       <c r="B509" s="4" t="n"/>
       <c r="C509" s="5" t="inlineStr">
         <is>
+          <t>AOI22INVCCMD2COT</t>
+        </is>
+      </c>
+      <c r="D509" s="5" t="n"/>
+    </row>
+    <row r="510">
+      <c r="A510" s="4" t="n"/>
+      <c r="B510" s="4" t="n"/>
+      <c r="C510" s="5" t="n"/>
+      <c r="D510" s="5" t="inlineStr">
+        <is>
+          <t>AOI211INVCCMD2COTA</t>
+        </is>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" s="6" t="n"/>
+      <c r="B511" s="6" t="n"/>
+      <c r="C511" s="7" t="n"/>
+      <c r="D511" s="7" t="inlineStr">
+        <is>
+          <t>AOI22INVCCMD1COTA</t>
+        </is>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" s="2" t="n"/>
+      <c r="B512" s="2" t="inlineStr">
+        <is>
+          <t>AOIND
+复合·AOIND</t>
+        </is>
+      </c>
+      <c r="C512" s="3" t="inlineStr">
+        <is>
+          <t>AOI21ND2CCBD1COT</t>
+        </is>
+      </c>
+      <c r="D512" s="3" t="n"/>
+    </row>
+    <row r="513">
+      <c r="A513" s="4" t="n"/>
+      <c r="B513" s="4" t="n"/>
+      <c r="C513" s="5" t="inlineStr">
+        <is>
           <t>AOI21ND2CCMD1COT</t>
         </is>
       </c>
-      <c r="D509" s="5" t="n"/>
-    </row>
-    <row r="510">
-      <c r="A510" s="6" t="n"/>
-      <c r="B510" s="6" t="n"/>
-      <c r="C510" s="7" t="n"/>
-      <c r="D510" s="7" t="inlineStr">
-        <is>
-          <t>AOI21ND2CCBD1COTA</t>
-        </is>
-      </c>
-    </row>
-    <row r="511">
-      <c r="A511" s="2" t="n"/>
-      <c r="B511" s="2" t="inlineStr">
-        <is>
-          <t>AOI21NR2</t>
-        </is>
-      </c>
-      <c r="C511" s="3" t="inlineStr">
-        <is>
-          <t>AOI21NR2CCBD1COT</t>
-        </is>
-      </c>
-      <c r="D511" s="3" t="n"/>
-    </row>
-    <row r="512">
-      <c r="A512" s="4" t="n"/>
-      <c r="B512" s="4" t="n"/>
-      <c r="C512" s="5" t="inlineStr">
-        <is>
-          <t>AOI21NR2CCMD2COTVIA</t>
-        </is>
-      </c>
-      <c r="D512" s="5" t="n"/>
-    </row>
-    <row r="513">
-      <c r="A513" s="6" t="n"/>
-      <c r="B513" s="6" t="n"/>
-      <c r="C513" s="7" t="n"/>
-      <c r="D513" s="7" t="inlineStr">
-        <is>
-          <t>AOI21NR2CCBD1COTA</t>
-        </is>
-      </c>
+      <c r="D513" s="5" t="n"/>
     </row>
     <row r="514">
-      <c r="A514" s="2" t="n"/>
-      <c r="B514" s="2" t="inlineStr">
-        <is>
-          <t>AOI21OAI21</t>
-        </is>
-      </c>
-      <c r="C514" s="3" t="inlineStr">
-        <is>
-          <t>AOI21OAI21CCAD2COT</t>
-        </is>
-      </c>
-      <c r="D514" s="3" t="n"/>
+      <c r="A514" s="4" t="n"/>
+      <c r="B514" s="4" t="n"/>
+      <c r="C514" s="5" t="inlineStr">
+        <is>
+          <t>AOI22ND2CCBD1COTVIAG</t>
+        </is>
+      </c>
+      <c r="D514" s="5" t="n"/>
     </row>
     <row r="515">
       <c r="A515" s="4" t="n"/>
       <c r="B515" s="4" t="n"/>
       <c r="C515" s="5" t="inlineStr">
         <is>
-          <t>AOI21OAI21CCMD2COT</t>
+          <t>AOI22ND2CCMD1COT</t>
         </is>
       </c>
       <c r="D515" s="5" t="n"/>
     </row>
     <row r="516">
-      <c r="A516" s="6" t="n"/>
-      <c r="B516" s="6" t="n"/>
-      <c r="C516" s="7" t="n"/>
-      <c r="D516" s="7" t="inlineStr">
-        <is>
-          <t>AOI21OAI21CCAD2COTA</t>
-        </is>
-      </c>
+      <c r="A516" s="4" t="n"/>
+      <c r="B516" s="4" t="n"/>
+      <c r="C516" s="5" t="inlineStr">
+        <is>
+          <t>AOI22ND2D1COTEEQ</t>
+        </is>
+      </c>
+      <c r="D516" s="5" t="n"/>
     </row>
     <row r="517">
-      <c r="A517" s="10" t="n"/>
-      <c r="B517" s="10" t="inlineStr">
-        <is>
-          <t>AOI22AOI21</t>
-        </is>
-      </c>
-      <c r="C517" s="11" t="inlineStr">
-        <is>
-          <t>AOI22AOI21CCMD2COTVIA</t>
-        </is>
-      </c>
-      <c r="D517" s="11" t="n"/>
+      <c r="A517" s="4" t="n"/>
+      <c r="B517" s="4" t="n"/>
+      <c r="C517" s="5" t="inlineStr">
+        <is>
+          <t>AOI22ND2D2COT</t>
+        </is>
+      </c>
+      <c r="D517" s="5" t="n"/>
     </row>
     <row r="518">
-      <c r="A518" s="10" t="n"/>
-      <c r="B518" s="10" t="inlineStr">
-        <is>
-          <t>AOI22AOI22</t>
-        </is>
-      </c>
-      <c r="C518" s="11" t="inlineStr">
-        <is>
-          <t>AOI22AOI22CCMD2COTM3CEQ</t>
-        </is>
-      </c>
-      <c r="D518" s="11" t="n"/>
+      <c r="A518" s="4" t="n"/>
+      <c r="B518" s="4" t="n"/>
+      <c r="C518" s="5" t="inlineStr">
+        <is>
+          <t>AOI22ND2D4COT</t>
+        </is>
+      </c>
+      <c r="D518" s="5" t="n"/>
     </row>
     <row r="519">
-      <c r="A519" s="2" t="n"/>
-      <c r="B519" s="2" t="inlineStr">
-        <is>
-          <t>AOI22INV</t>
-        </is>
-      </c>
-      <c r="C519" s="3" t="inlineStr">
-        <is>
-          <t>AOI22INVCCMD2COT</t>
-        </is>
-      </c>
-      <c r="D519" s="3" t="n"/>
+      <c r="A519" s="4" t="n"/>
+      <c r="B519" s="4" t="n"/>
+      <c r="C519" s="5" t="n"/>
+      <c r="D519" s="5" t="inlineStr">
+        <is>
+          <t>AOI21ND2CCBD1COTA</t>
+        </is>
+      </c>
     </row>
     <row r="520">
       <c r="A520" s="6" t="n"/>
@@ -6129,7 +6114,7 @@
       <c r="C520" s="7" t="n"/>
       <c r="D520" s="7" t="inlineStr">
         <is>
-          <t>AOI22INVCCMD1COTA</t>
+          <t>AOI22ND2CCBD4COTA</t>
         </is>
       </c>
     </row>
@@ -6137,12 +6122,13 @@
       <c r="A521" s="2" t="n"/>
       <c r="B521" s="2" t="inlineStr">
         <is>
-          <t>AOI22ND2</t>
+          <t>AOINR
+复合·AOINR</t>
         </is>
       </c>
       <c r="C521" s="3" t="inlineStr">
         <is>
-          <t>AOI22ND2CCBD1COTVIAG</t>
+          <t>AOI21NR2CCBD1COT</t>
         </is>
       </c>
       <c r="D521" s="3" t="n"/>
@@ -6152,7 +6138,7 @@
       <c r="B522" s="4" t="n"/>
       <c r="C522" s="5" t="inlineStr">
         <is>
-          <t>AOI22ND2CCMD1COT</t>
+          <t>AOI21NR2CCMD2COTVIA</t>
         </is>
       </c>
       <c r="D522" s="5" t="n"/>
@@ -6162,7 +6148,7 @@
       <c r="B523" s="4" t="n"/>
       <c r="C523" s="5" t="inlineStr">
         <is>
-          <t>AOI22ND2D1COTEEQ</t>
+          <t>AOI22NR2CCBD1COT</t>
         </is>
       </c>
       <c r="D523" s="5" t="n"/>
@@ -6172,7 +6158,7 @@
       <c r="B524" s="4" t="n"/>
       <c r="C524" s="5" t="inlineStr">
         <is>
-          <t>AOI22ND2D2COT</t>
+          <t>AOI22NR2CCMD1COT</t>
         </is>
       </c>
       <c r="D524" s="5" t="n"/>
@@ -6180,90 +6166,87 @@
     <row r="525">
       <c r="A525" s="4" t="n"/>
       <c r="B525" s="4" t="n"/>
-      <c r="C525" s="5" t="inlineStr">
-        <is>
-          <t>AOI22ND2D4COT</t>
-        </is>
-      </c>
-      <c r="D525" s="5" t="n"/>
+      <c r="C525" s="5" t="n"/>
+      <c r="D525" s="5" t="inlineStr">
+        <is>
+          <t>AOI21NR2CCBD1COTA</t>
+        </is>
+      </c>
     </row>
     <row r="526">
-      <c r="A526" s="6" t="n"/>
-      <c r="B526" s="6" t="n"/>
-      <c r="C526" s="7" t="n"/>
-      <c r="D526" s="7" t="inlineStr">
-        <is>
-          <t>AOI22ND2CCBD4COTA</t>
+      <c r="A526" s="4" t="n"/>
+      <c r="B526" s="4" t="n"/>
+      <c r="C526" s="5" t="n"/>
+      <c r="D526" s="5" t="inlineStr">
+        <is>
+          <t>AOI22NR2CCBD4COTA</t>
         </is>
       </c>
     </row>
     <row r="527">
-      <c r="A527" s="2" t="n"/>
-      <c r="B527" s="2" t="inlineStr">
-        <is>
-          <t>AOI22NR2</t>
-        </is>
-      </c>
-      <c r="C527" s="3" t="inlineStr">
-        <is>
-          <t>AOI22NR2CCBD1COT</t>
-        </is>
-      </c>
-      <c r="D527" s="3" t="n"/>
+      <c r="A527" s="6" t="n"/>
+      <c r="B527" s="6" t="n"/>
+      <c r="C527" s="7" t="n"/>
+      <c r="D527" s="7" t="inlineStr">
+        <is>
+          <t>AOI22NR2CCMD2COTA</t>
+        </is>
+      </c>
     </row>
     <row r="528">
-      <c r="A528" s="4" t="n"/>
-      <c r="B528" s="4" t="n"/>
-      <c r="C528" s="5" t="inlineStr">
-        <is>
-          <t>AOI22NR2CCMD1COT</t>
-        </is>
-      </c>
-      <c r="D528" s="5" t="n"/>
+      <c r="A528" s="2" t="n"/>
+      <c r="B528" s="2" t="inlineStr">
+        <is>
+          <t>AOIOAI
+复合·AOIOAI</t>
+        </is>
+      </c>
+      <c r="C528" s="3" t="inlineStr">
+        <is>
+          <t>AOI21OAI21CCAD2COT</t>
+        </is>
+      </c>
+      <c r="D528" s="3" t="n"/>
     </row>
     <row r="529">
       <c r="A529" s="4" t="n"/>
       <c r="B529" s="4" t="n"/>
-      <c r="C529" s="5" t="n"/>
-      <c r="D529" s="5" t="inlineStr">
-        <is>
-          <t>AOI22NR2CCBD4COTA</t>
-        </is>
-      </c>
+      <c r="C529" s="5" t="inlineStr">
+        <is>
+          <t>AOI21OAI21CCMD2COT</t>
+        </is>
+      </c>
+      <c r="D529" s="5" t="n"/>
     </row>
     <row r="530">
-      <c r="A530" s="6" t="n"/>
-      <c r="B530" s="6" t="n"/>
-      <c r="C530" s="7" t="n"/>
-      <c r="D530" s="7" t="inlineStr">
-        <is>
-          <t>AOI22NR2CCMD2COTA</t>
-        </is>
-      </c>
+      <c r="A530" s="4" t="n"/>
+      <c r="B530" s="4" t="n"/>
+      <c r="C530" s="5" t="inlineStr">
+        <is>
+          <t>AOI22OAI21CCAD1COT</t>
+        </is>
+      </c>
+      <c r="D530" s="5" t="n"/>
     </row>
     <row r="531">
-      <c r="A531" s="2" t="n"/>
-      <c r="B531" s="2" t="inlineStr">
-        <is>
-          <t>AOI22OAI21</t>
-        </is>
-      </c>
-      <c r="C531" s="3" t="inlineStr">
-        <is>
-          <t>AOI22OAI21CCAD1COT</t>
-        </is>
-      </c>
-      <c r="D531" s="3" t="n"/>
+      <c r="A531" s="4" t="n"/>
+      <c r="B531" s="4" t="n"/>
+      <c r="C531" s="5" t="inlineStr">
+        <is>
+          <t>AOI22OAI21CCMD1COT</t>
+        </is>
+      </c>
+      <c r="D531" s="5" t="n"/>
     </row>
     <row r="532">
       <c r="A532" s="4" t="n"/>
       <c r="B532" s="4" t="n"/>
-      <c r="C532" s="5" t="inlineStr">
-        <is>
-          <t>AOI22OAI21CCMD1COT</t>
-        </is>
-      </c>
-      <c r="D532" s="5" t="n"/>
+      <c r="C532" s="5" t="n"/>
+      <c r="D532" s="5" t="inlineStr">
+        <is>
+          <t>AOI21OAI21CCAD2COTA</t>
+        </is>
+      </c>
     </row>
     <row r="533">
       <c r="A533" s="4" t="n"/>
@@ -6289,32 +6272,41 @@
       <c r="A535" s="2" t="n"/>
       <c r="B535" s="2" t="inlineStr">
         <is>
-          <t>IAO21</t>
-        </is>
-      </c>
-      <c r="C535" s="3" t="inlineStr">
-        <is>
-          <t>IAO21D1COT</t>
-        </is>
-      </c>
-      <c r="D535" s="3" t="n"/>
+          <t>IAO
+复合·IAO</t>
+        </is>
+      </c>
+      <c r="C535" s="8" t="inlineStr">
+        <is>
+          <t>IAO22D2COT</t>
+        </is>
+      </c>
+      <c r="D535" s="8" t="inlineStr">
+        <is>
+          <t>IAO22D2COT</t>
+        </is>
+      </c>
     </row>
     <row r="536">
       <c r="A536" s="4" t="n"/>
       <c r="B536" s="4" t="n"/>
-      <c r="C536" s="5" t="inlineStr">
-        <is>
-          <t>IAO21D2COT</t>
-        </is>
-      </c>
-      <c r="D536" s="5" t="n"/>
+      <c r="C536" s="9" t="inlineStr">
+        <is>
+          <t>IAO22D4COT</t>
+        </is>
+      </c>
+      <c r="D536" s="9" t="inlineStr">
+        <is>
+          <t>IAO22D4COT</t>
+        </is>
+      </c>
     </row>
     <row r="537">
       <c r="A537" s="4" t="n"/>
       <c r="B537" s="4" t="n"/>
       <c r="C537" s="5" t="inlineStr">
         <is>
-          <t>IAO21D4COT</t>
+          <t>IAO21D1COT</t>
         </is>
       </c>
       <c r="D537" s="5" t="n"/>
@@ -6322,64 +6314,52 @@
     <row r="538">
       <c r="A538" s="4" t="n"/>
       <c r="B538" s="4" t="n"/>
-      <c r="C538" s="5" t="n"/>
-      <c r="D538" s="5" t="inlineStr">
-        <is>
-          <t>IAO21D2COT3FIN</t>
-        </is>
-      </c>
+      <c r="C538" s="5" t="inlineStr">
+        <is>
+          <t>IAO21D2COT</t>
+        </is>
+      </c>
+      <c r="D538" s="5" t="n"/>
     </row>
     <row r="539">
-      <c r="A539" s="6" t="n"/>
-      <c r="B539" s="6" t="n"/>
-      <c r="C539" s="7" t="n"/>
-      <c r="D539" s="7" t="inlineStr">
-        <is>
-          <t>IAO21EEQMBDD2COT</t>
-        </is>
-      </c>
+      <c r="A539" s="4" t="n"/>
+      <c r="B539" s="4" t="n"/>
+      <c r="C539" s="5" t="inlineStr">
+        <is>
+          <t>IAO21D4COT</t>
+        </is>
+      </c>
+      <c r="D539" s="5" t="n"/>
     </row>
     <row r="540">
-      <c r="A540" s="2" t="n"/>
-      <c r="B540" s="2" t="inlineStr">
-        <is>
-          <t>IAO22</t>
-        </is>
-      </c>
-      <c r="C540" s="8" t="inlineStr">
-        <is>
-          <t>IAO22D2COT</t>
-        </is>
-      </c>
-      <c r="D540" s="8" t="inlineStr">
-        <is>
-          <t>IAO22D2COT</t>
-        </is>
-      </c>
+      <c r="A540" s="4" t="n"/>
+      <c r="B540" s="4" t="n"/>
+      <c r="C540" s="5" t="inlineStr">
+        <is>
+          <t>IAO22D1COTVIAGMDB</t>
+        </is>
+      </c>
+      <c r="D540" s="5" t="n"/>
     </row>
     <row r="541">
       <c r="A541" s="4" t="n"/>
       <c r="B541" s="4" t="n"/>
-      <c r="C541" s="9" t="inlineStr">
-        <is>
-          <t>IAO22D4COT</t>
-        </is>
-      </c>
-      <c r="D541" s="9" t="inlineStr">
-        <is>
-          <t>IAO22D4COT</t>
+      <c r="C541" s="5" t="n"/>
+      <c r="D541" s="5" t="inlineStr">
+        <is>
+          <t>IAO21D2COT3FIN</t>
         </is>
       </c>
     </row>
     <row r="542">
       <c r="A542" s="4" t="n"/>
       <c r="B542" s="4" t="n"/>
-      <c r="C542" s="5" t="inlineStr">
-        <is>
-          <t>IAO22D1COTVIAGMDB</t>
-        </is>
-      </c>
-      <c r="D542" s="5" t="n"/>
+      <c r="C542" s="5" t="n"/>
+      <c r="D542" s="5" t="inlineStr">
+        <is>
+          <t>IAO21EEQMBDD2COT</t>
+        </is>
+      </c>
     </row>
     <row r="543">
       <c r="A543" s="4" t="n"/>
@@ -6405,7 +6385,8 @@
       <c r="A545" s="2" t="n"/>
       <c r="B545" s="2" t="inlineStr">
         <is>
-          <t>IAOI21</t>
+          <t>IAOI
+复合·IAOI</t>
         </is>
       </c>
       <c r="C545" s="8" t="inlineStr">
@@ -6463,7 +6444,8 @@
       <c r="A550" s="10" t="n"/>
       <c r="B550" s="10" t="inlineStr">
         <is>
-          <t>INVAAOI21</t>
+          <t>INVAAOI
+复合·INVAAOI</t>
         </is>
       </c>
       <c r="C550" s="11" t="inlineStr">
@@ -6477,7 +6459,8 @@
       <c r="A551" s="2" t="n"/>
       <c r="B551" s="2" t="inlineStr">
         <is>
-          <t>INVAOAI21</t>
+          <t>INVAOAI
+复合·INVAOAI</t>
         </is>
       </c>
       <c r="C551" s="3" t="inlineStr">
@@ -6501,7 +6484,8 @@
       <c r="A553" s="2" t="n"/>
       <c r="B553" s="2" t="inlineStr">
         <is>
-          <t>INVBAOI21</t>
+          <t>INVBAOI
+复合·INVBAOI</t>
         </is>
       </c>
       <c r="C553" s="3" t="inlineStr">
@@ -6525,7 +6509,8 @@
       <c r="A555" s="2" t="n"/>
       <c r="B555" s="2" t="inlineStr">
         <is>
-          <t>INVBOAI21</t>
+          <t>INVBOAI
+复合·INVBOAI</t>
         </is>
       </c>
       <c r="C555" s="3" t="inlineStr">
@@ -6549,7 +6534,8 @@
       <c r="A557" s="2" t="n"/>
       <c r="B557" s="2" t="inlineStr">
         <is>
-          <t>IOA21</t>
+          <t>IOA
+复合·IOA</t>
         </is>
       </c>
       <c r="C557" s="8" t="inlineStr">
@@ -6566,19 +6552,23 @@
     <row r="558">
       <c r="A558" s="4" t="n"/>
       <c r="B558" s="4" t="n"/>
-      <c r="C558" s="5" t="inlineStr">
-        <is>
-          <t>IOA21D1COTAROPUEEQ</t>
-        </is>
-      </c>
-      <c r="D558" s="5" t="n"/>
+      <c r="C558" s="9" t="inlineStr">
+        <is>
+          <t>IOA22D4COT</t>
+        </is>
+      </c>
+      <c r="D558" s="9" t="inlineStr">
+        <is>
+          <t>IOA22D4COT</t>
+        </is>
+      </c>
     </row>
     <row r="559">
       <c r="A559" s="4" t="n"/>
       <c r="B559" s="4" t="n"/>
       <c r="C559" s="5" t="inlineStr">
         <is>
-          <t>IOA21D2COTVIA</t>
+          <t>IOA21D1COTAROPUEEQ</t>
         </is>
       </c>
       <c r="D559" s="5" t="n"/>
@@ -6588,7 +6578,7 @@
       <c r="B560" s="4" t="n"/>
       <c r="C560" s="5" t="inlineStr">
         <is>
-          <t>IOA21D4COT</t>
+          <t>IOA21D2COTVIA</t>
         </is>
       </c>
       <c r="D560" s="5" t="n"/>
@@ -6598,7 +6588,7 @@
       <c r="B561" s="4" t="n"/>
       <c r="C561" s="5" t="inlineStr">
         <is>
-          <t>IOA21D6COTVIA</t>
+          <t>IOA21D4COT</t>
         </is>
       </c>
       <c r="D561" s="5" t="n"/>
@@ -6606,60 +6596,52 @@
     <row r="562">
       <c r="A562" s="4" t="n"/>
       <c r="B562" s="4" t="n"/>
-      <c r="C562" s="5" t="n"/>
-      <c r="D562" s="5" t="inlineStr">
-        <is>
-          <t>IOA21D0COT</t>
-        </is>
-      </c>
+      <c r="C562" s="5" t="inlineStr">
+        <is>
+          <t>IOA21D6COTVIA</t>
+        </is>
+      </c>
+      <c r="D562" s="5" t="n"/>
     </row>
     <row r="563">
-      <c r="A563" s="6" t="n"/>
-      <c r="B563" s="6" t="n"/>
-      <c r="C563" s="7" t="n"/>
-      <c r="D563" s="7" t="inlineStr">
-        <is>
-          <t>IOA21D4COT3FIN</t>
-        </is>
-      </c>
+      <c r="A563" s="4" t="n"/>
+      <c r="B563" s="4" t="n"/>
+      <c r="C563" s="5" t="inlineStr">
+        <is>
+          <t>IOA22D1COTVIAMDB</t>
+        </is>
+      </c>
+      <c r="D563" s="5" t="n"/>
     </row>
     <row r="564">
-      <c r="A564" s="2" t="n"/>
-      <c r="B564" s="2" t="inlineStr">
-        <is>
-          <t>IOA22</t>
-        </is>
-      </c>
-      <c r="C564" s="8" t="inlineStr">
-        <is>
-          <t>IOA22D4COT</t>
-        </is>
-      </c>
-      <c r="D564" s="8" t="inlineStr">
-        <is>
-          <t>IOA22D4COT</t>
-        </is>
-      </c>
+      <c r="A564" s="4" t="n"/>
+      <c r="B564" s="4" t="n"/>
+      <c r="C564" s="5" t="inlineStr">
+        <is>
+          <t>IOA22D2COT</t>
+        </is>
+      </c>
+      <c r="D564" s="5" t="n"/>
     </row>
     <row r="565">
       <c r="A565" s="4" t="n"/>
       <c r="B565" s="4" t="n"/>
-      <c r="C565" s="5" t="inlineStr">
-        <is>
-          <t>IOA22D1COTVIAMDB</t>
-        </is>
-      </c>
-      <c r="D565" s="5" t="n"/>
+      <c r="C565" s="5" t="n"/>
+      <c r="D565" s="5" t="inlineStr">
+        <is>
+          <t>IOA21D0COT</t>
+        </is>
+      </c>
     </row>
     <row r="566">
       <c r="A566" s="4" t="n"/>
       <c r="B566" s="4" t="n"/>
-      <c r="C566" s="5" t="inlineStr">
-        <is>
-          <t>IOA22D2COT</t>
-        </is>
-      </c>
-      <c r="D566" s="5" t="n"/>
+      <c r="C566" s="5" t="n"/>
+      <c r="D566" s="5" t="inlineStr">
+        <is>
+          <t>IOA21D4COT3FIN</t>
+        </is>
+      </c>
     </row>
     <row r="567">
       <c r="A567" s="6" t="n"/>
@@ -6675,7 +6657,8 @@
       <c r="A568" s="2" t="n"/>
       <c r="B568" s="2" t="inlineStr">
         <is>
-          <t>IOAI21</t>
+          <t>IOAI
+复合·IOAI</t>
         </is>
       </c>
       <c r="C568" s="8" t="inlineStr">
@@ -6737,12 +6720,13 @@
       <c r="A573" s="2" t="n"/>
       <c r="B573" s="2" t="inlineStr">
         <is>
-          <t>MAOI22</t>
+          <t>MAOI
+复合·MAOI</t>
         </is>
       </c>
       <c r="C573" s="3" t="inlineStr">
         <is>
-          <t>MAOI22D1COT</t>
+          <t>MAOI222D1COT</t>
         </is>
       </c>
       <c r="D573" s="3" t="n"/>
@@ -6752,7 +6736,7 @@
       <c r="B574" s="4" t="n"/>
       <c r="C574" s="5" t="inlineStr">
         <is>
-          <t>MAOI22D2COTVIA</t>
+          <t>MAOI222D2COTVIA</t>
         </is>
       </c>
       <c r="D574" s="5" t="n"/>
@@ -6762,41 +6746,37 @@
       <c r="B575" s="4" t="n"/>
       <c r="C575" s="5" t="inlineStr">
         <is>
-          <t>MAOI22D4COTVIA</t>
+          <t>MAOI222D4COTMDB</t>
         </is>
       </c>
       <c r="D575" s="5" t="n"/>
     </row>
     <row r="576">
-      <c r="A576" s="6" t="n"/>
-      <c r="B576" s="6" t="n"/>
-      <c r="C576" s="7" t="n"/>
-      <c r="D576" s="7" t="inlineStr">
-        <is>
-          <t>MAOI22D4COT</t>
-        </is>
-      </c>
+      <c r="A576" s="4" t="n"/>
+      <c r="B576" s="4" t="n"/>
+      <c r="C576" s="5" t="inlineStr">
+        <is>
+          <t>MAOI22D1COT</t>
+        </is>
+      </c>
+      <c r="D576" s="5" t="n"/>
     </row>
     <row r="577">
-      <c r="A577" s="2" t="n"/>
-      <c r="B577" s="2" t="inlineStr">
-        <is>
-          <t>MAOI222</t>
-        </is>
-      </c>
-      <c r="C577" s="3" t="inlineStr">
-        <is>
-          <t>MAOI222D1COT</t>
-        </is>
-      </c>
-      <c r="D577" s="3" t="n"/>
+      <c r="A577" s="4" t="n"/>
+      <c r="B577" s="4" t="n"/>
+      <c r="C577" s="5" t="inlineStr">
+        <is>
+          <t>MAOI22D2COTVIA</t>
+        </is>
+      </c>
+      <c r="D577" s="5" t="n"/>
     </row>
     <row r="578">
       <c r="A578" s="4" t="n"/>
       <c r="B578" s="4" t="n"/>
       <c r="C578" s="5" t="inlineStr">
         <is>
-          <t>MAOI222D2COTVIA</t>
+          <t>MAOI22D4COTVIA</t>
         </is>
       </c>
       <c r="D578" s="5" t="n"/>
@@ -6804,12 +6784,12 @@
     <row r="579">
       <c r="A579" s="4" t="n"/>
       <c r="B579" s="4" t="n"/>
-      <c r="C579" s="5" t="inlineStr">
-        <is>
-          <t>MAOI222D4COTMDB</t>
-        </is>
-      </c>
-      <c r="D579" s="5" t="n"/>
+      <c r="C579" s="5" t="n"/>
+      <c r="D579" s="5" t="inlineStr">
+        <is>
+          <t>MAOI222D2COT</t>
+        </is>
+      </c>
     </row>
     <row r="580">
       <c r="A580" s="4" t="n"/>
@@ -6817,7 +6797,7 @@
       <c r="C580" s="5" t="n"/>
       <c r="D580" s="5" t="inlineStr">
         <is>
-          <t>MAOI222D2COT</t>
+          <t>MAOI222D4COT</t>
         </is>
       </c>
     </row>
@@ -6827,7 +6807,7 @@
       <c r="C581" s="7" t="n"/>
       <c r="D581" s="7" t="inlineStr">
         <is>
-          <t>MAOI222D4COT</t>
+          <t>MAOI22D4COT</t>
         </is>
       </c>
     </row>
@@ -6835,7 +6815,8 @@
       <c r="A582" s="2" t="n"/>
       <c r="B582" s="2" t="inlineStr">
         <is>
-          <t>MOAI22</t>
+          <t>MOAI
+复合·MOAI</t>
         </is>
       </c>
       <c r="C582" s="8" t="inlineStr">
@@ -6893,7 +6874,8 @@
       <c r="A587" s="2" t="n"/>
       <c r="B587" s="2" t="inlineStr">
         <is>
-          <t>ND2AOI21</t>
+          <t>NDAOI
+复合·NDAOI</t>
         </is>
       </c>
       <c r="C587" s="3" t="inlineStr">
@@ -6917,7 +6899,8 @@
       <c r="A589" s="2" t="n"/>
       <c r="B589" s="2" t="inlineStr">
         <is>
-          <t>ND2IOA21</t>
+          <t>NDIOA
+复合·NDIOA</t>
         </is>
       </c>
       <c r="C589" s="3" t="inlineStr">
@@ -6951,7 +6934,8 @@
       <c r="A592" s="2" t="n"/>
       <c r="B592" s="2" t="inlineStr">
         <is>
-          <t>ND2OAI21</t>
+          <t>NDOAI
+复合·NDOAI</t>
         </is>
       </c>
       <c r="C592" s="3" t="inlineStr">
@@ -6975,7 +6959,8 @@
       <c r="A594" s="2" t="n"/>
       <c r="B594" s="2" t="inlineStr">
         <is>
-          <t>NR2AOI21</t>
+          <t>NRAOI
+复合·NRAOI</t>
         </is>
       </c>
       <c r="C594" s="3" t="inlineStr">
@@ -6999,7 +6984,8 @@
       <c r="A596" s="2" t="n"/>
       <c r="B596" s="2" t="inlineStr">
         <is>
-          <t>NR2ND2</t>
+          <t>NRND
+复合·NRND</t>
         </is>
       </c>
       <c r="C596" s="3" t="inlineStr">
@@ -7030,161 +7016,156 @@
       <c r="D598" s="7" t="n"/>
     </row>
     <row r="599">
-      <c r="A599" s="10" t="n"/>
-      <c r="B599" s="10" t="inlineStr">
-        <is>
-          <t>OAI211INV</t>
-        </is>
-      </c>
-      <c r="C599" s="11" t="inlineStr">
-        <is>
-          <t>OAI211INVCCAD1COTVIAG</t>
-        </is>
-      </c>
-      <c r="D599" s="11" t="n"/>
+      <c r="A599" s="2" t="n"/>
+      <c r="B599" s="2" t="inlineStr">
+        <is>
+          <t>OAIAOI
+复合·OAIAOI</t>
+        </is>
+      </c>
+      <c r="C599" s="3" t="inlineStr">
+        <is>
+          <t>OAI21AOI22D1COT</t>
+        </is>
+      </c>
+      <c r="D599" s="3" t="n"/>
     </row>
     <row r="600">
-      <c r="A600" s="10" t="n"/>
-      <c r="B600" s="10" t="inlineStr">
-        <is>
-          <t>OAI21AOI21</t>
-        </is>
-      </c>
-      <c r="C600" s="11" t="n"/>
-      <c r="D600" s="11" t="inlineStr">
-        <is>
-          <t>OAI21AOI21CCBD4COTA</t>
-        </is>
-      </c>
+      <c r="A600" s="4" t="n"/>
+      <c r="B600" s="4" t="n"/>
+      <c r="C600" s="5" t="inlineStr">
+        <is>
+          <t>OAI21AOI22D2COT</t>
+        </is>
+      </c>
+      <c r="D600" s="5" t="n"/>
     </row>
     <row r="601">
-      <c r="A601" s="2" t="n"/>
-      <c r="B601" s="2" t="inlineStr">
-        <is>
-          <t>OAI21AOI22</t>
-        </is>
-      </c>
-      <c r="C601" s="3" t="inlineStr">
-        <is>
-          <t>OAI21AOI22D1COT</t>
-        </is>
-      </c>
-      <c r="D601" s="3" t="n"/>
+      <c r="A601" s="4" t="n"/>
+      <c r="B601" s="4" t="n"/>
+      <c r="C601" s="5" t="inlineStr">
+        <is>
+          <t>OAI21AOI22D4COT</t>
+        </is>
+      </c>
+      <c r="D601" s="5" t="n"/>
     </row>
     <row r="602">
       <c r="A602" s="4" t="n"/>
       <c r="B602" s="4" t="n"/>
       <c r="C602" s="5" t="inlineStr">
         <is>
-          <t>OAI21AOI22D2COT</t>
+          <t>OAI22AOI21CCAD2COT</t>
         </is>
       </c>
       <c r="D602" s="5" t="n"/>
     </row>
     <row r="603">
-      <c r="A603" s="6" t="n"/>
-      <c r="B603" s="6" t="n"/>
-      <c r="C603" s="7" t="inlineStr">
-        <is>
-          <t>OAI21AOI22D4COT</t>
-        </is>
-      </c>
-      <c r="D603" s="7" t="n"/>
+      <c r="A603" s="4" t="n"/>
+      <c r="B603" s="4" t="n"/>
+      <c r="C603" s="5" t="inlineStr">
+        <is>
+          <t>OAI22AOI21CCMD1COT</t>
+        </is>
+      </c>
+      <c r="D603" s="5" t="n"/>
     </row>
     <row r="604">
-      <c r="A604" s="2" t="n"/>
-      <c r="B604" s="2" t="inlineStr">
-        <is>
-          <t>OAI21ND2</t>
-        </is>
-      </c>
-      <c r="C604" s="3" t="inlineStr">
-        <is>
-          <t>OAI21ND2CCAD1COTVIAG</t>
-        </is>
-      </c>
-      <c r="D604" s="3" t="n"/>
+      <c r="A604" s="4" t="n"/>
+      <c r="B604" s="4" t="n"/>
+      <c r="C604" s="5" t="n"/>
+      <c r="D604" s="5" t="inlineStr">
+        <is>
+          <t>OAI21AOI21CCBD4COTA</t>
+        </is>
+      </c>
     </row>
     <row r="605">
       <c r="A605" s="4" t="n"/>
       <c r="B605" s="4" t="n"/>
-      <c r="C605" s="5" t="inlineStr">
-        <is>
-          <t>OAI21ND2CCBD4COTVIA</t>
-        </is>
-      </c>
-      <c r="D605" s="5" t="n"/>
+      <c r="C605" s="5" t="n"/>
+      <c r="D605" s="5" t="inlineStr">
+        <is>
+          <t>OAI22AOI21CCBD4COTA</t>
+        </is>
+      </c>
     </row>
     <row r="606">
-      <c r="A606" s="4" t="n"/>
-      <c r="B606" s="4" t="n"/>
-      <c r="C606" s="5" t="inlineStr">
-        <is>
-          <t>OAI21ND2D1COT</t>
-        </is>
-      </c>
-      <c r="D606" s="5" t="n"/>
+      <c r="A606" s="6" t="n"/>
+      <c r="B606" s="6" t="n"/>
+      <c r="C606" s="7" t="n"/>
+      <c r="D606" s="7" t="inlineStr">
+        <is>
+          <t>OAI22AOI21CCMD2COTA</t>
+        </is>
+      </c>
     </row>
     <row r="607">
-      <c r="A607" s="4" t="n"/>
-      <c r="B607" s="4" t="n"/>
-      <c r="C607" s="5" t="inlineStr">
-        <is>
-          <t>OAI21ND2D2COT</t>
-        </is>
-      </c>
-      <c r="D607" s="5" t="n"/>
+      <c r="A607" s="2" t="n"/>
+      <c r="B607" s="2" t="inlineStr">
+        <is>
+          <t>OAIINV
+复合·OAIINV</t>
+        </is>
+      </c>
+      <c r="C607" s="3" t="inlineStr">
+        <is>
+          <t>OAI211INVCCAD1COTVIAG</t>
+        </is>
+      </c>
+      <c r="D607" s="3" t="n"/>
     </row>
     <row r="608">
       <c r="A608" s="4" t="n"/>
       <c r="B608" s="4" t="n"/>
       <c r="C608" s="5" t="inlineStr">
         <is>
-          <t>OAI21ND2D4COT</t>
+          <t>OAI22INVCCAD1COT</t>
         </is>
       </c>
       <c r="D608" s="5" t="n"/>
     </row>
     <row r="609">
-      <c r="A609" s="4" t="n"/>
-      <c r="B609" s="4" t="n"/>
-      <c r="C609" s="5" t="n"/>
-      <c r="D609" s="5" t="inlineStr">
-        <is>
-          <t>OAI21ND2CCAD1COTA</t>
+      <c r="A609" s="6" t="n"/>
+      <c r="B609" s="6" t="n"/>
+      <c r="C609" s="7" t="n"/>
+      <c r="D609" s="7" t="inlineStr">
+        <is>
+          <t>OAI22INVCCAD1COTA</t>
         </is>
       </c>
     </row>
     <row r="610">
-      <c r="A610" s="6" t="n"/>
-      <c r="B610" s="6" t="n"/>
-      <c r="C610" s="7" t="n"/>
-      <c r="D610" s="7" t="inlineStr">
-        <is>
-          <t>OAI21ND2CCBD4COTA</t>
-        </is>
-      </c>
+      <c r="A610" s="2" t="n"/>
+      <c r="B610" s="2" t="inlineStr">
+        <is>
+          <t>OAIND
+复合·OAIND</t>
+        </is>
+      </c>
+      <c r="C610" s="3" t="inlineStr">
+        <is>
+          <t>OAI21ND2CCAD1COTVIAG</t>
+        </is>
+      </c>
+      <c r="D610" s="3" t="n"/>
     </row>
     <row r="611">
-      <c r="A611" s="2" t="n"/>
-      <c r="B611" s="2" t="inlineStr">
-        <is>
-          <t>OAI21NR2</t>
-        </is>
-      </c>
-      <c r="C611" s="3" t="inlineStr">
-        <is>
-          <t>OAI21NR2CCAD1COT</t>
-        </is>
-      </c>
-      <c r="D611" s="3" t="n"/>
+      <c r="A611" s="4" t="n"/>
+      <c r="B611" s="4" t="n"/>
+      <c r="C611" s="5" t="inlineStr">
+        <is>
+          <t>OAI21ND2CCBD4COTVIA</t>
+        </is>
+      </c>
+      <c r="D611" s="5" t="n"/>
     </row>
     <row r="612">
       <c r="A612" s="4" t="n"/>
       <c r="B612" s="4" t="n"/>
       <c r="C612" s="5" t="inlineStr">
         <is>
-          <t>OAI21NR2CCBD2COT</t>
+          <t>OAI21ND2D1COT</t>
         </is>
       </c>
       <c r="D612" s="5" t="n"/>
@@ -7192,162 +7173,148 @@
     <row r="613">
       <c r="A613" s="4" t="n"/>
       <c r="B613" s="4" t="n"/>
-      <c r="C613" s="5" t="n"/>
-      <c r="D613" s="5" t="inlineStr">
-        <is>
-          <t>OAI21NR2CCAD2COTA</t>
-        </is>
-      </c>
+      <c r="C613" s="5" t="inlineStr">
+        <is>
+          <t>OAI21ND2D2COT</t>
+        </is>
+      </c>
+      <c r="D613" s="5" t="n"/>
     </row>
     <row r="614">
-      <c r="A614" s="6" t="n"/>
-      <c r="B614" s="6" t="n"/>
-      <c r="C614" s="7" t="n"/>
-      <c r="D614" s="7" t="inlineStr">
-        <is>
-          <t>OAI21NR2CCBD1COTA</t>
-        </is>
-      </c>
+      <c r="A614" s="4" t="n"/>
+      <c r="B614" s="4" t="n"/>
+      <c r="C614" s="5" t="inlineStr">
+        <is>
+          <t>OAI21ND2D4COT</t>
+        </is>
+      </c>
+      <c r="D614" s="5" t="n"/>
     </row>
     <row r="615">
-      <c r="A615" s="10" t="n"/>
-      <c r="B615" s="10" t="inlineStr">
-        <is>
-          <t>OAI21OAI21</t>
-        </is>
-      </c>
-      <c r="C615" s="11" t="n"/>
-      <c r="D615" s="11" t="inlineStr">
-        <is>
-          <t>OAI21OAI21CCBD4COTA</t>
-        </is>
-      </c>
+      <c r="A615" s="4" t="n"/>
+      <c r="B615" s="4" t="n"/>
+      <c r="C615" s="5" t="inlineStr">
+        <is>
+          <t>OAI22ND2CCBD4COT</t>
+        </is>
+      </c>
+      <c r="D615" s="5" t="n"/>
     </row>
     <row r="616">
-      <c r="A616" s="2" t="n"/>
-      <c r="B616" s="2" t="inlineStr">
-        <is>
-          <t>OAI22AOI21</t>
-        </is>
-      </c>
-      <c r="C616" s="3" t="inlineStr">
-        <is>
-          <t>OAI22AOI21CCAD2COT</t>
-        </is>
-      </c>
-      <c r="D616" s="3" t="n"/>
+      <c r="A616" s="4" t="n"/>
+      <c r="B616" s="4" t="n"/>
+      <c r="C616" s="5" t="n"/>
+      <c r="D616" s="5" t="inlineStr">
+        <is>
+          <t>OAI21ND2CCAD1COTA</t>
+        </is>
+      </c>
     </row>
     <row r="617">
       <c r="A617" s="4" t="n"/>
       <c r="B617" s="4" t="n"/>
-      <c r="C617" s="5" t="inlineStr">
-        <is>
-          <t>OAI22AOI21CCMD1COT</t>
-        </is>
-      </c>
-      <c r="D617" s="5" t="n"/>
+      <c r="C617" s="5" t="n"/>
+      <c r="D617" s="5" t="inlineStr">
+        <is>
+          <t>OAI21ND2CCBD4COTA</t>
+        </is>
+      </c>
     </row>
     <row r="618">
-      <c r="A618" s="4" t="n"/>
-      <c r="B618" s="4" t="n"/>
-      <c r="C618" s="5" t="n"/>
-      <c r="D618" s="5" t="inlineStr">
-        <is>
-          <t>OAI22AOI21CCBD4COTA</t>
+      <c r="A618" s="6" t="n"/>
+      <c r="B618" s="6" t="n"/>
+      <c r="C618" s="7" t="n"/>
+      <c r="D618" s="7" t="inlineStr">
+        <is>
+          <t>OAI22ND2CCBD4COTA</t>
         </is>
       </c>
     </row>
     <row r="619">
-      <c r="A619" s="6" t="n"/>
-      <c r="B619" s="6" t="n"/>
-      <c r="C619" s="7" t="n"/>
-      <c r="D619" s="7" t="inlineStr">
-        <is>
-          <t>OAI22AOI21CCMD2COTA</t>
-        </is>
-      </c>
+      <c r="A619" s="2" t="n"/>
+      <c r="B619" s="2" t="inlineStr">
+        <is>
+          <t>OAINR
+复合·OAINR</t>
+        </is>
+      </c>
+      <c r="C619" s="3" t="inlineStr">
+        <is>
+          <t>OAI21NR2CCAD1COT</t>
+        </is>
+      </c>
+      <c r="D619" s="3" t="n"/>
     </row>
     <row r="620">
-      <c r="A620" s="2" t="n"/>
-      <c r="B620" s="2" t="inlineStr">
-        <is>
-          <t>OAI22INV</t>
-        </is>
-      </c>
-      <c r="C620" s="3" t="inlineStr">
-        <is>
-          <t>OAI22INVCCAD1COT</t>
-        </is>
-      </c>
-      <c r="D620" s="3" t="n"/>
+      <c r="A620" s="4" t="n"/>
+      <c r="B620" s="4" t="n"/>
+      <c r="C620" s="5" t="inlineStr">
+        <is>
+          <t>OAI21NR2CCBD2COT</t>
+        </is>
+      </c>
+      <c r="D620" s="5" t="n"/>
     </row>
     <row r="621">
-      <c r="A621" s="6" t="n"/>
-      <c r="B621" s="6" t="n"/>
-      <c r="C621" s="7" t="n"/>
-      <c r="D621" s="7" t="inlineStr">
-        <is>
-          <t>OAI22INVCCAD1COTA</t>
-        </is>
-      </c>
+      <c r="A621" s="4" t="n"/>
+      <c r="B621" s="4" t="n"/>
+      <c r="C621" s="5" t="inlineStr">
+        <is>
+          <t>OAI22NR2CCBD4COT</t>
+        </is>
+      </c>
+      <c r="D621" s="5" t="n"/>
     </row>
     <row r="622">
-      <c r="A622" s="2" t="n"/>
-      <c r="B622" s="2" t="inlineStr">
-        <is>
-          <t>OAI22ND2</t>
-        </is>
-      </c>
-      <c r="C622" s="3" t="inlineStr">
-        <is>
-          <t>OAI22ND2CCBD4COT</t>
-        </is>
-      </c>
-      <c r="D622" s="3" t="n"/>
+      <c r="A622" s="4" t="n"/>
+      <c r="B622" s="4" t="n"/>
+      <c r="C622" s="5" t="n"/>
+      <c r="D622" s="5" t="inlineStr">
+        <is>
+          <t>OAI21NR2CCAD2COTA</t>
+        </is>
+      </c>
     </row>
     <row r="623">
-      <c r="A623" s="6" t="n"/>
-      <c r="B623" s="6" t="n"/>
-      <c r="C623" s="7" t="n"/>
-      <c r="D623" s="7" t="inlineStr">
-        <is>
-          <t>OAI22ND2CCBD4COTA</t>
+      <c r="A623" s="4" t="n"/>
+      <c r="B623" s="4" t="n"/>
+      <c r="C623" s="5" t="n"/>
+      <c r="D623" s="5" t="inlineStr">
+        <is>
+          <t>OAI21NR2CCBD1COTA</t>
         </is>
       </c>
     </row>
     <row r="624">
-      <c r="A624" s="2" t="n"/>
-      <c r="B624" s="2" t="inlineStr">
-        <is>
-          <t>OAI22NR2</t>
-        </is>
-      </c>
-      <c r="C624" s="3" t="inlineStr">
-        <is>
-          <t>OAI22NR2CCBD4COT</t>
-        </is>
-      </c>
-      <c r="D624" s="3" t="n"/>
+      <c r="A624" s="6" t="n"/>
+      <c r="B624" s="6" t="n"/>
+      <c r="C624" s="7" t="n"/>
+      <c r="D624" s="7" t="inlineStr">
+        <is>
+          <t>OAI22NR2CCBD4COTA</t>
+        </is>
+      </c>
     </row>
     <row r="625">
-      <c r="A625" s="6" t="n"/>
-      <c r="B625" s="6" t="n"/>
-      <c r="C625" s="7" t="n"/>
-      <c r="D625" s="7" t="inlineStr">
-        <is>
-          <t>OAI22NR2CCBD4COTA</t>
+      <c r="A625" s="2" t="n"/>
+      <c r="B625" s="2" t="inlineStr">
+        <is>
+          <t>OAIOAI
+复合·OAIOAI</t>
+        </is>
+      </c>
+      <c r="C625" s="3" t="n"/>
+      <c r="D625" s="3" t="inlineStr">
+        <is>
+          <t>OAI21OAI21CCBD4COTA</t>
         </is>
       </c>
     </row>
     <row r="626">
-      <c r="A626" s="10" t="n"/>
-      <c r="B626" s="10" t="inlineStr">
-        <is>
-          <t>OAI22OAI21</t>
-        </is>
-      </c>
-      <c r="C626" s="11" t="n"/>
-      <c r="D626" s="11" t="inlineStr">
+      <c r="A626" s="6" t="n"/>
+      <c r="B626" s="6" t="n"/>
+      <c r="C626" s="7" t="n"/>
+      <c r="D626" s="7" t="inlineStr">
         <is>
           <t>OAI22OAI21CCBD1COTA</t>
         </is>
@@ -7357,7 +7324,8 @@
       <c r="A627" s="2" t="n"/>
       <c r="B627" s="2" t="inlineStr">
         <is>
-          <t>OAOI211</t>
+          <t>OAOI
+复合·OAOI</t>
         </is>
       </c>
       <c r="C627" s="8" t="inlineStr">
@@ -7395,7 +7363,8 @@
       <c r="A630" s="2" t="n"/>
       <c r="B630" s="2" t="inlineStr">
         <is>
-          <t>OIAI21</t>
+          <t>OIAI
+复合·OIAI</t>
         </is>
       </c>
       <c r="C630" s="8" t="inlineStr">
@@ -7450,40 +7419,42 @@
       </c>
     </row>
     <row r="635">
-      <c r="A635" s="2" t="n"/>
-      <c r="B635" s="2" t="inlineStr">
-        <is>
-          <t>W2AO22</t>
-        </is>
-      </c>
-      <c r="C635" s="3" t="n"/>
-      <c r="D635" s="3" t="inlineStr">
+      <c r="A635" s="10" t="n"/>
+      <c r="B635" s="10" t="inlineStr">
+        <is>
+          <t>WANOR
+复合·WANOR</t>
+        </is>
+      </c>
+      <c r="C635" s="11" t="n"/>
+      <c r="D635" s="11" t="inlineStr">
+        <is>
+          <t>WAN2OR2COMD1COTA</t>
+        </is>
+      </c>
+    </row>
+    <row r="636">
+      <c r="A636" s="2" t="n"/>
+      <c r="B636" s="2" t="inlineStr">
+        <is>
+          <t>WAO
+复合·WAO</t>
+        </is>
+      </c>
+      <c r="C636" s="3" t="n"/>
+      <c r="D636" s="3" t="inlineStr">
         <is>
           <t>W2AO22D1COT</t>
         </is>
       </c>
     </row>
-    <row r="636">
-      <c r="A636" s="6" t="n"/>
-      <c r="B636" s="6" t="n"/>
-      <c r="C636" s="7" t="n"/>
-      <c r="D636" s="7" t="inlineStr">
+    <row r="637">
+      <c r="A637" s="6" t="n"/>
+      <c r="B637" s="6" t="n"/>
+      <c r="C637" s="7" t="n"/>
+      <c r="D637" s="7" t="inlineStr">
         <is>
           <t>W2AO22D2COT</t>
-        </is>
-      </c>
-    </row>
-    <row r="637">
-      <c r="A637" s="10" t="n"/>
-      <c r="B637" s="10" t="inlineStr">
-        <is>
-          <t>W2AOI22</t>
-        </is>
-      </c>
-      <c r="C637" s="11" t="n"/>
-      <c r="D637" s="11" t="inlineStr">
-        <is>
-          <t>W2AOI22D1COT</t>
         </is>
       </c>
     </row>
@@ -7491,39 +7462,37 @@
       <c r="A638" s="10" t="n"/>
       <c r="B638" s="10" t="inlineStr">
         <is>
-          <t>WAN2OR2</t>
+          <t>WAOI
+复合·WAOI</t>
         </is>
       </c>
       <c r="C638" s="11" t="n"/>
       <c r="D638" s="11" t="inlineStr">
         <is>
-          <t>WAN2OR2COMD1COTA</t>
+          <t>W2AOI22D1COT</t>
         </is>
       </c>
     </row>
     <row r="639">
-      <c r="A639" s="10" t="n"/>
-      <c r="B639" s="10" t="inlineStr">
-        <is>
-          <t>WAO21OA21</t>
-        </is>
-      </c>
-      <c r="C639" s="11" t="n"/>
-      <c r="D639" s="11" t="inlineStr">
+      <c r="A639" s="2" t="n"/>
+      <c r="B639" s="2" t="inlineStr">
+        <is>
+          <t>WAOOA
+复合·WAOOA</t>
+        </is>
+      </c>
+      <c r="C639" s="3" t="n"/>
+      <c r="D639" s="3" t="inlineStr">
         <is>
           <t>WAO21OA21COMD1COTA</t>
         </is>
       </c>
     </row>
     <row r="640">
-      <c r="A640" s="10" t="n"/>
-      <c r="B640" s="10" t="inlineStr">
-        <is>
-          <t>WAO22OA22</t>
-        </is>
-      </c>
-      <c r="C640" s="11" t="n"/>
-      <c r="D640" s="11" t="inlineStr">
+      <c r="A640" s="6" t="n"/>
+      <c r="B640" s="6" t="n"/>
+      <c r="C640" s="7" t="n"/>
+      <c r="D640" s="7" t="inlineStr">
         <is>
           <t>WAO22OA22COMD1COTA</t>
         </is>
@@ -7533,7 +7502,8 @@
       <c r="A641" s="2" t="n"/>
       <c r="B641" s="2" t="inlineStr">
         <is>
-          <t>XNR2AOI21</t>
+          <t>XNRAOI
+复合·XNRAOI</t>
         </is>
       </c>
       <c r="C641" s="3" t="inlineStr">
@@ -7554,35 +7524,31 @@
       <c r="D642" s="5" t="n"/>
     </row>
     <row r="643">
-      <c r="A643" s="6" t="n"/>
-      <c r="B643" s="6" t="n"/>
-      <c r="C643" s="7" t="n"/>
-      <c r="D643" s="7" t="inlineStr">
-        <is>
-          <t>XNR2AOI21D1COTA</t>
-        </is>
-      </c>
+      <c r="A643" s="4" t="n"/>
+      <c r="B643" s="4" t="n"/>
+      <c r="C643" s="5" t="inlineStr">
+        <is>
+          <t>XNR2AOI22D1COTVIAOPTTG</t>
+        </is>
+      </c>
+      <c r="D643" s="5" t="n"/>
     </row>
     <row r="644">
-      <c r="A644" s="2" t="n"/>
-      <c r="B644" s="2" t="inlineStr">
-        <is>
-          <t>XNR2AOI22</t>
-        </is>
-      </c>
-      <c r="C644" s="3" t="inlineStr">
-        <is>
-          <t>XNR2AOI22D1COTVIAOPTTG</t>
-        </is>
-      </c>
-      <c r="D644" s="3" t="n"/>
+      <c r="A644" s="4" t="n"/>
+      <c r="B644" s="4" t="n"/>
+      <c r="C644" s="5" t="inlineStr">
+        <is>
+          <t>XNR2AOI22D2COTOPTTGM3CEQ</t>
+        </is>
+      </c>
+      <c r="D644" s="5" t="n"/>
     </row>
     <row r="645">
       <c r="A645" s="4" t="n"/>
       <c r="B645" s="4" t="n"/>
       <c r="C645" s="5" t="inlineStr">
         <is>
-          <t>XNR2AOI22D2COTOPTTGM3CEQ</t>
+          <t>XNR2AOI22D4COT</t>
         </is>
       </c>
       <c r="D645" s="5" t="n"/>
@@ -7590,12 +7556,12 @@
     <row r="646">
       <c r="A646" s="4" t="n"/>
       <c r="B646" s="4" t="n"/>
-      <c r="C646" s="5" t="inlineStr">
-        <is>
-          <t>XNR2AOI22D4COT</t>
-        </is>
-      </c>
-      <c r="D646" s="5" t="n"/>
+      <c r="C646" s="5" t="n"/>
+      <c r="D646" s="5" t="inlineStr">
+        <is>
+          <t>XNR2AOI21D1COTA</t>
+        </is>
+      </c>
     </row>
     <row r="647">
       <c r="A647" s="6" t="n"/>
@@ -7611,7 +7577,8 @@
       <c r="A648" s="2" t="n"/>
       <c r="B648" s="2" t="inlineStr">
         <is>
-          <t>XNR2ND2</t>
+          <t>XNRND
+复合·XNRND</t>
         </is>
       </c>
       <c r="C648" s="3" t="inlineStr">
@@ -7645,7 +7612,8 @@
       <c r="A651" s="2" t="n"/>
       <c r="B651" s="2" t="inlineStr">
         <is>
-          <t>XNR2NR2</t>
+          <t>XNRNR
+复合·XNRNR</t>
         </is>
       </c>
       <c r="C651" s="3" t="inlineStr">
@@ -7666,32 +7634,29 @@
       <c r="D652" s="7" t="n"/>
     </row>
     <row r="653">
-      <c r="A653" s="10" t="n"/>
-      <c r="B653" s="10" t="inlineStr">
-        <is>
-          <t>XNR2OAI21</t>
-        </is>
-      </c>
-      <c r="C653" s="11" t="inlineStr">
+      <c r="A653" s="2" t="n"/>
+      <c r="B653" s="2" t="inlineStr">
+        <is>
+          <t>XNROAI
+复合·XNROAI</t>
+        </is>
+      </c>
+      <c r="C653" s="3" t="inlineStr">
         <is>
           <t>XNR2OAI21CCBD1COT</t>
         </is>
       </c>
-      <c r="D653" s="11" t="n"/>
+      <c r="D653" s="3" t="n"/>
     </row>
     <row r="654">
-      <c r="A654" s="2" t="n"/>
-      <c r="B654" s="2" t="inlineStr">
-        <is>
-          <t>XNR2OAI22</t>
-        </is>
-      </c>
-      <c r="C654" s="3" t="inlineStr">
+      <c r="A654" s="4" t="n"/>
+      <c r="B654" s="4" t="n"/>
+      <c r="C654" s="5" t="inlineStr">
         <is>
           <t>XNR2OAI22D1COT</t>
         </is>
       </c>
-      <c r="D654" s="3" t="n"/>
+      <c r="D654" s="5" t="n"/>
     </row>
     <row r="655">
       <c r="A655" s="4" t="n"/>
@@ -7727,7 +7692,8 @@
       <c r="A658" s="10" t="n"/>
       <c r="B658" s="10" t="inlineStr">
         <is>
-          <t>XNR2XNR2</t>
+          <t>XNRXNR
+复合·XNRXNR</t>
         </is>
       </c>
       <c r="C658" s="11" t="inlineStr">
@@ -7741,7 +7707,8 @@
       <c r="A659" s="10" t="n"/>
       <c r="B659" s="10" t="inlineStr">
         <is>
-          <t>XNR2XOR2</t>
+          <t>XNRXOR
+复合·XNRXOR</t>
         </is>
       </c>
       <c r="C659" s="11" t="inlineStr">
@@ -7752,32 +7719,29 @@
       <c r="D659" s="11" t="n"/>
     </row>
     <row r="660">
-      <c r="A660" s="10" t="n"/>
-      <c r="B660" s="10" t="inlineStr">
-        <is>
-          <t>XOR2AOI21</t>
-        </is>
-      </c>
-      <c r="C660" s="11" t="inlineStr">
+      <c r="A660" s="2" t="n"/>
+      <c r="B660" s="2" t="inlineStr">
+        <is>
+          <t>XORAOI
+复合·XORAOI</t>
+        </is>
+      </c>
+      <c r="C660" s="3" t="inlineStr">
         <is>
           <t>XOR2AOI21CCBD4COT</t>
         </is>
       </c>
-      <c r="D660" s="11" t="n"/>
+      <c r="D660" s="3" t="n"/>
     </row>
     <row r="661">
-      <c r="A661" s="2" t="n"/>
-      <c r="B661" s="2" t="inlineStr">
-        <is>
-          <t>XOR2AOI22</t>
-        </is>
-      </c>
-      <c r="C661" s="3" t="inlineStr">
+      <c r="A661" s="4" t="n"/>
+      <c r="B661" s="4" t="n"/>
+      <c r="C661" s="5" t="inlineStr">
         <is>
           <t>XOR2AOI22D1COTOPTTG</t>
         </is>
       </c>
-      <c r="D661" s="3" t="n"/>
+      <c r="D661" s="5" t="n"/>
     </row>
     <row r="662">
       <c r="A662" s="4" t="n"/>
@@ -7823,7 +7787,8 @@
       <c r="A666" s="2" t="n"/>
       <c r="B666" s="2" t="inlineStr">
         <is>
-          <t>XOR2ND2</t>
+          <t>XORND
+复合·XORND</t>
         </is>
       </c>
       <c r="C666" s="3" t="inlineStr">
@@ -7867,7 +7832,8 @@
       <c r="A670" s="2" t="n"/>
       <c r="B670" s="2" t="inlineStr">
         <is>
-          <t>XOR2NR2</t>
+          <t>XORNR
+复合·XORNR</t>
         </is>
       </c>
       <c r="C670" s="3" t="inlineStr">
@@ -7898,32 +7864,29 @@
       </c>
     </row>
     <row r="673">
-      <c r="A673" s="10" t="n"/>
-      <c r="B673" s="10" t="inlineStr">
-        <is>
-          <t>XOR2OAI21</t>
-        </is>
-      </c>
-      <c r="C673" s="11" t="inlineStr">
+      <c r="A673" s="2" t="n"/>
+      <c r="B673" s="2" t="inlineStr">
+        <is>
+          <t>XOROAI
+复合·XOROAI</t>
+        </is>
+      </c>
+      <c r="C673" s="3" t="inlineStr">
         <is>
           <t>XOR2OAI21CCBD4COT</t>
         </is>
       </c>
-      <c r="D673" s="11" t="n"/>
+      <c r="D673" s="3" t="n"/>
     </row>
     <row r="674">
-      <c r="A674" s="2" t="n"/>
-      <c r="B674" s="2" t="inlineStr">
-        <is>
-          <t>XOR2OAI22</t>
-        </is>
-      </c>
-      <c r="C674" s="3" t="inlineStr">
+      <c r="A674" s="4" t="n"/>
+      <c r="B674" s="4" t="n"/>
+      <c r="C674" s="5" t="inlineStr">
         <is>
           <t>XOR2OAI22D1COTTGOPU</t>
         </is>
       </c>
-      <c r="D674" s="3" t="n"/>
+      <c r="D674" s="5" t="n"/>
     </row>
     <row r="675">
       <c r="A675" s="4" t="n"/>
@@ -7969,7 +7932,8 @@
       <c r="A679" s="10" t="n"/>
       <c r="B679" s="10" t="inlineStr">
         <is>
-          <t>XOR2XNR2</t>
+          <t>XORXNR
+复合·XORXNR</t>
         </is>
       </c>
       <c r="C679" s="11" t="inlineStr">
@@ -7983,7 +7947,8 @@
       <c r="A680" s="10" t="n"/>
       <c r="B680" s="10" t="inlineStr">
         <is>
-          <t>XOR2XOR2</t>
+          <t>XORXOR
+复合·XORXOR</t>
         </is>
       </c>
       <c r="C680" s="11" t="inlineStr">
@@ -12222,8 +12187,8 @@
       </c>
       <c r="B1072" s="2" t="inlineStr">
         <is>
-          <t>GSDF
-门阵列ECO扫描</t>
+          <t>SCAN
+非Y扫描</t>
         </is>
       </c>
       <c r="C1072" s="8" t="inlineStr">
@@ -12248,96 +12213,81 @@
       <c r="D1073" s="5" t="n"/>
     </row>
     <row r="1074">
-      <c r="A1074" s="6" t="n"/>
-      <c r="B1074" s="6" t="n"/>
-      <c r="C1074" s="7" t="inlineStr">
+      <c r="A1074" s="4" t="n"/>
+      <c r="B1074" s="4" t="n"/>
+      <c r="C1074" s="5" t="inlineStr">
         <is>
           <t>GSDFRPQD1COT</t>
         </is>
       </c>
-      <c r="D1074" s="7" t="n"/>
+      <c r="D1074" s="5" t="n"/>
     </row>
     <row r="1075">
-      <c r="A1075" s="2" t="n"/>
-      <c r="B1075" s="2" t="inlineStr">
-        <is>
-          <t>RSDF
-R扫描SDF</t>
-        </is>
-      </c>
-      <c r="C1075" s="3" t="n"/>
-      <c r="D1075" s="3" t="inlineStr">
-        <is>
-          <t>RSDFQHDCWD1COT</t>
-        </is>
-      </c>
+      <c r="A1075" s="4" t="n"/>
+      <c r="B1075" s="4" t="n"/>
+      <c r="C1075" s="5" t="inlineStr">
+        <is>
+          <t>SDFKRPQD1COTVIASC4LPM3CEQ</t>
+        </is>
+      </c>
+      <c r="D1075" s="5" t="n"/>
     </row>
     <row r="1076">
       <c r="A1076" s="4" t="n"/>
       <c r="B1076" s="4" t="n"/>
-      <c r="C1076" s="5" t="n"/>
-      <c r="D1076" s="5" t="inlineStr">
-        <is>
-          <t>RSDFRPQHDCWD1COT</t>
-        </is>
-      </c>
+      <c r="C1076" s="5" t="inlineStr">
+        <is>
+          <t>SDFKSNQD1COT</t>
+        </is>
+      </c>
+      <c r="D1076" s="5" t="n"/>
     </row>
     <row r="1077">
       <c r="A1077" s="4" t="n"/>
       <c r="B1077" s="4" t="n"/>
-      <c r="C1077" s="5" t="n"/>
-      <c r="D1077" s="5" t="inlineStr">
-        <is>
-          <t>RSDFSNQHDCWD1COT</t>
-        </is>
-      </c>
+      <c r="C1077" s="5" t="inlineStr">
+        <is>
+          <t>SDFKSRPQD4COTOPU</t>
+        </is>
+      </c>
+      <c r="D1077" s="5" t="n"/>
     </row>
     <row r="1078">
-      <c r="A1078" s="6" t="n"/>
-      <c r="B1078" s="6" t="n"/>
-      <c r="C1078" s="7" t="n"/>
-      <c r="D1078" s="7" t="inlineStr">
-        <is>
-          <t>RSDFSRPQHDCWD1COT</t>
-        </is>
-      </c>
+      <c r="A1078" s="4" t="n"/>
+      <c r="B1078" s="4" t="n"/>
+      <c r="C1078" s="5" t="inlineStr">
+        <is>
+          <t>SDFMQD1COT</t>
+        </is>
+      </c>
+      <c r="D1078" s="5" t="n"/>
     </row>
     <row r="1079">
-      <c r="A1079" s="10" t="n"/>
-      <c r="B1079" s="10" t="inlineStr">
-        <is>
-          <t>SD2FF
-SD2FF</t>
-        </is>
-      </c>
-      <c r="C1079" s="11" t="n"/>
-      <c r="D1079" s="11" t="inlineStr">
-        <is>
-          <t>SD2FFQNX4AHQCOTC</t>
-        </is>
-      </c>
+      <c r="A1079" s="4" t="n"/>
+      <c r="B1079" s="4" t="n"/>
+      <c r="C1079" s="5" t="inlineStr">
+        <is>
+          <t>SDFNQD2COTOPU</t>
+        </is>
+      </c>
+      <c r="D1079" s="5" t="n"/>
     </row>
     <row r="1080">
-      <c r="A1080" s="2" t="n"/>
-      <c r="B1080" s="2" t="inlineStr">
-        <is>
-          <t>SDF
-扫描SDF</t>
-        </is>
-      </c>
-      <c r="C1080" s="3" t="inlineStr">
-        <is>
-          <t>SDFKRPQD1COTVIASC4LPM3CEQ</t>
-        </is>
-      </c>
-      <c r="D1080" s="3" t="n"/>
+      <c r="A1080" s="4" t="n"/>
+      <c r="B1080" s="4" t="n"/>
+      <c r="C1080" s="5" t="inlineStr">
+        <is>
+          <t>SDFNQND2COTOPU</t>
+        </is>
+      </c>
+      <c r="D1080" s="5" t="n"/>
     </row>
     <row r="1081">
       <c r="A1081" s="4" t="n"/>
       <c r="B1081" s="4" t="n"/>
       <c r="C1081" s="5" t="inlineStr">
         <is>
-          <t>SDFKSNQD1COT</t>
+          <t>SDFNRPQD4COT</t>
         </is>
       </c>
       <c r="D1081" s="5" t="n"/>
@@ -12347,7 +12297,7 @@
       <c r="B1082" s="4" t="n"/>
       <c r="C1082" s="5" t="inlineStr">
         <is>
-          <t>SDFKSRPQD4COTOPU</t>
+          <t>SDFNRPQND2COTMVM3OPU</t>
         </is>
       </c>
       <c r="D1082" s="5" t="n"/>
@@ -12357,7 +12307,7 @@
       <c r="B1083" s="4" t="n"/>
       <c r="C1083" s="5" t="inlineStr">
         <is>
-          <t>SDFMQD1COT</t>
+          <t>SDFNSNQD2COT</t>
         </is>
       </c>
       <c r="D1083" s="5" t="n"/>
@@ -12367,7 +12317,7 @@
       <c r="B1084" s="4" t="n"/>
       <c r="C1084" s="5" t="inlineStr">
         <is>
-          <t>SDFNQD2COTOPU</t>
+          <t>SDFNSNQND1COTM3CEQ</t>
         </is>
       </c>
       <c r="D1084" s="5" t="n"/>
@@ -12377,7 +12327,7 @@
       <c r="B1085" s="4" t="n"/>
       <c r="C1085" s="5" t="inlineStr">
         <is>
-          <t>SDFNQND2COTOPU</t>
+          <t>SDFNSRPQD4COT</t>
         </is>
       </c>
       <c r="D1085" s="5" t="n"/>
@@ -12387,7 +12337,7 @@
       <c r="B1086" s="4" t="n"/>
       <c r="C1086" s="5" t="inlineStr">
         <is>
-          <t>SDFNRPQD4COT</t>
+          <t>SDFQD2COTOPTTMIM3CEQ</t>
         </is>
       </c>
       <c r="D1086" s="5" t="n"/>
@@ -12397,7 +12347,7 @@
       <c r="B1087" s="4" t="n"/>
       <c r="C1087" s="5" t="inlineStr">
         <is>
-          <t>SDFNRPQND2COTMVM3OPU</t>
+          <t>SDFQND1COT</t>
         </is>
       </c>
       <c r="D1087" s="5" t="n"/>
@@ -12407,7 +12357,7 @@
       <c r="B1088" s="4" t="n"/>
       <c r="C1088" s="5" t="inlineStr">
         <is>
-          <t>SDFNSNQD2COT</t>
+          <t>SDFRPQD4COTOPTBB</t>
         </is>
       </c>
       <c r="D1088" s="5" t="n"/>
@@ -12417,7 +12367,7 @@
       <c r="B1089" s="4" t="n"/>
       <c r="C1089" s="5" t="inlineStr">
         <is>
-          <t>SDFNSNQND1COTM3CEQ</t>
+          <t>SDFRPQND4COTOPU</t>
         </is>
       </c>
       <c r="D1089" s="5" t="n"/>
@@ -12427,7 +12377,7 @@
       <c r="B1090" s="4" t="n"/>
       <c r="C1090" s="5" t="inlineStr">
         <is>
-          <t>SDFNSRPQD4COT</t>
+          <t>SDFSNQD8COTOPTBBM3CEQ</t>
         </is>
       </c>
       <c r="D1090" s="5" t="n"/>
@@ -12437,7 +12387,7 @@
       <c r="B1091" s="4" t="n"/>
       <c r="C1091" s="5" t="inlineStr">
         <is>
-          <t>SDFQD2COTOPTTMIM3CEQ</t>
+          <t>SDFSNQND4COTOPU</t>
         </is>
       </c>
       <c r="D1091" s="5" t="n"/>
@@ -12447,7 +12397,7 @@
       <c r="B1092" s="4" t="n"/>
       <c r="C1092" s="5" t="inlineStr">
         <is>
-          <t>SDFQND1COT</t>
+          <t>SDFSRPQD2COT</t>
         </is>
       </c>
       <c r="D1092" s="5" t="n"/>
@@ -12457,7 +12407,7 @@
       <c r="B1093" s="4" t="n"/>
       <c r="C1093" s="5" t="inlineStr">
         <is>
-          <t>SDFRPQD4COTOPTBB</t>
+          <t>SEDFQD1COT</t>
         </is>
       </c>
       <c r="D1093" s="5" t="n"/>
@@ -12467,7 +12417,7 @@
       <c r="B1094" s="4" t="n"/>
       <c r="C1094" s="5" t="inlineStr">
         <is>
-          <t>SDFRPQND4COTOPU</t>
+          <t>SEDFRPQD2COT</t>
         </is>
       </c>
       <c r="D1094" s="5" t="n"/>
@@ -12475,32 +12425,32 @@
     <row r="1095">
       <c r="A1095" s="4" t="n"/>
       <c r="B1095" s="4" t="n"/>
-      <c r="C1095" s="5" t="inlineStr">
-        <is>
-          <t>SDFSNQD8COTOPTBBM3CEQ</t>
-        </is>
-      </c>
-      <c r="D1095" s="5" t="n"/>
+      <c r="C1095" s="5" t="n"/>
+      <c r="D1095" s="5" t="inlineStr">
+        <is>
+          <t>RSDFQHDCWD1COT</t>
+        </is>
+      </c>
     </row>
     <row r="1096">
       <c r="A1096" s="4" t="n"/>
       <c r="B1096" s="4" t="n"/>
-      <c r="C1096" s="5" t="inlineStr">
-        <is>
-          <t>SDFSNQND4COTOPU</t>
-        </is>
-      </c>
-      <c r="D1096" s="5" t="n"/>
+      <c r="C1096" s="5" t="n"/>
+      <c r="D1096" s="5" t="inlineStr">
+        <is>
+          <t>RSDFRPQHDCWD1COT</t>
+        </is>
+      </c>
     </row>
     <row r="1097">
       <c r="A1097" s="4" t="n"/>
       <c r="B1097" s="4" t="n"/>
-      <c r="C1097" s="5" t="inlineStr">
-        <is>
-          <t>SDFSRPQD2COT</t>
-        </is>
-      </c>
-      <c r="D1097" s="5" t="n"/>
+      <c r="C1097" s="5" t="n"/>
+      <c r="D1097" s="5" t="inlineStr">
+        <is>
+          <t>RSDFSNQHDCWD1COT</t>
+        </is>
+      </c>
     </row>
     <row r="1098">
       <c r="A1098" s="4" t="n"/>
@@ -12508,7 +12458,7 @@
       <c r="C1098" s="5" t="n"/>
       <c r="D1098" s="5" t="inlineStr">
         <is>
-          <t>SDFKRPQD2ONECOT</t>
+          <t>RSDFSRPQHDCWD1COT</t>
         </is>
       </c>
     </row>
@@ -12518,7 +12468,7 @@
       <c r="C1099" s="5" t="n"/>
       <c r="D1099" s="5" t="inlineStr">
         <is>
-          <t>SDFKSRPQEEQMBDD2COT</t>
+          <t>SD2FFQNX4AHQCOTC</t>
         </is>
       </c>
     </row>
@@ -12528,7 +12478,7 @@
       <c r="C1100" s="5" t="n"/>
       <c r="D1100" s="5" t="inlineStr">
         <is>
-          <t>SDFMQD6COT</t>
+          <t>SDFFACPQX4ASBCOTC</t>
         </is>
       </c>
     </row>
@@ -12538,7 +12488,7 @@
       <c r="C1101" s="5" t="n"/>
       <c r="D1101" s="5" t="inlineStr">
         <is>
-          <t>SDFNQD0COT</t>
+          <t>SDFFASNQX2ATBCOTC</t>
         </is>
       </c>
     </row>
@@ -12548,7 +12498,7 @@
       <c r="C1102" s="5" t="n"/>
       <c r="D1102" s="5" t="inlineStr">
         <is>
-          <t>SDFNRPQND2COT</t>
+          <t>SDFFQNX0P5AHCCOTC</t>
         </is>
       </c>
     </row>
@@ -12558,7 +12508,7 @@
       <c r="C1103" s="5" t="n"/>
       <c r="D1103" s="5" t="inlineStr">
         <is>
-          <t>SDFNSNQD1COT</t>
+          <t>SDFFQNX0P5AHQCOTC</t>
         </is>
       </c>
     </row>
@@ -12568,7 +12518,7 @@
       <c r="C1104" s="5" t="n"/>
       <c r="D1104" s="5" t="inlineStr">
         <is>
-          <t>SDFNSNQND0COT</t>
+          <t>SDFFQNX4AHBCOTC</t>
         </is>
       </c>
     </row>
@@ -12578,7 +12528,7 @@
       <c r="C1105" s="5" t="n"/>
       <c r="D1105" s="5" t="inlineStr">
         <is>
-          <t>SDFQND2COT</t>
+          <t>SDFFQNX4AHQCOTC</t>
         </is>
       </c>
     </row>
@@ -12588,7 +12538,7 @@
       <c r="C1106" s="5" t="n"/>
       <c r="D1106" s="5" t="inlineStr">
         <is>
-          <t>SDFQOPTBBOPTLD4COT</t>
+          <t>SDFFQX1ASBCOTC</t>
         </is>
       </c>
     </row>
@@ -12598,7 +12548,7 @@
       <c r="C1107" s="5" t="n"/>
       <c r="D1107" s="5" t="inlineStr">
         <is>
-          <t>SDFQOPTBCUSS1D2COT</t>
+          <t>SDFFQX4ATBCOTC</t>
         </is>
       </c>
     </row>
@@ -12608,7 +12558,7 @@
       <c r="C1108" s="5" t="n"/>
       <c r="D1108" s="5" t="inlineStr">
         <is>
-          <t>SDFQOPTQD6COT</t>
+          <t>SDFFQX6AHCCOTC</t>
         </is>
       </c>
     </row>
@@ -12618,7 +12568,7 @@
       <c r="C1109" s="5" t="n"/>
       <c r="D1109" s="5" t="inlineStr">
         <is>
-          <t>SDFQOPTSV1D1COT</t>
+          <t>SDFFQX8COTC</t>
         </is>
       </c>
     </row>
@@ -12628,7 +12578,7 @@
       <c r="C1110" s="5" t="n"/>
       <c r="D1110" s="5" t="inlineStr">
         <is>
-          <t>SDFRPQD1COT</t>
+          <t>SDFKRPQD2ONECOT</t>
         </is>
       </c>
     </row>
@@ -12638,7 +12588,7 @@
       <c r="C1111" s="5" t="n"/>
       <c r="D1111" s="5" t="inlineStr">
         <is>
-          <t>SDFRPQOPTQD8COT</t>
+          <t>SDFKSRPQEEQMBDD2COT</t>
         </is>
       </c>
     </row>
@@ -12648,7 +12598,7 @@
       <c r="C1112" s="5" t="n"/>
       <c r="D1112" s="5" t="inlineStr">
         <is>
-          <t>SDFRPQOPTQV3D8COT</t>
+          <t>SDFMQD6COT</t>
         </is>
       </c>
     </row>
@@ -12658,7 +12608,7 @@
       <c r="C1113" s="5" t="n"/>
       <c r="D1113" s="5" t="inlineStr">
         <is>
-          <t>SDFRPQOPTQV4D8COT</t>
+          <t>SDFNQD0COT</t>
         </is>
       </c>
     </row>
@@ -12668,7 +12618,7 @@
       <c r="C1114" s="5" t="n"/>
       <c r="D1114" s="5" t="inlineStr">
         <is>
-          <t>SDFRPQOPTSV1D2COT</t>
+          <t>SDFNRPQND2COT</t>
         </is>
       </c>
     </row>
@@ -12678,32 +12628,27 @@
       <c r="C1115" s="5" t="n"/>
       <c r="D1115" s="5" t="inlineStr">
         <is>
-          <t>SDFSNQND2COT</t>
+          <t>SDFNSNQD1COT</t>
         </is>
       </c>
     </row>
     <row r="1116">
-      <c r="A1116" s="6" t="n"/>
-      <c r="B1116" s="6" t="n"/>
-      <c r="C1116" s="7" t="n"/>
-      <c r="D1116" s="7" t="inlineStr">
-        <is>
-          <t>SDFSRPQEEQMBDD1COT</t>
+      <c r="A1116" s="4" t="n"/>
+      <c r="B1116" s="4" t="n"/>
+      <c r="C1116" s="5" t="n"/>
+      <c r="D1116" s="5" t="inlineStr">
+        <is>
+          <t>SDFNSNQND0COT</t>
         </is>
       </c>
     </row>
     <row r="1117">
-      <c r="A1117" s="2" t="n"/>
-      <c r="B1117" s="2" t="inlineStr">
-        <is>
-          <t>SDFF
-扫描SDFF</t>
-        </is>
-      </c>
-      <c r="C1117" s="3" t="n"/>
-      <c r="D1117" s="3" t="inlineStr">
-        <is>
-          <t>SDFFACPQX4ASBCOTC</t>
+      <c r="A1117" s="4" t="n"/>
+      <c r="B1117" s="4" t="n"/>
+      <c r="C1117" s="5" t="n"/>
+      <c r="D1117" s="5" t="inlineStr">
+        <is>
+          <t>SDFQND2COT</t>
         </is>
       </c>
     </row>
@@ -12713,7 +12658,7 @@
       <c r="C1118" s="5" t="n"/>
       <c r="D1118" s="5" t="inlineStr">
         <is>
-          <t>SDFFASNQX2ATBCOTC</t>
+          <t>SDFQOPTBBOPTLD4COT</t>
         </is>
       </c>
     </row>
@@ -12723,7 +12668,7 @@
       <c r="C1119" s="5" t="n"/>
       <c r="D1119" s="5" t="inlineStr">
         <is>
-          <t>SDFFQNX0P5AHCCOTC</t>
+          <t>SDFQOPTBCUSS1D2COT</t>
         </is>
       </c>
     </row>
@@ -12733,7 +12678,7 @@
       <c r="C1120" s="5" t="n"/>
       <c r="D1120" s="5" t="inlineStr">
         <is>
-          <t>SDFFQNX0P5AHQCOTC</t>
+          <t>SDFQOPTQD6COT</t>
         </is>
       </c>
     </row>
@@ -12743,7 +12688,7 @@
       <c r="C1121" s="5" t="n"/>
       <c r="D1121" s="5" t="inlineStr">
         <is>
-          <t>SDFFQNX4AHBCOTC</t>
+          <t>SDFQOPTSV1D1COT</t>
         </is>
       </c>
     </row>
@@ -12753,7 +12698,7 @@
       <c r="C1122" s="5" t="n"/>
       <c r="D1122" s="5" t="inlineStr">
         <is>
-          <t>SDFFQNX4AHQCOTC</t>
+          <t>SDFRPQD1COT</t>
         </is>
       </c>
     </row>
@@ -12763,7 +12708,7 @@
       <c r="C1123" s="5" t="n"/>
       <c r="D1123" s="5" t="inlineStr">
         <is>
-          <t>SDFFQX1ASBCOTC</t>
+          <t>SDFRPQOPTQD8COT</t>
         </is>
       </c>
     </row>
@@ -12773,7 +12718,7 @@
       <c r="C1124" s="5" t="n"/>
       <c r="D1124" s="5" t="inlineStr">
         <is>
-          <t>SDFFQX4ATBCOTC</t>
+          <t>SDFRPQOPTQV3D8COT</t>
         </is>
       </c>
     </row>
@@ -12783,44 +12728,39 @@
       <c r="C1125" s="5" t="n"/>
       <c r="D1125" s="5" t="inlineStr">
         <is>
-          <t>SDFFQX6AHCCOTC</t>
+          <t>SDFRPQOPTQV4D8COT</t>
         </is>
       </c>
     </row>
     <row r="1126">
-      <c r="A1126" s="6" t="n"/>
-      <c r="B1126" s="6" t="n"/>
-      <c r="C1126" s="7" t="n"/>
-      <c r="D1126" s="7" t="inlineStr">
-        <is>
-          <t>SDFFQX8COTC</t>
+      <c r="A1126" s="4" t="n"/>
+      <c r="B1126" s="4" t="n"/>
+      <c r="C1126" s="5" t="n"/>
+      <c r="D1126" s="5" t="inlineStr">
+        <is>
+          <t>SDFRPQOPTSV1D2COT</t>
         </is>
       </c>
     </row>
     <row r="1127">
-      <c r="A1127" s="2" t="n"/>
-      <c r="B1127" s="2" t="inlineStr">
-        <is>
-          <t>SEDF
-使能扫描EDF</t>
-        </is>
-      </c>
-      <c r="C1127" s="3" t="inlineStr">
-        <is>
-          <t>SEDFQD1COT</t>
-        </is>
-      </c>
-      <c r="D1127" s="3" t="n"/>
+      <c r="A1127" s="4" t="n"/>
+      <c r="B1127" s="4" t="n"/>
+      <c r="C1127" s="5" t="n"/>
+      <c r="D1127" s="5" t="inlineStr">
+        <is>
+          <t>SDFSNQND2COT</t>
+        </is>
+      </c>
     </row>
     <row r="1128">
       <c r="A1128" s="4" t="n"/>
       <c r="B1128" s="4" t="n"/>
-      <c r="C1128" s="5" t="inlineStr">
-        <is>
-          <t>SEDFRPQD2COT</t>
-        </is>
-      </c>
-      <c r="D1128" s="5" t="n"/>
+      <c r="C1128" s="5" t="n"/>
+      <c r="D1128" s="5" t="inlineStr">
+        <is>
+          <t>SDFSRPQEEQMBDD1COT</t>
+        </is>
+      </c>
     </row>
     <row r="1129">
       <c r="A1129" s="4" t="n"/>
@@ -12846,8 +12786,8 @@
       <c r="A1131" s="2" t="n"/>
       <c r="B1131" s="2" t="inlineStr">
         <is>
-          <t>YSDF
-Y扫描SDF</t>
+          <t>YSCAN
+Y系列</t>
         </is>
       </c>
       <c r="C1131" s="3" t="inlineStr">
@@ -12928,25 +12868,20 @@
       <c r="D1138" s="5" t="n"/>
     </row>
     <row r="1139">
-      <c r="A1139" s="6" t="n"/>
-      <c r="B1139" s="6" t="n"/>
-      <c r="C1139" s="7" t="inlineStr">
+      <c r="A1139" s="4" t="n"/>
+      <c r="B1139" s="4" t="n"/>
+      <c r="C1139" s="5" t="inlineStr">
         <is>
           <t>YSDFSNQD1COT</t>
         </is>
       </c>
-      <c r="D1139" s="7" t="n"/>
+      <c r="D1139" s="5" t="n"/>
     </row>
     <row r="1140">
-      <c r="A1140" s="2" t="n"/>
-      <c r="B1140" s="2" t="inlineStr">
-        <is>
-          <t>YSDFF
-Y扫描SDFF</t>
-        </is>
-      </c>
-      <c r="C1140" s="3" t="n"/>
-      <c r="D1140" s="3" t="inlineStr">
+      <c r="A1140" s="4" t="n"/>
+      <c r="B1140" s="4" t="n"/>
+      <c r="C1140" s="5" t="n"/>
+      <c r="D1140" s="5" t="inlineStr">
         <is>
           <t>Y2SDFFQX1COTC</t>
         </is>
@@ -12970,7 +12905,7 @@
       </c>
       <c r="B1142" s="2" t="inlineStr">
         <is>
-          <t>CKAN2</t>
+          <t>CKAN</t>
         </is>
       </c>
       <c r="C1142" s="8" t="inlineStr">
@@ -13046,7 +12981,7 @@
       </c>
       <c r="B1148" s="2" t="inlineStr">
         <is>
-          <t>CKND2</t>
+          <t>CKND</t>
         </is>
       </c>
       <c r="C1148" s="3" t="inlineStr">
@@ -13142,7 +13077,7 @@
       </c>
       <c r="B1156" s="2" t="inlineStr">
         <is>
-          <t>CKMUX2</t>
+          <t>CKMUX</t>
         </is>
       </c>
       <c r="C1156" s="8" t="inlineStr">
@@ -13228,7 +13163,7 @@
       </c>
       <c r="B1163" s="2" t="inlineStr">
         <is>
-          <t>CKXOR2</t>
+          <t>CKXOR</t>
         </is>
       </c>
       <c r="C1163" s="8" t="inlineStr">
@@ -13290,7 +13225,7 @@
       </c>
       <c r="B1168" s="2" t="inlineStr">
         <is>
-          <t>CKOR2</t>
+          <t>CKOR</t>
         </is>
       </c>
       <c r="C1168" s="8" t="inlineStr">
@@ -13350,7 +13285,7 @@
       </c>
       <c r="B1172" s="2" t="inlineStr">
         <is>
-          <t>CKNR2</t>
+          <t>CKNR</t>
         </is>
       </c>
       <c r="C1172" s="8" t="inlineStr">
@@ -13499,8 +13434,8 @@
       </c>
       <c r="B1183" s="2" t="inlineStr">
         <is>
-          <t>CKLHQ
-高电平</t>
+          <t>LH
+高电平透明</t>
         </is>
       </c>
       <c r="C1183" s="3" t="inlineStr">
@@ -13521,69 +13456,59 @@
       </c>
     </row>
     <row r="1185">
-      <c r="A1185" s="10" t="n"/>
-      <c r="B1185" s="10" t="inlineStr">
-        <is>
-          <t>CKLNCNQ
-低电平·带CN</t>
-        </is>
-      </c>
-      <c r="C1185" s="11" t="inlineStr">
+      <c r="A1185" s="2" t="n"/>
+      <c r="B1185" s="2" t="inlineStr">
+        <is>
+          <t>LN
+低电平透明</t>
+        </is>
+      </c>
+      <c r="C1185" s="3" t="inlineStr">
         <is>
           <t>CKLNCNQD14COT</t>
         </is>
       </c>
-      <c r="D1185" s="11" t="n"/>
+      <c r="D1185" s="3" t="n"/>
     </row>
     <row r="1186">
-      <c r="A1186" s="2" t="n"/>
-      <c r="B1186" s="2" t="inlineStr">
-        <is>
-          <t>CKLNQ
-低电平</t>
-        </is>
-      </c>
-      <c r="C1186" s="3" t="inlineStr">
+      <c r="A1186" s="4" t="n"/>
+      <c r="B1186" s="4" t="n"/>
+      <c r="C1186" s="5" t="inlineStr">
         <is>
           <t>CKLNQD14COTOPTBB</t>
         </is>
       </c>
-      <c r="D1186" s="3" t="n"/>
+      <c r="D1186" s="5" t="n"/>
     </row>
     <row r="1187">
       <c r="A1187" s="4" t="n"/>
       <c r="B1187" s="4" t="n"/>
-      <c r="C1187" s="5" t="n"/>
-      <c r="D1187" s="5" t="inlineStr">
+      <c r="C1187" s="5" t="inlineStr">
+        <is>
+          <t>GCKLNQD2COT</t>
+        </is>
+      </c>
+      <c r="D1187" s="5" t="n"/>
+    </row>
+    <row r="1188">
+      <c r="A1188" s="4" t="n"/>
+      <c r="B1188" s="4" t="n"/>
+      <c r="C1188" s="5" t="n"/>
+      <c r="D1188" s="5" t="inlineStr">
         <is>
           <t>CKLNQD1MECOT</t>
         </is>
       </c>
     </row>
-    <row r="1188">
-      <c r="A1188" s="6" t="n"/>
-      <c r="B1188" s="6" t="n"/>
-      <c r="C1188" s="7" t="n"/>
-      <c r="D1188" s="7" t="inlineStr">
+    <row r="1189">
+      <c r="A1189" s="6" t="n"/>
+      <c r="B1189" s="6" t="n"/>
+      <c r="C1189" s="7" t="n"/>
+      <c r="D1189" s="7" t="inlineStr">
         <is>
           <t>CKLNQOPTBBD14COT</t>
         </is>
       </c>
-    </row>
-    <row r="1189">
-      <c r="A1189" s="10" t="n"/>
-      <c r="B1189" s="10" t="inlineStr">
-        <is>
-          <t>GCKLNQ
-门阵列ECO</t>
-        </is>
-      </c>
-      <c r="C1189" s="11" t="inlineStr">
-        <is>
-          <t>GCKLNQD2COT</t>
-        </is>
-      </c>
-      <c r="D1189" s="11" t="n"/>
     </row>
     <row r="1190">
       <c r="A1190" s="10" t="inlineStr">
@@ -13604,40 +13529,45 @@
       <c r="D1190" s="11" t="n"/>
     </row>
     <row r="1191">
-      <c r="A1191" s="2" t="inlineStr">
+      <c r="A1191" s="10" t="inlineStr">
         <is>
           <t>电平转换器</t>
         </is>
       </c>
-      <c r="B1191" s="2" t="inlineStr">
-        <is>
-          <t>CKLVL
+      <c r="B1191" s="10" t="inlineStr">
+        <is>
+          <t>CKLVU
 时钟域</t>
         </is>
       </c>
-      <c r="C1191" s="3" t="inlineStr">
+      <c r="C1191" s="11" t="n"/>
+      <c r="D1191" s="11" t="inlineStr">
+        <is>
+          <t>CKLVUX6COTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1192">
+      <c r="A1192" s="2" t="n"/>
+      <c r="B1192" s="2" t="inlineStr">
+        <is>
+          <t>LH
+高电平透明</t>
+        </is>
+      </c>
+      <c r="C1192" s="3" t="inlineStr">
         <is>
           <t>CKLVLLHBUFFSNKD6COT</t>
         </is>
       </c>
-      <c r="D1191" s="3" t="n"/>
-    </row>
-    <row r="1192">
-      <c r="A1192" s="4" t="n"/>
-      <c r="B1192" s="4" t="n"/>
-      <c r="C1192" s="5" t="inlineStr">
-        <is>
-          <t>CKLVLLHBUFFSRCD2COT</t>
-        </is>
-      </c>
-      <c r="D1192" s="5" t="n"/>
+      <c r="D1192" s="3" t="n"/>
     </row>
     <row r="1193">
       <c r="A1193" s="4" t="n"/>
       <c r="B1193" s="4" t="n"/>
       <c r="C1193" s="5" t="inlineStr">
         <is>
-          <t>CKLVLLHCHSNKD2COT</t>
+          <t>CKLVLLHBUFFSRCD2COT</t>
         </is>
       </c>
       <c r="D1193" s="5" t="n"/>
@@ -13647,7 +13577,7 @@
       <c r="B1194" s="4" t="n"/>
       <c r="C1194" s="5" t="inlineStr">
         <is>
-          <t>CKLVLLHCHSRCD4COT</t>
+          <t>CKLVLLHCHSNKD2COT</t>
         </is>
       </c>
       <c r="D1194" s="5" t="n"/>
@@ -13657,50 +13587,40 @@
       <c r="B1195" s="4" t="n"/>
       <c r="C1195" s="5" t="inlineStr">
         <is>
+          <t>CKLVLLHCHSRCD4COT</t>
+        </is>
+      </c>
+      <c r="D1195" s="5" t="n"/>
+    </row>
+    <row r="1196">
+      <c r="A1196" s="4" t="n"/>
+      <c r="B1196" s="4" t="n"/>
+      <c r="C1196" s="5" t="inlineStr">
+        <is>
           <t>CKLVLLHCLSNKD4COT</t>
         </is>
       </c>
-      <c r="D1195" s="5" t="n"/>
-    </row>
-    <row r="1196">
-      <c r="A1196" s="6" t="n"/>
-      <c r="B1196" s="6" t="n"/>
-      <c r="C1196" s="7" t="inlineStr">
+      <c r="D1196" s="5" t="n"/>
+    </row>
+    <row r="1197">
+      <c r="A1197" s="4" t="n"/>
+      <c r="B1197" s="4" t="n"/>
+      <c r="C1197" s="5" t="inlineStr">
         <is>
           <t>CKLVLLHCLSRCD2COT</t>
         </is>
       </c>
-      <c r="D1196" s="7" t="n"/>
-    </row>
-    <row r="1197">
-      <c r="A1197" s="10" t="n"/>
-      <c r="B1197" s="10" t="inlineStr">
-        <is>
-          <t>CKLVU
-时钟域</t>
-        </is>
-      </c>
-      <c r="C1197" s="11" t="n"/>
-      <c r="D1197" s="11" t="inlineStr">
-        <is>
-          <t>CKLVUX6COTC</t>
-        </is>
-      </c>
+      <c r="D1197" s="5" t="n"/>
     </row>
     <row r="1198">
-      <c r="A1198" s="2" t="n"/>
-      <c r="B1198" s="2" t="inlineStr">
-        <is>
-          <t>LVL
-LVL系列</t>
-        </is>
-      </c>
-      <c r="C1198" s="3" t="inlineStr">
+      <c r="A1198" s="4" t="n"/>
+      <c r="B1198" s="4" t="n"/>
+      <c r="C1198" s="5" t="inlineStr">
         <is>
           <t>LVLHLBUFFSNKD2COT</t>
         </is>
       </c>
-      <c r="D1198" s="3" t="n"/>
+      <c r="D1198" s="5" t="n"/>
     </row>
     <row r="1199">
       <c r="A1199" s="4" t="n"/>
@@ -14863,143 +14783,103 @@
       </c>
     </row>
     <row r="1302">
-      <c r="A1302" s="10" t="inlineStr">
+      <c r="A1302" s="2" t="inlineStr">
         <is>
           <t>锁存器</t>
         </is>
       </c>
-      <c r="B1302" s="10" t="inlineStr">
-        <is>
-          <t>GLAHQ
-门阵列·AH</t>
-        </is>
-      </c>
-      <c r="C1302" s="11" t="n"/>
-      <c r="D1302" s="11" t="inlineStr">
+      <c r="B1302" s="2" t="inlineStr">
+        <is>
+          <t>LH
+高电平透明</t>
+        </is>
+      </c>
+      <c r="C1302" s="3" t="inlineStr">
+        <is>
+          <t>GLHCNQD1COT</t>
+        </is>
+      </c>
+      <c r="D1302" s="3" t="n"/>
+    </row>
+    <row r="1303">
+      <c r="A1303" s="4" t="n"/>
+      <c r="B1303" s="4" t="n"/>
+      <c r="C1303" s="5" t="inlineStr">
+        <is>
+          <t>GLHQD1COT</t>
+        </is>
+      </c>
+      <c r="D1303" s="5" t="n"/>
+    </row>
+    <row r="1304">
+      <c r="A1304" s="4" t="n"/>
+      <c r="B1304" s="4" t="n"/>
+      <c r="C1304" s="5" t="inlineStr">
+        <is>
+          <t>LHCNQD4COTVIAOPPM3CEQ</t>
+        </is>
+      </c>
+      <c r="D1304" s="5" t="n"/>
+    </row>
+    <row r="1305">
+      <c r="A1305" s="4" t="n"/>
+      <c r="B1305" s="4" t="n"/>
+      <c r="C1305" s="5" t="inlineStr">
+        <is>
+          <t>LHCSNQD4COT</t>
+        </is>
+      </c>
+      <c r="D1305" s="5" t="n"/>
+    </row>
+    <row r="1306">
+      <c r="A1306" s="4" t="n"/>
+      <c r="B1306" s="4" t="n"/>
+      <c r="C1306" s="5" t="inlineStr">
+        <is>
+          <t>LHQD2COTOPP</t>
+        </is>
+      </c>
+      <c r="D1306" s="5" t="n"/>
+    </row>
+    <row r="1307">
+      <c r="A1307" s="4" t="n"/>
+      <c r="B1307" s="4" t="n"/>
+      <c r="C1307" s="5" t="inlineStr">
+        <is>
+          <t>LHSNQD2COT</t>
+        </is>
+      </c>
+      <c r="D1307" s="5" t="n"/>
+    </row>
+    <row r="1308">
+      <c r="A1308" s="4" t="n"/>
+      <c r="B1308" s="4" t="n"/>
+      <c r="C1308" s="5" t="n"/>
+      <c r="D1308" s="5" t="inlineStr">
         <is>
           <t>GLAHQD1COT</t>
         </is>
       </c>
     </row>
-    <row r="1303">
-      <c r="A1303" s="10" t="n"/>
-      <c r="B1303" s="10" t="inlineStr">
-        <is>
-          <t>GLAHRNQ
-门阵列·AH·RNQ</t>
-        </is>
-      </c>
-      <c r="C1303" s="11" t="n"/>
-      <c r="D1303" s="11" t="inlineStr">
+    <row r="1309">
+      <c r="A1309" s="4" t="n"/>
+      <c r="B1309" s="4" t="n"/>
+      <c r="C1309" s="5" t="n"/>
+      <c r="D1309" s="5" t="inlineStr">
         <is>
           <t>GLAHRNQD1COT</t>
         </is>
       </c>
     </row>
-    <row r="1304">
-      <c r="A1304" s="10" t="n"/>
-      <c r="B1304" s="10" t="inlineStr">
-        <is>
-          <t>GLHCNQ
-门阵列·高·CNQ</t>
-        </is>
-      </c>
-      <c r="C1304" s="11" t="inlineStr">
-        <is>
-          <t>GLHCNQD1COT</t>
-        </is>
-      </c>
-      <c r="D1304" s="11" t="n"/>
-    </row>
-    <row r="1305">
-      <c r="A1305" s="10" t="n"/>
-      <c r="B1305" s="10" t="inlineStr">
-        <is>
-          <t>GLHQ
-门阵列·高</t>
-        </is>
-      </c>
-      <c r="C1305" s="11" t="inlineStr">
-        <is>
-          <t>GLHQD1COT</t>
-        </is>
-      </c>
-      <c r="D1305" s="11" t="n"/>
-    </row>
-    <row r="1306">
-      <c r="A1306" s="10" t="n"/>
-      <c r="B1306" s="10" t="inlineStr">
-        <is>
-          <t>GLNCNQ
-门阵列·低·CNQ</t>
-        </is>
-      </c>
-      <c r="C1306" s="11" t="inlineStr">
-        <is>
-          <t>GLNCNQD1COT</t>
-        </is>
-      </c>
-      <c r="D1306" s="11" t="n"/>
-    </row>
-    <row r="1307">
-      <c r="A1307" s="10" t="n"/>
-      <c r="B1307" s="10" t="inlineStr">
-        <is>
-          <t>GLNQ
-门阵列·低</t>
-        </is>
-      </c>
-      <c r="C1307" s="11" t="inlineStr">
-        <is>
-          <t>GLNQD1COT</t>
-        </is>
-      </c>
-      <c r="D1307" s="11" t="n"/>
-    </row>
-    <row r="1308">
-      <c r="A1308" s="10" t="n"/>
-      <c r="B1308" s="10" t="inlineStr">
-        <is>
-          <t>LHCNQ
-高·CNQ</t>
-        </is>
-      </c>
-      <c r="C1308" s="11" t="inlineStr">
-        <is>
-          <t>LHCNQD4COTVIAOPPM3CEQ</t>
-        </is>
-      </c>
-      <c r="D1308" s="11" t="n"/>
-    </row>
-    <row r="1309">
-      <c r="A1309" s="10" t="n"/>
-      <c r="B1309" s="10" t="inlineStr">
-        <is>
-          <t>LHCSNQ
-高·CSNQ</t>
-        </is>
-      </c>
-      <c r="C1309" s="11" t="inlineStr">
-        <is>
-          <t>LHCSNQD4COT</t>
-        </is>
-      </c>
-      <c r="D1309" s="11" t="n"/>
-    </row>
     <row r="1310">
-      <c r="A1310" s="2" t="n"/>
-      <c r="B1310" s="2" t="inlineStr">
-        <is>
-          <t>LHQ
-高电平</t>
-        </is>
-      </c>
-      <c r="C1310" s="3" t="inlineStr">
-        <is>
-          <t>LHQD2COTOPP</t>
-        </is>
-      </c>
-      <c r="D1310" s="3" t="n"/>
+      <c r="A1310" s="4" t="n"/>
+      <c r="B1310" s="4" t="n"/>
+      <c r="C1310" s="5" t="n"/>
+      <c r="D1310" s="5" t="inlineStr">
+        <is>
+          <t>LHQD4ARCOT</t>
+        </is>
+      </c>
     </row>
     <row r="1311">
       <c r="A1311" s="6" t="n"/>
@@ -15007,7 +14887,7 @@
       <c r="C1311" s="7" t="n"/>
       <c r="D1311" s="7" t="inlineStr">
         <is>
-          <t>LHQD4ARCOT</t>
+          <t>LHSNQD1COT</t>
         </is>
       </c>
     </row>
@@ -15015,90 +14895,70 @@
       <c r="A1312" s="2" t="n"/>
       <c r="B1312" s="2" t="inlineStr">
         <is>
-          <t>LHSNQ
-高·SNQ</t>
-        </is>
-      </c>
-      <c r="C1312" s="3" t="inlineStr">
-        <is>
-          <t>LHSNQD2COT</t>
-        </is>
-      </c>
-      <c r="D1312" s="3" t="n"/>
+          <t>LN
+低电平透明</t>
+        </is>
+      </c>
+      <c r="C1312" s="8" t="inlineStr">
+        <is>
+          <t>LNCSNQD1COT</t>
+        </is>
+      </c>
+      <c r="D1312" s="8" t="inlineStr">
+        <is>
+          <t>LNCSNQD1COT</t>
+        </is>
+      </c>
     </row>
     <row r="1313">
-      <c r="A1313" s="6" t="n"/>
-      <c r="B1313" s="6" t="n"/>
-      <c r="C1313" s="7" t="n"/>
-      <c r="D1313" s="7" t="inlineStr">
-        <is>
-          <t>LHSNQD1COT</t>
-        </is>
-      </c>
+      <c r="A1313" s="4" t="n"/>
+      <c r="B1313" s="4" t="n"/>
+      <c r="C1313" s="5" t="inlineStr">
+        <is>
+          <t>GLNCNQD1COT</t>
+        </is>
+      </c>
+      <c r="D1313" s="5" t="n"/>
     </row>
     <row r="1314">
-      <c r="A1314" s="10" t="n"/>
-      <c r="B1314" s="10" t="inlineStr">
-        <is>
-          <t>LNCNQ
-低·CNQ</t>
-        </is>
-      </c>
-      <c r="C1314" s="11" t="inlineStr">
+      <c r="A1314" s="4" t="n"/>
+      <c r="B1314" s="4" t="n"/>
+      <c r="C1314" s="5" t="inlineStr">
+        <is>
+          <t>GLNQD1COT</t>
+        </is>
+      </c>
+      <c r="D1314" s="5" t="n"/>
+    </row>
+    <row r="1315">
+      <c r="A1315" s="4" t="n"/>
+      <c r="B1315" s="4" t="n"/>
+      <c r="C1315" s="5" t="inlineStr">
         <is>
           <t>LNCNQD4COT</t>
         </is>
       </c>
-      <c r="D1314" s="11" t="n"/>
-    </row>
-    <row r="1315">
-      <c r="A1315" s="10" t="n"/>
-      <c r="B1315" s="10" t="inlineStr">
-        <is>
-          <t>LNCSNQ
-低·CSNQ</t>
-        </is>
-      </c>
-      <c r="C1315" s="12" t="inlineStr">
-        <is>
-          <t>LNCSNQD1COT</t>
-        </is>
-      </c>
-      <c r="D1315" s="12" t="inlineStr">
-        <is>
-          <t>LNCSNQD1COT</t>
-        </is>
-      </c>
+      <c r="D1315" s="5" t="n"/>
     </row>
     <row r="1316">
-      <c r="A1316" s="10" t="n"/>
-      <c r="B1316" s="10" t="inlineStr">
-        <is>
-          <t>LNQ
-低电平</t>
-        </is>
-      </c>
-      <c r="C1316" s="11" t="inlineStr">
+      <c r="A1316" s="4" t="n"/>
+      <c r="B1316" s="4" t="n"/>
+      <c r="C1316" s="5" t="inlineStr">
         <is>
           <t>LNQD4COT</t>
         </is>
       </c>
-      <c r="D1316" s="11" t="n"/>
+      <c r="D1316" s="5" t="n"/>
     </row>
     <row r="1317">
-      <c r="A1317" s="2" t="n"/>
-      <c r="B1317" s="2" t="inlineStr">
-        <is>
-          <t>LNSNQ
-低·SNQ</t>
-        </is>
-      </c>
-      <c r="C1317" s="3" t="inlineStr">
+      <c r="A1317" s="4" t="n"/>
+      <c r="B1317" s="4" t="n"/>
+      <c r="C1317" s="5" t="inlineStr">
         <is>
           <t>LNSNQD1COTOPU</t>
         </is>
       </c>
-      <c r="D1317" s="3" t="n"/>
+      <c r="D1317" s="5" t="n"/>
     </row>
     <row r="1318">
       <c r="A1318" s="6" t="n"/>
@@ -15269,13 +15129,13 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="185">
+  <mergeCells count="169">
     <mergeCell ref="B179:B220"/>
     <mergeCell ref="B568:B572"/>
     <mergeCell ref="B34:B36"/>
     <mergeCell ref="B1289:B1290"/>
+    <mergeCell ref="B1312:B1318"/>
     <mergeCell ref="A225:A296"/>
-    <mergeCell ref="B611:B614"/>
     <mergeCell ref="B1248:B1252"/>
     <mergeCell ref="A1163:A1167"/>
     <mergeCell ref="A40:A71"/>
@@ -15284,17 +15144,14 @@
     <mergeCell ref="A1172:A1176"/>
     <mergeCell ref="B302:B311"/>
     <mergeCell ref="B1300:B1301"/>
-    <mergeCell ref="B573:B576"/>
+    <mergeCell ref="B508:B511"/>
+    <mergeCell ref="B1185:B1189"/>
     <mergeCell ref="B236:B247"/>
-    <mergeCell ref="B644:B647"/>
     <mergeCell ref="B422:B439"/>
     <mergeCell ref="B387:B414"/>
     <mergeCell ref="A1319:A1321"/>
-    <mergeCell ref="B1317:B1318"/>
-    <mergeCell ref="B1075:B1078"/>
     <mergeCell ref="A325:A340"/>
     <mergeCell ref="B596:B598"/>
-    <mergeCell ref="B604:B610"/>
     <mergeCell ref="A385:A414"/>
     <mergeCell ref="A696:A715"/>
     <mergeCell ref="B670:B672"/>
@@ -15302,14 +15159,11 @@
     <mergeCell ref="B814:B907"/>
     <mergeCell ref="A1142:A1147"/>
     <mergeCell ref="B911:B953"/>
-    <mergeCell ref="B564:B567"/>
     <mergeCell ref="A422:A477"/>
-    <mergeCell ref="B527:B530"/>
-    <mergeCell ref="B1080:B1116"/>
     <mergeCell ref="B40:B67"/>
     <mergeCell ref="B778:B781"/>
+    <mergeCell ref="B535:B544"/>
     <mergeCell ref="B230:B235"/>
-    <mergeCell ref="B1131:B1139"/>
     <mergeCell ref="B351:B361"/>
     <mergeCell ref="A302:A311"/>
     <mergeCell ref="B72:B170"/>
@@ -15317,13 +15171,17 @@
     <mergeCell ref="B1148:B1153"/>
     <mergeCell ref="B582:B586"/>
     <mergeCell ref="A1156:A1162"/>
+    <mergeCell ref="B625:B626"/>
     <mergeCell ref="A1168:A1171"/>
     <mergeCell ref="B221:B224"/>
+    <mergeCell ref="B639:B640"/>
     <mergeCell ref="B681:B683"/>
     <mergeCell ref="B782:B805"/>
     <mergeCell ref="B553:B554"/>
+    <mergeCell ref="B610:B618"/>
     <mergeCell ref="B959:B968"/>
     <mergeCell ref="B363:B367"/>
+    <mergeCell ref="B1072:B1130"/>
     <mergeCell ref="B551:B552"/>
     <mergeCell ref="A778:A805"/>
     <mergeCell ref="B1242:B1243"/>
@@ -15335,12 +15193,12 @@
     <mergeCell ref="A1302:A1318"/>
     <mergeCell ref="B415:B419"/>
     <mergeCell ref="B594:B595"/>
-    <mergeCell ref="B1191:B1196"/>
-    <mergeCell ref="B1117:B1126"/>
+    <mergeCell ref="B673:B678"/>
     <mergeCell ref="B1291:B1299"/>
     <mergeCell ref="A298:A301"/>
     <mergeCell ref="B1177:B1178"/>
     <mergeCell ref="B341:B350"/>
+    <mergeCell ref="B636:B637"/>
     <mergeCell ref="A1265:A1290"/>
     <mergeCell ref="B1258:B1261"/>
     <mergeCell ref="A1183:A1189"/>
@@ -15348,113 +15206,99 @@
     <mergeCell ref="A806:A907"/>
     <mergeCell ref="B555:B556"/>
     <mergeCell ref="B1179:B1180"/>
-    <mergeCell ref="B620:B621"/>
+    <mergeCell ref="B619:B624"/>
+    <mergeCell ref="B528:B534"/>
     <mergeCell ref="A1291:A1301"/>
-    <mergeCell ref="B508:B510"/>
-    <mergeCell ref="B654:B657"/>
-    <mergeCell ref="B661:B665"/>
+    <mergeCell ref="B521:B527"/>
     <mergeCell ref="B993:B1071"/>
     <mergeCell ref="B1244:B1245"/>
     <mergeCell ref="A72:A178"/>
     <mergeCell ref="A1324:A1331"/>
     <mergeCell ref="B748:B776"/>
-    <mergeCell ref="B1140:B1141"/>
-    <mergeCell ref="B514:B516"/>
     <mergeCell ref="B806:B813"/>
     <mergeCell ref="A369:A384"/>
+    <mergeCell ref="B641:B647"/>
     <mergeCell ref="B1163:B1167"/>
     <mergeCell ref="B420:B421"/>
     <mergeCell ref="B1172:B1176"/>
     <mergeCell ref="B1246:B1247"/>
     <mergeCell ref="B1262:B1264"/>
+    <mergeCell ref="B653:B657"/>
     <mergeCell ref="B627:B629"/>
     <mergeCell ref="A1246:A1257"/>
+    <mergeCell ref="B573:B581"/>
     <mergeCell ref="B696:B711"/>
-    <mergeCell ref="B1240:B1241"/>
     <mergeCell ref="B1183:B1184"/>
     <mergeCell ref="A1191:A1239"/>
     <mergeCell ref="B648:B650"/>
-    <mergeCell ref="B1310:B1311"/>
     <mergeCell ref="B371:B372"/>
     <mergeCell ref="A716:A733"/>
     <mergeCell ref="B589:B591"/>
     <mergeCell ref="B478:B491"/>
     <mergeCell ref="B497:B503"/>
     <mergeCell ref="A747:A776"/>
+    <mergeCell ref="B660:B665"/>
     <mergeCell ref="B1181:B1182"/>
-    <mergeCell ref="B1312:B1313"/>
-    <mergeCell ref="B511:B513"/>
     <mergeCell ref="A735:A746"/>
     <mergeCell ref="A2:A36"/>
     <mergeCell ref="A312:A324"/>
-    <mergeCell ref="B506:B507"/>
     <mergeCell ref="B2:B33"/>
     <mergeCell ref="A420:A421"/>
     <mergeCell ref="B1253:B1257"/>
-    <mergeCell ref="B1127:B1130"/>
     <mergeCell ref="B68:B71"/>
-    <mergeCell ref="B674:B678"/>
+    <mergeCell ref="B712:B715"/>
     <mergeCell ref="A1262:A1264"/>
-    <mergeCell ref="B712:B715"/>
     <mergeCell ref="B1324:B1331"/>
     <mergeCell ref="B1156:B1162"/>
     <mergeCell ref="B1168:B1171"/>
-    <mergeCell ref="B641:B643"/>
+    <mergeCell ref="B557:B567"/>
     <mergeCell ref="A38:A39"/>
     <mergeCell ref="B171:B178"/>
     <mergeCell ref="B1154:B1155"/>
     <mergeCell ref="A478:A491"/>
-    <mergeCell ref="B635:B636"/>
-    <mergeCell ref="B504:B505"/>
+    <mergeCell ref="B1131:B1141"/>
+    <mergeCell ref="B512:B520"/>
     <mergeCell ref="B1322:B1323"/>
     <mergeCell ref="B731:B733"/>
     <mergeCell ref="B373:B384"/>
     <mergeCell ref="A1177:A1182"/>
     <mergeCell ref="B666:B669"/>
     <mergeCell ref="A1322:A1323"/>
+    <mergeCell ref="B504:B507"/>
     <mergeCell ref="A492:A680"/>
     <mergeCell ref="A684:A695"/>
     <mergeCell ref="A908:A953"/>
     <mergeCell ref="B385:B386"/>
-    <mergeCell ref="B531:B534"/>
+    <mergeCell ref="B969:B992"/>
     <mergeCell ref="A681:A683"/>
-    <mergeCell ref="B535:B539"/>
-    <mergeCell ref="B969:B992"/>
     <mergeCell ref="A415:A419"/>
-    <mergeCell ref="B521:B526"/>
     <mergeCell ref="A1148:A1153"/>
     <mergeCell ref="B717:B730"/>
-    <mergeCell ref="B1186:B1188"/>
     <mergeCell ref="B38:B39"/>
-    <mergeCell ref="B540:B544"/>
     <mergeCell ref="B651:B652"/>
-    <mergeCell ref="B1198:B1222"/>
-    <mergeCell ref="B519:B520"/>
     <mergeCell ref="A1258:A1261"/>
+    <mergeCell ref="B1302:B1311"/>
     <mergeCell ref="B587:B588"/>
     <mergeCell ref="A179:A224"/>
-    <mergeCell ref="B622:B623"/>
+    <mergeCell ref="B607:B609"/>
     <mergeCell ref="B1265:B1286"/>
     <mergeCell ref="A954:A1071"/>
     <mergeCell ref="B1287:B1288"/>
-    <mergeCell ref="B1072:B1074"/>
     <mergeCell ref="B492:B496"/>
-    <mergeCell ref="B624:B625"/>
     <mergeCell ref="B298:B301"/>
-    <mergeCell ref="B557:B563"/>
     <mergeCell ref="B954:B958"/>
     <mergeCell ref="B248:B296"/>
     <mergeCell ref="A1154:A1155"/>
-    <mergeCell ref="B601:B603"/>
     <mergeCell ref="A341:A361"/>
     <mergeCell ref="B630:B634"/>
     <mergeCell ref="B908:B910"/>
     <mergeCell ref="B1319:B1321"/>
-    <mergeCell ref="B577:B581"/>
+    <mergeCell ref="B599:B606"/>
     <mergeCell ref="B1223:B1239"/>
     <mergeCell ref="B440:B477"/>
+    <mergeCell ref="B1192:B1222"/>
     <mergeCell ref="B225:B229"/>
-    <mergeCell ref="B616:B619"/>
+    <mergeCell ref="B1240:B1241"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Iterate A/B label check: fix FA/SDFSYNC and refresh Excel.
Round1 B findings: stop skeleton 复合· fallback for FA and SDFSYNC;
add explicit clock KEY families; use Chinese fine_zh for layout cells.
Regenerate preview Excel and ab_label_inventory for audit.
Round2 A/B both PASS (unmatched=0, missing fine_zh=0).

Co-authored-by: EsaLongs <EsaLongs@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/preview/NP1PP_vs_C1Y_preview.xlsx
+++ b/preview/NP1PP_vs_C1Y_preview.xlsx
@@ -14407,7 +14407,7 @@
       <c r="B1269" s="2" t="inlineStr">
         <is>
           <t>BOUNDARY
-BOUNDARY</t>
+边界单元</t>
         </is>
       </c>
       <c r="C1269" s="8" t="inlineStr">
@@ -14664,7 +14664,7 @@
       <c r="B1291" s="2" t="inlineStr">
         <is>
           <t>HDDICWY
-HDDICWY</t>
+版图单元</t>
         </is>
       </c>
       <c r="C1291" s="3" t="n"/>
@@ -14689,7 +14689,7 @@
       <c r="B1293" s="2" t="inlineStr">
         <is>
           <t>HDDID
-HDDID</t>
+版图单元</t>
         </is>
       </c>
       <c r="C1293" s="3" t="inlineStr">

</xml_diff>